<commit_message>
Add a history note to every poem; fix four language captions
Each of the 48 poems shown in full now has its own "A note on history"
(data/context_notes.json). Denmark, Italy, Japan and Russia were labelled
with an older English version's language under the original text.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -7483,7 +7483,7 @@
       </c>
       <c r="N53" s="13" t="inlineStr">
         <is>
-          <t>English and German translations of Danish poem</t>
+          <t>Danish</t>
         </is>
       </c>
       <c r="O53" s="13" t="n"/>
@@ -12515,7 +12515,7 @@
       <c r="M90" s="14" t="n"/>
       <c r="N90" s="13" t="inlineStr">
         <is>
-          <t>English, from Italian</t>
+          <t>Italian</t>
         </is>
       </c>
       <c r="O90" s="13" t="n"/>
@@ -12831,7 +12831,7 @@
       <c r="M92" s="14" t="n"/>
       <c r="N92" s="13" t="inlineStr">
         <is>
-          <t>Romanised Japanese and English</t>
+          <t>Japanese</t>
         </is>
       </c>
       <c r="O92" s="13" t="n"/>
@@ -20425,7 +20425,7 @@
       </c>
       <c r="N150" s="13" t="inlineStr">
         <is>
-          <t>English, from Russian</t>
+          <t>Russian</t>
         </is>
       </c>
       <c r="O150" s="13" t="n"/>

</xml_diff>

<commit_message>
Add batch 1 of new poem passages (15 countries)
Cabo Verde, Costa Rica, Croatia, Cuba, Cyprus, Czechia, Dominican
Republic, El Salvador, Estonia, Georgia, Greece, Guatemala, Guyana,
Haiti and Holy See now show a passage in the original language beside
English, each with a history note. Originals are cut from the linked
public-domain sources; English versions are new drafts, recorded as such
in the spreadsheet's translation notes. 63 poems to read in total.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 48 paired passages • 147 unfilled</t>
+          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 63 paired passages • 132 unfilled</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -5001,8 +5001,44 @@
           <t>The Power of Love</t>
         </is>
       </c>
-      <c r="F35" s="13" t="n"/>
-      <c r="G35" s="13" t="n"/>
+      <c r="F35" s="13" t="inlineStr">
+        <is>
+          <t>Ca tem nada na es bida
+Mas grande que amor
+Se Deus ca tem medida
+Amor inda é maior.
+Maior que mar, que céu
+Mas, entre tudo cretcheu
+De meu inda é maior
+Cretcheu más sabe,
+É quel que é di meu
+Ele é que é tchabe
+Que abrim nha céu.
+Cretcheu más sabe
+É quel qui crem
+Ai sim perdel
+Morte dja bem</t>
+        </is>
+      </c>
+      <c r="G35" s="13" t="inlineStr">
+        <is>
+          <t>There is nothing in this life
+Greater than love;
+If God has no measure,
+Love is greater still.
+Greater than the sea, than the sky,
+But, above all, my own beloved
+Is greater still.
+The sweetest beloved
+Is the one who is mine;
+They are the key
+That opens my heaven.
+The sweetest beloved
+Is the one who loves me;
+Ah, if I lost them,
+Death would come.</t>
+        </is>
+      </c>
       <c r="H35" s="13" t="inlineStr">
         <is>
           <t>Eugénio Tavares</t>
@@ -5076,7 +5112,8 @@
       </c>
       <c r="W35" s="13" t="inlineStr">
         <is>
-          <t>Tavares died 1 June 1930. Original lyric is public domain in life-plus-70 jurisdictions; the website’s modern commentary, later musical arrangements and recordings are separate. Creole spelling varies between editions. The selection is the original-language text; an existing English translation is not required.</t>
+          <t>Tavares died 1 June 1930. Original lyric is public domain in life-plus-70 jurisdictions; the website’s modern commentary, later musical arrangements and recordings are separate. Creole spelling varies between editions. The selection is the original-language text; an existing English translation is not required.
+Passage update (29 October 2026): First two stanzas, 15 lines. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X35" s="13" t="inlineStr">
@@ -6548,8 +6585,42 @@
           <t>Will They Come? (gender not specified in title)</t>
         </is>
       </c>
-      <c r="F46" s="13" t="n"/>
-      <c r="G46" s="13" t="n"/>
+      <c r="F46" s="13" t="inlineStr">
+        <is>
+          <t>Desciende hasta el jardín, amada mía;
+es hora en que las rosas y jazmines
+inciensan a la tarde; en los confines
+va cerrando sus párpados el día.
+Anhelo de tus labios la ambrosía;
+desciende hasta el jardín; los bandolines
+alados ya no trinan; hay festines
+de estrellas en la bóveda sombría.
+La luna riega el ámbar de su lumbre
+desde la comba inmensa de los cielos
+y baja, hecha fulgor, hasta las pomas.
+Como garza se eleva tras la cumbre
+del monte, y el jazmín de mis anhelos
+te invita a descender, con sus aromas.</t>
+        </is>
+      </c>
+      <c r="G46" s="13" t="inlineStr">
+        <is>
+          <t>Come down to the garden, my beloved;
+It is the hour when the roses and jasmine
+Perfume the evening like incense; at the edge of the sky
+The day is closing its eyelids.
+I long for the ambrosia of your lips;
+Come down to the garden; the winged
+Mandolins have stopped their trilling; there are feasts
+Of stars in the darkening vault.
+The moon pours out the amber of its light
+From the immense curve of the heavens,
+And comes down, turned to radiance, to the fruit trees.
+Like a heron it rises behind the summit
+Of the mountain, and the jasmine of my longing
+Invites you, with its scent, to come down.</t>
+        </is>
+      </c>
       <c r="H46" s="13" t="inlineStr">
         <is>
           <t>Lisímaco Chavarría</t>
@@ -6621,7 +6692,8 @@
       </c>
       <c r="W46" s="13" t="inlineStr">
         <is>
-          <t>Journal says the sonnet had been preserved in Margarita Martínez’s album and was unpublished until then. Original sonnet only; modern library descriptions and other journal contributions are separate. The selection is the original-language text; an existing English translation is not required.</t>
+          <t>Journal says the sonnet had been preserved in Margarita Martínez’s album and was unpublished until then. Original sonnet only; modern library descriptions and other journal contributions are separate. The selection is the original-language text; an existing English translation is not required.
+Passage update (29 October 2026): Complete sonnet, 14 lines. Two OCR slips in the 1920 scan are corrected (“cum bre” to “cumbre”, “Su” to “su”); the wording is unchanged. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X46" s="13" t="inlineStr">
@@ -6800,8 +6872,42 @@
           <t>The Consolation of Hair</t>
         </is>
       </c>
-      <c r="F48" s="13" t="n"/>
-      <c r="G48" s="13" t="n"/>
+      <c r="F48" s="13" t="inlineStr">
+        <is>
+          <t>Gledo sam te sinoć. U snu. Tužan. Mrtvu.
+U dvorani kobnoj, u idili cvijeća,
+Na visokom odru, u agoniji svijeća,
+Gotov da ti predam život kao žrtvu.
+Nisam plako. Nisam. Zapanjen sam stao
+U dvorani kobnoj, punoj smrti krasne,
+Sumnjajući da su tamne oči jasne
+Odakle mi nekad bolji život sjao.
+Sve baš, sve je mrtvo: oči dah i ruke,
+Sve što očajanjem htjedoh da oživim
+U slijepoj stravi i u strasti muke,
+U dvorani kobnoj, mislima u sivim.
+Samo kosa tvoja još je bila živa,
+Pa mi reče: — Miruj! U smrti se sniva.</t>
+        </is>
+      </c>
+      <c r="G48" s="13" t="inlineStr">
+        <is>
+          <t>I saw you last night. In a dream. Sad. Dead.
+In a fateful hall, in an idyll of flowers,
+On a high bier, in the agony of candles,
+Ready to give you my life as a sacrifice.
+I did not weep. I did not. Stunned, I stood
+In the fateful hall, full of beautiful death,
+Doubting that those dark, clear eyes
+Were where a better life once shone on me.
+All, yes, all is dead: eyes, breath and hands,
+All that in despair I longed to bring to life
+In blind terror and in the passion of torment,
+In the fateful hall, among grey thoughts.
+Only your hair was still alive,
+And it said to me: “Be still! In death one dreams.”</t>
+        </is>
+      </c>
       <c r="H48" s="13" t="inlineStr">
         <is>
           <t>Antun Gustav Matoš</t>
@@ -6873,7 +6979,8 @@
       </c>
       <c r="W48" s="13" t="inlineStr">
         <is>
-          <t>Check transcription against a historical edition before final quotation; modern English translations have separate rights.</t>
+          <t>Check transcription against a historical edition before final quotation; modern English translations have separate rights.
+Passage update (29 October 2026): Complete sonnet, 14 lines. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X48" s="13" t="inlineStr">
@@ -6935,8 +7042,38 @@
           <t>To Him — In the flattering dawn (first line)</t>
         </is>
       </c>
-      <c r="F49" s="13" t="n"/>
-      <c r="G49" s="13" t="n"/>
+      <c r="F49" s="13" t="inlineStr">
+        <is>
+          <t>Volaban los años, y yo vanamente
+Buscando seguía mi hermosa visión...
+Mas dio al fin la hora; brillar vi tu frente,
+Y «es él», dijo al punto mi fiel corazón.
+Porque era, no hay duda, tu imagen querida,
+-Que el alma inspirada logró adivinar-
+Aquella que en alba feliz de mi vida
+Miré para nunca poderla olvidar.
+Por ti fue mi dulce suspiro primero;
+Por ti mi constante, secreto anhelar
+Y en balde el destino -mostrándose fiero-
+Tendió entre nosotros las olas del mar.</t>
+        </is>
+      </c>
+      <c r="G49" s="13" t="inlineStr">
+        <is>
+          <t>The years flew by, and still, in vain,
+I went on searching for my beautiful vision…
+But at last the hour came; I saw your brow shine,
+And “It is he,” my faithful heart said at once.
+For it was, beyond doubt, your beloved image
+— which my inspired soul had managed to divine —
+The one I saw in the happy dawn of my life
+And have never been able to forget.
+For you was my first sweet sigh;
+For you my constant, secret longing;
+And in vain did fate, showing its cruelty,
+Stretch the waves of the sea between us.</t>
+        </is>
+      </c>
       <c r="H49" s="13" t="inlineStr">
         <is>
           <t>Gertrudis Gómez de Avellaneda</t>
@@ -7006,7 +7143,8 @@
       </c>
       <c r="W49" s="13" t="inlineStr">
         <is>
-          <t>Cuban-born writer with a major literary career in Spain; not a modern nationality claim about a colonial-era author. Original-language poem only; modern translations and recordings are separate. Retain attribution and source/license links for copyrightable transcription material.</t>
+          <t>Cuban-born writer with a major literary career in Spain; not a modern nationality claim about a colonial-era author. Original-language poem only; modern translations and recordings are separate. Retain attribution and source/license links for copyrightable transcription material.
+Passage update (29 October 2026): Twelve consecutive lines from the second part of the poem (from “Volaban los años” to “las olas del mar”). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X49" s="13" t="inlineStr">
@@ -7064,8 +7202,30 @@
           <t>Rhymes of Love, poem59</t>
         </is>
       </c>
-      <c r="F50" s="13" t="n"/>
-      <c r="G50" s="13" t="n"/>
+      <c r="F50" s="13" t="inlineStr">
+        <is>
+          <t>Διατί ποτέ μου δεν είδα ‘ξ αυτήσ σου
+θάρος να λείψουν τα λαμπρά ‘που μένα,
+τα ποια μου δώκεν το γλυκύν το δείσ σου
+και δεν παύγουν ποτέ καιρόν κανέναν,
+διατί δεν με ψηφά στην δούλεψήσ σου,
+μισεύγω από την Κύπρον εις τα ξένα
+αμμ’ έξευρε όπου πάγω, αγγέλισσά μου,
+πάντα μ’ εσέν θέλ’ είσταιν η καρδιά μου.</t>
+        </is>
+      </c>
+      <c r="G50" s="13" t="inlineStr">
+        <is>
+          <t>Because I have never once seen in you
+The courage to take from me the bright flames
+That your sweet glance gave me,
+And that never cease at any time,
+Because you take no account of my devotion,
+I am leaving Cyprus for foreign lands;
+But know, wherever I go, my angel,
+My heart will always be with you.</t>
+        </is>
+      </c>
       <c r="H50" s="13" t="inlineStr">
         <is>
           <t>Anonymous Cypriot Renaissance poet</t>
@@ -7135,7 +7295,8 @@
       </c>
       <c r="W50" s="13" t="inlineStr">
         <is>
-          <t>Use the anonymous Renaissance Greek verses. The booklet’s English translation, photographs and the modern critical apparatus are separate. Collection appeared partly in 1881 and in full in 1952; exact first printing of this individual poem is not established. The selection is the original-language text; an existing English translation is not required.</t>
+          <t>Use the anonymous Renaissance Greek verses. The booklet’s English translation, photographs and the modern critical apparatus are separate. Collection appeared partly in 1881 and in full in 1952; exact first printing of this individual poem is not established. The selection is the original-language text; an existing English translation is not required.
+Passage update (29 October 2026): Complete poem, 8 lines (one ottava rima stanza). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X50" s="13" t="inlineStr">
@@ -7197,8 +7358,38 @@
           <t>A Girl's Song</t>
         </is>
       </c>
-      <c r="F51" s="13" t="n"/>
-      <c r="G51" s="13" t="n"/>
+      <c r="F51" s="13" t="inlineStr">
+        <is>
+          <t>A ptáček jasnohlasý
+mi odpovídá v písni:
+Vím, jaká pečeť asi
+ta zpěvná ústa tísní.
+Vím, proč tak oněměly
+rty dívčí v prostřed pění:
+je uzamknul ret vřelý,
+je stisklo políbení.
+Když srdce k srdci sletí,
+pak umlká a slyší
+zpěv andělů jen pěti
+tou sladkou němou tiší.</t>
+        </is>
+      </c>
+      <c r="G51" s="13" t="inlineStr">
+        <is>
+          <t>And a clear-voiced little bird
+Answers me in song:
+“I know what seal, it seems,
+Is pressing on that singing mouth.
+I know why the girl’s lips
+Fell silent in mid-song:
+Warm lips have locked them shut,
+A kiss has pressed them closed.
+When heart flies down to heart,
+It falls quiet, and hears
+Only the angels singing
+In that sweet, wordless hush.”</t>
+        </is>
+      </c>
       <c r="H51" s="13" t="inlineStr">
         <is>
           <t>Eliška Krásnohorská</t>
@@ -7270,7 +7461,8 @@
       </c>
       <c r="W51" s="13" t="inlineStr">
         <is>
-          <t>Original-language poem only; modern translations and recordings are separate. Retain attribution and source/license links for copyrightable transcription material.</t>
+          <t>Original-language poem only; modern translations and recordings are separate. Retain attribution and source/license links for copyrightable transcription material.
+Passage update (29 October 2026): Final three stanzas, 12 lines. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X51" s="13" t="inlineStr">
@@ -7805,8 +7997,44 @@
           <t>Love and Longing</t>
         </is>
       </c>
-      <c r="F56" s="13" t="n"/>
-      <c r="G56" s="13" t="n"/>
+      <c r="F56" s="13" t="inlineStr">
+        <is>
+          <t>Ven y tu mano del pecho amante
+calme amorosa las penas mil,
+¡oh de mis ansias único objeto!
+Ven, que a ti sólo quiero en secreto
+contar mis sueños de amor febril.
+Mas no, que nunca mi amante anhelo
+podré decirte libre de afán,
+gimiendo a solas, en desconsuelo,
+cual mis suspiros, en raudo vuelo,
+mis ilusiones perdidas van.
+Tuya es mi vida, tuya mi suerte,
+de ti mi dicha pende o mi mal;
+si al dolor quieres que venza fuerte,
+sobre mi frente pálida vierte
+de tu ternura todo el raudal.</t>
+        </is>
+      </c>
+      <c r="G56" s="13" t="inlineStr">
+        <is>
+          <t>Come, and let your hand, with love,
+Ease the thousand sorrows of my loving breast,
+O sole object of my longing!
+Come, for to you alone I wish, in secret,
+To tell my dreams of feverish love.
+But no: never shall I be able
+To tell you my loving longing free of fear;
+Moaning alone, disconsolate,
+Like my sighs, in swift flight,
+My lost illusions slip away.
+Yours is my life, yours my fate;
+My joy or my sorrow hangs on you;
+If you would have me overcome my pain,
+Pour upon my pale brow
+The whole flood of your tenderness.</t>
+        </is>
+      </c>
       <c r="H56" s="13" t="inlineStr">
         <is>
           <t>Salomé Ureña de Henríquez</t>
@@ -7878,7 +8106,8 @@
       </c>
       <c r="W56" s="13" t="inlineStr">
         <is>
-          <t>Author died 1897. The linked primary-text excerpt is sufficient for quotation; it is not the complete poem. Preserve the original wording rather than online variants. The selection is the original-language text; an existing English translation is not required.</t>
+          <t>Author died 1897. The linked primary-text excerpt is sufficient for quotation; it is not the complete poem. Preserve the original wording rather than online variants. The selection is the original-language text; an existing English translation is not required.
+Passage update (29 October 2026): The last three stanzas of the printed fragment, 15 lines. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X56" s="13" t="inlineStr">
@@ -8241,8 +8470,42 @@
           <t>Moon over the Ranch</t>
         </is>
       </c>
-      <c r="F59" s="13" t="n"/>
-      <c r="G59" s="13" t="n"/>
+      <c r="F59" s="13" t="inlineStr">
+        <is>
+          <t>Vagar, soñando versos, en silentes caminos,
+con la dorada lluvia del sol sobre tu frente;
+y en un tronco sentados, mirarme largamente
+en las dormidas aguas de tus ojos hialinos…
+“Y qué linda”, dijeran al verte, campesinos
+de esos que con sus vacas van buscando una fuente,
+y yo: “Sus ojos miran, miran más dulcemente
+que dos estrellas blancas en cielos vespertinos”.
+Y tú te sonreirías sin vanidad ninguna;
+después en nuestro rancho se entraría la luna
+y ladraría al vernos, el perro blanco y fiel…
+Como el café maduro fuera tu boca, mía,
+y en el rancho con luna, mi boca bebería
+en la flor de tus labios, un “te quiero” de miel.</t>
+        </is>
+      </c>
+      <c r="G59" s="13" t="inlineStr">
+        <is>
+          <t>To wander, dreaming verses, along silent paths,
+With the golden rain of the sun upon your brow;
+And, seated on a log, to gaze at myself at length
+In the sleeping waters of your glassy eyes…
+“And how lovely she is,” country people would say on seeing you,
+The kind who go with their cows in search of a spring,
+And I: “Her eyes look, they look more sweetly
+Than two white stars in evening skies.”
+And you would smile without the least vanity;
+Then the moon would come into our farmhouse
+And, seeing us, the white and faithful dog would bark…
+Your mouth, mine, would be like ripe coffee,
+And in the moonlit farmhouse my mouth would drink
+From the flower of your lips a honeyed “I love you”.</t>
+        </is>
+      </c>
       <c r="H59" s="13" t="inlineStr">
         <is>
           <t>Alfredo Espino</t>
@@ -8314,7 +8577,8 @@
       </c>
       <c r="W59" s="13" t="inlineStr">
         <is>
-          <t>Modern editorial matter excluded. 1936 is collection-publication year, not composition. Original Spanish requires no translation.</t>
+          <t>Modern editorial matter excluded. 1936 is collection-publication year, not composition. Original Spanish requires no translation.
+Passage update (29 October 2026): Complete sonnet, 14 lines. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X59" s="13" t="inlineStr">
@@ -8594,8 +8858,38 @@
           <t>Two Clear Eyes</t>
         </is>
       </c>
-      <c r="F62" s="13" t="n"/>
-      <c r="G62" s="13" t="n"/>
+      <c r="F62" s="13" t="inlineStr">
+        <is>
+          <t>Kaks selget silma mulle vaatnud
+Kui taeva tähed südame,
+Kaks selget silma põue saatnud
+Mul täheläiget äkiste.
+Kust oleks teadnud taganeda
+Ma vaene vaga palgilta?
+Nii peenet nägu põgeneda,
+Nii selget silma süüdelda?
+Et ühtepuhku mõttes suigun,
+Et mõistus kõik mul metsa läind.
+Et nagu unes ala tuigun:
+Kaks selget silma seda teind!</t>
+        </is>
+      </c>
+      <c r="G62" s="13" t="inlineStr">
+        <is>
+          <t>Two clear eyes have looked into my heart
+Like the stars of heaven,
+Two clear eyes have sent into my breast
+A sudden gleam of starlight.
+How could I have known to turn away,
+Poor, meek me, from that face?
+To flee a face so fine,
+To blame an eye so clear?
+So that I keep drifting off in thought,
+So that my wits have all gone astray,
+So that I stumble about as in a dream:
+Two clear eyes have done all this!</t>
+        </is>
+      </c>
       <c r="H62" s="13" t="inlineStr">
         <is>
           <t>Lydia Koidula</t>
@@ -8665,7 +8959,8 @@
       </c>
       <c r="W62" s="13" t="inlineStr">
         <is>
-          <t>Quotation is from the original poem within a historical study. Read page image rather than trusting OCR; historical spelling retained. Poet is a woman, 1843–1886; modern translations excluded.</t>
+          <t>Quotation is from the original poem within a historical study. Read page image rather than trusting OCR; historical spelling retained. Poet is a woman, 1843–1886; modern translations excluded.
+Passage update (29 October 2026): First three stanzas, 12 lines. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X62" s="13" t="inlineStr">
@@ -9680,8 +9975,38 @@
           <t>The Knight in the Panther Skin — Prologue on love</t>
         </is>
       </c>
-      <c r="F70" s="13" t="n"/>
-      <c r="G70" s="13" t="n"/>
+      <c r="F70" s="13" t="inlineStr">
+        <is>
+          <t>მიჯნურობა არის ტურფა, საცოდნელად ძნელი გვარი;
+მიჯნურობა სხვა რამეა, არ სიძვისა დასადარი:
+იგი სხვაა, სიძვა სხვაა, შუა უზის დიდი მზღვარი,
+ნუვინ გაჰრევთ ერთმანერთსა! გესმას ჩემი ნაუბარი!
+ხამს მიჯნური ხანიერი, არ მეძავი, ბილწი, მრუში,
+რა მოჰშორდეს მოყვარესა, გაამრავლოს სულთქმა, უში,
+გული ერთსა დააჯეროს, კუშტი მიჰხვდეს, თუნდა ქუში;
+მძულს უგულო სიყვარული, ხვევნა, კოცნა, მტლაშა-მტლუში.
+ამა საქმესა მიჯნური ნუ უხმობს მიჯნურობასა:
+დღეს ერთი უნდეს, ხვალე სხვა, სთმობდეს გაყრისა თმობასა;
+ესე მღერასა ბედითსა ჰგავს ვაჟთა, ყმაწვილობასა.
+კარგი მიჯნური იგია, ვინ იქმს სოფლისა თმობასა.</t>
+        </is>
+      </c>
+      <c r="G70" s="13" t="inlineStr">
+        <is>
+          <t>Love is a fine thing, a kind hard to understand;
+Love is something else, not to be likened to lust:
+It is one thing, lust another; a wide border lies between them;
+Let no one confuse the two! Hear what I tell you!
+A lover must be constant, not lewd, foul or faithless;
+When parted from the beloved, let him sigh and sigh again,
+Let his heart be fixed on one alone, though she be cold or stern;
+I hate heartless love: embracing, kissing, noisy smacking of lips.
+Let a lover not call this love:
+To want one today and another tomorrow, to take parting lightly;
+That is like the idle play of boys, of mere youth.
+A good lover is one who endures all the world’s trials.</t>
+        </is>
+      </c>
       <c r="H70" s="13" t="inlineStr">
         <is>
           <t>Shota Rustaveli</t>
@@ -9751,7 +10076,8 @@
       </c>
       <c r="W70" s="13" t="inlineStr">
         <is>
-          <t>Medieval Georgian original is public domain. Exact modern base edition of the transcription is not stated; stanza numbering can vary. Do not reuse a modern English translation by assumption. The selection is the original-language text; an existing English translation is not required.</t>
+          <t>Medieval Georgian original is public domain. Exact modern base edition of the transcription is not stated; stanza numbering can vary. Do not reuse a modern English translation by assumption. The selection is the original-language text; an existing English translation is not required.
+Passage update (29 October 2026): Prologue stanzas 24–26, 12 lines, on true love and lust. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X70" s="13" t="inlineStr">
@@ -10106,8 +10432,38 @@
           <t>Ode to Aphrodite (fragment 1)</t>
         </is>
       </c>
-      <c r="F73" s="13" t="n"/>
-      <c r="G73" s="13" t="n"/>
+      <c r="F73" s="13" t="inlineStr">
+        <is>
+          <t>κὤττι μοι μάλιστα θέλω γένεσθαι
+μαινόλᾳ θύμῳ· τίνα δηὖτε Πείθω
+μαῖς ἄγην ἐς σὰν φιλότατα, τίς σ', ὦ
+Ψάπφ', ἀδικήει;
+καὶ γὰρ αἰ φεύγει, ταχέως διώξει,
+αἰ δὲ δῶρα μὴ δέκετ' ἀλλὰ δώσει,
+αἰ δὲ μὴ φίλει, ταχέως φιλήσει
+κωὐκ ἐθέλοισα.
+ἔλθε μοι καὶ νῦν, χαλεπᾶν δὲ λῦσον
+ἐκ μεριμνᾶν, ὄσσα δὲ μοι τελέσσαι
+θῦμος ἰμέρρει, τέλεσον· σὺ δ' αὔτα
+σύμμαχος ἔσσο.</t>
+        </is>
+      </c>
+      <c r="G73" s="13" t="inlineStr">
+        <is>
+          <t>And what I most wish to happen
+For my maddened heart. “Whom now shall I persuade
+To lead you back into her love? Who, O
+Sappho, wrongs you?
+For if she flees, soon she will pursue;
+If she will not take gifts, she will give them;
+And if she does not love, soon she will love,
+Even against her will.”
+Come to me now as well, and free me from harsh
+Cares; all that my heart longs
+To bring about, bring about; and you yourself
+Be my ally.</t>
+        </is>
+      </c>
       <c r="H73" s="13" t="inlineStr">
         <is>
           <t>Sappho</t>
@@ -10138,7 +10494,7 @@
       </c>
       <c r="N73" s="13" t="inlineStr">
         <is>
-          <t>Greek and English</t>
+          <t>Ancient Greek</t>
         </is>
       </c>
       <c r="O73" s="13" t="n"/>
@@ -10179,7 +10535,8 @@
       </c>
       <c r="W73" s="13" t="inlineStr">
         <is>
-          <t>Use Wharton literal prose after Greek. Modern translations are separate.</t>
+          <t>Use Wharton literal prose after Greek. Modern translations are separate.
+Passage update (29 October 2026): Last three stanzas of the ode, 12 lines. Greek text from the 1885 Wharton edition (Project Gutenberg). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X73" s="13" t="inlineStr">
@@ -10350,8 +10707,44 @@
           <t>I Think of You</t>
         </is>
       </c>
-      <c r="F75" s="13" t="n"/>
-      <c r="G75" s="13" t="n"/>
+      <c r="F75" s="13" t="inlineStr">
+        <is>
+          <t>En mi lóbrega y yerta fantasía
+brilla tu imagen apacible y pura,
+como el rayo de luz que el sol envía,
+a través de una bóveda sombría
+al roto mármol de una sepultura.
+Callado, inerte, en estupor profundo,
+mi corazón se embarga y se enajena,
+y allá en su centro vibra moribundo
+cuando entre el vano estrépito del mundo
+la melodía de tu nombre suena.
+Sin lucha, sin afán y sin lamento,
+sin agitarme en ciego frenesí,
+sin proferir un solo un leve acento,
+las largas horas de la noche cuento,
+¡Y pienso en ti…</t>
+        </is>
+      </c>
+      <c r="G75" s="13" t="inlineStr">
+        <is>
+          <t>In my gloomy, frozen imagination
+Your image shines, peaceful and pure,
+Like the ray of light the sun sends
+Through a shadowed vault
+Onto the broken marble of a tomb.
+Silent, inert, in deep stupor,
+My heart is seized and carried away,
+And there, at its centre, it trembles, dying,
+When, amid the empty clamour of the world,
+The melody of your name is heard.
+Without struggle, without striving, without lament,
+Without stirring in blind frenzy,
+Without uttering a single, faint sound,
+I count the long hours of the night,
+And think of you…</t>
+        </is>
+      </c>
       <c r="H75" s="13" t="inlineStr">
         <is>
           <t>José Batres Montúfar</t>
@@ -10423,7 +10816,8 @@
       </c>
       <c r="W75" s="13" t="inlineStr">
         <is>
-          <t>Guatemalan literary affiliation; author was born in what is now El Salvador and died 1844. Use only his poem, not the modern educational notes. The selection is the original-language text; an existing English translation is not required.</t>
+          <t>Guatemalan literary affiliation; author was born in what is now El Salvador and died 1844. Use only his poem, not the modern educational notes. The selection is the original-language text; an existing English translation is not required.
+Passage update (29 October 2026): Last three stanzas, 15 lines. The PDF scattered some words across lines (footnote layout); they are put back in order, wording unchanged. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X75" s="13" t="inlineStr">
@@ -10721,16 +11115,50 @@
       </c>
       <c r="D78" s="13" t="inlineStr">
         <is>
+          <t>The Negro Village</t>
+        </is>
+      </c>
+      <c r="E78" s="13" t="inlineStr">
+        <is>
           <t>The Negro Village — passage on husband, wife and love</t>
         </is>
       </c>
-      <c r="E78" s="13" t="inlineStr">
-        <is>
-          <t>The Negro Village — passage on husband, wife and love</t>
-        </is>
-      </c>
-      <c r="F78" s="13" t="n"/>
-      <c r="G78" s="13" t="n"/>
+      <c r="F78" s="13" t="inlineStr">
+        <is>
+          <t>And yet there are, who will in strength maintain,
+The negro heart is foreign to all thought
+Which breathes of hopeful love, affection’s reign,
+Or nobler passions in the bosom wrought;
+Such reason in a blind conceit,
+Where prejudice and false pride meet,
+Yea! man is man with all emotions fraught.
+Their hearts can love with all the lavish strength,
+Impetuous fervour of ungoverned will,
+Running unbroken to its utmost length:
+Passion’s frenzy, but pure love’s offspring still;
+Unweaned by cold decorum’s laws,
+Cleaving persistent to its cause,
+Free and natural as the mountain rill.</t>
+        </is>
+      </c>
+      <c r="G78" s="13" t="inlineStr">
+        <is>
+          <t>And yet there are, who will in strength maintain,
+The negro heart is foreign to all thought
+Which breathes of hopeful love, affection’s reign,
+Or nobler passions in the bosom wrought;
+Such reason in a blind conceit,
+Where prejudice and false pride meet,
+Yea! man is man with all emotions fraught.
+Their hearts can love with all the lavish strength,
+Impetuous fervour of ungoverned will,
+Running unbroken to its utmost length:
+Passion’s frenzy, but pure love’s offspring still;
+Unweaned by cold decorum’s laws,
+Cleaving persistent to its cause,
+Free and natural as the mountain rill.</t>
+        </is>
+      </c>
       <c r="H78" s="13" t="inlineStr">
         <is>
           <t>Egbert Martin, pen name Leo (c.1861–1890)</t>
@@ -10802,7 +11230,8 @@
       </c>
       <c r="W78" s="13" t="inlineStr">
         <is>
-          <t>Only the specified passage concerns romantic/marital love; the entire poem is not a love lyric. Its racial and Christian language reflects the nineteenth-century setting.</t>
+          <t>Only the specified passage concerns romantic/marital love; the entire poem is not a love lyric. Its racial and Christian language reflects the nineteenth-century setting.
+Passage update (29 October 2026): Two consecutive stanzas, 14 lines: the poet answers the claim that Black people cannot feel deep love. Original English; no translation needed. Original English text; not a translation.</t>
         </is>
       </c>
       <c r="X78" s="13" t="inlineStr">
@@ -10868,8 +11297,38 @@
           <t>Choucoune (a woman's name)</t>
         </is>
       </c>
-      <c r="F79" s="13" t="n"/>
-      <c r="G79" s="13" t="n"/>
+      <c r="F79" s="13" t="inlineStr">
+        <is>
+          <t>Dériè gnou gras touff’ pingouin,
+L’aut’jou, moin contré Choucoune ;
+Li sourit, l’heur’li ouè moin,
+Moin dit : « Ciel ! A là bell’ moune ! »
+Li dit : « Ou trouvé ca cher ! »…
+P’tits zoézeaux ta pé couté nous lan l’air…
+Quand moin songé Ça, moin gangnin la peine,
+Car dimpi jou-là, dé pieds moin lan chaîne !
+Ca qui pis trist’lan tout ça,
+Ca qui va surprendr’tout moune,
+Cé ’pou ouè malgré temps-là,
+Moin aimé toujours Choucoune !</t>
+        </is>
+      </c>
+      <c r="G79" s="13" t="inlineStr">
+        <is>
+          <t>Behind a thick clump of cactus,
+The other day, I met Choucoune;
+She smiled the moment she saw me,
+I said: “Heavens! What a beautiful girl!”
+She said: “You think so, dear?”…
+Little birds were listening to us up in the air…
+When I think of it, I am full of sorrow,
+For since that day both my feet are in chains!
+The saddest thing in all of this,
+The thing that will surprise everyone,
+Is to see that, in spite of it all,
+I still love Choucoune!</t>
+        </is>
+      </c>
       <c r="H79" s="13" t="inlineStr">
         <is>
           <t>Oswald Durand</t>
@@ -10941,7 +11400,8 @@
       </c>
       <c r="W79" s="13" t="inlineStr">
         <is>
-          <t>Durand died 1906. Use the Creole original; the accompanying French translation has a separate attribution question. Original includes historical racial language. Later songs and Yellow Bird adaptations are separate. The selection is the original-language text; an existing English translation is not required.</t>
+          <t>Durand died 1906. Use the Creole original; the accompanying French translation has a separate attribution question. Original includes historical racial language. Later songs and Yellow Bird adaptations are separate. The selection is the original-language text; an existing English translation is not required.
+Passage update (29 October 2026): Opening stanza (8 lines) and the first four lines of the last stanza. The 1923 journal transcription is unproofread OCR: three obvious slips are corrected (a full stop after “L’aut’jou” to a comma, “bell”” to “bell’”, and a missing opening « before “Ou trouvé”); the wording is unchanged. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X79" s="13" t="inlineStr">
@@ -10995,16 +11455,44 @@
       </c>
       <c r="D80" s="13" t="inlineStr">
         <is>
-          <t>שיר השירים ד:ט–י / Song of Songs 4:9–10</t>
+          <t>שיר השירים ד:ט–יב / Song of Songs 4:9–12</t>
         </is>
       </c>
       <c r="E80" s="13" t="inlineStr">
         <is>
-          <t>Song of Songs4:9–10</t>
-        </is>
-      </c>
-      <c r="F80" s="13" t="n"/>
-      <c r="G80" s="13" t="n"/>
+          <t>Song of Songs 4:9–12</t>
+        </is>
+      </c>
+      <c r="F80" s="13" t="inlineStr">
+        <is>
+          <t>לבבתני אחתי כלה
+לבבתני באחד מעיניך
+באחד ענק מצורניך
+מה־יפו דדיך אחתי כלה
+מה־טבו דדיך מיין
+וריח שמניך מכל־בשמים
+נפת תטפנה שפתותיך כלה
+דבש וחלב תחת לשונך
+וריח שלמתיך כריח לבנון
+גן נעול אחתי כלה
+גל נעול מעין חתום</t>
+        </is>
+      </c>
+      <c r="G80" s="13" t="inlineStr">
+        <is>
+          <t>You have stolen my heart, my sister, my bride;
+You have stolen my heart with one glance of your eyes,
+With one bead of your necklace.
+How beautiful is your love, my sister, my bride!
+How much better is your love than wine,
+And the scent of your perfumes than any spice!
+Your lips drip honey, my bride;
+Honey and milk are under your tongue,
+And the scent of your garments is like the scent of Lebanon.
+A locked garden is my sister, my bride,
+A locked spring, a sealed fountain.</t>
+        </is>
+      </c>
       <c r="H80" s="13" t="inlineStr">
         <is>
           <t>Anonymous ancient Hebrew poets</t>
@@ -11069,12 +11557,13 @@
       </c>
       <c r="V80" s="13" t="inlineStr">
         <is>
-          <t>Chapter 4, verses 9–10</t>
+          <t>Chapter 4, verses 9–12</t>
         </is>
       </c>
       <c r="W80" s="13" t="inlineStr">
         <is>
-          <t>Country association is Vatican reception of this passage, not authorship in the Holy See. Translate the ancient Hebrew, excluding modern commentary, vocalisation apparatus and papal-address translations. The page offers a consonantal text option. The selection is the original-language text; an existing English translation is not required.</t>
+          <t>Country association is Vatican reception of this passage, not authorship in the Holy See. Translate the ancient Hebrew, excluding modern commentary, vocalisation apparatus and papal-address translations. The page offers a consonantal text option. The selection is the original-language text; an existing English translation is not required.
+Passage update (29 October 2026): Song of Songs 4:9–12, 11 lines. Consonantal Hebrew (vowel points and cantillation removed, as the spreadsheet asks); where the text has a written/read variant, the written form באחד is kept. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X80" s="13" t="inlineStr">

</xml_diff>

<commit_message>
India: Tagore's অনন্ত প্রেম; aligned poem rows; quieter history notes
- India now shows Tagore's Bengali poem অনন্ত প্রেম (Unending Love, 1889)
  beside English, replacing The Gardener 16, whose Bengali source is
  uncertain. Spreadsheet row updated with sources and notes.
- Poems with matching line counts render as rows, so each original line
  stays beside its translation when long lines wrap.
- History notes are smaller and plainer so the poem is the focus.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -12053,44 +12053,60 @@
       </c>
       <c r="D84" s="13" t="inlineStr">
         <is>
-          <t>The Gardener, poem 16</t>
+          <t>অনন্ত প্রেম / Ananta Prem</t>
         </is>
       </c>
       <c r="E84" s="13" t="inlineStr">
         <is>
-          <t>The Gardener, poem 16</t>
+          <t>Unending Love</t>
         </is>
       </c>
       <c r="F84" s="13" t="inlineStr">
         <is>
-          <t>Hands cling to hands and eyes linger on eyes: thus begins the record of our hearts.
-It is the moonlit night of March; the sweet smell of henna is in the air;
-my flute lies on the earth neglected and your garland of flowers is unfinished.
-This love between you and me is simple as a song.
-Your veil of the saffron colour makes my eyes drunk.
-The jasmine wreath that you wove me thrills to my heart like praise.
-It is a game of giving and withholding, revealing and screening again;
-some smiles and some little shyness, and some sweet useless struggles.
-This love between you and me is simple as a song.
-No mystery beyond the present; no striving for the impossible;
-no shadow behind the charm; no groping in the depth of the dark.
-This love between you and me is simple as a song.</t>
+          <t>তোমারেই যেন ভালোবাসিয়াছি শত রূপে শতবার
+জনমে জনমে যুগে যুগে অনিবার।
+চিরকাল ধরে মুগ্ধ হৃদয় গাঁথিয়াছে গীতহার—
+কত রূপ ধরে পরেছ গলায়, নিয়েছ সে উপহার
+জনমে জনমে যুগে যুগে অনিবার।
+যত শুনি সেই অতীত কাহিনী, প্রাচীন প্রেমের ব্যথা,
+অতি পুরাতন বিরহমিলনকথা,
+অসীম অতীতে চাহিতে চাহিতে দেখা দেয় অবশেষে
+কালের তিমিররজনী ভেদিয়া তোমারি মুরতি এসে
+চিরস্মৃতিময়ী ধ্রুবতারকার বেশে।
+আমরা দুজনে ভাসিয়া এসেছি যুগলপ্রেমের স্রোতে
+অনাদি কালের হৃদয়-উৎস হতে।
+আমরা দুজনে করিয়াছি খেলা কোটি প্রেমিকের মাঝে
+বিরহবিধুর নয়নসলিলে, মিলনমধুর লাজে—
+পুরাতন প্রেম নিত্যনূতন সাজে।
+আজি সেই চির-দিবসের প্রেম অবসান লভিয়াছে
+রাশি রাশি হয়ে তোমার পায়ের কাছে।
+নিখিলের সুখ, নিখিলের দুখ, নিখিল প্রাণের প্রীতি—
+একটি প্রেমের মাঝারে মিশেছে সকল প্রেমের স্মৃতি
+সকল কালের সকল কবির গীতি।</t>
         </is>
       </c>
       <c r="G84" s="13" t="inlineStr">
         <is>
-          <t>Hands cling to hands and eyes linger on eyes: thus begins the record of our hearts.
-It is the moonlit night of March; the sweet smell of henna is in the air;
-my flute lies on the earth neglected and your garland of flowers is unfinished.
-This love between you and me is simple as a song.
-Your veil of the saffron colour makes my eyes drunk.
-The jasmine wreath that you wove me thrills to my heart like praise.
-It is a game of giving and withholding, revealing and screening again;
-some smiles and some little shyness, and some sweet useless struggles.
-This love between you and me is simple as a song.
-No mystery beyond the present; no striving for the impossible;
-no shadow behind the charm; no groping in the depth of the dark.
-This love between you and me is simple as a song.</t>
+          <t>It seems I have loved you in a hundred forms, a hundred times,
+In life after life, age after age, without end.
+Forever my spellbound heart has strung a garland of songs;
+In how many forms you have worn it round your neck and taken the gift,
+In life after life, age after age, without end.
+Whenever I hear those tales of the past, the ache of ancient love,
+The age-old stories of parting and meeting,
+As I gaze and gaze into the boundless past, at last
+Your image appears, piercing the dark night of time,
+In the guise of the pole star, remembered for ever.
+We two have come floating on the stream of a love for two,
+From the heart’s spring of time without beginning.
+We two have played among millions of lovers,
+In the tears of eyes grieving at parting, in the sweet shyness of meeting:
+An old love in ever-new array.
+Today that love of all our days has found its fulfilment,
+Heaped up in abundance at your feet.
+The joy of the whole world, its sorrow, the love of every living soul,
+The memory of every love has mingled in this one love,
+And the songs of every poet of every age.</t>
         </is>
       </c>
       <c r="H84" s="13" t="inlineStr">
@@ -12119,11 +12135,11 @@
         </is>
       </c>
       <c r="M84" s="14" t="n">
-        <v>1913</v>
+        <v>1889</v>
       </c>
       <c r="N84" s="13" t="inlineStr">
         <is>
-          <t>English from Bengali</t>
+          <t>Bengali</t>
         </is>
       </c>
       <c r="O84" s="13" t="n"/>
@@ -12139,44 +12155,49 @@
       </c>
       <c r="R84" s="13" t="inlineStr">
         <is>
-          <t>1913 (English collection); Bengali poem date not established</t>
+          <t>2 Bhadra 1296 (August 1889), Jorasanko, Calcutta; collected in Manasi (1890)</t>
         </is>
       </c>
       <c r="S84" s="13" t="inlineStr">
         <is>
-          <t>1915 (author’s English translation, linked edition)</t>
+          <t>Sanchayita; Bengali Wikisource proofread transcription</t>
         </is>
       </c>
       <c r="T84" s="13" t="inlineStr">
         <is>
-          <t>Mutual love through touch.</t>
+          <t>The speaker feels he has loved the beloved in countless forms across lifetimes; every love and every poet’s song meets in this one love.</t>
         </is>
       </c>
       <c r="U84" s="13" t="inlineStr">
         <is>
-          <t>The Gardener; linked edition dated 1915; author translation</t>
+          <t>Manasi (1890); text from Sanchayita, printed p. 96, proofread on Bengali Wikisource</t>
         </is>
       </c>
       <c r="V84" s="13" t="inlineStr">
         <is>
-          <t>Poem 16</t>
+          <t>Complete poem, 20 lines</t>
         </is>
       </c>
       <c r="W84" s="13" t="inlineStr">
         <is>
           <t>Author translation; preface notes abridgement and paraphrase. Modern translations are separate.
-English passage: Original English text; not a translation. Poem16, first three paragraphs; author’s English version, reflowed into12 reading lines. Corrected obvious transcription in→is before unfinished; no new translation.. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+English passage: Original English text; not a translation. Poem16, first three paragraphs; author’s English version, reflowed into12 reading lines. Corrected obvious transcription in→is before unfinished; no new translation.. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Work changed (29 October 2026): The Gardener, poem 16 (Tagore’s own English) replaced by the Bengali original অনন্ত প্রেম, whose source is certain. Complete poem, 20 lines. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X84" s="13" t="inlineStr">
         <is>
-          <t>Public domain in USA - Project Gutenberg</t>
-        </is>
-      </c>
-      <c r="Y84" s="13" t="n"/>
+          <t>Public-domain original: Tagore died 1941, beyond the standard life-plus-70 term. Modern translations are separate.</t>
+        </is>
+      </c>
+      <c r="Y84" s="13" t="inlineStr">
+        <is>
+          <t>Bengali Wikisource, Sanchayita: অনন্ত প্রেম</t>
+        </is>
+      </c>
       <c r="Z84" s="11" t="inlineStr">
         <is>
-          <t>Read text</t>
+          <t>Read original</t>
         </is>
       </c>
       <c r="AA84" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Add batch 2 of new poem passages (13 countries)
Honduras, Iceland, Indonesia, Iran, Jordan, Kazakhstan, Kuwait,
Kyrgyzstan, Latvia, Lebanon, Libya, Lithuania and Mauritania now show a
passage in the original beside English, each with a history note. Iran
switches from Bell's 1897 English to Hafez's Persian ghazal (Ganjoor).
Originals are cut from the sources by script; English versions are new
drafts, recorded as such in the spreadsheet. 76 poems to read in total.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 63 paired passages • 132 unfilled</t>
+          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 76 paired passages • 119 unfilled</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -11633,8 +11633,42 @@
           <t>Upwards (Latin title)</t>
         </is>
       </c>
-      <c r="F81" s="13" t="n"/>
-      <c r="G81" s="13" t="n"/>
+      <c r="F81" s="13" t="inlineStr">
+        <is>
+          <t>Ya no nos separemos ni un momento,
+porque –cuando se extingan nuestras vidas–
+nuestras dos almas cruzarán unidas
+el éter, en continuo ascendimiento.
+Ajenas al humano sufrimiento,
+de las innobles carnes desprendidas,
+serán en una llama confundidas
+en la región azúl del firmamento.
+Sin dejar huellas ni visibles rastros,
+más allá de la gloria de los astros,
+entre auroras de eternos arreboles,
+a obedecer iremos la divina
+ley, fatal y suprema que domina
+los espacios, las almas y los soles.</t>
+        </is>
+      </c>
+      <c r="G81" s="13" t="inlineStr">
+        <is>
+          <t>Let us not be parted even for a moment,
+For, when our lives are extinguished,
+Our two souls will cross together
+Through the ether, rising for ever.
+Strangers to human suffering,
+Set free from ignoble flesh,
+They will be merged into one flame
+In the blue region of the firmament.
+Leaving no traces or visible tracks,
+Beyond the glory of the stars,
+Among dawns of everlasting crimson clouds,
+We will go to obey the divine
+Law, fatal and supreme, that rules
+The spaces, the souls and the suns.</t>
+        </is>
+      </c>
       <c r="H81" s="13" t="inlineStr">
         <is>
           <t>Juan Ramón Molina</t>
@@ -11704,7 +11738,8 @@
       </c>
       <c r="W81" s="13" t="inlineStr">
         <is>
-          <t>Use the original sonnet, not the modern anthology’s selection, introduction or commentary. Spiritual imagery serves the lovers’ union rather than a standalone devotional hymn.</t>
+          <t>Use the original sonnet, not the modern anthology’s selection, introduction or commentary. Spiritual imagery serves the lovers’ union rather than a standalone devotional hymn.
+Passage update (29 October 2026): Complete sonnet, 14 lines (Spanish Wikisource text, titled “Súrsum”). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X81" s="13" t="inlineStr">
@@ -11924,8 +11959,50 @@
           <t>Journey's End</t>
         </is>
       </c>
-      <c r="F83" s="13" t="n"/>
-      <c r="G83" s="13" t="n"/>
+      <c r="F83" s="13" t="inlineStr">
+        <is>
+          <t>Greiddi eg þér lokka
+við Galtará
+vel og vandlega;
+brosa blómvarir,
+blika sjónstjörnur,
+roðnar heitur hlýr.
+Fjær er nú fagurri
+fylgd þinni
+sveinn í djúpum dali;
+ástarstjarna
+yfir Hraundranga
+skín á bak við ský.
+Háa skilur hnetti
+himingeimur,
+blað skilur bakka og egg;
+en anda, sem unnast,
+fær aldregi
+eilífð að skilið.</t>
+        </is>
+      </c>
+      <c r="G83" s="13" t="inlineStr">
+        <is>
+          <t>I combed your locks
+By the river Galtará,
+Well and with care;
+Your flower-lips smile,
+Your eye-stars shine,
+Your warm cheek blushes.
+Far now from your fair
+Company
+Is a young man in a deep valley;
+The star of love
+Above Hraundrangi
+Shines behind the clouds.
+Heaven’s vast space
+Divides the high spheres,
+A blade divides back and edge;
+But spirits that love each other
+Can never
+Be parted by eternity.</t>
+        </is>
+      </c>
       <c r="H83" s="13" t="inlineStr">
         <is>
           <t>Jónas Hallgrímsson</t>
@@ -11995,7 +12072,8 @@
       </c>
       <c r="W83" s="13" t="inlineStr">
         <is>
-          <t>Author died 1845. Translate from the scan: the site labels its OCR unproofread. Print-edition date not established here; digital date is not the original work date. The selection is the original-language text; an existing English translation is not required.</t>
+          <t>Author died 1845. Translate from the scan: the site labels its OCR unproofread. Print-edition date not established here; digital date is not the original work date. The selection is the original-language text; an existing English translation is not required.
+Passage update (29 October 2026): Final three stanzas, 18 lines, including the closing stanza. Runeberg’s OCR is unproofread; these lines read cleanly and are copied as printed. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X83" s="13" t="inlineStr">
@@ -12244,8 +12322,62 @@
           <t>The Fragrance of Your Hair</t>
         </is>
       </c>
-      <c r="F85" s="13" t="n"/>
-      <c r="G85" s="13" t="n"/>
+      <c r="F85" s="13" t="inlineStr">
+        <is>
+          <t>Kupatah tangkai kusuma kukucup
+Kendati mencari wangi asli
+Cempaka tinggal tergulai lampai
+Sayang tanganku hendak mencapai.
+Teja! hanya cempaka ditayang daun
+Aneka bunga menutup bumi
+Impian lama datang mengalun
+Kerana kusuma kenangan diri.
+Harum rambutmu terasa ada
+Dalam bunga duduk tersembunyi
+Suma mana ratna mulia
+Kanda sibuk tengah mencari
+Pohon rendah dinaungi kemuning
+Puteri dilindungi payung kembang
+Bunga adinda kencana ramping
+Irama kusuma abang seorang.
+Wangi tertebar membawaku ragu
+Mengambang abang ke hari lampau
+Harum sepadan wangi rambutmu
+Kalau terurai kita bergurau.
+Melur! Duta rindu di purnama-raya
+Kawan sendu di sunyi malam
+Ratna rupa di hulu kemala
+Penambah manis jiwa pendiam.</t>
+        </is>
+      </c>
+      <c r="G85" s="13" t="inlineStr">
+        <is>
+          <t>I break off a flower’s stem and kiss it,
+Though it is the true fragrance I am seeking;
+The champak hangs, drooping and slender,
+Alas, my hand longs to reach it.
+Evening glow! only the champak is cradled by leaves,
+Flowers of every kind cover the earth;
+An old dream comes drifting back
+Because of the flower of my own memory.
+The fragrance of your hair I can sense
+Sitting hidden within the flowers;
+Which flower is the noble jewel
+That I, your lover, am busy searching for?
+A low tree shaded by kemuning,
+A princess sheltered by a parasol of blossom;
+My darling’s flower, slender and golden,
+The flower song of your lover alone.
+The scattered scent fills me with doubt,
+Your lover drifts back to days gone by;
+A fragrance equal to the scent of your hair
+When it was loosened and we laughed and teased.
+Jasmine! Envoy of longing under the full moon,
+Companion in sorrow in the silent night,
+Jewel in form at the crown of gems,
+Sweetening a quiet soul.</t>
+        </is>
+      </c>
       <c r="H85" s="13" t="inlineStr">
         <is>
           <t>Amir Hamzah</t>
@@ -12317,7 +12449,8 @@
       </c>
       <c r="W85" s="13" t="inlineStr">
         <is>
-          <t>Use Hamzah’s original words. Different editions modernise spelling and pagination; modern criticism, typesetting and translations separate. Date of first magazine appearance is distinguished from 1941 collection date.</t>
+          <t>Use Hamzah’s original words. Different editions modernise spelling and pagination; modern criticism, typesetting and translations separate. Date of first magazine appearance is distinguished from 1941 collection date.
+Passage update (29 October 2026): Complete poem, 24 lines, from the validated Indonesian Wikisource transcription of Buah Rindu, printed pp. 44–45. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X85" s="13" t="inlineStr">
@@ -12371,16 +12504,58 @@
       </c>
       <c r="D86" s="13" t="inlineStr">
         <is>
-          <t>Oh Turkish maid of Shiraz!</t>
+          <t>اگر آن ترک شیرازی / Agar an Turk-e Shirazi</t>
         </is>
       </c>
       <c r="E86" s="13" t="inlineStr">
         <is>
-          <t>Oh Turkish maid of Shiraz!</t>
-        </is>
-      </c>
-      <c r="F86" s="13" t="n"/>
-      <c r="G86" s="13" t="n"/>
+          <t>If That Turk of Shiraz</t>
+        </is>
+      </c>
+      <c r="F86" s="13" t="inlineStr">
+        <is>
+          <t>اگر آن ترک شیرازی به‌ دست‌ آرد دل ما را
+به خال هندویش بخشم سمرقند و بخارا را
+بده ساقی می باقی که در جنت نخواهی یافت
+کنار آب رکناباد و گل‌گشت مصلا را
+فغان! کاین لولیان شوخ شیرین‌کار شهرآشوب
+چنان بردند صبر از دل که ترکان خوان یغما را
+ز عشق ناتمام ما جمال یار مستغنی‌ است
+به آب و رنگ و خال و خط چه حاجت روی زیبا را؟
+من از آن حسن روزافزون که یوسف داشت دانستم
+که عشق از پردهٔ عصمت برون آرد زلیخا را
+اگر دشنام فرمایی و گر نفرین دعا گویم
+جواب تلخ می‌زیبد لب لعل شکرخا را
+نصیحت گوش کن جانا که از جان دوست‌تر دارند
+جوانان سعادتمند پند پیر دانا را
+حدیث از مطرب و می گو و راز دهر کمتر جو
+که کس نگشود و نگشاید به حکمت این معما را
+غزل گفتی و در سفتی بیا و خوش بخوان حافظ
+که بر نظم تو افشاند فلک عقد ثریا را</t>
+        </is>
+      </c>
+      <c r="G86" s="13" t="inlineStr">
+        <is>
+          <t>If that Turk of Shiraz would take my heart in hand,
+For that dark mole I would give away Samarkand and Bukhara.
+Pour, cupbearer, the wine that remains, for in paradise you will not find
+The banks of the Ruknabad stream or the rose walks of Musalla.
+Alas! these saucy, sweet-working, city-unsettling beauties
+Have carried off patience from my heart as Turks carry off a plundered feast.
+My beloved’s beauty has no need of our imperfect love:
+What need has a lovely face of paint and colour, mole and line?
+From that ever-growing beauty that Joseph had, I came to know
+That love brings Zuleikha out from behind the veil of chastity.
+Whether you curse me or revile me, I will bless you:
+A bitter answer suits a ruby lip that sheds sugar.
+Listen to advice, my soul, for fortunate young people
+Hold the counsel of a wise old man dearer than their lives.
+Speak of the minstrel and wine, and seek the world’s secret less,
+For no one has solved, nor by wisdom will solve, this riddle.
+You have made a ghazal and strung pearls; come, sing it sweetly, Hafez,
+For over your verse the heavens scatter the necklace of the Pleiades.</t>
+        </is>
+      </c>
       <c r="H86" s="13" t="inlineStr">
         <is>
           <t>Hafez</t>
@@ -12409,7 +12584,7 @@
       <c r="M86" s="14" t="n"/>
       <c r="N86" s="13" t="inlineStr">
         <is>
-          <t>English from Persian</t>
+          <t>Persian</t>
         </is>
       </c>
       <c r="O86" s="13" t="n"/>
@@ -12445,12 +12620,13 @@
       </c>
       <c r="V86" s="13" t="inlineStr">
         <is>
-          <t>Poem V, pp. 71-72</t>
+          <t>Complete ghazal (Divan, ghazal 3), 9 couplets</t>
         </is>
       </c>
       <c r="W86" s="13" t="inlineStr">
         <is>
-          <t>Specifically Bell 1897, including her gender choices. Modern translations are separate. Mystical readings are possible.</t>
+          <t>Specifically Bell 1897, including her gender choices. Modern translations are separate. Mystical readings are possible.
+Passage update (29 October 2026): Complete ghazal, 9 couplets (18 half-lines). Persian text from Ganjoor (ghazal 3), with Ganjoor’s added short-vowel marks removed; the letters are unchanged. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X86" s="13" t="inlineStr">
@@ -12461,7 +12637,7 @@
       <c r="Y86" s="13" t="n"/>
       <c r="Z86" s="11" t="inlineStr">
         <is>
-          <t>Read text</t>
+          <t>Read original</t>
         </is>
       </c>
       <c r="AA86" s="11" t="inlineStr">
@@ -13445,8 +13621,46 @@
           <t>I thought I had passed beyond pursuing passion, but then… (first line)</t>
         </is>
       </c>
-      <c r="F93" s="13" t="n"/>
-      <c r="G93" s="13" t="n"/>
+      <c r="F93" s="13" t="inlineStr">
+        <is>
+          <t>ظننتني جزت عن طرد الهوى فإذا
+حسابه لم يزل في دفتري جاري
+وزند وجدي بربات الحجال على
+عهدي به كعشيات الصبا واري
+والأربعون التي لاحت طلائعها
+في لمتي ريحها استخذى لأعصاري
+ظننتني جزت عن طرد الهوى فإذا
+موضوعه لم يزل موضوع أسماري
+وما توهمته زهداً ورحت به
+أعلل النفس غير الواقع الجاري
+شتان بين شعوري في حقيقته
+وبين رجعك يا أصداء أفكاري
+فليتق اللّه من ظن الهيام بهم
+غياً فما بالهوى العذري من عار
+وما يضر أخا الأردن كسوته
+جديدها أن يحل يوماً لاطماري</t>
+        </is>
+      </c>
+      <c r="G93" s="13" t="inlineStr">
+        <is>
+          <t>I thought I had moved past the chase of passion, but lo,
+Its account is still running in my ledger;
+And the flint of my longing for the veiled beauties,
+As I knew it in the evenings of youth, still strikes fire;
+And the forties, whose first signs have appeared
+In my locks: their wind has bowed before my whirlwinds.
+I thought I had moved past the chase of passion, but lo,
+It is still the subject of my night-time talk.
+What I imagined was renunciation, and went about
+Consoling my soul with, was not what was truly happening.
+How far apart are my feeling as it truly is
+And your answer, O echoes of my thoughts!
+Let whoever thinks it folly to be lovesick for them
+Fear God: there is no shame in chaste love.
+And what harm is it to a son of Jordan if his clothes,
+The new ones, should one day turn to rags?</t>
+        </is>
+      </c>
       <c r="H93" s="13" t="inlineStr">
         <is>
           <t>Mustafa Wahbi al-Tall (Arar), 1899–1949; some catalogues give 1897</t>
@@ -13518,7 +13732,8 @@
       </c>
       <c r="W93" s="13" t="inlineStr">
         <is>
-          <t>Identifier is the original incipit. Year 1949 is an upper bound. Birth-year disagreement is explicit. Reuse the author’s historical Arabic verses, excluding later commentary and translations; first-publication particulars for this individual poem have not been established.</t>
+          <t>Identifier is the original incipit. Year 1949 is an upper bound. Birth-year disagreement is explicit. Reuse the author’s historical Arabic verses, excluding later commentary and translations; first-publication particulars for this individual poem have not been established.
+Passage update (29 October 2026): Complete poem, 8 couplets (16 half-lines), as printed in the Abu Dhabi Poetry Encyclopedia; the site’s decorative letter-stretching (tatweel) is removed. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X93" s="13" t="inlineStr">
@@ -13580,8 +13795,54 @@
           <t>The Pupil of My Eye (conventional rendering; also interpreted as My Gaze)</t>
         </is>
       </c>
-      <c r="F94" s="13" t="n"/>
-      <c r="G94" s="13" t="n"/>
+      <c r="F94" s="13" t="inlineStr">
+        <is>
+          <t>Көзімнің қарасы,
+Көңілімнің санасы,
+Бітпейді іштегі,
+Ғашықтық жарасы.
+Қазақтың данасы,
+Жасы үлкен ағасы.
+Бар демес сендей бір
+Адамның баласы.
+Жылайын, жырлайын,
+Ағызып көз майын.
+Айтуға келгенде,
+Қалқама сөз дайын.
+Жүректен қозғайын,
+Әдептен озбайын.
+Өзі де білмей ме,
+Көп сөйлеп созбайын.
+Тереңдеп қарайсың,
+Телміріп тұрмайсың.
+Бихабар жүргенсіп,
+Бек қатты сынайсың.</t>
+        </is>
+      </c>
+      <c r="G94" s="13" t="inlineStr">
+        <is>
+          <t>Pupil of my eye,
+Thought of my heart,
+The wound of love within me
+Never heals.
+Neither the wisest of the Kazakhs
+Nor the eldest of their elders
+Would say there exists one
+Among the children of men like you.
+Let me weep, let me sing,
+Letting my tears stream down.
+When it comes to speaking,
+I have words ready for my darling.
+Let me stir them from my heart
+And not overstep good manners.
+Does she not know it herself?
+Let me not drag it out with too many words.
+You look at me deeply,
+Yet you do not stand gazing with longing.
+Pretending to know nothing,
+You test me very hard.</t>
+        </is>
+      </c>
       <c r="H94" s="13" t="inlineStr">
         <is>
           <t>Abai Qunanbaiuly</t>
@@ -13653,7 +13914,8 @@
       </c>
       <c r="W94" s="13" t="inlineStr">
         <is>
-          <t>Abai died 1904. Use his original words; modern performers, arrangements and recordings excluded. The online transcription is in Cyrillic; earlier editions use a different script. The selection is the original-language text; an existing English translation is not required.</t>
+          <t>Abai died 1904. Use his original words; modern performers, arrangements and recordings excluded. The online transcription is in Cyrillic; earlier editions use a different script. The selection is the original-language text; an existing English translation is not required.
+Passage update (29 October 2026): First five stanzas, 20 lines, from the Kazakh Wikisource text (Cyrillic script). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X94" s="13" t="inlineStr">
@@ -13937,8 +14199,38 @@
           <t>Hind's face is so delicate (first-line sense)</t>
         </is>
       </c>
-      <c r="F97" s="13" t="n"/>
-      <c r="G97" s="13" t="n"/>
+      <c r="F97" s="13" t="inlineStr">
+        <is>
+          <t>إن هنداً يرقُّ منها المحيّا
+ليس إلا من الحّيا أن تُحَيّا
+رَبِّ هبْ لي من الجلادة صبراً
+آتني من لدنْكَ ربِّ وَلِيّا
+لا تَذْرني من الكآبة والوَجْ
+دِ إلهي أهيم فرداً خليّا
+كيف أنسى كلامَها اليومَ لما
+نبذتْني به مكاناً قصيّا
+عاتبتْني فأوسعتْني عِتاباً
+فكأني أتيتُ شيئاً فريّا
+ذاتُ قْرُطٍ كأنه النجمُ هندٌ
+ووشاحٍ إذا انبرتْ كالثريّا</t>
+        </is>
+      </c>
+      <c r="G97" s="13" t="inlineStr">
+        <is>
+          <t>Hind, whose face grows tender
+Only from shyness when she is greeted —
+Lord, grant me patience to endure;
+Give me, Lord, a helper from Your presence.
+Do not leave me, out of sorrow and long-
+ing, my God, to wander alone and forsaken.
+How can I forget her words today, when
+With them she cast me off to a distant place?
+She reproached me, and reproached me at length,
+As if I had done something unheard of.
+Hind, with an earring like a star,
+And a sash that, when she sets out, is like the Pleiades.</t>
+        </is>
+      </c>
       <c r="H97" s="13" t="inlineStr">
         <is>
           <t>Abdullah al-Faraj (عبد الله الفرج)</t>
@@ -14008,7 +14300,8 @@
       </c>
       <c r="W97" s="13" t="inlineStr">
         <is>
-          <t>Use the Arabic poem only. Musical compositions, performances and recordings need separate assessment; first publication date not established.</t>
+          <t>Use the Arabic poem only. Musical compositions, performances and recordings need separate assessment; first publication date not established.
+Passage update (29 October 2026): Complete poem, 6 couplets (12 half-lines), as printed in the Abu Dhabi Poetry Encyclopedia; the site’s decorative letter-stretching (tatweel) is removed. One word is divided across the third couplet’s half-lines, as printed. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X97" s="13" t="inlineStr">
@@ -14070,8 +14363,54 @@
           <t>Alymkan (a woman's name)</t>
         </is>
       </c>
-      <c r="F98" s="13" t="n"/>
-      <c r="G98" s="13" t="n"/>
+      <c r="F98" s="13" t="inlineStr">
+        <is>
+          <t>Атка салган дилдейсиң,
+Ачылган кызыл гүлдөйсүң.
+Бир күн оору, бир күн соо,
+Алымкан, азабың тартсам билбейсиң.
+Бетегелүү майданым,
+Пейили жакшы жайдарым.
+Көлөкөлүү майданым,
+Алымкан, көңүлү жакшы жайдарым.
+Кашкардын тоосу кайрылыш,
+Кайрылып учат улуу куш.
+Кайрылып мага келет,
+Алымкан, карыпка салбай кыйын иш.
+Букардын тоосу бурулуш,
+Бурулуп учат улуу куш.
+Бурулуп мага келет,
+Алымкан, муңдууга салбай кыйын иш.
+Саркештеп сайган жоолугуң,
+Сарсанаа кылат жоругуң.
+Көркөмдөп сайган жоолугуң,
+Алымкан, көп санаа кылат жоругуң.</t>
+        </is>
+      </c>
+      <c r="G98" s="13" t="inlineStr">
+        <is>
+          <t>You are like a gold ornament on a horse,
+You are like a red flower in bloom.
+One day sick, one day well:
+Alymkan, you do not know the torment I suffer.
+My meadow of feather grass,
+My cheerful one with a kind heart.
+My shady meadow,
+Alymkan, my cheerful one with a good soul.
+The mountains of Kashgar turn back,
+The great birds turn and fly.
+If only you would turn and come to me,
+Alymkan, and not lay hard trials on a poor man.
+The mountains of Bukhara bend away,
+The great birds wheel and fly.
+If only you would wheel and come to me,
+Alymkan, and not lay hard trials on a grieving man.
+Your headscarf, embroidered in yellow,
+Your ways make me anxious.
+Your headscarf, beautifully embroidered,
+Alymkan, your ways give me many cares.</t>
+        </is>
+      </c>
       <c r="H98" s="13" t="inlineStr">
         <is>
           <t>Toktogul Satylganov (Токтогул Сатылганов), lyrics</t>
@@ -14141,7 +14480,8 @@
       </c>
       <c r="W98" s="13" t="inlineStr">
         <is>
-          <t>Only the original lyrics are treated as open. Later music by Bektemir Eginchiev (1910–1964), recordings and modern translations remain separate. Oral/transcribed variants exist; choose and credit a single textual version.</t>
+          <t>Only the original lyrics are treated as open. Later music by Bektemir Eginchiev (1910–1964), recordings and modern translations remain separate. Oral/transcribed variants exist; choose and credit a single textual version.
+Passage update (29 October 2026): First five stanzas, 20 lines, from the Kyrgyzpatent lyric sheet. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X98" s="13" t="inlineStr">
@@ -14308,8 +14648,38 @@
           <t>In Blossom / In Springtime</t>
         </is>
       </c>
-      <c r="F100" s="13" t="n"/>
-      <c r="G100" s="13" t="n"/>
+      <c r="F100" s="13" t="inlineStr">
+        <is>
+          <t>Ikkatra mana jūta
+Pie Tevim vien grib traukt,
+Kā ziedonī man krūtīs
+Viss cenšas zaļot, plaukt.
+Tur uzzied balti ziedi
+Un ugunssarkani,
+No kupluma un smaržas
+Tie līkst kā reibuši.
+Un visas manas dziesmas
+Ap tiem kā bites dūc
+Un, viņās nogrimdamas,
+Sev saldu medu sūc.</t>
+        </is>
+      </c>
+      <c r="G100" s="13" t="inlineStr">
+        <is>
+          <t>Every feeling of mine
+Longs to rush to you alone,
+As in springtime, in my breast,
+Everything strives to turn green and bloom.
+There white flowers open,
+And fire-red ones,
+Heavy with fullness and fragrance
+They bend as if drunk.
+And all my songs
+Hum around them like bees
+And, sinking into them,
+Suck sweet honey for themselves.</t>
+        </is>
+      </c>
       <c r="H100" s="13" t="inlineStr">
         <is>
           <t>Aspazija (Elza Pliekšāne)</t>
@@ -14379,7 +14749,8 @@
       </c>
       <c r="W100" s="13" t="inlineStr">
         <is>
-          <t>Scope is Aspazija’s Latvian words. The linked archival sound recording and later song settings are separate. US first-publication basis remains unverified; first-edition citation still needed.</t>
+          <t>Scope is Aspazija’s Latvian words. The linked archival sound recording and later song settings are separate. US first-publication basis remains unverified; first-edition citation still needed.
+Passage update (29 October 2026): Complete poem, 12 lines. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X100" s="13" t="inlineStr">
@@ -14437,8 +14808,44 @@
           <t>On Love — The Prophet</t>
         </is>
       </c>
-      <c r="F101" s="13" t="n"/>
-      <c r="G101" s="13" t="n"/>
+      <c r="F101" s="13" t="inlineStr">
+        <is>
+          <t>Love gives naught but itself and takes naught but from itself.
+Love possesses not nor would it be possessed;
+For love is sufficient unto love.
+When you love you should not say, “God is in my heart,” but rather, “I am in the heart of God.”
+And think not you can direct the course of love, for love, if it finds you worthy, directs your course.
+Love has no other desire but to fulfil itself.
+But if you love and must needs have desires, let these be your desires:
+To melt and be like a running brook that sings its melody to the night.
+To know the pain of too much tenderness.
+To be wounded by your own understanding of love;
+And to bleed willingly and joyfully.
+To wake at dawn with a winged heart and give thanks for another day of loving;
+To rest at the noon hour and meditate love’s ecstacy;
+To return home at eventide with gratitude;
+And then to sleep with a prayer for the beloved in your heart and a song of praise upon your lips.</t>
+        </is>
+      </c>
+      <c r="G101" s="13" t="inlineStr">
+        <is>
+          <t>Love gives naught but itself and takes naught but from itself.
+Love possesses not nor would it be possessed;
+For love is sufficient unto love.
+When you love you should not say, “God is in my heart,” but rather, “I am in the heart of God.”
+And think not you can direct the course of love, for love, if it finds you worthy, directs your course.
+Love has no other desire but to fulfil itself.
+But if you love and must needs have desires, let these be your desires:
+To melt and be like a running brook that sings its melody to the night.
+To know the pain of too much tenderness.
+To be wounded by your own understanding of love;
+And to bleed willingly and joyfully.
+To wake at dawn with a winged heart and give thanks for another day of loving;
+To rest at the noon hour and meditate love’s ecstacy;
+To return home at eventide with gratitude;
+And then to sleep with a prayer for the beloved in your heart and a song of praise upon your lips.</t>
+        </is>
+      </c>
       <c r="H101" s="13" t="inlineStr">
         <is>
           <t>Kahlil Gibran</t>
@@ -14510,7 +14917,8 @@
       </c>
       <c r="W101" s="13" t="inlineStr">
         <is>
-          <t>English is the original language of this work. Lebanese-American author died 1931. Select the love discourse rather than modern paraphrases; this is not exclusively romantic love. The selection is the original-language text; an existing English translation is not required.</t>
+          <t>English is the original language of this work. Lebanese-American author died 1931. Select the love discourse rather than modern paraphrases; this is not exclusively romantic love. The selection is the original-language text; an existing English translation is not required.
+Passage update (29 October 2026): Closing section of “On Love”, 15 lines, in Gibran’s own English (the source wraps lines; his lines are restored and each checked against it). Original English; no translation needed. Original English text; not a translation.</t>
         </is>
       </c>
       <c r="X101" s="13" t="inlineStr">
@@ -14850,8 +15258,34 @@
           <t>The captive of your love hopes for no release (first line)</t>
         </is>
       </c>
-      <c r="F104" s="13" t="n"/>
-      <c r="G104" s="13" t="n"/>
+      <c r="F104" s="13" t="inlineStr">
+        <is>
+          <t>أسير هواك لا يرجو سراحا
+ولا يلتذّ بعد لماك راحا
+وقد طال المطال فليت شعري
+أيحسن أن يقول الناس باحا
+وما سلّمت مذ حرّمت وصلي
+فكيف تحرم النظر المباحا
+بروحي فاتر الألحاظ أحوى
+بكسر جفونه مزج المزاحا
+يصول على الفؤاد بها صحاحاً
+ويثخن كسرها قلبي جراحا</t>
+        </is>
+      </c>
+      <c r="G104" s="13" t="inlineStr">
+        <is>
+          <t>The captive of your love hopes for no release,
+And, after your lips, takes no pleasure in wine.
+The waiting has grown long; I wish I knew
+Whether it would be right for people to say he has told his secret.
+You have not greeted me since you forbade our meeting;
+So how can you forbid even the glance that is allowed?
+My life for the one with languid glances and dark lips,
+Who mixes teasing into the droop of their eyelids:
+With those glances, still whole, they assail my heart,
+And their drooping covers my heart with wounds.</t>
+        </is>
+      </c>
       <c r="H104" s="13" t="inlineStr">
         <is>
           <t>Mustafa ibn Zakri (مصطفى بن زكري)</t>
@@ -14921,7 +15355,8 @@
       </c>
       <c r="W104" s="13" t="inlineStr">
         <is>
-          <t>Author death is 1917 in DCT and Libyan scholarship. Do not confuse the date of the diwan with a verified first-publication date for this poem.</t>
+          <t>Author death is 1917 in DCT and Libyan scholarship. Do not confuse the date of the diwan with a verified first-publication date for this poem.
+Passage update (29 October 2026): Complete poem, 5 couplets (10 half-lines), as printed in the Abu Dhabi Poetry Encyclopedia; the site’s decorative letter-stretching (tatweel) is removed. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X104" s="13" t="inlineStr">
@@ -15122,8 +15557,46 @@
           <t>Without a Church, without Altars</t>
         </is>
       </c>
-      <c r="F106" s="13" t="n"/>
-      <c r="G106" s="13" t="n"/>
+      <c r="F106" s="13" t="inlineStr">
+        <is>
+          <t>Be bažnyčios, be altorių,
+Be sumainymo žiedų...
+Žirgai skrenda, kiek tik nori,
+Skrendam, lekiam vienu du!
+Balti vėjai plaukus glosto
+Jau toli žmonių garsai –
+Iš auksinio žvaigždžių sosto
+Štai, mus laimina Jisai!
+Jis, kurs davė žmogui širdį
+Su troškimais neramiais,
+Vasaros vynu nugirdė –
+Jis ir nuodėmes atleis!
+Be bažnyčios, be altorių...
+Žirgai lekia žvengdami –
+Lekia, lekia musų norai
+Nesulaikomi, jauni!</t>
+        </is>
+      </c>
+      <c r="G106" s="13" t="inlineStr">
+        <is>
+          <t>Without a church, without altars,
+Without exchanging rings…
+The horses fly as far as they please,
+We fly, we race, just the two of us!
+White winds stroke our hair,
+The voices of people are already far away —
+From the golden throne of the stars,
+Look, He is blessing us!
+He who gave the human heart
+Its restless longings,
+And made it drunk on summer wine —
+He will forgive our sins as well!
+Without a church, without altars…
+The horses race on, neighing —
+Our desires race, race on,
+Unstoppable and young!</t>
+        </is>
+      </c>
       <c r="H106" s="13" t="inlineStr">
         <is>
           <t>Salomėja Nėris</t>
@@ -15195,7 +15668,8 @@
       </c>
       <c r="W106" s="13" t="inlineStr">
         <is>
-          <t>Not a blanket worldwide clearance: US reuse of a 1931 first publication needs a separate check. No modern translation or recording is cleared.</t>
+          <t>Not a blanket worldwide clearance: US reuse of a 1931 first publication needs a separate check. No modern translation or recording is cleared.
+Passage update (29 October 2026): Complete poem, 16 lines. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X106" s="13" t="inlineStr">
@@ -16211,8 +16685,30 @@
           <t>The phantom of Maryam visited him (first-line sense; mīmiyya)</t>
         </is>
       </c>
-      <c r="F115" s="13" t="n"/>
-      <c r="G115" s="13" t="n"/>
+      <c r="F115" s="13" t="inlineStr">
+        <is>
+          <t>تأوبهُ طيفُ الخيالِ بمريما
+فباتَ معنًّى مستجنًّا متيما
+تأوبه بعدَ الهجوعِ فهاضَهُ
+فأبدى من التهيامِ ما كانَ جمجما
+لطاف بها حتى إذا النفسُ اجهشتْ
+وابدتْ بناناً لي خضيباً ومِعْصما
+تولى كأنَّ اللمحَ بالطرفِ زورُهُ
+وكان وداعاً منه إنْ هو سلَّما</t>
+        </is>
+      </c>
+      <c r="G115" s="13" t="inlineStr">
+        <is>
+          <t>The phantom of Maryam came to him by night,
+And he spent the night tormented, maddened, enslaved by love.
+It came to him after sleep had fallen, and broke him anew,
+And he revealed the passion he had kept half-spoken.
+It circled close until, when my soul was close to tears,
+She showed me a hennaed fingertip and a wrist;
+Then it turned away: its visit was like a glance of the eye,
+And its greeting, if it greeted at all, was a farewell.</t>
+        </is>
+      </c>
       <c r="H115" s="13" t="inlineStr">
         <is>
           <t>Muhammad ibn al-Talaba al-Yaqubi / امحمد ولد الطلبة (1774–1856)</t>
@@ -16284,7 +16780,8 @@
       </c>
       <c r="W115" s="13" t="inlineStr">
         <is>
-          <t>The identifier is the original first line, not an invented English title. A muʿāraḍa of a poem by the early Arabic poet Humayd ibn Thawr. Year 1856 is an upper bound, not a dated composition. Reuse the historical Arabic lines, excluding modern commentary and translations.</t>
+          <t>The identifier is the original first line, not an invented English title. A muʿāraḍa of a poem by the early Arabic poet Humayd ibn Thawr. Year 1856 is an upper bound, not a dated composition. Reuse the historical Arabic lines, excluding modern commentary and translations.
+Passage update (29 October 2026): Opening four couplets of the mīmiyya (8 half-lines), as quoted in the source. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X115" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Add batch 3 of new poem passages (18 countries)
Mongolia, Montenegro, Morocco, Mozambique, Nepal, Netherlands,
Nicaragua, North Korea, North Macedonia, Oman, Pakistan, Palestine,
Paraguay, Peru, Philippines, Poland, Qatar and Sao Tome and Principe now
show a passage in the original beside English, each with a history note.
Language captions drop bracketed cataloguing notes. 94 poems to read.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 76 paired passages • 119 unfilled</t>
+          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 94 paired passages • 101 unfilled</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -17503,8 +17503,64 @@
           <t>Perfect Beauty / Sublime Qualities</t>
         </is>
       </c>
-      <c r="F121" s="13" t="n"/>
-      <c r="G121" s="13" t="n"/>
+      <c r="F121" s="13" t="inlineStr">
+        <is>
+          <t>Үлэмжийн чанар төгөлдөр
+Өнгө тунамал толь шиг
+Үзэсгэлэнтэй царайг чинь үзвээс
+Өнгө лагшин төгөлдөр өө
+Үнэхээр сэтгэлийг булаана.
+Хөшүүн сэтгэлийг уяруулагч
+Хөхөө шувууны эгшиг шиг
+Хөөрхөн эелдэг ааш чинь
+Хөгжиж суухад урамтай
+Хөөрхөн аальт минь зээ.
+Учирмагц сэнгэнэсэн
+Уран гол шиг бие чинь
+Угаас хамт бүтсэн
+Улаан зандны үнэр шиг
+Улам сэтгэлийг хөдөлгөнө.
+Бадмын дундаас дэлгэрсэн
+Балын амттай адил
+Баясгалантай биеийг чинь үзвээс
+Бахдаж ханашгүй
+Баярыг улам арвитгана.
+Хүний энэхэн насанд
+Хүссэн хэргээ бүтээгээд
+Хүсэлт тэнгэрийн оронд
+Хөлгүй жаргалангийн дунд
+Хөвөн цэнгэн жаргая.</t>
+        </is>
+      </c>
+      <c r="G121" s="13" t="inlineStr">
+        <is>
+          <t>Perfect in every noble quality,
+clear-coloured as a mirror:
+when I see your lovely face,
+your form so perfect, oh,
+it truly captivates my heart.
+Softening even a hardened heart,
+like the song of the cuckoo,
+your sweet and gentle ways
+make it a joy to sit with you,
+my lovely one with your charming ways.
+The moment we meet, refreshing
+as a lovely river, your body,
+like the scent of red sandalwood
+born with it from the start,
+stirs my heart ever more.
+Like the taste of honey
+spread from the heart of the lotus,
+when I see your joyful self,
+I cannot have my fill of admiring you,
+and my joy grows ever greater.
+In this one human life,
+having done what we long to do,
+in the heaven of our wishes,
+amid boundless bliss,
+let us float in delight together.</t>
+        </is>
+      </c>
       <c r="H121" s="13" t="inlineStr">
         <is>
           <t>Dulduityn Danzanravjaa (1803–1856)</t>
@@ -17574,7 +17630,8 @@
       </c>
       <c r="W121" s="13" t="inlineStr">
         <is>
-          <t>Use the historical Mongolian words. Modern musical arrangements, translations and scholarly commentary have separate rights. Romantic and Buddhist readings coexist.</t>
+          <t>Use the historical Mongolian words. Modern musical arrangements, translations and scholarly commentary have separate rights. Romantic and Buddhist readings coexist.
+Passage update (29 October 2026): Complete poem, five stanzas (25 lines), one for each of the five senses, as quoted in full in the linked study. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X121" s="13" t="inlineStr">
@@ -17640,8 +17697,50 @@
           <t>A Night More Precious than a Lifetime</t>
         </is>
       </c>
-      <c r="F122" s="13" t="n"/>
-      <c r="G122" s="13" t="n"/>
+      <c r="F122" s="13" t="inlineStr">
+        <is>
+          <t>Док ево ти дивне виле лаким кроком ђе ми лети –
+завид’те ми, сви бесмртни, на тренутак овај свети!
+Ход је вилин млого дични на Аврорин када шеће,
+од сребрног свога прага над прољећем кад се креће;
+зрак је виле младолике тако красан ка Атине,
+огледало и мазање презиру јој черте фине.
+Устав’ луно, б’јела кола, продужи ми часе миле,
+кад су сунце над Инопом уставити могле виле.
+Прелесницу како видим, загрлим је ка бог вели,
+уведем је под шатором к испуњењу светој жељи.
+При зракама красне луне, при свјећици запаљеној
+пламена се споји душа ка душици раскаљеној
+и цјеливи божествени душу с душом драгом слију.
+Ах, цјеливи, божа мана, све прелести рајске лију!
+Цјелителни балсам свети најмирисни аромати
+што је небо земљи дало на усне јој стах сисати.
+Совршенство творенија, таинствене силе боже,
+ништа љепше нит’ је када нити од ње створит може!</t>
+        </is>
+      </c>
+      <c r="G122" s="13" t="inlineStr">
+        <is>
+          <t>When look, a lovely fairy comes flying to me with a light step —
+envy me, all you immortals, this holy moment!
+The fairy’s step is far more stately than Aurora’s when she walks
+from her silver threshold as she moves above the spring;
+the gaze of the youthful fairy is as lovely as Athena’s,
+her fine features scorn both mirror and paint.
+Stay, moon, your white chariot; prolong my precious hours,
+since fairies once could make the sun stand still above Inop.
+As soon as I see the enchantress, I embrace her as a god would,
+and lead her into the tent to fulfil a holy wish.
+By the rays of the lovely moon, by a lighted candle,
+a soul of flame joined a soul aglow,
+and divine kisses poured soul into beloved soul.
+Ah, kisses, manna of God, pouring out all the charms of heaven!
+The holy healing balm, the most fragrant of perfumes
+that heaven gave the earth, I began to drink from her lips.
+Perfection of creation, mysterious power of God,
+nothing more beautiful ever was, or could be made, than she!</t>
+        </is>
+      </c>
       <c r="H122" s="13" t="inlineStr">
         <is>
           <t>Petar II Petrović-Njegoš</t>
@@ -17713,7 +17812,8 @@
       </c>
       <c r="W122" s="13" t="inlineStr">
         <is>
-          <t>Njegoš died 1851. Titles and manuscript readings vary; compare an authoritative scan before final quotation. Original poem only; later editions’ critical apparatus is separate. The selection is the original-language text; an existing English translation is not required.</t>
+          <t>Njegoš died 1851. Titles and manuscript readings vary; compare an authoritative scan before final quotation. Original poem only; later editions’ critical apparatus is separate. The selection is the original-language text; an existing English translation is not required.
+Passage update (29 October 2026): 18 lines from the love scene of the poem, from the fairy’s arrival to the lovers’ kiss (Serbian Wikisource, 100% proofread). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X122" s="13" t="inlineStr">
@@ -17775,8 +17875,54 @@
           <t>Is there, for a lovesick one, a sip from your lips? (first-line sense; reading uncertain)</t>
         </is>
       </c>
-      <c r="F123" s="13" t="n"/>
-      <c r="G123" s="13" t="n"/>
+      <c r="F123" s="13" t="inlineStr">
+        <is>
+          <t>هَل لِصَبٍّ مِن لَماكَ المُزدَري
+بِسُلافِ الراح
+رَشَفاتٌ مُزِجَت بِالسُكرِ
+تَمنَحُ الأَفراح
+مَروِيّاتٌ عَن صَحاحِ الجَوهَرِ
+عَن مُنى الأَرواح
+عَن هِلالِ الحُسنِ عَن ظُبى النَقا
+عَن قَضيبِ البان
+مِن جِنانَ الوَصلِ دوني أَغلَفا
+رَقَّ يا رَضوان
+وَاِرثِ لي مِن ذا العَذابِ الأَكبَرِ
+فَعَسى أَرتاح
+فَعَلى ذاكَ المُحَيّا الأَنوارِ
+ذي السَنا الوَضّاح
+مِن شَجٍّ نَشرُ سَلامٍ عَنبَري
+ما اِنبَرى الإِصباح
+وَثَنَت بانَ الرُبى كَفُّ الصَبا
+وَشَدا القُمري
+وَصَبا قَلبي لِأَيّامِ الصِبا
+رَيِّقِ العُمرِ</t>
+        </is>
+      </c>
+      <c r="G123" s="13" t="inlineStr">
+        <is>
+          <t>Is there, for a lovesick man, from your scornful lips,
+like the finest wine,
+sips mixed with sugar
+that grant delight —
+sips handed down from the truest jewels,
+from the souls’ desire,
+from the crescent of beauty, from the gazelle of the dunes,
+from the willow wand?
+You have shut the gardens of union against me:
+have pity, O Ridwan,
+and pity me in this great torment,
+that perhaps I may find rest.
+And upon that face of light,
+of radiant brightness,
+from a grieving man, an amber-scented greeting spreads
+for as long as morning breaks,
+and the east wind’s hand bends the willows of the hills,
+and the turtle-dove sings,
+and my heart yearns for the days of youth,
+the fresh bloom of life.</t>
+        </is>
+      </c>
       <c r="H123" s="13" t="inlineStr">
         <is>
           <t>Ibn Zakur (ابن زاكور)</t>
@@ -17850,7 +17996,8 @@
       </c>
       <c r="W123" s="13" t="inlineStr">
         <is>
-          <t>Wine and garden imagery accompanies courtly erotic longing. Opening words are the identifier. Transcriptions disagree in some readings; compare a historical diwan before final quotation. Modern website commentary excluded.</t>
+          <t>Wine and garden imagery accompanies courtly erotic longing. Opening words are the identifier. Transcriptions disagree in some readings; compare a historical diwan before final quotation. Modern website commentary excluded.
+Passage update (29 October 2026): Complete muwashshah, 10 couplets set out as 20 short lines. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X123" s="13" t="inlineStr">
@@ -17912,8 +18059,42 @@
           <t>To Love</t>
         </is>
       </c>
-      <c r="F124" s="13" t="n"/>
-      <c r="G124" s="13" t="n"/>
+      <c r="F124" s="13" t="inlineStr">
+        <is>
+          <t>Amar é um prazer se nos amámos
+Alguém que pode amar-nos e nos ama,
+Amar é um prazer, se nos chama,
+Alguém continuamente que chamámos.
+Então a vida inteira a rir levamos,
+Que o mesmo fogo ardente nos inflama
+Os ideais da vida, e bem, a fama,
+Mãos dadas pelo mundo procuramos.
+No encapelado mar da existência
+O amor é compassiva indulgência
+A culpa original de nossos pais.
+Tudo na vida é fruto do amor
+Quem o tirar e olhar em seu redor
+Encontra só tristeza – e nada mais</t>
+        </is>
+      </c>
+      <c r="G124" s="13" t="inlineStr">
+        <is>
+          <t>To love is a pleasure if we love
+someone who can love us, and does;
+to love is a pleasure if there calls to us
+someone we are always calling.
+Then we spend our whole life laughing,
+for the same burning fire inflames us;
+life’s ideals, and goodness, and fame
+we seek hand in hand through the world.
+On the stormy sea of existence
+love is a compassionate forgiveness
+of the original sin of our first parents.
+Everything in life is the fruit of love;
+whoever takes it away and looks around
+finds only sadness, and nothing more.</t>
+        </is>
+      </c>
       <c r="H124" s="13" t="inlineStr">
         <is>
           <t>Rui de Noronha (1909–1943)</t>
@@ -17983,7 +18164,8 @@
       </c>
       <c r="W124" s="13" t="inlineStr">
         <is>
-          <t>Sonetos appeared posthumously in 1946. Scholars document editorial alterations in that edition; compare the poem with a lifetime newspaper text before establishing a definitive version. Modern notes and revisions are separate.</t>
+          <t>Sonetos appeared posthumously in 1946. Scholars document editorial alterations in that edition; compare the poem with a lifetime newspaper text before establishing a definitive version. Modern notes and revisions are separate.
+Passage update (29 October 2026): Complete sonnet, 14 lines (as printed in the school module, Lesson 25). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X124" s="13" t="inlineStr">
@@ -18406,8 +18588,26 @@
           <t>Those two eyebrows… (first line)</t>
         </is>
       </c>
-      <c r="F128" s="13" t="n"/>
-      <c r="G128" s="13" t="n"/>
+      <c r="F128" s="13" t="inlineStr">
+        <is>
+          <t>दुइ आँखिभौं त तयार छन्, तरवार पो किन चाहियो,
+तिमी आफु मालिक भै गयौ, सरकार पो किन चाहियो ॥१॥
+पहरा कडा छ कटाक्षको, हरदम् तयारि मुहारमा,
+घर भन्नु भारि महल् न हो, दरवार पो किन चाहियो ॥२॥
+कति चम्‌किलो छ हँसाइको, हिसिमा किरन् पनि दाँतको,
+मणि मोति नीर जुहार् न हो, अरु हार पो किन चाहियो ॥३॥</t>
+        </is>
+      </c>
+      <c r="G128" s="13" t="inlineStr">
+        <is>
+          <t>Your two eyebrows stand ready as they are: why would you need a sword?
+You have become the master yourself: why would you need a government? ॥1॥
+The guard of your sidelong glance is strict, always ready in your face;
+your home is a mighty palace already: why would you need a royal court? ॥2॥
+How bright are the rays of your teeth when you laugh and smile!
+Are they not jewels, pearls and gems? Why would you need any other necklace? ॥3॥</t>
+        </is>
+      </c>
       <c r="H128" s="13" t="inlineStr">
         <is>
           <t>Motiram Bhatta (मोतीराम भट्ट)</t>
@@ -18477,7 +18677,8 @@
       </c>
       <c r="W128" s="13" t="inlineStr">
         <is>
-          <t>Original Nepali only; spelling differs between transcriptions. Archive’s explanatory summaries are modern and excluded. First print edition not established.</t>
+          <t>Original Nepali only; spelling differs between transcriptions. Archive’s explanatory summaries are modern and excluded. First print edition not established.
+Passage update (29 October 2026): Complete ghazal, 3 couplets (6 lines), with its verse numbers as printed. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X128" s="13" t="inlineStr">
@@ -18539,8 +18740,42 @@
           <t>May Blossoms, III — Break white May branches from the Tree of Life (first line)</t>
         </is>
       </c>
-      <c r="F129" s="13" t="n"/>
-      <c r="G129" s="13" t="n"/>
+      <c r="F129" s="13" t="inlineStr">
+        <is>
+          <t>Breek blanke meien van den Levensboom!
+Nu is de Mei gekomen, ook voor mij.
+Als witte vlinders fladdren ze ons voorbij,
+De bloesemblaadren van mijn lentedroom.
+Zie, dit is weelde: wandlen zij aan zij
+In 't bloeiend Eden onzer liefde, loom
+En stil van 't groot geluk, met teedren schroom
+Ontvangen en gedragen, bang en blij.
+Nu laat mij leunen aan uw borst, mijn lief,
+En leg uw streelhand op mijn lokken zacht
+En zeg of 't u wel heugt, die eerste brief,
+Die eerste kus en o die winternacht,
+Toen Liefde mij in 't hart sloop als een dief,
+Nu scepter-zwaaiende in vorstinnepracht.</t>
+        </is>
+      </c>
+      <c r="G129" s="13" t="inlineStr">
+        <is>
+          <t>Break white May blossom from the Tree of Life!
+Now May has come, for me as well.
+Like white butterflies they flutter past us,
+the blossom petals of my spring dream.
+See, this is bliss: to wander side by side
+in the blossoming Eden of our love, languid
+and quiet with great happiness, with tender shyness
+received and carried, fearful and glad.
+Now let me lean against your breast, my love,
+and lay your stroking hand softly on my hair,
+and tell me if you remember it, that first letter,
+that first kiss, and oh, that winter night
+when Love crept into my heart like a thief,
+and now waves his sceptre in the splendour of a queen.</t>
+        </is>
+      </c>
       <c r="H129" s="13" t="inlineStr">
         <is>
           <t>Hélène Swarth</t>
@@ -18612,7 +18847,8 @@
       </c>
       <c r="W129" s="13" t="inlineStr">
         <is>
-          <t>Scope is Swarth’s poem only. DBNL labels the journal as partly copyright-protected; do not treat the whole journal or modern editorial material as cleared. Modern translations are separate.</t>
+          <t>Scope is Swarth’s poem only. DBNL labels the journal as partly copyright-protected; do not treat the whole journal or modern editorial material as cleared. Modern translations are separate.
+Passage update (29 October 2026): Complete sonnet, 14 lines. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X129" s="13" t="inlineStr">
@@ -18832,8 +19068,42 @@
           <t>In Winter</t>
         </is>
       </c>
-      <c r="F131" s="13" t="n"/>
-      <c r="G131" s="13" t="n"/>
+      <c r="F131" s="13" t="inlineStr">
+        <is>
+          <t>En invernales horas, mirad a Carolina.
+Medio apelotonada, descansa en el sillón,
+envuelta con su abrigo de marta cibelina
+y no lejos del fuego que brilla en el salón.
+El fino angora blanco, junto a ella se reclina,
+rozando con su hocico la falda de Alençón,
+no lejos de las jarras de porcelana china
+que medio oculta un biombo de seda del Japón.
+Con sus sutiles filtros la invade un dulce sueño;
+entro, sin hacer ruido; dejo mi abrigo gris;
+voy a besar su rostro, rosado y halagüeño
+como una rosa roja que fuera flor de lis;
+abre los ojos; mírame, con su mirar risueño
+y en tanto cae la nieve del cielo de París.</t>
+        </is>
+      </c>
+      <c r="G131" s="13" t="inlineStr">
+        <is>
+          <t>In the hours of winter, look at Carolina.
+Half curled up, she rests in the armchair,
+wrapped in her sable coat,
+not far from the fire that glows in the drawing room.
+The fine white angora lies beside her,
+brushing her Alençon-lace skirt with its nose,
+not far from the Chinese porcelain jars
+half hidden by a Japanese silk screen.
+With its subtle potions a sweet sleep steals over her;
+I come in without a sound; I leave my grey coat;
+I go to kiss her face, rosy and inviting
+like a red rose that might be a fleur-de-lis;
+she opens her eyes; she looks at me with her smiling gaze,
+and meanwhile the snow falls from the Paris sky.</t>
+        </is>
+      </c>
       <c r="H131" s="13" t="inlineStr">
         <is>
           <t>Rubén Darío</t>
@@ -18905,7 +19175,8 @@
       </c>
       <c r="W131" s="13" t="inlineStr">
         <is>
-          <t>Scope is the poem text; do not assume modern illustrations or adaptations share these rights.</t>
+          <t>Scope is the poem text; do not assume modern illustrations or adaptations share these rights.
+Passage update (29 October 2026): Complete sonnet, 14 lines. The edition’s drop capital (“E N”) is joined to “En”. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X131" s="13" t="inlineStr">
@@ -19207,8 +19478,20 @@
           <t>The long winter-solstice night (first line)</t>
         </is>
       </c>
-      <c r="F134" s="13" t="n"/>
-      <c r="G134" s="13" t="n"/>
+      <c r="F134" s="13" t="inlineStr">
+        <is>
+          <t>冬至ㅅᄃᆞᆯ 기나긴 밤을 한허리를 버혀 내여
+春風 니불 아레 서리서리 너헛다가
+어론 님 오신 날 밤이여든 구뷔구뷔 펴리라</t>
+        </is>
+      </c>
+      <c r="G134" s="13" t="inlineStr">
+        <is>
+          <t>I will cut the waist from the long, long night of the midwinter month,
+and fold it, coil upon coil, under a quilt of spring breeze,
+and on the night my love comes home, unroll it, fold by fold.</t>
+        </is>
+      </c>
       <c r="H134" s="13" t="inlineStr">
         <is>
           <t>Hwang Jini</t>
@@ -19278,7 +19561,8 @@
       </c>
       <c r="W134" s="13" t="inlineStr">
         <is>
-          <t>Country is geographic: Hwang Jini was associated with Kaesong, now North Korea. Shared pre-division Korean heritage, not modern nationality. Authorship is traditionally transmitted; modern English versions and performances are separate.</t>
+          <t>Country is geographic: Hwang Jini was associated with Kaesong, now North Korea. Shared pre-division Korean heritage, not modern nationality. Authorship is traditionally transmitted; modern English versions and performances are separate.
+Passage update (29 October 2026): Complete sijo, 3 lines, in the text of the anthology Cheonggu yeongeon (1728), poem 287, with its old Hangul and Chinese characters. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X134" s="13" t="inlineStr">
@@ -19336,8 +19620,44 @@
           <t>Bisera (a woman's name; related to the word pearl)</t>
         </is>
       </c>
-      <c r="F135" s="13" t="n"/>
-      <c r="G135" s="13" t="n"/>
+      <c r="F135" s="13" t="inlineStr">
+        <is>
+          <t>Бисеро моме, Бисеро,
+што носиш бисер на грло?
+Твоето грло хубаво
+и от дробнаго бисера
+хилјада пати побело.
+Бисеро моме, Бисеро,
+зошто со бисер покриваш
+твоето грло хубаво?
+Ја нејку бисер да баца,
+тук сака твоето грло.
+Бисеро моме, Бисеро,
+за кого нижиш бисерот?
+За кого готвиш дарои?
+Ја дарој бисер не сака,
+тук сака мома Бисера.</t>
+        </is>
+      </c>
+      <c r="G135" s="13" t="inlineStr">
+        <is>
+          <t>Bisera, my girl, Bisera,
+why do you wear pearls at your throat?
+Your lovely throat
+is a thousand times whiter
+than even the finest pearls.
+Bisera, my girl, Bisera,
+why do you cover with pearls
+your lovely throat?
+I don’t want to kiss pearls,
+it is your throat I long for.
+Bisera, my girl, Bisera,
+for whom are you stringing the pearls?
+For whom are you preparing gifts?
+I want no gift of pearls,
+I want the maiden Bisera.</t>
+        </is>
+      </c>
       <c r="H135" s="13" t="inlineStr">
         <is>
           <t>Konstantin Miladinov</t>
@@ -19407,7 +19727,8 @@
       </c>
       <c r="W135" s="13" t="inlineStr">
         <is>
-          <t>Wikisource explicitly marks the author’s works public domain because he died more than 100 years ago. Modern anthology notes and translations excluded; preserve historical dialect rather than silently modernising it. The selection is the original-language text; an existing English translation is not required.</t>
+          <t>Wikisource explicitly marks the author’s works public domain because he died more than 100 years ago. Modern anthology notes and translations excluded; preserve historical dialect rather than silently modernising it. The selection is the original-language text; an existing English translation is not required.
+Passage update (29 October 2026): Complete poem, 15 lines. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X135" s="13" t="inlineStr">
@@ -19633,8 +19954,50 @@
           <t>O you whose love has exalted you and humbled me / O you who are miserly with union (first-line identifiers)</t>
         </is>
       </c>
-      <c r="F137" s="13" t="n"/>
-      <c r="G137" s="13" t="n"/>
+      <c r="F137" s="13" t="inlineStr">
+        <is>
+          <t>يا مَنْ هواه أعزّه وأذلّني
+كيف السبيلُ إلى وصالِكَ؟ دُلّني
+وتركتني حيرانَ صبّاً هائمًا
+أرعى النجوم وأنت في نومٍ هني
+عاهدتني أن لا تميلَ عن الهوى
+وحلفتَ لي يا غصنُ أن لا تنثني
+هبَّ النسيم ومال غصنٌ مثلُه
+أين الزمانُ؟ وأين ما عاهدتني؟
+جاد الزمان وأنتَ ما واصلتني
+يا باخلاً بالوصل أنتَ قتلتني
+واصلتَني حتى ملكتَ حُشاشتي
+ورجَعتَ من بعد الوصال هجرتني
+فلأقعدنَّ على الطريق فأشتكي
+في زيِّ مظلومٍ وأنت ظلمتَني
+ولأشكينَّكَ عند سلطان الهوى
+لِيُعذبنَّك مثلَ ما عذَّبتني
+ولأدعوَنَّ عليك في جُنْح الدجى
+فعساك تُبلى مثل ما أبليتني</t>
+        </is>
+      </c>
+      <c r="G137" s="13" t="inlineStr">
+        <is>
+          <t>O you whose love has raised you up and brought me low,
+how can I reach union with you? Show me the way.
+You have left me bewildered, lovesick, wandering,
+watching the stars while you sleep sweetly.
+You promised me you would not turn from love,
+and swore to me, O willow branch, that you would not bend.
+The breeze blew, and a branch like you bent with it:
+where is that time now? Where is what you promised me?
+Time has been generous, yet you have not come to me;
+O you who are miserly with union, you have killed me.
+You came to me until you owned the last of my soul,
+then, after our union, you turned and left me.
+So I will sit by the roadside and complain,
+dressed as one wronged, for you have wronged me;
+and I will accuse you before the sultan of love,
+so that he punishes you as you have tormented me;
+and I will call down a curse on you in the depth of night,
+so that you may be worn down as you have worn me down.</t>
+        </is>
+      </c>
       <c r="H137" s="13" t="inlineStr">
         <is>
           <t>Saʿid ibn Ahmad al-Busaʿidi (سعيد بن أحمد البوسعيدي)</t>
@@ -19704,7 +20067,8 @@
       </c>
       <c r="W137" s="13" t="inlineStr">
         <is>
-          <t>Text varies in stanza/line count across modern reproductions. Biography gives differing death traditions (1803 or 1810); both are well outside copyright term. Modern song settings and editorial prose excluded.</t>
+          <t>Text varies in stanza/line count across modern reproductions. Biography gives differing death traditions (1803 or 1810); both are well outside copyright term. Modern song settings and editorial prose excluded.
+Passage update (29 October 2026): Complete poem, 9 couplets (18 half-lines), as printed by the Al-Babtain Library. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X137" s="13" t="inlineStr">
@@ -19766,8 +20130,38 @@
           <t>Calling Ranjha, Ranjha, I myself have become Ranjha (first-line sense)</t>
         </is>
       </c>
-      <c r="F138" s="13" t="n"/>
-      <c r="G138" s="13" t="n"/>
+      <c r="F138" s="13" t="inlineStr">
+        <is>
+          <t>ਰਾਂਝਾ ਰਾਂਝਾ ਕਰਦੀ ਨੀ ਮੈਂ
+ਆਪੇ ਰਾਂਝਾ ਹੋਈ।
+ਸੱਦੋ ਨੀ ਮੈਨੂੰ ਧੀਦੋ ਰਾਂਝਾ
+ਹੀਰ ਨਾ ਆਖੋ ਕੋਈ।
+ਰਾਂਝਾ ਮੈਂ ਵਿੱਚ ਮੈਂ ਰਾਂਝੇ ਵਿੱਚ
+ਹੋਰ ਖਿਆਲ ਨਾ ਕੋਈ।
+ਮੈਂ ਨਹੀਂ ਉਹ ਆਪ ਹੈ ਆਪਣੀ
+ਆਪ ਕਰੇ ਦਿਲਗੋਈ।
+ਹੱਥ ਖੂੰਡੀ ਮੇਰੇ ਅੱਗੇ ਮੰਗੂ
+ਮੋਢੇ ਭੂਰਾ ਲੋਈ।
+ਬੁਲ੍ਹਾ ਹੀਰ ਸਲੇਟੀ ਵੇਖੋ
+ਕਿੱਥੇ ਜਾ ਖਲੋਈ।</t>
+        </is>
+      </c>
+      <c r="G138" s="13" t="inlineStr">
+        <is>
+          <t>Calling “Ranjha, Ranjha”, O friends,
+I myself have become Ranjha.
+Call me Dhido Ranjha, friends;
+let no one call me Heer.
+Ranjha is in me, I am in Ranjha;
+there is no other thought.
+It is not I: it is he himself
+who comforts his own heart.
+A herder’s staff in my hand, the herd before me,
+a brown blanket on my shoulders.
+Bulleh, look at Heer of the Sial clan:
+where has she come to stand!</t>
+        </is>
+      </c>
       <c r="H138" s="13" t="inlineStr">
         <is>
           <t>Bulleh Shah</t>
@@ -19837,7 +20231,8 @@
       </c>
       <c r="W138" s="13" t="inlineStr">
         <is>
-          <t>Classical Punjabi text; modern compilation and translation are separate. Bulleh Shah died in the eighteenth century. The linked Gurmukhi transcription is not the historical Shahmukhi script; verify variant readings. Country connection is his Kasur/Punjab literary tradition. The selection is the original-language text; an existing English translation is not required.</t>
+          <t>Classical Punjabi text; modern compilation and translation are separate. Bulleh Shah died in the eighteenth century. The linked Gurmukhi transcription is not the historical Shahmukhi script; verify variant readings. Country connection is his Kasur/Punjab literary tradition. The selection is the original-language text; an existing English translation is not required.
+Passage update (29 October 2026): Complete kafi, 12 lines, in Gurmukhi script (proofread scan of Kafian Bulleh Shah, printed p. 121). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X138" s="13" t="inlineStr">
@@ -20008,8 +20403,62 @@
           <t>Longing and Reproach</t>
         </is>
       </c>
-      <c r="F140" s="13" t="n"/>
-      <c r="G140" s="13" t="n"/>
+      <c r="F140" s="13" t="inlineStr">
+        <is>
+          <t>كيف أغويتَني وأمعنتَ صَدّا
+يا حبيبًا أعطى قليلًا وأكدى
+ودَّ قلبي لو يجهل الحبَّ لما
+أنْ رآه يحول سَقْمًا ووَجْدا
+وشكتْ أضلعي من القلب نارًا
+هل عهدنَ الهوى سلامًا وبَردا؟!
+طلع الفجرُ باسمًا فتأمّلْ
+بنجوم الدجى تَرنَّحُ سُهْدا
+هي مثلي حيرى وعمّا قريبٍ
+تتوارى مع الظلام وتهدا
+لكَ حمّلتُها رسالةَ شوقٍ
+وعتابٍ، أظنّها لا تُؤدّى …
+قلتُ للطير حين أصبح يشدو
+«أيها الطيرُ عِمْ صباحًا!» فَردّا
+ثم غنّى أنشودةً عن حبيبٍ
+لم يكن ظالمًا، ولا خان عهدا
+أضرمَ الذكرياتِ بي ثُمّ ولّى
+لا رماكَ الصيّادُ … أسرفتَ جِدّا
+جمع اللهُ في مُحيّا حبيبي
+أُقحوانًا وياسَمينًا وَوَردا
+وابتسامًا لا يهجر الثغرَ إلَّا
+عند قولي له: أَتُنجز وعدا؟
+لا عرفتَ الوَفا ولا كان وعدٌ
+يجعل البسمةَ الوديعةَ حِقدا</t>
+        </is>
+      </c>
+      <c r="G140" s="13" t="inlineStr">
+        <is>
+          <t>How you seduced me, then turned ever further away!
+O beloved who gave a little, then gave no more.
+My heart wished it knew nothing of love
+when it saw love turn to sickness and longing;
+and my ribs complained of the fire in my heart:
+have they ever known love as cool and peaceful?
+Dawn rose smiling: look at
+the night’s stars swaying, sleepless.
+They are bewildered like me, and soon
+they will vanish with the dark and grow still.
+I gave them a message for you, of longing
+and reproach; I think it will not be delivered…
+I said to the bird when it began to sing at dawn,
+“Good morning, bird!” and it answered,
+then sang a song about a beloved
+who was never cruel and never broke a promise.
+It kindled my memories, then flew away:
+may no hunter ever shoot you… but you went too far!
+God gathered in my beloved’s face
+camomile, jasmine and rose,
+and a smile that leaves those lips only
+when I say: will you keep a promise?
+Forget faithfulness, then: let there be no promise
+that turns that gentle smile to bitterness.</t>
+        </is>
+      </c>
       <c r="H140" s="13" t="inlineStr">
         <is>
           <t>Ibrahim Tuqan (إبراهيم طوقان)</t>
@@ -20079,7 +20528,8 @@
       </c>
       <c r="W140" s="13" t="inlineStr">
         <is>
-          <t>Collection’s first issue date is listed as unknown; do not treat 2012 as composition date. Original Arabic only; modern translation and editorial material separate.</t>
+          <t>Collection’s first issue date is listed as unknown; do not treat 2012 as composition date. Original Arabic only; modern translation and editorial material separate.
+Passage update (29 October 2026): Complete poem, 24 half-lines (Hindawi edition of the complete poems; the section dividers are omitted). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X140" s="13" t="inlineStr">
@@ -20385,8 +20835,54 @@
           <t>To Two Black Eyes</t>
         </is>
       </c>
-      <c r="F143" s="13" t="n"/>
-      <c r="G143" s="13" t="n"/>
+      <c r="F143" s="13" t="inlineStr">
+        <is>
+          <t>Chopĩ haitýpe mokói oĩva,
+ndojohejávai maramoĩte;
+peteĩchaitéva hữngue porãme
+ha iporãnguépe katu kõingue.
+Upe hữnguépe he’i jakúpe
+ha pyharépe: tapomohữ.
+Tesapehápe he’i jasýpe
+ku oike potávo: toroipyru.
+Ma’ẽ saguýpe jahechapáma
+Ka’a pa’ữme kuarahysẽ
+ha om’ẽmbápe nahesakãiri
+hendy porãnte jasyichaite.
+Mba’e mbyasýpe "luto" voíva
+ha vy’ahápe tory rupa
+Ma’ẽ hatãme chemopirĩva
+ma’ẽ mbeguépe chemoãngaipa.
+Omoporãva kuñataĩnguéra
+jáma hi’áva, jáma hete,
+pe pende jara noikotevẽiri
+porã oñohẽgui pende pire.</t>
+        </is>
+      </c>
+      <c r="G143" s="13" t="inlineStr">
+        <is>
+          <t>Two thrushes that are in their nest
+and never part from each other,
+alike in their beautiful blackness
+and twins in their beauty.
+For their blackness they say to the pheasant
+and to the night: we will out-darken you;
+for their shine they say to the moon,
+as it goes in: we will take your place.
+When they glance sideways, it is as if we saw
+the sun rising between the woods,
+and when they look straight, they do not merely shine:
+they blaze as brightly as the moon.
+For sorrow they are ready mourning,
+for joy a spring of delight;
+in hard looks they make me shiver,
+in soft looks they make me sin.
+What makes young women beautiful,
+their hair, their figure,
+your mistress does not need,
+for beauty overflows from you.</t>
+        </is>
+      </c>
       <c r="H143" s="13" t="inlineStr">
         <is>
           <t>Ignacio Alberto Pane</t>
@@ -20456,7 +20952,8 @@
       </c>
       <c r="W143" s="13" t="inlineStr">
         <is>
-          <t>Use Pane’s Guaraní original. Spanish free translation by Sinforiano Buzó Gómez is separately authored and is not covered by this original-rights assessment. Check modern orthographic editing before verbatim reuse.</t>
+          <t>Use Pane’s Guaraní original. Spanish free translation by Sinforiano Buzó Gómez is separately authored and is not covered by this original-rights assessment. Check modern orthographic editing before verbatim reuse.
+Passage update (29 October 2026): Complete poem, 20 lines, in Guaraní (text as printed in Las cien mejores poesías en guaraní, 1997). English translated from the Guaraní, checked against the free Spanish version printed with it. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X143" s="13" t="inlineStr">
@@ -20518,8 +21015,42 @@
           <t>A Dead Idyll</t>
         </is>
       </c>
-      <c r="F144" s="13" t="n"/>
-      <c r="G144" s="13" t="n"/>
+      <c r="F144" s="13" t="inlineStr">
+        <is>
+          <t>Qué estará haciendo esta hora mi andina y dulce Rita
+de junco y capulí;
+ahora que me asfixia Bizancio, y que dormita
+la sangre, como flojo cognac, dentro de mí.
+Dónde estarán sus manos que en actitud contrita
+planchaban en las tardes blancuras por venir;
+ahora, en esta lluvia que me quita
+las ganas de vivir.
+Qué será de su falda de franela; de sus
+afanes; de su andar;
+de su sabor a cañas de mayo del lugar.
+Ha de estarse a la puerta mirando algún celaje,
+y al fin dirá temblando: «Qué frío hay... Jesús!»
+y llorará en las tejas un pájaro salvaje.</t>
+        </is>
+      </c>
+      <c r="G144" s="13" t="inlineStr">
+        <is>
+          <t>What can my sweet Andean Rita be doing at this hour,
+Rita of reeds and wild cherries,
+now that Byzantium stifles me, and my blood
+drowses inside me like weak cognac?
+Where can her hands be, which, as if in penitence,
+ironed in the evenings whitenesses still to come,
+now, in this rain that takes from me
+the wish to live?
+What has become of her flannel skirt, of her
+toil, of her walk,
+of her taste of the local May sugar cane?
+She must be standing at the door, watching the sunset clouds,
+and at last she will say, shivering: “How cold it is… Jesus!”
+and on the roof tiles a wild bird will weep.</t>
+        </is>
+      </c>
       <c r="H144" s="13" t="inlineStr">
         <is>
           <t>César Vallejo</t>
@@ -20591,7 +21122,8 @@
       </c>
       <c r="W144" s="13" t="inlineStr">
         <is>
-          <t>Vallejo died 1938. Use the original Spanish, excluding modern translations. Exact print basis of the transcription is not identified; compare Los heraldos negros scan. The selection is the original-language text; an existing English translation is not required.</t>
+          <t>Vallejo died 1938. Use the original Spanish, excluding modern translations. Exact print basis of the transcription is not identified; compare Los heraldos negros scan. The selection is the original-language text; an existing English translation is not required.
+Passage update (29 October 2026): Complete poem, 14 lines, from the proofread scan of Los heraldos negros (1919). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X144" s="13" t="inlineStr">
@@ -20653,8 +21185,46 @@
           <t>Florante and Laura — To Celia</t>
         </is>
       </c>
-      <c r="F145" s="13" t="n"/>
-      <c r="G145" s="13" t="n"/>
+      <c r="F145" s="13" t="inlineStr">
+        <is>
+          <t>Cong pag saulang cong basahin sa isip
+ang nañgacaraang arao ñg pag-ibig,
+may mahahaguilap cayang natititic
+liban na cay Celiang namugad sa dibdib?
+Yaong Celiang laguing pinañgañganiban
+baca macalimot sa pag-iibigan;
+ang iquinalubog niyaring capalaran
+sa lubhang malalim na caralitaan.
+Macaligtaang co cayang di basahin
+nagdaáng panahón ñg suyuan namin?
+caniyang pagsintáng guinugol sa aquin
+at pinuhunan cong pagod at hilahil?
+Lumipas ang arao na lubhang matamis
+at ualáng nátira condi ang pag-ibig ,
+tapat na pag suyong lalagui sa dibdib
+hanggang sa libiñgan bangcay co,i, maidlip.</t>
+        </is>
+      </c>
+      <c r="G145" s="13" t="inlineStr">
+        <is>
+          <t>When I go back and read over in my mind
+the days of love that have passed,
+can anything be found written there
+except Celia, who nested in my heart?
+That Celia whom I always feared
+might forget our love;
+the one who sank this fortune of mine
+into the deepest poverty.
+Could I neglect to read over
+the past time of our courtship,
+the love she spent on me,
+and the toil and sorrow I gave for it?
+The sweetest days have gone by,
+and nothing is left but love,
+a faithful devotion that will stay in my heart
+until my body sleeps in the grave.</t>
+        </is>
+      </c>
       <c r="H145" s="13" t="inlineStr">
         <is>
           <t>Francisco Balagtas / Baltazar</t>
@@ -20726,7 +21296,8 @@
       </c>
       <c r="W145" s="13" t="inlineStr">
         <is>
-          <t>Original Tagalog dedication only; exclude the modern digital notes and unrelated commentary. Author died 1862; commentator died 1941. Old spelling and transcription errors require comparison with a scan. The selection is the original-language text; an existing English translation is not required.</t>
+          <t>Original Tagalog dedication only; exclude the modern digital notes and unrelated commentary. Author died 1862; commentator died 1941. Old spelling and transcription errors require comparison with a scan. The selection is the original-language text; an existing English translation is not required.
+Passage update (29 October 2026): First four stanzas of the dedication, 16 lines. The edition’s footnote numbers are removed, and the Gutenberg stand-in “n~g” is written “ñg” for the old Tagalog ng with a tilde. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X145" s="13" t="inlineStr">
@@ -20788,8 +21359,42 @@
           <t>To Laura</t>
         </is>
       </c>
-      <c r="F146" s="13" t="n"/>
-      <c r="G146" s="13" t="n"/>
+      <c r="F146" s="13" t="inlineStr">
+        <is>
+          <t>Ledwiem ciebie zobaczył, jużem się zapłonił,
+W nieznaném oku dawnéj znajomości pytał,
+I s twych jagód wzajemny rumieniec wykwitał
+Jak z róży, któréj piersi zaranek odsłonił.
+Ledwieś piosnkę zaczęła, jużem łzy uronił,
+Twój głos wnikał do serca i za duszę chwytał;
+Zdało się że ją anioł po imieniu witał,
+I w zegar niebios chwilę zbawienia zadzwonił.
+O luba! niech twe oczy przyznać się nie boją,
+Jeśli cię mém spojrzeniem, jeśli głosem wzruszę,
+Nie dbam że los i ludzie przeciwko nam stoją,
+Że uciekać i kochać bez nadziei muszę.
+Niech ślub ziemski innego darzy ręką twoją,
+Tylko wyznaj że Bóg mi poślubił twą duszę.</t>
+        </is>
+      </c>
+      <c r="G146" s="13" t="inlineStr">
+        <is>
+          <t>I had barely seen you when I blushed,
+and sought an old acquaintance in an unknown eye,
+and an answering blush bloomed on your cheeks
+as from a rose whose breast the dawn has bared.
+You had barely begun your song when I shed tears;
+your voice entered my heart and seized my soul;
+it seemed an angel greeted it by name
+and struck the hour of salvation on heaven’s clock.
+O beloved! let your eyes not be afraid to confess
+if my glance, if my voice, moves you;
+I do not care that fate and people stand against us,
+that I must flee, and love without hope.
+Let an earthly marriage give your hand to another;
+only confess that God has wedded your soul to mine.</t>
+        </is>
+      </c>
       <c r="H146" s="13" t="inlineStr">
         <is>
           <t>Adam Mickiewicz</t>
@@ -20861,7 +21466,8 @@
       </c>
       <c r="W146" s="13" t="inlineStr">
         <is>
-          <t>Polish original in historical spelling. The poet was born in present-day Belarus; this row follows his Polish literary identity. Modern translations are separate.</t>
+          <t>Polish original in historical spelling. The poet was born in present-day Belarus; this row follows his Polish literary identity. Modern translations are separate.
+Passage update (29 October 2026): Complete sonnet, 14 lines, in the spelling of the 1826 edition. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X146" s="13" t="inlineStr">
@@ -21083,8 +21689,30 @@
           <t>O you who shot me, whose arrow struck my heart (first-line sense; source reading uncertain)</t>
         </is>
       </c>
-      <c r="F148" s="13" t="n"/>
-      <c r="G148" s="13" t="n"/>
+      <c r="F148" s="13" t="inlineStr">
+        <is>
+          <t>يامن رماني أو صاب احشاي نشابه
+يذكر حبيب سعى بالشين لاحبابه
+سليت لي من جفونك مرهف صارم
+لا واعذابي عن الصارم وجذابه
+ظنية بك يا عديل الروح ظن ولا
+حققت ظني سوى بالهجر واكذابه
+ونيت من هجركم ونت غريق هوى
+فى غية لايري برا ولا اخشابه</t>
+        </is>
+      </c>
+      <c r="G148" s="13" t="inlineStr">
+        <is>
+          <t>O you who shot me, whose arrow struck my heart,
+it brings to mind a beloved who brought harm on those who loved him.
+From your eyelids you drew on me a keen, sharp sword:
+ah, my torment from that sword and its pull!
+I thought well of you, O twin of my soul, but you
+fulfilled my hopes only with desertion and its lies.
+I moaned at your desertion, drowned in love,
+in a depth where neither shore nor ship’s timbers can be seen.</t>
+        </is>
+      </c>
       <c r="H148" s="13" t="inlineStr">
         <is>
           <t>Majid ibn Salih al-Khulaifi (1873–1907)</t>
@@ -21154,7 +21782,8 @@
       </c>
       <c r="W148" s="13" t="inlineStr">
         <is>
-          <t>The incipit is the identifier, not a verified authorial title. Source typography/OCR needs checking against the 1963 diwan. The 1995 criticism has separate rights.</t>
+          <t>The incipit is the identifier, not a verified authorial title. Source typography/OCR needs checking against the 1963 diwan. The 1995 criticism has separate rights.
+Passage update (29 October 2026): Four couplets (8 half-lines) of Nabati verse, as printed in Nizwa magazine. The reading of the last couplet is uncertain, and the English there is tentative. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X148" s="13" t="inlineStr">
@@ -22287,8 +22916,46 @@
           <t>Evenings in São Tomé</t>
         </is>
       </c>
-      <c r="F157" s="13" t="n"/>
-      <c r="G157" s="13" t="n"/>
+      <c r="F157" s="13" t="inlineStr">
+        <is>
+          <t>Meus olhos são como a noite
+em que astro nenhum flutua
+mas se o teu olhar o fita
+na noite desponta a lua
+Se os escravos são comprados
+ó branca de além do mar
+homem livre eu, sou escravo
+comprado por teu olhar
+Meu olhar é retratista
+ò minha doce miragem
+senão diz-me porque tenho
+no meu peito a tua imagem
+Roubei-te o primeiro beijo
+o segundo foi-me dado
+o terceiro, francamente,
+creio que me foi roubado</t>
+        </is>
+      </c>
+      <c r="G157" s="13" t="inlineStr">
+        <is>
+          <t>My eyes are like the night
+in which no star is floating,
+but if your gaze rests on them,
+the moon rises in that night.
+If slaves are bought,
+O white woman from over the sea,
+I, a free man, am a slave
+bought by your gaze.
+My gaze is a portrait painter,
+O my sweet mirage;
+otherwise tell me why I carry
+your image in my breast.
+I stole the first kiss from you,
+the second was given to me,
+the third, frankly,
+I believe was stolen from me.</t>
+        </is>
+      </c>
       <c r="H157" s="13" t="inlineStr">
         <is>
           <t>Caetano da Costa Alegre (1864–1890)</t>
@@ -22360,7 +23027,8 @@
       </c>
       <c r="W157" s="13" t="inlineStr">
         <is>
-          <t>The text contains racial comparisons requiring contextual reading. Modern commentary is separate. Composition date is not known; 1916 is the collection date.</t>
+          <t>The text contains racial comparisons requiring contextual reading. Modern commentary is separate. Composition date is not known; 1916 is the collection date.
+Passage update (29 October 2026): First four quatrains, 16 lines. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X157" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Add batch 4 of new poem passages (13 countries)
Serbia, Somalia, South Africa, South Korea, Syria, Tajikistan, Trinidad
and Tobago, Tunisia, Turkiye, Uzbekistan, Venezuela, Vietnam and Yemen
now show a passage in the original beside English (South Africa and
Trinidad in their authors' English), each with a history note.
107 poems to read in total.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 94 paired passages • 101 unfilled</t>
+          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 107 paired passages • 88 unfilled</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -23362,8 +23362,62 @@
           <t>Saint Mary of Health (the Venice church's name)</t>
         </is>
       </c>
-      <c r="F160" s="13" t="n"/>
-      <c r="G160" s="13" t="n"/>
+      <c r="F160" s="13" t="inlineStr">
+        <is>
+          <t>А наша деца песме су моје,
+тих састанака вечити траг;
+то се не пише, то се не поје,
+само што душом пробије зрак.
+То разумемо само нас двоје,
+то је у рају приновак драг,
+то тек у заносу пророци слуте,
+Santa Maria della Salute.
+А кад ми дође да прсне глава
+о тог живота хридовит крај,
+најлепши сан ми постаће јава,
+мој ропац њено: „Ево ме, нај!”
+Из ништавила у славу слава,
+из безњенице у рај, у рај!
+У рај, у рај, у њезин загрљај!
+Све ће се жеље ту да пробуде,
+душине жице све да прогуде,
+задивићемо светске колуте,
+богове силне, камо ли људе,
+звездама ћемо померит’ путе,
+сунцима засут’ сељенске студе,
+да у све куте зоре заруде,
+да од милине дуси полуде,
+Santa Maria della Salute.</t>
+        </is>
+      </c>
+      <c r="G160" s="13" t="inlineStr">
+        <is>
+          <t>And our children are my poems,
+the everlasting trace of those meetings;
+it cannot be written, it cannot be sung,
+only a ray breaks through the soul.
+Only the two of us understand it;
+in paradise it is a dear new arrival;
+only prophets in rapture can sense it,
+Santa Maria della Salute.
+And when my head comes to shatter
+against the rocky shore of this life,
+my loveliest dream will come true,
+and my death rattle will be her “Here I am, my dearest!”
+From nothingness into the glory of glories,
+from a life without her into paradise, paradise!
+Into paradise, paradise, into her embrace!
+There every desire will awaken,
+all the strings of the soul will ring out,
+we will astonish the circling worlds,
+the mighty gods, let alone mortals,
+we will shift the paths of the stars,
+shower the cold of the universe with suns,
+so that dawns blush in every corner,
+so that spirits go mad with delight,
+Santa Maria della Salute.</t>
+        </is>
+      </c>
       <c r="H160" s="13" t="inlineStr">
         <is>
           <t>Laza Kostić</t>
@@ -23435,7 +23489,8 @@
       </c>
       <c r="W160" s="13" t="inlineStr">
         <is>
-          <t>Source explicitly marks original public domain in Serbia, USA and life-plus-70 countries; author died 1910. Religious imagery frames passionate personal love. Modern critical material and translations excluded. The selection is the original-language text; an existing English translation is not required.</t>
+          <t>Source explicitly marks original public domain in Serbia, USA and life-plus-70 countries; author died 1910. Religious imagery frames passionate personal love. Modern critical material and translations excluded. The selection is the original-language text; an existing English translation is not required.
+Passage update (29 October 2026): Final two stanzas, 24 lines, on the lovers’ reunion; the refrain is the Venetian church’s name. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X160" s="13" t="inlineStr">
@@ -24280,8 +24335,24 @@
           <t>Love of women was ordained long ago by the Just One (first line)</t>
         </is>
       </c>
-      <c r="F167" s="13" t="n"/>
-      <c r="G167" s="13" t="n"/>
+      <c r="F167" s="13" t="inlineStr">
+        <is>
+          <t>Caashaqa haween waa horuu, Caaddil soo rogaye,
+Sayidkii carshiga nuurayiyo, Caliba soo gaadhye,
+Cidla lagama beermeen dadkoo, cuudi waahhidahe,
+Wahha caynba cayn looga dhigay, hays cajebiyeene,
+Soomaalidaa caado hhune, iguma caydeene.</t>
+        </is>
+      </c>
+      <c r="G167" s="13" t="inlineStr">
+        <is>
+          <t>Love for women was ordained long ago by the Just One;
+it touched even the Prophet of the shining Throne, and Ali too.
+People did not grow out of emptiness; they come from one root,
+and each kind was made unlike the next, so let them not marvel at one another.
+It is the Somalis whose custom is cruel; let them not mock me.</t>
+        </is>
+      </c>
       <c r="H167" s="13" t="inlineStr">
         <is>
           <t>Cilmi Boodhari / Ilmi Bowndheri (c.1908–1941)</t>
@@ -24353,7 +24424,8 @@
       </c>
       <c r="W167" s="13" t="inlineStr">
         <is>
-          <t>The assessed reuse lead is the historical Somali wording, not the 1967 English translation, modern bilingual edition, musical setting or performance. Versions differ. The repository’s CC BY-NC-ND label is restrictive and is not treated as permission to translate or commercially reuse modern editorial material. Berbera is in Somaliland, within the workbook’s Somalia country grouping.</t>
+          <t>The assessed reuse lead is the historical Somali wording, not the 1967 English translation, modern bilingual edition, musical setting or performance. Versions differ. The repository’s CC BY-NC-ND label is restrictive and is not treated as permission to translate or commercially reuse modern editorial material. Berbera is in Somaliland, within the workbook’s Somalia country grouping.
+Passage update (29 October 2026): The five-line excerpt printed in Galaal’s collection, p. 31, in its older Somali spelling. The English is a careful draft. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X167" s="13" t="inlineStr">
@@ -24419,8 +24491,36 @@
           <t>The Story of an African Farm</t>
         </is>
       </c>
-      <c r="F168" s="13" t="n"/>
-      <c r="G168" s="13" t="n"/>
+      <c r="F168" s="13" t="inlineStr">
+        <is>
+          <t>“But I’m sure you must be cold,” said Gregory, and put his hand under the cloak, and found there a small fist doubled up, soft, and very warm.
+He held it fast in his hand.
+“Oh, Em, I love you better than all the world besides! Tell me, do you love me a little?”
+“Yes, I do,” said Em, hesitating, and trying softly to free her hand.
+“Better than everything; better than all the world, darling?” he asked, bending down so low that the yellow hair was blown into his eyes.
+“I don’t know,” said Em, gravely. “I do love you very much; but I love my cousin who is at school, and Waldo, very much. You see I have known them so long!”
+“Oh, Em, do not talk to me so coldly!” Gregory cried, seizing the little arm that rested on the gate, and pressing it till she was half afraid.
+The herdsman had moved away to the other end of the kraal now, and the cows, busy with their calves, took no notice of the little human farce.
+“Em, if you talk so to me I will go mad! You must love me, love me better than all! You must give yourself to me. I have loved you since that first moment when I saw you walking by the stone wall with the jug in your hands. You were made for me, created for me! I will love you till I die! Oh, Em, do not be so cold, so cruel to me!”
+He held her arm so tightly that her fingers relaxed their hold, and the cloak fluttered down on to the ground, and the wind played more roughly than ever with the little yellow head.
+“I do love you very much,” she said; “but I do not know if I want to marry you. I love you better than Waldo, but I can’t tell if I love you better than Lyndall. If you would let me wait for a week I think perhaps I could tell you.”</t>
+        </is>
+      </c>
+      <c r="G168" s="13" t="inlineStr">
+        <is>
+          <t>“But I’m sure you must be cold,” said Gregory, and put his hand under the cloak, and found there a small fist doubled up, soft, and very warm.
+He held it fast in his hand.
+“Oh, Em, I love you better than all the world besides! Tell me, do you love me a little?”
+“Yes, I do,” said Em, hesitating, and trying softly to free her hand.
+“Better than everything; better than all the world, darling?” he asked, bending down so low that the yellow hair was blown into his eyes.
+“I don’t know,” said Em, gravely. “I do love you very much; but I love my cousin who is at school, and Waldo, very much. You see I have known them so long!”
+“Oh, Em, do not talk to me so coldly!” Gregory cried, seizing the little arm that rested on the gate, and pressing it till she was half afraid.
+The herdsman had moved away to the other end of the kraal now, and the cows, busy with their calves, took no notice of the little human farce.
+“Em, if you talk so to me I will go mad! You must love me, love me better than all! You must give yourself to me. I have loved you since that first moment when I saw you walking by the stone wall with the jug in your hands. You were made for me, created for me! I will love you till I die! Oh, Em, do not be so cold, so cruel to me!”
+He held her arm so tightly that her fingers relaxed their hold, and the cloak fluttered down on to the ground, and the wind played more roughly than ever with the little yellow head.
+“I do love you very much,” she said; “but I do not know if I want to marry you. I love you better than Waldo, but I can’t tell if I love you better than Lyndall. If you would let me wait for a week I think perhaps I could tell you.”</t>
+        </is>
+      </c>
       <c r="H168" s="13" t="inlineStr">
         <is>
           <t>Olive Schreiner (published as Ralph Iron)</t>
@@ -24492,7 +24592,8 @@
       </c>
       <c r="W168" s="13" t="inlineStr">
         <is>
-          <t>Prose novel rather than poem/song. Contains critical and painful relationships, not uniformly positive views. Historical racial language appears in the book. Gutenberg branding/licence separate from underlying novel.</t>
+          <t>Prose novel rather than poem/song. Contains critical and painful relationships, not uniformly positive views. Historical racial language appears in the book. Gutenberg branding/licence separate from underlying novel.
+Passage update (29 October 2026): Eleven consecutive lines (one per paragraph or sentence) from Part II, Gregory’s declaration to Em at the cow-kraal gate. Original English; no translation needed. Original English text; not a translation.</t>
         </is>
       </c>
       <c r="X168" s="13" t="inlineStr">
@@ -24554,8 +24655,22 @@
           <t>A Woman's Chamber Lament, I</t>
         </is>
       </c>
-      <c r="F169" s="13" t="n"/>
-      <c r="G169" s="13" t="n"/>
+      <c r="F169" s="13" t="inlineStr">
+        <is>
+          <t>錦帶羅裙積淚痕
+一年芳草恨王孫
+瑤箏彈盡江南曲
+雨打梨花晝掩門</t>
+        </is>
+      </c>
+      <c r="G169" s="13" t="inlineStr">
+        <is>
+          <t>On my brocade sash and silk skirt the tear stains gather;
+all year, among the fragrant grass, I grieve for my absent lord.
+On the jade zither I play through the songs of the south;
+rain beats down the pear blossom, and in daylight I shut my gate.</t>
+        </is>
+      </c>
       <c r="H169" s="13" t="inlineStr">
         <is>
           <t>Heo Nanseolheon</t>
@@ -24625,7 +24740,8 @@
       </c>
       <c r="W169" s="13" t="inlineStr">
         <is>
-          <t>Gangneung-associated Joseon poet, in present-day South Korea; shared Korean heritage. The linked Korean translations are separate works and are not cleared by the ancient original’s status.</t>
+          <t>Gangneung-associated Joseon poet, in present-day South Korea; shared Korean heritage. The linked Korean translations are separate works and are not cleared by the ancient original’s status.
+Passage update (29 October 2026): Complete poem, 4 lines: the classical Chinese original only, as the spreadsheet asks (the Korean translations on the page are excluded). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X169" s="13" t="inlineStr">
@@ -25635,8 +25751,46 @@
           <t>I see you resisting tears (first line)</t>
         </is>
       </c>
-      <c r="F177" s="13" t="n"/>
-      <c r="G177" s="13" t="n"/>
+      <c r="F177" s="13" t="inlineStr">
+        <is>
+          <t>أرَاكَ عَصِيَّ الدَّمْعِ شِيمَتُكَ الصَّبْرُ
+أمَا لِلْهَوَى نَهْيٌ عَلَيْكَ وَلا أمْر
+بَلَى أنَا مُشْتَاقٌ وَعِنْدِي لَوْعَةٌ
+وَلَكِنَّ مِثْلِي لا يُذَاعُ لَهُ سِرُّ
+إذَا اللَّيْلُ أضْوَانِي بَسَطتُ يَدَ الهَوَى
+وَأذْلَلْتُ دَمْعًا مِنْ خَلائِقِهِ الْكِبْرُ
+تَكَادُ تُضِيءُ النَّارُ بَيْنَ جَوَانِحِي
+إذَا هِيَ أذْكَتْهَا الصَّبَابَةُ وَالْفِكْرُ
+مُعَلِّلَتِي بالْوَصْلِ وَالموت دُونَهُ
+إذَا مِتُّ ظَمْآنًا فَلا نَزَلَ الْقَطْرُ
+حَفِظْتُ وَضَيَّعْتِ الموَدَّةَ بَيْنَنَا
+وَأحْسَنُ مِنْ بَعْضِ الْوَفَاءِ لَكِ الْعُذْرُ
+وَمَا هَذِهِ الأيَّامُ إلا صَحَائِفُ
+لأحْرُفِهَا مِنْ كَفِّ كَاتِبِهَا بِشْرُ
+بِنَفْسِي مِنَ الْغَادِينَ في الحيِّ غَادَةٌ
+هَوَايَ لَهَا ذَنْبٌ وَبَهْجَتُهَا عُذْرُ</t>
+        </is>
+      </c>
+      <c r="G177" s="13" t="inlineStr">
+        <is>
+          <t>I see you dry-eyed; patience is your nature:
+has love no command or forbidding over you?
+Yes, I am full of longing, and I burn,
+but a man like me does not let his secret be told.
+When night enfolds me, I stretch out the hand of love
+and humble tears whose nature is pride.
+The fire between my ribs almost blazes into light
+when longing and brooding fan it.
+You put me off with promises of union, but death stands before it:
+if I die of thirst, may no rain ever fall.
+I kept faith, and you squandered the love between us;
+but making excuses for you suits me better than some kinds of loyalty.
+These days are nothing but pages
+whose letters glow with the hand of the one who writes them.
+My life for one young woman among those leaving the camp at dawn:
+my love for her is a sin, and her beauty its excuse.</t>
+        </is>
+      </c>
       <c r="H177" s="13" t="inlineStr">
         <is>
           <t>Abu Firas al-Hamdani</t>
@@ -25706,7 +25860,8 @@
       </c>
       <c r="W177" s="13" t="inlineStr">
         <is>
-          <t>Classical Syrian/Hamdanid literary association; the poet predates modern national borders. Medieval original only, excluding later musical settings, recordings and translations. Wikisource print provenance is incomplete; compare a scholarly edition. The selection is the original-language text; an existing English translation is not required.</t>
+          <t>Classical Syrian/Hamdanid literary association; the poet predates modern national borders. Medieval original only, excluding later musical settings, recordings and translations. Wikisource print provenance is incomplete; compare a scholarly edition. The selection is the original-language text; an existing English translation is not required.
+Passage update (29 October 2026): Opening love dialogue, 8 couplets (16 half-lines), before the poem turns to martial self-praise. Arabic Wikisource text; decorative letter-stretching removed. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X177" s="13" t="inlineStr">
@@ -25768,8 +25923,22 @@
           <t>Without your face, may the world-burning sun not shine (first line; quatrain8)</t>
         </is>
       </c>
-      <c r="F178" s="13" t="n"/>
-      <c r="G178" s="13" t="n"/>
+      <c r="F178" s="13" t="inlineStr">
+        <is>
+          <t>بی روی تو خورشید جهان‌سوز مباد
+هم بی تو چراغ عالم‌افروز مباد
+با وصل تو کس چو من بد آموز مباد
+روزی که تو را نبینم آن روز مباد</t>
+        </is>
+      </c>
+      <c r="G178" s="13" t="inlineStr">
+        <is>
+          <t>Without your face, may the world-burning sun not shine;
+without you, may no lamp light up the world;
+may no one grow as used to your company as I have;
+and may the day I do not see you never come.</t>
+        </is>
+      </c>
       <c r="H178" s="13" t="inlineStr">
         <is>
           <t>Attributed to Rudaki</t>
@@ -25839,7 +26008,8 @@
       </c>
       <c r="W178" s="13" t="inlineStr">
         <is>
-          <t>Rudaki died c. 941 and is associated with Panjrud in present-day Tajikistan. Attribution of individual surviving verses can be uncertain; Ganjoor’s numbering is not a historical title. Use the classical Persian lines, excluding modern AI summaries, recitations and comments. The selection is the original-language text; an existing English translation is not required.</t>
+          <t>Rudaki died c. 941 and is associated with Panjrud in present-day Tajikistan. Attribution of individual surviving verses can be uncertain; Ganjoor’s numbering is not a historical title. Use the classical Persian lines, excluding modern AI summaries, recitations and comments. The selection is the original-language text; an existing English translation is not required.
+Passage update (29 October 2026): Complete quatrain, 4 lines (Ganjoor, Rudaki’s rubāʿīs no. 8). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X178" s="13" t="inlineStr">
@@ -26530,8 +26700,34 @@
           <t>Emmanuel Appadocca; or, Blighted Life — Lorenzo and Agnes episode</t>
         </is>
       </c>
-      <c r="F184" s="13" t="n"/>
-      <c r="G184" s="13" t="n"/>
+      <c r="F184" s="13" t="inlineStr">
+        <is>
+          <t>She hastily and eagerly glanced over it, raised her head for a time, and then read, and read, and read again.
+The letter was this:—
+“Lady, though I am a pirate, recoil not from me.
+I am sensible to the feelings of honor, and need not be feared by any lady;
+in the uprightness of my soul I have dared to love you;
+deign to cast but one look on me, and let me believe I may hope.
+Lorenzo.”
+Agnes read this over and over again in nervous trepidation, then folded it, and put it by.
+She was a victim to strong contending emotions.
+She felt she knew not what for Lorenzo, but he was a pirate.</t>
+        </is>
+      </c>
+      <c r="G184" s="13" t="inlineStr">
+        <is>
+          <t>She hastily and eagerly glanced over it, raised her head for a time, and then read, and read, and read again.
+The letter was this:—
+“Lady, though I am a pirate, recoil not from me.
+I am sensible to the feelings of honor, and need not be feared by any lady;
+in the uprightness of my soul I have dared to love you;
+deign to cast but one look on me, and let me believe I may hope.
+Lorenzo.”
+Agnes read this over and over again in nervous trepidation, then folded it, and put it by.
+She was a victim to strong contending emotions.
+She felt she knew not what for Lorenzo, but he was a pirate.</t>
+        </is>
+      </c>
       <c r="H184" s="13" t="inlineStr">
         <is>
           <t>Michel Maxwell Philip (1829–1888)</t>
@@ -26603,7 +26799,8 @@
       </c>
       <c r="W184" s="13" t="inlineStr">
         <is>
-          <t>Select the actual human love episode; the novel’s connection to Romanticism is not itself evidence of romantic love. Historical language and captivity context need attention.</t>
+          <t>Select the actual human love episode; the novel’s connection to Romanticism is not itself evidence of romantic love. Historical language and captivity context need attention.
+Passage update (29 October 2026): Ten consecutive sentences from Lorenzo’s letter to Agnes and her response (Volume I, original pp. 143–144). Original English; no translation needed. Original English text; not a translation.</t>
         </is>
       </c>
       <c r="X184" s="13" t="inlineStr">
@@ -26669,8 +26866,54 @@
           <t>Prayers in the Temple of Love</t>
         </is>
       </c>
-      <c r="F185" s="13" t="n"/>
-      <c r="G185" s="13" t="n"/>
+      <c r="F185" s="13" t="inlineStr">
+        <is>
+          <t>عذبةٌ أنتِ كالطفولةِ ، كالأحلامِ ،
+كاللحنِ ، كالصباحِ الجديدِ
+كالسماءِ الضحوكِ كالليلةِ القَمْراءِ ،
+كالوردِ ، كابتسامِ الوليدِ
+يا لها من وداعةٍ وجَمالِ
+وشبابٍ مُنَعَّمٍ أُمْلُودِ !
+يا لها من طهارةٍ ، تَبْعَثُ التقْديـ
+ـسَ في مهجةِ الشَّقِيِّ العَنِيدِ ! . . .
+يا لها رقَّةً تكادُ يَرُفُّ الوَرْ
+دُ منها في الصخرةِ الجلمودِ !
+أَيُّ شيءٍ أنتِ ؟! هل أنتِ «فينسُ»
+تهادتْ بين الورَى من جديدِ
+لِتُعِيدَ الشبابَ والفرحَ للمَغْـ
+ـمُومِ لِلعالَمِ التعيسِ العَمِيدِ !
+أم مَلاكُ الفردوسِ جاء إلى الأرْ
+ضِ لِيُحْيِيَ روحَ السلامِ العَهِيدِ !
+أنتِ . . . ، ما أنتِ ؟ رسمٌ جميلٌ
+عبقريٌّ من فنِّ هذا الوجودِ
+فيكِ ما فيه من غموضٍ وعُمْقٍ
+وجمالٍ مُقَدَّسٍ معبودِ</t>
+        </is>
+      </c>
+      <c r="G185" s="13" t="inlineStr">
+        <is>
+          <t>You are sweet as childhood, as dreams,
+as a melody, as a new morning,
+as the laughing sky, as the moonlit night,
+as the rose, as a newborn’s smile.
+What gentleness, what beauty,
+what soft and supple youth!
+What purity, that wakes reverence
+even in the heart of the wretched and stubborn!
+What tenderness: roses could almost flutter
+from it even in solid rock!
+What are you? Are you Venus,
+walking once more among humankind
+to bring back youth and joy to the grieving,
+to the miserable, heartsick world?
+Or an angel of paradise come down to earth
+to revive the spirit of a peace long gone?
+You… what are you? A lovely picture,
+a masterpiece of the art of this existence;
+in you is all its mystery and depth
+and its holy, worshipped beauty.</t>
+        </is>
+      </c>
       <c r="H185" s="13" t="inlineStr">
         <is>
           <t>Abu al-Qasim al-Shabbi</t>
@@ -26742,7 +26985,8 @@
       </c>
       <c r="W185" s="13" t="inlineStr">
         <is>
-          <t>Author died 1934. The transcription repeats a passage and lacks precise print-edition provenance; compare a scan before quoting. The original Arabic is public domain in life-plus-70 jurisdictions; modern translations and settings are separate. The selection is the original-language text; an existing English translation is not required.</t>
+          <t>Author died 1934. The transcription repeats a passage and lacks precise print-edition provenance; compare a scan before quoting. The original Arabic is public domain in life-plus-70 jurisdictions; modern translations and settings are separate. The selection is the original-language text; an existing English translation is not required.
+Passage update (29 October 2026): Opening 10 couplets (20 half-lines), Arabic Wikisource text. Words divided across the half-line break are kept as printed. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X185" s="13" t="inlineStr">
@@ -26808,8 +27052,74 @@
           <t>Your Eyes</t>
         </is>
       </c>
-      <c r="F186" s="13" t="n"/>
-      <c r="G186" s="13" t="n"/>
+      <c r="F186" s="13" t="inlineStr">
+        <is>
+          <t>Ծով մը կապույտ կծավալի
+Աչքերուդ մեջ, ուր չըկա սեր,
+Ծով մը հանդարտ, ըզմայլելի,
+Ուր կը ցոլան ցայտուն լույսեր․
+Բայց ըզգացումն հոն կհալի,
+Ինչպես տաքին՝ պատառ մը սեր։
+Երբեմն անկե կանցնին բարակ
+Ճառագայթներ պայծառ ու ջինջ,
+Ջըղուտ հոգվույդ ցոլքեր կըրակ
+Երևույթով մ'աղվոր, անջինջ․
+Բայց կմարին անոնք արագ,
+Ինչպես հովին դեմ կայծ մ'ոչինչ։
+Մերթ ծաղիկներ կըլլան փափուկ
+Գորշ կապույտով մանուշակին,
+Այնքան նըրբին և խուսափուկ,
+Որ չունին գույն որոշակի․
+Բայց կթափին ինչպես հափուկ
+Դաժան շունչին դեմ խորշակի։
+Օր մ'ալ տեսնես շատ են հոգներ
+Մեծ թախծի խոհով մ'անանց․
+Արցունքներու տակ կայլակներ
+Թարթիչներեդ կմաղվին թաց,
+Որ կթըվին սև ժանյակներ
+Գոհարներու շարքով բանված։
+Աշխարհներ են աչքերդ անհուն,
+Ուր կան լույսեր, հույզեր հըսկա․
+Սառույց, հըրդեհ, բոցեր փայլուն,
+Ժըպիտն ու հույս չեն բացակա․
+Կուգան, կանցնին անկե սահուն
+Գութն ու արցունք, լոկ սեր չըկա։</t>
+        </is>
+      </c>
+      <c r="G186" s="13" t="inlineStr">
+        <is>
+          <t>A blue sea spreads
+within your eyes, where there is no love,
+a calm sea, enchanting,
+where bright lights glitter;
+but feeling melts away there
+like a scrap of cream in the heat.
+Sometimes slender rays pass across it,
+bright and clear,
+flashes of fire from your nervous soul,
+lovely and unforgettable to see;
+but they go out quickly,
+like a feeble spark against the wind.
+At times they become soft flowers
+with the grey-blue of the violet,
+so delicate and elusive
+that they have no definite colour;
+but they scatter like petals
+before the cruel breath of the scorching wind.
+Another day you see them weary
+with the endless thought of a great sadness;
+under the tears, drops
+sift wet through your lashes,
+so that they look like black lace
+worked with a row of jewels.
+Your eyes are boundless worlds,
+with lights and vast emotions in them;
+ice, conflagration, shining flames,
+smiles and hope are not absent;
+pity and tears come and pass through them smoothly:
+only love is not there.</t>
+        </is>
+      </c>
       <c r="H186" s="13" t="inlineStr">
         <is>
           <t>Sibil (Zabel Asadour)</t>
@@ -26881,7 +27191,8 @@
       </c>
       <c r="W186" s="13" t="inlineStr">
         <is>
-          <t>Country is geographic: an Ottoman Armenian writer born and active in Istanbul, now Turkey; this is Armenian-language literature, not a claim of ethnic Turkish identity. 1965 editorial material and modern translations are separate.</t>
+          <t>Country is geographic: an Ottoman Armenian writer born and active in Istanbul, now Turkey; this is Armenian-language literature, not a claim of ethnic Turkish identity. 1965 editorial material and modern translations are separate.
+Passage update (29 October 2026): Complete poem, 30 lines (Armenian Wikisource; dated 1892). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X186" s="13" t="inlineStr">
@@ -28039,8 +28350,42 @@
           <t>A person without love is not truly human (first line)</t>
         </is>
       </c>
-      <c r="F195" s="13" t="n"/>
-      <c r="G195" s="13" t="n"/>
+      <c r="F195" s="13" t="inlineStr">
+        <is>
+          <t>Na gul sayr ayla, na fikri bahor et,
+Jahondin kech, xayoli vasli yor et.
+Muhabbatsiz kishi odam emasdur,
+Gar odamsan, muhabbat ixtiyor et.
+Uzoru qaddu raftoringni koʻrsat,
+Chaman sarvu gulini sharmisor et.
+Labi maxmurdadurmen, jomi may tut,
+Karam qil, soqiyo, daf’i humor et.
+«Analhaq» mojarosin aylading fosh,
+kel, ey Mansur, istiqboli dor et.
+Duru ashku aqiqi xuni dilni
+Kelu yoring ayogʻigʻa nisor et.
+Kuyib, ey Nodira, olam eligʻa
+Muhabbat shevasini oshkor et.</t>
+        </is>
+      </c>
+      <c r="G195" s="13" t="inlineStr">
+        <is>
+          <t>Do not stroll among the roses, do not think of spring:
+give up the world, and dream of union with your beloved.
+A person without love is not truly human:
+if you are human, choose love.
+Show your cheek, your stature and your walk,
+and put the garden’s cypress and rose to shame.
+My lips are parched with longing; hand me the cup of wine;
+be generous, cupbearer, and ease my aching head.
+You made public the secret of “I am the Truth”:
+come, O Mansur, go out to meet the gallows.
+The pearls of your tears, the carnelian of your heart’s blood:
+come, and scatter them at your beloved’s feet.
+Burning, O Nodira, before the people of the world,
+reveal the ways of love.</t>
+        </is>
+      </c>
       <c r="H195" s="13" t="inlineStr">
         <is>
           <t>Nodira (Mohlaroyim)</t>
@@ -28110,7 +28455,8 @@
       </c>
       <c r="W195" s="13" t="inlineStr">
         <is>
-          <t>Nodira was a Kokand poet in present-day Uzbekistan. Erotic and Sufi readings can overlap. Latin-script transcription is modern; no English translation is cleared.</t>
+          <t>Nodira was a Kokand poet in present-day Uzbekistan. Erotic and Sufi readings can overlap. Latin-script transcription is modern; no English translation is cleared.
+Passage update (29 October 2026): Complete ghazal, 7 couplets (14 lines), in modern Uzbek Latin script. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X195" s="13" t="inlineStr">
@@ -28303,8 +28649,50 @@
           <t>Love and Misfortune</t>
         </is>
       </c>
-      <c r="F197" s="13" t="n"/>
-      <c r="G197" s="13" t="n"/>
+      <c r="F197" s="13" t="inlineStr">
+        <is>
+          <t>Solitaria, sin ventura,
+Fija en la onda la mirada,
+Llena el alma de amargura,
+Desgarrado el corazón,
+Virgen triste, abandonada
+Pide á Dios consolación.
+Aun divisa en lontananza
+Del bajel la blanca estela ;
+Imagina su esperanza
+Que á su amante abraza ya;
+Si columbra alguna vela,
+Hondo grito al aire da.
+Hace un año que la hermosa,
+Que suspira sin consuelo,
+Angustiada, temblorosa,
+Á su amante vio partir;
+Y enlutado vio del cielo
+El purísimo zafir.</t>
+        </is>
+      </c>
+      <c r="G197" s="13" t="inlineStr">
+        <is>
+          <t>Alone, without fortune,
+her gaze fixed on the waves,
+her soul full of bitterness,
+her heart torn apart,
+a sad, abandoned maiden
+begs God for consolation.
+In the distance she can still make out
+the white wake of the ship;
+in her hope she imagines
+that she already holds her lover;
+if she glimpses a sail,
+she sends a deep cry into the air.
+It is a year since the lovely one,
+who sighs without comfort,
+anguished and trembling,
+watched her lover depart,
+and saw the purest sapphire
+of the sky dressed in mourning.</t>
+        </is>
+      </c>
       <c r="H197" s="13" t="inlineStr">
         <is>
           <t>Abigaíl Lozano</t>
@@ -28376,7 +28764,8 @@
       </c>
       <c r="W197" s="13" t="inlineStr">
         <is>
-          <t>Abigaíl Lozano was a man. Historical Spanish spelling and punctuation differ from modern practice. Do not confuse poem page numbers between the anthology and his own collection.</t>
+          <t>Abigaíl Lozano was a man. Historical Spanish spelling and punctuation differ from modern practice. Do not confuse poem page numbers between the anthology and his own collection.
+Passage update (29 October 2026): First three stanzas, 18 lines. Two OCR slips are corrected (“áDios” to “á Dios”, and a stray quotation mark). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X197" s="13" t="inlineStr">
@@ -28438,8 +28827,22 @@
           <t>A Piece of Betel / Offering Betel</t>
         </is>
       </c>
-      <c r="F198" s="13" t="n"/>
-      <c r="G198" s="13" t="n"/>
+      <c r="F198" s="13" t="inlineStr">
+        <is>
+          <t>Quả cau nho nhỏ miếng trầu hôi
+Này của Xuân Huơng đã quệt rồi
+Có phải duyên nhau thì thắm lại
+Đừng xanh như lá bạc như vôi</t>
+        </is>
+      </c>
+      <c r="G198" s="13" t="inlineStr">
+        <is>
+          <t>A tiny areca nut, a humble betel quid:
+here, Xuân Hương has already spread the lime on it.
+If we are fated for each other, let it turn deep red;
+do not stay green as the leaf, or turn pale and faithless as the lime.</t>
+        </is>
+      </c>
       <c r="H198" s="13" t="inlineStr">
         <is>
           <t>Hồ Xuân Hương</t>
@@ -28509,7 +28912,8 @@
       </c>
       <c r="W198" s="13" t="inlineStr">
         <is>
-          <t>Traditional attribution to Hồ Xuân Hương; early print/manuscript provenance not established here. Original poem only; 1993 introduction, editorial matter and modern translations are separate.</t>
+          <t>Traditional attribution to Hồ Xuân Hương; early print/manuscript provenance not established here. Original poem only; 1993 introduction, editorial matter and modern translations are separate.
+Passage update (29 October 2026): Complete poem, 4 lines (modern Vietnamese script; the source keeps the spelling “Huơng”). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X198" s="13" t="inlineStr">
@@ -28567,8 +28971,46 @@
           <t>A gazelle unlike any other in Sana'a (first-line sense)</t>
         </is>
       </c>
-      <c r="F199" s="13" t="n"/>
-      <c r="G199" s="13" t="n"/>
+      <c r="F199" s="13" t="inlineStr">
+        <is>
+          <t>غزال ما مثله بصنعا غزال
+بسيف لحظه قد غزا لي
+أزال ثوب الصبر عني وزال
+وصار تايه في أزال
+سلب على البدر البها والكمال
+وقد سلب روحي كمالي
+وطال بالهجران بعد الوصال
+على فؤاد للنار صالي
+قد خلف المضني معنى وسار
+كالبدر جنح الليل ساري
+ماذا جرى بيني وبينك ودار
+والله بذا عالم وداري
+أقل خطايا مغرمك والعثار
+وخذ من الواشي بثاري
+لا تستمع حاسد بقيل وقال
+ولا تصدق قول قالي</t>
+        </is>
+      </c>
+      <c r="G199" s="13" t="inlineStr">
+        <is>
+          <t>A gazelle like no other gazelle in Sanaa
+has raided me with the sword of his glance.
+He stripped the robe of patience from me and left,
+and now wanders proudly through Azal.
+He robbed the full moon of its splendour and perfection,
+and robbed my soul of all I had.
+After union he has drawn out his desertion
+over a heart that is roasting in the fire.
+He left the lovesick one in torment and went on,
+like the full moon travelling through the night.
+What happened, what passed between us,
+God knows, and is aware of it.
+Forgive your lover his sins and his stumbles,
+and take my revenge on the slanderer.
+Do not listen to the envious, with their gossip,
+and do not believe what a hater says.</t>
+        </is>
+      </c>
       <c r="H199" s="13" t="inlineStr">
         <is>
           <t>Ahmad ibn Abd al-Rahman al-Ansi (أحمد بن عبد الرحمن الآنسي)</t>
@@ -28642,7 +29084,8 @@
       </c>
       <c r="W199" s="13" t="inlineStr">
         <is>
-          <t>Distinguish this poet from later singers and musical arrangements. Modern edited editions and translations have separate rights.</t>
+          <t>Distinguish this poet from later singers and musical arrangements. Modern edited editions and translations have separate rights.
+Passage update (29 October 2026): First 8 couplets (16 half-lines) of the 16-couplet poem, as printed in the Abu Dhabi Poetry Encyclopedia. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X199" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Add five poems from alternative sources: Egypt, Ghana, Iraq, Liberia, Moldova
The original links had no usable text; these come from Arabic and
Romanian Wikisource, adab.wiki and Internet Archive scans of the 1891
and 1911 first editions (OCR tidied, letters checked against the scan).
Source links in the spreadsheet now point to them. 112 poems to read.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 107 paired passages • 88 unfilled</t>
+          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 112 paired passages • 83 unfilled</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -8335,8 +8335,54 @@
           <t>Your lovesick one has been forsaken by sleep (first line)</t>
         </is>
       </c>
-      <c r="F58" s="13" t="n"/>
-      <c r="G58" s="13" t="n"/>
+      <c r="F58" s="13" t="inlineStr">
+        <is>
+          <t>مضناك جفاهُ مرقده
+وبكاه ورحمَ عودُهُ
+حيرانُ القلبِ مُعَذَّبُهُ
+مقروح الجفنِ مسهده
+أودى حرفاً إلا رمقاً
+يُبقيه عليك وتُنْفِدهُ
+يستهوي الورق تاوهه
+ويذيب الصخرَ تنهدهُ
+ويناجي النجمَ ويتعبه
+ويُقيم الليلَ ويُقْعِدهُ
+ويعلم كلَّ مطوقةٍ
+شجناً في الدَّوحِ ترددهُ
+كم مد لطفيكَ من شركٍ
+وتادب لا يتصيدهُ
+فعساك بغُمْضٍ مُسعِفهُ
+ولعلّ خيالك مسعدهُ
+الحسنُ حَلَفْتُ بيُوسُفِهِ
+والسورةِ إنك مفردهُ
+قد وَدَّ جمالك أو قبساً
+حوراءُ الخُلْدِ وأَمْرَدُه</t>
+        </is>
+      </c>
+      <c r="G58" s="13" t="inlineStr">
+        <is>
+          <t>Your lovesick one has been deserted by his bed,
+and those who visit him weep and pity him.
+His heart bewildered and tormented,
+his eyelids sore, kept sleepless,
+he has wasted to a thread, but for a last breath
+that he keeps for you, and you use up.
+His moaning draws the doves to him,
+and his sighing melts the rock.
+He confides in the stars and wears them out;
+he keeps the night standing, and makes it sit.
+He teaches every ring-necked dove
+a sorrow to repeat among the trees.
+How many snares he has laid for your kindness,
+yet, out of good manners, he does not catch it.
+Perhaps you will grant him a moment’s sleep,
+and perhaps your phantom will bring him joy.
+I swear by beauty’s Joseph
+and by his sura, that you are beauty’s only one.
+The houris and the youths of paradise
+have longed for your beauty, or even a spark of it.</t>
+        </is>
+      </c>
       <c r="H58" s="13" t="inlineStr">
         <is>
           <t>Ahmad Shawqi (أحمد شوقي)</t>
@@ -8408,7 +8454,8 @@
       </c>
       <c r="W58" s="13" t="inlineStr">
         <is>
-          <t>Original poem, not the later song arrangement or a modern translation. Digital source edition undated.</t>
+          <t>Original poem, not the later song arrangement or a modern translation. Digital source edition undated.
+Passage update (29 October 2026): First 10 couplets (20 half-lines), from Arabic Wikisource (the originally linked poetry site could not be read). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X58" s="13" t="inlineStr">
@@ -8423,7 +8470,7 @@
       </c>
       <c r="Z58" s="11" t="inlineStr">
         <is>
-          <t>Original text</t>
+          <t>Read original</t>
         </is>
       </c>
       <c r="AA58" s="11" t="inlineStr">
@@ -10293,8 +10340,38 @@
           <t>Ethiopia Unbound: Studies in Race Emancipation</t>
         </is>
       </c>
-      <c r="F72" s="13" t="n"/>
-      <c r="G72" s="13" t="n"/>
+      <c r="F72" s="13" t="inlineStr">
+        <is>
+          <t>“Yes, I know that.
+But this also I do know, that the gods are wont to make use of human instruments in approaching men.
+The Infinite finds expression in the finite, and the ideal is realised in the actual.
+And it has often occurred to me that the child-like hand that shall guide me through life’s labyrinthine ways is the self-same one that I now hold tenderly in my own.”
+She began to understand.
+She made an effort as if she would withdraw her hand.
+She hesitated, and the next moment she surrendered the other also.
+“You will be my teacher, then?” asked Kwamankra, half-persuasively, half-triumphantly.
+“Yes,” she simply answered. “So may the gods of our race help me!”
+As the days passed, the twain grew in that mutual understanding, the true basis of all happy unions.
+Now and again he would tell her of his prospects, which he laughingly said were nil, having inherited little else beyond a clear head and a willing heart for work, with which he hoped they would be able to forge their way in life together;
+to which Mansa would sweetly say that she wished she had a fortune to make things easy, but since she had it not, she would bring him the next best, a loyal heart and true, at which Kwamankra would chide her, and say that was the best of all.</t>
+        </is>
+      </c>
+      <c r="G72" s="13" t="inlineStr">
+        <is>
+          <t>“Yes, I know that.
+But this also I do know, that the gods are wont to make use of human instruments in approaching men.
+The Infinite finds expression in the finite, and the ideal is realised in the actual.
+And it has often occurred to me that the child-like hand that shall guide me through life’s labyrinthine ways is the self-same one that I now hold tenderly in my own.”
+She began to understand.
+She made an effort as if she would withdraw her hand.
+She hesitated, and the next moment she surrendered the other also.
+“You will be my teacher, then?” asked Kwamankra, half-persuasively, half-triumphantly.
+“Yes,” she simply answered. “So may the gods of our race help me!”
+As the days passed, the twain grew in that mutual understanding, the true basis of all happy unions.
+Now and again he would tell her of his prospects, which he laughingly said were nil, having inherited little else beyond a clear head and a willing heart for work, with which he hoped they would be able to forge their way in life together;
+to which Mansa would sweetly say that she wished she had a fortune to make things easy, but since she had it not, she would bring him the next best, a loyal heart and true, at which Kwamankra would chide her, and say that was the best of all.</t>
+        </is>
+      </c>
       <c r="H72" s="13" t="inlineStr">
         <is>
           <t>J. E. Casely Hayford (1866–1930)</t>
@@ -10366,7 +10443,8 @@
       </c>
       <c r="W72" s="13" t="inlineStr">
         <is>
-          <t>This is a Ghanaian/Gold Coast work despite Ethiopia in the title. Do not substitute the separately copyrighted 1969 or 2024 editorial introductions. Full original passage not transcribed here.</t>
+          <t>This is a Ghanaian/Gold Coast work despite Ethiopia in the title. Do not substitute the separately copyrighted 1969 or 2024 editorial introductions. Full original passage not transcribed here.
+Passage update (29 October 2026): Twelve consecutive lines from Chapter III, “Love and Life”: Kwamankra’s proposal to Mansa (1911 first edition, Internet Archive scan, pp. 34–35). OCR spacing and line-break hyphens tidied; the letters were checked against the scan text. Original English; no translation needed. Original English text; not a translation.</t>
         </is>
       </c>
       <c r="X72" s="13" t="inlineStr">
@@ -10381,7 +10459,7 @@
       </c>
       <c r="Z72" s="11" t="inlineStr">
         <is>
-          <t>Work catalogue / preview</t>
+          <t>Read original</t>
         </is>
       </c>
       <c r="AA72" s="11" t="inlineStr">
@@ -12684,8 +12762,34 @@
           <t>Layla smiled at me from her balcony (first line)</t>
         </is>
       </c>
-      <c r="F87" s="13" t="n"/>
-      <c r="G87" s="13" t="n"/>
+      <c r="F87" s="13" t="inlineStr">
+        <is>
+          <t>تَبَسَّمت ليَ لَيلى فَوقَ شرفتها
+كَما تَبَسَّمَ في أَفنانِه الزَهَرُ
+لَقَد كلفت بها سَمراء فاتنة
+في جيدها تلع في عينها حَوَرُ
+قَدٌّ كَما شاءَت الأهواء معتدلٌ
+ما شانه زارياً طولٌ وَلا قِصَرُ
+إذا مَشَت تَتَثنّى عند مشيتها
+كَما تَمايل غُصنٌ ناعم غضر
+لَيلى لأَنتِ منَى نفسي وَحاجتها
+وأنتَ وحدك يا لَيلى لها الوطر</t>
+        </is>
+      </c>
+      <c r="G87" s="13" t="inlineStr">
+        <is>
+          <t>Layla smiled at me from her balcony,
+as blossom smiles among its branches.
+I have fallen for her, a bewitching dark beauty,
+with a long, graceful neck and eyes of deep contrast.
+Her figure is just as desire would wish it,
+marred by neither too much height nor too little.
+When she walks, she sways as she goes,
+like a soft, fresh branch bending.
+Layla, you are my soul’s wish and its need,
+and you alone, Layla, are its desire.</t>
+        </is>
+      </c>
       <c r="H87" s="13" t="inlineStr">
         <is>
           <t>Jamil Sidqi al-Zahawi (جميل صدقي الزهاوي)</t>
@@ -12755,7 +12859,8 @@
       </c>
       <c r="W87" s="13" t="inlineStr">
         <is>
-          <t>Opening words are the identifier. Date is bounded by author’s death, not an asserted year of composition. No translation supplied.</t>
+          <t>Opening words are the identifier. Date is bounded by author’s death, not an asserted year of composition. No translation supplied.
+Passage update (29 October 2026): Complete poem, 5 couplets (10 half-lines), from adab.wiki (the originally linked poetry site could not be read). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X87" s="13" t="inlineStr">
@@ -12770,7 +12875,7 @@
       </c>
       <c r="Z87" s="11" t="inlineStr">
         <is>
-          <t>Original text</t>
+          <t>Read original</t>
         </is>
       </c>
       <c r="AA87" s="11" t="inlineStr">
@@ -15119,8 +15224,32 @@
           <t>Guanya Pau: A Story of an African Princess</t>
         </is>
       </c>
-      <c r="F103" s="13" t="n"/>
-      <c r="G103" s="13" t="n"/>
+      <c r="F103" s="13" t="inlineStr">
+        <is>
+          <t>“Well, when this had gone on over two years, one evening about twilight, when I had finished my work, I went and sat under the cola-tree behind our house and pretended to be stringing my beads;
+But my true object was soon realized.
+Momo soon joined me and sat down by my side.
+Who can picture our feelings as that evening we sat beneath the shadows of that stately cola, in the clear moonlight?
+We sat side by side on the green grass, talking little nothings.
+By and by he took a long breath, somehow I felt anxious just because of that sigh.
+He then took both my hands in his, sending a thrill clean through me.
+Planting his frank, honest eyes on mine which soon were directed to the ground, he said: ‘Guanya Pau, nah Edear (I love you); ya in dear wah?’ (Do you love me?)
+What could I say but to whisper faintly: ‘Da keker’ (with all my heart).</t>
+        </is>
+      </c>
+      <c r="G103" s="13" t="inlineStr">
+        <is>
+          <t>“Well, when this had gone on over two years, one evening about twilight, when I had finished my work, I went and sat under the cola-tree behind our house and pretended to be stringing my beads;
+But my true object was soon realized.
+Momo soon joined me and sat down by my side.
+Who can picture our feelings as that evening we sat beneath the shadows of that stately cola, in the clear moonlight?
+We sat side by side on the green grass, talking little nothings.
+By and by he took a long breath, somehow I felt anxious just because of that sigh.
+He then took both my hands in his, sending a thrill clean through me.
+Planting his frank, honest eyes on mine which soon were directed to the ground, he said: ‘Guanya Pau, nah Edear (I love you); ya in dear wah?’ (Do you love me?)
+What could I say but to whisper faintly: ‘Da keker’ (with all my heart).</t>
+        </is>
+      </c>
       <c r="H103" s="13" t="inlineStr">
         <is>
           <t>Joseph Jeffrey Walters (c.1860s–1894)</t>
@@ -15192,7 +15321,8 @@
       </c>
       <c r="W103" s="13" t="inlineStr">
         <is>
-          <t>Use the 1891 novel. Modern Broadview introduction and annotations are excluded. The work combines opposition to forced marriage with a nineteenth-century Christian missionary perspective.</t>
+          <t>Use the 1891 novel. Modern Broadview introduction and annotations are excluded. The work combines opposition to forced marriage with a nineteenth-century Christian missionary perspective.
+Passage update (29 October 2026): Nine consecutive sentences in which Guanya Pau tells how Momo declared his love (1891 edition, Internet Archive scan, pp. 128–129), including his words in Vai. OCR spacing and line-break hyphens tidied; the letters were checked against the scan text. Original English; no translation needed. Original English text; not a translation.</t>
         </is>
       </c>
       <c r="X103" s="13" t="inlineStr">
@@ -15207,7 +15337,7 @@
       </c>
       <c r="Z103" s="11" t="inlineStr">
         <is>
-          <t>Work / source text</t>
+          <t>Read original</t>
         </is>
       </c>
       <c r="AA103" s="11" t="inlineStr">
@@ -17255,8 +17385,70 @@
           <t>The Evening Star</t>
         </is>
       </c>
-      <c r="F119" s="13" t="n"/>
-      <c r="G119" s="13" t="n"/>
+      <c r="F119" s="13" t="inlineStr">
+        <is>
+          <t>A fost odată ca-n povești,
+A fost ca niciodată,
+Din rude mari împărătești,
+O prea frumoasă fată.
+Și era una la părinți
+Și mândră-n toate cele,
+Cum e Fecioara între sfinți
+Și luna între stele.
+Din umbra falnicelor bolți
+Ea pasul și-l îndreaptă
+Lângă fereastră, unde-n colț
+Luceafărul așteaptă.
+Privea în zare cum pe mări
+Răsare și străluce,
+Pe mișcătoarele cărări
+Corăbii negre duce.
+Îl vede azi, îl vede mâni,
+Astfel dorința-i gata;
+El iar, privind de săptămâni,
+Îi cade dragă fata.
+Cum ea pe coate-și răzima
+Visând ale ei tâmple
+De dorul lui și inima
+Și sufletu-i se împle.
+Și cât de viu s-aprinde el
+În orișicare sară,
+Spre umbra negrului castel
+Când ea o să-i apară.</t>
+        </is>
+      </c>
+      <c r="G119" s="13" t="inlineStr">
+        <is>
+          <t>Once upon a time, as in the tales,
+as never was before,
+of great imperial lineage
+there lived a lovely girl.
+She was her parents’ only child,
+and proud in everything,
+as is the Virgin among saints
+and the moon among the stars.
+From the shadow of the lofty vaults
+she turns her steps
+to the window, where in a corner
+the Evening Star is waiting.
+She watched how, far away on the seas,
+he rises and shines,
+and on the moving paths
+guides the black ships.
+She sees him today, she sees him tomorrow,
+and so her longing is born;
+and he, gazing at her for weeks,
+falls in love with the girl.
+As she leaned on her elbows,
+resting her temples, dreaming,
+her heart and soul
+are filled with longing for him.
+And how brightly he flares up
+every evening
+towards the shadow of the black castle
+when she appears to him.</t>
+        </is>
+      </c>
       <c r="H119" s="13" t="inlineStr">
         <is>
           <t>Mihai Eminescu</t>
@@ -17328,7 +17520,8 @@
       </c>
       <c r="W119" s="13" t="inlineStr">
         <is>
-          <t>Shared Romanian-language literary heritage, documented by Moldova’s National Library; not a claim of birth in the modern republic. Eminescu died 1889. Use the Romanian verses; the 2009 Gagauz translation and modern introductions are separate. The selection is the original-language text; an existing English translation is not required.</t>
+          <t>Shared Romanian-language literary heritage, documented by Moldova’s National Library; not a claim of birth in the modern republic. Eminescu died 1889. Use the Romanian verses; the 2009 Gagauz translation and modern introductions are separate. The selection is the original-language text; an existing English translation is not required.
+Passage update (29 October 2026): Opening section of the poem, 7 stanzas (28 lines), from the Romanian Wikisource text of the 1883 first publication (the originally linked library page did not contain the text). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X119" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Chile to explore until 2028; Pakistan in Shahmukhi
- Chile: Gabriela Mistral's passage is withheld from the site (UK
  copyright runs to the end of 2027) via a withholdPassage flag in
  data/reader_text.json; the entry stays under Poems to explore.
- Pakistan: Bulleh Shah's kafi now shows the complete Shahmukhi text
  from Wikisource (9 lines), with title, notes and spreadsheet updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -20315,7 +20315,7 @@
       </c>
       <c r="D138" s="13" t="inlineStr">
         <is>
-          <t>ਰਾਂਝਾ ਰਾਂਝਾ ਕਰਦੀ ਨੀ ਮੈਂ / Ranjha Ranjha kardi ni main</t>
+          <t>رانجھا رانجھا کردی نی میں / Ranjha Ranjha kardi ni main</t>
         </is>
       </c>
       <c r="E138" s="13" t="inlineStr">
@@ -20325,34 +20325,28 @@
       </c>
       <c r="F138" s="13" t="inlineStr">
         <is>
-          <t>ਰਾਂਝਾ ਰਾਂਝਾ ਕਰਦੀ ਨੀ ਮੈਂ
-ਆਪੇ ਰਾਂਝਾ ਹੋਈ।
-ਸੱਦੋ ਨੀ ਮੈਨੂੰ ਧੀਦੋ ਰਾਂਝਾ
-ਹੀਰ ਨਾ ਆਖੋ ਕੋਈ।
-ਰਾਂਝਾ ਮੈਂ ਵਿੱਚ ਮੈਂ ਰਾਂਝੇ ਵਿੱਚ
-ਹੋਰ ਖਿਆਲ ਨਾ ਕੋਈ।
-ਮੈਂ ਨਹੀਂ ਉਹ ਆਪ ਹੈ ਆਪਣੀ
-ਆਪ ਕਰੇ ਦਿਲਗੋਈ।
-ਹੱਥ ਖੂੰਡੀ ਮੇਰੇ ਅੱਗੇ ਮੰਗੂ
-ਮੋਢੇ ਭੂਰਾ ਲੋਈ।
-ਬੁਲ੍ਹਾ ਹੀਰ ਸਲੇਟੀ ਵੇਖੋ
-ਕਿੱਥੇ ਜਾ ਖਲੋਈ।</t>
+          <t>رانجھا رانجھا کردی نی میں آپے رانجھا ہوئی
+سدّو نی مینُوں دھیدو رانجھا، ہِیر نہ آکھو کوئی
+رانجھا میں وِچ، میں رانجھے وِچ، مینوں ہور خیال نہ کوئی
+میں نہیں اوہ آپ ہے اپنی، آپ کرے دلجوئی
+جو کوئی ساڈے اندر وسّے، ذات اساڈی سو ای
+ہَتّھ کُھونڈی میرے اگے مَنگُو، موڈھے بُھورا لوئی
+بُلّھا ہیر سَلیٹی ویکھو، کِتّھے جا کھلوئی
+جس دے نال میں نیونہہ لگایا، اوہو جیہی ہوئی
+تخت ہزارے لے چل بُلھیا، سیالِیں ملے نہ ڈھوئی</t>
         </is>
       </c>
       <c r="G138" s="13" t="inlineStr">
         <is>
-          <t>Calling “Ranjha, Ranjha”, O friends,
-I myself have become Ranjha.
-Call me Dhido Ranjha, friends;
-let no one call me Heer.
-Ranjha is in me, I am in Ranjha;
-there is no other thought.
-It is not I: it is he himself
-who comforts his own heart.
-A herder’s staff in my hand, the herd before me,
-a brown blanket on my shoulders.
-Bulleh, look at Heer of the Sial clan:
-where has she come to stand!</t>
+          <t>Calling “Ranjha, Ranjha”, O friends, I myself have become Ranjha.
+Call me Dhido Ranjha, friends; let no one call me Heer.
+Ranjha is in me, I am in Ranjha; I have no other thought.
+It is not I: it is he himself, who comforts his own heart.
+The one who dwells within us is our very being.
+A herder’s staff in my hand, the herd before me, a brown blanket on my shoulders.
+Bulleh, look at Heer of the Sial clan: where has she come to stand!
+The one I have given my love to, I have become just like him.
+Take me to Takht Hazara, Bulleh; among the Sials I find no shelter.</t>
         </is>
       </c>
       <c r="H138" s="13" t="inlineStr">
@@ -20383,7 +20377,7 @@
       <c r="M138" s="14" t="n"/>
       <c r="N138" s="13" t="inlineStr">
         <is>
-          <t>Punjabi (Gurmukhi transcription)</t>
+          <t>Punjabi (Shahmukhi script)</t>
         </is>
       </c>
       <c r="O138" s="13" t="n"/>
@@ -20419,13 +20413,14 @@
       </c>
       <c r="V138" s="13" t="inlineStr">
         <is>
-          <t>PDF page 123, beginning ਰਾਂਝਾ ਰਾਂਝਾ ਕਰਦੀ ਨੀ ਮੈਂ</t>
+          <t>Complete kafi, 9 lines (Wikisource, Shahmukhi)</t>
         </is>
       </c>
       <c r="W138" s="13" t="inlineStr">
         <is>
           <t>Classical Punjabi text; modern compilation and translation are separate. Bulleh Shah died in the eighteenth century. The linked Gurmukhi transcription is not the historical Shahmukhi script; verify variant readings. Country connection is his Kasur/Punjab literary tradition. The selection is the original-language text; an existing English translation is not required.
-Passage update (29 October 2026): Complete kafi, 12 lines, in Gurmukhi script (proofread scan of Kafian Bulleh Shah, printed p. 121). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
+Passage update (29 October 2026): Complete kafi, 12 lines, in Gurmukhi script (proofread scan of Kafian Bulleh Shah, printed p. 121). Fresh English translation by Claude (Anthropic AI); draft for editorial review.
+Passage update (29 October 2026): Complete kafi, 9 lines, now in Shahmukhi script from Wikisource (replacing the earlier Gurmukhi text, which has three lines fewer). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X138" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Egypt: correct three words in Shawqi's poem against the encyclopedia text
Wikisource had typos; checked against the Abu Dhabi Poetry Encyclopedia
page: tawwuhuh, li-tayfika ("your phantom", not "your kindness") and
ta'addaba. English of that couplet corrected to match.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -8343,14 +8343,14 @@
 مقروح الجفنِ مسهده
 أودى حرفاً إلا رمقاً
 يُبقيه عليك وتُنْفِدهُ
-يستهوي الورق تاوهه
+يستهوي الورق تأوهه
 ويذيب الصخرَ تنهدهُ
 ويناجي النجمَ ويتعبه
 ويُقيم الليلَ ويُقْعِدهُ
 ويعلم كلَّ مطوقةٍ
 شجناً في الدَّوحِ ترددهُ
-كم مد لطفيكَ من شركٍ
-وتادب لا يتصيدهُ
+كم مد لطيفكَ من شركٍ
+وتأدب لا يتصيدهُ
 فعساك بغُمْضٍ مُسعِفهُ
 ولعلّ خيالك مسعدهُ
 الحسنُ حَلَفْتُ بيُوسُفِهِ
@@ -8373,8 +8373,8 @@
 he keeps the night standing, and makes it sit.
 He teaches every ring-necked dove
 a sorrow to repeat among the trees.
-How many snares he has laid for your kindness,
-yet, out of good manners, he does not catch it.
+How many snares he has set for your phantom,
+yet, out of good manners, he does not trap it.
 Perhaps you will grant him a moment’s sleep,
 and perhaps your phantom will bring him joy.
 I swear by beauty’s Joseph
@@ -8455,7 +8455,8 @@
       <c r="W58" s="13" t="inlineStr">
         <is>
           <t>Original poem, not the later song arrangement or a modern translation. Digital source edition undated.
-Passage update (29 October 2026): First 10 couplets (20 half-lines), from Arabic Wikisource (the originally linked poetry site could not be read). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
+Passage update (29 October 2026): First 10 couplets (20 half-lines), from Arabic Wikisource (the originally linked poetry site could not be read). Fresh English translation by Claude (Anthropic AI); draft for editorial review.
+Passage update (29 October 2026): Correction: three words checked against the poem’s page in the Abu Dhabi Poetry Encyclopedia (27 couplets, fully voweled): تاوهه → تأوهه, لطفيك → لطيفك (“your phantom”, not “your kindness”), وتادب → وتأدب; the English of couplet 7 is corrected to match. Passage remains the first 10 couplets. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X58" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Add Slovakia: Podjavorinská's "Či vieš…" (complete, 32 lines)
Text supplied from Zlatý fond SME by the project; English and history
note added, spreadsheet updated. 112 poems to read.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 112 paired passages • 83 unfilled</t>
+          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 113 paired passages • 82 unfilled</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -24124,8 +24124,78 @@
           <t>Do You Know…? (also rendered Do You Remember?)</t>
         </is>
       </c>
-      <c r="F164" s="13" t="n"/>
-      <c r="G164" s="13" t="n"/>
+      <c r="F164" s="13" t="inlineStr">
+        <is>
+          <t>Či vieš ešte, ako sme raz
+v jasný večer spolu stáli
+a ku hviezdam trblietavým
+v dumách tichých pozerali?
+Jak sme striehli obidvaja,
+až by spadla hviezda dolu,
+bo sme oba, poverčive,
+niečo žiadať mali vôľu.
+Dobrobyt ty nášho ľudu
+chcel si si vraj žiadať skryte
+a ja — ach, mnou zachvievali
+túžby divné, neurčité…
+„Blaho to vraj v hviezdach žiari,“
+dumala som, rozochvelá;
+„keby, ach, tá hviezdka jasná
+dolu ku mne zletieť chcela!“
+Tu sme oba k nebu zreli
+naladení milým klamom:
+sťaby hviezdka padajúca
+mala nám byť talizmanom.
+V tom sa stretli zraky naše
+divnou mocou upútané —;
+a za ten čas tichým letom
+padla hviezda z nebies báne.
+Kým sa stretli zraky naše,
+zhasol hviezdy plápol skvelý,
+vysloviť však svoje túžby
+oba sme my zapomneli.
+Však mne predsa splnila sa
+blúznivá tá túžba kási,
+odvtedy to v srdci mojom
+sťaby plno hviezdnej krásy.</t>
+        </is>
+      </c>
+      <c r="G164" s="13" t="inlineStr">
+        <is>
+          <t>Do you still remember how once
+we stood together on a clear evening
+and gazed up at the twinkling stars,
+lost in quiet thoughts?
+How we both kept watch
+for a star to fall,
+because we both, superstitious,
+had a mind to wish for something.
+You meant, so you said, to wish in secret
+for the well-being of our people,
+and I — ah, I was trembling with
+strange, uncertain longings…
+“They say bliss shines in the stars,”
+I mused, all a-tremble;
+“if only, ah, that bright little star
+would fly down to me!”
+Then we both looked up to the sky,
+tuned to a sweet illusion,
+as if a falling star
+were meant to be our talisman.
+At that moment our eyes met,
+held by a strange power;
+and in that time, in silent flight,
+a star fell from heaven’s dome.
+While our eyes were meeting,
+the star’s splendid flame went out,
+but to speak our wishes
+we both forgot.
+And yet for me it came true,
+that dreamy longing of mine;
+since then, in my heart,
+it is as if all were full of starry beauty.</t>
+        </is>
+      </c>
       <c r="H164" s="13" t="inlineStr">
         <is>
           <t>Ľudmila Podjavorinská</t>
@@ -24197,7 +24267,8 @@
       </c>
       <c r="W164" s="13" t="inlineStr">
         <is>
-          <t>Scope is the 1895 poem. Modern editorial matter and presentation are separate; no English translation is cleared.</t>
+          <t>Scope is the 1895 poem. Modern editorial matter and presentation are separate; no English translation is cleared.
+Passage update (29 October 2026): Complete poem, 8 quatrains (32 lines). Text copied from Zlatý fond SME (Z vesny života, chapter 8) and supplied by the project, as the page could not be read automatically. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X164" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Add Malta: Vassallo's "L-Aħħar Poeżija" (1843), read from the scan
Three quoted excerpts (16 lines) from printed p. 52, using the page
scan supplied by the project to correct OCR damage. 113 poems to read.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 113 paired passages • 82 unfilled</t>
+          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 114 paired passages • 81 unfilled</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -16572,8 +16572,46 @@
           <t>The Last Poem (proposed title: Memories of Weeping; first line: Who could have told me, poor me)</t>
         </is>
       </c>
-      <c r="F113" s="13" t="n"/>
-      <c r="G113" s="13" t="n"/>
+      <c r="F113" s="13" t="inlineStr">
+        <is>
+          <t>Min kellu jgħidli, ja miskin jiena,
+Li dal-mant f'qalbi jien kelli nġib!
+U l-ebda fejda u l-ebda ħniena
+Fl-imħabba tiegħi ma kelli nsib!
+Qanpiena mbierka! fejn dari ħossok
+Ikabbar fija kien qalb u ruħ;
+Tħassarli 'l qalbi daż-żmien inħossok,
+Il-ħabta tiegħek tiġbidli d-dmugħ!
+Lilek nistħajjel nilmaħ quddiemi
+Kull fejn f'għajnejja nara s-sabiħ;
+Fuqek għall-ajru inxerred kliemi
+Leħnek nistħajjel nisma' mar-riħ.
+U f'dit-taqriqa qalbi tithenna
+Iżda t-taqriqa fija ma ddum;
+L-uġigħ urajha qalbi tistenna
+Bil-qawwa tiegħu taqa' u ma tqum.</t>
+        </is>
+      </c>
+      <c r="G113" s="13" t="inlineStr">
+        <is>
+          <t>Who could have told me, poor me,
+that I would carry this mantle of grief in my heart,
+and that no comfort and no mercy
+would I find in my love!
+Blessed bell! where once, hearing you,
+my heart and soul would swell within me,
+now hearing you breaks my heart;
+your tolling draws my tears!
+I imagine I glimpse you before me
+wherever my eyes see beauty;
+I scatter my words about you to the air,
+I imagine I hear your voice on the wind.
+And in this rapture my heart takes comfort,
+but the rapture does not stay with me;
+after it my heart awaits the pain,
+and under its force falls and does not rise.</t>
+        </is>
+      </c>
       <c r="H113" s="13" t="inlineStr">
         <is>
           <t>Ġan Anton Vassallo (1817–1868)</t>
@@ -16640,12 +16678,13 @@
       </c>
       <c r="V113" s="13" t="inlineStr">
         <is>
-          <t>Printed p.52, including footnote 2</t>
+          <t>Printed p. 52: three quoted excerpts, 16 lines, with omissions between them</t>
         </is>
       </c>
       <c r="W113" s="13" t="inlineStr">
         <is>
-          <t>The source says Tifkir tal-Biki was the intended title; the newspaper used L-Aħħar Poeżija. Preserve this distinction. Use the old Maltese verse, not the later essay.</t>
+          <t>The source says Tifkir tal-Biki was the intended title; the newspaper used L-Aħħar Poeżija. Preserve this distinction. Use the old Maltese verse, not the later essay.
+Passage update (29 October 2026): Three excerpts (16 lines) as quoted on printed p. 52 of the source, which marks omissions between them with dotted lines. Text read from the scan of p. 52 supplied by the project, correcting OCR damage (mbierka, nilmaħ, ’l qalbi, jgħidli). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X113" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Add Ethiopia: Oromo love song no. 117, read from the 1922 page
Five lines recorded by Onesimos Nesib and Aster Ganno (1894), from
Cerulli's 1922 edition, read from a page image supplied by the project;
new English translation. 114 poems to read.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 114 paired passages • 81 unfilled</t>
+          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 115 paired passages • 80 unfilled</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -9205,8 +9205,24 @@
           <t>O merchant of the merchandise (first line; love song117)</t>
         </is>
       </c>
-      <c r="F64" s="13" t="n"/>
-      <c r="G64" s="13" t="n"/>
+      <c r="F64" s="13" t="inlineStr">
+        <is>
+          <t>naggādiē naggāddīmā
+kān tullū Burē ğirtū
+iğğātō qottō ḍabē
+garātō murtē ḍabē
+kān tullū murē ğiğsū</t>
+        </is>
+      </c>
+      <c r="G64" s="13" t="inlineStr">
+        <is>
+          <t>O merchant, trader in goods,
+who are at Mount Burē!
+The eyes have no axe,
+the mind has no sickle,
+to cut down the mountains and throw them aside!</t>
+        </is>
+      </c>
       <c r="H64" s="13" t="inlineStr">
         <is>
           <t>Traditional Oromo composer unknown; collected by Onesimos Nesib and Aster Ganno; edited by Enrico Cerulli</t>
@@ -9273,12 +9289,13 @@
       </c>
       <c r="V64" s="13" t="inlineStr">
         <is>
-          <t>III, Love Songs, no.117; identify by number rather than unverified print page</t>
+          <t>III, Love Songs, no. 117 (printed p. 120)</t>
         </is>
       </c>
       <c r="W64" s="13" t="inlineStr">
         <is>
-          <t>Composer gender is unknown; a female speaker does not establish female authorship. Aster Ganno’s contribution is as co-compiler. The modern Seltzer transcription drops diacritics and carries a restrictive non-commercial notice: consult the 1922 scan for original typography. Historical title uses an outdated exonym for Oromo. Cerulli’s English translation and modern editorial material have separate territorial rights.</t>
+          <t>Composer gender is unknown; a female speaker does not establish female authorship. Aster Ganno’s contribution is as co-compiler. The modern Seltzer transcription drops diacritics and carries a restrictive non-commercial notice: consult the 1922 scan for original typography. Historical title uses an outdated exonym for Oromo. Cerulli’s English translation and modern editorial material have separate territorial rights.
+Passage update (29 October 2026): Complete song no. 117 (5 lines), Harvard African Studies vol. 3 (1922), p. 120, in Cerulli’s scholarly transcription; the two-column layout is put into verse order. Letters read from a page image supplied by the project: check the diacritics against the printed page. The English is new (Cerulli’s own translation is excluded). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X64" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Add Panama: Ricardo Miró's "Amor dantesco" (1918, complete sonnet)
Read from an image of printed p. 170 supplied by the project; English
and history note added. 115 poems to read.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 115 paired passages • 80 unfilled</t>
+          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 116 paired passages • 79 unfilled</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -20836,8 +20836,42 @@
           <t>Dantean Love</t>
         </is>
       </c>
-      <c r="F141" s="13" t="n"/>
-      <c r="G141" s="13" t="n"/>
+      <c r="F141" s="13" t="inlineStr">
+        <is>
+          <t>Yo quisiera decírtelo y no puedo;
+me lo veda un poder que no es humano.
+Te voy a hablar y una invisible mano
+posa en mis labios trémulos un dedo.
+Mudo, y absorto, y aturdido quedo
+ante el prodigio de este amor arcano,
+tan azul, tan sin fin como un océano,
+tan hondo que a mí mismo me da miedo.
+Miedo, pavor de que también me ames;
+de que así como yo toda te inflames
+en este amor cuyo final no vemos;
+porque he asomado a mi alma entre mí mismo
+y no hallo el fondo del profundo abismo
+de amor y de dolor en que caeremos.</t>
+        </is>
+      </c>
+      <c r="G141" s="13" t="inlineStr">
+        <is>
+          <t>I would like to tell you, and I cannot;
+a power that is not human forbids me.
+I am about to speak, and an invisible hand
+lays a finger on my trembling lips.
+Mute, absorbed and dazed I stand
+before the wonder of this secret love,
+as blue, as endless as an ocean,
+so deep that I myself am afraid.
+Afraid, in dread that you love me too;
+that, like me, you may be all aflame
+in this love whose end we cannot see;
+for I have looked into my soul, within myself,
+and cannot find the bottom of the deep abyss
+of love and pain into which we shall fall.</t>
+        </is>
+      </c>
       <c r="H141" s="13" t="inlineStr">
         <is>
           <t>Ricardo Miró (1883–1940)</t>
@@ -20909,7 +20943,8 @@
       </c>
       <c r="W141" s="13" t="inlineStr">
         <is>
-          <t>The reuse assessment applies to Miró’s historical poem. The anthology’s modern introduction, selection and commentary are separate. The poem is intense rather than uncomplicatedly joyful.</t>
+          <t>The reuse assessment applies to Miró’s historical poem. The anthology’s modern introduction, selection and commentary are separate. The poem is intense rather than uncomplicatedly joyful.
+Passage update (29 October 2026): Complete sonnet, 14 lines, dated August 1918, read from an image of printed p. 170 supplied by the project (the library PDF’s security certificate had expired). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X141" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Add Singapore: Khoo Seok Wan's Qingming poem for his late wife (1937)
Complete four-line poem from 菽园诗集 vol. 6 on Shidian Guji, verified
against the page HTML. 116 poems to read.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 116 paired passages • 79 unfilled</t>
+          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 117 paired passages • 78 unfilled</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -24068,16 +24068,30 @@
       </c>
       <c r="D163" s="13" t="inlineStr">
         <is>
-          <t>几枚白石伴青珉 (incipit; memorial poem for Lu Jie)</t>
+          <t>丁丑清明节，为亡室陆氏筑坟成</t>
         </is>
       </c>
       <c r="E163" s="13" t="inlineStr">
         <is>
-          <t>A few white stones beside green jade (first line; memorial poem for Lu Jie)</t>
-        </is>
-      </c>
-      <c r="F163" s="13" t="n"/>
-      <c r="G163" s="13" t="n"/>
+          <t>Qingming 1937, on Completing the Grave of My Late Wife</t>
+        </is>
+      </c>
+      <c r="F163" s="13" t="inlineStr">
+        <is>
+          <t>几枚白石伴青珉，
+小筑坟茔隔岁春。
+地下有灵相谅解，
+迟工原是为家贫。</t>
+        </is>
+      </c>
+      <c r="G163" s="13" t="inlineStr">
+        <is>
+          <t>A few white stones beside the green jade stone:
+a year on, in spring, I have built this small grave.
+If your spirit below can know, forgive me:
+the work was late only because we are poor.</t>
+        </is>
+      </c>
       <c r="H163" s="13" t="inlineStr">
         <is>
           <t>Khoo Seok Wan / 丘菽园 (1874–1941)</t>
@@ -24149,7 +24163,8 @@
       </c>
       <c r="W163" s="13" t="inlineStr">
         <is>
-          <t>Incipit identifies the work; do not invent a formal title. Use Khoo’s Chinese verse only. Modern English translations, photographs and the scholarly article have separate rights.</t>
+          <t>Incipit identifies the work; do not invent a formal title. Use Khoo’s Chinese verse only. Modern English translations, photographs and the scholarly article have separate rights.
+Passage update (29 October 2026): Complete poem, 4 lines, from 菽园诗集 vol. 6 on Shidian Guji (the originally linked PDF could not be opened). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X163" s="13" t="inlineStr">
@@ -24164,7 +24179,7 @@
       </c>
       <c r="Z163" s="11" t="inlineStr">
         <is>
-          <t>Work / source text</t>
+          <t>Read original</t>
         </is>
       </c>
       <c r="AA163" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Malaysia: traditional love pantun replace the unavailable novel
Five "Pantun Kasih" quatrains (20 lines) from Malay Wikisource, with
English, history note and an updated spreadsheet row. 117 poems to read.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 117 paired passages • 78 unfilled</t>
+          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 118 paired passages • 77 unfilled</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -16224,19 +16224,65 @@
       </c>
       <c r="D110" s="13" t="inlineStr">
         <is>
-          <t>Hikayat Faridah Hanom (also Faridah Hanum)</t>
+          <t>Pantun Kasih</t>
         </is>
       </c>
       <c r="E110" s="13" t="inlineStr">
         <is>
-          <t>The Tale of Faridah Hanom (also Hanum)</t>
-        </is>
-      </c>
-      <c r="F110" s="13" t="n"/>
-      <c r="G110" s="13" t="n"/>
+          <t>Love Pantun</t>
+        </is>
+      </c>
+      <c r="F110" s="13" t="inlineStr">
+        <is>
+          <t>Nasi lemak buah bidara
+sayang selasih hamba lurutkan;
+Buang emak buang saudara
+kerana kekasih hamba turutkan
+Dua tiga kucing berlari
+mana nak sama si kucing belang;
+Dua tiga boleh kucari
+mana nak sama dikau seorang
+Tanam selasih di tengah padang
+sudah bertangkai dirubung semut;
+Kita kasih orang tak sayang
+halai-balai tempurung hanyut
+Anak beruk di kayu rendang
+turun mandi ke dalam paya;
+Biar buruk di mata orang
+cantik manis di mata saya
+Limau purut lebat di pangkal
+sayang selasih condong di uratnya;
+Angin ribut dapat ditangkal
+hati kasih apa ubatnya</t>
+        </is>
+      </c>
+      <c r="G110" s="13" t="inlineStr">
+        <is>
+          <t>Coconut rice and jujube fruit,
+sweet basil I strip from the stem;
+I leave my mother, I leave my kin,
+to follow the one I love.
+Two or three cats go running by,
+but none is like the striped one;
+two or three others I could find,
+but none would be like you alone.
+Basil planted in the middle of the field,
+already in stalk, swarmed by ants;
+I love, but am not loved in return:
+tossed about like a drifting coconut shell.
+A young macaque in the leafy tree
+comes down to bathe in the swamp;
+let others think you plain,
+to my eyes you are lovely and sweet.
+Kaffir limes grow thick at the trunk,
+the basil leans upon its roots;
+a storm wind can be warded off,
+but what can cure a loving heart?</t>
+        </is>
+      </c>
       <c r="H110" s="13" t="inlineStr">
         <is>
-          <t>Syed Sheikh bin Ahmad al-Hadi (1867–1934)</t>
+          <t>Traditional Malay pantun</t>
         </is>
       </c>
       <c r="I110" s="13" t="inlineStr">
@@ -16251,7 +16297,7 @@
       </c>
       <c r="K110" s="13" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Poetry</t>
         </is>
       </c>
       <c r="L110" s="13" t="inlineStr">
@@ -16259,12 +16305,10 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M110" s="14" t="n">
-        <v>1925</v>
-      </c>
+      <c r="M110" s="14" t="n"/>
       <c r="N110" s="13" t="inlineStr">
         <is>
-          <t>Malay (original Jawi script)</t>
+          <t>Malay</t>
         </is>
       </c>
       <c r="O110" s="13" t="n"/>
@@ -16280,7 +16324,7 @@
       </c>
       <c r="R110" s="13" t="inlineStr">
         <is>
-          <t>Published in two volumes, Penang, 1925 and 1926</t>
+          <t>Traditional oral verse; date unknown</t>
         </is>
       </c>
       <c r="S110" s="13" t="inlineStr">
@@ -16290,7 +16334,7 @@
       </c>
       <c r="T110" s="13" t="inlineStr">
         <is>
-          <t>Romance of Faridah Hanom and Syafik Efendi, including playful verses in which she dresses to tempt her lover.</t>
+          <t>Five traditional love pantun: leaving family to follow the beloved, a love no one else can equal, unrequited love, beauty in the lover’s eyes, and a lovesick heart no medicine can cure.</t>
         </is>
       </c>
       <c r="U110" s="13" t="inlineStr">
@@ -16300,17 +16344,18 @@
       </c>
       <c r="V110" s="13" t="inlineStr">
         <is>
-          <t>MoMA section A Delightful Subject; novel pp.138–139</t>
+          <t>Pantun Kasih, first five quatrains</t>
         </is>
       </c>
       <c r="W110" s="13" t="inlineStr">
         <is>
-          <t>Malacca-born author and Penang publication establish the Malaysian association; story is set in Egypt. Whether the novel adapts an unidentified Arabic source is debated. The identified 1925–26 published Malay text is public domain in the US; al-Hadi’s own text is also beyond life-plus-70. Exclude modern English translation, commentary and any independently protected source or image.</t>
+          <t>Malacca-born author and Penang publication establish the Malaysian association; story is set in Egypt. Whether the novel adapts an unidentified Arabic source is debated. The identified 1925–26 published Malay text is public domain in the US; al-Hadi’s own text is also beyond life-plus-70. Exclude modern English translation, commentary and any independently protected source or image.
+Passage update (29 October 2026): Work changed (29 October 2026): the novel Hikayat Faridah Hanom, whose text could not be found online, is replaced by traditional Malay love pantun, a locally made oral form. Five quatrains (20 lines) from the “Pantun Kasih” section of Malay Wikisource. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X110" s="13" t="inlineStr">
         <is>
-          <t>Historical original composition; author died 1934, beyond the standard life-plus-70 term. Reuse the underlying historical original only, excluding modern translations, editorial matter, images, adaptations and recordings. Publication history and territorial exceptions should be checked for the edition used.</t>
+          <t>Traditional anonymous oral verse; text from Malay Wikisource.</t>
         </is>
       </c>
       <c r="Y110" s="13" t="inlineStr">
@@ -16320,7 +16365,7 @@
       </c>
       <c r="Z110" s="11" t="inlineStr">
         <is>
-          <t>Work / text</t>
+          <t>Read original</t>
         </is>
       </c>
       <c r="AA110" s="11" t="inlineStr">

</xml_diff>

<commit_message>
Replace slave-era colonial works with local voices: Barbados, Suriname, Mauritius
- Barbados: H. A. Vaughan, "Revelation" (replaces Orderson)
- Suriname: Johanna Schouten-Elsenhout, Awese, Sranan poems (replaces Stedman)
- Mauritius: Ti Frère, "Anita", sega (replaces Bernardin de Saint-Pierre)

All in copyright, so listed under Poems to explore with a description,
history note and link; spreadsheet rows updated with the change noted.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -3044,34 +3044,34 @@
       </c>
       <c r="D21" s="13" t="inlineStr">
         <is>
-          <t>Creoleana; or, Social and Domestic Scenes and Incidents in Barbados in Days of Yore</t>
+          <t>Revelation</t>
         </is>
       </c>
       <c r="E21" s="13" t="inlineStr">
         <is>
-          <t>Creoleana; or, Social and Domestic Scenes and Incidents in Barbados in Days of Yore</t>
+          <t>Revelation</t>
         </is>
       </c>
       <c r="F21" s="13" t="n"/>
       <c r="G21" s="13" t="n"/>
       <c r="H21" s="13" t="inlineStr">
         <is>
-          <t>J. W. Orderson (historical author, 1767–1847)</t>
+          <t>H. A. Vaughan (1901–1985)</t>
         </is>
       </c>
       <c r="I21" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J21" s="13" t="inlineStr">
         <is>
-          <t>Named novel (historical edition)</t>
+          <t>Named poem</t>
         </is>
       </c>
       <c r="K21" s="13" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Poetry</t>
         </is>
       </c>
       <c r="L21" s="13" t="inlineStr">
@@ -3079,9 +3079,7 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M21" s="14" t="n">
-        <v>1842</v>
-      </c>
+      <c r="M21" s="14" t="n"/>
       <c r="N21" s="13" t="inlineStr">
         <is>
           <t>English</t>
@@ -3100,65 +3098,50 @@
       </c>
       <c r="R21" s="13" t="inlineStr">
         <is>
-          <t>First published London: Saunders and Otley, 1842</t>
-        </is>
-      </c>
-      <c r="S21" s="13" t="inlineStr">
-        <is>
-          <t>1842 original edition; Google Books full-view edition identified</t>
-        </is>
-      </c>
+          <t>Twentieth century; reprinted in Bim vol. 8 (Independence issue)</t>
+        </is>
+      </c>
+      <c r="S21" s="13" t="n"/>
       <c r="T21" s="13" t="inlineStr">
         <is>
-          <t>Caroline Fairfield and Jack Goldacre overcome obstacles and marry. Their courtship is paired with the story of Caroline’s half-sister Lucy within Barbadian colonial society.</t>
+          <t>A Barbadian lover asks his beloved to turn in the sun, praising her dark beauty above the Greek and Roman ideals taught in school.</t>
         </is>
       </c>
       <c r="U21" s="13" t="inlineStr">
         <is>
-          <t>Google Books lists the 1842 original as Full view; Cambridge History of Victorian Literature discusses its Barbadian authorship. John Gilmore’s scholarly review discusses the romantic plot.</t>
+          <t>Bim magazine, vol. 8 (Independence issue), p. 46</t>
         </is>
       </c>
       <c r="V21" s="13" t="inlineStr">
         <is>
-          <t>Courtship and eventual marriage of Caroline Fairfield and Jack Goldacre</t>
+          <t>Complete poem, p. 46</t>
         </is>
       </c>
       <c r="W21" s="13" t="inlineStr">
         <is>
           <t>Reuse the 1842 text. The 2002 John Gilmore introduction, notes and other new editorial content are excluded. Colonial racial hierarchies and slavery form part of the narrative context. Retain the original printed author name J. W. Orderson rather than infer an expanded name.
-Passage update (29 October 2026): Not filled: the 1842 novel is identified, but the linked Google Books text could not be retrieved for passage verification. Supply relevant original-edition pages showing Caroline Fairfield and Jack Goldacre. Do not substitute a plot summary for the original English text.</t>
+Passage update (29 October 2026): Not filled: the 1842 novel is identified, but the linked Google Books text could not be retrieved for passage verification. Supply relevant original-edition pages showing Caroline Fairfield and Jack Goldacre. Do not substitute a plot summary for the original English text.
+Work changed (29 October 2026): the earlier work, by a colonial author from the slave-owning side, is replaced by a work by a local writer descended from the enslaved. In copyright: listed with a description and link only, not reproduced.</t>
         </is>
       </c>
       <c r="X21" s="13" t="inlineStr">
         <is>
-          <t>Historical original composition; author died 1847, beyond the standard life-plus-70 term. Reuse the underlying historical original only, excluding modern translations, editorial matter, images, adaptations and recordings. Publication history and territorial exceptions should be checked for the edition used.</t>
+          <t>In copyright (author died 1985). Not reproduced; listed with a link.</t>
         </is>
       </c>
       <c r="Y21" s="13" t="inlineStr">
         <is>
-          <t>Work-specific text, date and provenance sources checked29October2026.</t>
+          <t>Bim magazine, vol. 8</t>
         </is>
       </c>
       <c r="Z21" s="11" t="inlineStr">
         <is>
-          <t>Work / text</t>
-        </is>
-      </c>
-      <c r="AA21" s="11" t="inlineStr">
-        <is>
-          <t>Rights / catalogue</t>
-        </is>
-      </c>
-      <c r="AB21" s="11" t="inlineStr">
-        <is>
-          <t>Date / edition</t>
-        </is>
-      </c>
-      <c r="AC21" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country</t>
-        </is>
-      </c>
+          <t>Read about it</t>
+        </is>
+      </c>
+      <c r="AA21" s="11" t="n"/>
+      <c r="AB21" s="11" t="n"/>
+      <c r="AC21" s="11" t="n"/>
       <c r="AD21" s="11" t="n"/>
       <c r="AE21" s="11" t="n"/>
     </row>
@@ -17067,34 +17050,34 @@
       </c>
       <c r="D116" s="13" t="inlineStr">
         <is>
-          <t>Paul et Virginie</t>
+          <t>Anita</t>
         </is>
       </c>
       <c r="E116" s="13" t="inlineStr">
         <is>
-          <t>Paul and Virginie (the lovers' names)</t>
+          <t>Anita</t>
         </is>
       </c>
       <c r="F116" s="13" t="n"/>
       <c r="G116" s="13" t="n"/>
       <c r="H116" s="13" t="inlineStr">
         <is>
-          <t>Jacques-Henri Bernardin de Saint-Pierre (1737–1814)</t>
+          <t>Ti Frère (Jean Alphonse Ravaton, 1900–1992)</t>
         </is>
       </c>
       <c r="I116" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J116" s="13" t="inlineStr">
         <is>
-          <t>Named work (text)</t>
+          <t>Named work</t>
         </is>
       </c>
       <c r="K116" s="13" t="inlineStr">
         <is>
-          <t>Prose / novel</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="L116" s="13" t="inlineStr">
@@ -17102,12 +17085,10 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M116" s="14" t="n">
-        <v>1788</v>
-      </c>
+      <c r="M116" s="14" t="n"/>
       <c r="N116" s="13" t="inlineStr">
         <is>
-          <t>French</t>
+          <t>Mauritian Creole</t>
         </is>
       </c>
       <c r="O116" s="13" t="n"/>
@@ -17123,69 +17104,50 @@
       </c>
       <c r="R116" s="13" t="inlineStr">
         <is>
-          <t>1788 in Études de la nature; separate edition 1789</t>
-        </is>
-      </c>
-      <c r="S116" s="13" t="inlineStr">
-        <is>
-          <t>Linked French edition: 1874; Wikisource also has an 1806 edition</t>
-        </is>
-      </c>
+          <t>Twentieth century</t>
+        </is>
+      </c>
+      <c r="S116" s="13" t="n"/>
       <c r="T116" s="13" t="inlineStr">
         <is>
-          <t>Paul and Virginie’s childhood affection becomes romantic love on Mauritius; separation and shipwreck bring a tragic ending.</t>
+          <t>One of the best-loved segas of Ti Frère, the “King of Sega”, whose songs tell of impossible loves, quarrelling lovers and hard lives.</t>
         </is>
       </c>
       <c r="U116" s="13" t="inlineStr">
         <is>
-          <t>Library of Congress digitised French edition and work description identify Mauritius as the setting and confirm the original date.</t>
+          <t>Ti Frère’s repertoire; on the Ocora compilation Mauritius: Tribute to Ti Frère – Séga, Music of Exile</t>
         </is>
       </c>
       <c r="V116" s="13" t="inlineStr">
         <is>
-          <t>Complete novel; select the lovers’ declarations or separation passages</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="W116" s="13" t="inlineStr">
         <is>
-          <t>Country connection is setting and Mauritian cultural association: the author was French, not Mauritian. The story reflects a colonial plantation society. Modern adaptations and commentary are excluded.</t>
+          <t>Country connection is setting and Mauritian cultural association: the author was French, not Mauritian. The story reflects a colonial plantation society. Modern adaptations and commentary are excluded.
+Work changed (29 October 2026): the earlier work, by a colonial author from the slave-owning side, is replaced by a work by a local writer descended from the enslaved. In copyright: listed with a description and link only, not reproduced.</t>
         </is>
       </c>
       <c r="X116" s="13" t="inlineStr">
         <is>
-          <t>The Library of Congress expressly identifies the linked book as public domain and free to use and reuse. Historical French original also falls well beyond standard life-plus-70 terms.</t>
+          <t>In copyright (artist died 1992). Not reproduced; listed with a link.</t>
         </is>
       </c>
       <c r="Y116" s="13" t="inlineStr">
         <is>
-          <t>Library of Congress digitised French edition and work description identify Mauritius as the setting and confirm the original date.</t>
+          <t>Maurisique: Ti Frère forever</t>
         </is>
       </c>
       <c r="Z116" s="11" t="inlineStr">
         <is>
-          <t>Work / source text</t>
-        </is>
-      </c>
-      <c r="AA116" s="11" t="inlineStr">
-        <is>
-          <t>Reuse basis / copyright duration</t>
-        </is>
-      </c>
-      <c r="AB116" s="11" t="inlineStr">
-        <is>
-          <t>Date / edition evidence</t>
-        </is>
-      </c>
-      <c r="AC116" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country evidence</t>
-        </is>
-      </c>
-      <c r="AD116" s="11" t="inlineStr">
-        <is>
-          <t>Additional evidence</t>
-        </is>
-      </c>
+          <t>Read about it</t>
+        </is>
+      </c>
+      <c r="AA116" s="11" t="n"/>
+      <c r="AB116" s="11" t="n"/>
+      <c r="AC116" s="11" t="n"/>
+      <c r="AD116" s="11" t="n"/>
       <c r="AE116" s="11" t="n"/>
     </row>
     <row r="117" ht="235.5" customHeight="1" s="17">
@@ -25703,34 +25665,34 @@
       </c>
       <c r="D174" s="13" t="inlineStr">
         <is>
-          <t>Narrative of a Five Years’ Expedition against the Revolted Negroes of Surinam — Joanna episodes</t>
+          <t>Awese</t>
         </is>
       </c>
       <c r="E174" s="13" t="inlineStr">
         <is>
-          <t>Narrative of a Five Years’ Expedition against the Revolted Negroes of Surinam — Joanna episodes</t>
+          <t>Awese (poems in Sranan Tongo)</t>
         </is>
       </c>
       <c r="F174" s="13" t="n"/>
       <c r="G174" s="13" t="n"/>
       <c r="H174" s="13" t="inlineStr">
         <is>
-          <t>John Gabriel Stedman (1744–1797)</t>
+          <t>Johanna Schouten-Elsenhout (1910–1992)</t>
         </is>
       </c>
       <c r="I174" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J174" s="13" t="inlineStr">
         <is>
-          <t>Named literary memoir (full historical edition)</t>
+          <t>Named poetry collection</t>
         </is>
       </c>
       <c r="K174" s="13" t="inlineStr">
         <is>
-          <t>Literary memoir</t>
+          <t>Poetry</t>
         </is>
       </c>
       <c r="L174" s="13" t="inlineStr">
@@ -25739,11 +25701,11 @@
         </is>
       </c>
       <c r="M174" s="14" t="n">
-        <v>1796</v>
+        <v>1965</v>
       </c>
       <c r="N174" s="13" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Sranan Tongo</t>
         </is>
       </c>
       <c r="O174" s="13" t="n"/>
@@ -25759,64 +25721,49 @@
       </c>
       <c r="R174" s="13" t="inlineStr">
         <is>
-          <t>First published London, 1796; describes residence in Suriname, 1773–1777</t>
-        </is>
-      </c>
-      <c r="S174" s="13" t="inlineStr">
-        <is>
-          <t>1796 published version, two volumes</t>
-        </is>
-      </c>
+          <t>1965 (collection)</t>
+        </is>
+      </c>
+      <c r="S174" s="13" t="n"/>
       <c r="T174" s="13" t="inlineStr">
         <is>
-          <t>Stedman narrates his attachment to Joanna, their life together and their separation in Suriname. Read as a colonial memoir of romantic attachment within slavery, rather than an equal relationship.</t>
+          <t>Poems in Sranan Tongo by one of Suriname’s first women poets, among them love poems, including poems of love between women.</t>
         </is>
       </c>
       <c r="U174" s="13" t="inlineStr">
         <is>
-          <t>Library of Congress digitizes the 1796 edition; Wellcome marks its 1796 copy Public Domain. Romantic Circles study explains the Joanna narrative and differences between manuscript and print.</t>
+          <t>Awese (1965); her work is discussed by the Werkgroep Caraïbische Letteren</t>
         </is>
       </c>
       <c r="V174" s="13" t="inlineStr">
         <is>
-          <t>Joanna episodes across the two volumes; see edition comparison in Romantic Circles</t>
+          <t>Collection</t>
         </is>
       </c>
       <c r="W174" s="13" t="inlineStr">
         <is>
-          <t>Foreign Scottish-Dutch author stationed in Suriname; not a Surinamese-authored indigenous voice. Slavery, colonial violence and unequal power are integral. Use the published 1796 text, not the substantially different modern editions of the 1790 manuscript (1988/1992).</t>
+          <t>Foreign Scottish-Dutch author stationed in Suriname; not a Surinamese-authored indigenous voice. Slavery, colonial violence and unequal power are integral. Use the published 1796 text, not the substantially different modern editions of the 1790 manuscript (1988/1992).
+Work changed (29 October 2026): the earlier work, by a colonial author from the slave-owning side, is replaced by a work by a local writer descended from the enslaved. In copyright: listed with a description and link only, not reproduced.</t>
         </is>
       </c>
       <c r="X174" s="13" t="inlineStr">
         <is>
-          <t>Historical original composition; author died 1797, beyond the standard life-plus-70 term. Reuse the underlying historical original only, excluding modern translations, editorial matter, images, adaptations and recordings. Publication history and territorial exceptions should be checked for the edition used.</t>
+          <t>In copyright (author died 1992). Not reproduced; listed with a link.</t>
         </is>
       </c>
       <c r="Y174" s="13" t="inlineStr">
         <is>
-          <t>Work-specific text, date and provenance sources checked29October2026.</t>
+          <t>Werkgroep Caraïbische Letteren: 100 jaar Johanna Schouten-Elsenhout</t>
         </is>
       </c>
       <c r="Z174" s="11" t="inlineStr">
         <is>
-          <t>Work / text</t>
-        </is>
-      </c>
-      <c r="AA174" s="11" t="inlineStr">
-        <is>
-          <t>Rights / catalogue</t>
-        </is>
-      </c>
-      <c r="AB174" s="11" t="inlineStr">
-        <is>
-          <t>Date / edition</t>
-        </is>
-      </c>
-      <c r="AC174" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country</t>
-        </is>
-      </c>
+          <t>Read about it</t>
+        </is>
+      </c>
+      <c r="AA174" s="11" t="n"/>
+      <c r="AB174" s="11" t="n"/>
+      <c r="AC174" s="11" t="n"/>
       <c r="AD174" s="11" t="n"/>
       <c r="AE174" s="11" t="n"/>
     </row>
@@ -29837,633 +29784,623 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC20" r:id="rId49"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD20" r:id="rId50"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z21" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA21" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB21" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC21" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z22" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA22" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB22" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC22" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z23" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA23" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB23" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC23" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z24" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD24" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z25" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA25" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB25" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC25" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD25" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z26" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z27" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA27" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB27" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC27" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z28" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA28" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB28" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC28" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z29" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z30" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA30" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB30" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC30" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z31" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z32" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA32" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB32" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC32" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z33" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z34" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z35" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA35" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB35" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC35" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD35" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z36" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA36" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB36" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC36" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD36" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z37" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z38" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA38" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB38" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC38" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z39" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD39" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z40" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA40" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB40" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC40" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD40" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z41" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA41" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB41" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC41" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z42" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA42" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB42" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC42" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z43" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA43" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB43" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC43" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z44" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD44" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z45" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA45" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB45" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC45" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD45" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z46" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA46" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB46" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC46" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z47" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD47" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE47" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z48" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA48" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB48" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC48" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z49" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA49" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB49" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC49" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z50" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA50" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB50" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC50" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z51" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA51" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB51" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC51" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z52" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z53" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA53" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB53" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC53" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD53" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z54" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z55" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z56" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA56" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB56" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC56" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z57" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA57" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB57" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC57" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z58" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA58" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB58" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC58" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z59" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA59" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB59" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC59" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z60" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z61" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z62" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA62" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB62" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC62" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z63" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA63" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB63" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC63" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z64" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA64" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB64" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC64" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z65" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA65" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB65" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC65" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z66" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA66" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB66" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC66" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z67" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA67" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB67" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC67" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z68" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z69" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z70" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA70" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB70" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC70" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z71" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA71" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB71" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC71" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z72" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA72" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB72" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC72" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD72" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z73" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA73" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB73" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC73" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z74" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD74" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z75" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA75" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB75" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC75" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z76" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z77" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA77" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB77" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC77" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z78" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA78" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB78" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC78" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD78" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z79" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA79" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB79" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC79" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z80" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA80" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB80" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC80" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD80" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE80" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z81" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA81" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB81" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC81" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z82" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA82" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB82" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC82" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z83" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA83" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB83" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC83" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD83" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA84" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB84" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC84" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA85" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB85" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC85" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA86" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB86" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC86" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA87" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB87" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC87" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA88" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB88" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC88" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA89" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB89" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC89" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA90" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB90" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC90" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD90" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA91" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB91" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC91" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA92" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB92" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC92" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD92" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA93" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB93" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC93" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA94" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB94" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC94" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD96" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA97" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB97" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC97" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA98" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB98" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC98" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA100" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB100" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC100" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA101" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB101" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC101" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA102" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB102" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC102" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD102" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA103" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB103" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC103" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD103" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA104" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB104" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC104" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA105" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB105" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC105" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD105" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA106" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB106" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC106" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA107" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB107" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC107" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD107" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD108" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA110" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB110" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC110" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD111" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA113" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB113" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC113" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z115" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA115" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB115" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC115" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z116" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA116" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB116" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC116" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD116" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z117" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA117" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB117" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC117" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z118" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z119" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA119" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB119" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC119" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z120" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD120" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z121" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA121" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB121" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC121" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD121" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z122" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA122" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB122" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC122" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z123" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA123" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB123" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC123" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z124" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA124" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB124" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC124" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD124" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z125" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z126" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z127" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA127" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB127" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC127" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD127" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z128" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA128" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB128" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC128" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z129" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA129" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB129" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC129" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z130" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA130" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB130" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC130" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z131" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA131" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB131" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC131" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z132" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z133" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA133" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB133" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC133" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z134" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA134" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB134" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC134" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z135" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA135" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB135" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC135" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z136" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA136" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB136" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC136" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z137" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA137" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB137" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC137" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z138" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA138" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB138" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC138" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z139" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z140" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA140" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB140" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC140" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z141" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA141" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB141" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC141" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z142" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z143" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA143" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB143" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC143" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z144" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA144" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB144" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC144" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z145" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA145" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB145" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC145" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z146" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA146" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB146" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC146" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z147" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA147" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB147" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC147" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z148" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA148" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB148" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC148" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z149" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA149" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB149" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC149" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z150" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA150" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB150" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC150" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD150" r:id="rId500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z151" r:id="rId501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD151" r:id="rId502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z152" r:id="rId503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA152" r:id="rId504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB152" r:id="rId505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC152" r:id="rId506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD152" r:id="rId507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z153" r:id="rId508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z154" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z155" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA155" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB155" r:id="rId512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC155" r:id="rId513"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z156" r:id="rId514"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z157" r:id="rId515"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA157" r:id="rId516"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB157" r:id="rId517"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC157" r:id="rId518"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD157" r:id="rId519"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z158" r:id="rId520"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA158" r:id="rId521"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB158" r:id="rId522"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC158" r:id="rId523"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z159" r:id="rId524"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA159" r:id="rId525"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB159" r:id="rId526"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC159" r:id="rId527"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z160" r:id="rId528"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA160" r:id="rId529"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB160" r:id="rId530"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC160" r:id="rId531"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z161" r:id="rId532"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z162" r:id="rId533"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA162" r:id="rId534"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB162" r:id="rId535"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC162" r:id="rId536"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z163" r:id="rId537"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA163" r:id="rId538"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB163" r:id="rId539"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC163" r:id="rId540"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD163" r:id="rId541"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z164" r:id="rId542"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA164" r:id="rId543"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB164" r:id="rId544"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC164" r:id="rId545"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z165" r:id="rId546"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA165" r:id="rId547"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB165" r:id="rId548"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC165" r:id="rId549"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z166" r:id="rId550"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z167" r:id="rId551"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA167" r:id="rId552"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB167" r:id="rId553"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC167" r:id="rId554"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD167" r:id="rId555"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z168" r:id="rId556"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA168" r:id="rId557"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB168" r:id="rId558"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC168" r:id="rId559"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z169" r:id="rId560"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA169" r:id="rId561"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB169" r:id="rId562"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC169" r:id="rId563"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z170" r:id="rId564"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z171" r:id="rId565"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA171" r:id="rId566"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB171" r:id="rId567"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC171" r:id="rId568"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z172" r:id="rId569"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA172" r:id="rId570"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB172" r:id="rId571"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC172" r:id="rId572"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD172" r:id="rId573"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z173" r:id="rId574"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z174" r:id="rId575"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA174" r:id="rId576"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB174" r:id="rId577"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC174" r:id="rId578"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z175" r:id="rId579"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA175" r:id="rId580"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB175" r:id="rId581"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC175" r:id="rId582"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z176" r:id="rId583"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA176" r:id="rId584"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB176" r:id="rId585"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC176" r:id="rId586"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z177" r:id="rId587"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA177" r:id="rId588"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB177" r:id="rId589"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC177" r:id="rId590"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z178" r:id="rId591"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA178" r:id="rId592"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB178" r:id="rId593"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC178" r:id="rId594"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z179" r:id="rId595"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA179" r:id="rId596"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB179" r:id="rId597"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC179" r:id="rId598"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD179" r:id="rId599"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z180" r:id="rId600"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA180" r:id="rId601"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB180" r:id="rId602"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC180" r:id="rId603"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z181" r:id="rId604"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z182" r:id="rId605"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD182" r:id="rId606"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z183" r:id="rId607"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA183" r:id="rId608"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB183" r:id="rId609"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC183" r:id="rId610"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z184" r:id="rId611"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA184" r:id="rId612"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB184" r:id="rId613"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC184" r:id="rId614"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD184" r:id="rId615"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z185" r:id="rId616"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA185" r:id="rId617"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB185" r:id="rId618"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC185" r:id="rId619"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD185" r:id="rId620"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z186" r:id="rId621"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA186" r:id="rId622"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB186" r:id="rId623"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC186" r:id="rId624"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z187" r:id="rId625"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD187" r:id="rId626"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z188" r:id="rId627"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z189" r:id="rId628"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z190" r:id="rId629"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA190" r:id="rId630"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB190" r:id="rId631"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC190" r:id="rId632"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD190" r:id="rId633"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z191" r:id="rId634"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD191" r:id="rId635"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z192" r:id="rId636"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA192" r:id="rId637"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB192" r:id="rId638"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC192" r:id="rId639"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z193" r:id="rId640"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA193" r:id="rId641"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB193" r:id="rId642"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC193" r:id="rId643"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z194" r:id="rId644"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA194" r:id="rId645"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB194" r:id="rId646"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC194" r:id="rId647"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z195" r:id="rId648"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA195" r:id="rId649"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB195" r:id="rId650"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC195" r:id="rId651"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z196" r:id="rId652"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA196" r:id="rId653"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB196" r:id="rId654"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC196" r:id="rId655"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z197" r:id="rId656"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA197" r:id="rId657"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB197" r:id="rId658"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC197" r:id="rId659"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z198" r:id="rId660"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA198" r:id="rId661"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB198" r:id="rId662"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC198" r:id="rId663"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z199" r:id="rId664"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA199" r:id="rId665"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB199" r:id="rId666"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC199" r:id="rId667"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z200" r:id="rId668"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD200" r:id="rId669"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z201" r:id="rId670"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA201" r:id="rId671"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB201" r:id="rId672"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC201" r:id="rId673"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD201" r:id="rId674"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z22" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA22" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB22" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC22" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z23" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA23" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB23" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC23" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z24" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD24" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z25" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA25" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB25" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC25" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD25" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z26" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z27" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA27" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB27" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC27" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z28" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA28" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB28" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC28" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z29" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z30" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA30" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB30" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC30" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z31" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z32" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA32" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB32" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC32" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z33" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z34" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z35" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA35" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB35" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC35" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD35" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z36" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA36" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB36" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC36" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD36" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z37" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z38" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA38" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB38" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC38" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z39" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD39" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z40" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA40" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB40" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC40" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD40" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z41" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA41" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB41" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC41" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z42" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA42" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB42" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC42" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z43" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA43" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB43" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC43" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z44" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD44" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z45" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA45" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB45" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC45" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD45" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z46" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA46" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB46" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC46" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z47" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD47" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE47" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z48" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA48" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB48" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC48" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z49" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA49" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB49" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC49" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z50" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA50" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB50" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC50" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z51" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA51" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB51" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC51" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z52" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z53" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA53" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB53" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC53" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD53" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z54" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z55" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z56" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA56" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB56" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC56" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z57" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA57" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB57" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC57" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z58" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA58" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB58" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC58" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z59" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA59" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB59" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC59" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z60" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z61" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z62" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA62" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB62" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC62" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z63" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA63" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB63" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC63" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z64" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA64" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB64" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC64" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z65" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA65" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB65" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC65" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z66" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA66" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB66" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC66" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z67" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA67" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB67" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC67" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z68" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z69" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z70" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA70" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB70" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC70" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z71" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA71" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB71" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC71" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z72" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA72" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB72" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC72" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD72" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z73" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA73" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB73" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC73" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z74" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD74" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z75" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA75" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB75" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC75" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z76" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z77" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA77" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB77" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC77" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z78" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA78" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB78" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC78" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD78" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z79" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA79" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB79" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC79" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z80" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA80" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB80" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC80" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD80" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE80" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z81" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA81" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB81" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC81" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z82" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA82" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB82" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC82" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z83" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA83" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB83" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC83" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD83" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA84" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB84" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC84" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA85" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB85" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC85" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA86" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB86" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC86" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA87" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB87" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC87" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA88" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB88" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC88" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA89" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB89" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC89" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA90" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB90" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC90" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD90" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA91" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB91" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC91" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA92" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB92" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC92" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD92" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA93" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB93" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC93" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA94" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB94" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC94" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD96" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA97" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB97" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC97" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA98" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB98" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC98" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA100" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB100" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC100" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA101" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB101" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC101" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA102" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB102" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC102" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD102" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA103" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB103" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC103" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD103" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA104" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB104" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC104" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA105" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB105" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC105" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD105" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA106" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB106" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC106" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA107" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB107" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC107" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD107" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD108" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA110" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB110" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC110" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD111" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA113" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB113" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC113" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z115" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA115" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB115" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC115" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z116" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z117" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA117" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB117" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC117" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z118" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z119" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA119" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB119" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC119" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z120" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD120" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z121" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA121" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB121" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC121" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD121" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z122" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA122" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB122" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC122" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z123" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA123" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB123" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC123" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z124" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA124" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB124" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC124" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD124" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z125" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z126" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z127" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA127" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB127" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC127" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD127" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z128" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA128" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB128" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC128" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z129" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA129" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB129" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC129" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z130" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA130" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB130" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC130" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z131" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA131" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB131" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC131" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z132" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z133" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA133" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB133" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC133" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z134" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA134" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB134" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC134" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z135" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA135" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB135" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC135" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z136" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA136" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB136" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC136" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z137" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA137" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB137" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC137" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z138" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA138" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB138" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC138" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z139" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z140" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA140" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB140" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC140" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z141" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA141" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB141" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC141" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z142" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z143" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA143" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB143" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC143" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z144" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA144" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB144" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC144" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z145" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA145" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB145" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC145" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z146" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA146" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB146" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC146" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z147" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA147" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB147" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC147" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z148" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA148" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB148" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC148" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z149" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA149" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB149" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC149" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z150" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA150" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB150" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC150" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD150" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z151" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD151" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z152" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA152" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB152" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC152" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD152" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z153" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z154" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z155" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA155" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB155" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC155" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z156" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z157" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA157" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB157" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC157" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD157" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z158" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA158" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB158" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC158" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z159" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA159" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB159" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC159" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z160" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA160" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB160" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC160" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z161" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z162" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA162" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB162" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC162" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z163" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA163" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB163" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC163" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD163" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z164" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA164" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB164" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC164" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z165" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA165" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB165" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC165" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z166" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z167" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA167" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB167" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC167" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD167" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z168" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA168" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB168" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC168" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z169" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA169" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB169" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC169" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z170" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z171" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA171" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB171" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC171" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z172" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA172" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB172" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC172" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD172" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z173" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z174" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z175" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA175" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB175" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC175" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z176" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA176" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB176" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC176" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z177" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA177" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB177" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC177" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z178" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA178" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB178" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC178" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z179" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA179" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB179" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC179" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD179" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z180" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA180" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB180" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC180" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z181" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z182" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD182" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z183" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA183" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB183" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC183" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z184" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA184" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB184" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC184" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD184" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z185" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA185" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB185" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC185" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD185" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z186" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA186" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB186" r:id="rId613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC186" r:id="rId614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z187" r:id="rId615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD187" r:id="rId616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z188" r:id="rId617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z189" r:id="rId618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z190" r:id="rId619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA190" r:id="rId620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB190" r:id="rId621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC190" r:id="rId622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD190" r:id="rId623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z191" r:id="rId624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD191" r:id="rId625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z192" r:id="rId626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA192" r:id="rId627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB192" r:id="rId628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC192" r:id="rId629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z193" r:id="rId630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA193" r:id="rId631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB193" r:id="rId632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC193" r:id="rId633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z194" r:id="rId634"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA194" r:id="rId635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB194" r:id="rId636"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC194" r:id="rId637"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z195" r:id="rId638"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA195" r:id="rId639"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB195" r:id="rId640"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC195" r:id="rId641"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z196" r:id="rId642"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA196" r:id="rId643"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB196" r:id="rId644"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC196" r:id="rId645"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z197" r:id="rId646"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA197" r:id="rId647"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB197" r:id="rId648"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC197" r:id="rId649"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z198" r:id="rId650"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA198" r:id="rId651"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB198" r:id="rId652"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC198" r:id="rId653"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z199" r:id="rId654"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA199" r:id="rId655"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB199" r:id="rId656"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC199" r:id="rId657"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z200" r:id="rId658"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD200" r:id="rId659"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z201" r:id="rId660"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA201" r:id="rId661"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB201" r:id="rId662"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC201" r:id="rId663"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD201" r:id="rId664"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId675"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId665"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Replace outsider works with local voices: Senegal, Zimbabwe, Fiji, Guinea-Bissau, Samoa, St Kitts
- Senegal: Senghor, "Femme noire" (replaces Loti)
- Zimbabwe: Oliver Mtukudzi, "Svovi Yangu" (replaces Haggard)
- Fiji: "Isa Lei" (replaces Basil Thomson)
- Guinea-Bissau: Odete Semedo, Entre o Ser e o Amar (replaces Duarte)
- Samoa: "Le Teine Ea" (replaces R. L. Stevenson; moves to explore)
- Saint Kitts and Nevis: Infamus, "Love St Kitts" (replaces Grainger)

All listed under Poems to explore with description, history note and link.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -569,7 +569,7 @@
     <row r="2">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 118 paired passages • 77 unfilled</t>
+          <t>195 countries • 134 open-original leads • 9 historical versions • 52 not verified • 117 paired passages • 78 unfilled</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -9332,34 +9332,34 @@
       </c>
       <c r="D65" s="13" t="inlineStr">
         <is>
-          <t>Raluve</t>
+          <t>Isa Lei</t>
         </is>
       </c>
       <c r="E65" s="13" t="inlineStr">
         <is>
-          <t>Raluve (character's name; retained)</t>
+          <t>Isa Lei (farewell song)</t>
         </is>
       </c>
       <c r="F65" s="13" t="n"/>
       <c r="G65" s="13" t="n"/>
       <c r="H65" s="13" t="inlineStr">
         <is>
-          <t>Basil Thomson (1861–1939)</t>
+          <t>Traditional Fijian song</t>
         </is>
       </c>
       <c r="I65" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J65" s="13" t="inlineStr">
         <is>
-          <t>Named short story (full text)</t>
+          <t>Named work</t>
         </is>
       </c>
       <c r="K65" s="13" t="inlineStr">
         <is>
-          <t>Short story</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="L65" s="13" t="inlineStr">
@@ -9367,12 +9367,10 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M65" s="14" t="n">
-        <v>1894</v>
-      </c>
+      <c r="M65" s="14" t="n"/>
       <c r="N65" s="13" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Fijian</t>
         </is>
       </c>
       <c r="O65" s="13" t="n"/>
@@ -9388,64 +9386,45 @@
       </c>
       <c r="R65" s="13" t="inlineStr">
         <is>
-          <t>Published in South Sea Yarns, Edinburgh and London, 1894</t>
-        </is>
-      </c>
-      <c r="S65" s="13" t="inlineStr">
-        <is>
-          <t>William Blackwood and Sons, 1894, pp.68–110</t>
-        </is>
-      </c>
+          <t>Early twentieth century; origins disputed</t>
+        </is>
+      </c>
+      <c r="S65" s="13" t="n"/>
       <c r="T65" s="13" t="inlineStr">
         <is>
-          <t>Vere and the Fijian woman Raluve fall in love and meet secretly while confronting colonial racial barriers and family opposition.</t>
+          <t>Fiji’s best-known song, a tender farewell sung to a departing loved one, now sung whenever visitors leave the islands.</t>
         </is>
       </c>
       <c r="U65" s="13" t="inlineStr">
         <is>
-          <t>Original English story in South Sea Yarns (1894), chapter Raluve. National Library of New Zealand confirms author dates; Royal Anthropological Institute records Fiji residence.</t>
-        </is>
-      </c>
-      <c r="V65" s="13" t="inlineStr">
-        <is>
-          <t>Raluve, pp.68–110; love and meeting scenes especially pp.89–94</t>
-        </is>
-      </c>
+          <t>Traditional song</t>
+        </is>
+      </c>
+      <c r="V65" s="13" t="n"/>
       <c r="W65" s="13" t="inlineStr">
         <is>
-          <t>British colonial administrator writing fiction set in Fiji, not an indigenous Fijian-authored work. The text contains racial stereotypes and unequal colonial assumptions. Reuse original prose; modern editions and illustrations require separate assessment.</t>
+          <t>British colonial administrator writing fiction set in Fiji, not an indigenous Fijian-authored work. The text contains racial stereotypes and unequal colonial assumptions. Reuse original prose; modern editions and illustrations require separate assessment.
+Work changed (29 October 2026): the earlier work, by an outsider writing about the country, is replaced by a work by a local poet or musician. Listed with a description and link only.</t>
         </is>
       </c>
       <c r="X65" s="13" t="inlineStr">
         <is>
-          <t>Historical original composition; author died 1939, beyond the standard life-plus-70 term. Reuse the underlying historical original only, excluding modern translations, editorial matter, images, adaptations and recordings. Publication history and territorial exceptions should be checked for the edition used.</t>
+          <t>Origins and authorship disputed. Listed with a link.</t>
         </is>
       </c>
       <c r="Y65" s="13" t="inlineStr">
         <is>
-          <t>Work-specific text, date and provenance sources checked29October2026.</t>
+          <t>Wikipedia: Isa Lei</t>
         </is>
       </c>
       <c r="Z65" s="11" t="inlineStr">
         <is>
-          <t>Work / text</t>
-        </is>
-      </c>
-      <c r="AA65" s="11" t="inlineStr">
-        <is>
-          <t>Rights / catalogue</t>
-        </is>
-      </c>
-      <c r="AB65" s="11" t="inlineStr">
-        <is>
-          <t>Date / edition</t>
-        </is>
-      </c>
-      <c r="AC65" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country</t>
-        </is>
-      </c>
+          <t>Read about it</t>
+        </is>
+      </c>
+      <c r="AA65" s="11" t="n"/>
+      <c r="AB65" s="11" t="n"/>
+      <c r="AC65" s="11" t="n"/>
       <c r="AD65" s="11" t="n"/>
       <c r="AE65" s="11" t="n"/>
     </row>
@@ -11059,34 +11038,34 @@
       </c>
       <c r="D77" s="13" t="inlineStr">
         <is>
-          <t>Auá: novela negra</t>
+          <t>Entre o Ser e o Amar</t>
         </is>
       </c>
       <c r="E77" s="13" t="inlineStr">
         <is>
-          <t>Auá: A Black Novel (Auá is a character's name; historical subtitle)</t>
+          <t>Between Being and Loving</t>
         </is>
       </c>
       <c r="F77" s="13" t="n"/>
       <c r="G77" s="13" t="n"/>
       <c r="H77" s="13" t="inlineStr">
         <is>
-          <t>Fausto Duarte (1902/1903–1953)</t>
+          <t>Odete Semedo (born 1959)</t>
         </is>
       </c>
       <c r="I77" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J77" s="13" t="inlineStr">
         <is>
-          <t>Named novel (excerpts in scholarly study)</t>
+          <t>Named poetry collection</t>
         </is>
       </c>
       <c r="K77" s="13" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Poetry</t>
         </is>
       </c>
       <c r="L77" s="13" t="inlineStr">
@@ -11095,11 +11074,11 @@
         </is>
       </c>
       <c r="M77" s="14" t="n">
-        <v>1934</v>
+        <v>1996</v>
       </c>
       <c r="N77" s="13" t="inlineStr">
         <is>
-          <t>Portuguese, with Fula and other local expressions</t>
+          <t>Portuguese and Guinean Kriol</t>
         </is>
       </c>
       <c r="O77" s="13" t="n"/>
@@ -11115,64 +11094,45 @@
       </c>
       <c r="R77" s="13" t="inlineStr">
         <is>
-          <t>First published Lisbon, 1934</t>
-        </is>
-      </c>
-      <c r="S77" s="13" t="inlineStr">
-        <is>
-          <t>Historical novel; excerpts and analysis in UNILAB study (2018)</t>
-        </is>
-      </c>
+          <t>1996</t>
+        </is>
+      </c>
+      <c r="S77" s="13" t="n"/>
       <c r="T77" s="13" t="inlineStr">
         <is>
-          <t>The marriage of Malam and Auá, her attachment to Abdulai, and Malam’s jealousy and longing shape a tragic story set in Guinea-Bissau.</t>
+          <t>Odete Semedo’s first collection of poems, written in both Portuguese and Guinean Kriol, a choice she calls “double belonging”.</t>
         </is>
       </c>
       <c r="U77" s="13" t="inlineStr">
         <is>
-          <t>UNILAB, Trindade Gomes Nanque, Auá: a representação da personagem feminina Fula no romance colonial de Fausto Duarte, 2018; original work published 1934. UNL thesis p.61 records author dates and residence in Guinea.</t>
-        </is>
-      </c>
-      <c r="V77" s="13" t="inlineStr">
-        <is>
-          <t>UNILAB study, discussion and quotations of Malam, Auá and Abdulai</t>
-        </is>
-      </c>
+          <t>Entre o Ser e o Amar (1996)</t>
+        </is>
+      </c>
+      <c r="V77" s="13" t="n"/>
       <c r="W77" s="13" t="inlineStr">
         <is>
-          <t>Cape Verde-born author lived and worked in Guinea; country association is residence and the novel’s Guinean setting. Colonial stereotypes, sexual violence and revenge require context. Modern scholarship is excluded. Aquilino Ribeiro’s preface and the cover photograph have separate rights and are excluded.</t>
+          <t>Cape Verde-born author lived and worked in Guinea; country association is residence and the novel’s Guinean setting. Colonial stereotypes, sexual violence and revenge require context. Modern scholarship is excluded. Aquilino Ribeiro’s preface and the cover photograph have separate rights and are excluded.
+Work changed (29 October 2026): the earlier work, by an outsider writing about the country, is replaced by a work by a local poet or musician. Listed with a description and link only.</t>
         </is>
       </c>
       <c r="X77" s="13" t="inlineStr">
         <is>
-          <t>Historical original composition; author died 1953, beyond the standard life-plus-70 term. Reuse the underlying historical original only, excluding modern translations, editorial matter, images, adaptations and recordings. Publication history and territorial exceptions should be checked for the edition used.</t>
+          <t>In copyright (living author). Not reproduced; listed with a link.</t>
         </is>
       </c>
       <c r="Y77" s="13" t="inlineStr">
         <is>
-          <t>Work-specific text, date and provenance sources checked29October2026.</t>
+          <t>Wikipedia: Odete Semedo</t>
         </is>
       </c>
       <c r="Z77" s="11" t="inlineStr">
         <is>
-          <t>Work / text</t>
-        </is>
-      </c>
-      <c r="AA77" s="11" t="inlineStr">
-        <is>
-          <t>Rights / catalogue</t>
-        </is>
-      </c>
-      <c r="AB77" s="11" t="inlineStr">
-        <is>
-          <t>Date / edition</t>
-        </is>
-      </c>
-      <c r="AC77" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country</t>
-        </is>
-      </c>
+          <t>Read about it</t>
+        </is>
+      </c>
+      <c r="AA77" s="11" t="n"/>
+      <c r="AB77" s="11" t="n"/>
+      <c r="AC77" s="11" t="n"/>
       <c r="AD77" s="11" t="n"/>
       <c r="AE77" s="11" t="n"/>
     </row>
@@ -22557,34 +22517,34 @@
       </c>
       <c r="D152" s="13" t="inlineStr">
         <is>
-          <t>Bryan and Pereene. A West Indian Ballad</t>
+          <t>Love St Kitts</t>
         </is>
       </c>
       <c r="E152" s="13" t="inlineStr">
         <is>
-          <t>Bryan and Pereene. A West Indian Ballad</t>
+          <t>Love St Kitts</t>
         </is>
       </c>
       <c r="F152" s="13" t="n"/>
       <c r="G152" s="13" t="n"/>
       <c r="H152" s="13" t="inlineStr">
         <is>
-          <t>James Grainger (c.1721–1766)</t>
+          <t>Infamus</t>
         </is>
       </c>
       <c r="I152" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J152" s="13" t="inlineStr">
         <is>
-          <t>Named work (text)</t>
+          <t>Named work</t>
         </is>
       </c>
       <c r="K152" s="13" t="inlineStr">
         <is>
-          <t>Poetry</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="L152" s="13" t="inlineStr">
@@ -22592,9 +22552,7 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M152" s="14" t="n">
-        <v>1765</v>
-      </c>
+      <c r="M152" s="14" t="n"/>
       <c r="N152" s="13" t="inlineStr">
         <is>
           <t>English</t>
@@ -22613,69 +22571,46 @@
       </c>
       <c r="R152" s="13" t="inlineStr">
         <is>
-          <t>Published in Percy’s Reliques, 1765; linked source edition 1767</t>
-        </is>
-      </c>
-      <c r="S152" s="13" t="inlineStr">
-        <is>
-          <t>Historical work reproduced in linked digital source; modern editorial material is separate</t>
-        </is>
-      </c>
+          <t>Twenty-first century</t>
+        </is>
+      </c>
+      <c r="S152" s="13" t="n"/>
       <c r="T152" s="13" t="inlineStr">
         <is>
-          <t>Separated lovers eagerly anticipate reunion, but Bryan is killed by a shark as he swims to shore and Pereene dies of grief.</t>
+          <t>A song of love for St Kitts by the Kittitian artist Infamus.</t>
         </is>
       </c>
       <c r="U152" s="13" t="inlineStr">
         <is>
-          <t>Eighteenth-Century Poetry Archive supplies text and Bodleian facsimile. Percy’s historical note places the anecdote on St Christopher; Grainger lived and died on St Kitts.</t>
-        </is>
-      </c>
-      <c r="V152" s="13" t="inlineStr">
-        <is>
-          <t>Complete 56-line ballad; lines 5–40 concern fidelity and anticipated reunion</t>
-        </is>
-      </c>
+          <t>Official music video (TRUCAPO channel, YouTube)</t>
+        </is>
+      </c>
+      <c r="V152" s="13" t="n"/>
       <c r="W152" s="13" t="inlineStr">
         <is>
-          <t>Scottish-born colonial resident author, not an Indigenous island voice. Graphic tragic ending and colonial racial representation. First-publication date should not be confused with the linked 1767 anthology.</t>
+          <t>Scottish-born colonial resident author, not an Indigenous island voice. Graphic tragic ending and colonial racial representation. First-publication date should not be confused with the linked 1767 anthology.
+Work changed (29 October 2026): James Grainger’s ballad, by a Scottish plantation doctor, is replaced by a song by a Kittitian artist, chosen by the project. Listed with a description and link only.</t>
         </is>
       </c>
       <c r="X152" s="13" t="inlineStr">
         <is>
-          <t>Historical original text: standard life-plus-70 term has expired; author died 1766. Assessment excludes modern translations, commentary, editorial alterations, musical settings and recordings. Territorial and unusual publication-history exceptions are not comprehensively assessed.</t>
+          <t>In copyright. Not reproduced; listed with a link.</t>
         </is>
       </c>
       <c r="Y152" s="13" t="inlineStr">
         <is>
-          <t>Eighteenth-Century Poetry Archive supplies text and Bodleian facsimile. Percy’s historical note places the anecdote on St Christopher; Grainger lived and died on St Kitts.</t>
+          <t>YouTube: Infamus – Love St Kitts (official music video)</t>
         </is>
       </c>
       <c r="Z152" s="11" t="inlineStr">
         <is>
-          <t>Work / source text</t>
-        </is>
-      </c>
-      <c r="AA152" s="11" t="inlineStr">
-        <is>
-          <t>Reuse basis / copyright duration</t>
-        </is>
-      </c>
-      <c r="AB152" s="11" t="inlineStr">
-        <is>
-          <t>Date / edition evidence</t>
-        </is>
-      </c>
-      <c r="AC152" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country evidence</t>
-        </is>
-      </c>
-      <c r="AD152" s="11" t="inlineStr">
-        <is>
-          <t>Additional evidence</t>
-        </is>
-      </c>
+          <t>Watch the video</t>
+        </is>
+      </c>
+      <c r="AA152" s="11" t="n"/>
+      <c r="AB152" s="11" t="n"/>
+      <c r="AC152" s="11" t="n"/>
+      <c r="AD152" s="11" t="n"/>
       <c r="AE152" s="11" t="n"/>
     </row>
     <row r="153" ht="43.5" customHeight="1" s="17">
@@ -22914,70 +22849,34 @@
       </c>
       <c r="D155" s="13" t="inlineStr">
         <is>
-          <t>My Wife (Songs of Travel, XXVI)</t>
+          <t>Le Teine Ea</t>
         </is>
       </c>
       <c r="E155" s="13" t="inlineStr">
         <is>
-          <t>My Wife (Songs of Travel, XXVI)</t>
-        </is>
-      </c>
-      <c r="F155" s="13" t="inlineStr">
-        <is>
-          <t>Trusty, dusky, vivid, true,
-With eyes of gold and bramble-dew,
-Steel-true and blade-straight,
-The great artificer
-Made my mate.
-Honour, anger, valour, fire;
-A love that life could never tire,
-Death quench or evil stir,
-The mighty master
-Gave to her.
-Teacher, tender, comrade, wife,
-A fellow-farer true through life,
-Heart-whole and soul-free
-The august father
-Gave to me.</t>
-        </is>
-      </c>
-      <c r="G155" s="13" t="inlineStr">
-        <is>
-          <t>Trusty, dusky, vivid, true,
-With eyes of gold and bramble-dew,
-Steel-true and blade-straight,
-The great artificer
-Made my mate.
-Honour, anger, valour, fire;
-A love that life could never tire,
-Death quench or evil stir,
-The mighty master
-Gave to her.
-Teacher, tender, comrade, wife,
-A fellow-farer true through life,
-Heart-whole and soul-free
-The august father
-Gave to me.</t>
-        </is>
-      </c>
+          <t>Dream Girl</t>
+        </is>
+      </c>
+      <c r="F155" s="13" t="n"/>
+      <c r="G155" s="13" t="n"/>
       <c r="H155" s="13" t="inlineStr">
         <is>
-          <t>Robert Louis Stevenson (1850–1894)</t>
+          <t>Traditional Samoan song</t>
         </is>
       </c>
       <c r="I155" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J155" s="13" t="inlineStr">
         <is>
-          <t>Named poem (full text)</t>
+          <t>Named work</t>
         </is>
       </c>
       <c r="K155" s="13" t="inlineStr">
         <is>
-          <t>Poetry</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="L155" s="13" t="inlineStr">
@@ -22985,12 +22884,10 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M155" s="14" t="n">
-        <v>1896</v>
-      </c>
+      <c r="M155" s="14" t="n"/>
       <c r="N155" s="13" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Samoan</t>
         </is>
       </c>
       <c r="O155" s="13" t="n"/>
@@ -23006,65 +22903,46 @@
       </c>
       <c r="R155" s="13" t="inlineStr">
         <is>
-          <t>Written before December 1894; collected posthumously in Songs of Travel, 1896</t>
-        </is>
-      </c>
-      <c r="S155" s="13" t="inlineStr">
-        <is>
-          <t>Songs of Travel and Other Verses, London: Chatto &amp; Windus, 1896, p.39</t>
-        </is>
-      </c>
+          <t>Twentieth century</t>
+        </is>
+      </c>
+      <c r="S155" s="13" t="n"/>
       <c r="T155" s="13" t="inlineStr">
         <is>
-          <t>An affirmative poem praising his wife Fanny as a lifelong companion whose love survives adversity and death.</t>
+          <t>A popular Samoan song whose title means “Dream Girl”.</t>
         </is>
       </c>
       <c r="U155" s="13" t="inlineStr">
         <is>
-          <t>Full English poem in Project Gutenberg, Songs of Travel, XXVI. The 1896 edition’s contents identify p.39. National Library of New Zealand documents Stevenson’s residence at Vailima, Samoa, from 1889 to 1894.</t>
-        </is>
-      </c>
-      <c r="V155" s="13" t="inlineStr">
-        <is>
-          <t>XXVI — My Wife, beginning Trusty, dusky, vivid, true</t>
-        </is>
-      </c>
+          <t>Huapala song archive</t>
+        </is>
+      </c>
+      <c r="V155" s="13" t="n"/>
       <c r="W155" s="13" t="inlineStr">
         <is>
           <t>Country link is the Scottish author’s established residence in Samoa, not Samoan origin or language. Exact place and date of composition are not established. This is an original English poem, not a translation of Samoan oral tradition.
-English passage: Original English text; not a translation. Complete poem,15 lines; Scottish author resident in Samoa, as qualified in country notes. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+English passage: Original English text; not a translation. Complete poem,15 lines; Scottish author resident in Samoa, as qualified in country notes. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Work changed (29 October 2026): the earlier work, by an outsider writing about the country, is replaced by a work by a local poet or musician. Listed with a description and link only.</t>
         </is>
       </c>
       <c r="X155" s="13" t="inlineStr">
         <is>
-          <t>Historical original composition; author died 1894, beyond the standard life-plus-70 term. Reuse the underlying historical original only, excluding modern translations, editorial matter, images, adaptations and recordings. Publication history and territorial exceptions should be checked for the edition used.</t>
+          <t>Not reproduced; listed with a link.</t>
         </is>
       </c>
       <c r="Y155" s="13" t="inlineStr">
         <is>
-          <t>Work-specific text, date and provenance sources checked29October2026.</t>
+          <t>Huapala: Le Teine Ea</t>
         </is>
       </c>
       <c r="Z155" s="11" t="inlineStr">
         <is>
-          <t>Work / text</t>
-        </is>
-      </c>
-      <c r="AA155" s="11" t="inlineStr">
-        <is>
-          <t>Rights / catalogue</t>
-        </is>
-      </c>
-      <c r="AB155" s="11" t="inlineStr">
-        <is>
-          <t>Date / edition</t>
-        </is>
-      </c>
-      <c r="AC155" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country</t>
-        </is>
-      </c>
+          <t>Read about it</t>
+        </is>
+      </c>
+      <c r="AA155" s="11" t="n"/>
+      <c r="AB155" s="11" t="n"/>
+      <c r="AC155" s="11" t="n"/>
       <c r="AD155" s="11" t="n"/>
       <c r="AE155" s="11" t="n"/>
     </row>
@@ -23506,34 +23384,34 @@
       </c>
       <c r="D159" s="13" t="inlineStr">
         <is>
-          <t>Le Roman d’un spahi</t>
+          <t>Femme noire</t>
         </is>
       </c>
       <c r="E159" s="13" t="inlineStr">
         <is>
-          <t>The Story of a Spahi (a colonial cavalry soldier)</t>
+          <t>Black Woman</t>
         </is>
       </c>
       <c r="F159" s="13" t="n"/>
       <c r="G159" s="13" t="n"/>
       <c r="H159" s="13" t="inlineStr">
         <is>
-          <t>Pierre Loti (1850–1923)</t>
+          <t>Léopold Sédar Senghor (1906–2001)</t>
         </is>
       </c>
       <c r="I159" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J159" s="13" t="inlineStr">
         <is>
-          <t>Named literary work (full original-language text; setting association)</t>
+          <t>Named poem</t>
         </is>
       </c>
       <c r="K159" s="13" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Poetry</t>
         </is>
       </c>
       <c r="L159" s="13" t="inlineStr">
@@ -23542,7 +23420,7 @@
         </is>
       </c>
       <c r="M159" s="14" t="n">
-        <v>1881</v>
+        <v>1945</v>
       </c>
       <c r="N159" s="13" t="inlineStr">
         <is>
@@ -23562,64 +23440,45 @@
       </c>
       <c r="R159" s="13" t="inlineStr">
         <is>
-          <t>First published1881; linked historical edition1910</t>
-        </is>
-      </c>
-      <c r="S159" s="13" t="inlineStr">
-        <is>
-          <t>Calmann-Lévy1910, original French text</t>
-        </is>
-      </c>
+          <t>1945 (Chants d’ombre)</t>
+        </is>
+      </c>
+      <c r="S159" s="13" t="n"/>
       <c r="T159" s="13" t="inlineStr">
         <is>
-          <t>French soldier Jean Peyral and Senegalese Fatou-Gaye fall in love in Senegal. Their relationship ends in death, suicide and the death of their child; tragic romantic love, not an affirmative model.</t>
+          <t>A praise poem to a Black woman, celebrating her beauty as the beauty of Africa itself; Senghor’s best-known poem.</t>
         </is>
       </c>
       <c r="U159" s="13" t="inlineStr">
         <is>
-          <t>An original French novel by a visiting French naval officer, associated with Senegal through its setting and Senegalese heroine. It is not an indigenous Senegalese voice. Institut Français catalogue confirms the love plot and Senegal setting; Wikisource supplies a historical French edition and1881 facsimile.</t>
-        </is>
-      </c>
-      <c r="V159" s="13" t="inlineStr">
-        <is>
-          <t>Full novel; use historical French text, not a later adaptation</t>
-        </is>
-      </c>
+          <t>Chants d’ombre (1945)</t>
+        </is>
+      </c>
+      <c r="V159" s="13" t="n"/>
       <c r="W159" s="13" t="inlineStr">
         <is>
-          <t>Country association is setting and author’s experience there, rather than nationality. Colonial racial stereotypes and unequal power shape the romance. The plot includes suicide and infanticide. Select critically; illustrations and later editions require separate assessment.</t>
+          <t>Country association is setting and author’s experience there, rather than nationality. Colonial racial stereotypes and unequal power shape the romance. The plot includes suicide and infanticide. Select critically; illustrations and later editions require separate assessment.
+Work changed (29 October 2026): the earlier work, by an outsider writing about the country, is replaced by a work by a local poet or musician. Listed with a description and link only.</t>
         </is>
       </c>
       <c r="X159" s="13" t="inlineStr">
         <is>
-          <t>Original French prose published1881; Loti died1923, beyond standard life-plus-70 and US publication terms. Reuse the historical text only; modern translations, editorial matter, cover art and adaptations are separate.</t>
+          <t>In copyright (author died 2001). Not reproduced; listed with a link.</t>
         </is>
       </c>
       <c r="Y159" s="13" t="inlineStr">
         <is>
-          <t>Work-specific text, date and provenance sources checked29October2026.</t>
+          <t>La langue française: commentary on “Femme noire”</t>
         </is>
       </c>
       <c r="Z159" s="11" t="inlineStr">
         <is>
-          <t>Work / text</t>
-        </is>
-      </c>
-      <c r="AA159" s="11" t="inlineStr">
-        <is>
-          <t>Rights / catalogue</t>
-        </is>
-      </c>
-      <c r="AB159" s="11" t="inlineStr">
-        <is>
-          <t>Date / edition</t>
-        </is>
-      </c>
-      <c r="AC159" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country</t>
-        </is>
-      </c>
+          <t>Read about it</t>
+        </is>
+      </c>
+      <c r="AA159" s="11" t="n"/>
+      <c r="AB159" s="11" t="n"/>
+      <c r="AC159" s="11" t="n"/>
       <c r="AD159" s="11" t="n"/>
       <c r="AE159" s="11" t="n"/>
     </row>
@@ -29610,34 +29469,34 @@
       </c>
       <c r="D201" s="13" t="inlineStr">
         <is>
-          <t>Benita: An African Romance</t>
+          <t>Svovi Yangu</t>
         </is>
       </c>
       <c r="E201" s="13" t="inlineStr">
         <is>
-          <t>Benita: An African Romance</t>
+          <t>My Svovi (My Darling)</t>
         </is>
       </c>
       <c r="F201" s="13" t="n"/>
       <c r="G201" s="13" t="n"/>
       <c r="H201" s="13" t="inlineStr">
         <is>
-          <t>H. Rider Haggard (1856–1925)</t>
+          <t>Oliver Mtukudzi (1952–2019)</t>
         </is>
       </c>
       <c r="I201" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J201" s="13" t="inlineStr">
         <is>
-          <t>Named literary work (full original-language text; setting association)</t>
+          <t>Named work</t>
         </is>
       </c>
       <c r="K201" s="13" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="L201" s="13" t="inlineStr">
@@ -29645,12 +29504,10 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M201" s="14" t="n">
-        <v>1906</v>
-      </c>
+      <c r="M201" s="14" t="n"/>
       <c r="N201" s="13" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Shona</t>
         </is>
       </c>
       <c r="O201" s="13" t="n"/>
@@ -29666,69 +29523,46 @@
       </c>
       <c r="R201" s="13" t="inlineStr">
         <is>
-          <t>Book edition1906; earlier serialization1903–1904</t>
-        </is>
-      </c>
-      <c r="S201" s="13" t="inlineStr">
-        <is>
-          <t>Historical English novel; Project Gutenberg2761</t>
-        </is>
-      </c>
+          <t>Twentieth century</t>
+        </is>
+      </c>
+      <c r="S201" s="13" t="n"/>
       <c r="T201" s="13" t="inlineStr">
         <is>
-          <t>Benita Clifford and Robert Seymour are reunited after shipwreck and danger. The closing chapters contrast their love with the treasure hunt and Jacob Meyer’s possessive obsession.</t>
+          <t>Mtukudzi’s love song for his wife, Daisy: his devotion to her and his sorrow at being far from the love of his life.</t>
         </is>
       </c>
       <c r="U201" s="13" t="inlineStr">
         <is>
-          <t>British colonial adventure fiction associated with Zimbabwe through the fictional Bambatse ruins and Khumalo/Matabele kingdom setting. The scholarly chapter Great Zimbabwe in Rhodesian Fiction discusses its Zimbabwe landscape; Cambridge includes it in central-African literary history. It is not Zimbabwean indigenous authorship.</t>
-        </is>
-      </c>
-      <c r="V201" s="13" t="inlineStr">
-        <is>
-          <t>XXIII, Benita Gives Her Answer; XXIV, The True Gold</t>
-        </is>
-      </c>
+          <t>Recording by Oliver Mtukudzi</t>
+        </is>
+      </c>
+      <c r="V201" s="13" t="n"/>
       <c r="W201" s="13" t="inlineStr">
         <is>
-          <t>Foreign British author; country association is the imagined Zimbabwe setting. Colonial stereotypes, antisemitism and coercive obsession occur in the novel. The mutual love of Benita and Robert is distinct from Meyer’s pursuit. Use original text critically.</t>
+          <t>Foreign British author; country association is the imagined Zimbabwe setting. Colonial stereotypes, antisemitism and coercive obsession occur in the novel. The mutual love of Benita and Robert is distinct from Meyer’s pursuit. Use original text critically.
+Work changed (29 October 2026): the earlier work, by an outsider writing about the country, is replaced by a work by a local poet or musician. Listed with a description and link only.</t>
         </is>
       </c>
       <c r="X201" s="13" t="inlineStr">
         <is>
-          <t>Original English text published1906 and public domain in the USA; author died1925, beyond standard life-plus-70. New editorial work, translations, art and adaptations are excluded.</t>
+          <t>In copyright. Not reproduced; listed with a link.</t>
         </is>
       </c>
       <c r="Y201" s="13" t="inlineStr">
         <is>
-          <t>Work-specific text, date and provenance sources checked29October2026.</t>
+          <t>African Arguments: tribute to Oliver Mtukudzi</t>
         </is>
       </c>
       <c r="Z201" s="11" t="inlineStr">
         <is>
-          <t>Work / text</t>
-        </is>
-      </c>
-      <c r="AA201" s="11" t="inlineStr">
-        <is>
-          <t>Rights / catalogue</t>
-        </is>
-      </c>
-      <c r="AB201" s="11" t="inlineStr">
-        <is>
-          <t>Date / edition</t>
-        </is>
-      </c>
-      <c r="AC201" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country</t>
-        </is>
-      </c>
-      <c r="AD201" s="11" t="inlineStr">
-        <is>
-          <t>Additional evidence</t>
-        </is>
-      </c>
+          <t>Read about it</t>
+        </is>
+      </c>
+      <c r="AA201" s="11" t="n"/>
+      <c r="AB201" s="11" t="n"/>
+      <c r="AC201" s="11" t="n"/>
+      <c r="AD201" s="11" t="n"/>
       <c r="AE201" s="11" t="n"/>
     </row>
   </sheetData>
@@ -29923,484 +29757,464 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB64" r:id="rId188"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC64" r:id="rId189"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z65" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA65" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB65" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC65" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z66" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA66" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB66" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC66" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z67" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA67" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB67" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC67" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z68" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z69" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z70" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA70" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB70" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC70" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z71" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA71" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB71" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC71" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z72" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA72" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB72" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC72" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD72" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z73" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA73" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB73" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC73" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z74" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD74" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z75" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA75" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB75" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC75" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z76" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z77" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA77" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB77" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC77" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z78" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA78" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB78" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC78" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD78" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z79" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA79" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB79" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC79" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z80" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA80" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB80" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC80" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD80" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE80" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z81" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA81" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB81" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC81" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z82" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA82" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB82" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC82" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z83" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA83" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB83" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC83" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD83" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA84" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB84" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC84" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA85" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB85" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC85" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA86" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB86" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC86" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA87" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB87" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC87" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA88" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB88" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC88" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA89" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB89" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC89" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA90" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB90" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC90" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD90" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA91" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB91" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC91" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA92" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB92" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC92" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD92" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA93" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB93" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC93" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA94" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB94" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC94" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD96" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA97" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB97" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC97" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA98" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB98" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC98" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA100" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB100" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC100" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA101" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB101" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC101" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA102" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB102" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC102" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD102" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA103" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB103" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC103" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD103" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA104" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB104" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC104" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA105" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB105" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC105" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD105" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA106" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB106" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC106" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA107" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB107" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC107" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD107" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD108" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA110" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB110" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC110" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD111" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA113" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB113" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC113" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z115" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA115" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB115" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC115" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z116" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z117" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA117" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB117" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC117" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z118" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z119" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA119" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB119" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC119" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z120" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD120" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z121" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA121" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB121" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC121" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD121" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z122" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA122" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB122" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC122" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z123" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA123" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB123" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC123" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z124" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA124" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB124" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC124" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD124" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z125" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z126" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z127" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA127" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB127" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC127" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD127" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z128" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA128" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB128" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC128" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z129" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA129" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB129" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC129" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z130" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA130" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB130" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC130" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z131" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA131" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB131" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC131" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z132" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z133" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA133" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB133" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC133" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z134" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA134" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB134" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC134" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z135" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA135" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB135" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC135" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z136" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA136" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB136" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC136" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z137" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA137" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB137" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC137" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z138" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA138" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB138" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC138" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z139" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z140" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA140" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB140" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC140" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z141" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA141" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB141" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC141" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z142" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z143" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA143" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB143" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC143" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z144" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA144" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB144" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC144" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z145" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA145" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB145" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC145" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z146" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA146" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB146" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC146" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z147" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA147" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB147" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC147" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z148" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA148" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB148" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC148" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z149" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA149" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB149" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC149" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z150" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA150" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB150" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC150" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD150" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z151" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD151" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z152" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA152" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB152" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC152" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD152" r:id="rId500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z153" r:id="rId501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z154" r:id="rId502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z155" r:id="rId503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA155" r:id="rId504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB155" r:id="rId505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC155" r:id="rId506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z156" r:id="rId507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z157" r:id="rId508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA157" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB157" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC157" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD157" r:id="rId512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z158" r:id="rId513"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA158" r:id="rId514"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB158" r:id="rId515"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC158" r:id="rId516"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z159" r:id="rId517"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA159" r:id="rId518"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB159" r:id="rId519"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC159" r:id="rId520"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z160" r:id="rId521"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA160" r:id="rId522"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB160" r:id="rId523"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC160" r:id="rId524"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z161" r:id="rId525"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z162" r:id="rId526"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA162" r:id="rId527"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB162" r:id="rId528"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC162" r:id="rId529"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z163" r:id="rId530"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA163" r:id="rId531"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB163" r:id="rId532"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC163" r:id="rId533"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD163" r:id="rId534"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z164" r:id="rId535"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA164" r:id="rId536"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB164" r:id="rId537"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC164" r:id="rId538"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z165" r:id="rId539"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA165" r:id="rId540"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB165" r:id="rId541"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC165" r:id="rId542"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z166" r:id="rId543"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z167" r:id="rId544"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA167" r:id="rId545"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB167" r:id="rId546"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC167" r:id="rId547"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD167" r:id="rId548"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z168" r:id="rId549"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA168" r:id="rId550"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB168" r:id="rId551"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC168" r:id="rId552"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z169" r:id="rId553"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA169" r:id="rId554"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB169" r:id="rId555"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC169" r:id="rId556"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z170" r:id="rId557"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z171" r:id="rId558"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA171" r:id="rId559"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB171" r:id="rId560"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC171" r:id="rId561"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z172" r:id="rId562"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA172" r:id="rId563"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB172" r:id="rId564"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC172" r:id="rId565"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD172" r:id="rId566"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z173" r:id="rId567"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z174" r:id="rId568"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z175" r:id="rId569"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA175" r:id="rId570"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB175" r:id="rId571"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC175" r:id="rId572"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z176" r:id="rId573"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA176" r:id="rId574"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB176" r:id="rId575"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC176" r:id="rId576"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z177" r:id="rId577"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA177" r:id="rId578"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB177" r:id="rId579"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC177" r:id="rId580"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z178" r:id="rId581"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA178" r:id="rId582"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB178" r:id="rId583"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC178" r:id="rId584"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z179" r:id="rId585"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA179" r:id="rId586"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB179" r:id="rId587"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC179" r:id="rId588"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD179" r:id="rId589"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z180" r:id="rId590"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA180" r:id="rId591"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB180" r:id="rId592"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC180" r:id="rId593"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z181" r:id="rId594"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z182" r:id="rId595"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD182" r:id="rId596"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z183" r:id="rId597"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA183" r:id="rId598"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB183" r:id="rId599"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC183" r:id="rId600"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z184" r:id="rId601"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA184" r:id="rId602"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB184" r:id="rId603"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC184" r:id="rId604"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD184" r:id="rId605"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z185" r:id="rId606"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA185" r:id="rId607"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB185" r:id="rId608"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC185" r:id="rId609"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD185" r:id="rId610"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z186" r:id="rId611"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA186" r:id="rId612"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB186" r:id="rId613"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC186" r:id="rId614"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z187" r:id="rId615"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD187" r:id="rId616"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z188" r:id="rId617"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z189" r:id="rId618"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z190" r:id="rId619"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA190" r:id="rId620"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB190" r:id="rId621"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC190" r:id="rId622"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD190" r:id="rId623"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z191" r:id="rId624"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD191" r:id="rId625"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z192" r:id="rId626"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA192" r:id="rId627"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB192" r:id="rId628"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC192" r:id="rId629"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z193" r:id="rId630"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA193" r:id="rId631"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB193" r:id="rId632"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC193" r:id="rId633"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z194" r:id="rId634"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA194" r:id="rId635"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB194" r:id="rId636"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC194" r:id="rId637"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z195" r:id="rId638"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA195" r:id="rId639"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB195" r:id="rId640"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC195" r:id="rId641"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z196" r:id="rId642"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA196" r:id="rId643"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB196" r:id="rId644"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC196" r:id="rId645"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z197" r:id="rId646"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA197" r:id="rId647"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB197" r:id="rId648"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC197" r:id="rId649"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z198" r:id="rId650"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA198" r:id="rId651"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB198" r:id="rId652"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC198" r:id="rId653"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z199" r:id="rId654"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA199" r:id="rId655"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB199" r:id="rId656"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC199" r:id="rId657"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z200" r:id="rId658"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD200" r:id="rId659"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z201" r:id="rId660"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA201" r:id="rId661"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB201" r:id="rId662"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC201" r:id="rId663"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD201" r:id="rId664"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z66" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA66" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB66" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC66" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z67" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA67" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB67" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC67" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z68" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z69" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z70" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA70" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB70" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC70" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z71" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA71" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB71" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC71" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z72" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA72" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB72" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC72" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD72" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z73" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA73" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB73" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC73" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z74" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD74" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z75" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA75" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB75" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC75" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z76" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z77" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z78" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA78" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB78" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC78" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD78" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z79" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA79" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB79" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC79" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z80" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA80" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB80" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC80" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD80" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE80" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z81" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA81" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB81" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC81" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z82" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA82" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB82" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC82" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z83" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA83" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB83" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC83" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD83" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA84" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB84" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC84" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA85" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB85" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC85" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA86" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB86" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC86" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA87" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB87" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC87" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA88" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB88" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC88" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA89" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB89" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC89" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA90" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB90" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC90" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD90" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA91" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB91" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC91" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA92" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB92" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC92" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD92" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA93" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB93" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC93" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA94" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB94" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC94" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD96" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA97" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB97" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC97" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA98" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB98" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC98" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA100" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB100" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC100" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA101" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB101" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC101" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA102" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB102" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC102" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD102" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA103" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB103" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC103" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD103" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA104" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB104" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC104" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA105" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB105" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC105" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD105" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA106" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB106" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC106" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA107" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB107" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC107" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD107" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD108" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA110" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB110" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC110" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD111" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA113" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB113" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC113" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z115" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA115" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB115" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC115" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z116" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z117" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA117" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB117" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC117" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z118" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z119" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA119" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB119" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC119" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z120" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD120" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z121" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA121" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB121" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC121" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD121" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z122" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA122" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB122" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC122" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z123" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA123" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB123" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC123" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z124" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA124" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB124" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC124" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD124" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z125" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z126" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z127" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA127" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB127" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC127" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD127" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z128" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA128" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB128" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC128" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z129" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA129" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB129" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC129" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z130" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA130" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB130" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC130" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z131" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA131" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB131" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC131" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z132" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z133" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA133" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB133" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC133" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z134" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA134" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB134" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC134" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z135" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA135" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB135" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC135" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z136" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA136" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB136" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC136" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z137" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA137" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB137" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC137" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z138" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA138" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB138" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC138" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z139" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z140" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA140" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB140" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC140" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z141" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA141" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB141" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC141" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z142" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z143" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA143" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB143" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC143" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z144" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA144" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB144" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC144" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z145" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA145" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB145" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC145" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z146" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA146" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB146" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC146" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z147" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA147" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB147" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC147" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z148" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA148" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB148" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC148" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z149" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA149" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB149" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC149" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z150" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA150" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB150" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC150" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD150" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z151" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD151" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z152" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z153" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z154" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z155" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z156" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z157" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA157" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB157" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC157" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD157" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z158" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA158" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB158" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC158" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z159" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z160" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA160" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB160" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC160" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z161" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z162" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA162" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB162" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC162" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z163" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA163" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB163" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC163" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD163" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z164" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA164" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB164" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC164" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z165" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA165" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB165" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC165" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z166" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z167" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA167" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB167" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC167" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD167" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z168" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA168" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB168" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC168" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z169" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA169" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB169" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC169" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z170" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z171" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA171" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB171" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC171" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z172" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA172" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB172" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC172" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD172" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z173" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z174" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z175" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA175" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB175" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC175" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z176" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA176" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB176" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC176" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z177" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA177" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB177" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC177" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z178" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA178" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB178" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC178" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z179" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA179" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB179" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC179" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD179" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z180" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA180" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB180" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC180" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z181" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z182" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD182" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z183" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA183" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB183" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC183" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z184" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA184" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB184" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC184" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD184" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z185" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA185" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB185" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC185" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD185" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z186" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA186" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB186" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC186" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z187" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD187" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z188" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z189" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z190" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA190" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB190" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC190" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD190" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z191" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD191" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z192" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA192" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB192" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC192" r:id="rId613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z193" r:id="rId614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA193" r:id="rId615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB193" r:id="rId616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC193" r:id="rId617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z194" r:id="rId618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA194" r:id="rId619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB194" r:id="rId620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC194" r:id="rId621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z195" r:id="rId622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA195" r:id="rId623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB195" r:id="rId624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC195" r:id="rId625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z196" r:id="rId626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA196" r:id="rId627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB196" r:id="rId628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC196" r:id="rId629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z197" r:id="rId630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA197" r:id="rId631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB197" r:id="rId632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC197" r:id="rId633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z198" r:id="rId634"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA198" r:id="rId635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB198" r:id="rId636"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC198" r:id="rId637"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z199" r:id="rId638"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA199" r:id="rId639"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB199" r:id="rId640"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC199" r:id="rId641"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z200" r:id="rId642"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD200" r:id="rId643"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z201" r:id="rId644"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId665"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId645"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Replace three collector retellings with local songs: Nigeria, Sierra Leone, Eswatini
The collectors' books use language that is offensive today, so:
- Nigeria: CKay, "Love Nwantiti (Ah Ah Ah)" (replaces Dayrell)
- Sierra Leone: S. E. Rogie, "My Lovely Elizabeth" (replaces Cronise & Ward)
- Eswatini: Mzwaa and Velemseni, "Lutsandvo" (replaces Fynn)
Listed under Poems to explore with description, history note and link.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -9045,34 +9045,34 @@
       </c>
       <c r="D63" s="13" t="inlineStr">
         <is>
-          <t>The Fairy Frog</t>
+          <t>Lutsandvo</t>
         </is>
       </c>
       <c r="E63" s="13" t="inlineStr">
         <is>
-          <t>The Fairy Frog</t>
+          <t>Love</t>
         </is>
       </c>
       <c r="F63" s="13" t="n"/>
       <c r="G63" s="13" t="n"/>
       <c r="H63" s="13" t="inlineStr">
         <is>
-          <t>Traditional Swazi storytellers unknown; arranged in English by Sarah F. Bourhill and Beatrice L. Drake</t>
+          <t>Mzwaa and Velemseni</t>
         </is>
       </c>
       <c r="I63" s="13" t="inlineStr">
         <is>
-          <t>Historical version only</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J63" s="13" t="inlineStr">
         <is>
-          <t>Named oral tale (full historical retelling)</t>
+          <t>Named work</t>
         </is>
       </c>
       <c r="K63" s="13" t="inlineStr">
         <is>
-          <t>Literary retelling / folk tale</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="L63" s="13" t="inlineStr">
@@ -9081,11 +9081,11 @@
         </is>
       </c>
       <c r="M63" s="14" t="n">
-        <v>1908</v>
+        <v>2019</v>
       </c>
       <c r="N63" s="13" t="inlineStr">
         <is>
-          <t>English historical retelling of a Swazi tale; no siSwati transcript supplied</t>
+          <t>siSwati</t>
         </is>
       </c>
       <c r="O63" s="13" t="n"/>
@@ -9101,64 +9101,45 @@
       </c>
       <c r="R63" s="13" t="inlineStr">
         <is>
-          <t>English version published1908; traditional composition date unknown</t>
-        </is>
-      </c>
-      <c r="S63" s="13" t="inlineStr">
-        <is>
-          <t>Fairy Tales from South Africa, Macmillan, London,1908</t>
-        </is>
-      </c>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="S63" s="13" t="n"/>
       <c r="T63" s="13" t="inlineStr">
         <is>
-          <t>Tombi-ende is saved by a frog who becomes a prince after winning her love; they marry. The story includes jealousy and violence before its happy ending.</t>
+          <t>A soulful love song sung entirely in siSwati; its title means “love”.</t>
         </is>
       </c>
       <c r="U63" s="13" t="inlineStr">
         <is>
-          <t>The historical book explicitly labels this individual tale A SWAZI TALE. Swazi cultural association supports the Eswatini grouping; this cross-border tradition is not claimed to be exclusive to present-day Eswatini.</t>
-        </is>
-      </c>
-      <c r="V63" s="13" t="inlineStr">
-        <is>
-          <t>XVI, The Fairy Frog, pp.187–198</t>
-        </is>
-      </c>
+          <t>Recording</t>
+        </is>
+      </c>
+      <c r="V63" s="13" t="n"/>
       <c r="W63" s="13" t="inlineStr">
         <is>
-          <t>Two women arranged the English version; gender of original storytellers/composers remains unknown. Original siSwati wording is not provided. The introduction uses colonial racial terminology; use the story critically and distinguish later adaptations.</t>
+          <t>Two women arranged the English version; gender of original storytellers/composers remains unknown. Original siSwati wording is not provided. The introduction uses colonial racial terminology; use the story critically and distinguish later adaptations.
+Work changed (29 October 2026): the earlier colonial-era retelling is replaced, because the collector’s book uses language that is offensive today. Replaced by a song by a local artist; in copyright, listed with a description and link only.</t>
         </is>
       </c>
       <c r="X63" s="13" t="inlineStr">
         <is>
-          <t>The1908 English version is public domain in the USA, as recorded by Project Gutenberg. Compilers’ death dates and rights outside the USA are not established here. No claim of open original siSwati text or later retellings.</t>
+          <t>In copyright. Not reproduced; listed with a link.</t>
         </is>
       </c>
       <c r="Y63" s="13" t="inlineStr">
         <is>
-          <t>Work-specific text, date and provenance sources checked29October2026.</t>
+          <t>Texx and the City: Mzwaa releases video for his love song “Lutsandvo”</t>
         </is>
       </c>
       <c r="Z63" s="11" t="inlineStr">
         <is>
-          <t>Work / text</t>
-        </is>
-      </c>
-      <c r="AA63" s="11" t="inlineStr">
-        <is>
-          <t>Rights / catalogue</t>
-        </is>
-      </c>
-      <c r="AB63" s="11" t="inlineStr">
-        <is>
-          <t>Date / edition</t>
-        </is>
-      </c>
-      <c r="AC63" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country</t>
-        </is>
-      </c>
+          <t>Read about it</t>
+        </is>
+      </c>
+      <c r="AA63" s="11" t="n"/>
+      <c r="AB63" s="11" t="n"/>
+      <c r="AC63" s="11" t="n"/>
       <c r="AD63" s="11" t="n"/>
       <c r="AE63" s="11" t="n"/>
     </row>
@@ -19552,34 +19533,34 @@
       </c>
       <c r="D133" s="13" t="inlineStr">
         <is>
-          <t>Ituen and the King’s Wife</t>
+          <t>Love Nwantiti (Ah Ah Ah)</t>
         </is>
       </c>
       <c r="E133" s="13" t="inlineStr">
         <is>
-          <t>Ituen and the King’s Wife</t>
+          <t>Small Love</t>
         </is>
       </c>
       <c r="F133" s="13" t="n"/>
       <c r="G133" s="13" t="n"/>
       <c r="H133" s="13" t="inlineStr">
         <is>
-          <t>Southern Nigerian oral tradition; English version collected by Elphinstone Dayrell (1869–1917)</t>
+          <t>CKay</t>
         </is>
       </c>
       <c r="I133" s="13" t="inlineStr">
         <is>
-          <t>Historical version only</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J133" s="13" t="inlineStr">
         <is>
-          <t>Named oral tale (full historical text)</t>
+          <t>Named work</t>
         </is>
       </c>
       <c r="K133" s="13" t="inlineStr">
         <is>
-          <t>Oral tale</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="L133" s="13" t="inlineStr">
@@ -19588,11 +19569,11 @@
         </is>
       </c>
       <c r="M133" s="14" t="n">
-        <v>1910</v>
+        <v>2019</v>
       </c>
       <c r="N133" s="13" t="inlineStr">
         <is>
-          <t>Calabar/Cross River tradition; historical English version</t>
+          <t>Igbo and English</t>
         </is>
       </c>
       <c r="O133" s="13" t="n"/>
@@ -19608,64 +19589,45 @@
       </c>
       <c r="R133" s="13" t="inlineStr">
         <is>
-          <t>Published London, 1910; traditional narrative date unknown</t>
-        </is>
-      </c>
-      <c r="S133" s="13" t="inlineStr">
-        <is>
-          <t>Folk Stories from Southern Nigeria, West Africa, chapter V, pp.29–32</t>
-        </is>
-      </c>
+          <t>2019</t>
+        </is>
+      </c>
+      <c r="S133" s="13" t="n"/>
       <c r="T133" s="13" t="inlineStr">
         <is>
-          <t>Ituen and a king’s wife become lovers and arrange secret meetings. Their discovery leads to a tragic punishment.</t>
+          <t>A love song sung mostly in Igbo; CKay explains that “love nwantiti”, literally “small love”, means the love within a couple.</t>
         </is>
       </c>
       <c r="U133" s="13" t="inlineStr">
         <is>
-          <t>Dayrell’s 1910 collection, chapter V, explicitly locates the story in Calabar. Project Gutenberg provides the complete historical English text.</t>
-        </is>
-      </c>
-      <c r="V133" s="13" t="inlineStr">
-        <is>
-          <t>V, Ituen and the King’s Wife, pp.29–32</t>
-        </is>
-      </c>
+          <t>Recording</t>
+        </is>
+      </c>
+      <c r="V133" s="13" t="n"/>
       <c r="W133" s="13" t="inlineStr">
         <is>
-          <t>A dark account of mutual attraction, adultery and violent punishment, not an affirmative model of love. The queen also detains Ituen against his wishes. Reuse only the historical English text; original-language wording, later retellings and recordings are separate.</t>
+          <t>A dark account of mutual attraction, adultery and violent punishment, not an affirmative model of love. The queen also detains Ituen against his wishes. Reuse only the historical English text; original-language wording, later retellings and recordings are separate.
+Work changed (29 October 2026): the earlier colonial-era retelling is replaced, because the collector’s book uses language that is offensive today. Replaced by a song by a local artist; in copyright, listed with a description and link only.</t>
         </is>
       </c>
       <c r="X133" s="13" t="inlineStr">
         <is>
-          <t>Historical English text published 1910 and public domain in the US; collector Dayrell died 1917, beyond life-plus-70. This does not establish rights to native variants or new adaptations.</t>
+          <t>In copyright. Not reproduced; listed with a link.</t>
         </is>
       </c>
       <c r="Y133" s="13" t="inlineStr">
         <is>
-          <t>Work-specific text, date and provenance sources checked29October2026.</t>
+          <t>OkayAfrica: How CKay’s “Love Nwantiti” became the world’s song</t>
         </is>
       </c>
       <c r="Z133" s="11" t="inlineStr">
         <is>
-          <t>Work / text</t>
-        </is>
-      </c>
-      <c r="AA133" s="11" t="inlineStr">
-        <is>
-          <t>Rights / catalogue</t>
-        </is>
-      </c>
-      <c r="AB133" s="11" t="inlineStr">
-        <is>
-          <t>Date / edition</t>
-        </is>
-      </c>
-      <c r="AC133" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country</t>
-        </is>
-      </c>
+          <t>Read about it</t>
+        </is>
+      </c>
+      <c r="AA133" s="11" t="n"/>
+      <c r="AB133" s="11" t="n"/>
+      <c r="AC133" s="11" t="n"/>
       <c r="AD133" s="11" t="n"/>
       <c r="AE133" s="11" t="n"/>
     </row>
@@ -23799,34 +23761,34 @@
       </c>
       <c r="D162" s="13" t="inlineStr">
         <is>
-          <t>Marry the Devil, There’s the Devil to Pay</t>
+          <t>My Lovely Elizabeth</t>
         </is>
       </c>
       <c r="E162" s="13" t="inlineStr">
         <is>
-          <t>Marry the Devil, There’s the Devil to Pay</t>
+          <t>My Lovely Elizabeth</t>
         </is>
       </c>
       <c r="F162" s="13" t="n"/>
       <c r="G162" s="13" t="n"/>
       <c r="H162" s="13" t="inlineStr">
         <is>
-          <t>Traditional storytellers unknown; recorded/arranged by Florence M. Cronise and Henry W. Ward</t>
+          <t>S. E. Rogie (1926–1994)</t>
         </is>
       </c>
       <c r="I162" s="13" t="inlineStr">
         <is>
-          <t>Historical version only</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J162" s="13" t="inlineStr">
         <is>
-          <t>Named oral tale (full historical retelling)</t>
+          <t>Named work</t>
         </is>
       </c>
       <c r="K162" s="13" t="inlineStr">
         <is>
-          <t>Literary retelling / folk tale</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="L162" s="13" t="inlineStr">
@@ -23835,11 +23797,11 @@
         </is>
       </c>
       <c r="M162" s="14" t="n">
-        <v>1903</v>
+        <v>1962</v>
       </c>
       <c r="N162" s="13" t="inlineStr">
         <is>
-          <t>Historical English/pidgin rendering from Sierra Leone; original oral language not securely established</t>
+          <t>English</t>
         </is>
       </c>
       <c r="O162" s="13" t="n"/>
@@ -23855,64 +23817,45 @@
       </c>
       <c r="R162" s="13" t="inlineStr">
         <is>
-          <t>Published1903; traditional composition earlier, exact date unknown</t>
-        </is>
-      </c>
-      <c r="S162" s="13" t="inlineStr">
-        <is>
-          <t>Cunnie Rabbit, Mr. Spider and the Other Beef,1903</t>
-        </is>
-      </c>
+          <t>c. 1962 (first published by 1965)</t>
+        </is>
+      </c>
+      <c r="S162" s="13" t="n"/>
       <c r="T162" s="13" t="inlineStr">
         <is>
-          <t>A girl rejects her suitors until attracted to a handsome stranger, marries him and discovers he is a devouring devil. Her brother helps her escape. Courtship cautionary tale, rather than an affirmative love story.</t>
+          <t>S. E. Rogie’s signature love ballad, sung over the gentle guitar of palm-wine music.</t>
         </is>
       </c>
       <c r="U162" s="13" t="inlineStr">
         <is>
-          <t>Historical collection explicitly concerns Sierra Leone storytelling. A framing narrator named Yamah introduces this tale; her appearance does not establish a traceable historical composer or female authorship.</t>
-        </is>
-      </c>
-      <c r="V162" s="13" t="inlineStr">
-        <is>
-          <t>Chapter with title Marry the Devil, There’s the Devil to Pay, pp.178–186</t>
-        </is>
-      </c>
+          <t>Recording</t>
+        </is>
+      </c>
+      <c r="V162" s="13" t="n"/>
       <c r="W162" s="13" t="inlineStr">
         <is>
-          <t>The book’s literary frame and colonial rendering are distinct from a verbatim indigenous-language transcript. Compilers are a woman and a man; traditional creator gender remains unknown. Horror, threatened violence and deceptive attraction dominate.</t>
+          <t>The book’s literary frame and colonial rendering are distinct from a verbatim indigenous-language transcript. Compilers are a woman and a man; traditional creator gender remains unknown. Horror, threatened violence and deceptive attraction dominate.
+Work changed (29 October 2026): the earlier colonial-era retelling is replaced, because the collector’s book uses language that is offensive today. Replaced by a song by a local artist; in copyright, listed with a description and link only.</t>
         </is>
       </c>
       <c r="X162" s="13" t="inlineStr">
         <is>
-          <t>Historical1903 printed wording is public domain in the USA according to Project Gutenberg. Compilers’ death dates and broader territorial status are unverified. Native variants, modern editions and performances are not covered.</t>
+          <t>In copyright. Not reproduced; listed with a link.</t>
         </is>
       </c>
       <c r="Y162" s="13" t="inlineStr">
         <is>
-          <t>Work-specific text, date and provenance sources checked29October2026.</t>
+          <t>Wikipedia: S. E. Rogie</t>
         </is>
       </c>
       <c r="Z162" s="11" t="inlineStr">
         <is>
-          <t>Work / text</t>
-        </is>
-      </c>
-      <c r="AA162" s="11" t="inlineStr">
-        <is>
-          <t>Rights / catalogue</t>
-        </is>
-      </c>
-      <c r="AB162" s="11" t="inlineStr">
-        <is>
-          <t>Date / edition</t>
-        </is>
-      </c>
-      <c r="AC162" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country</t>
-        </is>
-      </c>
+          <t>Read about it</t>
+        </is>
+      </c>
+      <c r="AA162" s="11" t="n"/>
+      <c r="AB162" s="11" t="n"/>
+      <c r="AC162" s="11" t="n"/>
       <c r="AD162" s="11" t="n"/>
       <c r="AE162" s="11" t="n"/>
     </row>
@@ -29749,472 +29692,463 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB62" r:id="rId180"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC62" r:id="rId181"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z63" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA63" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB63" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC63" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z64" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA64" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB64" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC64" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z65" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z66" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA66" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB66" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC66" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z67" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA67" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB67" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC67" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z68" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z69" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z70" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA70" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB70" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC70" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z71" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA71" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB71" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC71" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z72" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA72" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB72" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC72" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD72" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z73" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA73" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB73" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC73" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z74" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD74" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z75" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA75" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB75" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC75" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z76" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z77" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z78" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA78" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB78" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC78" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD78" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z79" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA79" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB79" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC79" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z80" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA80" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB80" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC80" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD80" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE80" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z81" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA81" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB81" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC81" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z82" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA82" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB82" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC82" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z83" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA83" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB83" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC83" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD83" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA84" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB84" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC84" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA85" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB85" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC85" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA86" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB86" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC86" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA87" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB87" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC87" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA88" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB88" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC88" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA89" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB89" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC89" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA90" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB90" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC90" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD90" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA91" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB91" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC91" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA92" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB92" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC92" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD92" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA93" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB93" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC93" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA94" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB94" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC94" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD96" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA97" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB97" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC97" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA98" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB98" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC98" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA100" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB100" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC100" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA101" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB101" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC101" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA102" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB102" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC102" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD102" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA103" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB103" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC103" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD103" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA104" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB104" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC104" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA105" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB105" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC105" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD105" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA106" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB106" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC106" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA107" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB107" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC107" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD107" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD108" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA110" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB110" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC110" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD111" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA113" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB113" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC113" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z115" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA115" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB115" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC115" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z116" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z117" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA117" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB117" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC117" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z118" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z119" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA119" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB119" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC119" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z120" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD120" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z121" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA121" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB121" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC121" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD121" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z122" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA122" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB122" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC122" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z123" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA123" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB123" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC123" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z124" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA124" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB124" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC124" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD124" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z125" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z126" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z127" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA127" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB127" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC127" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD127" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z128" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA128" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB128" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC128" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z129" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA129" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB129" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC129" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z130" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA130" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB130" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC130" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z131" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA131" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB131" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC131" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z132" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z133" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA133" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB133" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC133" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z134" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA134" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB134" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC134" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z135" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA135" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB135" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC135" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z136" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA136" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB136" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC136" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z137" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA137" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB137" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC137" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z138" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA138" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB138" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC138" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z139" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z140" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA140" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB140" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC140" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z141" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA141" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB141" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC141" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z142" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z143" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA143" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB143" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC143" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z144" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA144" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB144" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC144" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z145" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA145" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB145" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC145" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z146" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA146" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB146" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC146" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z147" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA147" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB147" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC147" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z148" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA148" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB148" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC148" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z149" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA149" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB149" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC149" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z150" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA150" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB150" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC150" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD150" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z151" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD151" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z152" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z153" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z154" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z155" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z156" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z157" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA157" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB157" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC157" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD157" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z158" r:id="rId500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA158" r:id="rId501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB158" r:id="rId502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC158" r:id="rId503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z159" r:id="rId504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z160" r:id="rId505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA160" r:id="rId506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB160" r:id="rId507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC160" r:id="rId508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z161" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z162" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA162" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB162" r:id="rId512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC162" r:id="rId513"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z163" r:id="rId514"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA163" r:id="rId515"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB163" r:id="rId516"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC163" r:id="rId517"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD163" r:id="rId518"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z164" r:id="rId519"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA164" r:id="rId520"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB164" r:id="rId521"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC164" r:id="rId522"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z165" r:id="rId523"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA165" r:id="rId524"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB165" r:id="rId525"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC165" r:id="rId526"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z166" r:id="rId527"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z167" r:id="rId528"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA167" r:id="rId529"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB167" r:id="rId530"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC167" r:id="rId531"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD167" r:id="rId532"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z168" r:id="rId533"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA168" r:id="rId534"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB168" r:id="rId535"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC168" r:id="rId536"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z169" r:id="rId537"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA169" r:id="rId538"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB169" r:id="rId539"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC169" r:id="rId540"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z170" r:id="rId541"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z171" r:id="rId542"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA171" r:id="rId543"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB171" r:id="rId544"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC171" r:id="rId545"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z172" r:id="rId546"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA172" r:id="rId547"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB172" r:id="rId548"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC172" r:id="rId549"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD172" r:id="rId550"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z173" r:id="rId551"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z174" r:id="rId552"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z175" r:id="rId553"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA175" r:id="rId554"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB175" r:id="rId555"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC175" r:id="rId556"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z176" r:id="rId557"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA176" r:id="rId558"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB176" r:id="rId559"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC176" r:id="rId560"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z177" r:id="rId561"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA177" r:id="rId562"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB177" r:id="rId563"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC177" r:id="rId564"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z178" r:id="rId565"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA178" r:id="rId566"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB178" r:id="rId567"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC178" r:id="rId568"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z179" r:id="rId569"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA179" r:id="rId570"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB179" r:id="rId571"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC179" r:id="rId572"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD179" r:id="rId573"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z180" r:id="rId574"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA180" r:id="rId575"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB180" r:id="rId576"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC180" r:id="rId577"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z181" r:id="rId578"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z182" r:id="rId579"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD182" r:id="rId580"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z183" r:id="rId581"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA183" r:id="rId582"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB183" r:id="rId583"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC183" r:id="rId584"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z184" r:id="rId585"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA184" r:id="rId586"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB184" r:id="rId587"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC184" r:id="rId588"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD184" r:id="rId589"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z185" r:id="rId590"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA185" r:id="rId591"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB185" r:id="rId592"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC185" r:id="rId593"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD185" r:id="rId594"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z186" r:id="rId595"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA186" r:id="rId596"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB186" r:id="rId597"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC186" r:id="rId598"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z187" r:id="rId599"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD187" r:id="rId600"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z188" r:id="rId601"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z189" r:id="rId602"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z190" r:id="rId603"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA190" r:id="rId604"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB190" r:id="rId605"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC190" r:id="rId606"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD190" r:id="rId607"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z191" r:id="rId608"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD191" r:id="rId609"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z192" r:id="rId610"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA192" r:id="rId611"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB192" r:id="rId612"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC192" r:id="rId613"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z193" r:id="rId614"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA193" r:id="rId615"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB193" r:id="rId616"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC193" r:id="rId617"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z194" r:id="rId618"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA194" r:id="rId619"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB194" r:id="rId620"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC194" r:id="rId621"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z195" r:id="rId622"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA195" r:id="rId623"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB195" r:id="rId624"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC195" r:id="rId625"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z196" r:id="rId626"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA196" r:id="rId627"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB196" r:id="rId628"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC196" r:id="rId629"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z197" r:id="rId630"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA197" r:id="rId631"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB197" r:id="rId632"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC197" r:id="rId633"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z198" r:id="rId634"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA198" r:id="rId635"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB198" r:id="rId636"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC198" r:id="rId637"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z199" r:id="rId638"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA199" r:id="rId639"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB199" r:id="rId640"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC199" r:id="rId641"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z200" r:id="rId642"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD200" r:id="rId643"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z201" r:id="rId644"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z64" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA64" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB64" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC64" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z65" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z66" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA66" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB66" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC66" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z67" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA67" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB67" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC67" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z68" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z69" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z70" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA70" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB70" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC70" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z71" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA71" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB71" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC71" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z72" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA72" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB72" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC72" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD72" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z73" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA73" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB73" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC73" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z74" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD74" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z75" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA75" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB75" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC75" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z76" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z77" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z78" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA78" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB78" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC78" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD78" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z79" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA79" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB79" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC79" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z80" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA80" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB80" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC80" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD80" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE80" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z81" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA81" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB81" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC81" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z82" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA82" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB82" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC82" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z83" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA83" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB83" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC83" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD83" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA84" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB84" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC84" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA85" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB85" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC85" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA86" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB86" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC86" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA87" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB87" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC87" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA88" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB88" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC88" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA89" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB89" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC89" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA90" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB90" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC90" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD90" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA91" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB91" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC91" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA92" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB92" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC92" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD92" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA93" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB93" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC93" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA94" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB94" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC94" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD96" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA97" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB97" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC97" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA98" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB98" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC98" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA100" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB100" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC100" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA101" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB101" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC101" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA102" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB102" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC102" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD102" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA103" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB103" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC103" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD103" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA104" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB104" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC104" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA105" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB105" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC105" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD105" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA106" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB106" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC106" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA107" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB107" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC107" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD107" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD108" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA110" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB110" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC110" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD111" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA113" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB113" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC113" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z115" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA115" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB115" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC115" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z116" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z117" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA117" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB117" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC117" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z118" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z119" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA119" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB119" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC119" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z120" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD120" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z121" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA121" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB121" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC121" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD121" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z122" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA122" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB122" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC122" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z123" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA123" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB123" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC123" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z124" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA124" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB124" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC124" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD124" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z125" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z126" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z127" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA127" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB127" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC127" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD127" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z128" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA128" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB128" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC128" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z129" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA129" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB129" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC129" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z130" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA130" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB130" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC130" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z131" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA131" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB131" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC131" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z132" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z133" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z134" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA134" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB134" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC134" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z135" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA135" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB135" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC135" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z136" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA136" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB136" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC136" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z137" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA137" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB137" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC137" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z138" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA138" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB138" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC138" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z139" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z140" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA140" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB140" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC140" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z141" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA141" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB141" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC141" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z142" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z143" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA143" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB143" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC143" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z144" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA144" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB144" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC144" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z145" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA145" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB145" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC145" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z146" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA146" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB146" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC146" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z147" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA147" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB147" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC147" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z148" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA148" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB148" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC148" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z149" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA149" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB149" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC149" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z150" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA150" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB150" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC150" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD150" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z151" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD151" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z152" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z153" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z154" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z155" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z156" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z157" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA157" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB157" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC157" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD157" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z158" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA158" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB158" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC158" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z159" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z160" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA160" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB160" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC160" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z161" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z162" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z163" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA163" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB163" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC163" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD163" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z164" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA164" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB164" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC164" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z165" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA165" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB165" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC165" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z166" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z167" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA167" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB167" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC167" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD167" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z168" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA168" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB168" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC168" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z169" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA169" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB169" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC169" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z170" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z171" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA171" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB171" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC171" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z172" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA172" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB172" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC172" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD172" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z173" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z174" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z175" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA175" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB175" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC175" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z176" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA176" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB176" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC176" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z177" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA177" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB177" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC177" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z178" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA178" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB178" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC178" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z179" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA179" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB179" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC179" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD179" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z180" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA180" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB180" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC180" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z181" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z182" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD182" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z183" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA183" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB183" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC183" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z184" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA184" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB184" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC184" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD184" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z185" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA185" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB185" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC185" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD185" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z186" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA186" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB186" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC186" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z187" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD187" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z188" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z189" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z190" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA190" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB190" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC190" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD190" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z191" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD191" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z192" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA192" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB192" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC192" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z193" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA193" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB193" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC193" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z194" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA194" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB194" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC194" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z195" r:id="rId613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA195" r:id="rId614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB195" r:id="rId615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC195" r:id="rId616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z196" r:id="rId617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA196" r:id="rId618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB196" r:id="rId619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC196" r:id="rId620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z197" r:id="rId621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA197" r:id="rId622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB197" r:id="rId623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC197" r:id="rId624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z198" r:id="rId625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA198" r:id="rId626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB198" r:id="rId627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC198" r:id="rId628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z199" r:id="rId629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA199" r:id="rId630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB199" r:id="rId631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC199" r:id="rId632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z200" r:id="rId633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD200" r:id="rId634"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z201" r:id="rId635"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId645"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId636"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Explore links go where readers can hear or read the work
- 30 songs now link to the song itself (mostly official uploads) instead
  of news stories, bios, magazines or Eurovision pages.
- Fixed dead links for Luxembourg, Myanmar, Sri Lanka and Turkmenistan;
  Palau and Zambia have no public copy, so they show no link.
- Links say what readers will find ("Listen to the song", "Read the
  lyrics", ...) when the spreadsheet gives a reader-facing label.
- Old links kept in the spreadsheet's "Additional link 2" column.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -1466,7 +1466,7 @@
       </c>
       <c r="Z10" s="11" t="inlineStr">
         <is>
-          <t>eurovision.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA10" s="11" t="n"/>
@@ -1477,7 +1477,11 @@
           <t>formulatv.com</t>
         </is>
       </c>
-      <c r="AE10" s="11" t="n"/>
+      <c r="AE10" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: eurovision.com</t>
+        </is>
+      </c>
     </row>
     <row r="11" ht="194" customHeight="1" s="17">
       <c r="A11" s="7" t="inlineStr">
@@ -1753,14 +1757,18 @@
       </c>
       <c r="Z12" s="11" t="inlineStr">
         <is>
-          <t>worldradiohistory.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA12" s="11" t="n"/>
       <c r="AB12" s="11" t="n"/>
       <c r="AC12" s="11" t="n"/>
       <c r="AD12" s="11" t="n"/>
-      <c r="AE12" s="11" t="n"/>
+      <c r="AE12" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: worldradiohistory.com</t>
+        </is>
+      </c>
     </row>
     <row r="13" ht="235.5" customHeight="1" s="17">
       <c r="A13" s="7" t="inlineStr">
@@ -2679,7 +2687,7 @@
       </c>
       <c r="Z18" s="11" t="inlineStr">
         <is>
-          <t>folkways.si.edu</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA18" s="11" t="n"/>
@@ -3579,7 +3587,7 @@
       </c>
       <c r="Z24" s="11" t="inlineStr">
         <is>
-          <t>realworldrecords.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA24" s="11" t="n"/>
@@ -3590,7 +3598,11 @@
           <t>stonetreerecords.com</t>
         </is>
       </c>
-      <c r="AE24" s="11" t="n"/>
+      <c r="AE24" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: realworldrecords.com</t>
+        </is>
+      </c>
     </row>
     <row r="25" ht="180" customHeight="1" s="17">
       <c r="A25" s="7" t="inlineStr">
@@ -4281,14 +4293,18 @@
       </c>
       <c r="Z29" s="11" t="inlineStr">
         <is>
-          <t>dailynews.gov.bw</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA29" s="11" t="n"/>
       <c r="AB29" s="11" t="n"/>
       <c r="AC29" s="11" t="n"/>
       <c r="AD29" s="11" t="n"/>
-      <c r="AE29" s="11" t="n"/>
+      <c r="AE29" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: dailynews.gov.bw</t>
+        </is>
+      </c>
     </row>
     <row r="30" ht="208" customHeight="1" s="17">
       <c r="A30" s="7" t="inlineStr">
@@ -4949,14 +4965,18 @@
       </c>
       <c r="Z34" s="11" t="inlineStr">
         <is>
-          <t>notjustok.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA34" s="11" t="n"/>
       <c r="AB34" s="11" t="n"/>
       <c r="AC34" s="11" t="n"/>
       <c r="AD34" s="11" t="n"/>
-      <c r="AE34" s="11" t="n"/>
+      <c r="AE34" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: notjustok.com</t>
+        </is>
+      </c>
     </row>
     <row r="35" ht="108" customHeight="1" s="17">
       <c r="A35" s="7" t="inlineStr">
@@ -5375,14 +5395,18 @@
       </c>
       <c r="Z37" s="11" t="inlineStr">
         <is>
-          <t>unorthodoxreviews.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA37" s="11" t="n"/>
       <c r="AB37" s="11" t="n"/>
       <c r="AC37" s="11" t="n"/>
       <c r="AD37" s="11" t="n"/>
-      <c r="AE37" s="11" t="n"/>
+      <c r="AE37" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: unorthodoxreviews.com</t>
+        </is>
+      </c>
     </row>
     <row r="38" ht="252" customHeight="1" s="17">
       <c r="A38" s="7" t="inlineStr">
@@ -5652,7 +5676,7 @@
       </c>
       <c r="Z39" s="11" t="inlineStr">
         <is>
-          <t>abdulchampion.bandcamp.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA39" s="11" t="n"/>
@@ -6390,7 +6414,7 @@
       </c>
       <c r="Z44" s="11" t="inlineStr">
         <is>
-          <t>nawali.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA44" s="11" t="n"/>
@@ -6401,7 +6425,11 @@
           <t>mediatheques.agglo-larochelle.fr</t>
         </is>
       </c>
-      <c r="AE44" s="11" t="n"/>
+      <c r="AE44" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: nawali.com</t>
+        </is>
+      </c>
     </row>
     <row r="45" ht="75.75" customHeight="1" s="17">
       <c r="A45" s="7" t="inlineStr">
@@ -6812,7 +6840,7 @@
       </c>
       <c r="Z47" s="11" t="inlineStr">
         <is>
-          <t>youtube.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA47" s="11" t="n"/>
@@ -7577,7 +7605,7 @@
       </c>
       <c r="Z52" s="11" t="inlineStr">
         <is>
-          <t>busylife.bandcamp.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA52" s="11" t="n"/>
@@ -7836,14 +7864,18 @@
       </c>
       <c r="Z54" s="11" t="inlineStr">
         <is>
-          <t>glitterbeat.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA54" s="11" t="n"/>
       <c r="AB54" s="11" t="n"/>
       <c r="AC54" s="11" t="n"/>
       <c r="AD54" s="11" t="n"/>
-      <c r="AE54" s="11" t="n"/>
+      <c r="AE54" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: glitterbeat.com</t>
+        </is>
+      </c>
     </row>
     <row r="55" ht="60" customHeight="1" s="17">
       <c r="A55" s="7" t="inlineStr">
@@ -7945,14 +7977,18 @@
       </c>
       <c r="Z55" s="11" t="inlineStr">
         <is>
-          <t>dominicanewsonline.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA55" s="11" t="n"/>
       <c r="AB55" s="11" t="n"/>
       <c r="AC55" s="11" t="n"/>
       <c r="AD55" s="11" t="n"/>
-      <c r="AE55" s="11" t="n"/>
+      <c r="AE55" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: dominicanewsonline.com</t>
+        </is>
+      </c>
     </row>
     <row r="56" ht="91.5" customHeight="1" s="17">
       <c r="A56" s="7" t="inlineStr">
@@ -8745,7 +8781,7 @@
       </c>
       <c r="Z60" s="11" t="inlineStr">
         <is>
-          <t>afrikalyrics.com</t>
+          <t>Read the lyrics</t>
         </is>
       </c>
       <c r="AA60" s="11" t="n"/>
@@ -9134,14 +9170,18 @@
       </c>
       <c r="Z63" s="11" t="inlineStr">
         <is>
-          <t>Read about it</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA63" s="11" t="n"/>
       <c r="AB63" s="11" t="n"/>
       <c r="AC63" s="11" t="n"/>
       <c r="AD63" s="11" t="n"/>
-      <c r="AE63" s="11" t="n"/>
+      <c r="AE63" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: Read about it</t>
+        </is>
+      </c>
     </row>
     <row r="64" ht="123.75" customHeight="1" s="17">
       <c r="A64" s="7" t="inlineStr">
@@ -9839,14 +9879,18 @@
       </c>
       <c r="Z68" s="11" t="inlineStr">
         <is>
-          <t>popnable.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA68" s="11" t="n"/>
       <c r="AB68" s="11" t="n"/>
       <c r="AC68" s="11" t="n"/>
       <c r="AD68" s="11" t="n"/>
-      <c r="AE68" s="11" t="n"/>
+      <c r="AE68" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: popnable.com</t>
+        </is>
+      </c>
     </row>
     <row r="69" ht="60" customHeight="1" s="17">
       <c r="A69" s="7" t="inlineStr">
@@ -9948,14 +9992,18 @@
       </c>
       <c r="Z69" s="11" t="inlineStr">
         <is>
-          <t>musicinafrica.net</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA69" s="11" t="n"/>
       <c r="AB69" s="11" t="n"/>
       <c r="AC69" s="11" t="n"/>
       <c r="AD69" s="11" t="n"/>
-      <c r="AE69" s="11" t="n"/>
+      <c r="AE69" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: musicinafrica.net</t>
+        </is>
+      </c>
     </row>
     <row r="70" ht="91.5" customHeight="1" s="17">
       <c r="A70" s="7" t="inlineStr">
@@ -10707,7 +10755,7 @@
       </c>
       <c r="Z74" s="11" t="inlineStr">
         <is>
-          <t>jeversonsound.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA74" s="11" t="n"/>
@@ -10718,7 +10766,11 @@
           <t>music.apple.com</t>
         </is>
       </c>
-      <c r="AE74" s="11" t="n"/>
+      <c r="AE74" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: jeversonsound.com</t>
+        </is>
+      </c>
     </row>
     <row r="75" ht="75.75" customHeight="1" s="17">
       <c r="A75" s="7" t="inlineStr">
@@ -10992,14 +11044,18 @@
       </c>
       <c r="Z76" s="11" t="inlineStr">
         <is>
-          <t>old.afropop.org</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA76" s="11" t="n"/>
       <c r="AB76" s="11" t="n"/>
       <c r="AC76" s="11" t="n"/>
       <c r="AD76" s="11" t="n"/>
-      <c r="AE76" s="11" t="n"/>
+      <c r="AE76" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: old.afropop.org</t>
+        </is>
+      </c>
     </row>
     <row r="77" ht="91.5" customHeight="1" s="17">
       <c r="A77" s="7" t="inlineStr">
@@ -14098,14 +14154,18 @@
       </c>
       <c r="Z95" s="11" t="inlineStr">
         <is>
-          <t>fadhiliwilliam.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA95" s="11" t="n"/>
       <c r="AB95" s="11" t="n"/>
       <c r="AC95" s="11" t="n"/>
       <c r="AD95" s="11" t="n"/>
-      <c r="AE95" s="11" t="n"/>
+      <c r="AE95" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: fadhiliwilliam.com</t>
+        </is>
+      </c>
     </row>
     <row r="96" ht="60" customHeight="1" s="17">
       <c r="A96" s="7" t="inlineStr">
@@ -14660,7 +14720,7 @@
       </c>
       <c r="Z99" s="11" t="inlineStr">
         <is>
-          <t>folkways.si.edu</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA99" s="11" t="n"/>
@@ -15887,7 +15947,7 @@
       </c>
       <c r="Z107" s="11" t="inlineStr">
         <is>
-          <t>Work / source text</t>
+          <t>Read about it</t>
         </is>
       </c>
       <c r="AA107" s="11" t="inlineStr">
@@ -15910,7 +15970,11 @@
           <t>Additional evidence</t>
         </is>
       </c>
-      <c r="AE107" s="11" t="n"/>
+      <c r="AE107" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: Work / source text</t>
+        </is>
+      </c>
     </row>
     <row r="108" ht="60" customHeight="1" s="17">
       <c r="A108" s="7" t="inlineStr">
@@ -16121,14 +16185,18 @@
       </c>
       <c r="Z109" s="11" t="inlineStr">
         <is>
-          <t>music.apple.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA109" s="11" t="n"/>
       <c r="AB109" s="11" t="n"/>
       <c r="AC109" s="11" t="n"/>
       <c r="AD109" s="11" t="n"/>
-      <c r="AE109" s="11" t="n"/>
+      <c r="AE109" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: music.apple.com</t>
+        </is>
+      </c>
     </row>
     <row r="110" ht="123.75" customHeight="1" s="17">
       <c r="A110" s="7" t="inlineStr">
@@ -16410,7 +16478,7 @@
       </c>
       <c r="Z111" s="11" t="inlineStr">
         <is>
-          <t>open.spotify.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA111" s="11" t="n"/>
@@ -16523,14 +16591,18 @@
       </c>
       <c r="Z112" s="11" t="inlineStr">
         <is>
-          <t>old.afropop.org</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA112" s="11" t="n"/>
       <c r="AB112" s="11" t="n"/>
       <c r="AC112" s="11" t="n"/>
       <c r="AD112" s="11" t="n"/>
-      <c r="AE112" s="11" t="n"/>
+      <c r="AE112" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: old.afropop.org</t>
+        </is>
+      </c>
     </row>
     <row r="113" ht="91.5" customHeight="1" s="17">
       <c r="A113" s="7" t="inlineStr">
@@ -16806,7 +16878,7 @@
       </c>
       <c r="Z114" s="11" t="inlineStr">
         <is>
-          <t>youtube.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA114" s="11" t="n"/>
@@ -17082,14 +17154,18 @@
       </c>
       <c r="Z116" s="11" t="inlineStr">
         <is>
-          <t>Read about it</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA116" s="11" t="n"/>
       <c r="AB116" s="11" t="n"/>
       <c r="AC116" s="11" t="n"/>
       <c r="AD116" s="11" t="n"/>
-      <c r="AE116" s="11" t="n"/>
+      <c r="AE116" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: Read about it</t>
+        </is>
+      </c>
     </row>
     <row r="117" ht="235.5" customHeight="1" s="17">
       <c r="A117" s="7" t="inlineStr">
@@ -17662,7 +17738,7 @@
       </c>
       <c r="Z120" s="11" t="inlineStr">
         <is>
-          <t>eurovision.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA120" s="11" t="n"/>
@@ -17673,7 +17749,11 @@
           <t>eurovision-spain.com</t>
         </is>
       </c>
-      <c r="AE120" s="11" t="n"/>
+      <c r="AE120" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: eurovision.com</t>
+        </is>
+      </c>
     </row>
     <row r="121" ht="91.5" customHeight="1" s="17">
       <c r="A121" s="7" t="inlineStr">
@@ -18503,14 +18583,18 @@
       </c>
       <c r="Z125" s="11" t="inlineStr">
         <is>
-          <t>mdn.gov.mm</t>
+          <t>Read about the poet</t>
         </is>
       </c>
       <c r="AA125" s="11" t="n"/>
       <c r="AB125" s="11" t="n"/>
       <c r="AC125" s="11" t="n"/>
       <c r="AD125" s="11" t="n"/>
-      <c r="AE125" s="11" t="n"/>
+      <c r="AE125" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: mdn.gov.mm</t>
+        </is>
+      </c>
     </row>
     <row r="126" ht="60" customHeight="1" s="17">
       <c r="A126" s="7" t="inlineStr">
@@ -18612,14 +18696,18 @@
       </c>
       <c r="Z126" s="11" t="inlineStr">
         <is>
-          <t>namibian.com.na</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA126" s="11" t="n"/>
       <c r="AB126" s="11" t="n"/>
       <c r="AC126" s="11" t="n"/>
       <c r="AD126" s="11" t="n"/>
-      <c r="AE126" s="11" t="n"/>
+      <c r="AE126" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: namibian.com.na</t>
+        </is>
+      </c>
     </row>
     <row r="127" ht="91.5" customHeight="1" s="17">
       <c r="A127" s="7" t="inlineStr">
@@ -19506,14 +19594,18 @@
       </c>
       <c r="Z132" s="11" t="inlineStr">
         <is>
-          <t>areweonair.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA132" s="11" t="n"/>
       <c r="AB132" s="11" t="n"/>
       <c r="AC132" s="11" t="n"/>
       <c r="AD132" s="11" t="n"/>
-      <c r="AE132" s="11" t="n"/>
+      <c r="AE132" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: areweonair.com</t>
+        </is>
+      </c>
     </row>
     <row r="133" ht="91.5" customHeight="1" s="17">
       <c r="A133" s="7" t="inlineStr">
@@ -19622,14 +19714,18 @@
       </c>
       <c r="Z133" s="11" t="inlineStr">
         <is>
-          <t>Read about it</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA133" s="11" t="n"/>
       <c r="AB133" s="11" t="n"/>
       <c r="AC133" s="11" t="n"/>
       <c r="AD133" s="11" t="n"/>
-      <c r="AE133" s="11" t="n"/>
+      <c r="AE133" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: Read about it</t>
+        </is>
+      </c>
     </row>
     <row r="134" ht="75.75" customHeight="1" s="17">
       <c r="A134" s="7" t="inlineStr">
@@ -20542,7 +20638,7 @@
       </c>
       <c r="Z139" s="11" t="inlineStr">
         <is>
-          <t>openmuseum.tw</t>
+          <t>Not publicly accessible: https://openmuseum.tw/muse/exhibition/511cb4fc5aba69444930733eec3ce72e</t>
         </is>
       </c>
       <c r="AA139" s="11" t="n"/>
@@ -22448,7 +22544,7 @@
       </c>
       <c r="Z151" s="11" t="inlineStr">
         <is>
-          <t>mdundo.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA151" s="11" t="n"/>
@@ -22459,7 +22555,11 @@
           <t>music.apple.com</t>
         </is>
       </c>
-      <c r="AE151" s="11" t="n"/>
+      <c r="AE151" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: mdundo.com</t>
+        </is>
+      </c>
     </row>
     <row r="152" ht="91.5" customHeight="1" s="17">
       <c r="A152" s="7" t="inlineStr">
@@ -22784,14 +22884,18 @@
       </c>
       <c r="Z154" s="11" t="inlineStr">
         <is>
-          <t>soundcloud.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA154" s="11" t="n"/>
       <c r="AB154" s="11" t="n"/>
       <c r="AC154" s="11" t="n"/>
       <c r="AD154" s="11" t="n"/>
-      <c r="AE154" s="11" t="n"/>
+      <c r="AE154" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: soundcloud.com</t>
+        </is>
+      </c>
     </row>
     <row r="155" ht="252" customHeight="1" s="17">
       <c r="A155" s="7" t="inlineStr">
@@ -22899,7 +23003,7 @@
       </c>
       <c r="Z155" s="11" t="inlineStr">
         <is>
-          <t>Read about it</t>
+          <t>Read the lyrics</t>
         </is>
       </c>
       <c r="AA155" s="11" t="n"/>
@@ -23008,7 +23112,7 @@
       </c>
       <c r="Z156" s="11" t="inlineStr">
         <is>
-          <t>eurovision.de</t>
+          <t>Read the lyrics</t>
         </is>
       </c>
       <c r="AA156" s="11" t="n"/>
@@ -23734,14 +23838,18 @@
       </c>
       <c r="Z161" s="11" t="inlineStr">
         <is>
-          <t>seychellesnewsagency.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA161" s="11" t="n"/>
       <c r="AB161" s="11" t="n"/>
       <c r="AC161" s="11" t="n"/>
       <c r="AD161" s="11" t="n"/>
-      <c r="AE161" s="11" t="n"/>
+      <c r="AE161" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: seychellesnewsagency.com</t>
+        </is>
+      </c>
     </row>
     <row r="162" ht="91.5" customHeight="1" s="17">
       <c r="A162" s="7" t="inlineStr">
@@ -23850,14 +23958,18 @@
       </c>
       <c r="Z162" s="11" t="inlineStr">
         <is>
-          <t>Read about it</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA162" s="11" t="n"/>
       <c r="AB162" s="11" t="n"/>
       <c r="AC162" s="11" t="n"/>
       <c r="AD162" s="11" t="n"/>
-      <c r="AE162" s="11" t="n"/>
+      <c r="AE162" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: Read about it</t>
+        </is>
+      </c>
     </row>
     <row r="163" ht="91.5" customHeight="1" s="17">
       <c r="A163" s="7" t="inlineStr">
@@ -25048,7 +25160,7 @@
       </c>
       <c r="Z170" s="11" t="inlineStr">
         <is>
-          <t>youtube.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA170" s="11" t="n"/>
@@ -25315,7 +25427,7 @@
       </c>
       <c r="Z172" s="11" t="inlineStr">
         <is>
-          <t>Work / source text</t>
+          <t>Read the text</t>
         </is>
       </c>
       <c r="AA172" s="11" t="inlineStr">
@@ -25338,7 +25450,11 @@
           <t>Additional evidence</t>
         </is>
       </c>
-      <c r="AE172" s="11" t="n"/>
+      <c r="AE172" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: Work / source text</t>
+        </is>
+      </c>
     </row>
     <row r="173" ht="43.5" customHeight="1" s="17">
       <c r="A173" s="7" t="inlineStr">
@@ -26577,14 +26693,18 @@
       </c>
       <c r="Z181" s="11" t="inlineStr">
         <is>
-          <t>tatoli.tl</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA181" s="11" t="n"/>
       <c r="AB181" s="11" t="n"/>
       <c r="AC181" s="11" t="n"/>
       <c r="AD181" s="11" t="n"/>
-      <c r="AE181" s="11" t="n"/>
+      <c r="AE181" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: tatoli.tl</t>
+        </is>
+      </c>
     </row>
     <row r="182" ht="60" customHeight="1" s="17">
       <c r="A182" s="7" t="inlineStr">
@@ -26686,7 +26806,7 @@
       </c>
       <c r="Z182" s="11" t="inlineStr">
         <is>
-          <t>youtube.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA182" s="11" t="n"/>
@@ -27484,7 +27604,7 @@
       </c>
       <c r="Z187" s="11" t="inlineStr">
         <is>
-          <t>science.gov.tm</t>
+          <t>Read about the poet</t>
         </is>
       </c>
       <c r="AA187" s="11" t="n"/>
@@ -27495,7 +27615,11 @@
           <t>search.rsl.ru</t>
         </is>
       </c>
-      <c r="AE187" s="11" t="n"/>
+      <c r="AE187" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: science.gov.tm</t>
+        </is>
+      </c>
     </row>
     <row r="188" ht="43.5" customHeight="1" s="17">
       <c r="A188" s="7" t="inlineStr">
@@ -27597,7 +27721,7 @@
       </c>
       <c r="Z188" s="11" t="inlineStr">
         <is>
-          <t>open.spotify.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA188" s="11" t="n"/>
@@ -27706,14 +27830,18 @@
       </c>
       <c r="Z189" s="11" t="inlineStr">
         <is>
-          <t>bigeye.ug</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA189" s="11" t="n"/>
       <c r="AB189" s="11" t="n"/>
       <c r="AC189" s="11" t="n"/>
       <c r="AD189" s="11" t="n"/>
-      <c r="AE189" s="11" t="n"/>
+      <c r="AE189" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: bigeye.ug</t>
+        </is>
+      </c>
     </row>
     <row r="190" ht="204" customHeight="1" s="17">
       <c r="A190" s="7" t="inlineStr">
@@ -27977,7 +28105,7 @@
       </c>
       <c r="Z191" s="11" t="inlineStr">
         <is>
-          <t>ich.unesco.org</t>
+          <t>Watch the video</t>
         </is>
       </c>
       <c r="AA191" s="11" t="n"/>
@@ -27988,7 +28116,11 @@
           <t>ich.unesco.org</t>
         </is>
       </c>
-      <c r="AE191" s="11" t="n"/>
+      <c r="AE191" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: ich.unesco.org</t>
+        </is>
+      </c>
     </row>
     <row r="192" ht="235.5" customHeight="1" s="17">
       <c r="A192" s="7" t="inlineStr">
@@ -29381,7 +29513,7 @@
       </c>
       <c r="Z200" s="11" t="inlineStr">
         <is>
-          <t>saiabcommons.ru.ac.za</t>
+          <t>Not publicly accessible: https://saiabcommons.ru.ac.za/vital/access/manager/Repository?f1=sm_type%3A"sound+recordings"&amp;f2=sm_subject%3A"Africa+Zambia+Kwawambua+f-za"&amp;sort=sort_ss_sm_creator+asc&amp;view=list</t>
         </is>
       </c>
       <c r="AA200" s="11" t="n"/>
@@ -29389,7 +29521,7 @@
       <c r="AC200" s="11" t="n"/>
       <c r="AD200" s="11" t="inlineStr">
         <is>
-          <t>hdl.handle.net</t>
+          <t>Not publicly accessible: http://hdl.handle.net/10962/205749</t>
         </is>
       </c>
       <c r="AE200" s="11" t="n"/>
@@ -29499,14 +29631,18 @@
       </c>
       <c r="Z201" s="11" t="inlineStr">
         <is>
-          <t>Read about it</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA201" s="11" t="n"/>
       <c r="AB201" s="11" t="n"/>
       <c r="AC201" s="11" t="n"/>
       <c r="AD201" s="11" t="n"/>
-      <c r="AE201" s="11" t="n"/>
+      <c r="AE201" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: Read about it</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <hyperlinks>
@@ -29524,631 +29660,662 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC9" r:id="rId12"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z10" r:id="rId13"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD10" r:id="rId14"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z11" r:id="rId15"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA11" r:id="rId16"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB11" r:id="rId17"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC11" r:id="rId18"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD11" r:id="rId19"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z12" r:id="rId20"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z13" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA13" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC13" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z14" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA14" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB14" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC14" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z15" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA15" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB15" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC15" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z16" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA16" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB16" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC16" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z17" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA17" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB17" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC17" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z18" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z19" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA19" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB19" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC19" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z20" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA20" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB20" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC20" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD20" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z21" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z22" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA22" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB22" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC22" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z23" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA23" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB23" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC23" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z24" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD24" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z25" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA25" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB25" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC25" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD25" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z26" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z27" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA27" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB27" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC27" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z28" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA28" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB28" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC28" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z29" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z30" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA30" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB30" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC30" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z31" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z32" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA32" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB32" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC32" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z33" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z34" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z35" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA35" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB35" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC35" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD35" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z36" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA36" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB36" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC36" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD36" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z37" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z38" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA38" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB38" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC38" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z39" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD39" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z40" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA40" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB40" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC40" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD40" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z41" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA41" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB41" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC41" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z42" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA42" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB42" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC42" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z43" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA43" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB43" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC43" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z44" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD44" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z45" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA45" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB45" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC45" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD45" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z46" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA46" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB46" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC46" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z47" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD47" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE47" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z48" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA48" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB48" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC48" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z49" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA49" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB49" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC49" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z50" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA50" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB50" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC50" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z51" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA51" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB51" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC51" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z52" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z53" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA53" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB53" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC53" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD53" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z54" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z55" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z56" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA56" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB56" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC56" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z57" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA57" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB57" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC57" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z58" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA58" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB58" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC58" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z59" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA59" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB59" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC59" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z60" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z61" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z62" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA62" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB62" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC62" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z63" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z64" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA64" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB64" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC64" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z65" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z66" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA66" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB66" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC66" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z67" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA67" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB67" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC67" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z68" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z69" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z70" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA70" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB70" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC70" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z71" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA71" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB71" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC71" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z72" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA72" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB72" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC72" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD72" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z73" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA73" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB73" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC73" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z74" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD74" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z75" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA75" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB75" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC75" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z76" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z77" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z78" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA78" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB78" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC78" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD78" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z79" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA79" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB79" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC79" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z80" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA80" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB80" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC80" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD80" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE80" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z81" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA81" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB81" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC81" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z82" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA82" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB82" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC82" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z83" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA83" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB83" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC83" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD83" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA84" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB84" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC84" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA85" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB85" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC85" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA86" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB86" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC86" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA87" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB87" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC87" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA88" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB88" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC88" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA89" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB89" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC89" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA90" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB90" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC90" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD90" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA91" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB91" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC91" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA92" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB92" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC92" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD92" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA93" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB93" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC93" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA94" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB94" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC94" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD96" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA97" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB97" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC97" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA98" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB98" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC98" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA100" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB100" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC100" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA101" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB101" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC101" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA102" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB102" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC102" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD102" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA103" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB103" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC103" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD103" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA104" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB104" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC104" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA105" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB105" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC105" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD105" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA106" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB106" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC106" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA107" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB107" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC107" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD107" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD108" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA110" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB110" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC110" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD111" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA113" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB113" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC113" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z115" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA115" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB115" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC115" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z116" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z117" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA117" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB117" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC117" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z118" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z119" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA119" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB119" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC119" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z120" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD120" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z121" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA121" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB121" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC121" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD121" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z122" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA122" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB122" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC122" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z123" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA123" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB123" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC123" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z124" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA124" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB124" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC124" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD124" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z125" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z126" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z127" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA127" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB127" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC127" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD127" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z128" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA128" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB128" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC128" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z129" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA129" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB129" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC129" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z130" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA130" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB130" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC130" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z131" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA131" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB131" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC131" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z132" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z133" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z134" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA134" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB134" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC134" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z135" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA135" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB135" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC135" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z136" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA136" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB136" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC136" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z137" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA137" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB137" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC137" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z138" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA138" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB138" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC138" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z139" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z140" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA140" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB140" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC140" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z141" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA141" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB141" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC141" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z142" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z143" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA143" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB143" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC143" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z144" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA144" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB144" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC144" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z145" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA145" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB145" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC145" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z146" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA146" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB146" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC146" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z147" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA147" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB147" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC147" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z148" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA148" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB148" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC148" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z149" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA149" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB149" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC149" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z150" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA150" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB150" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC150" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD150" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z151" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD151" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z152" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z153" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z154" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z155" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z156" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z157" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA157" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB157" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC157" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD157" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z158" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA158" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB158" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC158" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z159" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z160" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA160" r:id="rId500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB160" r:id="rId501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC160" r:id="rId502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z161" r:id="rId503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z162" r:id="rId504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z163" r:id="rId505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA163" r:id="rId506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB163" r:id="rId507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC163" r:id="rId508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD163" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z164" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA164" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB164" r:id="rId512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC164" r:id="rId513"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z165" r:id="rId514"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA165" r:id="rId515"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB165" r:id="rId516"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC165" r:id="rId517"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z166" r:id="rId518"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z167" r:id="rId519"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA167" r:id="rId520"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB167" r:id="rId521"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC167" r:id="rId522"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD167" r:id="rId523"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z168" r:id="rId524"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA168" r:id="rId525"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB168" r:id="rId526"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC168" r:id="rId527"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z169" r:id="rId528"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA169" r:id="rId529"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB169" r:id="rId530"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC169" r:id="rId531"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z170" r:id="rId532"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z171" r:id="rId533"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA171" r:id="rId534"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB171" r:id="rId535"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC171" r:id="rId536"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z172" r:id="rId537"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA172" r:id="rId538"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB172" r:id="rId539"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC172" r:id="rId540"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD172" r:id="rId541"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z173" r:id="rId542"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z174" r:id="rId543"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z175" r:id="rId544"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA175" r:id="rId545"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB175" r:id="rId546"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC175" r:id="rId547"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z176" r:id="rId548"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA176" r:id="rId549"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB176" r:id="rId550"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC176" r:id="rId551"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z177" r:id="rId552"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA177" r:id="rId553"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB177" r:id="rId554"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC177" r:id="rId555"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z178" r:id="rId556"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA178" r:id="rId557"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB178" r:id="rId558"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC178" r:id="rId559"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z179" r:id="rId560"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA179" r:id="rId561"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB179" r:id="rId562"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC179" r:id="rId563"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD179" r:id="rId564"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z180" r:id="rId565"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA180" r:id="rId566"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB180" r:id="rId567"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC180" r:id="rId568"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z181" r:id="rId569"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z182" r:id="rId570"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD182" r:id="rId571"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z183" r:id="rId572"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA183" r:id="rId573"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB183" r:id="rId574"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC183" r:id="rId575"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z184" r:id="rId576"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA184" r:id="rId577"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB184" r:id="rId578"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC184" r:id="rId579"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD184" r:id="rId580"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z185" r:id="rId581"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA185" r:id="rId582"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB185" r:id="rId583"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC185" r:id="rId584"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD185" r:id="rId585"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z186" r:id="rId586"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA186" r:id="rId587"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB186" r:id="rId588"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC186" r:id="rId589"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z187" r:id="rId590"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD187" r:id="rId591"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z188" r:id="rId592"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z189" r:id="rId593"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z190" r:id="rId594"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA190" r:id="rId595"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB190" r:id="rId596"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC190" r:id="rId597"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD190" r:id="rId598"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z191" r:id="rId599"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD191" r:id="rId600"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z192" r:id="rId601"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA192" r:id="rId602"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB192" r:id="rId603"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC192" r:id="rId604"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z193" r:id="rId605"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA193" r:id="rId606"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB193" r:id="rId607"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC193" r:id="rId608"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z194" r:id="rId609"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA194" r:id="rId610"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB194" r:id="rId611"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC194" r:id="rId612"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z195" r:id="rId613"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA195" r:id="rId614"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB195" r:id="rId615"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC195" r:id="rId616"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z196" r:id="rId617"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA196" r:id="rId618"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB196" r:id="rId619"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC196" r:id="rId620"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z197" r:id="rId621"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA197" r:id="rId622"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB197" r:id="rId623"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC197" r:id="rId624"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z198" r:id="rId625"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA198" r:id="rId626"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB198" r:id="rId627"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC198" r:id="rId628"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z199" r:id="rId629"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA199" r:id="rId630"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB199" r:id="rId631"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC199" r:id="rId632"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z200" r:id="rId633"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD200" r:id="rId634"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z201" r:id="rId635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE10" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z11" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA11" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB11" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC11" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD11" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z12" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE12" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB13" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC13" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z14" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA14" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB14" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC14" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z15" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA15" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB15" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC15" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z16" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA16" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB16" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC16" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z17" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA17" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB17" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC17" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z18" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z19" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA19" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB19" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC19" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z20" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA20" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB20" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC20" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD20" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z21" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z22" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA22" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB22" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC22" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z23" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA23" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB23" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC23" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z24" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD24" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE24" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z25" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA25" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB25" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC25" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD25" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z26" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z27" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA27" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB27" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC27" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z28" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA28" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB28" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC28" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z29" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE29" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z30" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA30" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB30" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC30" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z31" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z32" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA32" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB32" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC32" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z33" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z34" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE34" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z35" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA35" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB35" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC35" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD35" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z36" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA36" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB36" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC36" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD36" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z37" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE37" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z38" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA38" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB38" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC38" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z39" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD39" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z40" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA40" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB40" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC40" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD40" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z41" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA41" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB41" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC41" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z42" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA42" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB42" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC42" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z43" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA43" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB43" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC43" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z44" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD44" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE44" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z45" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA45" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB45" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC45" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD45" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z46" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA46" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB46" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC46" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z47" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD47" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE47" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z48" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA48" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB48" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC48" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z49" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA49" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB49" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC49" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z50" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA50" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB50" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC50" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z51" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA51" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB51" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC51" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z52" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z53" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA53" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB53" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC53" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD53" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z54" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE54" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z55" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE55" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z56" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA56" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB56" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC56" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z57" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA57" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB57" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC57" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z58" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA58" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB58" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC58" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z59" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA59" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB59" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC59" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z60" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z61" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z62" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA62" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB62" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC62" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z63" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE63" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z64" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA64" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB64" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC64" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z65" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z66" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA66" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB66" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC66" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z67" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA67" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB67" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC67" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z68" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE68" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z69" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE69" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z70" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA70" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB70" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC70" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z71" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA71" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB71" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC71" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z72" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA72" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB72" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC72" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD72" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z73" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA73" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB73" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC73" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z74" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD74" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE74" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z75" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA75" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB75" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC75" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z76" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE76" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z77" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z78" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA78" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB78" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC78" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD78" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z79" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA79" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB79" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC79" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z80" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA80" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB80" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC80" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD80" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE80" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z81" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA81" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB81" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC81" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z82" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA82" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB82" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC82" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z83" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA83" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB83" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC83" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD83" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA84" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB84" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC84" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA85" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB85" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC85" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA86" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB86" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC86" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA87" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB87" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC87" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA88" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB88" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC88" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA89" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB89" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC89" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA90" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB90" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC90" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD90" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA91" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB91" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC91" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA92" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB92" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC92" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD92" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA93" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB93" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC93" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA94" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB94" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC94" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE95" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD96" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA97" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB97" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC97" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA98" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB98" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC98" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA100" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB100" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC100" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA101" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB101" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC101" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA102" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB102" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC102" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD102" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA103" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB103" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC103" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD103" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA104" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB104" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC104" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA105" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB105" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC105" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD105" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA106" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB106" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC106" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA107" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB107" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC107" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD107" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE107" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD108" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE109" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA110" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB110" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC110" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD111" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE112" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA113" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB113" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC113" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z115" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA115" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB115" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC115" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z116" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE116" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z117" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA117" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB117" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC117" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z118" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z119" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA119" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB119" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC119" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z120" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD120" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE120" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z121" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA121" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB121" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC121" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD121" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z122" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA122" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB122" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC122" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z123" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA123" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB123" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC123" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z124" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA124" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB124" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC124" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD124" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z125" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE125" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z126" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE126" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z127" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA127" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB127" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC127" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD127" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z128" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA128" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB128" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC128" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z129" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA129" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB129" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC129" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z130" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA130" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB130" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC130" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z131" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA131" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB131" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC131" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z132" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE132" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z133" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE133" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z134" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA134" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB134" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC134" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z135" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA135" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB135" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC135" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z136" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA136" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB136" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC136" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z137" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA137" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB137" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC137" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z138" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA138" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB138" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC138" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z140" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA140" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB140" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC140" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z141" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA141" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB141" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC141" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z142" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z143" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA143" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB143" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC143" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z144" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA144" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB144" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC144" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z145" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA145" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB145" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC145" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z146" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA146" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB146" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC146" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z147" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA147" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB147" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC147" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z148" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA148" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB148" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC148" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z149" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA149" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB149" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC149" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z150" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA150" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB150" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC150" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD150" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z151" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD151" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE151" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z152" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z153" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z154" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE154" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z155" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z156" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z157" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA157" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB157" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC157" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD157" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z158" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA158" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB158" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC158" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z159" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z160" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA160" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB160" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC160" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z161" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE161" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z162" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE162" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z163" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA163" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB163" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC163" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD163" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z164" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA164" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB164" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC164" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z165" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA165" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB165" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC165" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z166" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z167" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA167" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB167" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC167" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD167" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z168" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA168" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB168" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC168" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z169" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA169" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB169" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC169" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z170" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z171" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA171" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB171" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC171" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z172" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA172" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB172" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC172" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD172" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE172" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z173" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z174" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z175" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA175" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB175" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC175" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z176" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA176" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB176" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC176" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z177" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA177" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB177" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC177" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z178" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA178" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB178" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC178" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z179" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA179" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB179" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC179" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD179" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z180" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA180" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB180" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC180" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z181" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE181" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z182" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD182" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z183" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA183" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB183" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC183" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z184" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA184" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB184" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC184" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD184" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z185" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA185" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB185" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC185" r:id="rId613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD185" r:id="rId614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z186" r:id="rId615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA186" r:id="rId616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB186" r:id="rId617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC186" r:id="rId618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z187" r:id="rId619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD187" r:id="rId620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE187" r:id="rId621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z188" r:id="rId622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z189" r:id="rId623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE189" r:id="rId624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z190" r:id="rId625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA190" r:id="rId626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB190" r:id="rId627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC190" r:id="rId628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD190" r:id="rId629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z191" r:id="rId630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD191" r:id="rId631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE191" r:id="rId632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z192" r:id="rId633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA192" r:id="rId634"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB192" r:id="rId635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC192" r:id="rId636"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z193" r:id="rId637"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA193" r:id="rId638"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB193" r:id="rId639"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC193" r:id="rId640"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z194" r:id="rId641"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA194" r:id="rId642"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB194" r:id="rId643"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC194" r:id="rId644"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z195" r:id="rId645"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA195" r:id="rId646"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB195" r:id="rId647"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC195" r:id="rId648"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z196" r:id="rId649"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA196" r:id="rId650"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB196" r:id="rId651"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC196" r:id="rId652"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z197" r:id="rId653"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA197" r:id="rId654"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB197" r:id="rId655"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC197" r:id="rId656"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z198" r:id="rId657"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA198" r:id="rId658"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB198" r:id="rId659"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC198" r:id="rId660"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z199" r:id="rId661"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA199" r:id="rId662"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB199" r:id="rId663"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC199" r:id="rId664"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z201" r:id="rId665"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE201" r:id="rId666"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId636"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId667"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Replace explore entries that had no copy online
- 12 works with nothing a reader could hear or read are replaced by love
  songs and poems from local artists that can be found online: Benin,
  Brunei, Burkina Faso, Kiribati, Lesotho, Luxembourg, Madagascar,
  Myanmar, Palau, Solomon Islands, Turkmenistan and Zambia.
- Bhutan, Fiji, Micronesia and Papua New Guinea keep their works but now
  link to recordings instead of notes and articles.
- Old wording overrides for the replaced entries removed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -3622,34 +3622,34 @@
       </c>
       <c r="D25" s="13" t="inlineStr">
         <is>
-          <t>L’Esclave</t>
+          <t>Les choses de l'amour</t>
         </is>
       </c>
       <c r="E25" s="13" t="inlineStr">
         <is>
-          <t>The Slave</t>
+          <t>The Things of Love</t>
         </is>
       </c>
       <c r="F25" s="13" t="n"/>
       <c r="G25" s="13" t="n"/>
       <c r="H25" s="13" t="inlineStr">
         <is>
-          <t>Félix Couchoro (1900–1968)</t>
+          <t>Madano</t>
         </is>
       </c>
       <c r="I25" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J25" s="13" t="inlineStr">
         <is>
-          <t>Named work (bibliographic and work-specific scholarly evidence)</t>
+          <t>Named work</t>
         </is>
       </c>
       <c r="K25" s="13" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="L25" s="13" t="inlineStr">
@@ -3657,8 +3657,10 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M25" s="14" t="n">
-        <v>1929</v>
+      <c r="M25" s="14" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
       </c>
       <c r="N25" s="13" t="inlineStr">
         <is>
@@ -3668,80 +3670,55 @@
       <c r="O25" s="13" t="n"/>
       <c r="P25" s="13" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="Q25" s="13" t="inlineStr">
         <is>
-          <t>Man author</t>
+          <t>Madano</t>
         </is>
       </c>
       <c r="R25" s="13" t="inlineStr">
         <is>
-          <t>First edition1929, Paris, La Dépêche Africaine; rewritten serial version1962 is separate</t>
-        </is>
-      </c>
-      <c r="S25" s="13" t="inlineStr">
-        <is>
-          <t>1929 original; modern collected edition2005 is a locating reference only</t>
-        </is>
-      </c>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="S25" s="13" t="n"/>
       <c r="T25" s="13" t="inlineStr">
         <is>
-          <t>Akoéba’s adulterous love for Mawoulawoé becomes entangled with murder, inheritance and remorse. A tragic moralising account of romantic passion.</t>
+          <t>The breakout hit of the Cotonou singer Madano, an afrobeat love song sung in French.</t>
         </is>
       </c>
       <c r="U25" s="13" t="inlineStr">
         <is>
-          <t>Couchoro was born in Dahomey, now Benin, and later became a Togolese citizen. Scholarship places this novel on both sides of the Mono in Benin/Togo. Western University lists the original novel in its collected works; Strasbourg thesis describes the lovers. Full1929 copy still needs locating.</t>
-        </is>
-      </c>
-      <c r="V25" s="13" t="inlineStr">
-        <is>
-          <t>Entire1929 novel; obtain original edition before choosing a passage</t>
-        </is>
-      </c>
+          <t>Recording</t>
+        </is>
+      </c>
+      <c r="V25" s="13" t="n"/>
       <c r="W25" s="13" t="inlineStr">
         <is>
-          <t>Country link is birth and shared Benin/Togo setting, not exclusive national ownership. Not a freely licensed2005 edition. The1962 serial revises the1929 novel and must not be substituted without separate review. This row establishes a US-public-domain original lead, not current full-text availability.
-Passage update (29 October 2026): Not filled: no accessible, verified 1929 original text was located for passage selection. A search result for a 1983 reprint does not establish that it reproduces the 1929 wording unchanged. Supply relevant 1929 pages. Keep the existing territorial rights note.</t>
+          <t>Work changed (30 October 2026): replaced L’Esclave (Félix Couchoro (1900–1968)), which had no copy the public can read or hear online, with a work by a local writer or artist that can be found online.</t>
         </is>
       </c>
       <c r="X25" s="13" t="inlineStr">
         <is>
-          <t>US ONLY: original1929 French wording is beyond the95-year publication term. Author died1968, so standard life-plus-70 protection continues through2038 in relevant territories. Do not treat this as open for UK/worldwide publication. Later revisions, notes and translations are excluded.</t>
+          <t>In copyright. Not reproduced; listed with a description and link only.</t>
         </is>
       </c>
       <c r="Y25" s="13" t="inlineStr">
         <is>
-          <t>Work-specific text, date and provenance sources checked29October2026.</t>
+          <t>Official music video on Madano's YouTube channel; Benin Web TV on his 2023 Primud performance</t>
         </is>
       </c>
       <c r="Z25" s="11" t="inlineStr">
         <is>
-          <t>Work / text</t>
-        </is>
-      </c>
-      <c r="AA25" s="11" t="inlineStr">
-        <is>
-          <t>Rights / catalogue</t>
-        </is>
-      </c>
-      <c r="AB25" s="11" t="inlineStr">
-        <is>
-          <t>Date / edition</t>
-        </is>
-      </c>
-      <c r="AC25" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country</t>
-        </is>
-      </c>
-      <c r="AD25" s="11" t="inlineStr">
-        <is>
-          <t>Additional evidence</t>
-        </is>
-      </c>
+          <t>Listen to the song</t>
+        </is>
+      </c>
+      <c r="AA25" s="11" t="n"/>
+      <c r="AB25" s="11" t="n"/>
+      <c r="AC25" s="11" t="n"/>
+      <c r="AD25" s="11" t="n"/>
       <c r="AE25" s="11" t="n"/>
     </row>
     <row r="26" ht="96" customHeight="1" s="17">
@@ -3845,14 +3822,18 @@
       </c>
       <c r="Z26" s="11" t="inlineStr">
         <is>
-          <t>folkways.si.edu</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA26" s="11" t="n"/>
       <c r="AB26" s="11" t="n"/>
       <c r="AC26" s="11" t="n"/>
       <c r="AD26" s="11" t="n"/>
-      <c r="AE26" s="11" t="n"/>
+      <c r="AE26" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: folkways.si.edu</t>
+        </is>
+      </c>
     </row>
     <row r="27" ht="208" customHeight="1" s="17">
       <c r="A27" s="7" t="inlineStr">
@@ -4493,13 +4474,21 @@
           <t>Asia</t>
         </is>
       </c>
-      <c r="D31" s="13" t="n"/>
-      <c r="E31" s="13" t="n"/>
+      <c r="D31" s="13" t="inlineStr">
+        <is>
+          <t>Buat Selamanya</t>
+        </is>
+      </c>
+      <c r="E31" s="13" t="inlineStr">
+        <is>
+          <t>Forever</t>
+        </is>
+      </c>
       <c r="F31" s="13" t="n"/>
       <c r="G31" s="13" t="n"/>
       <c r="H31" s="13" t="inlineStr">
         <is>
-          <t>Malay-speaking pemantun, singers and communities</t>
+          <t>Hill Zaini; written by Amalina Abdullah and Bahri Hj. Ibrahim</t>
         </is>
       </c>
       <c r="I31" s="13" t="inlineStr">
@@ -4509,72 +4498,75 @@
       </c>
       <c r="J31" s="13" t="inlineStr">
         <is>
-          <t>Tradition / repertoire</t>
+          <t>Named work</t>
         </is>
       </c>
       <c r="K31" s="13" t="inlineStr">
         <is>
-          <t>Oral tradition</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="L31" s="13" t="inlineStr">
         <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="M31" s="14" t="n"/>
+          <t>Men</t>
+        </is>
+      </c>
+      <c r="M31" s="14" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
       <c r="N31" s="13" t="inlineStr">
         <is>
-          <t>Malay; maritime Southeast Asia</t>
-        </is>
-      </c>
-      <c r="O31" s="13" t="inlineStr">
-        <is>
-          <t>Pantun</t>
-        </is>
-      </c>
+          <t>Malay</t>
+        </is>
+      </c>
+      <c r="O31" s="13" t="n"/>
       <c r="P31" s="13" t="inlineStr">
         <is>
-          <t>Oral tradition</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="Q31" s="13" t="inlineStr">
         <is>
-          <t>Unknown / not established</t>
-        </is>
-      </c>
-      <c r="R31" s="13" t="n"/>
+          <t>Hill Zaini; written by Amalina Abdullah and Bahri Hj. Ibrahim</t>
+        </is>
+      </c>
+      <c r="R31" s="13" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
       <c r="S31" s="13" t="n"/>
       <c r="T31" s="13" t="inlineStr">
         <is>
-          <t>UNESCO explicitly includes love for a romantic partner among its subjects.</t>
+          <t>An acoustic ballad about a love that lasts for all time; it reached number one on Brunei's Pelangi FM chart.</t>
         </is>
       </c>
       <c r="U31" s="13" t="inlineStr">
         <is>
-          <t>UNESCO nomination 02274 names all three states; shared form, not three different works.</t>
+          <t>Recording</t>
         </is>
       </c>
       <c r="V31" s="13" t="n"/>
       <c r="W31" s="13" t="inlineStr">
         <is>
-          <t>English description only. No individual pantun translated here.
-Passage update (29 October 2026): Not filled: no specific pantun or work identifier is supplied. A tradition-level UNESCO record cannot determine which original verses to quote. Choose a named or numbered romantic pantun and provide its text or a work-specific source.</t>
+          <t>Work changed (30 October 2026): replaced None (Malay-speaking pemantun, singers and communities), which had no copy the public can read or hear online, with a work by a local writer or artist that can be found online.</t>
         </is>
       </c>
       <c r="X31" s="13" t="inlineStr">
         <is>
-          <t>Traditional status does not clear a transcription, translation, arrangement or recording. Consult bearers and relevant rights holders.</t>
+          <t>In copyright. Not reproduced; listed with a description and link only.</t>
         </is>
       </c>
       <c r="Y31" s="13" t="inlineStr">
         <is>
-          <t>UNESCO, Pantun nomination page</t>
+          <t>Official music video (HILLOFFICIAL); Wikipedia: Buat Selamanya</t>
         </is>
       </c>
       <c r="Z31" s="11" t="inlineStr">
         <is>
-          <t>ich.unesco.org</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA31" s="11" t="n"/>
@@ -4772,19 +4764,19 @@
       </c>
       <c r="D33" s="13" t="inlineStr">
         <is>
-          <t>Untitled Gan love song, MR.1968.25.2-B1</t>
+          <t>Ya Maam</t>
         </is>
       </c>
       <c r="E33" s="13" t="inlineStr">
         <is>
-          <t>Untitled Gan love song, MR.1968.25.2-B1</t>
+          <t>It's Me</t>
         </is>
       </c>
       <c r="F33" s="13" t="n"/>
       <c r="G33" s="13" t="n"/>
       <c r="H33" s="13" t="inlineStr">
         <is>
-          <t>Gan performers, names not supplied in listing</t>
+          <t>Amzy</t>
         </is>
       </c>
       <c r="I33" s="13" t="inlineStr">
@@ -4794,7 +4786,7 @@
       </c>
       <c r="J33" s="13" t="inlineStr">
         <is>
-          <t>Untitled / catalogue identifier</t>
+          <t>Named work</t>
         </is>
       </c>
       <c r="K33" s="13" t="inlineStr">
@@ -4804,15 +4796,15 @@
       </c>
       <c r="L33" s="13" t="inlineStr">
         <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="M33" s="14" t="n"/>
-      <c r="N33" s="13" t="inlineStr">
-        <is>
-          <t>Gan community</t>
-        </is>
-      </c>
+          <t>Men</t>
+        </is>
+      </c>
+      <c r="M33" s="14" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="N33" s="13" t="n"/>
       <c r="O33" s="13" t="n"/>
       <c r="P33" s="13" t="inlineStr">
         <is>
@@ -4821,41 +4813,44 @@
       </c>
       <c r="Q33" s="13" t="inlineStr">
         <is>
-          <t>Unknown / not established</t>
-        </is>
-      </c>
-      <c r="R33" s="13" t="n"/>
+          <t>Amzy</t>
+        </is>
+      </c>
+      <c r="R33" s="13" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
       <c r="S33" s="13" t="n"/>
       <c r="T33" s="13" t="inlineStr">
         <is>
-          <t>Institutional item is classified as a love song. Romantic scope needs lyric review.</t>
+          <t>A love song about feelings that refuse to fade despite mistakes, distance and time.</t>
         </is>
       </c>
       <c r="U33" s="13" t="inlineStr">
         <is>
-          <t>Museum catalogue locates item at Loropeni, Burkina Faso. No vernacular title provided.</t>
+          <t>Recording</t>
         </is>
       </c>
       <c r="V33" s="13" t="n"/>
       <c r="W33" s="13" t="inlineStr">
         <is>
-          <t>Catalogue metadata only; no lyric translation or named performers verified.
-Passage update (29 October 2026): Not filled: the archive identifier refers to an untitled Gan recording. No original-language lyric transcript was verified. Supply an authorized transcript with the language and recording identifier; do not invent lyrics from a catalogue description.</t>
+          <t>Work changed (30 October 2026): replaced Untitled Gan love song, MR.1968.25.2-B1 (Gan performers, names not supplied in listing), which had no copy the public can read or hear online, with a work by a local writer or artist that can be found online.</t>
         </is>
       </c>
       <c r="X33" s="13" t="inlineStr">
         <is>
-          <t>Lyric, musical setting, translation, performance and recording rights require separate review. Age or online access is not permission.</t>
+          <t>In copyright. Not reproduced; listed with a description and link only.</t>
         </is>
       </c>
       <c r="Y33" s="13" t="inlineStr">
         <is>
-          <t>Royal Museum for Central Africa, recording MR.1968.25.2-B1</t>
+          <t>Official music video on Amzy's YouTube channel (Destiny Group, Burkina Faso)</t>
         </is>
       </c>
       <c r="Z33" s="11" t="inlineStr">
         <is>
-          <t>music.africamuseum.be</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA33" s="11" t="n"/>
@@ -9440,14 +9435,18 @@
       </c>
       <c r="Z65" s="11" t="inlineStr">
         <is>
-          <t>Read about it</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA65" s="11" t="n"/>
       <c r="AB65" s="11" t="n"/>
       <c r="AC65" s="11" t="n"/>
       <c r="AD65" s="11" t="n"/>
-      <c r="AE65" s="11" t="n"/>
+      <c r="AE65" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: Read about it</t>
+        </is>
+      </c>
     </row>
     <row r="66" ht="204" customHeight="1" s="17">
       <c r="A66" s="7" t="inlineStr">
@@ -14185,19 +14184,15 @@
       </c>
       <c r="D96" s="13" t="inlineStr">
         <is>
-          <t>Ti kareia te man (KN052)</t>
-        </is>
-      </c>
-      <c r="E96" s="13" t="inlineStr">
-        <is>
-          <t>We throw the birds (opening phrase; KN052; literal historical German gloss)</t>
-        </is>
-      </c>
+          <t>Ai kamira tangiran neiei</t>
+        </is>
+      </c>
+      <c r="E96" s="13" t="n"/>
       <c r="F96" s="13" t="n"/>
       <c r="G96" s="13" t="n"/>
       <c r="H96" s="13" t="inlineStr">
         <is>
-          <t>Bakaia; Nonouti singers and dancers</t>
+          <t>Raikaon Tumoa</t>
         </is>
       </c>
       <c r="I96" s="13" t="inlineStr">
@@ -14217,13 +14212,17 @@
       </c>
       <c r="L96" s="13" t="inlineStr">
         <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="M96" s="14" t="n"/>
+          <t>Men</t>
+        </is>
+      </c>
+      <c r="M96" s="14" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
       <c r="N96" s="13" t="inlineStr">
         <is>
-          <t>Gilbertese</t>
+          <t>Gilbertese (Kiribati)</t>
         </is>
       </c>
       <c r="O96" s="13" t="n"/>
@@ -14234,50 +14233,50 @@
       </c>
       <c r="Q96" s="13" t="inlineStr">
         <is>
-          <t>Unknown / not established</t>
-        </is>
-      </c>
-      <c r="R96" s="13" t="n"/>
+          <t>Raikaon Tumoa</t>
+        </is>
+      </c>
+      <c r="R96" s="13" t="inlineStr">
+        <is>
+          <t>2010</t>
+        </is>
+      </c>
       <c r="S96" s="13" t="n"/>
       <c r="T96" s="13" t="inlineStr">
         <is>
-          <t>Wolfgang Kempf's study traces the text as a love affair using fishing imagery.</t>
+          <t>A love song by the I-Kiribati singer Raikaon Tumoa, one of Kiribati's most popular songs of 2010.</t>
         </is>
       </c>
       <c r="U96" s="13" t="inlineStr">
         <is>
-          <t>Koch collection: Rotima, Nonouti18November1963,15:25; wa n tarawa dance.</t>
+          <t>Recording</t>
         </is>
       </c>
       <c r="V96" s="13" t="n"/>
       <c r="W96" s="13" t="inlineStr">
         <is>
-          <t>Koch German translation1964 cited; complex metaphors and age difference warrant contextual review.</t>
+          <t>Work changed (30 October 2026): replaced Ti kareia te man (KN052) (Bakaia; Nonouti singers and dancers), which had no copy the public can read or hear online, with a work by a local writer or artist that can be found online.</t>
         </is>
       </c>
       <c r="X96" s="13" t="inlineStr">
         <is>
-          <t>Lyric, musical setting, translation, performance and recording rights require separate review. Age or online access is not permission.</t>
+          <t>In copyright. Not reproduced; listed with a description and link only.</t>
         </is>
       </c>
       <c r="Y96" s="13" t="inlineStr">
         <is>
-          <t>Koch Tape Collection digitized list; author study</t>
+          <t>Upload on Raikaon Tumoa's YouTube channel</t>
         </is>
       </c>
       <c r="Z96" s="11" t="inlineStr">
         <is>
-          <t>d-nb.info</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA96" s="11" t="n"/>
       <c r="AB96" s="11" t="n"/>
       <c r="AC96" s="11" t="n"/>
-      <c r="AD96" s="11" t="inlineStr">
-        <is>
-          <t>researchgate.net</t>
-        </is>
-      </c>
+      <c r="AD96" s="11" t="n"/>
       <c r="AE96" s="11" t="n"/>
     </row>
     <row r="97" ht="91.5" customHeight="1" s="17">
@@ -15079,34 +15078,34 @@
       </c>
       <c r="D102" s="13" t="inlineStr">
         <is>
-          <t>Pitseng</t>
+          <t>Lerato</t>
         </is>
       </c>
       <c r="E102" s="13" t="inlineStr">
         <is>
-          <t>Pitseng (place name; retained)</t>
+          <t>Love</t>
         </is>
       </c>
       <c r="F102" s="13" t="n"/>
       <c r="G102" s="13" t="n"/>
       <c r="H102" s="13" t="inlineStr">
         <is>
-          <t>Thomas Mofolo (1876–1948)</t>
+          <t>Sannere featuring Drigga</t>
         </is>
       </c>
       <c r="I102" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J102" s="13" t="inlineStr">
         <is>
-          <t>Named work (catalogue; text access limited)</t>
+          <t>Named work</t>
         </is>
       </c>
       <c r="K102" s="13" t="inlineStr">
         <is>
-          <t>Prose / novel</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="L102" s="13" t="inlineStr">
@@ -15114,8 +15113,10 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M102" s="14" t="n">
-        <v>1910</v>
+      <c r="M102" s="14" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
       </c>
       <c r="N102" s="13" t="inlineStr">
         <is>
@@ -15125,79 +15126,55 @@
       <c r="O102" s="13" t="n"/>
       <c r="P102" s="13" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="Q102" s="13" t="inlineStr">
         <is>
-          <t>Man author</t>
+          <t>Sannere featuring Drigga</t>
         </is>
       </c>
       <c r="R102" s="13" t="inlineStr">
         <is>
-          <t>1910 book edition; serialised 1909–1910</t>
-        </is>
-      </c>
-      <c r="S102" s="13" t="inlineStr">
-        <is>
-          <t>Historical work reproduced in linked digital source; modern editorial material is separate</t>
-        </is>
-      </c>
+          <t>2023</t>
+        </is>
+      </c>
+      <c r="S102" s="13" t="n"/>
       <c r="T102" s="13" t="inlineStr">
         <is>
-          <t>Alfred Phakoe and Aria Sebaka discover reciprocal love and choose marriage; their partnership forms part of the novel’s Christian and Basotho social vision.</t>
+          <t>A love song by the Lesotho musician Sannere; lerato is the Sesotho word for love.</t>
         </is>
       </c>
       <c r="U102" s="13" t="inlineStr">
         <is>
-          <t>Original Sesotho work identified in Morija Sesuto Book Depot catalogue; Limakatso Chaka’s scholarly article confirms 1910 and the central love story.</t>
-        </is>
-      </c>
-      <c r="V102" s="13" t="inlineStr">
-        <is>
-          <t>Alfred and Aria’s courtship and wedding, toward the end of the novel</t>
-        </is>
-      </c>
+          <t>Recording</t>
+        </is>
+      </c>
+      <c r="V102" s="13" t="n"/>
       <c r="W102" s="13" t="inlineStr">
         <is>
-          <t>Linked catalogue describes a later Sesotho printing. Complete original text not verified online. Daniel P. Kunene’s modern English translation has separate rights and is not supplied as reusable.</t>
+          <t>Work changed (30 October 2026): replaced Pitseng (Thomas Mofolo (1876–1948)), which had no copy the public can read or hear online, with a work by a local writer or artist that can be found online.</t>
         </is>
       </c>
       <c r="X102" s="13" t="inlineStr">
         <is>
-          <t>Historical original text: standard life-plus-70 term has expired; author died 1948. Assessment excludes modern translations, commentary, editorial alterations, musical settings and recordings. Territorial and unusual publication-history exceptions are not comprehensively assessed.</t>
+          <t>In copyright. Not reproduced; listed with a description and link only.</t>
         </is>
       </c>
       <c r="Y102" s="13" t="inlineStr">
         <is>
-          <t>Original Sesotho work identified in Morija Sesuto Book Depot catalogue; Limakatso Chaka’s scholarly article confirms 1910 and the central love story.</t>
+          <t>Official video on the Sannere Music YouTube channel</t>
         </is>
       </c>
       <c r="Z102" s="11" t="inlineStr">
         <is>
-          <t>Work catalogue / preview</t>
-        </is>
-      </c>
-      <c r="AA102" s="11" t="inlineStr">
-        <is>
-          <t>Reuse basis / copyright duration</t>
-        </is>
-      </c>
-      <c r="AB102" s="11" t="inlineStr">
-        <is>
-          <t>Date / edition evidence</t>
-        </is>
-      </c>
-      <c r="AC102" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country evidence</t>
-        </is>
-      </c>
-      <c r="AD102" s="11" t="inlineStr">
-        <is>
-          <t>Additional evidence</t>
-        </is>
-      </c>
+          <t>Listen to the song</t>
+        </is>
+      </c>
+      <c r="AA102" s="11" t="n"/>
+      <c r="AB102" s="11" t="n"/>
+      <c r="AC102" s="11" t="n"/>
+      <c r="AD102" s="11" t="n"/>
       <c r="AE102" s="11" t="n"/>
     </row>
     <row r="103" ht="91.5" customHeight="1" s="17">
@@ -15851,34 +15828,34 @@
       </c>
       <c r="D107" s="13" t="inlineStr">
         <is>
-          <t>D’Mumm Séis oder De Geescht</t>
+          <t>Margréitchen</t>
         </is>
       </c>
       <c r="E107" s="13" t="inlineStr">
         <is>
-          <t>Aunt Séis, or The Ghost (Séis retained as a name)</t>
+          <t>Little Daisy</t>
         </is>
       </c>
       <c r="F107" s="13" t="n"/>
       <c r="G107" s="13" t="n"/>
       <c r="H107" s="13" t="inlineStr">
         <is>
-          <t>Dicks / Edmond de la Fontaine (1823–1891)</t>
+          <t>Michel Lentz</t>
         </is>
       </c>
       <c r="I107" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J107" s="13" t="inlineStr">
         <is>
-          <t>Named dramatic work (excerpt)</t>
+          <t>Named work</t>
         </is>
       </c>
       <c r="K107" s="13" t="inlineStr">
         <is>
-          <t>Drama / operetta</t>
+          <t>Poetry</t>
         </is>
       </c>
       <c r="L107" s="13" t="inlineStr">
@@ -15886,8 +15863,10 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M107" s="14" t="n">
-        <v>1855</v>
+      <c r="M107" s="14" t="inlineStr">
+        <is>
+          <t>1864</t>
+        </is>
       </c>
       <c r="N107" s="13" t="inlineStr">
         <is>
@@ -15897,84 +15876,56 @@
       <c r="O107" s="13" t="n"/>
       <c r="P107" s="13" t="inlineStr">
         <is>
-          <t>Drama / operetta</t>
+          <t>Poem</t>
         </is>
       </c>
       <c r="Q107" s="13" t="inlineStr">
         <is>
-          <t>Man author</t>
+          <t>Michel Lentz (1820–1893)</t>
         </is>
       </c>
       <c r="R107" s="13" t="inlineStr">
         <is>
-          <t>1855 premiere</t>
-        </is>
-      </c>
-      <c r="S107" s="13" t="inlineStr">
-        <is>
-          <t>Historical work reproduced in linked digital source; modern editorial material is separate</t>
-        </is>
-      </c>
+          <t>1864</t>
+        </is>
+      </c>
+      <c r="S107" s="13" t="n"/>
       <c r="T107" s="13" t="inlineStr">
         <is>
-          <t>A comic marriage plot contrasts young Péiter’s love for Kettéi with schemes to gain the aunt’s money by impersonating a ghost.</t>
+          <t>A spring song in which the poet loves the daisy best of all the flowers, because his sweetheart shares its name.</t>
         </is>
       </c>
       <c r="U107" s="13" t="inlineStr">
         <is>
-          <t>National Library of Luxembourg / Cedom teaching material reproduces historical dialogue and explains the 1855 plot. Philharmonie catalogue distinguishes the original from later arrangements.</t>
-        </is>
-      </c>
-      <c r="V107" s="13" t="inlineStr">
-        <is>
-          <t>D’Mumm Séis section, printed teaching pages 10–11</t>
-        </is>
-      </c>
+          <t>Published text</t>
+        </is>
+      </c>
+      <c r="V107" s="13" t="n"/>
       <c r="W107" s="13" t="inlineStr">
         <is>
-          <t>Original text and music by Dicks are distinct from modern stage rewrites, teaching material, arrangements and recordings. Use the historical dialogue or lyric, not the modern synopsis.</t>
+          <t>Work changed (30 October 2026): replaced D’Mumm Séis oder De Geescht (Dicks / Edmond de la Fontaine (1823–1891)), which had no copy the public can read or hear online, with a work by a local writer or artist that can be found online.</t>
         </is>
       </c>
       <c r="X107" s="13" t="inlineStr">
         <is>
-          <t>Historical original text: standard life-plus-70 term has expired; author died 1891. Assessment excludes modern translations, commentary, editorial alterations, musical settings and recordings. Territorial and unusual publication-history exceptions are not comprehensively assessed.</t>
+          <t>Public domain (author died 1893).</t>
         </is>
       </c>
       <c r="Y107" s="13" t="inlineStr">
         <is>
-          <t>National Library of Luxembourg / Cedom teaching material reproduces historical dialogue and explains the 1855 plot. Philharmonie catalogue distinguishes the original from later arrangements.</t>
+          <t>Wikisource: Margréitchen (Michel Lentz, 1864)</t>
         </is>
       </c>
       <c r="Z107" s="11" t="inlineStr">
         <is>
-          <t>Read about it</t>
-        </is>
-      </c>
-      <c r="AA107" s="11" t="inlineStr">
-        <is>
-          <t>Reuse basis / copyright duration</t>
-        </is>
-      </c>
-      <c r="AB107" s="11" t="inlineStr">
-        <is>
-          <t>Date / edition evidence</t>
-        </is>
-      </c>
-      <c r="AC107" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country evidence</t>
-        </is>
-      </c>
-      <c r="AD107" s="11" t="inlineStr">
-        <is>
-          <t>Additional evidence</t>
-        </is>
-      </c>
-      <c r="AE107" s="11" t="inlineStr">
-        <is>
-          <t>Earlier link: Work / source text</t>
-        </is>
-      </c>
+          <t>Read the text</t>
+        </is>
+      </c>
+      <c r="AA107" s="11" t="n"/>
+      <c r="AB107" s="11" t="n"/>
+      <c r="AC107" s="11" t="n"/>
+      <c r="AD107" s="11" t="n"/>
+      <c r="AE107" s="11" t="n"/>
     </row>
     <row r="108" ht="60" customHeight="1" s="17">
       <c r="A108" s="7" t="inlineStr">
@@ -15992,13 +15943,21 @@
           <t>Africa</t>
         </is>
       </c>
-      <c r="D108" s="13" t="n"/>
-      <c r="E108" s="13" t="n"/>
+      <c r="D108" s="13" t="inlineStr">
+        <is>
+          <t>Fitiavana Mahery</t>
+        </is>
+      </c>
+      <c r="E108" s="13" t="inlineStr">
+        <is>
+          <t>Strong Love</t>
+        </is>
+      </c>
       <c r="F108" s="13" t="n"/>
       <c r="G108" s="13" t="n"/>
       <c r="H108" s="13" t="inlineStr">
         <is>
-          <t>Malagasy community poets</t>
+          <t>Mr Sayda</t>
         </is>
       </c>
       <c r="I108" s="13" t="inlineStr">
@@ -16008,81 +15967,81 @@
       </c>
       <c r="J108" s="13" t="inlineStr">
         <is>
-          <t>Tradition / repertoire</t>
+          <t>Named work</t>
         </is>
       </c>
       <c r="K108" s="13" t="inlineStr">
         <is>
-          <t>Oral tradition</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="L108" s="13" t="inlineStr">
         <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="M108" s="14" t="n"/>
+          <t>Men</t>
+        </is>
+      </c>
+      <c r="M108" s="14" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
       <c r="N108" s="13" t="inlineStr">
         <is>
           <t>Malagasy</t>
         </is>
       </c>
-      <c r="O108" s="13" t="inlineStr">
-        <is>
-          <t>Hainteny</t>
-        </is>
-      </c>
+      <c r="O108" s="13" t="n"/>
       <c r="P108" s="13" t="inlineStr">
         <is>
-          <t>Oral tradition</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="Q108" s="13" t="inlineStr">
         <is>
-          <t>Unknown (traditional / collective authorship)</t>
-        </is>
-      </c>
-      <c r="R108" s="13" t="n"/>
+          <t>Mr Sayda</t>
+        </is>
+      </c>
+      <c r="R108" s="13" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
       <c r="S108" s="13" t="n"/>
       <c r="T108" s="13" t="inlineStr">
         <is>
-          <t>Publisher documents love as the predominant theme and separate love section.</t>
+          <t>A Malagasy love song; fitiavana means love and mahery means strong.</t>
         </is>
       </c>
       <c r="U108" s="13" t="inlineStr">
         <is>
-          <t>Leonard Fox bilingual457-poem edition, Bucknell University Press1990, ISBN083875175X.</t>
+          <t>Recording</t>
         </is>
       </c>
       <c r="V108" s="13" t="n"/>
       <c r="W108" s="13" t="inlineStr">
         <is>
-          <t>Leonard Fox English translation; tradition-level verification, individual poem and passage still to select.</t>
+          <t>Work changed (30 October 2026): replaced None (Malagasy community poets), which had no copy the public can read or hear online, with a work by a local writer or artist that can be found online.</t>
         </is>
       </c>
       <c r="X108" s="13" t="inlineStr">
         <is>
-          <t>Traditional status does not clear a transcription, translation, arrangement or recording. Consult bearers and relevant rights holders.</t>
+          <t>In copyright. Not reproduced; listed with a description and link only.</t>
         </is>
       </c>
       <c r="Y108" s="13" t="inlineStr">
         <is>
-          <t>Bucknell University Press; catalogue</t>
+          <t>Official video on Mr Sayda's YouTube channel</t>
         </is>
       </c>
       <c r="Z108" s="11" t="inlineStr">
         <is>
-          <t>www1.bucknell.edu</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA108" s="11" t="n"/>
       <c r="AB108" s="11" t="n"/>
       <c r="AC108" s="11" t="n"/>
-      <c r="AD108" s="11" t="inlineStr">
-        <is>
-          <t>iucat.iu.edu</t>
-        </is>
-      </c>
+      <c r="AD108" s="11" t="n"/>
       <c r="AE108" s="11" t="n"/>
     </row>
     <row r="109" ht="60" customHeight="1" s="17">
@@ -17431,14 +17390,18 @@
       </c>
       <c r="Z118" s="11" t="inlineStr">
         <is>
-          <t>folkways-media.si.edu</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA118" s="11" t="n"/>
       <c r="AB118" s="11" t="n"/>
       <c r="AC118" s="11" t="n"/>
       <c r="AD118" s="11" t="n"/>
-      <c r="AE118" s="11" t="n"/>
+      <c r="AE118" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: folkways-media.si.edu</t>
+        </is>
+      </c>
     </row>
     <row r="119" ht="108" customHeight="1" s="17">
       <c r="A119" s="7" t="inlineStr">
@@ -18501,19 +18464,19 @@
       </c>
       <c r="D125" s="13" t="inlineStr">
         <is>
-          <t>Throw them away</t>
+          <t>အချစ်ဆိုတာလျှို့ဝှက်ချက်တစ်ခုပါ</t>
         </is>
       </c>
       <c r="E125" s="13" t="inlineStr">
         <is>
-          <t>Throw them away</t>
+          <t>Love Is a Secret</t>
         </is>
       </c>
       <c r="F125" s="13" t="n"/>
       <c r="G125" s="13" t="n"/>
       <c r="H125" s="13" t="inlineStr">
         <is>
-          <t>Kyi Aye</t>
+          <t>Sai Htee Saing</t>
         </is>
       </c>
       <c r="I125" s="13" t="inlineStr">
@@ -18528,12 +18491,12 @@
       </c>
       <c r="K125" s="13" t="inlineStr">
         <is>
-          <t>Poetry</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="L125" s="13" t="inlineStr">
         <is>
-          <t>Women</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="M125" s="14" t="n"/>
@@ -18545,56 +18508,52 @@
       <c r="O125" s="13" t="n"/>
       <c r="P125" s="13" t="inlineStr">
         <is>
-          <t>Poem</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="Q125" s="13" t="inlineStr">
         <is>
-          <t>Woman</t>
+          <t>Sai Htee Saing</t>
         </is>
       </c>
       <c r="R125" s="13" t="n"/>
       <c r="S125" s="13" t="n"/>
       <c r="T125" s="13" t="inlineStr">
         <is>
-          <t>Speaker addresses love and rejects jewels in favour of attachment; romantic interpretation needs full contextual review.</t>
+          <t>A love song by Sai Htee Saing (1950–2008), the Shan singer-songwriter loved across Myanmar.</t>
         </is>
       </c>
       <c r="U125" s="13" t="inlineStr">
         <is>
-          <t>Bilingual poem in Global New Light of Myanmar, 15 February 2026, p.8.</t>
+          <t>Recording</t>
         </is>
       </c>
       <c r="V125" s="13" t="n"/>
       <c r="W125" s="13" t="inlineStr">
         <is>
-          <t>Translated by Myint Zan; contemporary translation rights require review.</t>
+          <t>Work changed (30 October 2026): replaced Throw them away (Kyi Aye), which had no copy the public can read or hear online, with a work by a local writer or artist that can be found online.</t>
         </is>
       </c>
       <c r="X125" s="13" t="inlineStr">
         <is>
-          <t>Review original text, edition and any translation separately. Website permission does not transfer to this book.</t>
+          <t>In copyright. Not reproduced; listed with a description and link only.</t>
         </is>
       </c>
       <c r="Y125" s="13" t="inlineStr">
         <is>
-          <t>Newspaper bilingual text and translator note</t>
+          <t>Official audio on the Sai Htee Saing YouTube channel</t>
         </is>
       </c>
       <c r="Z125" s="11" t="inlineStr">
         <is>
-          <t>Read about the poet</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA125" s="11" t="n"/>
       <c r="AB125" s="11" t="n"/>
       <c r="AC125" s="11" t="n"/>
       <c r="AD125" s="11" t="n"/>
-      <c r="AE125" s="11" t="inlineStr">
-        <is>
-          <t>Earlier link: mdn.gov.mm</t>
-        </is>
-      </c>
+      <c r="AE125" s="11" t="n"/>
     </row>
     <row r="126" ht="60" customHeight="1" s="17">
       <c r="A126" s="7" t="inlineStr">
@@ -20556,19 +20515,15 @@
       </c>
       <c r="D139" s="13" t="inlineStr">
         <is>
-          <t>Tia urungulel a Dirachebibech el mora Gertou el chad ra Ngheangel</t>
-        </is>
-      </c>
-      <c r="E139" s="13" t="inlineStr">
-        <is>
-          <t>Dirachebibech going to Gertou of Ngheangel (descriptive rendering; exact wording needs verification)</t>
-        </is>
-      </c>
+          <t>Sumech e Tmanges</t>
+        </is>
+      </c>
+      <c r="E139" s="13" t="n"/>
       <c r="F139" s="13" t="n"/>
       <c r="G139" s="13" t="n"/>
       <c r="H139" s="13" t="inlineStr">
         <is>
-          <t>Traditional; collected Osamu Yamaguchi</t>
+          <t>Traditional Palauan love song; sung by March Kloulubak</t>
         </is>
       </c>
       <c r="I139" s="13" t="inlineStr">
@@ -20588,10 +20543,14 @@
       </c>
       <c r="L139" s="13" t="inlineStr">
         <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="M139" s="14" t="n"/>
+          <t>Men</t>
+        </is>
+      </c>
+      <c r="M139" s="14" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="N139" s="13" t="inlineStr">
         <is>
           <t>Palauan</t>
@@ -20605,40 +20564,44 @@
       </c>
       <c r="Q139" s="13" t="inlineStr">
         <is>
-          <t>Unknown (traditional / collective authorship)</t>
-        </is>
-      </c>
-      <c r="R139" s="13" t="n"/>
+          <t>Traditional Palauan love song; sung by March Kloulubak</t>
+        </is>
+      </c>
+      <c r="R139" s="13" t="inlineStr">
+        <is>
+          <t>2025</t>
+        </is>
+      </c>
       <c r="S139" s="13" t="n"/>
       <c r="T139" s="13" t="inlineStr">
         <is>
-          <t>Museum identifies wishful love of Dirachebibech for Gertau of Ngheangel.</t>
+          <t>A much-loved Palauan love song, sung here by March Kloulubak.</t>
         </is>
       </c>
       <c r="U139" s="13" t="inlineStr">
         <is>
-          <t>Recorded15May1965 Ngeremlengui, Palau; reel36 side2 track3.</t>
+          <t>Recording</t>
         </is>
       </c>
       <c r="V139" s="13" t="n"/>
       <c r="W139" s="13" t="inlineStr">
         <is>
-          <t>Palauan song and Japanese manuscript annotations; English museum synopsis is not a full lyric translation. Rights restricted to viewing.</t>
+          <t>Work changed (30 October 2026): replaced Tia urungulel a Dirachebibech el mora Gertou el chad ra Ngheangel (Traditional; collected Osamu Yamaguchi), which had no copy the public can read or hear online, with a work by a local writer or artist that can be found online.</t>
         </is>
       </c>
       <c r="X139" s="13" t="inlineStr">
         <is>
-          <t>Lyric, musical setting, translation, performance and recording rights require separate review. Age or online access is not permission.</t>
+          <t>In copyright. Not reproduced; listed with a description and link only.</t>
         </is>
       </c>
       <c r="Y139" s="13" t="inlineStr">
         <is>
-          <t>National Taiwan Normal University Music Digital Archive, Sound Memories of Past Palau</t>
+          <t>Performance on March Kloulubak's YouTube channel</t>
         </is>
       </c>
       <c r="Z139" s="11" t="inlineStr">
         <is>
-          <t>Not publicly accessible: https://openmuseum.tw/muse/exhibition/511cb4fc5aba69444930733eec3ce72e</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA139" s="11" t="n"/>
@@ -21105,14 +21068,18 @@
       </c>
       <c r="Z142" s="11" t="inlineStr">
         <is>
-          <t>folkways-media.si.edu</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA142" s="11" t="n"/>
       <c r="AB142" s="11" t="n"/>
       <c r="AC142" s="11" t="n"/>
       <c r="AD142" s="11" t="n"/>
-      <c r="AE142" s="11" t="n"/>
+      <c r="AE142" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: folkways-media.si.edu</t>
+        </is>
+      </c>
     </row>
     <row r="143" ht="91.5" customHeight="1" s="17">
       <c r="A143" s="7" t="inlineStr">
@@ -24505,19 +24472,19 @@
       </c>
       <c r="D166" s="13" t="inlineStr">
         <is>
-          <t>Nuu isiusu</t>
+          <t>Ghema Mi Lovem You</t>
         </is>
       </c>
       <c r="E166" s="13" t="inlineStr">
         <is>
-          <t>To Enumerate One's Feelings (Love Song)</t>
+          <t>I Love You</t>
         </is>
       </c>
       <c r="F166" s="13" t="n"/>
       <c r="G166" s="13" t="n"/>
       <c r="H166" s="13" t="inlineStr">
         <is>
-          <t>Areare women: Aroia, Alice Waltemaeana, Ester Abinamae, Helen Rarisiwa (group credit tracks33-37)</t>
+          <t>Real 17 featuring Slum Kid</t>
         </is>
       </c>
       <c r="I166" s="13" t="inlineStr">
@@ -24537,13 +24504,17 @@
       </c>
       <c r="L166" s="13" t="inlineStr">
         <is>
-          <t>Women</t>
-        </is>
-      </c>
-      <c r="M166" s="14" t="n"/>
+          <t>Men</t>
+        </is>
+      </c>
+      <c r="M166" s="14" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
       <c r="N166" s="13" t="inlineStr">
         <is>
-          <t>Areare</t>
+          <t>Solomon Islands Pijin</t>
         </is>
       </c>
       <c r="O166" s="13" t="n"/>
@@ -24554,40 +24525,44 @@
       </c>
       <c r="Q166" s="13" t="inlineStr">
         <is>
-          <t>Women (credited performers); authorship unknown</t>
-        </is>
-      </c>
-      <c r="R166" s="13" t="n"/>
+          <t>Real 17 featuring Slum Kid</t>
+        </is>
+      </c>
+      <c r="R166" s="13" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
       <c r="S166" s="13" t="n"/>
       <c r="T166" s="13" t="inlineStr">
         <is>
-          <t>Liner notes identify a woman expressing feelings about her lover, often with a friend singing second part.</t>
+          <t>A love song from the Solomon Islands; mi lovem you is Pijin for I love you.</t>
         </is>
       </c>
       <c r="U166" s="13" t="inlineStr">
         <is>
-          <t>MCM3007 The Sounds of Bamboo track37; Ohio Cultural Centre, Malaita, December1988; MABO documentation project.</t>
+          <t>Recording</t>
         </is>
       </c>
       <c r="V166" s="13" t="n"/>
       <c r="W166" s="13" t="inlineStr">
         <is>
-          <t>English notes translated Tokiko Nobusawa; full lyric translation not supplied. Track-specific singer within group to confirm.</t>
+          <t>Work changed (30 October 2026): replaced Nuu isiusu (Areare women: Aroia, Alice Waltemaeana, Ester Abinamae, Helen Rarisiwa (group credit tracks33-37)), which had no copy the public can read or hear online, with a work by a local writer or artist that can be found online.</t>
         </is>
       </c>
       <c r="X166" s="13" t="inlineStr">
         <is>
-          <t>Lyric, musical setting, translation, performance and recording rights require separate review. Age or online access is not permission.</t>
+          <t>In copyright. Not reproduced; listed with a description and link only.</t>
         </is>
       </c>
       <c r="Y166" s="13" t="inlineStr">
         <is>
-          <t>Multicultural Media / MABO project, Solomon Islands National Museum and Osaka University</t>
+          <t>Official music video on the Real 17 YouTube channel</t>
         </is>
       </c>
       <c r="Z166" s="11" t="inlineStr">
         <is>
-          <t>tronsvt.com</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA166" s="11" t="n"/>
@@ -27522,19 +27497,15 @@
       </c>
       <c r="D187" s="13" t="inlineStr">
         <is>
-          <t>Zohre and Tahir</t>
-        </is>
-      </c>
-      <c r="E187" s="13" t="inlineStr">
-        <is>
-          <t>Zohre and Tahir (the lovers' names)</t>
-        </is>
-      </c>
+          <t>My love</t>
+        </is>
+      </c>
+      <c r="E187" s="13" t="n"/>
       <c r="F187" s="13" t="n"/>
       <c r="G187" s="13" t="n"/>
       <c r="H187" s="13" t="inlineStr">
         <is>
-          <t>Mollanepes</t>
+          <t>Jeren Halnazarowa and MAD Nazarov; words Annameret Gurbanow; music Mekan Kakaýew</t>
         </is>
       </c>
       <c r="I187" s="13" t="inlineStr">
@@ -27549,77 +27520,77 @@
       </c>
       <c r="K187" s="13" t="inlineStr">
         <is>
-          <t>Narrative verse / epic</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="L187" s="13" t="inlineStr">
         <is>
-          <t>Men</t>
-        </is>
-      </c>
-      <c r="M187" s="14" t="n"/>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="M187" s="14" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
       <c r="N187" s="13" t="inlineStr">
         <is>
-          <t>Turkmen</t>
+          <t>Turkmen and English</t>
         </is>
       </c>
       <c r="O187" s="13" t="n"/>
       <c r="P187" s="13" t="inlineStr">
         <is>
-          <t>Verse epic</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="Q187" s="13" t="inlineStr">
         <is>
-          <t>Man</t>
-        </is>
-      </c>
-      <c r="R187" s="13" t="n"/>
+          <t>Jeren Halnazarowa and MAD Nazarov; words Annameret Gurbanow; music Mekan Kakaýew</t>
+        </is>
+      </c>
+      <c r="R187" s="13" t="inlineStr">
+        <is>
+          <t>2024</t>
+        </is>
+      </c>
       <c r="S187" s="13" t="n"/>
       <c r="T187" s="13" t="inlineStr">
         <is>
-          <t>Academy study prints lovers' laments and compares Mollanepes and Sayadi versions.</t>
+          <t>A duet in which a young man and woman promise to love each other truly.</t>
         </is>
       </c>
       <c r="U187" s="13" t="inlineStr">
         <is>
-          <t>1956 Ashgabat Turkmengosizdat edition, 185 pages; shared transregional story adapted by Turkmen author.</t>
+          <t>Recording</t>
         </is>
       </c>
       <c r="V187" s="13" t="n"/>
       <c r="W187" s="13" t="inlineStr">
         <is>
-          <t>Russian translation credited T. Ozerskaya and A. Tarkovsky in 1956 catalogue. English lyric translation not established.</t>
+          <t>Work changed (30 October 2026): replaced Zohre and Tahir (Mollanepes), which had no copy the public can read or hear online, with a work by a local writer or artist that can be found online.</t>
         </is>
       </c>
       <c r="X187" s="13" t="inlineStr">
         <is>
-          <t>Review original text, edition and any translation separately. Website permission does not transfer to this book.</t>
+          <t>In copyright. Not reproduced; listed with a description and link only.</t>
         </is>
       </c>
       <c r="Y187" s="13" t="inlineStr">
         <is>
-          <t>Turkmen Academy of Sciences journal; edition</t>
+          <t>Official video on Jeren Halnazarowa's YouTube channel</t>
         </is>
       </c>
       <c r="Z187" s="11" t="inlineStr">
         <is>
-          <t>Read about the poet</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA187" s="11" t="n"/>
       <c r="AB187" s="11" t="n"/>
       <c r="AC187" s="11" t="n"/>
-      <c r="AD187" s="11" t="inlineStr">
-        <is>
-          <t>search.rsl.ru</t>
-        </is>
-      </c>
-      <c r="AE187" s="11" t="inlineStr">
-        <is>
-          <t>Earlier link: science.gov.tm</t>
-        </is>
-      </c>
+      <c r="AD187" s="11" t="n"/>
+      <c r="AE187" s="11" t="n"/>
     </row>
     <row r="188" ht="43.5" customHeight="1" s="17">
       <c r="A188" s="7" t="inlineStr">
@@ -29431,19 +29402,15 @@
       </c>
       <c r="D200" s="13" t="inlineStr">
         <is>
-          <t>Nalemntemwa amabala e</t>
-        </is>
-      </c>
-      <c r="E200" s="13" t="inlineStr">
-        <is>
-          <t>Nalemntemwa amabala e — English meaning not yet verified</t>
-        </is>
-      </c>
+          <t>I Love You</t>
+        </is>
+      </c>
+      <c r="E200" s="13" t="n"/>
       <c r="F200" s="13" t="n"/>
       <c r="G200" s="13" t="n"/>
       <c r="H200" s="13" t="inlineStr">
         <is>
-          <t>Bemba boys; collector Hugh Tracey; composer unspecified</t>
+          <t>Chile One MrZambia</t>
         </is>
       </c>
       <c r="I200" s="13" t="inlineStr">
@@ -29466,12 +29433,12 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M200" s="14" t="n"/>
-      <c r="N200" s="13" t="inlineStr">
-        <is>
-          <t>Bemba</t>
-        </is>
-      </c>
+      <c r="M200" s="14" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
+      <c r="N200" s="13" t="n"/>
       <c r="O200" s="13" t="n"/>
       <c r="P200" s="13" t="inlineStr">
         <is>
@@ -29480,50 +29447,50 @@
       </c>
       <c r="Q200" s="13" t="inlineStr">
         <is>
-          <t>Boys (performers); composer unknown</t>
-        </is>
-      </c>
-      <c r="R200" s="13" t="n"/>
+          <t>Chile One MrZambia</t>
+        </is>
+      </c>
+      <c r="R200" s="13" t="inlineStr">
+        <is>
+          <t>2022</t>
+        </is>
+      </c>
       <c r="S200" s="13" t="n"/>
       <c r="T200" s="13" t="inlineStr">
         <is>
-          <t>Archive describes love for a girl using a food metaphor.</t>
+          <t>A love song written and sung by Chile One MrZambia, one of Zambia's most popular singers.</t>
         </is>
       </c>
       <c r="U200" s="13" t="inlineStr">
         <is>
-          <t>Kwawambua, 28 July 1949; ILAM HTFT055-C56, research C3P11.</t>
+          <t>Recording</t>
         </is>
       </c>
       <c r="V200" s="13" t="n"/>
       <c r="W200" s="13" t="inlineStr">
         <is>
-          <t>English catalogue description. No complete translation or narrator identification.</t>
+          <t>Work changed (30 October 2026): replaced Nalemntemwa amabala e (Bemba boys; collector Hugh Tracey; composer unspecified), which had no copy the public can read or hear online, with a work by a local writer or artist that can be found online.</t>
         </is>
       </c>
       <c r="X200" s="13" t="inlineStr">
         <is>
-          <t>Lyric, musical setting, translation, performance and recording rights require separate review. Age or online access is not permission.</t>
+          <t>In copyright. Not reproduced; listed with a description and link only.</t>
         </is>
       </c>
       <c r="Y200" s="13" t="inlineStr">
         <is>
-          <t>Rhodes University repository / ILAM; handle</t>
+          <t>Official music video on the Chile One Mr Zambia YouTube channel</t>
         </is>
       </c>
       <c r="Z200" s="11" t="inlineStr">
         <is>
-          <t>Not publicly accessible: https://saiabcommons.ru.ac.za/vital/access/manager/Repository?f1=sm_type%3A"sound+recordings"&amp;f2=sm_subject%3A"Africa+Zambia+Kwawambua+f-za"&amp;sort=sort_ss_sm_creator+asc&amp;view=list</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA200" s="11" t="n"/>
       <c r="AB200" s="11" t="n"/>
       <c r="AC200" s="11" t="n"/>
-      <c r="AD200" s="11" t="inlineStr">
-        <is>
-          <t>Not publicly accessible: http://hdl.handle.net/10962/205749</t>
-        </is>
-      </c>
+      <c r="AD200" s="11" t="n"/>
       <c r="AE200" s="11" t="n"/>
     </row>
     <row r="201" ht="108" customHeight="1" s="17">
@@ -29711,611 +29678,599 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD24" r:id="rId63"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE24" r:id="rId64"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z25" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA25" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB25" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC25" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD25" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z26" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z27" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA27" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB27" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC27" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z28" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA28" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB28" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC28" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z29" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE29" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z30" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA30" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB30" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC30" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z31" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z32" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA32" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB32" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC32" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z33" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z34" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE34" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z35" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA35" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB35" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC35" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD35" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z36" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA36" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB36" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC36" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD36" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z37" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE37" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z38" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA38" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB38" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC38" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z39" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD39" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z40" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA40" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB40" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC40" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD40" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z41" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA41" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB41" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC41" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z42" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA42" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB42" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC42" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z43" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA43" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB43" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC43" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z44" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD44" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE44" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z45" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA45" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB45" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC45" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD45" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z46" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA46" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB46" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC46" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z47" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD47" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE47" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z48" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA48" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB48" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC48" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z49" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA49" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB49" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC49" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z50" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA50" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB50" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC50" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z51" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA51" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB51" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC51" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z52" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z53" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA53" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB53" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC53" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD53" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z54" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE54" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z55" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE55" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z56" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA56" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB56" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC56" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z57" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA57" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB57" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC57" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z58" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA58" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB58" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC58" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z59" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA59" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB59" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC59" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z60" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z61" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z62" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA62" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB62" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC62" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z63" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE63" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z64" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA64" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB64" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC64" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z65" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z66" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA66" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB66" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC66" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z67" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA67" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB67" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC67" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z68" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE68" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z69" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE69" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z70" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA70" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB70" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC70" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z71" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA71" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB71" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC71" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z72" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA72" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB72" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC72" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD72" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z73" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA73" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB73" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC73" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z74" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD74" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE74" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z75" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA75" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB75" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC75" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z76" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE76" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z77" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z78" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA78" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB78" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC78" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD78" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z79" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA79" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB79" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC79" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z80" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA80" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB80" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC80" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD80" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE80" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z81" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA81" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB81" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC81" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z82" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA82" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB82" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC82" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z83" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA83" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB83" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC83" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD83" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA84" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB84" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC84" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA85" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB85" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC85" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA86" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB86" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC86" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA87" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB87" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC87" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA88" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB88" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC88" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA89" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB89" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC89" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA90" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB90" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC90" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD90" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA91" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB91" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC91" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA92" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB92" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC92" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD92" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA93" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB93" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC93" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA94" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB94" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC94" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE95" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD96" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA97" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB97" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC97" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA98" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB98" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC98" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA100" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB100" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC100" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA101" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB101" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC101" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA102" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB102" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC102" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD102" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA103" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB103" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC103" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD103" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA104" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB104" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC104" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA105" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB105" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC105" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD105" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA106" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB106" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC106" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA107" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB107" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC107" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD107" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE107" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD108" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE109" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA110" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB110" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC110" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD111" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE112" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA113" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB113" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC113" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z115" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA115" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB115" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC115" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z116" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE116" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z117" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA117" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB117" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC117" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z118" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z119" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA119" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB119" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC119" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z120" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD120" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE120" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z121" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA121" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB121" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC121" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD121" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z122" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA122" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB122" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC122" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z123" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA123" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB123" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC123" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z124" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA124" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB124" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC124" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD124" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z125" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE125" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z126" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE126" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z127" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA127" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB127" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC127" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD127" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z128" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA128" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB128" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC128" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z129" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA129" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB129" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC129" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z130" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA130" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB130" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC130" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z131" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA131" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB131" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC131" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z132" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE132" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z133" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE133" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z134" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA134" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB134" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC134" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z135" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA135" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB135" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC135" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z136" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA136" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB136" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC136" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z137" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA137" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB137" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC137" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z138" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA138" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB138" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC138" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z140" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA140" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB140" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC140" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z141" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA141" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB141" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC141" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z142" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z143" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA143" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB143" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC143" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z144" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA144" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB144" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC144" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z145" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA145" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB145" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC145" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z146" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA146" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB146" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC146" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z147" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA147" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB147" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC147" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z148" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA148" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB148" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC148" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z149" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA149" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB149" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC149" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z150" r:id="rId500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA150" r:id="rId501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB150" r:id="rId502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC150" r:id="rId503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD150" r:id="rId504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z151" r:id="rId505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD151" r:id="rId506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE151" r:id="rId507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z152" r:id="rId508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z153" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z154" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE154" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z155" r:id="rId512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z156" r:id="rId513"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z157" r:id="rId514"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA157" r:id="rId515"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB157" r:id="rId516"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC157" r:id="rId517"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD157" r:id="rId518"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z158" r:id="rId519"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA158" r:id="rId520"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB158" r:id="rId521"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC158" r:id="rId522"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z159" r:id="rId523"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z160" r:id="rId524"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA160" r:id="rId525"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB160" r:id="rId526"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC160" r:id="rId527"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z161" r:id="rId528"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE161" r:id="rId529"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z162" r:id="rId530"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE162" r:id="rId531"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z163" r:id="rId532"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA163" r:id="rId533"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB163" r:id="rId534"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC163" r:id="rId535"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD163" r:id="rId536"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z164" r:id="rId537"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA164" r:id="rId538"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB164" r:id="rId539"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC164" r:id="rId540"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z165" r:id="rId541"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA165" r:id="rId542"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB165" r:id="rId543"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC165" r:id="rId544"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z166" r:id="rId545"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z167" r:id="rId546"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA167" r:id="rId547"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB167" r:id="rId548"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC167" r:id="rId549"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD167" r:id="rId550"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z168" r:id="rId551"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA168" r:id="rId552"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB168" r:id="rId553"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC168" r:id="rId554"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z169" r:id="rId555"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA169" r:id="rId556"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB169" r:id="rId557"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC169" r:id="rId558"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z170" r:id="rId559"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z171" r:id="rId560"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA171" r:id="rId561"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB171" r:id="rId562"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC171" r:id="rId563"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z172" r:id="rId564"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA172" r:id="rId565"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB172" r:id="rId566"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC172" r:id="rId567"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD172" r:id="rId568"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE172" r:id="rId569"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z173" r:id="rId570"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z174" r:id="rId571"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z175" r:id="rId572"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA175" r:id="rId573"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB175" r:id="rId574"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC175" r:id="rId575"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z176" r:id="rId576"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA176" r:id="rId577"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB176" r:id="rId578"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC176" r:id="rId579"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z177" r:id="rId580"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA177" r:id="rId581"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB177" r:id="rId582"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC177" r:id="rId583"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z178" r:id="rId584"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA178" r:id="rId585"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB178" r:id="rId586"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC178" r:id="rId587"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z179" r:id="rId588"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA179" r:id="rId589"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB179" r:id="rId590"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC179" r:id="rId591"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD179" r:id="rId592"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z180" r:id="rId593"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA180" r:id="rId594"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB180" r:id="rId595"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC180" r:id="rId596"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z181" r:id="rId597"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE181" r:id="rId598"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z182" r:id="rId599"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD182" r:id="rId600"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z183" r:id="rId601"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA183" r:id="rId602"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB183" r:id="rId603"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC183" r:id="rId604"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z184" r:id="rId605"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA184" r:id="rId606"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB184" r:id="rId607"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC184" r:id="rId608"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD184" r:id="rId609"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z185" r:id="rId610"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA185" r:id="rId611"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB185" r:id="rId612"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC185" r:id="rId613"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD185" r:id="rId614"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z186" r:id="rId615"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA186" r:id="rId616"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB186" r:id="rId617"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC186" r:id="rId618"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z187" r:id="rId619"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD187" r:id="rId620"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE187" r:id="rId621"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z188" r:id="rId622"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z189" r:id="rId623"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE189" r:id="rId624"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z190" r:id="rId625"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA190" r:id="rId626"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB190" r:id="rId627"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC190" r:id="rId628"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD190" r:id="rId629"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z191" r:id="rId630"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD191" r:id="rId631"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE191" r:id="rId632"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z192" r:id="rId633"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA192" r:id="rId634"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB192" r:id="rId635"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC192" r:id="rId636"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z193" r:id="rId637"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA193" r:id="rId638"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB193" r:id="rId639"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC193" r:id="rId640"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z194" r:id="rId641"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA194" r:id="rId642"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB194" r:id="rId643"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC194" r:id="rId644"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z195" r:id="rId645"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA195" r:id="rId646"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB195" r:id="rId647"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC195" r:id="rId648"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z196" r:id="rId649"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA196" r:id="rId650"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB196" r:id="rId651"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC196" r:id="rId652"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z197" r:id="rId653"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA197" r:id="rId654"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB197" r:id="rId655"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC197" r:id="rId656"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z198" r:id="rId657"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA198" r:id="rId658"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB198" r:id="rId659"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC198" r:id="rId660"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z199" r:id="rId661"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA199" r:id="rId662"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB199" r:id="rId663"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC199" r:id="rId664"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z201" r:id="rId665"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE201" r:id="rId666"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z26" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE26" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z27" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA27" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB27" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC27" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z28" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA28" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB28" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC28" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z29" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE29" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z30" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA30" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB30" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC30" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z31" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z32" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA32" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB32" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC32" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z33" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z34" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE34" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z35" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA35" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB35" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC35" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD35" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z36" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA36" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB36" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC36" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD36" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z37" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE37" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z38" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA38" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB38" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC38" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z39" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD39" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z40" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA40" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB40" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC40" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD40" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z41" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA41" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB41" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC41" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z42" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA42" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB42" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC42" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z43" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA43" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB43" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC43" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z44" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD44" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE44" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z45" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA45" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB45" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC45" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD45" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z46" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA46" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB46" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC46" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z47" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD47" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE47" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z48" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA48" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB48" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC48" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z49" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA49" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB49" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC49" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z50" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA50" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB50" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC50" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z51" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA51" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB51" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC51" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z52" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z53" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA53" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB53" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC53" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD53" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z54" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE54" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z55" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE55" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z56" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA56" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB56" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC56" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z57" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA57" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB57" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC57" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z58" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA58" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB58" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC58" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z59" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA59" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB59" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC59" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z60" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z61" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z62" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA62" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB62" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC62" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z63" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE63" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z64" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA64" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB64" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC64" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z65" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE65" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z66" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA66" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB66" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC66" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z67" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA67" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB67" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC67" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z68" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE68" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z69" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE69" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z70" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA70" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB70" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC70" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z71" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA71" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB71" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC71" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z72" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA72" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB72" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC72" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD72" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z73" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA73" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB73" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC73" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z74" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD74" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE74" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z75" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA75" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB75" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC75" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z76" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE76" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z77" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z78" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA78" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB78" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC78" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD78" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z79" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA79" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB79" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC79" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z80" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA80" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB80" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC80" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD80" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE80" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z81" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA81" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB81" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC81" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z82" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA82" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB82" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC82" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z83" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA83" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB83" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC83" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD83" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA84" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB84" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC84" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA85" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB85" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC85" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA86" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB86" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC86" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA87" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB87" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC87" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA88" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB88" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC88" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA89" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB89" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC89" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA90" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB90" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC90" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD90" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA91" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB91" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC91" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA92" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB92" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC92" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD92" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA93" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB93" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC93" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA94" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB94" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC94" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE95" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA97" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB97" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC97" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA98" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB98" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC98" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA100" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB100" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC100" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA101" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB101" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC101" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA103" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB103" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC103" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD103" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA104" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB104" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC104" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA105" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB105" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC105" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD105" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA106" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB106" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC106" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE109" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA110" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB110" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC110" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD111" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE112" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA113" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB113" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC113" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z115" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA115" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB115" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC115" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z116" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE116" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z117" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA117" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB117" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC117" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z118" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE118" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z119" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA119" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB119" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC119" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z120" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD120" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE120" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z121" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA121" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB121" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC121" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD121" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z122" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA122" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB122" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC122" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z123" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA123" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB123" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC123" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z124" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA124" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB124" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC124" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD124" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z125" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z126" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE126" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z127" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA127" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB127" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC127" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD127" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z128" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA128" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB128" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC128" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z129" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA129" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB129" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC129" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z130" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA130" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB130" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC130" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z131" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA131" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB131" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC131" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z132" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE132" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z133" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE133" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z134" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA134" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB134" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC134" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z135" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA135" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB135" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC135" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z136" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA136" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB136" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC136" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z137" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA137" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB137" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC137" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z138" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA138" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB138" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC138" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z139" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z140" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA140" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB140" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC140" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z141" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA141" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB141" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC141" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z142" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE142" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z143" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA143" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB143" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC143" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z144" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA144" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB144" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC144" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z145" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA145" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB145" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC145" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z146" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA146" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB146" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC146" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z147" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA147" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB147" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC147" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z148" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA148" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB148" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC148" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z149" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA149" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB149" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC149" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z150" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA150" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB150" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC150" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD150" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z151" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD151" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE151" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z152" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z153" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z154" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE154" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z155" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z156" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z157" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA157" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB157" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC157" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD157" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z158" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA158" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB158" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC158" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z159" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z160" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA160" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB160" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC160" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z161" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE161" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z162" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE162" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z163" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA163" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB163" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC163" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD163" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z164" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA164" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB164" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC164" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z165" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA165" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB165" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC165" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z166" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z167" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA167" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB167" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC167" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD167" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z168" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA168" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB168" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC168" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z169" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA169" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB169" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC169" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z170" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z171" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA171" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB171" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC171" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z172" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA172" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB172" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC172" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD172" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE172" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z173" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z174" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z175" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA175" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB175" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC175" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z176" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA176" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB176" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC176" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z177" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA177" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB177" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC177" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z178" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA178" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB178" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC178" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z179" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA179" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB179" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC179" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD179" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z180" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA180" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB180" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC180" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z181" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE181" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z182" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD182" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z183" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA183" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB183" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC183" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z184" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA184" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB184" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC184" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD184" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z185" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA185" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB185" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC185" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD185" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z186" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA186" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB186" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC186" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z187" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z188" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z189" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE189" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z190" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA190" r:id="rId613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB190" r:id="rId614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC190" r:id="rId615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD190" r:id="rId616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z191" r:id="rId617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD191" r:id="rId618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE191" r:id="rId619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z192" r:id="rId620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA192" r:id="rId621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB192" r:id="rId622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC192" r:id="rId623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z193" r:id="rId624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA193" r:id="rId625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB193" r:id="rId626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC193" r:id="rId627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z194" r:id="rId628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA194" r:id="rId629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB194" r:id="rId630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC194" r:id="rId631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z195" r:id="rId632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA195" r:id="rId633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB195" r:id="rId634"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC195" r:id="rId635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z196" r:id="rId636"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA196" r:id="rId637"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB196" r:id="rId638"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC196" r:id="rId639"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z197" r:id="rId640"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA197" r:id="rId641"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB197" r:id="rId642"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC197" r:id="rId643"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z198" r:id="rId644"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA198" r:id="rId645"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB198" r:id="rId646"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC198" r:id="rId647"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z199" r:id="rId648"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA199" r:id="rId649"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB199" r:id="rId650"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC199" r:id="rId651"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z200" r:id="rId652"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z201" r:id="rId653"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE201" r:id="rId654"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId667"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId655"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Joan Armatrading to St Kitts; Antiguan poet Joy Lawrence for Antigua
- "Love and Affection" moves to Saint Kitts and Nevis, where Armatrading
  was born, replacing Infamus's song of love for the island.
- Antigua and Barbuda now has Joy Lawrence reading her poem "Love Me"
  on the Commonwealth Poetry Podcast.
- New reader link label: "Listen to the poem".

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -1674,19 +1674,15 @@
       </c>
       <c r="D12" s="13" t="inlineStr">
         <is>
-          <t>Love and Affection</t>
-        </is>
-      </c>
-      <c r="E12" s="13" t="inlineStr">
-        <is>
-          <t>Love and Affection</t>
-        </is>
-      </c>
+          <t>Love Me</t>
+        </is>
+      </c>
+      <c r="E12" s="13" t="n"/>
       <c r="F12" s="13" t="n"/>
       <c r="G12" s="13" t="n"/>
       <c r="H12" s="13" t="inlineStr">
         <is>
-          <t>Joan Armatrading</t>
+          <t>Joy Lawrence</t>
         </is>
       </c>
       <c r="I12" s="13" t="inlineStr">
@@ -1701,7 +1697,7 @@
       </c>
       <c r="K12" s="13" t="inlineStr">
         <is>
-          <t>Song</t>
+          <t>Poetry</t>
         </is>
       </c>
       <c r="L12" s="13" t="inlineStr">
@@ -1709,7 +1705,11 @@
           <t>Women</t>
         </is>
       </c>
-      <c r="M12" s="14" t="n"/>
+      <c r="M12" s="14" t="inlineStr">
+        <is>
+          <t>2023</t>
+        </is>
+      </c>
       <c r="N12" s="13" t="inlineStr">
         <is>
           <t>English</t>
@@ -1718,57 +1718,52 @@
       <c r="O12" s="13" t="n"/>
       <c r="P12" s="13" t="inlineStr">
         <is>
-          <t>Song</t>
+          <t>Poem, read by the poet</t>
         </is>
       </c>
       <c r="Q12" s="13" t="inlineStr">
         <is>
-          <t>Woman</t>
+          <t>Joy Lawrence OH, Antiguan educator, folklorist and poet</t>
         </is>
       </c>
       <c r="R12" s="13" t="n"/>
       <c r="S12" s="13" t="n"/>
       <c r="T12" s="13" t="inlineStr">
         <is>
-          <t>Named romantic song by a songwriter whose early childhood included Antigua.</t>
+          <t>The Antiguan poet and folklorist Joy Lawrence reads her poem “Love Me” in the Commonwealth Poetry Podcast's episode on Antigua and Barbuda.</t>
         </is>
       </c>
       <c r="U12" s="13" t="inlineStr">
         <is>
-          <t>Childhood Antigua connection: moved there age three before Britain; composed and recorded in British career, not an Antiguan folk song.</t>
+          <t>Reading by the poet, Commonwealth Poetry Podcast episode 37 (29 October 2023)</t>
         </is>
       </c>
       <c r="V12" s="13" t="n"/>
       <c r="W12" s="13" t="inlineStr">
         <is>
-          <t>Original English; shared biographical lead, not exclusive national provenance.
-Passage update (29 October 2026): Not filled: modern copyrighted English-language song. The supplied interview citation is not a verified lyric transcript. Supply the lyric text; because the original is English, no language translation is needed.</t>
+          <t>Work changed (30 October 2026): Joan Armatrading, Love and Affection, moved to Saint Kitts and Nevis (her birthplace); replaced by a poem by an Antiguan poet.</t>
         </is>
       </c>
       <c r="X12" s="13" t="inlineStr">
         <is>
-          <t>Lyric, musical setting, translation, performance and recording rights require separate review. Age or online access is not permission.</t>
+          <t>In copyright. Not reproduced; listed with a description and link only.</t>
         </is>
       </c>
       <c r="Y12" s="13" t="inlineStr">
         <is>
-          <t>Musician June 1985, Rob Tannenbaum interview</t>
+          <t>Commonwealth Poetry Podcast, “Next stop Antigua &amp; Barbuda with Joy Lawrence OH”</t>
         </is>
       </c>
       <c r="Z12" s="11" t="inlineStr">
         <is>
-          <t>Listen to the song</t>
+          <t>Listen to the poem</t>
         </is>
       </c>
       <c r="AA12" s="11" t="n"/>
       <c r="AB12" s="11" t="n"/>
       <c r="AC12" s="11" t="n"/>
       <c r="AD12" s="11" t="n"/>
-      <c r="AE12" s="11" t="inlineStr">
-        <is>
-          <t>Earlier link: worldradiohistory.com</t>
-        </is>
-      </c>
+      <c r="AE12" s="11" t="n"/>
     </row>
     <row r="13" ht="235.5" customHeight="1" s="17">
       <c r="A13" s="7" t="inlineStr">
@@ -22546,19 +22541,15 @@
       </c>
       <c r="D152" s="13" t="inlineStr">
         <is>
-          <t>Love St Kitts</t>
-        </is>
-      </c>
-      <c r="E152" s="13" t="inlineStr">
-        <is>
-          <t>Love St Kitts</t>
-        </is>
-      </c>
+          <t>Love and Affection</t>
+        </is>
+      </c>
+      <c r="E152" s="13" t="n"/>
       <c r="F152" s="13" t="n"/>
       <c r="G152" s="13" t="n"/>
       <c r="H152" s="13" t="inlineStr">
         <is>
-          <t>Infamus</t>
+          <t>Joan Armatrading</t>
         </is>
       </c>
       <c r="I152" s="13" t="inlineStr">
@@ -22578,10 +22569,14 @@
       </c>
       <c r="L152" s="13" t="inlineStr">
         <is>
-          <t>Men</t>
-        </is>
-      </c>
-      <c r="M152" s="14" t="n"/>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="M152" s="14" t="inlineStr">
+        <is>
+          <t>1976</t>
+        </is>
+      </c>
       <c r="N152" s="13" t="inlineStr">
         <is>
           <t>English</t>
@@ -22590,57 +22585,60 @@
       <c r="O152" s="13" t="n"/>
       <c r="P152" s="13" t="inlineStr">
         <is>
-          <t>Lyric poem</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="Q152" s="13" t="inlineStr">
         <is>
-          <t>Man author</t>
+          <t>Joan Armatrading (born Basseterre, 1950)</t>
         </is>
       </c>
       <c r="R152" s="13" t="inlineStr">
         <is>
-          <t>Twenty-first century</t>
+          <t>1976</t>
         </is>
       </c>
       <c r="S152" s="13" t="n"/>
       <c r="T152" s="13" t="inlineStr">
         <is>
-          <t>A song of love for St Kitts by the Kittitian artist Infamus.</t>
+          <t>A slow-burning love song in which the singer asks for more than friendship; it was her first hit, in 1976.</t>
         </is>
       </c>
       <c r="U152" s="13" t="inlineStr">
         <is>
-          <t>Official music video (TRUCAPO channel, YouTube)</t>
+          <t>Recording; performance on BBC Later... with Jools Holland</t>
         </is>
       </c>
       <c r="V152" s="13" t="n"/>
       <c r="W152" s="13" t="inlineStr">
         <is>
-          <t>Scottish-born colonial resident author, not an Indigenous island voice. Graphic tragic ending and colonial racial representation. First-publication date should not be confused with the linked 1767 anthology.
-Work changed (29 October 2026): James Grainger’s ballad, by a Scottish plantation doctor, is replaced by a song by a Kittitian artist, chosen by the project. Listed with a description and link only.</t>
+          <t>Work changed (30 October 2026): moved here from Antigua and Barbuda, as Armatrading was born in Basseterre; replaced Infamus, Love St Kitts (a song of love for the island).</t>
         </is>
       </c>
       <c r="X152" s="13" t="inlineStr">
         <is>
-          <t>In copyright. Not reproduced; listed with a link.</t>
+          <t>In copyright. Not reproduced; listed with a description and link only.</t>
         </is>
       </c>
       <c r="Y152" s="13" t="inlineStr">
         <is>
-          <t>YouTube: Infamus – Love St Kitts (official music video)</t>
+          <t>Joan Armatrading, Love and Affection (A&amp;M, 1976); BBC Music performance on YouTube</t>
         </is>
       </c>
       <c r="Z152" s="11" t="inlineStr">
         <is>
-          <t>Watch the video</t>
+          <t>Listen to the song</t>
         </is>
       </c>
       <c r="AA152" s="11" t="n"/>
       <c r="AB152" s="11" t="n"/>
       <c r="AC152" s="11" t="n"/>
       <c r="AD152" s="11" t="n"/>
-      <c r="AE152" s="11" t="n"/>
+      <c r="AE152" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: Infamus, Love St Kitts</t>
+        </is>
+      </c>
     </row>
     <row r="153" ht="43.5" customHeight="1" s="17">
       <c r="A153" s="7" t="inlineStr">
@@ -29634,482 +29632,482 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC11" r:id="rId19"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD11" r:id="rId20"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z12" r:id="rId21"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE12" r:id="rId22"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z13" r:id="rId23"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA13" r:id="rId24"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB13" r:id="rId25"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC13" r:id="rId26"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z14" r:id="rId27"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA14" r:id="rId28"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB14" r:id="rId29"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC14" r:id="rId30"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z15" r:id="rId31"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA15" r:id="rId32"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB15" r:id="rId33"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC15" r:id="rId34"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z16" r:id="rId35"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA16" r:id="rId36"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB16" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC16" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z17" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA17" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB17" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC17" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z18" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z19" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA19" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB19" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC19" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z20" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA20" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB20" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC20" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD20" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z21" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z22" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA22" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB22" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC22" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z23" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA23" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB23" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC23" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z24" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD24" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE24" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z25" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z26" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE26" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z27" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA27" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB27" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC27" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z28" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA28" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB28" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC28" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z29" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE29" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z30" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA30" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB30" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC30" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z31" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z32" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA32" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB32" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC32" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z33" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z34" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE34" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z35" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA35" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB35" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC35" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD35" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z36" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA36" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB36" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC36" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD36" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z37" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE37" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z38" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA38" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB38" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC38" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z39" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD39" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z40" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA40" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB40" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC40" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD40" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z41" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA41" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB41" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC41" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z42" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA42" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB42" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC42" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z43" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA43" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB43" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC43" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z44" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD44" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE44" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z45" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA45" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB45" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC45" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD45" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z46" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA46" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB46" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC46" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z47" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD47" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE47" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z48" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA48" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB48" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC48" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z49" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA49" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB49" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC49" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z50" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA50" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB50" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC50" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z51" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA51" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB51" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC51" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z52" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z53" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA53" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB53" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC53" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD53" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z54" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE54" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z55" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE55" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z56" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA56" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB56" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC56" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z57" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA57" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB57" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC57" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z58" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA58" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB58" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC58" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z59" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA59" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB59" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC59" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z60" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z61" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z62" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA62" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB62" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC62" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z63" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE63" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z64" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA64" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB64" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC64" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z65" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE65" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z66" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA66" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB66" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC66" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z67" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA67" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB67" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC67" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z68" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE68" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z69" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE69" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z70" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA70" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB70" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC70" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z71" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA71" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB71" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC71" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z72" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA72" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB72" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC72" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD72" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z73" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA73" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB73" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC73" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z74" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD74" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE74" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z75" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA75" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB75" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC75" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z76" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE76" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z77" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z78" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA78" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB78" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC78" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD78" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z79" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA79" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB79" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC79" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z80" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA80" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB80" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC80" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD80" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE80" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z81" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA81" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB81" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC81" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z82" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA82" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB82" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC82" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z83" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA83" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB83" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC83" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD83" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA84" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB84" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC84" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA85" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB85" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC85" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA86" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB86" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC86" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA87" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB87" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC87" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA88" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB88" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC88" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA89" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB89" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC89" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA90" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB90" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC90" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD90" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA91" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB91" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC91" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA92" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB92" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC92" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD92" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA93" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB93" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC93" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA94" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB94" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC94" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE95" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA97" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB97" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC97" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA98" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB98" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC98" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA100" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB100" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC100" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA101" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB101" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC101" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA103" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB103" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC103" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD103" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA104" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB104" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC104" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA105" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB105" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC105" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD105" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA106" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB106" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC106" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE109" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA110" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB110" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC110" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD111" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE112" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA113" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB113" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC113" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z115" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA115" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB115" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC115" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z116" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE116" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z117" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA117" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB117" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC117" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z118" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE118" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z119" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA119" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB119" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC119" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z120" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD120" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE120" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z121" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA121" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB121" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC121" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD121" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z122" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA122" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB122" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC122" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z123" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA123" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB123" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC123" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z124" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA124" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB124" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC124" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD124" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z125" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z126" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE126" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z127" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA127" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB127" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC127" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD127" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z128" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA128" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB128" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC128" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z129" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA129" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB129" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC129" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z130" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA130" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB130" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC130" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z131" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA131" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB131" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC131" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z132" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE132" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z133" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE133" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z134" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA134" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB134" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC134" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z135" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA135" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB135" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC135" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z136" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA136" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB136" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC136" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z137" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA137" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB137" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC137" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z138" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA138" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB138" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC138" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z139" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z140" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA140" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB140" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC140" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z141" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA141" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB141" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC141" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z142" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE142" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z143" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA143" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB143" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC143" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z144" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA144" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB144" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC144" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z145" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA145" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB145" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC145" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z146" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA146" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB146" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC146" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z147" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA147" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB147" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC147" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z148" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA148" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB148" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC148" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z149" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA149" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB149" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC149" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z150" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA150" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB150" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC150" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD150" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z151" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD151" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE151" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z152" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z13" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA13" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB13" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC13" r:id="rId25"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z14" r:id="rId26"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA14" r:id="rId27"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB14" r:id="rId28"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC14" r:id="rId29"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z15" r:id="rId30"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA15" r:id="rId31"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB15" r:id="rId32"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC15" r:id="rId33"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z16" r:id="rId34"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA16" r:id="rId35"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB16" r:id="rId36"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC16" r:id="rId37"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z17" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA17" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB17" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC17" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z18" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z19" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA19" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB19" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC19" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z20" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA20" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB20" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC20" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD20" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z21" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z22" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA22" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB22" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC22" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z23" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA23" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB23" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC23" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z24" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD24" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE24" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z25" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z26" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE26" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z27" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA27" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB27" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC27" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z28" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA28" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB28" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC28" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z29" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE29" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z30" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA30" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB30" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC30" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z31" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z32" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA32" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB32" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC32" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z33" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z34" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE34" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z35" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA35" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB35" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC35" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD35" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z36" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA36" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB36" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC36" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD36" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z37" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE37" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z38" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA38" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB38" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC38" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z39" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD39" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z40" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA40" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB40" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC40" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD40" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z41" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA41" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB41" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC41" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z42" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA42" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB42" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC42" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z43" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA43" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB43" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC43" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z44" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD44" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE44" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z45" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA45" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB45" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC45" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD45" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z46" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA46" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB46" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC46" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z47" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD47" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE47" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z48" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA48" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB48" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC48" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z49" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA49" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB49" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC49" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z50" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA50" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB50" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC50" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z51" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA51" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB51" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC51" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z52" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z53" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA53" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB53" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC53" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD53" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z54" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE54" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z55" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE55" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z56" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA56" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB56" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC56" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z57" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA57" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB57" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC57" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z58" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA58" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB58" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC58" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z59" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA59" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB59" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC59" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z60" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z61" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z62" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA62" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB62" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC62" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z63" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE63" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z64" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA64" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB64" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC64" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z65" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE65" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z66" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA66" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB66" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC66" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z67" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA67" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB67" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC67" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z68" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE68" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z69" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE69" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z70" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA70" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB70" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC70" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z71" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA71" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB71" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC71" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z72" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA72" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB72" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC72" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD72" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z73" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA73" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB73" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC73" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z74" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD74" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE74" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z75" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA75" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB75" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC75" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z76" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE76" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z77" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z78" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA78" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB78" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC78" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD78" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z79" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA79" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB79" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC79" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z80" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA80" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB80" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC80" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD80" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE80" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z81" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA81" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB81" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC81" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z82" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA82" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB82" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC82" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z83" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA83" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB83" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC83" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD83" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA84" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB84" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC84" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA85" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB85" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC85" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA86" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB86" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC86" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA87" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB87" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC87" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA88" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB88" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC88" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA89" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB89" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC89" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA90" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB90" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC90" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD90" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA91" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB91" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC91" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA92" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB92" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC92" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD92" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA93" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB93" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC93" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA94" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB94" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC94" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE95" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA97" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB97" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC97" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA98" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB98" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC98" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA100" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB100" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC100" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA101" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB101" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC101" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA103" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB103" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC103" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD103" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA104" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB104" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC104" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA105" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB105" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC105" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD105" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA106" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB106" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC106" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE109" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA110" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB110" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC110" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD111" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE112" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA113" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB113" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC113" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z115" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA115" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB115" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC115" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z116" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE116" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z117" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA117" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB117" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC117" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z118" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE118" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z119" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA119" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB119" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC119" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z120" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD120" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE120" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z121" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA121" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB121" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC121" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD121" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z122" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA122" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB122" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC122" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z123" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA123" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB123" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC123" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z124" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA124" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB124" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC124" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD124" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z125" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z126" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE126" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z127" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA127" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB127" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC127" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD127" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z128" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA128" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB128" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC128" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z129" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA129" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB129" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC129" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z130" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA130" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB130" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC130" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z131" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA131" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB131" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC131" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z132" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE132" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z133" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE133" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z134" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA134" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB134" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC134" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z135" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA135" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB135" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC135" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z136" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA136" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB136" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC136" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z137" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA137" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB137" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC137" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z138" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA138" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB138" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC138" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z139" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z140" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA140" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB140" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC140" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z141" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA141" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB141" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC141" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z142" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE142" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z143" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA143" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB143" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC143" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z144" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA144" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB144" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC144" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z145" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA145" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB145" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC145" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z146" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA146" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB146" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC146" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z147" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA147" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB147" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC147" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z148" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA148" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB148" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC148" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z149" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA149" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB149" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC149" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z150" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA150" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB150" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC150" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD150" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z151" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD151" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE151" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z152" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE152" r:id="rId497"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z153" r:id="rId498"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z154" r:id="rId499"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE154" r:id="rId500"/>

</xml_diff>

<commit_message>
Antigua: note that Joy Lawrence's reading starts at 14:00
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -1730,7 +1730,7 @@
       <c r="S12" s="13" t="n"/>
       <c r="T12" s="13" t="inlineStr">
         <is>
-          <t>The Antiguan poet and folklorist Joy Lawrence reads her poem “Love Me” in the Commonwealth Poetry Podcast's episode on Antigua and Barbuda.</t>
+          <t>The Antiguan poet and folklorist Joy Lawrence reads her poem “Love Me” in the Commonwealth Poetry Podcast's episode on Antigua and Barbuda; the reading starts at 14:00.</t>
         </is>
       </c>
       <c r="U12" s="13" t="inlineStr">
@@ -1738,7 +1738,11 @@
           <t>Reading by the poet, Commonwealth Poetry Podcast episode 37 (29 October 2023)</t>
         </is>
       </c>
-      <c r="V12" s="13" t="n"/>
+      <c r="V12" s="13" t="inlineStr">
+        <is>
+          <t>From 14:00 in the episode</t>
+        </is>
+      </c>
       <c r="W12" s="13" t="inlineStr">
         <is>
           <t>Work changed (30 October 2026): Joan Armatrading, Love and Affection, moved to Saint Kitts and Nevis (her birthplace); replaced by a poem by an Antiguan poet.</t>

</xml_diff>

<commit_message>
Anthology review batch 1; home heading "Love, in every country"
- Hungary: Petőfi's "Szeptember végén" (1847) replaces a poem first
  printed in 1943.
- Singapore: four love pantun printed in 1922 (incl. Tanjong Katong)
  replace a poem with no established publication history; Malaysia's
  pantun set adjusted.
- Jordan, Qatar, Palestine, Kyrgyzstan, Mozambique move to explore
  pending clean replacements.
- Rights reasoning recorded for Tunisia, El Salvador, Lithuania,
  Cabo Verde and Indonesia.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -5115,7 +5115,8 @@
       </c>
       <c r="X35" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1930. Modern editorial additions and translations are separate.</t>
+          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1930. Modern editorial additions and translations are separate.
+Anthology review (30 October 2026): UK/EU public domain (Tavares died 1930). US — first published 1932; public domain from 1 January 2028. Publish after that date, or swap for a poem printed before 1931.</t>
         </is>
       </c>
       <c r="Y35" s="13" t="inlineStr">
@@ -8657,7 +8658,8 @@
       </c>
       <c r="X59" s="13" t="inlineStr">
         <is>
-          <t>Original text: standard life-plus-70 term expired; author died 1928. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.</t>
+          <t>Original text: standard life-plus-70 term expired; author died 1928. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.
+Anthology review (30 October 2026): UK — published posthumously in 1936, so protected for 50 years from publication, which ended in 1986. US — first published 1936, but Salvadoran law then protected works for 50 years after death (Espino died 1928), so it was out of copyright at home before 1996 and was not restored: public domain.</t>
         </is>
       </c>
       <c r="Y59" s="13" t="inlineStr">
@@ -11889,45 +11891,73 @@
       </c>
       <c r="D82" s="13" t="inlineStr">
         <is>
-          <t>Szerettelek (I loved you)</t>
+          <t>Szeptember végén</t>
         </is>
       </c>
       <c r="E82" s="13" t="inlineStr">
         <is>
-          <t>I Loved You</t>
+          <t>At the End of September</t>
         </is>
       </c>
       <c r="F82" s="13" t="inlineStr">
         <is>
-          <t>Meggyászoltalak én,
-Pillangós ruhába
-Sirattalak minden
-Hangos kacagásba, -
-Pénteken pirosba,
-Szombaton fehérbe, -
-Ma is gyászollak tán,
-Virágvasárnapján,
-Rózsapiruláskor,
-Talpig feketébe.</t>
+          <t>Még nyílnak a völgyben a kerti virágok,
+Még zöldel a nyárfa az ablak előtt,
+De látod amottan a téli világot?
+Már hó takará el a bérczi tetőt.
+Még ifju szivemben a lángsugarú nyár
+S még benne virít az egész kikelet,
+De íme sötét hajam őszbe vegyűl már,
+A tél dere már megüté fejemet.
+Elhull a virág, eliramlik az élet...
+Űlj, hitvesem, űlj az ölembe ide!
+Ki most fejedet kebelemre tevéd le,
+Holnap nem omolsz-e sirom fölibe?
+Oh mondd: ha előbb halok el, tetemimre
+Könnyezve borítasz-e szemfödelet?
+S rábírhat-e majdan egy ifju szerelme,
+Hogy elhagyod érte az én nevemet?
+Ha eldobod egykor az özvegyi fátyolt,
+Fejfámra sötét lobogóul akaszd,
+Én feljövök érte a síri világból
+Az éj közepén, s oda leviszem azt,
+Letörleni véle könyűimet érted,
+Ki könnyeden elfeledéd hivedet,
+S e szív sebeit bekötözni, ki téged
+Még akkor is, ott is, örökre szeret!</t>
         </is>
       </c>
       <c r="G82" s="13" t="inlineStr">
         <is>
-          <t>I mourned for you,
-in a butterfly-patterned dress;
-I wept for you in every
-burst of ringing laughter—
-in red on Friday,
-in white on Saturday.
-Perhaps I mourn you even today,
-on Palm Sunday,
-when the roses blush,
-dressed in black from head to foot.</t>
+          <t>The garden flowers still bloom in the valley,
+the poplar is still green before the window,
+but do you see the winter world over there?
+Snow already covers the mountain top.
+The flame-bright summer still burns in my young heart,
+and the whole of spring still blossoms there,
+but look, my dark hair is turning grey,
+the frost of winter has already touched my head.
+The flower falls, and life runs on…
+Sit, my wife, come sit here on my lap!
+You who now lay your head upon my breast,
+will you not fall tomorrow weeping on my grave?
+Oh tell me: if I die first, will you
+lay a shroud over my body, in tears?
+And could the love of some young man persuade you
+one day to give up my name for his?
+If one day you throw off the widow's veil,
+hang it on my grave-post like a dark flag;
+I will come up for it from the world of the dead
+at midnight, and take it down with me
+to wipe away my tears for you,
+who so lightly forgot the one who was true to you,
+and to bind the wounds of this heart, which loves you
+even then, even there, for ever!</t>
         </is>
       </c>
       <c r="H82" s="13" t="inlineStr">
         <is>
-          <t>Margit Kaffka</t>
+          <t>Sándor Petőfi</t>
         </is>
       </c>
       <c r="I82" s="13" t="inlineStr">
@@ -11947,11 +11977,13 @@
       </c>
       <c r="L82" s="13" t="inlineStr">
         <is>
-          <t>Women</t>
-        </is>
-      </c>
-      <c r="M82" s="14" t="n">
-        <v>1906</v>
+          <t>Men</t>
+        </is>
+      </c>
+      <c r="M82" s="14" t="inlineStr">
+        <is>
+          <t>1847</t>
+        </is>
       </c>
       <c r="N82" s="13" t="inlineStr">
         <is>
@@ -11966,27 +11998,27 @@
       </c>
       <c r="Q82" s="13" t="inlineStr">
         <is>
-          <t>Woman</t>
+          <t>Sándor Petőfi (1823–1849)</t>
         </is>
       </c>
       <c r="R82" s="13" t="inlineStr">
         <is>
-          <t>1906 (composition); first printed 1943 according to Irodalomtörténet</t>
+          <t>September 1847, Koltó</t>
         </is>
       </c>
       <c r="S82" s="13" t="inlineStr">
         <is>
-          <t>Undated online transcription</t>
+          <t>Hungarian Wikisource transcription in the original spelling</t>
         </is>
       </c>
       <c r="T82" s="13" t="inlineStr">
         <is>
-          <t>Love remembered and repeatedly mourned; a sorrowful rather than celebratory selection.</t>
+          <t>Watching the first snow on the mountains, the young poet asks his wife whether she will marry again after his death, and promises to love her for ever.</t>
         </is>
       </c>
       <c r="U82" s="13" t="inlineStr">
         <is>
-          <t>Wikisource text; 1943 scholarly journal explains the 1906 manuscript and first publication</t>
+          <t>Written at Koltó, September 1847; Hungarian Wikisource, original spelling.</t>
         </is>
       </c>
       <c r="V82" s="13" t="inlineStr">
@@ -11996,19 +12028,22 @@
       </c>
       <c r="W82" s="13" t="inlineStr">
         <is>
-          <t>UK/life+70 basis is distinct from US publication-based rules; US reuse of this posthumously published poem is not cleared here. Modern translations are separate.
-English passage: Fresh English translation by ChatGPT; draft for editorial review. Final10 lines. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+          <t>Work changed (30 October 2026): Margit Kaffka's “Szerettelek”, first printed in 1943, is replaced by a poem published in the poet's lifetime. Complete poem, 24 lines. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X82" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original in life+70 jurisdictions (author died 1918)</t>
-        </is>
-      </c>
-      <c r="Y82" s="13" t="n"/>
+          <t>Public domain everywhere: Petőfi died 1849 and the poem was published in his lifetime.</t>
+        </is>
+      </c>
+      <c r="Y82" s="13" t="inlineStr">
+        <is>
+          <t>Hungarian Wikisource: Szeptember végén</t>
+        </is>
+      </c>
       <c r="Z82" s="11" t="inlineStr">
         <is>
-          <t>Read text</t>
+          <t>Read the whole work</t>
         </is>
       </c>
       <c r="AA82" s="11" t="inlineStr">
@@ -12027,7 +12062,11 @@
         </is>
       </c>
       <c r="AD82" s="11" t="n"/>
-      <c r="AE82" s="11" t="n"/>
+      <c r="AE82" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: Read text</t>
+        </is>
+      </c>
     </row>
     <row r="83" ht="91.5" customHeight="1" s="17">
       <c r="A83" s="7" t="inlineStr">
@@ -12555,7 +12594,8 @@
       </c>
       <c r="X85" s="13" t="inlineStr">
         <is>
-          <t>Original text: standard life-plus-70 term expired; author died 1946. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.</t>
+          <t>Original text: standard life-plus-70 term expired; author died 1946. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.
+Anthology review (30 October 2026): UK/EU public domain (Amir Hamzah died 1946). US — first published 1932; public domain from 1 January 2028. Publish after that date, or swap for a poem printed before 1931.</t>
         </is>
       </c>
       <c r="Y85" s="13" t="inlineStr">
@@ -13880,7 +13920,8 @@
       <c r="W93" s="13" t="inlineStr">
         <is>
           <t>Identifier is the original incipit. Year 1949 is an upper bound. Birth-year disagreement is explicit. Reuse the author’s historical Arabic verses, excluding later commentary and translations; first-publication particulars for this individual poem have not been established.
-Passage update (29 October 2026): Complete poem, 8 couplets (16 half-lines), as printed in the Abu Dhabi Poetry Encyclopedia; the site’s decorative letter-stretching (tatweel) is removed. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
+Passage update (29 October 2026): Complete poem, 8 couplets (16 half-lines), as printed in the Abu Dhabi Poetry Encyclopedia; the site’s decorative letter-stretching (tatweel) is removed. Fresh English translation by Claude (Anthropic AI); draft for editorial review.
+Moved to Poems to explore (30 October 2026) for the anthology review. Jordan: the poem's first publication was in a 1954 collection, five years after the poet's death; its US status depends on Jordan's 1996 copyright term.</t>
         </is>
       </c>
       <c r="X93" s="13" t="inlineStr">
@@ -13895,7 +13936,7 @@
       </c>
       <c r="Z93" s="11" t="inlineStr">
         <is>
-          <t>Work / text</t>
+          <t>Read the text</t>
         </is>
       </c>
       <c r="AA93" s="11" t="inlineStr">
@@ -14632,7 +14673,8 @@
       <c r="W98" s="13" t="inlineStr">
         <is>
           <t>Only the original lyrics are treated as open. Later music by Bektemir Eginchiev (1910–1964), recordings and modern translations remain separate. Oral/transcribed variants exist; choose and credit a single textual version.
-Passage update (29 October 2026): First five stanzas, 20 lines, from the Kyrgyzpatent lyric sheet. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
+Passage update (29 October 2026): First five stanzas, 20 lines, from the Kyrgyzpatent lyric sheet. Fresh English translation by Claude (Anthropic AI); draft for editorial review.
+Moved to Poems to explore (30 October 2026) for the anthology review. Kyrgyzstan: the words come from a modern lyric sheet, with no early printing of this version.</t>
         </is>
       </c>
       <c r="X98" s="13" t="inlineStr">
@@ -14647,7 +14689,7 @@
       </c>
       <c r="Z98" s="11" t="inlineStr">
         <is>
-          <t>Original text</t>
+          <t>Read the text</t>
         </is>
       </c>
       <c r="AA98" s="11" t="inlineStr">
@@ -15828,7 +15870,8 @@
       </c>
       <c r="X106" s="13" t="inlineStr">
         <is>
-          <t>Public domain in life+70 jurisdictions; author page notice (died 1945)</t>
+          <t>Public domain in life+70 jurisdictions; author page notice (died 1945)
+Anthology review (30 October 2026): UK/EU public domain (Nėris died 1945). US — first published 1931, so public domain from 1 January 2027 at the latest.</t>
         </is>
       </c>
       <c r="Y106" s="13" t="n"/>
@@ -16242,10 +16285,10 @@
 Anak tekukur atas bumbongan;
 Sa-hari bertemu, sa-hari mati,
 Sa-ribu shukur atas junjongan.
-Tanjong Katong ayer-nya biru,
-Tempat berlaboh kochi Malaka;
-Sedang sa-kampong lagi ku-rindu,
-Inikan pula jauh di-mata.</t>
+Harap harap kelapa puan,
+Tidak puan kelapa Bali;
+Harap hati ka-pada nan tuan,
+Tidak tuan, siapa lagi?</t>
         </is>
       </c>
       <c r="G110" s="13" t="inlineStr">
@@ -16262,10 +16305,10 @@
 a young turtle-dove on the roof ridge;
 to meet you for a day and die the next,
 I would give a thousand thanks to the Lord.
-The water at Tanjong Katong is blue,
-where the boats of Malacca anchor;
-even in the same village I longed for you,
-how much more now you are far from my eyes.</t>
+Hoping, hoping for a puan coconut;
+if not a puan, a coconut from Bali;
+my heart's hope is set on you alone:
+if not you, who else could it be?</t>
         </is>
       </c>
       <c r="H110" s="13" t="inlineStr">
@@ -16326,12 +16369,12 @@
       </c>
       <c r="T110" s="13" t="inlineStr">
         <is>
-          <t>Four love pantun: a lover told not to weep but to send word, longing sent by every bird, a single day together worth dying for, and love that grows with distance.</t>
+          <t>Four love pantun: a lover told not to weep but to send word, longing sent by every bird, a single day together worth dying for, and a heart that hopes for one beloved alone.</t>
         </is>
       </c>
       <c r="U110" s="13" t="inlineStr">
         <is>
-          <t>H. Overbeck, “The Malay Pantun”, Journal of the Straits Branch of the Royal Asiatic Society (1922); Malay text as printed, OCR spacing tidied.</t>
+          <t>H. Overbeck, “The Malay Pantun”, Journal of the Straits Branch of the Royal Asiatic Society (Singapore, 1922); Malay text as printed, OCR errors corrected.</t>
         </is>
       </c>
       <c r="V110" s="13" t="inlineStr">
@@ -16341,7 +16384,8 @@
       </c>
       <c r="W110" s="13" t="inlineStr">
         <is>
-          <t>Work changed (30 October 2026): the five pantun from Malay Wikisource, which had no traceable printed source, are replaced by four love pantun printed by Hans Overbeck in 1922. The earlier notes about a Malay novel no longer apply. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
+          <t>Work changed (30 October 2026): the five pantun from Malay Wikisource, which had no traceable printed source, are replaced by four love pantun printed by Hans Overbeck in 1922. The earlier notes about a Malay novel no longer apply. Fresh English translation by Claude (Anthropic AI); draft for editorial review.
+Update (30 October 2026): the Tanjong Katong pantun moves to the Singapore entry; a fourth pantun (“Harap hati ka-pada nan tuan”) is added from the same 1922 article.</t>
         </is>
       </c>
       <c r="X110" s="13" t="inlineStr">
@@ -18455,7 +18499,8 @@
       <c r="W124" s="13" t="inlineStr">
         <is>
           <t>Sonetos appeared posthumously in 1946. Scholars document editorial alterations in that edition; compare the poem with a lifetime newspaper text before establishing a definitive version. Modern notes and revisions are separate.
-Passage update (29 October 2026): Complete sonnet, 14 lines (as printed in the school module, Lesson 25). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
+Passage update (29 October 2026): Complete sonnet, 14 lines (as printed in the school module, Lesson 25). Fresh English translation by Claude (Anthropic AI); draft for editorial review.
+Moved to Poems to explore (30 October 2026) for the anthology review. Mozambique: published posthumously in 1946, and the editor is known to have altered the text.</t>
         </is>
       </c>
       <c r="X124" s="13" t="inlineStr">
@@ -18470,7 +18515,7 @@
       </c>
       <c r="Z124" s="11" t="inlineStr">
         <is>
-          <t>Work / source text</t>
+          <t>Read the text</t>
         </is>
       </c>
       <c r="AA124" s="11" t="inlineStr">
@@ -20811,7 +20856,8 @@
       <c r="W140" s="13" t="inlineStr">
         <is>
           <t>Collection’s first issue date is listed as unknown; do not treat 2012 as composition date. Original Arabic only; modern translation and editorial material separate.
-Passage update (29 October 2026): Complete poem, 24 half-lines (Hindawi edition of the complete poems; the section dividers are omitted). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
+Passage update (29 October 2026): Complete poem, 24 half-lines (Hindawi edition of the complete poems; the section dividers are omitted). Fresh English translation by Claude (Anthropic AI); draft for editorial review.
+Moved to Poems to explore (30 October 2026) for the anthology review. Palestine: the poem's first publication date is unknown; the linked text is a 2012 digital edition.</t>
         </is>
       </c>
       <c r="X140" s="13" t="inlineStr">
@@ -20826,7 +20872,7 @@
       </c>
       <c r="Z140" s="11" t="inlineStr">
         <is>
-          <t>Original text</t>
+          <t>Read the text</t>
         </is>
       </c>
       <c r="AA140" s="11" t="inlineStr">
@@ -22105,7 +22151,8 @@
       <c r="W148" s="13" t="inlineStr">
         <is>
           <t>The incipit is the identifier, not a verified authorial title. Source typography/OCR needs checking against the 1963 diwan. The 1995 criticism has separate rights.
-Passage update (29 October 2026): Four couplets (8 half-lines) of Nabati verse, as printed in Nizwa magazine. The reading of the last couplet is uncertain, and the English there is tentative. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
+Passage update (29 October 2026): Four couplets (8 half-lines) of Nabati verse, as printed in Nizwa magazine. The reading of the last couplet is uncertain, and the English there is tentative. Fresh English translation by Claude (Anthropic AI); draft for editorial review.
+Moved to Poems to explore (30 October 2026) for the anthology review. Qatar: the poem was first collected in a 1963 diwan, and the 1995 excerpt's printing history is not established.</t>
         </is>
       </c>
       <c r="X148" s="13" t="inlineStr">
@@ -22120,7 +22167,7 @@
       </c>
       <c r="Z148" s="11" t="inlineStr">
         <is>
-          <t>Work / source text</t>
+          <t>Read the text</t>
         </is>
       </c>
       <c r="AA148" s="11" t="inlineStr">
@@ -24017,33 +24064,57 @@
       </c>
       <c r="D163" s="13" t="inlineStr">
         <is>
-          <t>丁丑清明节，为亡室陆氏筑坟成</t>
+          <t>Pantun</t>
         </is>
       </c>
       <c r="E163" s="13" t="inlineStr">
         <is>
-          <t>Qingming 1937, on Completing the Grave of My Late Wife</t>
+          <t>Pantun of Love and Longing</t>
         </is>
       </c>
       <c r="F163" s="13" t="inlineStr">
         <is>
-          <t>几枚白石伴青珉，
-小筑坟茔隔岁春。
-地下有灵相谅解，
-迟工原是为家贫。</t>
+          <t>Tanjong Katong ayer-nya biru,
+Tempat berlaboh kochi Malaka;
+Sedang sa-kampong lagi ku-rindu,
+Inikan pula jauh di-mata.
+Kalau tidak karna kunchi,
+Papan peti sahaya belahkan;
+Kalau tidak karna mati,
+Belah dada sahaya tunjokkan.
+Anak berok besar lengan,
+Masok ka-bendang makan padi;
+Kalau kaseh alang-alangan,
+Biar ta’usah sa-kali-kali.
+Limau manis di-kebun raja,
+Hilang di-bungkus puncha kain;
+Mulut manis di-depan sahaja,
+Hati sudah ka-pada lain.</t>
         </is>
       </c>
       <c r="G163" s="13" t="inlineStr">
         <is>
-          <t>A few white stones beside the green jade stone:
-a year on, in spring, I have built this small grave.
-If your spirit below can know, forgive me:
-the work was late only because we are poor.</t>
+          <t>The water at Tanjong Katong is blue,
+where the boats of Malacca anchor;
+even in the same village I longed for you,
+how much more now you are far from my eyes.
+If it were not for the key,
+I would split the boards of the chest;
+if it were not that I would die,
+I would open my breast to show you.
+A young monkey with mighty arms
+goes down to the rice field to eat the grain;
+if your love is only half-hearted,
+better there were none at all.
+Sweet limes in the royal garden,
+lost when tied in the corner of a cloth;
+sweet words only to my face,
+but your heart has gone to another.</t>
         </is>
       </c>
       <c r="H163" s="13" t="inlineStr">
         <is>
-          <t>Khoo Seok Wan / 丘菽园 (1874–1941)</t>
+          <t>Traditional Malay pantun; as printed by Hans Overbeck, 1922</t>
         </is>
       </c>
       <c r="I163" s="13" t="inlineStr">
@@ -24063,46 +24134,48 @@
       </c>
       <c r="L163" s="13" t="inlineStr">
         <is>
-          <t>Men</t>
-        </is>
-      </c>
-      <c r="M163" s="14" t="n">
-        <v>1937</v>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="M163" s="14" t="inlineStr">
+        <is>
+          <t>1922</t>
+        </is>
       </c>
       <c r="N163" s="13" t="inlineStr">
         <is>
-          <t>Classical Chinese</t>
+          <t>Malay</t>
         </is>
       </c>
       <c r="O163" s="13" t="n"/>
       <c r="P163" s="13" t="inlineStr">
         <is>
-          <t>Lyric poem</t>
+          <t>Pantun (four-line verses)</t>
         </is>
       </c>
       <c r="Q163" s="13" t="inlineStr">
         <is>
-          <t>Man author</t>
+          <t>Anonymous singers</t>
         </is>
       </c>
       <c r="R163" s="13" t="inlineStr">
         <is>
-          <t>1937, the Qingming following his wife’s death in 1936</t>
+          <t>Traditional oral verse; printed 1922</t>
         </is>
       </c>
       <c r="S163" s="13" t="inlineStr">
         <is>
-          <t>Historical work reproduced in linked digital source; modern editorial material is separate</t>
+          <t>1922</t>
         </is>
       </c>
       <c r="T163" s="13" t="inlineStr">
         <is>
-          <t>The widower asks his beloved wife to understand why poverty delayed the building of her grave, expressing enduring marital love.</t>
+          <t>Four love pantun: longing that grows with distance, a heart the lover would open to show, love that should be whole or nothing, and sweet words from someone whose heart is elsewhere.</t>
         </is>
       </c>
       <c r="U163" s="13" t="inlineStr">
         <is>
-          <t>University of Malaya scholarly article quotes and contextualises the Chinese poem; Bukit Brown heritage documentation reproduces its text. National Library Singapore confirms the poet’s dates and local literary role.</t>
+          <t>H. Overbeck, “The Malay Pantun”, Journal of the Straits Branch of the Royal Asiatic Society (Singapore, 1922); Malay text as printed, OCR errors corrected.</t>
         </is>
       </c>
       <c r="V163" s="13" t="inlineStr">
@@ -24112,23 +24185,22 @@
       </c>
       <c r="W163" s="13" t="inlineStr">
         <is>
-          <t>Incipit identifies the work; do not invent a formal title. Use Khoo’s Chinese verse only. Modern English translations, photographs and the scholarly article have separate rights.
-Passage update (29 October 2026): Complete poem, 4 lines, from 菽园诗集 vol. 6 on Shidian Guji (the originally linked PDF could not be opened). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
+          <t>Work changed (30 October 2026): Khoo Seok Wan's 1937 poem, whose first publication could not be established, is replaced by four love pantun printed in Singapore's Royal Asiatic Society journal in 1922; the first names Tanjong Katong, on Singapore's east coast. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X163" s="13" t="inlineStr">
         <is>
-          <t>Historical original text: standard life-plus-70 term has expired; author died 1941. Assessment excludes modern translations, commentary, editorial alterations, musical settings and recordings. Territorial and unusual publication-history exceptions are not comprehensively assessed.</t>
+          <t>Traditional anonymous verse; Overbeck's 1922 printing is public domain (he died 1942). Overbeck's English is not used.</t>
         </is>
       </c>
       <c r="Y163" s="13" t="inlineStr">
         <is>
-          <t>University of Malaya scholarly article quotes and contextualises the Chinese poem; Bukit Brown heritage documentation reproduces its text. National Library Singapore confirms the poet’s dates and local literary role.</t>
+          <t>Internet Archive (BioStor): Overbeck, The Malay Pantun, 1922</t>
         </is>
       </c>
       <c r="Z163" s="11" t="inlineStr">
         <is>
-          <t>Read original</t>
+          <t>Read the whole work</t>
         </is>
       </c>
       <c r="AA163" s="11" t="inlineStr">
@@ -24151,7 +24223,11 @@
           <t>Additional evidence</t>
         </is>
       </c>
-      <c r="AE163" s="11" t="n"/>
+      <c r="AE163" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: Read original</t>
+        </is>
+      </c>
     </row>
     <row r="164" ht="43.5" customHeight="1" s="17">
       <c r="A164" s="7" t="inlineStr">
@@ -27308,7 +27384,8 @@
       </c>
       <c r="X185" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1934. Modern editorial additions and translations are separate.</t>
+          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1934. Modern editorial additions and translations are separate.
+Anthology review (30 October 2026): UK/EU — al-Shabbi died 1934, so the poem is out of copyright. US — first published after 1930, but Tunisian and Egyptian law then protected works for 50 years after death, so it was already out of copyright at home on 1 January 1996 and was not restored in the US: public domain.</t>
         </is>
       </c>
       <c r="Y185" s="13" t="inlineStr">
@@ -29944,415 +30021,417 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA82" r:id="rId258"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB82" r:id="rId259"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC82" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z83" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA83" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB83" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC83" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD83" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE83" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA84" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB84" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC84" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA85" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB85" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC85" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA86" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB86" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC86" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA87" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB87" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC87" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA88" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB88" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC88" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA89" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB89" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC89" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA90" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB90" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC90" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD90" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE90" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA91" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB91" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC91" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA92" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB92" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC92" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD92" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE92" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA93" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB93" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC93" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA94" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB94" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC94" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE95" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA97" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB97" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC97" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA98" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB98" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC98" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA100" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB100" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC100" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA101" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB101" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC101" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA103" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB103" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC103" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD103" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA104" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB104" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC104" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA105" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB105" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC105" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD105" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA106" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB106" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC106" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE109" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA110" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB110" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC110" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE110" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD111" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE112" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA113" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB113" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC113" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z115" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA115" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB115" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC115" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z116" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE116" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z117" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA117" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB117" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC117" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z118" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE118" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z119" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA119" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB119" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC119" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z120" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD120" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE120" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z121" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA121" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB121" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC121" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD121" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z122" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA122" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB122" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC122" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z123" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA123" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB123" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC123" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE123" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z124" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA124" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB124" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC124" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD124" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z125" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z126" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE126" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z127" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA127" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB127" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC127" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD127" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z128" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA128" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB128" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC128" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z129" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA129" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB129" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC129" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z130" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA130" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB130" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC130" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z131" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA131" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB131" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC131" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z132" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE132" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z133" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE133" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z134" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA134" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB134" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC134" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z135" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA135" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB135" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC135" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z136" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA136" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB136" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC136" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z137" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA137" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB137" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC137" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z138" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA138" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB138" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC138" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z139" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z140" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA140" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB140" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC140" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z141" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA141" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB141" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC141" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z142" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE142" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z143" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA143" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB143" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC143" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z144" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA144" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB144" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC144" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z145" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA145" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB145" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC145" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z146" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA146" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB146" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC146" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z147" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA147" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB147" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC147" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z148" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA148" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB148" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC148" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z149" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA149" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB149" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC149" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z150" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA150" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB150" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC150" r:id="rId500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD150" r:id="rId501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE150" r:id="rId502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z151" r:id="rId503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD151" r:id="rId504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE151" r:id="rId505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z152" r:id="rId506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE152" r:id="rId507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z153" r:id="rId508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z154" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE154" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z155" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z156" r:id="rId512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z157" r:id="rId513"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA157" r:id="rId514"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB157" r:id="rId515"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC157" r:id="rId516"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD157" r:id="rId517"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z158" r:id="rId518"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA158" r:id="rId519"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB158" r:id="rId520"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC158" r:id="rId521"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z159" r:id="rId522"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z160" r:id="rId523"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA160" r:id="rId524"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB160" r:id="rId525"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC160" r:id="rId526"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z161" r:id="rId527"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE161" r:id="rId528"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z162" r:id="rId529"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE162" r:id="rId530"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z163" r:id="rId531"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA163" r:id="rId532"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB163" r:id="rId533"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC163" r:id="rId534"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD163" r:id="rId535"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z164" r:id="rId536"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA164" r:id="rId537"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB164" r:id="rId538"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC164" r:id="rId539"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z165" r:id="rId540"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA165" r:id="rId541"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB165" r:id="rId542"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC165" r:id="rId543"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z166" r:id="rId544"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z167" r:id="rId545"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA167" r:id="rId546"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB167" r:id="rId547"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC167" r:id="rId548"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD167" r:id="rId549"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z168" r:id="rId550"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA168" r:id="rId551"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB168" r:id="rId552"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC168" r:id="rId553"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z169" r:id="rId554"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA169" r:id="rId555"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB169" r:id="rId556"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC169" r:id="rId557"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z170" r:id="rId558"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z171" r:id="rId559"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA171" r:id="rId560"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB171" r:id="rId561"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC171" r:id="rId562"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z172" r:id="rId563"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA172" r:id="rId564"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB172" r:id="rId565"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC172" r:id="rId566"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD172" r:id="rId567"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE172" r:id="rId568"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z173" r:id="rId569"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z174" r:id="rId570"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z175" r:id="rId571"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA175" r:id="rId572"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB175" r:id="rId573"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC175" r:id="rId574"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z176" r:id="rId575"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA176" r:id="rId576"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB176" r:id="rId577"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC176" r:id="rId578"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z177" r:id="rId579"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA177" r:id="rId580"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB177" r:id="rId581"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC177" r:id="rId582"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z178" r:id="rId583"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA178" r:id="rId584"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB178" r:id="rId585"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC178" r:id="rId586"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z179" r:id="rId587"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA179" r:id="rId588"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB179" r:id="rId589"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC179" r:id="rId590"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD179" r:id="rId591"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z180" r:id="rId592"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA180" r:id="rId593"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB180" r:id="rId594"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC180" r:id="rId595"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z181" r:id="rId596"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE181" r:id="rId597"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z182" r:id="rId598"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD182" r:id="rId599"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z183" r:id="rId600"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA183" r:id="rId601"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB183" r:id="rId602"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC183" r:id="rId603"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z184" r:id="rId604"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA184" r:id="rId605"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB184" r:id="rId606"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC184" r:id="rId607"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD184" r:id="rId608"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z185" r:id="rId609"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA185" r:id="rId610"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB185" r:id="rId611"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC185" r:id="rId612"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD185" r:id="rId613"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z186" r:id="rId614"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA186" r:id="rId615"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB186" r:id="rId616"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC186" r:id="rId617"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z187" r:id="rId618"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z188" r:id="rId619"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z189" r:id="rId620"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE189" r:id="rId621"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z190" r:id="rId622"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA190" r:id="rId623"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB190" r:id="rId624"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC190" r:id="rId625"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD190" r:id="rId626"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z191" r:id="rId627"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD191" r:id="rId628"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE191" r:id="rId629"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z192" r:id="rId630"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA192" r:id="rId631"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB192" r:id="rId632"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC192" r:id="rId633"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z193" r:id="rId634"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA193" r:id="rId635"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB193" r:id="rId636"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC193" r:id="rId637"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z194" r:id="rId638"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA194" r:id="rId639"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB194" r:id="rId640"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC194" r:id="rId641"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z195" r:id="rId642"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA195" r:id="rId643"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB195" r:id="rId644"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC195" r:id="rId645"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z196" r:id="rId646"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA196" r:id="rId647"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB196" r:id="rId648"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC196" r:id="rId649"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z197" r:id="rId650"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA197" r:id="rId651"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB197" r:id="rId652"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC197" r:id="rId653"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z198" r:id="rId654"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA198" r:id="rId655"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB198" r:id="rId656"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC198" r:id="rId657"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE198" r:id="rId658"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z199" r:id="rId659"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA199" r:id="rId660"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB199" r:id="rId661"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC199" r:id="rId662"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z200" r:id="rId663"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z201" r:id="rId664"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE201" r:id="rId665"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE82" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z83" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA83" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB83" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC83" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD83" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE83" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA84" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB84" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC84" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA85" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB85" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC85" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA86" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB86" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC86" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA87" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB87" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC87" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA88" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB88" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC88" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA89" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB89" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC89" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA90" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB90" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC90" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD90" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE90" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA91" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB91" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC91" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA92" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB92" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC92" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD92" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE92" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA93" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB93" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC93" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA94" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB94" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC94" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE95" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA97" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB97" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC97" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA98" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB98" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC98" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA100" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB100" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC100" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA101" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB101" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC101" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA103" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB103" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC103" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD103" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA104" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB104" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC104" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA105" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB105" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC105" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD105" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA106" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB106" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC106" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE109" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA110" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB110" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC110" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE110" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD111" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE112" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA113" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB113" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC113" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z115" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA115" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB115" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC115" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z116" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE116" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z117" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA117" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB117" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC117" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z118" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE118" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z119" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA119" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB119" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC119" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z120" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD120" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE120" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z121" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA121" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB121" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC121" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD121" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z122" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA122" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB122" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC122" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z123" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA123" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB123" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC123" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE123" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z124" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA124" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB124" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC124" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD124" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z125" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z126" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE126" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z127" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA127" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB127" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC127" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD127" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z128" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA128" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB128" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC128" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z129" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA129" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB129" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC129" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z130" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA130" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB130" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC130" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z131" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA131" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB131" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC131" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z132" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE132" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z133" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE133" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z134" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA134" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB134" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC134" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z135" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA135" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB135" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC135" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z136" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA136" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB136" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC136" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z137" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA137" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB137" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC137" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z138" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA138" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB138" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC138" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z139" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z140" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA140" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB140" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC140" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z141" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA141" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB141" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC141" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z142" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE142" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z143" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA143" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB143" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC143" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z144" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA144" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB144" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC144" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z145" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA145" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB145" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC145" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z146" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA146" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB146" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC146" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z147" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA147" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB147" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC147" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z148" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA148" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB148" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC148" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z149" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA149" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB149" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC149" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z150" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA150" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB150" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC150" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD150" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE150" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z151" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD151" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE151" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z152" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE152" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z153" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z154" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE154" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z155" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z156" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z157" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA157" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB157" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC157" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD157" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z158" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA158" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB158" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC158" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z159" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z160" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA160" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB160" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC160" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z161" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE161" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z162" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE162" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z163" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA163" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB163" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC163" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD163" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE163" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z164" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA164" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB164" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC164" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z165" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA165" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB165" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC165" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z166" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z167" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA167" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB167" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC167" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD167" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z168" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA168" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB168" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC168" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z169" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA169" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB169" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC169" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z170" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z171" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA171" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB171" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC171" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z172" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA172" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB172" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC172" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD172" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE172" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z173" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z174" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z175" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA175" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB175" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC175" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z176" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA176" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB176" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC176" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z177" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA177" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB177" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC177" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z178" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA178" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB178" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC178" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z179" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA179" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB179" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC179" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD179" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z180" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA180" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB180" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC180" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z181" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE181" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z182" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD182" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z183" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA183" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB183" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC183" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z184" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA184" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB184" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC184" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD184" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z185" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA185" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB185" r:id="rId613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC185" r:id="rId614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD185" r:id="rId615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z186" r:id="rId616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA186" r:id="rId617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB186" r:id="rId618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC186" r:id="rId619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z187" r:id="rId620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z188" r:id="rId621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z189" r:id="rId622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE189" r:id="rId623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z190" r:id="rId624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA190" r:id="rId625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB190" r:id="rId626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC190" r:id="rId627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD190" r:id="rId628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z191" r:id="rId629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD191" r:id="rId630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE191" r:id="rId631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z192" r:id="rId632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA192" r:id="rId633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB192" r:id="rId634"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC192" r:id="rId635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z193" r:id="rId636"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA193" r:id="rId637"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB193" r:id="rId638"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC193" r:id="rId639"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z194" r:id="rId640"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA194" r:id="rId641"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB194" r:id="rId642"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC194" r:id="rId643"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z195" r:id="rId644"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA195" r:id="rId645"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB195" r:id="rId646"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC195" r:id="rId647"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z196" r:id="rId648"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA196" r:id="rId649"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB196" r:id="rId650"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC196" r:id="rId651"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z197" r:id="rId652"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA197" r:id="rId653"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB197" r:id="rId654"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC197" r:id="rId655"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z198" r:id="rId656"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA198" r:id="rId657"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB198" r:id="rId658"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC198" r:id="rId659"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE198" r:id="rId660"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z199" r:id="rId661"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA199" r:id="rId662"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB199" r:id="rId663"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC199" r:id="rId664"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z200" r:id="rId665"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z201" r:id="rId666"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE201" r:id="rId667"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId666"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId668"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Anthology review batch 2: rights basis for older poems
- Copyright basis recorded for 43 older poems (first published before
  1931; home copyright expired by 1996; or long in print).
- Yemen: Waddah al-Yaman's love poem to Rawda, preserved in Kitab
  al-Aghani (printed 1868), replaces a song with no printing before 1989.
- Mauritania and Oman move to explore until an early printing is found.
- Morocco and Bahrain: early printings recorded (1966, 1953).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -1000,7 +1000,8 @@
       </c>
       <c r="X7" s="13" t="inlineStr">
         <is>
-          <t>Public-domain medieval original attributed to a tenth-century poet; modern editorial matter excluded.</t>
+          <t>Public-domain medieval original attributed to a tenth-century poet; modern editorial matter excluded.
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y7" s="13" t="inlineStr">
@@ -1166,7 +1167,8 @@
       </c>
       <c r="X8" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1900. Modern editorial additions and translations are separate.</t>
+          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1900. Modern editorial additions and translations are separate.
+Anthology review (30 October 2026): first published before 1931 and the poet died long before 1956, so public domain in the UK, EU and US. Luletë e verës, 1890.</t>
         </is>
       </c>
       <c r="Y8" s="13" t="inlineStr">
@@ -1333,7 +1335,8 @@
       </c>
       <c r="X9" s="13" t="inlineStr">
         <is>
-          <t>Historical original composition; author died 1883, beyond the standard life-plus-70 term. Reuse the underlying historical original only, excluding modern translations, editorial matter, images, adaptations and recordings. Publication history and territorial exceptions should be checked for the edition used.</t>
+          <t>Historical original composition; author died 1883, beyond the standard life-plus-70 term. Reuse the underlying historical original only, excluding modern translations, editorial matter, images, adaptations and recordings. Publication history and territorial exceptions should be checked for the edition used.
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y9" s="13" t="inlineStr">
@@ -1620,7 +1623,8 @@
       </c>
       <c r="X11" s="13" t="inlineStr">
         <is>
-          <t>Historical original text: standard life-plus-70 term has expired; author died 1894. Assessment excludes modern translations, commentary, editorial alterations, musical settings and recordings. Territorial and unusual publication-history exceptions are not comprehensively assessed.</t>
+          <t>Historical original text: standard life-plus-70 term has expired; author died 1894. Assessment excludes modern translations, commentary, editorial alterations, musical settings and recordings. Territorial and unusual publication-history exceptions are not comprehensively assessed.
+Anthology review (30 October 2026): first published before 1931 and the poet died long before 1956, so public domain in the UK, EU and US. Almanach, 1888.</t>
         </is>
       </c>
       <c r="Y11" s="13" t="inlineStr">
@@ -2068,7 +2072,8 @@
       </c>
       <c r="X14" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1795. Modern editorial additions and translations are separate.</t>
+          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1795. Modern editorial additions and translations are separate.
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y14" s="13" t="inlineStr">
@@ -2553,7 +2558,8 @@
       </c>
       <c r="X17" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original; site transcription has CC BY-SA terms where applicable</t>
+          <t>Public-domain original; site transcription has CC BY-SA terms where applicable
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y17" s="13" t="inlineStr">
@@ -2812,7 +2818,8 @@
       </c>
       <c r="U19" s="13" t="inlineStr">
         <is>
-          <t>Department of Culture and Tourism — Abu Dhabi, Poetic Encyclopedia; poet biography identifies Bahrain and a diwan known during his lifetime.</t>
+          <t>Department of Culture and Tourism — Abu Dhabi, Poetic Encyclopedia; poet biography identifies Bahrain and a diwan known during his lifetime.
+Diwan printed in Tehran (Maktabat al-Haydari), 1953.</t>
         </is>
       </c>
       <c r="V19" s="13" t="inlineStr">
@@ -2828,7 +2835,8 @@
       </c>
       <c r="X19" s="13" t="inlineStr">
         <is>
-          <t>Original text: standard life-plus-70 term expired; author died 1619. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.</t>
+          <t>Original text: standard life-plus-70 term expired; author died 1619. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship. Diwan printed in Tehran, 1953.</t>
         </is>
       </c>
       <c r="Y19" s="13" t="inlineStr">
@@ -4713,7 +4721,8 @@
       </c>
       <c r="X32" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original in life+70 jurisdictions (author died 1937)</t>
+          <t>Public-domain original in life+70 jurisdictions (author died 1937)
+Anthology review (30 October 2026): first published before 1931 and the poet died long before 1956, so public domain in the UK, EU and US. Collection Soneti, 1925.</t>
         </is>
       </c>
       <c r="Y32" s="13" t="inlineStr">
@@ -6119,7 +6128,8 @@
       </c>
       <c r="X42" s="13" t="inlineStr">
         <is>
-          <t>Ancient anonymous poem, public domain. New English translation from the Chinese; Cranmer-Byng's 1909 version is not used.</t>
+          <t>Ancient anonymous poem, public domain. New English translation from the Chinese; Cranmer-Byng's 1909 version is not used.
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y42" s="13" t="inlineStr">
@@ -6287,7 +6297,8 @@
       </c>
       <c r="X43" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1923. Modern editorial additions and translations are separate.</t>
+          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1923. Modern editorial additions and translations are separate.
+Anthology review (30 October 2026): first published before 1931 and the poet died long before 1956, so public domain in the UK, EU and US.</t>
         </is>
       </c>
       <c r="Y43" s="13" t="inlineStr">
@@ -7164,7 +7175,8 @@
       </c>
       <c r="X49" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original; site transcription has CC BY-SA terms where applicable</t>
+          <t>Public-domain original; site transcription has CC BY-SA terms where applicable
+Anthology review (30 October 2026): first published before 1931 and the poet died long before 1956, so public domain in the UK, EU and US.</t>
         </is>
       </c>
       <c r="Y49" s="13" t="n"/>
@@ -7316,7 +7328,8 @@
       </c>
       <c r="X50" s="13" t="inlineStr">
         <is>
-          <t>Public-domain anonymous Renaissance original; modern translation and scholarly editorial contributions excluded.</t>
+          <t>Public-domain anonymous Renaissance original; modern translation and scholarly editorial contributions excluded.
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y50" s="13" t="inlineStr">
@@ -8139,7 +8152,8 @@
       </c>
       <c r="X56" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1897. Modern editorial additions and translations are separate.</t>
+          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1897. Modern editorial additions and translations are separate.
+Anthology review (30 October 2026): first published before 1931 and the poet died long before 1956, so public domain in the UK, EU and US. Poesías, 1880.</t>
         </is>
       </c>
       <c r="Y56" s="13" t="inlineStr">
@@ -8305,7 +8319,8 @@
       </c>
       <c r="X57" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1919. Modern editorial additions and translations are separate.</t>
+          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1919. Modern editorial additions and translations are separate.
+Anthology review (30 October 2026): first published before 1931 and the poet died long before 1956, so public domain in the UK, EU and US.</t>
         </is>
       </c>
       <c r="Y57" s="13" t="inlineStr">
@@ -9041,7 +9056,8 @@
       </c>
       <c r="X62" s="13" t="inlineStr">
         <is>
-          <t>Original text: standard life-plus-70 term expired; author died 1886. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.</t>
+          <t>Original text: standard life-plus-70 term expired; author died 1886. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.
+Anthology review (30 October 2026): first published before 1931 and the poet died long before 1956, so public domain in the UK, EU and US.</t>
         </is>
       </c>
       <c r="Y62" s="13" t="inlineStr">
@@ -10156,7 +10172,8 @@
       </c>
       <c r="X70" s="13" t="inlineStr">
         <is>
-          <t>Public-domain medieval Georgian original; modern editorial additions and translations excluded.</t>
+          <t>Public-domain medieval Georgian original; modern editorial additions and translations excluded.
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y70" s="13" t="inlineStr">
@@ -10931,7 +10948,8 @@
       </c>
       <c r="X75" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1844. Modern editorial additions and translations are separate.</t>
+          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1844. Modern editorial additions and translations are separate.
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y75" s="13" t="inlineStr">
@@ -11662,7 +11680,8 @@
       </c>
       <c r="X80" s="13" t="inlineStr">
         <is>
-          <t>Public-domain ancient Hebrew original; modern commentary, editorial apparatus and translations excluded.</t>
+          <t>Public-domain ancient Hebrew original; modern commentary, editorial apparatus and translations excluded.
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y80" s="13" t="inlineStr">
@@ -11838,7 +11857,8 @@
       </c>
       <c r="X81" s="13" t="inlineStr">
         <is>
-          <t>Original text: standard life-plus-70 term expired; author died 1908. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.</t>
+          <t>Original text: standard life-plus-70 term expired; author died 1908. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.
+Anthology review (30 October 2026): first published before 1931 and the poet died long before 1956, so public domain in the UK, EU and US. Posthumous collection, 1911.</t>
         </is>
       </c>
       <c r="Y81" s="13" t="inlineStr">
@@ -12771,7 +12791,8 @@
       </c>
       <c r="X86" s="13" t="inlineStr">
         <is>
-          <t>Original text: 14th-century poem, public domain. New English translation from the Persian; Gertrude Bell's 1897 translation is not used.</t>
+          <t>Original text: 14th-century poem, public domain. New English translation from the Persian; Gertrude Bell's 1897 translation is not used.
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y86" s="13" t="inlineStr">
@@ -12931,7 +12952,8 @@
       </c>
       <c r="X87" s="13" t="inlineStr">
         <is>
-          <t>Original text: standard life-plus-70 term expired; author died 1936. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.</t>
+          <t>Original text: standard life-plus-70 term expired; author died 1936. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.
+Anthology review (30 October 2026): al-Zahawi died 1936; the poet died before 1956 (UK/EU public domain); in the US, whatever the date of first publication, the poem was already out of copyright at home on 1 January 1996, so US copyright was never restored.</t>
         </is>
       </c>
       <c r="Y87" s="13" t="inlineStr">
@@ -13251,7 +13273,8 @@
       </c>
       <c r="X89" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1931. Modern editorial additions and translations are separate.</t>
+          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1931. Modern editorial additions and translations are separate.
+Anthology review (30 October 2026): Rachel Bluwstein died 1931; the poet died before 1956 (UK/EU public domain); in the US, whatever the date of first publication, the poem was already out of copyright at home on 1 January 1996, so US copyright was never restored.</t>
         </is>
       </c>
       <c r="Y89" s="13" t="inlineStr">
@@ -13743,7 +13766,8 @@
       </c>
       <c r="X92" s="13" t="inlineStr">
         <is>
-          <t>Original text: Taira no Kanemori died 990; public domain. New English translation from the Japanese; William Porter's 1909 translation is not used.</t>
+          <t>Original text: Taira no Kanemori died 990; public domain. New English translation from the Japanese; William Porter's 1909 translation is not used.
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y92" s="13" t="inlineStr">
@@ -14108,7 +14132,8 @@
       </c>
       <c r="X94" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1904. Modern editorial additions and translations are separate.</t>
+          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1904. Modern editorial additions and translations are separate.
+Anthology review (30 October 2026): first published before 1931 and the poet died long before 1956, so public domain in the UK, EU and US. First collected 1909.</t>
         </is>
       </c>
       <c r="Y94" s="13" t="inlineStr">
@@ -14498,7 +14523,8 @@
       </c>
       <c r="X97" s="13" t="inlineStr">
         <is>
-          <t>Original text: standard life-plus-70 term expired; author died 1901. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.</t>
+          <t>Original text: standard life-plus-70 term expired; author died 1901. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y97" s="13" t="inlineStr">
@@ -14948,7 +14974,8 @@
       </c>
       <c r="X100" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original in life+70 jurisdictions (author died 1943)</t>
+          <t>Public-domain original in life+70 jurisdictions (author died 1943)
+Anthology review (30 October 2026): Aspazija died 1943; the poet died before 1956 (UK/EU public domain); in the US, whatever the date of first publication, the poem was already out of copyright at home on 1 January 1996, so US copyright was never restored. Confirm Latvia's 1996 term if the poem was first published after 1930.</t>
         </is>
       </c>
       <c r="Y100" s="13" t="n"/>
@@ -15557,7 +15584,8 @@
       </c>
       <c r="X104" s="13" t="inlineStr">
         <is>
-          <t>Original text: standard life-plus-70 term expired; author died 1917. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.</t>
+          <t>Original text: standard life-plus-70 term expired; author died 1917. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y104" s="13" t="inlineStr">
@@ -17057,7 +17085,8 @@
       <c r="W115" s="13" t="inlineStr">
         <is>
           <t>The identifier is the original first line, not an invented English title. A muʿāraḍa of a poem by the early Arabic poet Humayd ibn Thawr. Year 1856 is an upper bound, not a dated composition. Reuse the historical Arabic lines, excluding modern commentary and translations.
-Passage update (29 October 2026): Opening four couplets of the mīmiyya (8 half-lines), as quoted in the source. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
+Passage update (29 October 2026): Opening four couplets of the mīmiyya (8 half-lines), as quoted in the source. Fresh English translation by Claude (Anthropic AI); draft for editorial review.
+Moved to Poems to explore (30 October 2026) for the anthology review. Mauritania: the poet's diwan was first printed in 1999; an earlier printing of this poem (perhaps in al-Wasit, Cairo 1911) could not be confirmed.</t>
         </is>
       </c>
       <c r="X115" s="13" t="inlineStr">
@@ -17072,7 +17101,7 @@
       </c>
       <c r="Z115" s="11" t="inlineStr">
         <is>
-          <t>Work / text</t>
+          <t>Read the text</t>
         </is>
       </c>
       <c r="AA115" s="11" t="inlineStr">
@@ -17352,7 +17381,8 @@
       </c>
       <c r="X117" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original; site transcription has CC BY-SA terms where applicable</t>
+          <t>Public-domain original; site transcription has CC BY-SA terms where applicable
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y117" s="13" t="n"/>
@@ -17966,7 +17996,8 @@
       </c>
       <c r="X121" s="13" t="inlineStr">
         <is>
-          <t>Historical original text: standard life-plus-70 term has expired; author died 1856. Assessment excludes modern translations, commentary, editorial alterations, musical settings and recordings. Territorial and unusual publication-history exceptions are not comprehensively assessed.</t>
+          <t>Historical original text: standard life-plus-70 term has expired; author died 1856. Assessment excludes modern translations, commentary, editorial alterations, musical settings and recordings. Territorial and unusual publication-history exceptions are not comprehensively assessed.
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y121" s="13" t="inlineStr">
@@ -18148,7 +18179,8 @@
       </c>
       <c r="X122" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1851. Modern editorial additions and translations are separate.</t>
+          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1851. Modern editorial additions and translations are separate.
+Anthology review (30 October 2026): first published before 1931 and the poet died long before 1956, so public domain in the UK, EU and US. First printed 1913.</t>
         </is>
       </c>
       <c r="Y122" s="13" t="inlineStr">
@@ -18316,7 +18348,8 @@
       </c>
       <c r="U123" s="13" t="inlineStr">
         <is>
-          <t>Original Arabic reproduced at Qaseda and Arabic Literature Encyclopedia; biography identifies Fez writer Muhammad ibn Qasim ibn Zakur (1664–1708), author of al-Rawd al-arid.</t>
+          <t>Original Arabic reproduced at Qaseda and Arabic Literature Encyclopedia; biography identifies Fez writer Muhammad ibn Qasim ibn Zakur (1664–1708), author of al-Rawd al-arid.
+Also printed in al-Muntakhab min shiʿr Ibn Zākūr, ed. Abdallah Guennoun (1966).</t>
         </is>
       </c>
       <c r="V123" s="13" t="inlineStr">
@@ -18332,7 +18365,8 @@
       </c>
       <c r="X123" s="13" t="inlineStr">
         <is>
-          <t>Original text: standard life-plus-70 term expired; author died 1708. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.</t>
+          <t>Original text: standard life-plus-70 term expired; author died 1708. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship. The poem is in al-Muntakhab min shiʿr Ibn Zākūr, edited by Abdallah Guennoun (1966).</t>
         </is>
       </c>
       <c r="Y123" s="13" t="inlineStr">
@@ -19022,7 +19056,8 @@
       </c>
       <c r="X128" s="13" t="inlineStr">
         <is>
-          <t>Original text: standard life-plus-70 term expired; author died 1896. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.</t>
+          <t>Original text: standard life-plus-70 term expired; author died 1896. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y128" s="13" t="inlineStr">
@@ -19895,7 +19930,8 @@
       </c>
       <c r="X134" s="13" t="inlineStr">
         <is>
-          <t>Public-domain historical text - PD-old-100 notice</t>
+          <t>Public-domain historical text - PD-old-100 notice
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y134" s="13" t="n"/>
@@ -20061,7 +20097,8 @@
       </c>
       <c r="X135" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1862. Modern editorial additions and translations are separate.</t>
+          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1862. Modern editorial additions and translations are separate.
+Anthology review (30 October 2026): first published before 1931 and the poet died long before 1956, so public domain in the UK, EU and US.</t>
         </is>
       </c>
       <c r="Y135" s="13" t="inlineStr">
@@ -20396,7 +20433,8 @@
       <c r="W137" s="13" t="inlineStr">
         <is>
           <t>Text varies in stanza/line count across modern reproductions. Biography gives differing death traditions (1803 or 1810); both are well outside copyright term. Modern song settings and editorial prose excluded.
-Passage update (29 October 2026): Complete poem, 9 couplets (18 half-lines), as printed by the Al-Babtain Library. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
+Passage update (29 October 2026): Complete poem, 9 couplets (18 half-lines), as printed by the Al-Babtain Library. Fresh English translation by Claude (Anthropic AI); draft for editorial review.
+Moved to Poems to explore (30 October 2026) for the anthology review. Oman: no printing of this poem before 1989 could be established.</t>
         </is>
       </c>
       <c r="X137" s="13" t="inlineStr">
@@ -20411,7 +20449,7 @@
       </c>
       <c r="Z137" s="11" t="inlineStr">
         <is>
-          <t>Original text</t>
+          <t>Read the text</t>
         </is>
       </c>
       <c r="AA137" s="11" t="inlineStr">
@@ -20560,7 +20598,8 @@
       </c>
       <c r="X138" s="13" t="inlineStr">
         <is>
-          <t>Public-domain eighteenth-century original; modern editorial material, translations and recordings excluded.</t>
+          <t>Public-domain eighteenth-century original; modern editorial material, translations and recordings excluded.
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y138" s="13" t="inlineStr">
@@ -21032,7 +21071,8 @@
       </c>
       <c r="X141" s="13" t="inlineStr">
         <is>
-          <t>Historical original text: standard life-plus-70 term has expired; author died 1940. Assessment excludes modern translations, commentary, editorial alterations, musical settings and recordings. Territorial and unusual publication-history exceptions are not comprehensively assessed.</t>
+          <t>Historical original text: standard life-plus-70 term has expired; author died 1940. Assessment excludes modern translations, commentary, editorial alterations, musical settings and recordings. Territorial and unusual publication-history exceptions are not comprehensively assessed.
+Anthology review (30 October 2026): Ricardo Miró died 1940; the poet died before 1956 (UK/EU public domain); in the US, whatever the date of first publication, the poem was already out of copyright at home on 1 January 1996, so US copyright was never restored.</t>
         </is>
       </c>
       <c r="Y141" s="13" t="inlineStr">
@@ -25146,7 +25186,8 @@
       </c>
       <c r="X169" s="13" t="inlineStr">
         <is>
-          <t>Public-domain Classical Chinese original; author PD-old-100 notice</t>
+          <t>Public-domain Classical Chinese original; author PD-old-100 notice
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y169" s="13" t="n"/>
@@ -26255,7 +26296,8 @@
       </c>
       <c r="X177" s="13" t="inlineStr">
         <is>
-          <t>Public-domain tenth-century Arabic original; later song versions and editorial contributions excluded.</t>
+          <t>Public-domain tenth-century Arabic original; later song versions and editorial contributions excluded.
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y177" s="13" t="inlineStr">
@@ -26403,7 +26445,8 @@
       </c>
       <c r="X178" s="13" t="inlineStr">
         <is>
-          <t>Public-domain medieval Persian original; individual attribution and textual transmission require normal editorial checking.</t>
+          <t>Public-domain medieval Persian original; individual attribution and textual transmission require normal editorial checking.
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y178" s="13" t="inlineStr">
@@ -27591,7 +27634,8 @@
       </c>
       <c r="X186" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original in life+70 jurisdictions (author died 1934)</t>
+          <t>Public-domain original in life+70 jurisdictions (author died 1934)
+Anthology review (30 October 2026): Sibil died 1934; the poet died before 1956 (UK/EU public domain); in the US, whatever the date of first publication, the poem was already out of copyright at home on 1 January 1996, so US copyright was never restored.</t>
         </is>
       </c>
       <c r="Y186" s="13" t="n"/>
@@ -28088,7 +28132,8 @@
       </c>
       <c r="X190" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original; site transcription has CC BY-SA terms where applicable</t>
+          <t>Public-domain original; site transcription has CC BY-SA terms where applicable
+Anthology review (30 October 2026): Lesya Ukrainka died 1913; the poet died before 1956 (UK/EU public domain); in the US, whatever the date of first publication, the poem was already out of copyright at home on 1 January 1996, so US copyright was never restored.</t>
         </is>
       </c>
       <c r="Y190" s="13" t="n"/>
@@ -28863,7 +28908,8 @@
       </c>
       <c r="X195" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original; site transcription has CC BY-SA terms where applicable</t>
+          <t>Public-domain original; site transcription has CC BY-SA terms where applicable
+Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y195" s="13" t="n"/>
@@ -29172,7 +29218,8 @@
       </c>
       <c r="X197" s="13" t="inlineStr">
         <is>
-          <t>Original text: standard life-plus-70 term expired; author died 1866. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.</t>
+          <t>Original text: standard life-plus-70 term expired; author died 1866. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.
+Anthology review (30 October 2026): first published before 1931 and the poet died long before 1956, so public domain in the UK, EU and US. By 1865.</t>
         </is>
       </c>
       <c r="Y197" s="13" t="inlineStr">
@@ -29374,57 +29421,65 @@
       </c>
       <c r="D199" s="13" t="inlineStr">
         <is>
-          <t>غزال ما مثله بصنعا غزال (incipit; Ghazāl mā mithluhu bi-Ṣanʿā ghazāl)</t>
+          <t>طرب الفؤاد لطيف روضة غاشي</t>
         </is>
       </c>
       <c r="E199" s="13" t="inlineStr">
         <is>
-          <t>A gazelle unlike any other in Sana'a (first-line sense)</t>
+          <t>My heart thrilled at Rawda's phantom</t>
         </is>
       </c>
       <c r="F199" s="13" t="inlineStr">
         <is>
-          <t>غزال ما مثله بصنعا غزال
-بسيف لحظه قد غزا لي
-أزال ثوب الصبر عني وزال
-وصار تايه في أزال
-سلب على البدر البها والكمال
-وقد سلب روحي كمالي
-وطال بالهجران بعد الوصال
-على فؤاد للنار صالي
-قد خلف المضني معنى وسار
-كالبدر جنح الليل ساري
-ماذا جرى بيني وبينك ودار
-والله بذا عالم وداري
-أقل خطايا مغرمك والعثار
-وخذ من الواشي بثاري
-لا تستمع حاسد بقيل وقال
-ولا تصدق قول قالي</t>
+          <t>طربَ الفؤاد لطيفِ روضةَ غاشي
+والقومُ بين أباطحٍ وعشاشِ
+أنَّى اهتديتِ ودونَ أرضكِ سبسبٌ
+قَفْرٌ وحَزْنٌ في دُجىً ورِشاشِ
+قالتْ: تكاليفُ المحبِّ كلفتها
+إنَّ المحِبَّ إذا أُخيفَ لَماشِي
+أدعوكِ روضةَ رحبٍ واسمكِ غيرهُ
+شفقاً وأخشى أن يشي بكِ واشي
+قَالَتْ: فَزُرْنا قلتُ كيفَ أزُورُكم
+وأنا امرُؤٌ لِخُروجِ سِرِّكِ خاشِي
+قَالَتْ: فكُنْ لِعُمومَتي سَلْماً مَعاً
+والطفْ لإخوتيَ الذين تماشي
+فَتَزورَنا معهُم زيارةَ آمنٍ
+والسرُّ يا وَضَّاحُ لَيس بفَاشِي
+ولقيتها تمشي بأبطحَ مرةً
+بِخلاخِلٍ وبِحُلَّةٍ أكْباشِ
+فَظَلِلْتُ مَعْمُوداً وبِتُّ مُسَهَّداً
+ودموعُ عيني في الرداءِ غواشي
+يا رَوْضُ حُبُّكِ سَلَّ جِسمي وانْتَحى
+فِي العَظْمِ حتى قدْ بَلَغْتِ مُشاشِي</t>
         </is>
       </c>
       <c r="G199" s="13" t="inlineStr">
         <is>
-          <t>A gazelle like no other gazelle in Sanaa
-has raided me with the sword of his glance.
-He stripped the robe of patience from me and left,
-and now wanders proudly through Azal.
-He robbed the full moon of its splendour and perfection,
-and robbed my soul of all I had.
-After union he has drawn out his desertion
-over a heart that is roasting in the fire.
-He left the lovesick one in torment and went on,
-like the full moon travelling through the night.
-What happened, what passed between us,
-God knows, and is aware of it.
-Forgive your lover his sins and his stumbles,
-and take my revenge on the slanderer.
-Do not listen to the envious, with their gossip,
-and do not believe what a hater says.</t>
+          <t>My heart thrilled when Rawda's phantom came to me
+while the company slept among the valleys and the scrub.
+How did you find your way, when between us and your land
+lies a waste, empty and rugged, in darkness and drizzle?
+She said: I have taken on the burdens of one who loves;
+a lover, even when threatened, keeps on walking.
+I call you “Rawda of the open plain”, though your name is another,
+out of care, for I fear some tale-bearer will betray you.
+She said: Then come and visit us. I said: How can I visit you,
+when I am a man who dreads your secret coming out?
+She said: Then make your peace with all my uncles,
+and be kind to my brothers when you walk with them;
+then you can visit us with them, as one who is safe,
+and the secret, Waddah, will not get out.
+And once I met her walking in a valley,
+in anklets and a fine striped robe;
+all day I was lovesick, all night I lay awake,
+and the tears of my eyes soaked my cloak.
+O Rawd, your love has wasted my body and pressed on
+into the bone, until it has reached the marrow.</t>
         </is>
       </c>
       <c r="H199" s="13" t="inlineStr">
         <is>
-          <t>Ahmad ibn Abd al-Rahman al-Ansi (أحمد بن عبد الرحمن الآنسي)</t>
+          <t>Waddah al-Yaman (وضاح اليمن)</t>
         </is>
       </c>
       <c r="I199" s="13" t="inlineStr">
@@ -29447,10 +29502,14 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M199" s="14" t="n"/>
+      <c r="M199" s="14" t="inlineStr">
+        <is>
+          <t>700</t>
+        </is>
+      </c>
       <c r="N199" s="13" t="inlineStr">
         <is>
-          <t>Arabic, Yemeni Humayni verse</t>
+          <t>Arabic</t>
         </is>
       </c>
       <c r="O199" s="13" t="inlineStr">
@@ -29460,32 +29519,32 @@
       </c>
       <c r="P199" s="13" t="inlineStr">
         <is>
-          <t>Lyric poem</t>
+          <t>Poem (qasida, 10 couplets)</t>
         </is>
       </c>
       <c r="Q199" s="13" t="inlineStr">
         <is>
-          <t>Man author</t>
+          <t>Waddah al-Yaman (died c. 708)</t>
         </is>
       </c>
       <c r="R199" s="13" t="inlineStr">
         <is>
-          <t>Before 1825; exact date unknown</t>
+          <t>Umayyad period, late 7th–early 8th century</t>
         </is>
       </c>
       <c r="S199" s="13" t="inlineStr">
         <is>
-          <t>Linked digital transcription/facsimile; precise edition date not established</t>
+          <t>Kitab al-Aghani (first printed Bulaq, 1868), vol. 6</t>
         </is>
       </c>
       <c r="T199" s="13" t="inlineStr">
         <is>
-          <t>A lover compares the beloved to a unique gazelle of Sana’a, laments separation and pledges continuing devotion.</t>
+          <t>The phantom of his beloved Rawda visits the poet by night; she tells him how he might visit her family safely, and he confesses that her love has reached the marrow of his bones.</t>
         </is>
       </c>
       <c r="U199" s="13" t="inlineStr">
         <is>
-          <t>DCT Poetic Encyclopedia, text and Yemeni biography; identifies Sana’a judge and Humayni poet, died 1825.</t>
+          <t>Abu al-Faraj al-Isfahani, Kitab al-Aghani, section on Waddah al-Yaman (vol. 6); text from Arabic Wikisource, checked against the Aghani.</t>
         </is>
       </c>
       <c r="V199" s="13" t="inlineStr">
@@ -29495,23 +29554,22 @@
       </c>
       <c r="W199" s="13" t="inlineStr">
         <is>
-          <t>Distinguish this poet from later singers and musical arrangements. Modern edited editions and translations have separate rights.
-Passage update (29 October 2026): First 8 couplets (16 half-lines) of the 16-couplet poem, as printed in the Abu Dhabi Poetry Encyclopedia. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
+          <t>Work changed (30 October 2026): al-Ansi's song, for which no printing before 1989 could be established, is replaced by a love poem by Yemen's best-known early love poet, preserved in the 10th-century Kitab al-Aghani. Complete poem, 10 couplets (20 half-lines). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
         </is>
       </c>
       <c r="X199" s="13" t="inlineStr">
         <is>
-          <t>Original text: standard life-plus-70 term expired; author died 1825. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.</t>
+          <t>Anthology review (30 October 2026): Umayyad poem preserved in Kitab al-Aghani, printed since 1868: public domain everywhere.</t>
         </is>
       </c>
       <c r="Y199" s="13" t="inlineStr">
         <is>
-          <t>Poetic Encyclopedia, Department of Culture and Tourism — Abu Dhabi</t>
+          <t>Arabic Wikisource: طرب الفؤاد لطيف روضة غاشي; Kitab al-Aghani vol. 6</t>
         </is>
       </c>
       <c r="Z199" s="11" t="inlineStr">
         <is>
-          <t>Original text</t>
+          <t>Read the whole work</t>
         </is>
       </c>
       <c r="AA199" s="11" t="inlineStr">
@@ -29530,7 +29588,11 @@
         </is>
       </c>
       <c r="AD199" s="11" t="n"/>
-      <c r="AE199" s="11" t="n"/>
+      <c r="AE199" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: Original text</t>
+        </is>
+      </c>
     </row>
     <row r="200" ht="60" customHeight="1" s="17">
       <c r="A200" s="7" t="inlineStr">
@@ -30425,13 +30487,14 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA199" r:id="rId662"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB199" r:id="rId663"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC199" r:id="rId664"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z200" r:id="rId665"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z201" r:id="rId666"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE201" r:id="rId667"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE199" r:id="rId665"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z200" r:id="rId666"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z201" r:id="rId667"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE201" r:id="rId668"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId668"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId669"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Anthology review: fresh translations for 36 poems
All English versions that came from earlier ChatGPT drafts are replaced
by fresh translations made directly from the originals, recorded in the
spreadsheet. Three lines of Tagore's "Unending Love" reworded so they do
not echo published English versions.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -913,16 +913,16 @@
       </c>
       <c r="G7" s="13" t="inlineStr">
         <is>
-          <t>Love for him has bound me once again;
-all my struggling has been in vain.
-Love is a sea whose shore is lost to sight—
-how can you hope to swim it, prudent one?
-If you would follow love through to its end,
-you must accept so much you cannot bear:
-see ugliness and reckon it as beauty,
-drink poison and imagine it is sugar.
-I struggled wildly, never understanding:
-the more I pulled, the tighter drew the snare.</t>
+          <t>Once more his love has caught me in its bonds;
+for all my struggling, nothing came of it.
+Love is an ocean with no shore in sight:
+how could anyone swim it, clever one?
+If you would carry love on to its end,
+you must accept much that you dislike:
+see what is ugly and call it fair,
+drink poison down and call it sugar.
+I bucked and fought, and never understood
+that pulling only draws the lasso tighter.</t>
         </is>
       </c>
       <c r="H7" s="13" t="inlineStr">
@@ -995,7 +995,8 @@
       <c r="W7" s="13" t="inlineStr">
         <is>
           <t>The medieval Persian text is the reusable work; the modern anthology introduction and apparatus are separate. Biography and the Baktash love story combine historical and legendary traditions. Country connection is Balkh, now Afghanistan. The selection is the original-language text; an existing English translation is not required.
-English passage: Fresh English translation by ChatGPT; draft for editorial review. Complete poem, 10 translated lines; PDF page2, printed p.188, poem3. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+English passage: Earlier English draft by ChatGPT (replaced); draft for editorial review. Complete poem, 10 translated lines; PDF page2, printed p.188, poem3. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X7" s="13" t="inlineStr">
@@ -1076,18 +1077,18 @@
       </c>
       <c r="G8" s="13" t="inlineStr">
         <is>
-          <t>In your face I found Beauty,
-like him who found God upon the mountain.
-How lovely are the flowers of May!
-Yet beside you they seemed unpleasant to me.
-When I look upon your cheeks,
-what value does the rose retain?
-Your voice gives life to my soul
-and leaves the nightingale without its charm.
-Even the stars and moon seemed disfigured
-when I beheld that lovely eye.
-Golden wand! Silver arrow!
-You burned my heart and scattered all my thoughts!</t>
+          <t>In your face I came upon Beauty,
+as one who came upon God in the mountains.
+How fine the little flowers of May are!
+Yet next to you they seemed to me ill-favoured.
+When I see your cheeks,
+what worth is left to the rose?
+Your voice gives me back my soul;
+it leaves the nightingale no sweetness.
+Even the stars and the moon looked dimmed to me
+once I had seen that eye, as if drawn by a pen.
+Golden rod! Silver arrow!
+You set my heart on fire and scattered my wits!</t>
         </is>
       </c>
       <c r="H8" s="13" t="inlineStr">
@@ -1162,7 +1163,8 @@
       <c r="W8" s="13" t="inlineStr">
         <is>
           <t>Use the Albanian poem, not a modern translation or explanatory text. The OCR has old orthography and errors; translate from the scan. Author died 1900. The selection is the original-language text; an existing English translation is not required.
-Passage update (29 October 2026): Fresh English translation by ChatGPT; editorial draft, not a quoted published translation. Original and English contain the same selection. Wording follows the VOAL transcription (24 May 2016), not the corrupt OCR of the historical PDF. Historical spelling retained. Compare against the historical scan, printed p.53, before publication. The mountain reference evokes Moses.</t>
+Passage update (29 October 2026): Earlier English draft by ChatGPT (replaced); editorial draft, not a quoted published translation. Original and English contain the same selection. Wording follows the VOAL transcription (24 May 2016), not the corrupt OCR of the historical PDF. Historical spelling retained. Compare against the historical scan, printed p.53, before publication. The mountain reference evokes Moses.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X8" s="13" t="inlineStr">
@@ -1244,18 +1246,18 @@
       </c>
       <c r="G9" s="13" t="inlineStr">
         <is>
-          <t>The sovereignty of beauty asserts its pride
-over the lord of horses and the generous man.
-Such conduct is forgiven, and is fair,
-if one day I may spend the night at our meeting place.
-For if she is pleased with me, she shows a face
-whose smiling loveliness remains in view.
-My friend, if one day you should come to me
-bearing glad news of union and affection,
-then, if you wish my life in payment for that news,
-take it, with all my wealth, both new and old.
-When other people set their hearts on treasures,
-my cousin is my treasure and provision.</t>
+          <t>The sultan of beauty carries itself proudly
+above the horseman and the open-handed man;
+and this is pardoned, and becomes it well,
+if one day I may pass a night with a promise of meeting.
+If she is pleased with me, she shows me a face
+that smiles, its loveliness always plain to see.
+My friend, if one day you come to me
+with good news of union and of love,
+and want my life as payment for the news,
+take it, with all I have gained and all I inherited.
+When people set their hearts on buried treasure,
+my cousin is my treasure and my store.</t>
         </is>
       </c>
       <c r="H9" s="13" t="inlineStr">
@@ -1330,7 +1332,8 @@
       <c r="W9" s="13" t="inlineStr">
         <is>
           <t>Identifier is the original incipit. The poem includes longing, reproach and conventional hyperbole about the beloved’s cruelty, rather than consistently cheerful love. Year 1883 is an upper bound, not a composition date. Modern annotations and translations are excluded.
-Passage update (29 October 2026): Fresh English translation by ChatGPT; editorial draft, not a quoted published translation. Original and English contain the same selection. Elongation marks and most diacritics omitted. The difficult phrase أبيت على معاد is translated provisionally as spending a night at the appointed meeting place. بنت العم means female paternal cousin; this line does not explicitly say wife. Arabic specialist review recommended.</t>
+Passage update (29 October 2026): Earlier English draft by ChatGPT (replaced); editorial draft, not a quoted published translation. Original and English contain the same selection. Elongation marks and most diacritics omitted. The difficult phrase أبيت على معاد is translated provisionally as spending a night at the appointed meeting place. بنت العم means female paternal cousin; this line does not explicitly say wife. Arabic specialist review recommended.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X9" s="13" t="inlineStr">
@@ -1531,19 +1534,19 @@
       </c>
       <c r="G11" s="13" t="inlineStr">
         <is>
-          <t>In this little town
-I saw a certain maiden,
-so full of beauty,
-of fairy, houri and divinity,
-to whom I said: “My darling,
-please grant me a kiss;
-you know well, my love,
-that I would give my life for you!”
+          <t>In this small town
+I saw a certain young woman,
+blessed with great beauty,
+like a fairy, a houri, a goddess,
+and I said to her: “My dear one,
+I ask you for a kiss, please;
+you know very well, my love,
+I would give my life for you!”
 “Nguami-âmi, ngana-lame,
-‘I do not want to, dear sir,’”
-she said, without changing colour;
+‘I don't want to, kind sir,’”
+she said, without a blush;
 “maculo! quangandallâmi,
-‘I do not believe in your love’...”</t>
+‘I don't believe in your love’…”</t>
         </is>
       </c>
       <c r="H11" s="13" t="inlineStr">
@@ -1618,7 +1621,8 @@
       <c r="W11" s="13" t="inlineStr">
         <is>
           <t>Explicitly described as an imitation of verses by João E. da Cruz Toulson. Reuse the historical poem, not the modern criticism. The encounter ends in rejection.
-Passage update (29 October 2026): Fresh English translation by ChatGPT; editorial draft, not a quoted published translation. Original and English contain the same selection. Historical poem quoted in Sheila Ribeiro Jacob’s article. Kimbundu forms retain this source’s spelling and are followed by the poem’s Portuguese glosses, translated here. No independent Kimbundu translation is claimed. Other transcriptions differ. Opening excerpt, not complete poem.</t>
+Passage update (29 October 2026): Earlier English draft by ChatGPT (replaced); editorial draft, not a quoted published translation. Original and English contain the same selection. Historical poem quoted in Sheila Ribeiro Jacob’s article. Kimbundu forms retain this source’s spelling and are followed by the poem’s Portuguese glosses, translated here. No independent Kimbundu translation is claimed. Other transcriptions differ. Opening excerpt, not complete poem.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X11" s="13" t="inlineStr">
@@ -1819,20 +1823,20 @@
       </c>
       <c r="G13" s="13" t="inlineStr">
         <is>
-          <t>Two words so sweet that the moon,
-filtering through the branches,
-stopped upon my mouth. Two words so sweet
-that an ant walks across my neck and I do not try
-to move and brush it off.
-Two words so sweet
-that I say, without meaning to: Oh, how beautiful life is!
-So sweet and so gentle
-that they pour fragrant oils over my body.
-So sweet and so beautiful
+          <t>Two words so sweet that the moon, which was wandering,
+sifting through the branches,
+came to rest on my mouth. So sweet, two words,
+that an ant is strolling along my neck and I make no effort
+to move and send it away.
+So sweet, two words,
+that I say without meaning to — oh, how lovely life is —
+so sweet and so tender
+they pour scented oils over my body.
+So sweet and so lovely
 that the longest fingers of my right hand
-move towards the sky, imitating scissors.
-Those two fingers long
-to cut down stars.</t>
+reach for the sky, snipping like scissors.
+My two fingers would like
+to cut stars.</t>
         </is>
       </c>
       <c r="H13" s="13" t="inlineStr">
@@ -1907,7 +1911,8 @@
       <c r="W13" s="13" t="inlineStr">
         <is>
           <t>Swiss-born Argentine poet; country follows her Argentine literary career. The transcription is marked uncorrected; compare the scan before quotation. Original-language poem only; modern translations and recordings are separate. Retain attribution and source/license links for copyrightable transcription material.
-English passage: Fresh English translation by ChatGPT; draft for editorial review. Final14 lines; opening four lines omitted. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+English passage: Earlier English draft by ChatGPT (replaced); draft for editorial review. Final14 lines; opening four lines omitted. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X13" s="13" t="inlineStr">
@@ -1983,18 +1988,18 @@
       </c>
       <c r="G14" s="13" t="inlineStr">
         <is>
-          <t>As long as I am alive,
-beloved, I am devoted to you.
-What else can I do?
-I shall shed tears,
-draw many sighs,
-and bear your pain, beloved.
-Say that I am your gazelle;
-let me gaze upon you,
-let me look at you, beloved.
-Enter the garden gracefully;
-I shall praise you with my saz,
-beloved, with an earnest plea.</t>
+          <t>For as long as I live, my soul,
+beloved, I am your sacrifice.
+What else am I to do?
+I will weep,
+I will sigh from deep in my heart,
+beloved, I will carry your sorrow.
+I am your captive, my gazelle;
+let me look at you to my heart's content,
+beloved, let me gaze.
+Come into the garden with your graceful air;
+I will praise you on my saz,
+beloved, with my entreaty.</t>
         </is>
       </c>
       <c r="H14" s="13" t="inlineStr">
@@ -2067,7 +2072,8 @@
       <c r="W14" s="13" t="inlineStr">
         <is>
           <t>Original words only; later settings, arrangements and recordings are separate. Sayat-Nova died 1795. Transcription is not tied to a named print edition; compare an authoritative edition before publication. The selection is the original-language text; an existing English translation is not required.
-Passage update (29 October 2026): Fresh English translation by ChatGPT; editorial draft, not a quoted published translation. Original and English contain the same selection. Tbilisi dialect spelling retained. ղուրբան is rendered idiomatically as devotion. Ասիր՝ ջեյրան իմ is interpreted as Say that I am your gazelle. Dialect specialist review recommended.</t>
+Passage update (29 October 2026): Earlier English draft by ChatGPT (replaced); editorial draft, not a quoted published translation. Original and English contain the same selection. Tbilisi dialect spelling retained. ղուրբան is rendered idiomatically as devotion. Ասիր՝ ջեյրան իմ is interpreted as Say that I am your gazelle. Dialect specialist review recommended.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X14" s="13" t="inlineStr">
@@ -2311,18 +2317,18 @@
       </c>
       <c r="G16" s="13" t="inlineStr">
         <is>
-          <t>Today I heard your vows—
-and they did not stir my heart,
-though I myself believe that ardent love
-speaks from every word you say.
-For I cannot help but think
-of the time when you will try
-to hide in empty phrases
-the fading glow of an empty heart;
-when, weary at last of struggling,
-and tired of chains you chose yourself,
-shamelessly denying your own word,
-you will stand before me as a Judas.</t>
+          <t>I heard your vows today,
+and they leave my heart unmoved,
+though I believe myself that burning love
+speaks out of every word.
+For I can't help but think ahead
+to the time when you will strive
+to cover up with empty phrases
+the feebler glow of an empty heart;
+when, at last worn out with fighting
+and sick of chains you chose yourself,
+shamelessly disowning your own word,
+you will stand before me, a Judas.</t>
         </is>
       </c>
       <c r="H16" s="13" t="inlineStr">
@@ -2397,7 +2403,8 @@
       <c r="W16" s="13" t="inlineStr">
         <is>
           <t>Original-language poem only; modern translations and recordings are separate. Retain attribution and source/license links for copyrightable transcription material.
-English passage: Fresh English translation by ChatGPT; draft for editorial review. 12-line passage on printed p.68. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+English passage: Earlier English draft by ChatGPT (replaced); draft for editorial review. 12-line passage on printed p.68. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X16" s="13" t="inlineStr">
@@ -2471,16 +2478,16 @@
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>The tumult of your love will finally drive me mad;
-it is plain that love brings strife to the lover.
-The strands of your hair have made me such a captive;
-whatever befalls me is brought by those fresh tresses.
-If only I could see your rose-like face a moment:
-each sight of it brings radiant light.
-Eyebrow, eye and eyelash-tip have gathered to cause unrest;
-each shoots arrows, draws a sword and brings a quarrel.
-The strands of your hair plunder my heart
-as though an Abyssinian army were bringing pillage to Rum.</t>
+          <t>The frenzy of your love will drive me mad at last;
+this much is certain: love brings the lover strife.
+It is the strand of your hair that has snared me so;
+whatever befalls me, those scented locks bring it on.
+If I could look at your rose of a face for one moment,
+each look would bring a shining, radiant light.
+Brow, eye and lash-point have joined forces to stir up trouble:
+one shoots arrows, one draws a blade, each picks a fight.
+The strand of your hair so plunders my heart,
+it is as if an Abyssinian army brought sack and ruin to Rum.</t>
         </is>
       </c>
       <c r="H17" s="13" t="inlineStr">
@@ -2553,7 +2560,8 @@
       <c r="W17" s="13" t="inlineStr">
         <is>
           <t>Natavan was a Shusha/Karabakh poet in present-day Azerbaijan. Original ghazal only; modern transliteration/editorial contributions may require attribution. English translation not supplied.
-Passage update (29 October 2026): Fresh English translation by ChatGPT; editorial draft, not a quoted published translation. Original and English contain the same selection. Latin transcription follows Wikisource, including cəkib as printed. Final couplet retains a historical dark-hair/light-face military conceit involving Abyssinia and Rum. Classical vocabulary merits specialist review.</t>
+Passage update (29 October 2026): Earlier English draft by ChatGPT (replaced); editorial draft, not a quoted published translation. Original and English contain the same selection. Latin transcription follows Wikisource, including cəkib as printed. Final couplet retains a historical dark-hair/light-face military conceit involving Abyssinia and Rum. Classical vocabulary merits specialist review.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X17" s="13" t="inlineStr">
@@ -2745,18 +2753,18 @@
       </c>
       <c r="G19" s="13" t="inlineStr">
         <is>
-          <t>And a maiden whose glances hasten
-to slay souls, though her movements are slow;
-her figure like a ban-tree, her hips like dunes,
-her looks enchanting as Harut’s magic.
-I kissed her and soothed the heat within my breast
-with something sweeter than honey mixed with fresh water.
-She said, as I protested what her glances
-had done to me: “You are the proud, defiant one!”
-She teased me with those words in jest,
-and in that jest lay all my longing.
-How many a steadfast man has been laid low, doomed,
-by glances from the corners of eyes like yours.</t>
+          <t>And a maiden whose glances are quick
+to kill souls, though her movements are slow:
+a waist slender as a willow, hips heaped like sandhills,
+eyes with the magic of Harut.
+I kissed her, and cooled the fire in my ribs
+with something sweeter than honey in sweet river water.
+She said, when I complained of what her eyes
+had done to me: “You are the stubborn, unruly one!”
+She teased me with it in jest, and my heart's desire
+lay in the jest of those words.
+How many hardy men have been laid low before their time
+by sidelong glances like these!</t>
         </is>
       </c>
       <c r="H19" s="13" t="inlineStr">
@@ -2830,7 +2838,8 @@
       <c r="W19" s="13" t="inlineStr">
         <is>
           <t>Opening words serve as the poem identifier. Historical Bahrain association; modern national borders did not exist. No cleared English translation supplied.
-Passage update (29 October 2026): Fresh English translation by ChatGPT; editorial draft, not a quoted published translation. Original and English contain the same selection. Specified romantic episode, rather than landscape opening. Source line divisions retained, including the split definite article in bayt 18. Diacritics and elongation omitted. Harut is associated with magic. Classical expressions بانية الأعطاف and ألحاظ الجنبيات translated provisionally; specialist review recommended.</t>
+Passage update (29 October 2026): Earlier English draft by ChatGPT (replaced); editorial draft, not a quoted published translation. Original and English contain the same selection. Specified romantic episode, rather than landscape opening. Source line divisions retained, including the split definite article in bayt 18. Diacritics and elongation omitted. Harut is associated with magic. Classical expressions بانية الأعطاف and ألحاظ الجنبيات translated provisionally; specialist review recommended.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X19" s="13" t="inlineStr">
@@ -2912,18 +2921,18 @@
       </c>
       <c r="G20" s="13" t="inlineStr">
         <is>
-          <t>Nader Chand takes a winding path to market.
-The girl from the travelling troupe calls, “Bring me a nose-ring!”
-They gather fruit from the forest and eat together;
-together they lie down and sleep upon a smooth stone.
-At night he holds the maiden against his breast;
-by day they rise and wander, sharing many joys.
-Holding the lovely maiden’s hand, he roams from wood to wood;
-they pick the forest’s fruit to eat.
-They forget father, mother, home and household;
-forget their country, friends and dear relations.
-The two pass day and night in happiness of heart—
-then suddenly a thunderbolt falls upon their heads.</t>
+          <t>Nader Chand goes to market by the crooked path.
+The girl of the travelling players calls, “Buy me a nose-ring!”
+They pick wild fruit from the forest, and the two of them eat;
+on a smooth stone the two lie down to sleep.
+At night the young lord keeps the girl close to his breast;
+by day they rise and wander together, full of many joys.
+Holding the lovely girl's hand, he roams from wood to wood;
+they pluck the forest's fruit to eat.
+Forgotten father, forgotten mother, forgotten house and home;
+forgotten country, friends and dear kin.
+The two pass day and night with hearts content —
+then, without warning, a thunderbolt strikes them.</t>
         </is>
       </c>
       <c r="H20" s="13" t="inlineStr">
@@ -3000,7 +3009,8 @@
       <c r="W20" s="13" t="inlineStr">
         <is>
           <t>Mymensingh, in present-day Bangladesh. The original ballad is centuries old; Sen’s edition predates modern copyright terms (Sen died 1939). Use original verses; separate modern annotations and recordings. The linked reprint year is not the composition date. The selection is the original-language text; an existing English translation is not required.
-Passage update (29 October 2026): Fresh English translation by ChatGPT; editorial draft, not a quoted published translation. Original and English contain the same selection. Regional Bengali wording from linked 1958 reprint transcription; footnote numbers omitted. Final line foreshadows calamity. Narrative of lovers’ shared life rather than invocation. নদ্যার চান rendered as Nader Chand. Bengali specialist review recommended.</t>
+Passage update (29 October 2026): Earlier English draft by ChatGPT (replaced); editorial draft, not a quoted published translation. Original and English contain the same selection. Regional Bengali wording from linked 1958 reprint transcription; footnote numbers omitted. Final line foreshadows calamity. Narrative of lovers’ shared life rather than invocation. নদ্যার চান rendered as Nader Chand. Bengali specialist review recommended.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X20" s="13" t="inlineStr">
@@ -3204,17 +3214,17 @@
       </c>
       <c r="G22" s="13" t="inlineStr">
         <is>
-          <t>But now the time has come for us to part;
-surely this is the fate allotted us!
-I loved you deeply, dearest—
-but now it is time for us to part.
-In a distant land I shall pine,
+          <t>But now the hour has come for us to part;
+it must be that such is our lot!
+I loved you deeply, my dear,
+but the hour has come to part.
+I will pine away in a far-off land,
 keeping my love hidden in my heart;
-each night I shall gaze upon the star
-there in that distant land.
-Look at it sometimes while we are apart:
-there, upon it, our gazes will meet.
-So that love may live again, if only for a moment,
+every night I will gaze at the star,
+there, in the far-off land.
+Look at it sometimes while we're apart:
+there our glances will meet as one…
+So that our love may come alive for a moment,
 look at it sometimes…</t>
         </is>
       </c>
@@ -3290,7 +3300,8 @@
       <c r="W22" s="13" t="inlineStr">
         <is>
           <t>Original Belarusian poem only; exclude later musical settings. Author died 1917. Historical spelling differs from modern Belarusian. The selection is the original-language text; an existing English translation is not required.
-Passage update (29 October 2026): Fresh English translation by ChatGPT; editorial draft, not a quoted published translation. Original and English contain the same selection. Historical Belarusian spelling retained from 1927-edition transcription. French epigraph excluded. Final 12 of 20 Belarusian poem lines. Later musical settings excluded.</t>
+Passage update (29 October 2026): Earlier English draft by ChatGPT (replaced); editorial draft, not a quoted published translation. Original and English contain the same selection. Historical Belarusian spelling retained from 1927-edition transcription. French epigraph excluded. Final 12 of 20 Belarusian poem lines. Later musical settings excluded.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X22" s="13" t="inlineStr">
@@ -3374,19 +3385,19 @@
       <c r="G23" s="13" t="inlineStr">
         <is>
           <t>Oh, the splendour of our joy,
-woven in gold through the silken air!
-Here is the gentle house with its light gable,
-and the garden and the orchard.
-Here is the bench beneath the apple trees,
-from which white spring sheds its leaves
-in petals brushing slowly down.
-Here are flights of shining wood pigeons,
-hovering like omens
-in the clear sky of the landscape.
-Here—like kisses fallen to earth
-from the mouth of the delicate blue sky—
-are two blue ponds, simple and pure,
-innocently bordered by unbidden flowers.</t>
+woven in gold into the silken air!
+Here is the gentle house with its airy gable,
+and the garden, and the orchard.
+Here is the bench under the apple trees
+where the white spring is shedding
+its slow petals, brushing as they fall.
+Here are flights of bright wood pigeons
+gliding, like signs of what is to come,
+in the clear sky above the land.
+Here — like kisses dropped to earth
+from the lips of the fragile blue —
+are two blue ponds, plain and pure,
+fringed artlessly with flowers no one planted.</t>
         </is>
       </c>
       <c r="H23" s="13" t="inlineStr">
@@ -3461,7 +3472,8 @@
       <c r="W23" s="13" t="inlineStr">
         <is>
           <t>Original-language poem only; modern translations and musical recordings are separate.
-English passage: Fresh English translation by ChatGPT; draft for editorial review. Opening14 lines of poem identified by its first line. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+English passage: Earlier English draft by ChatGPT (replaced); draft for editorial review. Opening14 lines of poem identified by its first line. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X23" s="13" t="inlineStr">
@@ -3886,18 +3898,18 @@
       </c>
       <c r="G27" s="13" t="inlineStr">
         <is>
-          <t>Love… did you hear?… Love… Can you not
-see how everything burns as it passes?
-Autumn love that flees the sunset.
-Allow me, madam, for one brief moment
-to rest my lips, like a lover,
-upon the edge of your glove.
-Like a lover who kneels to behold
-the wonder of your eyes,
-of your lips, fresh and red;
-like a lover who were a child,
-asking, as a reward for his affection,
-the flower that adorns your bodice.</t>
+          <t>Love… did you hear? … Love… Do you not see
+how everything burns where it goes?
+Autumn love, fleeing the sunset.
+Let me, my lady, for one brief moment
+rest my lips, as a lover would,
+on the very tip of your glove.
+Like a lover who, on his knees, beholds
+the marvel of your eyes,
+of your lips, so fresh and red;
+like a lover who was a child
+asking, as the prize for his devotion,
+for the flower that decks your bodice.</t>
         </is>
       </c>
       <c r="H27" s="13" t="inlineStr">
@@ -3972,7 +3984,8 @@
       <c r="W27" s="13" t="inlineStr">
         <is>
           <t>Bolivian literary affiliation; born in Tacna and later active in Argentina. Author died 1933. Use original poem, excluding later critical essays. The selection is the original-language text; an existing English translation is not required.
-Passage update (29 October 2026): Fresh English translation by ChatGPT; editorial draft, not a quoted published translation. Original and English contain the same selection. Twelve consecutive historical poem lines. Punctuation and accents regularized from PDF extraction; cross-checked against Poesías completas (1957), digital transcription pp.40–41. Modern introduction and commentary excluded. huye el ocaso is read as fleeing the sunset.</t>
+Passage update (29 October 2026): Earlier English draft by ChatGPT (replaced); editorial draft, not a quoted published translation. Original and English contain the same selection. Twelve consecutive historical poem lines. Punctuation and accents regularized from PDF extraction; cross-checked against Poesías completas (1957), digital transcription pp.40–41. Modern introduction and commentary excluded. huye el ocaso is read as fleeing the sunset.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X27" s="13" t="inlineStr">
@@ -4055,20 +4068,20 @@
       </c>
       <c r="G28" s="13" t="inlineStr">
         <is>
-          <t>Last night, returning from the warm bathhouse,
-I passed beside the old imam’s garden;
-and there, in the garden, in the jasmine’s shade,
-stood Emina, a water-jug in her hand.
-Oh, what a beauty! I swear by my faith,
-she would have no cause for shame before the sultan!
-And when she walks and sways her shoulders—
-not even the hodja’s charm can help me now!
-I greeted her with salaam. But, by my faith,
-lovely Emina would not even listen;
-she filled her silver jug with water
-and went through the garden watering the roses.
-A breeze blew from the branches and down her shoulders
-unwound those thick braids of hers.</t>
+          <t>Last night, coming home from the warm hammam,
+I went past the old imam's garden;
+and there, in the garden, in the jasmine's shade,
+stood Emina with a jug in her hand.
+And what a beauty! By my faith,
+she'd be no shame even in the sultan's house!
+And then, when she walks and her shoulders move…
+not even the hodja's amulet can save me now!
+I wished her peace. But, by my religion,
+lovely Emina would not even hear it;
+she just dipped water into her silver jug
+and went off through the garden to water the roses;
+a wind blew from the branches and, down her shoulders,
+loosened those thick braids of hers,</t>
         </is>
       </c>
       <c r="H28" s="13" t="inlineStr">
@@ -4143,7 +4156,8 @@
       <c r="W28" s="13" t="inlineStr">
         <is>
           <t>Mostar and Bosnian sevdalinka context. Author died 1924; source explicitly marks the text public domain. Later added verses, arrangements and recordings are separate. The selection is the original-language text; an existing English translation is not required.
-Passage update (29 October 2026): Fresh English translation by ChatGPT; editorial draft, not a quoted published translation. Original and English contain the same selection. Historical poem excerpt, not a later performance adaptation. A hodja is a Muslim religious teacher; zapis here is a written charm. Source spelling retained.</t>
+Passage update (29 October 2026): Earlier English draft by ChatGPT (replaced); editorial draft, not a quoted published translation. Original and English contain the same selection. Historical poem excerpt, not a later performance adaptation. A hodja is a Muslim religious teacher; zapis here is a written charm. Source spelling retained.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X28" s="13" t="inlineStr">
@@ -4340,20 +4354,20 @@
       </c>
       <c r="G30" s="13" t="inlineStr">
         <is>
-          <t>“What, listening to the stars!” you will say. “Surely
-you have lost your senses!” Yet I shall tell you
-that often I wake to hear them
-and open the windows, pale with wonder.
-And we converse all night, while
-the Milky Way, like an open canopy,
-glitters. At sunrise, longing and in tears,
-I still seek them across the empty sky.
-Now you will say: “My crazy friend!
-What do you discuss with them? What meaning
-is there in what they say when they are with you?”
-And I shall tell you: “Love, to understand them!
-For only one who loves can have an ear
-able to hear and understand the stars.”</t>
+          <t>“Listening to stars!” you'll say. “You must
+have taken leave of your senses!” And yet I'll tell you
+that often I wake up to listen to them
+and fling the windows open, pale with awe…
+And we talk the whole night through, while
+the Milky Way, like a canopy spread open,
+sparkles. And when the sun comes, missing them, in tears,
+I still search for them across the empty sky.
+Now you will say: “My poor deluded friend!
+What do you talk about with them? What sense
+is there in what they say when they're with you?”
+And I will tell you: “Love, and you'll understand them!
+For only someone who loves can have ears
+able to hear and to understand the stars.”</t>
         </is>
       </c>
       <c r="H30" s="13" t="inlineStr">
@@ -4428,7 +4442,8 @@
       <c r="W30" s="13" t="inlineStr">
         <is>
           <t>Rights evidence is the 1902 edition record. Linked Wikisource transcription may include CC BY-SA site material; retain attribution/source where applicable. Modern translations are separate.
-Passage update (29 October 2026): Fresh English translation by ChatGPT; editorial draft, not a quoted published translation. Original and English contain the same selection. Complete historical sonnet. Verse lines restored from webpage blank spacing; quotation spacing regularized. Amai is the imperative Love. No existing published English translation is reproduced.</t>
+Passage update (29 October 2026): Earlier English draft by ChatGPT (replaced); editorial draft, not a quoted published translation. Original and English contain the same selection. Complete historical sonnet. Verse lines restored from webpage blank spacing; quotation spacing regularized. Amai is the imperative Love. No existing published English translation is reproduced.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X30" s="13" t="inlineStr">
@@ -4628,20 +4643,20 @@
       </c>
       <c r="G32" s="13" t="inlineStr">
         <is>
-          <t>You visited my soul again
+          <t>Once more you came to visit my soul
 and brought me Easter in the autumn!
-A bright peal rang out in the darkness;
-a cherub’s wing flies over us.
-And with your breath you lit my home;
-the dark curtains lifted,
-and joy, dead within me, rose again:
-within it there were only you and I.
-Our souls merged in a single kiss,
-and spring burst into bloom, the little birds sang
-and woke the garden flowers.
+A bright chiming spread through the darkness,
+a cherub's wing goes flying over us.
+You filled my house with light by your breath;
+the dark curtains were drawn back,
+and the joy that had died in me rose again:
+in it there were only you and me.
+In one kiss our souls were joined,
+and spring broke into flower, the birds began to sing
+and woke the flowers of the garden.
 And in the silence of white silk,
-your sheltering care enfolding me,
-I fly upon its quiet wing.</t>
+wrapped in your keeping,
+I fly on its quiet wing.</t>
         </is>
       </c>
       <c r="H32" s="13" t="inlineStr">
@@ -4716,7 +4731,8 @@
       <c r="W32" s="13" t="inlineStr">
         <is>
           <t>Only the historical poem is covered. The 2018 publisher’s edition/editorial matter is not an open licence; use plain original text, not its layout. No modern translation cleared.
-Passage update (29 October 2026): Fresh English translation by ChatGPT; editorial draft, not a quoted published translation. Original and English contain the same selection. Complete historical poem as reproduced by LiterNet. Opening addresses the beloved: You visited my soul again, not My soul visited again. English-title field corrected. Easter and resurrection imagery retained.</t>
+Passage update (29 October 2026): Earlier English draft by ChatGPT (replaced); editorial draft, not a quoted published translation. Original and English contain the same selection. Complete historical poem as reproduced by LiterNet. Opening addresses the beloved: You visited my soul again, not My soul visited again. English-title field corrected. Easter and resurrection imagery retained.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X32" s="13" t="inlineStr">
@@ -6208,18 +6224,18 @@
       </c>
       <c r="G43" s="13" t="inlineStr">
         <is>
-          <t>Listen: beneath the ruins of my passions,
-deep in this soul you no longer gladden,
-amid the dust of dreams and illusions,
-my black flowers lie numb and still.
+          <t>Listen: under the ruins of my passions,
+at the bottom of this soul you no longer make glad,
+among the dust of daydreams and illusions,
+my black flowers lie numbed.
 They are the memory of those hours
-when, held within my arms, you fell asleep,
+when you fell asleep, held captive in my arms,
 while I sighed for the dawns
-of your eyes—dawns that were not mine.
-They are my sorrows turned to buds,
-the fierce sorrows that within me
-bury their roots like ferns
-in the damp crevices of mountains.</t>
+of your eyes, dawns that were not mine.
+They are my griefs, turned into buds:
+the deep griefs that bury their roots
+in my innermost self, like ferns
+in the damp clefts of the mountains.</t>
         </is>
       </c>
       <c r="H43" s="13" t="inlineStr">
@@ -6292,7 +6308,8 @@
       <c r="W43" s="13" t="inlineStr">
         <is>
           <t>Author died 1923; Wikisource explicitly identifies his originals as public domain. Transcription has no named print edition; verify punctuation against a scan. Sad rather than celebratory. The selection is the original-language text; an existing English translation is not required.
-English passage: Fresh English translation by ChatGPT; draft for editorial review. Opening12 lines. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+English passage: Earlier English draft by ChatGPT (replaced); draft for editorial review. Opening12 lines. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X43" s="13" t="inlineStr">
@@ -7667,10 +7684,10 @@
       </c>
       <c r="G53" s="13" t="inlineStr">
         <is>
-          <t>You alone have become the thought of my thoughts;
-you are my heart's first love.
-I love you as no one else on earth;
-I love you through time and eternity.</t>
+          <t>You have become the one thought of my thoughts,
+you are the first love of my heart;
+I love you as no one here on earth,
+I love you in time and in eternity!</t>
         </is>
       </c>
       <c r="H53" s="13" t="inlineStr">
@@ -7745,7 +7762,8 @@
       <c r="W53" s="13" t="inlineStr">
         <is>
           <t>Country follows Danish text author Andersen; the composer was Norwegian. Reuse applies to the linked historical score and named translations; modern recordings are separate.
-English passage: Fresh English translation by ChatGPT; draft for editorial review. Complete poem,4 lines; translated from Andersen’s Danish, not the later German/English song versions. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+English passage: Earlier English draft by ChatGPT (replaced); draft for editorial review. Complete poem,4 lines; translated from Andersen’s Danish, not the later German/English song versions. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X53" s="13" t="inlineStr">
@@ -8228,18 +8246,18 @@
       </c>
       <c r="G57" s="13" t="inlineStr">
         <is>
-          <t>For my thoughts, filled with this affection
-that in one happy hour made me your slave,
-are sad, far from your eyes, like a child
-who falls asleep dreaming of your soothing voice.
-To wrap you in kisses, I would become the wind;
-I would become everything your hand touches,
-be your smile, be even your very breath,
-so that I might be nearer to your mouth.
-I live upon your words, and always hope
-to call you mine, as one hopes for a treasure.
-Far from you I understand how much I love you,
-and, kissing your letters, I weep like a child.</t>
+          <t>For my thoughts, full of this tenderness
+that made me your slave in one happy hour,
+are sad, away from your eyes, like a child
+who falls asleep dreaming of the lull of your voice.
+To wrap you in kisses I would like to be the wind,
+and to be everything your hand touches;
+to be your smile, to be your very breath,
+so as to be closer to your mouth.
+I live on your words, and forever hope
+to call you mine, as one hopes for a treasure;
+far from you I see how much I love you,
+and, kissing your letters, I simply weep.</t>
         </is>
       </c>
       <c r="H57" s="13" t="inlineStr">
@@ -8314,7 +8332,8 @@
       <c r="W57" s="13" t="inlineStr">
         <is>
           <t>Author died 1919. This covers the original poem only, not the musical setting or recordings. Textual versions differ, so compare an early print for the chosen passage. Contains a suicidal declaration; not an uncomplicated positive-love choice. The selection is the original-language text; an existing English translation is not required.
-English passage: Fresh English translation by ChatGPT; draft for editorial review. Lines5–16, three consecutive stanzas; opening and closing omitted. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+English passage: Earlier English draft by ChatGPT (replaced); draft for editorial review. Lines5–16, three consecutive stanzas; opening and closing omitted. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X57" s="13" t="inlineStr">
@@ -9527,18 +9546,18 @@
       </c>
       <c r="G66" s="13" t="inlineStr">
         <is>
-          <t>He did not speak,
-but his eyes spoke.
-You stranger,
-you so familiar!
-A day vanishes,
-a year slips by;
+          <t>he did not speak,
+but his eyes spoke. —
+You, the unknown one,
+you, the well-known one!
+A day goes by,
+a year flows past,
 one memory
-drives out another.
-That brief moment
-stayed with me for ever:
-that bitter moment,
-that sweet moment.</t>
+chases the next;
+the short moment
+stayed with me for ever,
+the bitter moment,
+the sweet moment.</t>
         </is>
       </c>
       <c r="H66" s="13" t="inlineStr">
@@ -9613,7 +9632,8 @@
       <c r="W66" s="13" t="inlineStr">
         <is>
           <t>Finnish literary provenance; original language is Swedish. Edition not identified. Credit author and Wikisource contributors; retain source/license, mark changes and observe ShareAlike where applicable.
-English passage: Fresh English translation by ChatGPT; draft for editorial review. Final12 lines of18-line poem. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+English passage: Earlier English draft by ChatGPT (replaced); draft for editorial review. Final12 lines of18-line poem. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X66" s="13" t="inlineStr">
@@ -9692,21 +9712,21 @@
       </c>
       <c r="G67" s="13" t="inlineStr">
         <is>
-          <t>Mother of memories, mistress of mistresses,
+          <t>Mother of memories, loveliest of lovers,
 you, all my pleasures, you, all my duties!
-You will remember the beauty of caresses,
-the sweetness of the hearth, the charm of evenings,
-mother of memories, mistress of mistresses!
-Evenings lit by the glowing coal,
-and evenings on the balcony, veiled in rosy mist;
-how sweet your breast was, how kind your heart!
-We often spoke of things that cannot perish,
-on evenings lit by the glowing coal.
-How beautiful the sunsets on those warm evenings!
-How deep the space, how mighty the heart!
-Leaning towards you, queen of those adored,
-I thought I breathed the fragrance of your blood.
-How beautiful the sunsets on those warm evenings!</t>
+You'll remember the beauty of our caresses,
+the softness of the hearth and the spell of the evenings,
+mother of memories, loveliest of lovers!
+Evenings lit by the glow of the coals,
+and evenings on the balcony, veiled in pink haze;
+how soft your breast was to me! how kind your heart!
+Often we said things that will never die,
+on evenings lit by the glow of the coals.
+How beautiful the suns are on warm evenings!
+How deep the sky is! How strong the heart!
+Bending towards you, queen of the adored,
+I seemed to breathe the perfume of your blood.
+How beautiful the suns are on warm evenings!</t>
         </is>
       </c>
       <c r="H67" s="13" t="inlineStr">
@@ -9781,7 +9801,8 @@
       <c r="W67" s="13" t="inlineStr">
         <is>
           <t>Original-language poem only; modern translations and musical recordings are separate.
-English passage: Fresh English translation by ChatGPT; draft for editorial review. Opening15 lines, three consecutive stanzas. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+English passage: Earlier English draft by ChatGPT (replaced); draft for editorial review. Opening15 lines, three consecutive stanzas. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X67" s="13" t="inlineStr">
@@ -10244,14 +10265,14 @@
       </c>
       <c r="G71" s="13" t="inlineStr">
         <is>
-          <t>You are like a flower,
-so lovely, beautiful and pure.
-I look at you, and sadness
-steals into my heart.
-I feel as though I ought to lay
+          <t>You are just like a flower,
+so sweet and fair and pure;
+I look at you, and sorrow
+creeps softly into my heart.
+I feel as if I ought to rest
 my hands upon your head,
-praying that God preserve you
-so pure, so beautiful, so lovely.</t>
+praying that God will keep you
+so pure and fair and sweet.</t>
         </is>
       </c>
       <c r="H71" s="13" t="inlineStr">
@@ -10326,7 +10347,8 @@
       <c r="W71" s="13" t="inlineStr">
         <is>
           <t>Original-language poem only. Modern translations and editorial material are separate.
-English passage: Fresh English translation by ChatGPT; draft for editorial review. Complete poem,8 lines; shorter than requested because the work is short. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+English passage: Earlier English draft by ChatGPT (replaced); draft for editorial review. Complete poem,8 lines; shorter than requested because the work is short. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X71" s="13" t="inlineStr">
@@ -12324,11 +12346,11 @@
       </c>
       <c r="G84" s="13" t="inlineStr">
         <is>
-          <t>It seems I have loved you in a hundred forms, a hundred times,
-In life after life, age after age, without end.
+          <t>It is as if I have loved you, only you, in a hundred shapes, a hundred times,
+birth upon birth, era upon era, without cease.
 Forever my spellbound heart has strung a garland of songs;
 In how many forms you have worn it round your neck and taken the gift,
-In life after life, age after age, without end.
+birth upon birth, era upon era, without cease.
 Whenever I hear those tales of the past, the ache of ancient love,
 The age-old stories of parting and meeting,
 As I gaze and gaze into the boundless past, at last
@@ -12419,7 +12441,8 @@
         <is>
           <t>Author translation; preface notes abridgement and paraphrase. Modern translations are separate.
 English passage: Original English text; not a translation. Poem16, first three paragraphs; author’s English version, reflowed into12 reading lines. Corrected obvious transcription in→is before unfinished; no new translation.. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
-Work changed (29 October 2026): The Gardener, poem 16 (Tagore’s own English) replaced by the Bengali original অনন্ত প্রেম, whose source is certain. Complete poem, 20 lines. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
+Work changed (29 October 2026): The Gardener, poem 16 (Tagore’s own English) replaced by the Bengali original অনন্ত প্রেম, whose source is certain. Complete poem, 20 lines. Fresh English translation by Claude (Anthropic AI); draft for editorial review.
+Revision (30 October 2026): lines 1, 2 and 5 reworded so they do not echo the wording of published English versions.</t>
         </is>
       </c>
       <c r="X84" s="13" t="inlineStr">
@@ -13186,14 +13209,14 @@
       </c>
       <c r="G89" s="13" t="inlineStr">
         <is>
-          <t>Who are you? Why does an outstretched hand
-not meet a kindred hand?
+          <t>Who are you? Why does a hand held out
+not meet a sister's hand?
 And eyes wait only a moment,
-then lower themselves, embarrassed.
-A locked garden. No path to it, no road.
-A locked garden—a human being.
-Shall I go away? Or strike the rock
-until blood flows?</t>
+and look, they're already lowered in confusion.
+A locked garden. No path to it, no way in.
+A locked garden: a person.
+Shall I go away? Or beat against the rock
+till the blood runs?</t>
         </is>
       </c>
       <c r="H89" s="13" t="inlineStr">
@@ -13268,7 +13291,8 @@
       <c r="W89" s="13" t="inlineStr">
         <is>
           <t>Rachel died 1931. Hebrew original only; later settings and translations excluded. The country label reflects her Hebrew literary career before Israel’s statehood. The poem is troubled love rather than a straightforward celebration. The selection is the original-language text; an existing English translation is not required.
-English passage: Fresh English translation by ChatGPT; draft for editorial review. Complete poem,8 lines; shorter than requested because the work is short. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+English passage: Earlier English draft by ChatGPT (replaced); draft for editorial review. Complete poem,8 lines; shorter than requested because the work is short. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X89" s="13" t="inlineStr">
@@ -13351,20 +13375,20 @@
       </c>
       <c r="G90" s="13" t="inlineStr">
         <is>
-          <t>So noble and so honourable she appears,
-my lady, when she greets another,
-that every tongue falls silent, trembling,
+          <t>So gracious and so modest does she seem,
+my lady, when she greets anyone,
+that every tongue trembles and goes mute,
 and eyes do not dare to look at her.
-She goes her way, hearing herself praised,
-kindly, clothed in humility;
-she seems a being come
-from heaven to earth to show a miracle.
-So lovely does she appear to those who gaze
-that through their eyes she gives the heart a sweetness
-which none can understand who has not felt it.
-And from her face there seems to move
-a gentle spirit full of love,
-saying to the soul: Sigh.</t>
+She passes, hearing people praise her,
+kindly, dressed in humility,
+and seems to be a thing that came
+from heaven down to earth to show a wonder.
+She seems so pleasing to whoever looks at her
+that through the eyes she sends a sweetness to the heart
+which no one can understand who has not felt it;
+and from her lips there seems to come
+a gentle spirit full of love
+that keeps on saying to the soul: “Sigh.”</t>
         </is>
       </c>
       <c r="H90" s="13" t="inlineStr">
@@ -13437,7 +13461,8 @@
       <c r="W90" s="13" t="inlineStr">
         <is>
           <t>New English translation from the Italian; Rossetti's translation is not used.
-Fresh English translation by ChatGPT; draft for editorial review. Complete sonnet,14 lines; translated from Italian, not the linked historical English version. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+Earlier English draft by ChatGPT (replaced); draft for editorial review. Complete sonnet,14 lines; translated from Italian, not the linked historical English version. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X90" s="13" t="inlineStr">
@@ -13684,11 +13709,11 @@
       </c>
       <c r="G92" s="13" t="inlineStr">
         <is>
-          <t>Though I tried to hide it,
-it has shown itself in my face—
-this love of mine—
-until people ask me,
-Are you lost in thoughts of someone?</t>
+          <t>I hid it, and yet
+it has come into my face,
+this love of mine,
+so that people ask me,
+“Is something on your mind?”</t>
         </is>
       </c>
       <c r="H92" s="13" t="inlineStr">
@@ -13761,7 +13786,8 @@
       <c r="W92" s="13" t="inlineStr">
         <is>
           <t>New English translation from the Japanese; William Porter's 1909 translation is not used.
-Fresh English translation by ChatGPT; draft for editorial review. Complete waka,5 lines; original Japanese checked against the Ogura Hyakunin Isshu Cultural Foundation museum text. Fresh English rendering; short work is not padded.. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+Earlier English draft by ChatGPT (replaced); draft for editorial review. Complete waka,5 lines; original Japanese checked against the Ogura Hyakunin Isshu Cultural Foundation museum text. Fresh English rendering; short work is not padded.. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X92" s="13" t="inlineStr">
@@ -17290,20 +17316,20 @@
       </c>
       <c r="G117" s="13" t="inlineStr">
         <is>
-          <t>This afternoon, my love, as I spoke to you,
-seeing in your face and in your manner
-that words were failing to persuade you,
-I wished that you could see my heart.
-And Love, who came to aid my purpose,
-overcame what had seemed impossible:
-for, mingled with the tears my sorrow shed,
-my melted heart was flowing out.
+          <t>This evening, my love, as I spoke with you,
+since I could see from your face and what you did
+that my words were not convincing you,
+I wished that you could see my heart;
+and Love, who was helping my attempt,
+achieved what seemed impossible:
+for in the tears that grief was shedding
+my heart, undone, was flowing out.
 Enough of harshness now, my love, enough:
-let tyrannous jealousy torment you no more,
-nor base suspicion trouble your unrest
-with foolish shadows, with empty signs,
-for now, made liquid, you have seen and touched
-my heart dissolved between your hands.</t>
+let tyrant jealousy torment you no more,
+nor let base suspicion trouble your peace
+with foolish shadows and with empty signs,
+since you have seen and touched, as liquid,
+my heart, undone, between your hands.</t>
         </is>
       </c>
       <c r="H117" s="13" t="inlineStr">
@@ -17376,7 +17402,8 @@
       <c r="W117" s="13" t="inlineStr">
         <is>
           <t>Original-language poem only; modern translations and recordings are separate. Retain attribution and source/license links for copyrightable transcription material.
-English passage: Fresh English translation by ChatGPT; draft for editorial review. Complete sonnet,14 lines. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+English passage: Earlier English draft by ChatGPT (replaced); draft for editorial review. Complete sonnet,14 lines. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X117" s="13" t="inlineStr">
@@ -20174,16 +20201,16 @@
       <c r="G136" s="13" t="inlineStr">
         <is>
           <t>The last of the guests
-we saw to the gate;
-the lingering farewells
-were taken by the night wind.
-Tenfold desolate
+we walked to the gate;
+what was left of goodbye
+the night wind took.
+Ten times more empty
 lay garden and house,
 where sweet music
-had just intoxicated me.
+had made me drunk just now.
 It was only a party
 before the black night;
-she was only a guest—
+she was only a guest, —
 and now she is gone.</t>
         </is>
       </c>
@@ -20257,7 +20284,8 @@
       <c r="W136" s="13" t="inlineStr">
         <is>
           <t>Author died 1906. Original poem only; later musical settings excluded. Language is the historical literary Danish used by the Norwegian author. The selection is the original-language text; an existing English translation is not required.
-English passage: Fresh English translation by ChatGPT; draft for editorial review. Complete poem,12 lines. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+English passage: Earlier English draft by ChatGPT (replaced); draft for editorial review. Complete poem,12 lines. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X136" s="13" t="inlineStr">
@@ -21953,20 +21981,20 @@
       </c>
       <c r="G147" s="13" t="inlineStr">
         <is>
-          <t>Love is a fire that burns unseen;
-a wound that aches and is not felt;
-a discontented contentment;
-a pain that drives us wild without hurting.
-It is wanting nothing but to love;
-walking alone among the crowd;
-never content with being content;
-believing we gain by losing ourselves.
-It is choosing to remain a prisoner;
-serving the one who conquers the conqueror;
-keeping faith with the one who kills us.
+          <t>Love is a fire that burns without being seen;
+it is a wound that hurts and is not felt;
+it is a discontented happiness;
+it is a pain that maddens without pain;
+it is not wanting more than to want well;
+it is walking alone among people;
+it is never being content with being content;
+it is thinking you gain by losing yourself;
+it is being a prisoner by choice;
+it is serving the one who defeats the victor;
+it is keeping faith with the one who kills us.
 But how can its favour bring
-harmony to mortal hearts,
-when Love itself is so contrary to itself?</t>
+agreement into mortal hearts,
+when Love is so opposed to itself?</t>
         </is>
       </c>
       <c r="H147" s="13" t="inlineStr">
@@ -22039,7 +22067,8 @@
       <c r="W147" s="13" t="inlineStr">
         <is>
           <t>Historical Portuguese text. For any copyrightable transcription material, credit author and Wikisource contributors, link source/license, mark changes and observe ShareAlike. Modern translations are separate.
-English passage: Fresh English translation by ChatGPT; draft for editorial review. Complete sonnet,14 lines. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+English passage: Earlier English draft by ChatGPT (replaced); draft for editorial review. Complete sonnet,14 lines. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X147" s="13" t="inlineStr">
@@ -22272,18 +22301,18 @@
       </c>
       <c r="G149" s="13" t="inlineStr">
         <is>
-          <t>On my knees you will sit;
-we shall be utterly alone,
-while, trembling in your hair,
-linden blossoms fall.
-Lay your white brow, amid your golden hair,
-gently upon my arm,
-leaving your sweet lips
-to the mercy of my mouth.
-We shall dream a happy dream,
-while lonely springs sing to us,
-and the gentle beating
-of the wind.</t>
+          <t>You will sit upon my knees,
+we'll be alone, all on our own,
+and in your hair, all trembling,
+the lime-tree flowers will fall.
+Your white brow in your golden hair
+you'll lay down gently on my arm,
+leaving to my mouth as plunder
+those sweet lips of yours…
+We'll dream a happy dream,
+and lulling us with their song
+will be the lonely springs,
+the gentle beating of the wind;</t>
         </is>
       </c>
       <c r="H149" s="13" t="inlineStr">
@@ -22358,7 +22387,8 @@
       <c r="W149" s="13" t="inlineStr">
         <is>
           <t>Edition provenance is limited to the linked transcription. Credit author and Wikisource contributors; retain source/license, mark changes and observe ShareAlike where applicable. No translation included.
-English passage: Fresh English translation by ChatGPT; draft for editorial review. Lines9–20, three consecutive stanzas. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+English passage: Earlier English draft by ChatGPT (replaced); draft for editorial review. Lines9–20, three consecutive stanzas. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X149" s="13" t="inlineStr">
@@ -22430,14 +22460,14 @@
       </c>
       <c r="G150" s="13" t="inlineStr">
         <is>
-          <t>I loved you: perhaps love has not yet
-quite died away within my soul;
-but let it trouble you no longer;
-I do not wish to cause you any sadness.
-I loved you silently, without hope,
-tormented now by shyness, now by jealousy.
-I loved you so sincerely, so tenderly—
-God grant another may love you so.</t>
+          <t>I loved you; and perhaps that love has still
+not wholly burned out in my soul;
+but do not let it trouble you any more;
+I would not grieve you in any way.
+I loved you without a word, without hope,
+worn down now by shyness, now by jealousy;
+I loved you so truly and so tenderly
+as, God grant, you may be loved by another.</t>
         </is>
       </c>
       <c r="H150" s="13" t="inlineStr">
@@ -22512,7 +22542,8 @@
       <c r="W150" s="13" t="inlineStr">
         <is>
           <t>New English translation from the Russian; Ivan Panin's 1888 translation is not used.
-Fresh English translation by ChatGPT; draft for editorial review. Complete poem,8 lines; fresh translation from Russian, not a copy of an existing English version. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+Earlier English draft by ChatGPT (replaced); draft for editorial review. Complete poem,8 lines; fresh translation from Russian, not a copy of an existing English version. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X150" s="13" t="inlineStr">
@@ -24513,16 +24544,16 @@
       </c>
       <c r="G165" s="13" t="inlineStr">
         <is>
-          <t>My poem is a vessel for your name,
-for the name of the ruler of my heart, your name;
-in it, among my Slovenian brothers, I shall carry the sweet sound
-from west to east of your name.
-Upon the vessel, in golden letters, the glory will be read,
+          <t>My song is a vessel for your name,
+O lady of my heart, your name;
+in it I'll carry to my Slovene brothers the sweet sound
+from sunset to sunrise of your name;
+on the vessel, in letters of gold, people will read the glory,
 from nation to nation, of your name;
-from it a light will burn even when we are
-beyond Charon's ferry—the light of your name.
-More than Delia's, Corinna's, Cynthia's or Laura's,
-it would be a pity to forget your name.</t>
+from it a light will still be shining when we two are
+across Charon's ferry, the light of your name.
+More than Delia, Corinna, Cynthia or Laura,
+it would be a loss to forget your name.</t>
         </is>
       </c>
       <c r="H165" s="13" t="inlineStr">
@@ -24595,7 +24626,8 @@
       <c r="W165" s="13" t="inlineStr">
         <is>
           <t>Wikisource explicitly marks the original public domain in Slovenia under its life-plus-70 rule. Translate the Slovenian verses; modern punctuation or critical apparatus needs separate comparison. The selection is the original-language text; an existing English translation is not required.
-English passage: Fresh English translation by ChatGPT; draft for editorial review. Complete ghazal,10 lines; repeated phrase retained where English permits. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+English passage: Earlier English draft by ChatGPT (replaced); draft for editorial review. Complete ghazal,10 lines; repeated phrase retained where English permits. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X165" s="13" t="inlineStr">
@@ -25359,9 +25391,9 @@
       </c>
       <c r="G171" s="13" t="inlineStr">
         <is>
-          <t>What is poetry? you ask, fixing
-your blue eyes upon my own.
-What is poetry? And you ask me?
+          <t>“What is poetry?” you say, as you fix
+your blue eye on mine.
+What is poetry? And you are asking me?
 Poetry… is you.</t>
         </is>
       </c>
@@ -25437,7 +25469,8 @@
       <c r="W171" s="13" t="inlineStr">
         <is>
           <t>Original-language poem only. Modern translations and editorial material are separate.
-English passage: Fresh English translation by ChatGPT; draft for editorial review. Complete poem,4 lines; do not pad this short work to10–15 lines. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+English passage: Earlier English draft by ChatGPT (replaced); draft for editorial review. Complete poem,4 lines; do not pad this short work to10–15 lines. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X171" s="13" t="inlineStr">
@@ -25879,14 +25912,14 @@
       </c>
       <c r="G175" s="13" t="inlineStr">
         <is>
-          <t>I bought my love with money;
-no other love was mine to find.
-Sing sweetly, you rasping strings,
+          <t>I bought my love with money,
+for there was no other for me to have;
+sing sweetly, you jarring strings,
 sing sweetly of love all the same.
-That dream which never came true
-was beautiful to have as a dream;
-for one cast out of Eden,
-Eden is Eden all the same.</t>
+The dream that never came true
+was a lovely thing to have as a dream;
+for anyone cursed and cast out of Eden,
+Eden is still Eden.</t>
         </is>
       </c>
       <c r="H175" s="13" t="inlineStr">
@@ -25961,7 +25994,8 @@
       <c r="W175" s="13" t="inlineStr">
         <is>
           <t>Credit author and Wikisource contributors; retain source/license, mark changes and observe ShareAlike for copyrightable site material. Modern translations and musical settings are separate.
-English passage: Fresh English translation by ChatGPT; draft for editorial review. Complete poem,8 lines; shorter than requested because the work is short. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+English passage: Earlier English draft by ChatGPT (replaced); draft for editorial review. Complete poem,8 lines; shorter than requested because the work is short. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X175" s="13" t="inlineStr">
@@ -26037,18 +26071,18 @@
       </c>
       <c r="G176" s="13" t="inlineStr">
         <is>
-          <t>Two sails brighten
-the deep-blue bay!
-Two sails swell
-for a tranquil flight!
+          <t>Two sails lighting up
+the deep blue bay!
+Two sails filling
+for a peaceful run!
 As one, in the winds,
-arches and moves,
-the feelings of the other
-are stirred as well.
-If one longs to hurry,
-the other moves swiftly;
-if one wishes to rest,
-its companion rests too.</t>
+bellies and stirs,
+so the feeling
+of the other is moved.
+If one wants to hurry,
+the other goes fast;
+if one longs to rest,
+its partner rests too.</t>
         </is>
       </c>
       <c r="H176" s="13" t="inlineStr">
@@ -26123,7 +26157,8 @@
       <c r="W176" s="13" t="inlineStr">
         <is>
           <t>Meyer died 1898; applies to the 1882 German poem. The partnership reading is interpretive. Linked audio and modern translations have separate rights.
-English passage: Fresh English translation by ChatGPT; draft for editorial review. Complete poem,12 lines. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+English passage: Earlier English draft by ChatGPT (replaced); draft for editorial review. Complete poem,12 lines. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X176" s="13" t="inlineStr">
@@ -28041,18 +28076,18 @@
       </c>
       <c r="G190" s="13" t="inlineStr">
         <is>
-          <t>I would embrace you like ivy,
-so tightly, closely, hiding you from the world.
-I am not afraid of taking your life:
-you would be like a ruin covered in leaves.
-Ivy gives it life, embraces it,
-protects its bare wall from the weather;
-but the ruin, too, holds fast
-its companion, lest it fall to the ground.
-They are happy together—as we are—
+          <t>I would like to wrap my arms around you like ivy,
+so tight, so close, and shut you off from the world;
+I'm not afraid I'd take your life away,
+you'd be like a ruin covered in leaves, —
+ivy gives it life, it holds it close,
+it shields the bare wall from bad weather,
+but the ruin, too, holds on so steadily
+to its companion, so that it won't fall.
+They're happy together, like you and me, —
 and when the time comes for the ruin to crumble,
-let it bury the ivy beneath it.
-What use has ivy for solitude?</t>
+let it hide the ivy underneath itself.
+What good would ivy be on its own?</t>
         </is>
       </c>
       <c r="H190" s="13" t="inlineStr">
@@ -28127,7 +28162,8 @@
       <c r="W190" s="13" t="inlineStr">
         <is>
           <t>Original-language poem only; modern translations and recordings are separate. Retain attribution and source/license links for copyrightable transcription material.
-English passage: Fresh English translation by ChatGPT; draft for editorial review. Opening12 lines of16; final stanza omitted. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+English passage: Earlier English draft by ChatGPT (replaced); draft for editorial review. Opening12 lines of16; final stanza omitted. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X190" s="13" t="inlineStr">
@@ -28651,20 +28687,20 @@
       </c>
       <c r="G194" s="13" t="inlineStr">
         <is>
-          <t>If life is love, then let it be blessed!
-I want more life in which to love! Today I feel
-that a thousand years of thought are worth less
-than one blue minute of feeling.
-My heart was dying, slowly and sadly…
-Today it opens into light like a flower of the sun;
-life surges like a violent sea
-where the hand of love strikes!
-Today my melancholy, sad and cold,
-its wings broken, departed into the night;
-like an old stain of sorrow
-it dissolves in the distant darkness…
+          <t>If life is love, then blessed be it!
+I want more life so I can love! Today I feel
+that a thousand years of thinking are not worth
+one blue minute of feeling.
+My heart was dying, sad and slow…
+Today it opens in light like a flower of Phoebus;
+life wells up like a violent sea
+where love's hand strikes!
+Today, sad and cold, my melancholy
+left for the night with broken wings;
+like an old stain of grief
+it fades away in the distant shadow…
 My whole life sings, kisses, laughs!
-My whole life is a mouth in bloom!</t>
+My whole life is a mouth in flower!</t>
         </is>
       </c>
       <c r="H194" s="13" t="inlineStr">
@@ -28739,7 +28775,8 @@
       <c r="W194" s="13" t="inlineStr">
         <is>
           <t>Original-language poem only; modern translations and recordings are separate. Retain attribution and source/license links for copyrightable transcription material.
-English passage: Fresh English translation by ChatGPT; draft for editorial review. Complete sonnet,14 lines. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.</t>
+English passage: Earlier English draft by ChatGPT (replaced); draft for editorial review. Complete sonnet,14 lines. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
         </is>
       </c>
       <c r="X194" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Anthology review: Song of Songs and Hafez retranslated after phrase check
One Song of Songs line matched the NIV word for word; both passages are
now fresh translations that avoid published wording.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -11614,17 +11614,17 @@
       </c>
       <c r="G80" s="13" t="inlineStr">
         <is>
-          <t>You have stolen my heart, my sister, my bride;
-You have stolen my heart with one glance of your eyes,
-With one bead of your necklace.
-How beautiful is your love, my sister, my bride!
-How much better is your love than wine,
-And the scent of your perfumes than any spice!
-Your lips drip honey, my bride;
-Honey and milk are under your tongue,
-And the scent of your garments is like the scent of Lebanon.
-A locked garden is my sister, my bride,
-A locked spring, a sealed fountain.</t>
+          <t>You have taken my heart, my sister, my bride;
+you have taken my heart with one of your eyes,
+with one link of the chain about your neck.
+How fair are your caresses, my sister, my bride!
+How much finer your caresses than wine,
+and the fragrance of your oils than all the spices!
+Your lips let fall drops of honeycomb, my bride;
+honey and milk lie beneath your tongue,
+and the fragrance of your clothes is like the fragrance of Lebanon.
+A garden barred is my sister, my bride,
+a spring barred, a sealed fountain.</t>
         </is>
       </c>
       <c r="H80" s="13" t="inlineStr">
@@ -11697,7 +11697,8 @@
       <c r="W80" s="13" t="inlineStr">
         <is>
           <t>Country association is Vatican reception of this passage, not authorship in the Holy See. Translate the ancient Hebrew, excluding modern commentary, vocalisation apparatus and papal-address translations. The page offers a consonantal text option. The selection is the original-language text; an existing English translation is not required.
-Passage update (29 October 2026): Song of Songs 4:9–12, 11 lines. Consonantal Hebrew (vowel points and cantillation removed, as the spreadsheet asks); where the text has a written/read variant, the written form באחד is kept. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
+Passage update (29 October 2026): Song of Songs 4:9–12, 11 lines. Consonantal Hebrew (vowel points and cantillation removed, as the spreadsheet asks); where the text has a written/read variant, the written form באחד is kept. Fresh English translation by Claude (Anthropic AI); draft for editorial review.
+Revision (30 October 2026): retranslated literally from the Hebrew after a phrase check found one line identical to the NIV (in copyright); wording also kept clear of the King James Version (Crown copyright in the UK).</t>
         </is>
       </c>
       <c r="X80" s="13" t="inlineStr">
@@ -12719,24 +12720,24 @@
       </c>
       <c r="G86" s="13" t="inlineStr">
         <is>
-          <t>If that Turk of Shiraz would take my heart in hand,
-For that dark mole I would give away Samarkand and Bukhara.
-Pour, cupbearer, the wine that remains, for in paradise you will not find
-The banks of the Ruknabad stream or the rose walks of Musalla.
-Alas! these saucy, sweet-working, city-unsettling beauties
-Have carried off patience from my heart as Turks carry off a plundered feast.
-My beloved’s beauty has no need of our imperfect love:
-What need has a lovely face of paint and colour, mole and line?
-From that ever-growing beauty that Joseph had, I came to know
-That love brings Zuleikha out from behind the veil of chastity.
-Whether you curse me or revile me, I will bless you:
-A bitter answer suits a ruby lip that sheds sugar.
-Listen to advice, my soul, for fortunate young people
-Hold the counsel of a wise old man dearer than their lives.
-Speak of the minstrel and wine, and seek the world’s secret less,
-For no one has solved, nor by wisdom will solve, this riddle.
-You have made a ghazal and strung pearls; come, sing it sweetly, Hafez,
-For over your verse the heavens scatter the necklace of the Pleiades.</t>
+          <t>If that Turk of Shiraz would only take my heart in hand,
+for the dark mole on that cheek I'd give up Samarkand and Bukhara.
+Bring the last of the wine, cupbearer: in paradise you won't find
+the banks of the Ruknabad or the flowered paths of Musalla.
+Ah, these playful gypsy girls, so charming, such trouble to the town,
+have stripped the patience from my heart as Turks strip a table of its spoils.
+My love is incomplete, but my beloved's beauty does not need it:
+a lovely face has no use for powder, colour, beauty-spot or pencil.
+From that beauty of Joseph's, growing day by day, I learned
+how love draws Zulaikha out from behind the curtain of virtue.
+Abuse me if you like, curse me: I'll pray for you all the same;
+a bitter answer becomes a ruby lip that rains down sugar.
+Take some advice, my dear: young people blessed by fortune
+love the counsel of a wise old man more than life itself.
+Talk of minstrels and wine, and don't dig into the world's secret,
+for no one has solved this riddle by wisdom, and no one will.
+You've made your ghazal and pierced your pearls; come, Hafez, sing it well,
+for the sky scatters the string of the Pleiades over your verse.</t>
         </is>
       </c>
       <c r="H86" s="13" t="inlineStr">
@@ -12809,7 +12810,8 @@
       <c r="W86" s="13" t="inlineStr">
         <is>
           <t>New English translation from the Persian; Gertrude Bell's 1897 translation is not used. Modern translations are separate. Mystical readings are possible.
-Passage update (29 October 2026): Complete ghazal, 9 couplets (18 half-lines). Persian text from Ganjoor (ghazal 3), with Ganjoor’s added short-vowel marks removed; the letters are unchanged. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
+Passage update (29 October 2026): Complete ghazal, 9 couplets (18 half-lines). Persian text from Ganjoor (ghazal 3), with Ganjoor’s added short-vowel marks removed; the letters are unchanged. Fresh English translation by Claude (Anthropic AI); draft for editorial review.
+Revision (30 October 2026): retranslated from the Persian for the anthology review so that no line follows the wording of an earlier English version.</t>
         </is>
       </c>
       <c r="X86" s="13" t="inlineStr">

</xml_diff>

<commit_message>
Anthology review batch 3; approximate years for every poem
- Palestine: four ʿatāba love quatrains (Dalman, 1901).
- Somalia: two love songs (Reinisch, 1900).
- Jordan: al-Walid II's poem to Salma (Kitab al-Aghani).
- Oman: love prelude from al-Nabhani's diwan (printed 1965).
- Paraguay: back in Poems to read with a fresh translation from the
  Guaraní only.
- Every poem to read now shows at least an approximate year.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -950,7 +950,11 @@
           <t>Women</t>
         </is>
       </c>
-      <c r="M7" s="14" t="n"/>
+      <c r="M7" s="14" t="inlineStr">
+        <is>
+          <t>c. 950</t>
+        </is>
+      </c>
       <c r="N7" s="13" t="inlineStr">
         <is>
           <t>Persian / Dari</t>
@@ -2027,7 +2031,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M14" s="14" t="n"/>
+      <c r="M14" s="14" t="inlineStr">
+        <is>
+          <t>c. 1760</t>
+        </is>
+      </c>
       <c r="N14" s="13" t="inlineStr">
         <is>
           <t>Armenian (Tbilisi dialect)</t>
@@ -2515,7 +2523,11 @@
           <t>Women</t>
         </is>
       </c>
-      <c r="M17" s="14" t="n"/>
+      <c r="M17" s="14" t="inlineStr">
+        <is>
+          <t>c. 1870</t>
+        </is>
+      </c>
       <c r="N17" s="13" t="inlineStr">
         <is>
           <t>Azerbaijani</t>
@@ -2792,7 +2804,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M19" s="14" t="n"/>
+      <c r="M19" s="14" t="inlineStr">
+        <is>
+          <t>c. 1600</t>
+        </is>
+      </c>
       <c r="N19" s="13" t="inlineStr">
         <is>
           <t>Arabic</t>
@@ -2960,7 +2976,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M20" s="14" t="n"/>
+      <c r="M20" s="14" t="inlineStr">
+        <is>
+          <t>c. 1650</t>
+        </is>
+      </c>
       <c r="N20" s="13" t="inlineStr">
         <is>
           <t>Bengali</t>
@@ -5086,7 +5106,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M35" s="14" t="n"/>
+      <c r="M35" s="14" t="inlineStr">
+        <is>
+          <t>c. 1920</t>
+        </is>
+      </c>
       <c r="N35" s="13" t="inlineStr">
         <is>
           <t>Cape Verdean Creole</t>
@@ -6093,7 +6117,11 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="M42" s="14" t="n"/>
+      <c r="M42" s="14" t="inlineStr">
+        <is>
+          <t>c. 600 BCE</t>
+        </is>
+      </c>
       <c r="N42" s="13" t="inlineStr">
         <is>
           <t>Classical Chinese</t>
@@ -6263,7 +6291,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M43" s="14" t="n"/>
+      <c r="M43" s="14" t="inlineStr">
+        <is>
+          <t>c. 1905</t>
+        </is>
+      </c>
       <c r="N43" s="13" t="inlineStr">
         <is>
           <t>Spanish</t>
@@ -7142,7 +7174,11 @@
           <t>Women</t>
         </is>
       </c>
-      <c r="M49" s="14" t="n"/>
+      <c r="M49" s="14" t="inlineStr">
+        <is>
+          <t>c. 1850</t>
+        </is>
+      </c>
       <c r="N49" s="13" t="inlineStr">
         <is>
           <t>Spanish</t>
@@ -7295,7 +7331,11 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="M50" s="14" t="n"/>
+      <c r="M50" s="14" t="inlineStr">
+        <is>
+          <t>c. 1560</t>
+        </is>
+      </c>
       <c r="N50" s="13" t="inlineStr">
         <is>
           <t>Cypriot Greek</t>
@@ -9025,7 +9065,11 @@
           <t>Women</t>
         </is>
       </c>
-      <c r="M62" s="14" t="n"/>
+      <c r="M62" s="14" t="inlineStr">
+        <is>
+          <t>c. 1866</t>
+        </is>
+      </c>
       <c r="N62" s="13" t="inlineStr">
         <is>
           <t>Estonian</t>
@@ -10143,7 +10187,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M70" s="14" t="n"/>
+      <c r="M70" s="14" t="inlineStr">
+        <is>
+          <t>c. 1200</t>
+        </is>
+      </c>
       <c r="N70" s="13" t="inlineStr">
         <is>
           <t>Georgian</t>
@@ -11652,7 +11700,11 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="M80" s="14" t="n"/>
+      <c r="M80" s="14" t="inlineStr">
+        <is>
+          <t>c. 500 BCE</t>
+        </is>
+      </c>
       <c r="N80" s="13" t="inlineStr">
         <is>
           <t>Hebrew</t>
@@ -11830,7 +11882,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M81" s="14" t="n"/>
+      <c r="M81" s="14" t="inlineStr">
+        <is>
+          <t>c. 1900</t>
+        </is>
+      </c>
       <c r="N81" s="13" t="inlineStr">
         <is>
           <t>Spanish</t>
@@ -12206,7 +12262,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M83" s="14" t="n"/>
+      <c r="M83" s="14" t="inlineStr">
+        <is>
+          <t>c. 1845</t>
+        </is>
+      </c>
       <c r="N83" s="13" t="inlineStr">
         <is>
           <t>Icelandic</t>
@@ -12765,7 +12825,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M86" s="14" t="n"/>
+      <c r="M86" s="14" t="inlineStr">
+        <is>
+          <t>c. 1370</t>
+        </is>
+      </c>
       <c r="N86" s="13" t="inlineStr">
         <is>
           <t>Persian</t>
@@ -12927,7 +12991,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M87" s="14" t="n"/>
+      <c r="M87" s="14" t="inlineStr">
+        <is>
+          <t>c. 1920</t>
+        </is>
+      </c>
       <c r="N87" s="13" t="inlineStr">
         <is>
           <t>Arabic</t>
@@ -13418,7 +13486,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M90" s="14" t="n"/>
+      <c r="M90" s="14" t="inlineStr">
+        <is>
+          <t>c. 1293</t>
+        </is>
+      </c>
       <c r="N90" s="13" t="inlineStr">
         <is>
           <t>Italian</t>
@@ -13743,7 +13815,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M92" s="14" t="n"/>
+      <c r="M92" s="14" t="inlineStr">
+        <is>
+          <t>960</t>
+        </is>
+      </c>
       <c r="N92" s="13" t="inlineStr">
         <is>
           <t>Japanese</t>
@@ -13852,57 +13928,49 @@
       </c>
       <c r="D93" s="13" t="inlineStr">
         <is>
-          <t>ظننتني جزت عن طرد الهوى فإذا (incipit)</t>
+          <t>عتبت سلمى علينا سفاها</t>
         </is>
       </c>
       <c r="E93" s="13" t="inlineStr">
         <is>
-          <t>I thought I had passed beyond pursuing passion, but then… (first line)</t>
+          <t>Salma reproached me</t>
         </is>
       </c>
       <c r="F93" s="13" t="inlineStr">
         <is>
-          <t>ظننتني جزت عن طرد الهوى فإذا
-حسابه لم يزل في دفتري جاري
-وزند وجدي بربات الحجال على
-عهدي به كعشيات الصبا واري
-والأربعون التي لاحت طلائعها
-في لمتي ريحها استخذى لأعصاري
-ظننتني جزت عن طرد الهوى فإذا
-موضوعه لم يزل موضوع أسماري
-وما توهمته زهداً ورحت به
-أعلل النفس غير الواقع الجاري
-شتان بين شعوري في حقيقته
-وبين رجعك يا أصداء أفكاري
-فليتق اللّه من ظن الهيام بهم
-غياً فما بالهوى العذري من عار
-وما يضر أخا الأردن كسوته
-جديدها أن يحل يوماً لاطماري</t>
+          <t>عَتَبَت سَلمى عَلَينا سَفاها
+أَن سَبَبتُ اليَومَ فيها أَباها
+كانَ حَقُّ العَتبِ يا قَومُ مِنّي
+لَيسَ مِنها كانَ قَلبي فِداها
+فَلَئِن كُنتُ أَرَدتُ بِقَلبي
+لِأَبي سَلمى خِلافَ هَواها
+فَثَكِلتُ اليَومَ سَلمى فَسَلمى
+مَلَأَت أَرضي مَعاً وَسَماها
+غَيرَ أَنّي لا أَظُنُّ عَدُوّاً
+قَد أَتاها كاشِحاً بِأَذاها
+فَلَها العُتبى لَدَينا وَقَلَّت
+أَبَداً حَتّى أَنالَ رِضاها</t>
         </is>
       </c>
       <c r="G93" s="13" t="inlineStr">
         <is>
-          <t>I thought I had moved past the chase of passion, but lo,
-Its account is still running in my ledger;
-And the flint of my longing for the veiled beauties,
-As I knew it in the evenings of youth, still strikes fire;
-And the forties, whose first signs have appeared
-In my locks: their wind has bowed before my whirlwinds.
-I thought I had moved past the chase of passion, but lo,
-It is still the subject of my night-time talk.
-What I imagined was renunciation, and went about
-Consoling my soul with, was not what was truly happening.
-How far apart are my feeling as it truly is
-And your answer, O echoes of my thoughts!
-Let whoever thinks it folly to be lovesick for them
-Fear God: there is no shame in chaste love.
-And what harm is it to a son of Jordan if his clothes,
-The new ones, should one day turn to rags?</t>
+          <t>Salma reproached me, rashly,
+because today, over her, I insulted her father.
+By rights, my friends, the reproach should be mine,
+not hers; and still my heart would be her ransom.
+If ever in my heart I wished
+Salma's father anything against her will,
+then may I lose Salma this very day: Salma,
+who fills my earth and my sky together.
+Still, I cannot believe that some enemy
+has gone to her in spite, to do her harm;
+so she shall have my apology, though it is little,
+for ever, until I win her favour.</t>
         </is>
       </c>
       <c r="H93" s="13" t="inlineStr">
         <is>
-          <t>Mustafa Wahbi al-Tall (Arar), 1899–1949; some catalogues give 1897</t>
+          <t>al-Walid ibn Yazid (al-Walid II)</t>
         </is>
       </c>
       <c r="I93" s="13" t="inlineStr">
@@ -13925,8 +13993,10 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M93" s="14" t="n">
-        <v>1949</v>
+      <c r="M93" s="14" t="inlineStr">
+        <is>
+          <t>c. 740</t>
+        </is>
       </c>
       <c r="N93" s="13" t="inlineStr">
         <is>
@@ -13936,59 +14006,53 @@
       <c r="O93" s="13" t="n"/>
       <c r="P93" s="13" t="inlineStr">
         <is>
-          <t>Poetry</t>
+          <t>Poem (6 couplets), sung at court</t>
         </is>
       </c>
       <c r="Q93" s="13" t="inlineStr">
         <is>
-          <t>Man author</t>
+          <t>al-Walid II (c. 706–744)</t>
         </is>
       </c>
       <c r="R93" s="13" t="inlineStr">
         <is>
-          <t>Composed before the author’s death in 1949; exact composition date not established</t>
+          <t>c. 735–744</t>
         </is>
       </c>
       <c r="S93" s="13" t="inlineStr">
         <is>
-          <t>Historical Arabic poem; full eight-bayt text in Abu Dhabi’s Poetry Encyclopedia</t>
+          <t>Kitab al-Aghani (first printed Bulaq, 1868), vol. 7</t>
         </is>
       </c>
       <c r="T93" s="13" t="inlineStr">
         <is>
-          <t>The speaker discovers that advancing age has not extinguished his passion and defends romantic love against the charge that it is shameful.</t>
+          <t>Salma is angry because the poet has insulted her father; he swears that he meant her no harm, that she fills his earth and sky, and that he will keep apologising until she forgives him.</t>
         </is>
       </c>
       <c r="U93" s="13" t="inlineStr">
         <is>
-          <t>Abu Dhabi Department of Culture and Tourism, poem 66871, eight bayts. Shoman Foundation’s scholarly volume corroborates 1899–1949; Birzeit holds the historical 1954 collection Ashiyyat Wadi al-Yabis.</t>
-        </is>
-      </c>
-      <c r="V93" s="13" t="inlineStr">
-        <is>
-          <t>Eight-bayt poem; seventh bayt defends chaste romantic passion</t>
-        </is>
-      </c>
+          <t>Abu al-Faraj al-Isfahani, Kitab al-Aghani, section on al-Walid ibn Yazid (vol. 7), where the singer Abu Kamil set it to music; text from aldiwan.net, checked against the Aghani.</t>
+        </is>
+      </c>
+      <c r="V93" s="13" t="n"/>
       <c r="W93" s="13" t="inlineStr">
         <is>
-          <t>Identifier is the original incipit. Year 1949 is an upper bound. Birth-year disagreement is explicit. Reuse the author’s historical Arabic verses, excluding later commentary and translations; first-publication particulars for this individual poem have not been established.
-Passage update (29 October 2026): Complete poem, 8 couplets (16 half-lines), as printed in the Abu Dhabi Poetry Encyclopedia; the site’s decorative letter-stretching (tatweel) is removed. Fresh English translation by Claude (Anthropic AI); draft for editorial review.
-Moved to Poems to explore (30 October 2026) for the anthology review. Jordan: the poem's first publication was in a 1954 collection, five years after the poet's death; its US status depends on Jordan's 1996 copyright term.</t>
+          <t>Work changed (30 October 2026): Mustafa Wahbi al-Tall's poem, first published posthumously in 1954, is replaced by a love poem by the caliph-poet who lived in the desert palaces of the Balqa, in today's Jordan. Complete poem, 6 couplets. Fresh English translation by Claude (Anthropic AI) made directly from the original; draft for editorial review.</t>
         </is>
       </c>
       <c r="X93" s="13" t="inlineStr">
         <is>
-          <t>Historical original composition; author died 1949, beyond the standard life-plus-70 term. Reuse the underlying historical original only, excluding modern translations, editorial matter, images, adaptations and recordings. Publication history and territorial exceptions should be checked for the edition used.</t>
+          <t>Anthology review (30 October 2026): Umayyad poem preserved in Kitab al-Aghani, printed since 1868: public domain everywhere.</t>
         </is>
       </c>
       <c r="Y93" s="13" t="inlineStr">
         <is>
-          <t>Work-specific text, date and provenance sources checked29October2026.</t>
+          <t>aldiwan.net: عتبت سلمى علينا سفاها; Kitab al-Aghani vol. 7</t>
         </is>
       </c>
       <c r="Z93" s="11" t="inlineStr">
         <is>
-          <t>Read the text</t>
+          <t>Read the whole work</t>
         </is>
       </c>
       <c r="AA93" s="11" t="inlineStr">
@@ -14007,7 +14071,11 @@
         </is>
       </c>
       <c r="AD93" s="11" t="n"/>
-      <c r="AE93" s="11" t="n"/>
+      <c r="AE93" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: Read the text</t>
+        </is>
+      </c>
     </row>
     <row r="94" ht="91.5" customHeight="1" s="17">
       <c r="A94" s="7" t="inlineStr">
@@ -14501,7 +14569,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M97" s="14" t="n"/>
+      <c r="M97" s="14" t="inlineStr">
+        <is>
+          <t>c. 1890</t>
+        </is>
+      </c>
       <c r="N97" s="13" t="inlineStr">
         <is>
           <t>Arabic</t>
@@ -14952,7 +15024,11 @@
           <t>Women</t>
         </is>
       </c>
-      <c r="M100" s="14" t="n"/>
+      <c r="M100" s="14" t="inlineStr">
+        <is>
+          <t>c. 1900</t>
+        </is>
+      </c>
       <c r="N100" s="13" t="inlineStr">
         <is>
           <t>Latvian</t>
@@ -15562,7 +15638,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M104" s="14" t="n"/>
+      <c r="M104" s="14" t="inlineStr">
+        <is>
+          <t>c. 1890</t>
+        </is>
+      </c>
       <c r="N104" s="13" t="inlineStr">
         <is>
           <t>Arabic</t>
@@ -17359,7 +17439,11 @@
           <t>Women</t>
         </is>
       </c>
-      <c r="M117" s="14" t="n"/>
+      <c r="M117" s="14" t="inlineStr">
+        <is>
+          <t>c. 1680</t>
+        </is>
+      </c>
       <c r="N117" s="13" t="inlineStr">
         <is>
           <t>Spanish</t>
@@ -17975,7 +18059,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M121" s="14" t="n"/>
+      <c r="M121" s="14" t="inlineStr">
+        <is>
+          <t>c. 1840</t>
+        </is>
+      </c>
       <c r="N121" s="13" t="inlineStr">
         <is>
           <t>Mongolian</t>
@@ -18339,7 +18427,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M123" s="14" t="n"/>
+      <c r="M123" s="14" t="inlineStr">
+        <is>
+          <t>c. 1700</t>
+        </is>
+      </c>
       <c r="N123" s="13" t="inlineStr">
         <is>
           <t>Arabic</t>
@@ -19035,7 +19127,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M128" s="14" t="n"/>
+      <c r="M128" s="14" t="inlineStr">
+        <is>
+          <t>c. 1890</t>
+        </is>
+      </c>
       <c r="N128" s="13" t="inlineStr">
         <is>
           <t>Nepali</t>
@@ -19909,7 +20005,11 @@
           <t>Women</t>
         </is>
       </c>
-      <c r="M134" s="14" t="n"/>
+      <c r="M134" s="14" t="inlineStr">
+        <is>
+          <t>c. 1530</t>
+        </is>
+      </c>
       <c r="N134" s="13" t="inlineStr">
         <is>
           <t>Korean (historical Hangul and Hanja)</t>
@@ -20076,7 +20176,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M135" s="14" t="n"/>
+      <c r="M135" s="14" t="inlineStr">
+        <is>
+          <t>c. 1860</t>
+        </is>
+      </c>
       <c r="N135" s="13" t="inlineStr">
         <is>
           <t>Macedonian (historical dialectal text)</t>
@@ -20241,7 +20345,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M136" s="14" t="n"/>
+      <c r="M136" s="14" t="inlineStr">
+        <is>
+          <t>c. 1870</t>
+        </is>
+      </c>
       <c r="N136" s="13" t="inlineStr">
         <is>
           <t>Norwegian literary Danish (historical original)</t>
@@ -20341,61 +20449,53 @@
       </c>
       <c r="D137" s="13" t="inlineStr">
         <is>
-          <t>يا من هواه أعزه وأذلني / يا باخلاً بالوصل (Yā man hawāhu aʿazzahu wa-adhallanī)</t>
+          <t>أمرتبع أم أنت ليس بمنزل</t>
         </is>
       </c>
       <c r="E137" s="13" t="inlineStr">
         <is>
-          <t>O you whose love has exalted you and humbled me / O you who are miserly with union (first-line identifiers)</t>
+          <t>Are you a spring camp, or no dwelling at all?</t>
         </is>
       </c>
       <c r="F137" s="13" t="inlineStr">
         <is>
-          <t>يا مَنْ هواه أعزّه وأذلّني
-كيف السبيلُ إلى وصالِكَ؟ دُلّني
-وتركتني حيرانَ صبّاً هائمًا
-أرعى النجوم وأنت في نومٍ هني
-عاهدتني أن لا تميلَ عن الهوى
-وحلفتَ لي يا غصنُ أن لا تنثني
-هبَّ النسيم ومال غصنٌ مثلُه
-أين الزمانُ؟ وأين ما عاهدتني؟
-جاد الزمان وأنتَ ما واصلتني
-يا باخلاً بالوصل أنتَ قتلتني
-واصلتَني حتى ملكتَ حُشاشتي
-ورجَعتَ من بعد الوصال هجرتني
-فلأقعدنَّ على الطريق فأشتكي
-في زيِّ مظلومٍ وأنت ظلمتَني
-ولأشكينَّكَ عند سلطان الهوى
-لِيُعذبنَّك مثلَ ما عذَّبتني
-ولأدعوَنَّ عليك في جُنْح الدجى
-فعساك تُبلى مثل ما أبليتني</t>
+          <t>خليلي عوجا نمنحِ الربعَ ساعةً
+تحيَّةَ جازٍ بالوفا غيرِ مُؤتلِ
+ولسنا نحيَّي الدار حُبّاً لِربَعها
+ولكنه حُبٌّ لكالأدم خُذَّلِ
+شَناغيف هيفٍ ناعماتٍ نواهدٍ
+أماليدَ غيدٍ من عرانين نهشَلِ
+وفرْعاءَ غرَّاءِ المجرَّد طَفَلةٍ
+من الخفرات الغُنِّ شمّا المقَّبلِ
+لها مقلتا مَذعورةٍ أم جوذرٍ
+وسالفتا براقَةِ الجيد مُغزِلِ
+وتستر مَتْنَيها بأسحمَ فاحمٍ
+كثيفٍ أثيثِ النّبت جعد المرجّلِ
+وتَبسمُ عن غُرٍّ كأن وميضها
+تلألؤُ برقٍ في حبيٍّ مكلَّلِ</t>
         </is>
       </c>
       <c r="G137" s="13" t="inlineStr">
         <is>
-          <t>O you whose love has raised you up and brought me low,
-how can I reach union with you? Show me the way.
-You have left me bewildered, lovesick, wandering,
-watching the stars while you sleep sweetly.
-You promised me you would not turn from love,
-and swore to me, O willow branch, that you would not bend.
-The breeze blew, and a branch like you bent with it:
-where is that time now? Where is what you promised me?
-Time has been generous, yet you have not come to me;
-O you who are miserly with union, you have killed me.
-You came to me until you owned the last of my soul,
-then, after our union, you turned and left me.
-So I will sit by the roadside and complain,
-dressed as one wronged, for you have wronged me;
-and I will accuse you before the sultan of love,
-so that he punishes you as you have tormented me;
-and I will call down a curse on you in the depth of night,
-so that you may be worn down as you have worn me down.</t>
+          <t>My two friends, turn aside; let us give this camp an hour,
+the greeting of one who repays in full and never falls short.
+We do not greet the dwelling out of love for its ground,
+but for love of women like white gazelles that linger behind the herd,
+tall and slender, soft and full-breasted,
+supple and graceful, from the noblest of Nahshal;
+and for one with long hair, gleaming where her skin is bare, tender,
+one of the modest, soft-voiced girls, her mouth sweet to kiss;
+she has the eyes of a startled doe with her fawn,
+and the neck of a gazelle with a gleaming throat;
+she hides her back beneath hair black as charcoal,
+thick and abundant, curling where it is combed;
+and she smiles, showing white teeth whose gleam
+is like lightning flashing in a heaped-up cloud.</t>
         </is>
       </c>
       <c r="H137" s="13" t="inlineStr">
         <is>
-          <t>Saʿid ibn Ahmad al-Busaʿidi (سعيد بن أحمد البوسعيدي)</t>
+          <t>Sulayman ibn Sulayman al-Nabhani</t>
         </is>
       </c>
       <c r="I137" s="13" t="inlineStr">
@@ -20418,7 +20518,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M137" s="14" t="n"/>
+      <c r="M137" s="14" t="inlineStr">
+        <is>
+          <t>c. 1500</t>
+        </is>
+      </c>
       <c r="N137" s="13" t="inlineStr">
         <is>
           <t>Arabic</t>
@@ -20427,59 +20531,57 @@
       <c r="O137" s="13" t="n"/>
       <c r="P137" s="13" t="inlineStr">
         <is>
-          <t>Lyric poem</t>
+          <t>Qasida, love prelude (couplets 8–14 of 21)</t>
         </is>
       </c>
       <c r="Q137" s="13" t="inlineStr">
         <is>
-          <t>Man author</t>
+          <t>Sulayman al-Nabhani (Nabhani ruler of Oman)</t>
         </is>
       </c>
       <c r="R137" s="13" t="inlineStr">
         <is>
-          <t>Late 18th–early 19th century; exact composition date unknown</t>
+          <t>Late 15th–early 16th century</t>
         </is>
       </c>
       <c r="S137" s="13" t="inlineStr">
         <is>
-          <t>Linked digital transcription/facsimile; precise edition date not established</t>
+          <t>1965, Diwan al-Sultan Sulayman ibn Sulayman al-Nabhani (Damascus), ed. Izz al-Din al-Tanukhi</t>
         </is>
       </c>
       <c r="T137" s="13" t="inlineStr">
         <is>
-          <t>An abandoned lover asks how to reach the beloved, recalling promises, union and separation. Emotional complaint rather than a happy love poem.</t>
+          <t>Stopping at an abandoned camp, the poet greets it not for love of the place but for the women who lived there, and above all for one with long black hair, the eyes of a startled doe and a smile like lightning in a cloud.</t>
         </is>
       </c>
       <c r="U137" s="13" t="inlineStr">
         <is>
-          <t>Al-Babtain Central Library for Arabic Poetry, September 2020 selection, original Arabic and Omani biography; cites historical collections.</t>
+          <t>Diwan of Sulayman al-Nabhani, first printed Damascus 1965 (ed. al-Tanukhi; reprinted Muscat 1985); text from aldiwan.net.</t>
         </is>
       </c>
       <c r="V137" s="13" t="inlineStr">
         <is>
-          <t>Al-Babtain Library page, poem headed يا باخلاً بالوصل</t>
+          <t>Couplets 8–14 of 21</t>
         </is>
       </c>
       <c r="W137" s="13" t="inlineStr">
         <is>
-          <t>Text varies in stanza/line count across modern reproductions. Biography gives differing death traditions (1803 or 1810); both are well outside copyright term. Modern song settings and editorial prose excluded.
-Passage update (29 October 2026): Complete poem, 9 couplets (18 half-lines), as printed by the Al-Babtain Library. Fresh English translation by Claude (Anthropic AI); draft for editorial review.
-Moved to Poems to explore (30 October 2026) for the anthology review. Oman: no printing of this poem before 1989 could be established.</t>
+          <t>Work changed (30 October 2026): Saʿid al-Busaʿidi's poem, for which no printing before 1989 could be established, is replaced by the love prelude of a qasida by Oman's best-known classical poet. Couplets 8–14 of 21. Fresh English translation by Claude (Anthropic AI) made directly from the original; draft for editorial review.</t>
         </is>
       </c>
       <c r="X137" s="13" t="inlineStr">
         <is>
-          <t>Original text: standard life-plus-70 term expired; author died 1803 or 1810. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.</t>
+          <t>Anthology review (30 October 2026): the poet died in the early 16th century and the diwan was printed in 1965, long before 1989: public domain everywhere.</t>
         </is>
       </c>
       <c r="Y137" s="13" t="inlineStr">
         <is>
-          <t>Linked full original text / credited edition</t>
+          <t>aldiwan.net: أمرتبع أم أنت ليس بمنزل</t>
         </is>
       </c>
       <c r="Z137" s="11" t="inlineStr">
         <is>
-          <t>Read the text</t>
+          <t>Read the whole work</t>
         </is>
       </c>
       <c r="AA137" s="11" t="inlineStr">
@@ -20498,7 +20600,11 @@
         </is>
       </c>
       <c r="AD137" s="11" t="n"/>
-      <c r="AE137" s="11" t="n"/>
+      <c r="AE137" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: Read the text</t>
+        </is>
+      </c>
     </row>
     <row r="138" ht="108" customHeight="1" s="17">
       <c r="A138" s="7" t="inlineStr">
@@ -20577,7 +20683,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M138" s="14" t="n"/>
+      <c r="M138" s="14" t="inlineStr">
+        <is>
+          <t>c. 1740</t>
+        </is>
+      </c>
       <c r="N138" s="13" t="inlineStr">
         <is>
           <t>Punjabi (Shahmukhi script)</t>
@@ -20791,73 +20901,57 @@
       </c>
       <c r="D140" s="13" t="inlineStr">
         <is>
-          <t>شوق وعتاب (Shawq wa-ʿitāb; Longing and Reproach)</t>
+          <t>ʿAtāba</t>
         </is>
       </c>
       <c r="E140" s="13" t="inlineStr">
         <is>
-          <t>Longing and Reproach</t>
+          <t>Four Love Quatrains</t>
         </is>
       </c>
       <c r="F140" s="13" t="inlineStr">
         <is>
-          <t>كيف أغويتَني وأمعنتَ صَدّا
-يا حبيبًا أعطى قليلًا وأكدى
-ودَّ قلبي لو يجهل الحبَّ لما
-أنْ رآه يحول سَقْمًا ووَجْدا
-وشكتْ أضلعي من القلب نارًا
-هل عهدنَ الهوى سلامًا وبَردا؟!
-طلع الفجرُ باسمًا فتأمّلْ
-بنجوم الدجى تَرنَّحُ سُهْدا
-هي مثلي حيرى وعمّا قريبٍ
-تتوارى مع الظلام وتهدا
-لكَ حمّلتُها رسالةَ شوقٍ
-وعتابٍ، أظنّها لا تُؤدّى …
-قلتُ للطير حين أصبح يشدو
-«أيها الطيرُ عِمْ صباحًا!» فَردّا
-ثم غنّى أنشودةً عن حبيبٍ
-لم يكن ظالمًا، ولا خان عهدا
-أضرمَ الذكرياتِ بي ثُمّ ولّى
-لا رماكَ الصيّادُ … أسرفتَ جِدّا
-جمع اللهُ في مُحيّا حبيبي
-أُقحوانًا وياسَمينًا وَوَردا
-وابتسامًا لا يهجر الثغرَ إلَّا
-عند قولي له: أَتُنجز وعدا؟
-لا عرفتَ الوَفا ولا كان وعدٌ
-يجعل البسمةَ الوديعةَ حِقدا</t>
+          <t>Ṭalʿat nigmet il-ġarrār min rād,
+u-marbāha gabal Ḥaurān min rād;
+billa yā hawa l-ġaddār indār min rād,
+nada wa-kṭur ʿala ṣidr il-ḥabāba.
+Nizil maʿ bēn Yāfa u-bēn Maʿlūl,
+tiḥkīni u-band it-tōb maḥlūl;
+ana-lli min frāḳ il-ḥubb maʿlūl,
+u-mā yišfīni ġēr šōf il-iḥbāba.
+Nizil maʿ bēn Ṣāfīta u-ʿAkkār,
+u-kāsi kān ṣāfīli tʿakkar;
+ḥabābi lau saḳūni samm sukkar,
+ʿala ḳalbi aladd min eš-šarāba.
+Nizil maʿ bēn Zaḥle w-il-Ksaijir,
+ḥabībi lā ṭawīl walā ksaijir;
+ḥalafna dīn ʿannak mā nġaijir,
+mā zāl er-rūḥ wi-ggitti ṣawāba.</t>
         </is>
       </c>
       <c r="G140" s="13" t="inlineStr">
         <is>
-          <t>How you seduced me, then turned ever further away!
-O beloved who gave a little, then gave no more.
-My heart wished it knew nothing of love
-when it saw love turn to sickness and longing;
-and my ribs complained of the fire in my heart:
-have they ever known love as cool and peaceful?
-Dawn rose smiling: look at
-the night’s stars swaying, sleepless.
-They are bewildered like me, and soon
-they will vanish with the dark and grow still.
-I gave them a message for you, of longing
-and reproach; I think it will not be delivered…
-I said to the bird when it began to sing at dawn,
-“Good morning, bird!” and it answered,
-then sang a song about a beloved
-who was never cruel and never broke a promise.
-It kindled my memories, then flew away:
-may no hunter ever shoot you… but you went too far!
-God gathered in my beloved’s face
-camomile, jasmine and rose,
-and a smile that leaves those lips only
-when I say: will you keep a promise?
-Forget faithfulness, then: let there be no promise
-that turns that gentle smile to bitterness.</t>
+          <t>The morning star has risen over there,
+its home is the Hauran mountains, over there;
+by God, faithless wind, turn round, over there,
+and fall as dew upon my darling's breast.
+He made camp between Yafa and Maʿlul;
+she talks with me, the sash of her dress untied;
+I am the one made sick by love's parting,
+and nothing cures me but the sight of my love.
+He made camp between Safita and Akkar;
+my cup was clear for me, then it grew cloudy;
+if my loves gave me poison, it would be sugar,
+sweeter to my heart than any drink.
+He made camp between Zahle and Ksaijir;
+my darling is neither tall nor short;
+we swore an oath: I will never turn from you,
+as long as my soul and body hold together.</t>
         </is>
       </c>
       <c r="H140" s="13" t="inlineStr">
         <is>
-          <t>Ibrahim Tuqan (إبراهيم طوقان)</t>
+          <t>Traditional Palestinian ʿatāba; as printed by Gustaf Dalman, 1901</t>
         </is>
       </c>
       <c r="I140" s="13" t="inlineStr">
@@ -20877,71 +20971,73 @@
       </c>
       <c r="L140" s="13" t="inlineStr">
         <is>
-          <t>Men</t>
-        </is>
-      </c>
-      <c r="M140" s="14" t="n"/>
+          <t>Unknown</t>
+        </is>
+      </c>
+      <c r="M140" s="14" t="inlineStr">
+        <is>
+          <t>1901</t>
+        </is>
+      </c>
       <c r="N140" s="13" t="inlineStr">
         <is>
-          <t>Arabic</t>
+          <t>Palestinian Arabic (Dalman's transcription)</t>
         </is>
       </c>
       <c r="O140" s="13" t="n"/>
       <c r="P140" s="13" t="inlineStr">
         <is>
-          <t>Lyric poem</t>
+          <t>ʿAtāba (sung four-line verses)</t>
         </is>
       </c>
       <c r="Q140" s="13" t="inlineStr">
         <is>
-          <t>Man author</t>
+          <t>Anonymous singers</t>
         </is>
       </c>
       <c r="R140" s="13" t="inlineStr">
         <is>
-          <t>Before 1941; precise date unknown</t>
+          <t>Traditional sung verse; printed 1901</t>
         </is>
       </c>
       <c r="S140" s="13" t="inlineStr">
         <is>
-          <t>Hindawi digital edition, 2012</t>
+          <t>1901, Palästinischer Diwan (Leipzig)</t>
         </is>
       </c>
       <c r="T140" s="13" t="inlineStr">
         <is>
-          <t>The speaker addresses a rejecting beloved, sending longing and reproach through the stars and a singing bird. Romantic separation and unfulfilled affection.</t>
+          <t>Four love quatrains: dew sent on the wind to the beloved's breast, a lover whom only the sight of his love can cure, poison that would taste like sugar from her hand, and an oath to stay faithful as long as body and soul hold together.</t>
         </is>
       </c>
       <c r="U140" s="13" t="inlineStr">
         <is>
-          <t>Hindawi complete poetry, 2012 edition, book 25090535; Hindawi URL redirects to Safahat. Publisher explicitly declares the underlying text public domain.</t>
+          <t>Gustaf Dalman, Palästinischer Diwan (Leipzig, 1901), nos. 30–33; Arabic as transcribed by Dalman, OCR errors corrected.</t>
         </is>
       </c>
       <c r="V140" s="13" t="inlineStr">
         <is>
-          <t>Named chapter شوق وعتاب</t>
+          <t>Nos. 30–33</t>
         </is>
       </c>
       <c r="W140" s="13" t="inlineStr">
         <is>
-          <t>Collection’s first issue date is listed as unknown; do not treat 2012 as composition date. Original Arabic only; modern translation and editorial material separate.
-Passage update (29 October 2026): Complete poem, 24 half-lines (Hindawi edition of the complete poems; the section dividers are omitted). Fresh English translation by Claude (Anthropic AI); draft for editorial review.
-Moved to Poems to explore (30 October 2026) for the anthology review. Palestine: the poem's first publication date is unknown; the linked text is a 2012 digital edition.</t>
+          <t>Work changed (30 October 2026): Ibrahim Tuqan's poem, whose first publication could not be established, is replaced by four traditional love quatrains collected in Palestine and printed in 1901; one names Yafa and Maʿlul, villages near Nazareth. Fresh English translation by Claude (Anthropic AI) made directly from the original; draft for editorial review.</t>
         </is>
       </c>
       <c r="X140" s="13" t="inlineStr">
         <is>
-          <t>Publisher explicitly states the underlying text is public domain. Author died 1941; standard life-plus-70 term expired. Modern translations and editorial additions excluded.</t>
+          <t>Anthology review (30 October 2026): traditional anonymous verse; Dalman's 1901 printing is public domain (he died 1941). Dalman's German is not used.</t>
         </is>
       </c>
       <c r="Y140" s="13" t="inlineStr">
         <is>
-          <t>Linked full original text / credited edition</t>
+          <t>Internet Archive: Dalman, Palästinischer Diwan (1901)</t>
         </is>
       </c>
       <c r="Z140" s="11" t="inlineStr">
         <is>
-          <t>Read the text</t>
+          <t>Read the whole work</t>
         </is>
       </c>
       <c r="AA140" s="11" t="inlineStr">
@@ -20960,7 +21056,11 @@
         </is>
       </c>
       <c r="AD140" s="11" t="n"/>
-      <c r="AE140" s="11" t="n"/>
+      <c r="AE140" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: Read the text</t>
+        </is>
+      </c>
     </row>
     <row r="141" ht="91.5" customHeight="1" s="17">
       <c r="A141" s="7" t="inlineStr">
@@ -21298,26 +21398,26 @@
       </c>
       <c r="G143" s="13" t="inlineStr">
         <is>
-          <t>Two thrushes that are in their nest
-and never part from each other,
-alike in their beautiful blackness
-and twins in their beauty.
-For their blackness they say to the pheasant
-and to the night: we will out-darken you;
-for their shine they say to the moon,
-as it goes in: we will take your place.
-When they glance sideways, it is as if we saw
-the sun rising between the woods,
-and when they look straight, they do not merely shine:
-they blaze as brightly as the moon.
-For sorrow they are ready mourning,
-for joy a spring of delight;
-in hard looks they make me shiver,
-in soft looks they make me sin.
-What makes young women beautiful,
-their hair, their figure,
-your mistress does not need,
-for beauty overflows from you.</t>
+          <t>Two chopí birds that share one nest
+never leave each other at all;
+exactly alike in their lovely blackness,
+and in their beauty, twins indeed.
+With that blackness they tell the jacu bird
+and the night: “Let me make you darker.”
+With their brightness they tell the moon,
+as it is about to set: “Let me step over you.”
+In a sidelong glance we see already
+the sunrise between the woods;
+and when they look full on, they are not only bright:
+they blaze with beauty, just like the moon.
+In sorrow, mourning ready-made;
+in gladness, a bed of joy;
+with a hard look they make me shiver,
+with a gentle look they lead me into sin.
+What makes young women lovely,
+be it their hair, be it their body,
+the one who owns you has no need of:
+beauty spills from your very skin.</t>
         </is>
       </c>
       <c r="H143" s="13" t="inlineStr">
@@ -21345,7 +21445,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M143" s="14" t="n"/>
+      <c r="M143" s="14" t="inlineStr">
+        <is>
+          <t>before 1920</t>
+        </is>
+      </c>
       <c r="N143" s="13" t="inlineStr">
         <is>
           <t>Guaraní</t>
@@ -21391,12 +21495,14 @@
         <is>
           <t>Use Pane’s Guaraní original. Spanish free translation by Sinforiano Buzó Gómez is separately authored and is not covered by this original-rights assessment. Check modern orthographic editing before verbatim reuse.
 Passage update (29 October 2026): Complete poem, 20 lines, in Guaraní (text as printed in Las cien mejores poesías en guaraní, 1997). English translated from the Guaraní, checked against the free Spanish version printed with it. Fresh English translation by Claude (Anthropic AI); draft for editorial review.
-Moved to Poems to explore (30 October 2026): the English was checked against a modern Spanish translation still in copyright, so the passage is withheld until a fresh translation from the Guaraní has been reviewed by a Guaraní speaker.</t>
+Moved to Poems to explore (30 October 2026): the English was checked against a modern Spanish translation still in copyright, so the passage is withheld until a fresh translation from the Guaraní has been reviewed by a Guaraní speaker.
+Translation redone (30 October 2026): fresh English translation by Claude (Anthropic AI) made only from the Guaraní, without reference to any Spanish or other translation; returned to Poems to read. Review by a Guaraní speaker recommended.</t>
         </is>
       </c>
       <c r="X143" s="13" t="inlineStr">
         <is>
-          <t>Original text: standard life-plus-70 term expired; author died 1920. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.</t>
+          <t>Original text: standard life-plus-70 term expired; author died 1920. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.
+Anthology review (30 October 2026): Pane died 1920 and the poem was published in his lifetime; the 1997 anthology modernises the spelling only.</t>
         </is>
       </c>
       <c r="Y143" s="13" t="inlineStr">
@@ -21406,7 +21512,7 @@
       </c>
       <c r="Z143" s="11" t="inlineStr">
         <is>
-          <t>Read the text</t>
+          <t>Read the whole work</t>
         </is>
       </c>
       <c r="AA143" s="11" t="inlineStr">
@@ -22024,7 +22130,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M147" s="14" t="n"/>
+      <c r="M147" s="14" t="inlineStr">
+        <is>
+          <t>c. 1570</t>
+        </is>
+      </c>
       <c r="N147" s="13" t="inlineStr">
         <is>
           <t>Portuguese</t>
@@ -24583,7 +24693,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M165" s="14" t="n"/>
+      <c r="M165" s="14" t="inlineStr">
+        <is>
+          <t>c. 1833</t>
+        </is>
+      </c>
       <c r="N165" s="13" t="inlineStr">
         <is>
           <t>Slovenian</t>
@@ -24800,35 +24914,51 @@
       </c>
       <c r="D167" s="13" t="inlineStr">
         <is>
-          <t>Caashaqa haween waa horuu Caaddil soo rogaye (incipit; Caashaqa Haween)</t>
+          <t>Šáqlan Gédi-bā</t>
         </is>
       </c>
       <c r="E167" s="13" t="inlineStr">
         <is>
-          <t>Love of women was ordained long ago by the Just One (first line)</t>
+          <t>Two Somali Love Songs</t>
         </is>
       </c>
       <c r="F167" s="13" t="inlineStr">
         <is>
-          <t>Caashaqa haween waa horuu, Caaddil soo rogaye,
-Sayidkii carshiga nuurayiyo, Caliba soo gaadhye,
-Cidla lagama beermeen dadkoo, cuudi waahhidahe,
-Wahha caynba cayn looga dhigay, hays cajebiyeene,
-Soomaalidaa caado hhune, iguma caydeene.</t>
+          <t>Šáqlan Gédi-bā šára-ʾál-áy
+lō šir tágayá-yay,
+wáḥan ḥámar šakamádda
+ū gū ḥiḍay,
+šámis rúgtōdi-yay.
+šeḥyáda ʿílmiga šéga-yáy
+šáraf wádagán-i.
+Gāšánka ī šaqal,
+míd-dan šegayá tímid-i.
+Marākíbta badáha márta
+ē málabka díqaysa;
+wáḥa ī ga gá muq ḍēr Ijo
+an méher kū tūbáyay.</t>
         </is>
       </c>
       <c r="G167" s="13" t="inlineStr">
         <is>
-          <t>Love for women was ordained long ago by the Just One;
-it touched even the Prophet of the shining Throne, and Ali too.
-People did not grow out of emptiness; they come from one root,
-and each kind was made unlike the next, so let them not marvel at one another.
-It is the Somalis whose custom is cruel; let them not mock me.</t>
+          <t>Shaqlan, daughter of Gedi, truly:
+crowds go out to her;
+I too put the reins
+on a bay horse
+and rode towards the house of the sun.
+The sheikhs who teach learning
+have a share in her refinement.
+Cover my shield for me:
+the one I speak of has come.
+The ships sail the seas
+and bring precious things;
+but I would rather gaze at Ijo,
+for whom I paid the bride-price.</t>
         </is>
       </c>
       <c r="H167" s="13" t="inlineStr">
         <is>
-          <t>Cilmi Boodhari / Ilmi Bowndheri (c.1908–1941)</t>
+          <t>Traditional Somali songs; as printed by Leo Reinisch, 1900</t>
         </is>
       </c>
       <c r="I167" s="13" t="inlineStr">
@@ -24851,70 +24981,70 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M167" s="14" t="n">
-        <v>1934</v>
+      <c r="M167" s="14" t="inlineStr">
+        <is>
+          <t>1900</t>
+        </is>
       </c>
       <c r="N167" s="13" t="inlineStr">
         <is>
-          <t>Somali; older Roman orthography in Galaal’s typescript</t>
+          <t>Somali (Reinisch's transcription)</t>
         </is>
       </c>
       <c r="O167" s="13" t="n"/>
       <c r="P167" s="13" t="inlineStr">
         <is>
-          <t>Poetry</t>
+          <t>Two love songs</t>
         </is>
       </c>
       <c r="Q167" s="13" t="inlineStr">
         <is>
-          <t>Man author</t>
+          <t>Anonymous singers</t>
         </is>
       </c>
       <c r="R167" s="13" t="inlineStr">
         <is>
-          <t>1930s, after the love encounter dated 1934 in the 1967 account; exact composition date uncertain</t>
+          <t>Traditional sung verse; printed 1900</t>
         </is>
       </c>
       <c r="S167" s="13" t="inlineStr">
         <is>
-          <t>Five original Somali lines in M.H.I. Galaal, A Collection of Somali Literature, c.1964, p.31; fuller modern version 2016</t>
+          <t>1900, Die Somali-Sprache, vol. 1 (Vienna), pp. 257–258</t>
         </is>
       </c>
       <c r="T167" s="13" t="inlineStr">
         <is>
-          <t>The poet defends love of women as a natural human feeling and protests against those who shame him for being lovesick.</t>
+          <t>Two short love songs: the singer saddles his horse to join the crowds who court Shaqlan, Gedi's daughter, and a man who would rather look at Ijo, for whom he paid the bride-price, than at all the treasure ships bring.</t>
         </is>
       </c>
       <c r="U167" s="13" t="inlineStr">
         <is>
-          <t>Roma Tre Centro Studi Somali preserves Galaal’s unmodernized typescript; Andrzejewski’s prefatory note dates its mimeographed publication to about 1964. Original Somali excerpt at p.31 under ILMI – BOONDHERI. Oxford scholarly source corroborates death in 1941.</t>
+          <t>Leo Reinisch, Die Somali-Sprache, vol. 1: Texte (Vienna, 1900), nos. 120–121, pp. 257–258; Somali as printed, read from the page images.</t>
         </is>
       </c>
       <c r="V167" s="13" t="inlineStr">
         <is>
-          <t>Galaal p.31, five-line excerpt; 2016 bilingual collection pp.64–65 for a longer variant</t>
+          <t>Nos. 120–121, pp. 257–258</t>
         </is>
       </c>
       <c r="W167" s="13" t="inlineStr">
         <is>
-          <t>The assessed reuse lead is the historical Somali wording, not the 1967 English translation, modern bilingual edition, musical setting or performance. Versions differ. The repository’s CC BY-NC-ND label is restrictive and is not treated as permission to translate or commercially reuse modern editorial material. Berbera is in Somaliland, within the workbook’s Somalia country grouping.
-Passage update (29 October 2026): The five-line excerpt printed in Galaal’s collection, p. 31, in its older Somali spelling. The English is a careful draft. Fresh English translation by Claude (Anthropic AI); draft for editorial review.
-Moved to Poems to explore (30 October 2026): the passage is withheld while rights in Galaal's c.1964 written record of the oral poem are reviewed; the site links to the typescript instead.</t>
+          <t>Work changed (30 October 2026): Ilmi Boodhari's poem, whose only early written record (c.1964) may still carry the transcriber's rights, is replaced by two Somali love songs printed in 1900. Fresh English translation by Claude (Anthropic AI) made directly from the original; draft for editorial review.</t>
         </is>
       </c>
       <c r="X167" s="13" t="inlineStr">
         <is>
-          <t>Poet died 1941: original composition is beyond the standard life-plus-70 term. A Somali excerpt was published c.1964. Reuse only the underlying historical Somali lines; later translations, editorial contributions, melodies, recordings and repository licence restrictions remain separate.</t>
+          <t>Anthology review (30 October 2026): traditional anonymous songs; Reinisch's 1900 printing is public domain (he died 1919). Reinisch's German is not used.</t>
         </is>
       </c>
       <c r="Y167" s="13" t="inlineStr">
         <is>
-          <t>Work-specific text, date and provenance sources checked29October2026.</t>
+          <t>Internet Archive: Reinisch, Die Somali-Sprache, vol. 1 (1900)</t>
         </is>
       </c>
       <c r="Z167" s="11" t="inlineStr">
         <is>
-          <t>Read the text</t>
+          <t>Read the whole work</t>
         </is>
       </c>
       <c r="AA167" s="11" t="inlineStr">
@@ -24937,7 +25067,11 @@
           <t>Additional evidence</t>
         </is>
       </c>
-      <c r="AE167" s="11" t="n"/>
+      <c r="AE167" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: Read the text</t>
+        </is>
+      </c>
     </row>
     <row r="168" ht="91.5" customHeight="1" s="17">
       <c r="A168" s="7" t="inlineStr">
@@ -25170,7 +25304,11 @@
           <t>Women</t>
         </is>
       </c>
-      <c r="M169" s="14" t="n"/>
+      <c r="M169" s="14" t="inlineStr">
+        <is>
+          <t>c. 1580</t>
+        </is>
+      </c>
       <c r="N169" s="13" t="inlineStr">
         <is>
           <t>Classical Chinese (Hanja original)</t>
@@ -26283,7 +26421,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M177" s="14" t="n"/>
+      <c r="M177" s="14" t="inlineStr">
+        <is>
+          <t>c. 960</t>
+        </is>
+      </c>
       <c r="N177" s="13" t="inlineStr">
         <is>
           <t>Arabic</t>
@@ -26432,7 +26574,11 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M178" s="14" t="n"/>
+      <c r="M178" s="14" t="inlineStr">
+        <is>
+          <t>c. 930</t>
+        </is>
+      </c>
       <c r="N178" s="13" t="inlineStr">
         <is>
           <t>Persian (Arabic script)</t>
@@ -28897,7 +29043,11 @@
           <t>Women</t>
         </is>
       </c>
-      <c r="M195" s="14" t="n"/>
+      <c r="M195" s="14" t="inlineStr">
+        <is>
+          <t>c. 1830</t>
+        </is>
+      </c>
       <c r="N195" s="13" t="inlineStr">
         <is>
           <t>Uzbek / Chagatai literary tradition</t>
@@ -29356,7 +29506,11 @@
           <t>Women</t>
         </is>
       </c>
-      <c r="M198" s="14" t="n"/>
+      <c r="M198" s="14" t="inlineStr">
+        <is>
+          <t>c. 1800</t>
+        </is>
+      </c>
       <c r="N198" s="13" t="inlineStr">
         <is>
           <t>Vietnamese, modern Quốc ngữ transcription of Nôm verse</t>
@@ -29543,7 +29697,7 @@
       </c>
       <c r="M199" s="14" t="inlineStr">
         <is>
-          <t>700</t>
+          <t>c. 700</t>
         </is>
       </c>
       <c r="N199" s="13" t="inlineStr">
@@ -30173,367 +30327,371 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA93" r:id="rId309"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB93" r:id="rId310"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC93" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA94" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB94" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC94" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE95" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA97" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB97" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC97" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA98" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB98" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC98" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA100" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB100" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC100" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA101" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB101" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC101" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA103" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB103" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC103" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD103" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA104" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB104" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC104" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA105" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB105" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC105" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD105" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA106" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB106" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC106" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE109" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA110" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB110" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC110" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE110" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD111" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE112" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA113" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB113" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC113" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z115" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA115" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB115" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC115" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z116" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE116" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z117" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA117" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB117" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC117" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z118" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE118" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z119" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA119" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB119" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC119" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z120" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD120" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE120" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z121" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA121" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB121" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC121" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD121" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z122" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA122" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB122" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC122" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z123" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA123" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB123" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC123" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE123" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z124" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA124" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB124" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC124" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD124" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z125" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z126" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE126" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z127" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA127" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB127" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC127" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD127" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z128" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA128" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB128" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC128" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z129" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA129" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB129" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC129" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z130" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA130" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB130" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC130" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z131" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA131" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB131" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC131" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z132" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE132" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z133" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE133" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z134" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA134" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB134" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC134" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z135" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA135" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB135" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC135" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z136" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA136" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB136" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC136" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z137" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA137" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB137" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC137" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z138" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA138" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB138" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC138" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z139" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z140" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA140" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB140" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC140" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z141" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA141" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB141" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC141" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z142" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE142" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z143" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA143" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB143" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC143" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z144" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA144" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB144" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC144" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z145" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA145" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB145" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC145" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z146" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA146" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB146" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC146" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z147" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA147" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB147" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC147" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z148" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA148" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB148" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC148" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z149" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA149" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB149" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC149" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z150" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA150" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB150" r:id="rId500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC150" r:id="rId501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD150" r:id="rId502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE150" r:id="rId503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z151" r:id="rId504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD151" r:id="rId505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE151" r:id="rId506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z152" r:id="rId507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE152" r:id="rId508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z153" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z154" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE154" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z155" r:id="rId512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z156" r:id="rId513"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z157" r:id="rId514"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA157" r:id="rId515"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB157" r:id="rId516"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC157" r:id="rId517"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD157" r:id="rId518"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z158" r:id="rId519"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA158" r:id="rId520"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB158" r:id="rId521"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC158" r:id="rId522"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z159" r:id="rId523"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z160" r:id="rId524"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA160" r:id="rId525"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB160" r:id="rId526"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC160" r:id="rId527"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z161" r:id="rId528"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE161" r:id="rId529"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z162" r:id="rId530"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE162" r:id="rId531"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z163" r:id="rId532"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA163" r:id="rId533"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB163" r:id="rId534"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC163" r:id="rId535"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD163" r:id="rId536"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE163" r:id="rId537"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z164" r:id="rId538"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA164" r:id="rId539"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB164" r:id="rId540"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC164" r:id="rId541"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z165" r:id="rId542"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA165" r:id="rId543"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB165" r:id="rId544"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC165" r:id="rId545"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z166" r:id="rId546"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z167" r:id="rId547"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA167" r:id="rId548"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB167" r:id="rId549"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC167" r:id="rId550"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD167" r:id="rId551"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z168" r:id="rId552"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA168" r:id="rId553"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB168" r:id="rId554"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC168" r:id="rId555"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z169" r:id="rId556"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA169" r:id="rId557"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB169" r:id="rId558"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC169" r:id="rId559"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z170" r:id="rId560"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z171" r:id="rId561"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA171" r:id="rId562"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB171" r:id="rId563"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC171" r:id="rId564"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z172" r:id="rId565"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA172" r:id="rId566"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB172" r:id="rId567"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC172" r:id="rId568"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD172" r:id="rId569"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE172" r:id="rId570"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z173" r:id="rId571"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z174" r:id="rId572"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z175" r:id="rId573"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA175" r:id="rId574"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB175" r:id="rId575"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC175" r:id="rId576"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z176" r:id="rId577"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA176" r:id="rId578"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB176" r:id="rId579"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC176" r:id="rId580"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z177" r:id="rId581"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA177" r:id="rId582"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB177" r:id="rId583"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC177" r:id="rId584"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z178" r:id="rId585"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA178" r:id="rId586"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB178" r:id="rId587"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC178" r:id="rId588"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z179" r:id="rId589"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA179" r:id="rId590"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB179" r:id="rId591"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC179" r:id="rId592"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD179" r:id="rId593"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z180" r:id="rId594"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA180" r:id="rId595"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB180" r:id="rId596"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC180" r:id="rId597"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z181" r:id="rId598"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE181" r:id="rId599"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z182" r:id="rId600"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD182" r:id="rId601"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z183" r:id="rId602"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA183" r:id="rId603"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB183" r:id="rId604"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC183" r:id="rId605"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z184" r:id="rId606"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA184" r:id="rId607"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB184" r:id="rId608"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC184" r:id="rId609"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD184" r:id="rId610"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z185" r:id="rId611"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA185" r:id="rId612"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB185" r:id="rId613"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC185" r:id="rId614"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD185" r:id="rId615"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z186" r:id="rId616"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA186" r:id="rId617"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB186" r:id="rId618"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC186" r:id="rId619"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z187" r:id="rId620"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z188" r:id="rId621"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z189" r:id="rId622"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE189" r:id="rId623"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z190" r:id="rId624"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA190" r:id="rId625"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB190" r:id="rId626"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC190" r:id="rId627"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD190" r:id="rId628"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z191" r:id="rId629"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD191" r:id="rId630"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE191" r:id="rId631"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z192" r:id="rId632"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA192" r:id="rId633"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB192" r:id="rId634"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC192" r:id="rId635"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z193" r:id="rId636"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA193" r:id="rId637"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB193" r:id="rId638"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC193" r:id="rId639"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z194" r:id="rId640"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA194" r:id="rId641"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB194" r:id="rId642"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC194" r:id="rId643"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z195" r:id="rId644"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA195" r:id="rId645"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB195" r:id="rId646"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC195" r:id="rId647"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z196" r:id="rId648"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA196" r:id="rId649"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB196" r:id="rId650"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC196" r:id="rId651"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z197" r:id="rId652"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA197" r:id="rId653"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB197" r:id="rId654"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC197" r:id="rId655"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z198" r:id="rId656"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA198" r:id="rId657"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB198" r:id="rId658"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC198" r:id="rId659"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE198" r:id="rId660"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z199" r:id="rId661"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA199" r:id="rId662"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB199" r:id="rId663"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC199" r:id="rId664"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE199" r:id="rId665"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z200" r:id="rId666"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z201" r:id="rId667"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE201" r:id="rId668"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE93" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA94" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB94" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC94" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE95" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA97" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB97" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC97" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA98" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB98" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC98" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA100" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB100" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC100" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA101" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB101" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC101" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA103" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB103" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC103" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD103" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA104" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB104" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC104" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA105" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB105" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC105" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD105" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA106" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB106" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC106" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE109" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA110" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB110" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC110" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE110" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD111" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE112" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA113" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB113" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC113" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z115" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA115" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB115" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC115" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z116" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE116" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z117" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA117" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB117" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC117" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z118" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE118" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z119" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA119" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB119" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC119" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z120" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD120" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE120" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z121" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA121" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB121" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC121" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD121" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z122" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA122" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB122" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC122" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z123" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA123" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB123" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC123" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE123" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z124" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA124" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB124" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC124" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD124" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z125" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z126" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE126" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z127" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA127" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB127" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC127" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD127" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z128" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA128" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB128" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC128" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z129" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA129" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB129" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC129" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z130" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA130" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB130" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC130" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z131" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA131" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB131" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC131" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z132" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE132" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z133" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE133" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z134" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA134" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB134" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC134" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z135" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA135" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB135" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC135" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z136" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA136" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB136" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC136" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z137" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA137" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB137" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC137" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE137" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z138" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA138" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB138" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC138" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z139" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z140" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA140" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB140" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC140" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE140" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z141" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA141" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB141" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC141" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z142" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE142" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z143" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA143" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB143" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC143" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z144" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA144" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB144" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC144" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z145" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA145" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB145" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC145" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z146" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA146" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB146" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC146" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z147" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA147" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB147" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC147" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z148" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA148" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB148" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC148" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z149" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA149" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB149" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC149" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z150" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA150" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB150" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC150" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD150" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE150" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z151" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD151" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE151" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z152" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE152" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z153" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z154" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE154" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z155" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z156" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z157" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA157" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB157" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC157" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD157" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z158" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA158" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB158" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC158" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z159" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z160" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA160" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB160" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC160" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z161" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE161" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z162" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE162" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z163" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA163" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB163" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC163" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD163" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE163" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z164" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA164" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB164" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC164" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z165" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA165" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB165" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC165" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z166" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z167" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA167" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB167" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC167" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD167" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE167" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z168" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA168" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB168" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC168" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z169" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA169" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB169" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC169" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z170" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z171" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA171" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB171" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC171" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z172" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA172" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB172" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC172" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD172" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE172" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z173" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z174" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z175" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA175" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB175" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC175" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z176" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA176" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB176" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC176" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z177" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA177" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB177" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC177" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z178" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA178" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB178" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC178" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z179" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA179" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB179" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC179" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD179" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z180" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA180" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB180" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC180" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z181" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE181" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z182" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD182" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z183" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA183" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB183" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC183" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z184" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA184" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB184" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC184" r:id="rId613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD184" r:id="rId614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z185" r:id="rId615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA185" r:id="rId616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB185" r:id="rId617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC185" r:id="rId618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD185" r:id="rId619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z186" r:id="rId620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA186" r:id="rId621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB186" r:id="rId622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC186" r:id="rId623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z187" r:id="rId624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z188" r:id="rId625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z189" r:id="rId626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE189" r:id="rId627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z190" r:id="rId628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA190" r:id="rId629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB190" r:id="rId630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC190" r:id="rId631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD190" r:id="rId632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z191" r:id="rId633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD191" r:id="rId634"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE191" r:id="rId635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z192" r:id="rId636"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA192" r:id="rId637"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB192" r:id="rId638"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC192" r:id="rId639"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z193" r:id="rId640"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA193" r:id="rId641"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB193" r:id="rId642"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC193" r:id="rId643"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z194" r:id="rId644"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA194" r:id="rId645"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB194" r:id="rId646"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC194" r:id="rId647"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z195" r:id="rId648"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA195" r:id="rId649"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB195" r:id="rId650"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC195" r:id="rId651"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z196" r:id="rId652"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA196" r:id="rId653"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB196" r:id="rId654"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC196" r:id="rId655"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z197" r:id="rId656"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA197" r:id="rId657"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB197" r:id="rId658"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC197" r:id="rId659"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z198" r:id="rId660"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA198" r:id="rId661"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB198" r:id="rId662"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC198" r:id="rId663"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE198" r:id="rId664"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z199" r:id="rId665"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA199" r:id="rId666"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB199" r:id="rId667"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC199" r:id="rId668"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE199" r:id="rId669"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z200" r:id="rId670"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z201" r:id="rId671"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE201" r:id="rId672"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId669"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId673"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Austria: Rilke's "Liebes-Lied" (1907) replaces Ada Christen's "Erklärung"
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -2299,49 +2299,51 @@
       </c>
       <c r="D16" s="13" t="inlineStr">
         <is>
-          <t>Erklärung (Declaration)</t>
+          <t>Liebes-Lied</t>
         </is>
       </c>
       <c r="E16" s="13" t="inlineStr">
         <is>
-          <t>Declaration</t>
+          <t>Love Song</t>
         </is>
       </c>
       <c r="F16" s="13" t="inlineStr">
         <is>
-          <t>Ich hörte heute deine Schwüre –
-Und es bewegt das Herz mir nicht,
-Glaub’ ich auch selbst, daß heiße Liebe
-Aus jedem deiner Worte spricht.
-Denn unwillkürlich muß ich denken
-Der Zeit, wo du dich wirst bemühn,
-Mit leeren Phrasen zu verhüllen
-Des leeren Herzens matt’res Glühn.
-Wo endlich du des Kämpfens müde
-Und satt der selbstgewählten Ketten,
-Schamlos dein eignes Wort verleugnend,
-Ein Judas vor mich hin wirst treten.</t>
+          <t>Wie soll ich meine Seele halten, daß
+sie nicht an deine rührt? Wie soll ich sie
+hinheben über dich zu andern Dingen?
+Ach gerne möcht ich sie bei irgendwas
+Verlorenem im Dunkel unterbringen
+an einer fremden stillen Stelle, die
+nicht weiterschwingt wenn deine Tiefen schwingen.
+Doch alles was uns anrührt, dich und mich,
+nimmt uns zusammen wie ein Bogenstrich,
+der aus zwei Saiten eine Stimme zieht.
+Auf welches Instrument sind wir gespannt?
+Und welcher Spieler hat uns in der Hand?
+O süßes Lied.</t>
         </is>
       </c>
       <c r="G16" s="13" t="inlineStr">
         <is>
-          <t>I heard your vows today,
-and they leave my heart unmoved,
-though I believe myself that burning love
-speaks out of every word.
-For I can't help but think ahead
-to the time when you will strive
-to cover up with empty phrases
-the feebler glow of an empty heart;
-when, at last worn out with fighting
-and sick of chains you chose yourself,
-shamelessly disowning your own word,
-you will stand before me, a Judas.</t>
+          <t>How am I to hold my soul so that
+it does not touch on yours? How am I to
+lift it over you to other things?
+Oh, I would gladly lodge it somewhere
+with something lost in the dark,
+in a strange, still place
+that does not go on trembling when your depths tremble.
+Yet all that stirs us, you and me,
+gathers us up like a stroke of the bow
+that pulls a single voice from two strings.
+On what instrument are we strung?
+And which player has us in hand?
+O sweet song.</t>
         </is>
       </c>
       <c r="H16" s="13" t="inlineStr">
         <is>
-          <t>Ada Christen</t>
+          <t>Rainer Maria Rilke</t>
         </is>
       </c>
       <c r="I16" s="13" t="inlineStr">
@@ -2361,11 +2363,13 @@
       </c>
       <c r="L16" s="13" t="inlineStr">
         <is>
-          <t>Women</t>
-        </is>
-      </c>
-      <c r="M16" s="14" t="n">
-        <v>1868</v>
+          <t>Men</t>
+        </is>
+      </c>
+      <c r="M16" s="14" t="inlineStr">
+        <is>
+          <t>1907</t>
+        </is>
       </c>
       <c r="N16" s="13" t="inlineStr">
         <is>
@@ -2380,27 +2384,27 @@
       </c>
       <c r="Q16" s="13" t="inlineStr">
         <is>
-          <t>Woman</t>
+          <t>Rainer Maria Rilke (1875–1926)</t>
         </is>
       </c>
       <c r="R16" s="13" t="inlineStr">
         <is>
-          <t>1868 (Lieder einer Verlorenen)</t>
+          <t>1907 (Neue Gedichte)</t>
         </is>
       </c>
       <c r="S16" s="13" t="inlineStr">
         <is>
-          <t>1868, Hoffmann und Campe, Hamburg</t>
+          <t>1907, Neue Gedichte (Leipzig: Insel-Verlag), p. 3</t>
         </is>
       </c>
       <c r="T16" s="13" t="inlineStr">
         <is>
-          <t>Sceptical: the speaker hears declarations of love but fears future betrayal.</t>
+          <t>Two lovers are so bound together that the poet cannot keep his soul from touching hers: everything that moves them draws one voice from two strings, like a bow.</t>
         </is>
       </c>
       <c r="U16" s="13" t="inlineStr">
         <is>
-          <t>Scan-backed transcription, Lieder einer Verlorenen</t>
+          <t>Rilke, Neue Gedichte (Leipzig: Insel-Verlag, 1907), p. 3; German Wikisource, transcribed from the 1907 scans.</t>
         </is>
       </c>
       <c r="V16" s="13" t="inlineStr">
@@ -2410,20 +2414,22 @@
       </c>
       <c r="W16" s="13" t="inlineStr">
         <is>
-          <t>Original-language poem only; modern translations and recordings are separate. Retain attribution and source/license links for copyrightable transcription material.
-English passage: Earlier English draft by ChatGPT (replaced); draft for editorial review. 12-line passage on printed p.68. Original and English cells contain the same selection; line breaks are reading lines, not a claim of manuscript typography.
-Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
+          <t>Work changed (30 October 2026): Ada Christen's “Erklärung”, a poem of distrust rather than love, is replaced by Rilke's best-known love poem. Complete poem, 13 lines. Fresh English translation by Claude (Anthropic AI) made directly from the German, deliberately not following published translations; draft for editorial review.</t>
         </is>
       </c>
       <c r="X16" s="13" t="inlineStr">
         <is>
-          <t>Public-domain German original; author died 1901</t>
-        </is>
-      </c>
-      <c r="Y16" s="13" t="n"/>
+          <t>Anthology review (30 October 2026): published 1907; Rilke died 1926, so public domain in the UK, EU and US. Modern English translations (for example Stephen Mitchell's) are in copyright and are not used.</t>
+        </is>
+      </c>
+      <c r="Y16" s="13" t="inlineStr">
+        <is>
+          <t>German Wikisource: Liebes-Lied (Neue Gedichte, 1907)</t>
+        </is>
+      </c>
       <c r="Z16" s="11" t="inlineStr">
         <is>
-          <t>Read text</t>
+          <t>Read the whole work</t>
         </is>
       </c>
       <c r="AA16" s="11" t="inlineStr">
@@ -2442,7 +2448,11 @@
         </is>
       </c>
       <c r="AD16" s="11" t="n"/>
-      <c r="AE16" s="11" t="n"/>
+      <c r="AE16" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: Read text</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="180" customHeight="1" s="17">
       <c r="A17" s="7" t="inlineStr">
@@ -30053,645 +30063,646 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA16" r:id="rId35"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB16" r:id="rId36"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC16" r:id="rId37"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z17" r:id="rId38"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA17" r:id="rId39"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB17" r:id="rId40"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC17" r:id="rId41"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z18" r:id="rId42"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z19" r:id="rId43"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA19" r:id="rId44"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB19" r:id="rId45"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC19" r:id="rId46"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z20" r:id="rId47"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA20" r:id="rId48"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB20" r:id="rId49"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC20" r:id="rId50"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD20" r:id="rId51"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z21" r:id="rId52"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z22" r:id="rId53"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA22" r:id="rId54"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB22" r:id="rId55"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC22" r:id="rId56"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z23" r:id="rId57"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA23" r:id="rId58"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB23" r:id="rId59"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC23" r:id="rId60"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z24" r:id="rId61"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD24" r:id="rId62"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE24" r:id="rId63"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z25" r:id="rId64"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z26" r:id="rId65"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE26" r:id="rId66"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z27" r:id="rId67"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA27" r:id="rId68"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB27" r:id="rId69"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC27" r:id="rId70"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z28" r:id="rId71"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA28" r:id="rId72"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB28" r:id="rId73"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC28" r:id="rId74"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z29" r:id="rId75"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE29" r:id="rId76"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z30" r:id="rId77"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA30" r:id="rId78"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB30" r:id="rId79"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC30" r:id="rId80"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z31" r:id="rId81"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z32" r:id="rId82"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA32" r:id="rId83"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB32" r:id="rId84"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC32" r:id="rId85"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z33" r:id="rId86"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z34" r:id="rId87"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE34" r:id="rId88"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z35" r:id="rId89"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA35" r:id="rId90"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB35" r:id="rId91"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC35" r:id="rId92"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD35" r:id="rId93"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z36" r:id="rId94"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA36" r:id="rId95"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB36" r:id="rId96"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC36" r:id="rId97"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD36" r:id="rId98"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z37" r:id="rId99"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE37" r:id="rId100"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z38" r:id="rId101"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA38" r:id="rId102"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB38" r:id="rId103"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC38" r:id="rId104"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z39" r:id="rId105"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD39" r:id="rId106"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z40" r:id="rId107"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA40" r:id="rId108"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB40" r:id="rId109"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC40" r:id="rId110"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD40" r:id="rId111"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z41" r:id="rId112"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA41" r:id="rId113"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB41" r:id="rId114"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC41" r:id="rId115"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z42" r:id="rId116"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA42" r:id="rId117"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB42" r:id="rId118"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC42" r:id="rId119"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE42" r:id="rId120"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z43" r:id="rId121"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA43" r:id="rId122"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB43" r:id="rId123"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC43" r:id="rId124"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z44" r:id="rId125"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD44" r:id="rId126"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE44" r:id="rId127"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z45" r:id="rId128"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA45" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB45" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC45" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD45" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z46" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA46" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB46" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC46" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z47" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD47" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE47" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z48" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA48" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB48" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC48" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z49" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA49" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB49" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC49" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z50" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA50" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB50" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC50" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z51" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA51" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB51" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC51" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z52" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z53" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA53" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB53" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC53" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD53" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE53" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z54" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE54" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z55" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE55" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z56" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA56" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB56" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC56" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z57" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA57" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB57" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC57" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z58" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA58" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB58" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC58" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z59" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA59" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB59" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC59" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z60" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z61" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z62" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA62" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB62" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC62" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z63" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE63" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z64" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA64" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB64" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC64" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE64" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z65" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE65" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z66" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA66" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB66" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC66" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z67" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA67" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB67" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC67" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z68" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE68" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z69" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE69" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z70" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA70" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB70" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC70" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z71" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA71" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB71" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC71" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z72" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA72" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB72" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC72" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD72" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z73" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA73" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB73" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC73" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z74" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD74" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE74" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z75" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA75" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB75" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC75" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z76" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE76" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z77" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z78" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA78" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB78" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC78" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD78" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z79" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA79" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB79" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC79" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z80" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA80" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB80" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC80" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD80" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE80" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z81" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA81" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB81" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC81" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE81" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z82" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA82" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB82" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC82" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE82" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z83" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA83" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB83" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC83" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD83" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE83" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA84" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB84" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC84" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA85" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB85" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC85" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA86" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB86" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC86" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA87" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB87" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC87" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA88" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB88" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC88" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA89" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB89" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC89" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA90" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB90" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC90" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD90" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE90" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA91" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB91" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC91" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA92" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB92" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC92" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD92" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE92" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA93" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB93" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC93" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE93" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA94" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB94" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC94" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE95" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA97" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB97" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC97" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA98" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB98" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC98" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA100" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB100" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC100" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA101" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB101" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC101" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA103" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB103" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC103" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD103" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA104" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB104" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC104" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA105" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB105" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC105" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD105" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA106" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB106" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC106" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE109" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA110" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB110" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC110" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE110" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD111" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE112" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA113" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB113" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC113" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z115" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA115" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB115" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC115" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z116" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE116" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z117" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA117" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB117" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC117" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z118" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE118" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z119" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA119" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB119" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC119" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z120" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD120" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE120" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z121" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA121" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB121" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC121" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD121" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z122" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA122" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB122" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC122" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z123" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA123" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB123" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC123" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE123" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z124" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA124" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB124" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC124" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD124" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z125" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z126" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE126" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z127" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA127" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB127" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC127" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD127" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z128" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA128" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB128" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC128" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z129" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA129" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB129" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC129" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z130" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA130" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB130" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC130" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z131" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA131" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB131" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC131" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z132" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE132" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z133" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE133" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z134" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA134" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB134" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC134" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z135" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA135" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB135" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC135" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z136" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA136" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB136" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC136" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z137" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA137" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB137" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC137" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE137" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z138" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA138" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB138" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC138" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z139" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z140" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA140" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB140" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC140" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE140" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z141" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA141" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB141" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC141" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z142" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE142" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z143" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA143" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB143" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC143" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z144" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA144" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB144" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC144" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z145" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA145" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB145" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC145" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z146" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA146" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB146" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC146" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z147" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA147" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB147" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC147" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z148" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA148" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB148" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC148" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z149" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA149" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB149" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC149" r:id="rId500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z150" r:id="rId501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA150" r:id="rId502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB150" r:id="rId503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC150" r:id="rId504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD150" r:id="rId505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE150" r:id="rId506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z151" r:id="rId507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD151" r:id="rId508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE151" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z152" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE152" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z153" r:id="rId512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z154" r:id="rId513"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE154" r:id="rId514"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z155" r:id="rId515"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z156" r:id="rId516"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z157" r:id="rId517"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA157" r:id="rId518"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB157" r:id="rId519"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC157" r:id="rId520"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD157" r:id="rId521"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z158" r:id="rId522"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA158" r:id="rId523"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB158" r:id="rId524"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC158" r:id="rId525"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z159" r:id="rId526"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z160" r:id="rId527"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA160" r:id="rId528"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB160" r:id="rId529"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC160" r:id="rId530"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z161" r:id="rId531"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE161" r:id="rId532"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z162" r:id="rId533"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE162" r:id="rId534"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z163" r:id="rId535"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA163" r:id="rId536"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB163" r:id="rId537"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC163" r:id="rId538"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD163" r:id="rId539"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE163" r:id="rId540"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z164" r:id="rId541"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA164" r:id="rId542"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB164" r:id="rId543"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC164" r:id="rId544"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z165" r:id="rId545"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA165" r:id="rId546"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB165" r:id="rId547"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC165" r:id="rId548"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z166" r:id="rId549"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z167" r:id="rId550"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA167" r:id="rId551"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB167" r:id="rId552"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC167" r:id="rId553"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD167" r:id="rId554"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE167" r:id="rId555"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z168" r:id="rId556"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA168" r:id="rId557"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB168" r:id="rId558"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC168" r:id="rId559"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z169" r:id="rId560"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA169" r:id="rId561"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB169" r:id="rId562"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC169" r:id="rId563"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z170" r:id="rId564"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z171" r:id="rId565"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA171" r:id="rId566"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB171" r:id="rId567"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC171" r:id="rId568"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z172" r:id="rId569"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA172" r:id="rId570"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB172" r:id="rId571"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC172" r:id="rId572"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD172" r:id="rId573"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE172" r:id="rId574"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z173" r:id="rId575"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z174" r:id="rId576"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z175" r:id="rId577"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA175" r:id="rId578"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB175" r:id="rId579"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC175" r:id="rId580"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z176" r:id="rId581"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA176" r:id="rId582"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB176" r:id="rId583"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC176" r:id="rId584"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z177" r:id="rId585"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA177" r:id="rId586"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB177" r:id="rId587"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC177" r:id="rId588"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z178" r:id="rId589"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA178" r:id="rId590"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB178" r:id="rId591"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC178" r:id="rId592"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z179" r:id="rId593"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA179" r:id="rId594"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB179" r:id="rId595"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC179" r:id="rId596"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD179" r:id="rId597"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z180" r:id="rId598"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA180" r:id="rId599"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB180" r:id="rId600"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC180" r:id="rId601"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z181" r:id="rId602"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE181" r:id="rId603"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z182" r:id="rId604"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD182" r:id="rId605"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z183" r:id="rId606"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA183" r:id="rId607"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB183" r:id="rId608"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC183" r:id="rId609"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z184" r:id="rId610"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA184" r:id="rId611"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB184" r:id="rId612"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC184" r:id="rId613"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD184" r:id="rId614"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z185" r:id="rId615"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA185" r:id="rId616"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB185" r:id="rId617"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC185" r:id="rId618"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD185" r:id="rId619"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z186" r:id="rId620"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA186" r:id="rId621"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB186" r:id="rId622"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC186" r:id="rId623"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z187" r:id="rId624"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z188" r:id="rId625"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z189" r:id="rId626"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE189" r:id="rId627"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z190" r:id="rId628"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA190" r:id="rId629"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB190" r:id="rId630"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC190" r:id="rId631"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD190" r:id="rId632"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z191" r:id="rId633"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD191" r:id="rId634"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE191" r:id="rId635"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z192" r:id="rId636"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA192" r:id="rId637"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB192" r:id="rId638"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC192" r:id="rId639"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z193" r:id="rId640"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA193" r:id="rId641"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB193" r:id="rId642"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC193" r:id="rId643"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z194" r:id="rId644"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA194" r:id="rId645"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB194" r:id="rId646"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC194" r:id="rId647"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z195" r:id="rId648"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA195" r:id="rId649"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB195" r:id="rId650"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC195" r:id="rId651"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z196" r:id="rId652"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA196" r:id="rId653"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB196" r:id="rId654"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC196" r:id="rId655"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z197" r:id="rId656"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA197" r:id="rId657"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB197" r:id="rId658"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC197" r:id="rId659"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z198" r:id="rId660"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA198" r:id="rId661"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB198" r:id="rId662"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC198" r:id="rId663"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE198" r:id="rId664"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z199" r:id="rId665"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA199" r:id="rId666"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB199" r:id="rId667"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC199" r:id="rId668"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE199" r:id="rId669"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z200" r:id="rId670"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z201" r:id="rId671"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE201" r:id="rId672"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE16" r:id="rId38"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z17" r:id="rId39"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA17" r:id="rId40"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB17" r:id="rId41"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC17" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z18" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z19" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA19" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB19" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC19" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z20" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA20" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB20" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC20" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD20" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z21" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z22" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA22" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB22" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC22" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z23" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA23" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB23" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC23" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z24" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD24" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE24" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z25" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z26" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE26" r:id="rId67"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z27" r:id="rId68"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA27" r:id="rId69"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB27" r:id="rId70"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC27" r:id="rId71"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z28" r:id="rId72"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA28" r:id="rId73"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB28" r:id="rId74"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC28" r:id="rId75"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z29" r:id="rId76"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE29" r:id="rId77"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z30" r:id="rId78"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA30" r:id="rId79"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB30" r:id="rId80"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC30" r:id="rId81"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z31" r:id="rId82"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z32" r:id="rId83"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA32" r:id="rId84"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB32" r:id="rId85"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC32" r:id="rId86"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z33" r:id="rId87"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z34" r:id="rId88"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE34" r:id="rId89"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z35" r:id="rId90"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA35" r:id="rId91"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB35" r:id="rId92"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC35" r:id="rId93"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD35" r:id="rId94"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z36" r:id="rId95"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA36" r:id="rId96"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB36" r:id="rId97"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC36" r:id="rId98"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD36" r:id="rId99"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z37" r:id="rId100"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE37" r:id="rId101"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z38" r:id="rId102"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA38" r:id="rId103"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB38" r:id="rId104"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC38" r:id="rId105"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z39" r:id="rId106"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD39" r:id="rId107"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z40" r:id="rId108"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA40" r:id="rId109"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB40" r:id="rId110"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC40" r:id="rId111"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD40" r:id="rId112"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z41" r:id="rId113"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA41" r:id="rId114"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB41" r:id="rId115"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC41" r:id="rId116"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z42" r:id="rId117"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA42" r:id="rId118"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB42" r:id="rId119"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC42" r:id="rId120"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE42" r:id="rId121"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z43" r:id="rId122"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA43" r:id="rId123"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB43" r:id="rId124"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC43" r:id="rId125"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z44" r:id="rId126"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD44" r:id="rId127"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE44" r:id="rId128"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z45" r:id="rId129"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA45" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB45" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC45" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD45" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z46" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA46" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB46" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC46" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z47" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD47" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE47" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z48" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA48" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB48" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC48" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z49" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA49" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB49" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC49" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z50" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA50" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB50" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC50" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z51" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA51" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB51" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC51" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z52" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z53" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA53" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB53" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC53" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD53" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE53" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z54" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE54" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z55" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE55" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z56" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA56" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB56" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC56" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z57" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA57" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB57" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC57" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z58" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA58" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB58" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC58" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z59" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA59" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB59" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC59" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z60" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z61" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z62" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA62" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB62" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC62" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z63" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE63" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z64" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA64" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB64" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC64" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE64" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z65" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE65" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z66" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA66" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB66" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC66" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z67" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA67" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB67" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC67" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z68" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE68" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z69" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE69" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z70" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA70" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB70" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC70" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z71" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA71" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB71" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC71" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z72" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA72" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB72" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC72" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD72" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z73" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA73" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB73" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC73" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z74" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD74" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE74" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z75" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA75" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB75" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC75" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z76" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE76" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z77" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z78" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA78" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB78" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC78" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD78" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z79" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA79" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB79" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC79" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z80" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA80" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB80" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC80" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD80" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE80" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z81" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA81" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB81" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC81" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE81" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z82" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA82" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB82" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC82" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE82" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z83" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA83" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB83" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC83" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD83" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE83" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA84" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB84" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC84" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA85" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB85" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC85" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA86" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB86" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC86" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA87" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB87" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC87" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA88" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB88" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC88" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA89" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB89" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC89" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA90" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB90" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC90" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD90" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE90" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA91" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB91" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC91" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA92" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB92" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC92" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD92" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE92" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA93" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB93" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC93" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE93" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA94" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB94" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC94" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE95" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA97" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB97" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC97" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA98" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB98" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC98" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA100" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB100" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC100" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA101" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB101" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC101" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA103" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB103" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC103" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD103" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA104" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB104" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC104" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA105" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB105" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC105" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD105" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA106" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB106" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC106" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE109" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA110" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB110" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC110" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE110" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD111" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE112" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA113" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB113" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC113" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z115" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA115" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB115" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC115" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z116" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE116" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z117" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA117" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB117" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC117" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z118" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE118" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z119" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA119" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB119" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC119" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z120" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD120" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE120" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z121" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA121" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB121" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC121" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD121" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z122" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA122" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB122" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC122" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z123" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA123" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB123" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC123" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE123" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z124" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA124" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB124" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC124" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD124" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z125" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z126" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE126" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z127" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA127" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB127" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC127" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD127" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z128" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA128" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB128" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC128" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z129" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA129" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB129" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC129" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z130" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA130" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB130" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC130" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z131" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA131" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB131" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC131" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z132" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE132" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z133" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE133" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z134" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA134" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB134" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC134" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z135" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA135" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB135" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC135" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z136" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA136" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB136" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC136" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z137" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA137" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB137" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC137" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE137" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z138" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA138" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB138" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC138" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z139" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z140" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA140" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB140" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC140" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE140" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z141" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA141" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB141" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC141" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z142" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE142" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z143" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA143" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB143" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC143" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z144" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA144" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB144" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC144" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z145" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA145" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB145" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC145" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z146" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA146" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB146" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC146" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z147" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA147" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB147" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC147" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z148" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA148" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB148" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC148" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z149" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA149" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB149" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC149" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z150" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA150" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB150" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC150" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD150" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE150" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z151" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD151" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE151" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z152" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE152" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z153" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z154" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE154" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z155" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z156" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z157" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA157" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB157" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC157" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD157" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z158" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA158" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB158" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC158" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z159" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z160" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA160" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB160" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC160" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z161" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE161" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z162" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE162" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z163" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA163" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB163" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC163" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD163" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE163" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z164" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA164" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB164" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC164" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z165" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA165" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB165" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC165" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z166" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z167" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA167" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB167" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC167" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD167" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE167" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z168" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA168" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB168" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC168" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z169" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA169" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB169" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC169" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z170" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z171" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA171" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB171" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC171" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z172" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA172" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB172" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC172" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD172" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE172" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z173" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z174" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z175" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA175" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB175" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC175" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z176" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA176" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB176" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC176" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z177" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA177" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB177" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC177" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z178" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA178" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB178" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC178" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z179" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA179" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB179" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC179" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD179" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z180" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA180" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB180" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC180" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z181" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE181" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z182" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD182" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z183" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA183" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB183" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC183" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z184" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA184" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB184" r:id="rId613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC184" r:id="rId614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD184" r:id="rId615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z185" r:id="rId616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA185" r:id="rId617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB185" r:id="rId618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC185" r:id="rId619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD185" r:id="rId620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z186" r:id="rId621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA186" r:id="rId622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB186" r:id="rId623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC186" r:id="rId624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z187" r:id="rId625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z188" r:id="rId626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z189" r:id="rId627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE189" r:id="rId628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z190" r:id="rId629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA190" r:id="rId630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB190" r:id="rId631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC190" r:id="rId632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD190" r:id="rId633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z191" r:id="rId634"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD191" r:id="rId635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE191" r:id="rId636"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z192" r:id="rId637"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA192" r:id="rId638"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB192" r:id="rId639"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC192" r:id="rId640"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z193" r:id="rId641"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA193" r:id="rId642"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB193" r:id="rId643"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC193" r:id="rId644"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z194" r:id="rId645"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA194" r:id="rId646"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB194" r:id="rId647"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC194" r:id="rId648"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z195" r:id="rId649"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA195" r:id="rId650"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB195" r:id="rId651"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC195" r:id="rId652"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z196" r:id="rId653"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA196" r:id="rId654"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB196" r:id="rId655"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC196" r:id="rId656"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z197" r:id="rId657"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA197" r:id="rId658"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB197" r:id="rId659"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC197" r:id="rId660"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z198" r:id="rId661"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA198" r:id="rId662"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB198" r:id="rId663"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC198" r:id="rId664"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE198" r:id="rId665"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z199" r:id="rId666"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA199" r:id="rId667"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB199" r:id="rId668"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC199" r:id="rId669"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE199" r:id="rId670"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z200" r:id="rId671"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z201" r:id="rId672"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE201" r:id="rId673"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId673"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId674"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Sensitivity review: replace contentious and outsider-sourced entries
Guyana (Martin Carter), South Africa (Mazisi Kunene) and Türkiye (Karacaoğlan)
replaced; love songs by local artists for Congo, Tanzania, Mali, Guinea,
Burundi, Maldives and Tonga; São Tomé, Azerbaijan, Iran and Oman passages
trimmed or retranslated; notes updated.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -2489,9 +2489,7 @@
 Gül üzün görmək əgər mümkün olaydı bir dəm,
 Hər zaman görmək onu nuri-mücəlla gətirir.
 Qaşü göz, novki-mücə fitnə üçün cəm olmuş,
-Ox atıb, tiğ cəkib, hər biri dəva gətirir.
-Könlümü qarət edir eylə ki, tari-zülfün,
-Rumə, sanki həbəşi ləşgəri-yəğma gətirir.</t>
+Ox atıb, tiğ cəkib, hər biri dəva gətirir.</t>
         </is>
       </c>
       <c r="G17" s="13" t="inlineStr">
@@ -2503,9 +2501,7 @@
 If I could look at your rose of a face for one moment,
 each look would bring a shining, radiant light.
 Brow, eye and lash-point have joined forces to stir up trouble:
-one shoots arrows, one draws a blade, each picks a fight.
-The strand of your hair so plunders my heart,
-it is as if an Abyssinian army brought sack and ruin to Rum.</t>
+one shoots arrows, one draws a blade, each picks a fight.</t>
         </is>
       </c>
       <c r="H17" s="13" t="inlineStr">
@@ -2583,7 +2579,8 @@
         <is>
           <t>Natavan was a Shusha/Karabakh poet in present-day Azerbaijan. Original ghazal only; modern transliteration/editorial contributions may require attribution. English translation not supplied.
 Passage update (29 October 2026): Earlier English draft by ChatGPT (replaced); editorial draft, not a quoted published translation. Original and English contain the same selection. Latin transcription follows Wikisource, including cəkib as printed. Final couplet retains a historical dark-hair/light-face military conceit involving Abyssinia and Rum. Classical vocabulary merits specialist review.
-Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
+Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.
+Revision (30 October 2026, sensitivity review): final couplet left out (its image compares dark hair to an Abyssinian army); the passage is now couplets 1–4 of the ghazal.</t>
         </is>
       </c>
       <c r="X17" s="13" t="inlineStr">
@@ -4931,19 +4928,19 @@
       </c>
       <c r="D34" s="13" t="inlineStr">
         <is>
-          <t>Nakupenda</t>
+          <t>Amosozi y'urukundo</t>
         </is>
       </c>
       <c r="E34" s="13" t="inlineStr">
         <is>
-          <t>I Love You</t>
+          <t>Tears of Love</t>
         </is>
       </c>
       <c r="F34" s="13" t="n"/>
       <c r="G34" s="13" t="n"/>
       <c r="H34" s="13" t="inlineStr">
         <is>
-          <t>Iry Tina and Pallaso; co-writing Daddy Andre; production Diggy Baur</t>
+          <t>Kidum (Jean-Pierre Nimbona)</t>
         </is>
       </c>
       <c r="I34" s="13" t="inlineStr">
@@ -4963,53 +4960,60 @@
       </c>
       <c r="L34" s="13" t="inlineStr">
         <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="M34" s="14" t="n"/>
+          <t>Men</t>
+        </is>
+      </c>
+      <c r="M34" s="14" t="inlineStr">
+        <is>
+          <t>c. 2015</t>
+        </is>
+      </c>
       <c r="N34" s="13" t="inlineStr">
         <is>
-          <t>English, Swahili, Luganda and additional language not named</t>
+          <t>Kirundi</t>
         </is>
       </c>
       <c r="O34" s="13" t="n"/>
       <c r="P34" s="13" t="inlineStr">
         <is>
-          <t>Song</t>
+          <t>Love song</t>
         </is>
       </c>
       <c r="Q34" s="13" t="inlineStr">
         <is>
-          <t>Unknown / not established</t>
-        </is>
-      </c>
-      <c r="R34" s="13" t="n"/>
+          <t>Kidum</t>
+        </is>
+      </c>
+      <c r="R34" s="13" t="inlineStr">
+        <is>
+          <t>c. 2015</t>
+        </is>
+      </c>
       <c r="S34" s="13" t="n"/>
       <c r="T34" s="13" t="inlineStr">
         <is>
-          <t>Report describes mutual promises of loyalty and enduring romantic love.</t>
+          <t>A Kirundi ballad about the tears that love brings.</t>
         </is>
       </c>
       <c r="U34" s="13" t="inlineStr">
         <is>
-          <t>Burundian Iry Tina collaborates with Ugandan Pallaso, 2021. Shared modern performance.</t>
+          <t>Audio video with lyrics on Kidum's YouTube channel.</t>
         </is>
       </c>
       <c r="V34" s="13" t="n"/>
       <c r="W34" s="13" t="inlineStr">
         <is>
-          <t>No complete English translation verified. Original text, translation, edition and any recording require separate rights review.
-Passage update (29 October 2026): Not filled: a modern song and collaborators are identified, but no original lyrics have been supplied for translation. Supply the lyric text and the intended recorded version.</t>
+          <t>Work changed (30 October 2026) after the sensitivity review: the duet whose singer could not be confirmed as Burundian is replaced by a Kirundi love song by Burundi's best-known singer.</t>
         </is>
       </c>
       <c r="X34" s="13" t="inlineStr">
         <is>
-          <t>Lyric, musical setting, translation, performance and recording rights require separate review. Age or online access is not permission.</t>
+          <t>In copyright: described and linked only; no text or recording is reproduced here. Sensitivity review, 30 October 2026.</t>
         </is>
       </c>
       <c r="Y34" s="13" t="inlineStr">
         <is>
-          <t>Notjustok East Africa, 14 October 2021</t>
+          <t>Audio video with lyrics on Kidum's YouTube channel.</t>
         </is>
       </c>
       <c r="Z34" s="11" t="inlineStr">
@@ -6523,126 +6527,108 @@
       </c>
       <c r="D45" s="13" t="inlineStr">
         <is>
-          <t>The Vanishing Wife</t>
+          <t>Bolingo Ebomi Nga</t>
         </is>
       </c>
       <c r="E45" s="13" t="inlineStr">
         <is>
-          <t>The Vanishing Wife</t>
+          <t>Love Has Killed Me</t>
         </is>
       </c>
       <c r="F45" s="13" t="n"/>
       <c r="G45" s="13" t="n"/>
       <c r="H45" s="13" t="inlineStr">
         <is>
-          <t>Vili / Loango oral tradition; Richard Edward Dennett (1857–1921), published English version</t>
+          <t>Roga Roga</t>
         </is>
       </c>
       <c r="I45" s="13" t="inlineStr">
         <is>
-          <t>Historical version only</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J45" s="13" t="inlineStr">
         <is>
-          <t>Named work (text)</t>
+          <t>Named work</t>
         </is>
       </c>
       <c r="K45" s="13" t="inlineStr">
         <is>
-          <t>Prose / folktale</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="L45" s="13" t="inlineStr">
         <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="M45" s="14" t="n">
-        <v>1898</v>
+          <t>Men</t>
+        </is>
+      </c>
+      <c r="M45" s="14" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
       </c>
       <c r="N45" s="13" t="inlineStr">
         <is>
-          <t>English historical version; Vili / Loango source tradition</t>
+          <t>Lingala</t>
         </is>
       </c>
       <c r="O45" s="13" t="n"/>
       <c r="P45" s="13" t="inlineStr">
         <is>
-          <t>Prose / folktale</t>
+          <t>Love song</t>
         </is>
       </c>
       <c r="Q45" s="13" t="inlineStr">
         <is>
-          <t>Original oral creator / attribution not established</t>
+          <t>Roga Roga (Extra Musica)</t>
         </is>
       </c>
       <c r="R45" s="13" t="inlineStr">
         <is>
-          <t>1898, Notes on the Folklore of the Fjort, chapter V</t>
-        </is>
-      </c>
-      <c r="S45" s="13" t="inlineStr">
-        <is>
-          <t>Historical work reproduced in linked digital source; modern editorial material is separate</t>
-        </is>
-      </c>
+          <t>2026</t>
+        </is>
+      </c>
+      <c r="S45" s="13" t="n"/>
       <c r="T45" s="13" t="inlineStr">
         <is>
-          <t>Buite loves the mysterious woman who brings him comfort; breaking her condition causes her to disappear, leaving him grieving.</t>
+          <t>A rumba love song in which the singer confesses that love has overwhelmed him.</t>
         </is>
       </c>
       <c r="U45" s="13" t="inlineStr">
         <is>
-          <t>Dennett’s named Loango tale, published 1898; source places his work in what is now the Republic of the Congo.</t>
-        </is>
-      </c>
-      <c r="V45" s="13" t="inlineStr">
-        <is>
-          <t>Complete chapter V; the wife’s arrival and final disappearance</t>
-        </is>
-      </c>
+          <t>Official video on Roga Roga's YouTube channel.</t>
+        </is>
+      </c>
+      <c r="V45" s="13" t="n"/>
       <c r="W45" s="13" t="inlineStr">
         <is>
-          <t>Historical English retelling through a colonial collector. Country is the Republic of the Congo, not the Democratic Republic of the Congo. Original Vili wording is not supplied.</t>
+          <t>Work changed (30 October 2026) after the sensitivity review: the 1898 folktale recorded by a British trader is replaced by a love song by one of Brazzaville's best-known musicians.</t>
         </is>
       </c>
       <c r="X45" s="13" t="inlineStr">
         <is>
-          <t>The source identifies this historical English book as public domain. Dennett died 1921 and the 1898 version is beyond standard life-plus-70 terms. This does not clear all oral variants, community rights or later adaptations.</t>
+          <t>In copyright: described and linked only; no text or recording is reproduced here. Sensitivity review, 30 October 2026.</t>
         </is>
       </c>
       <c r="Y45" s="13" t="inlineStr">
         <is>
-          <t>Dennett’s named Loango tale, published 1898; source places his work in what is now the Republic of the Congo.</t>
+          <t>Official video on Roga Roga's YouTube channel.</t>
         </is>
       </c>
       <c r="Z45" s="11" t="inlineStr">
         <is>
-          <t>Work / source text</t>
-        </is>
-      </c>
-      <c r="AA45" s="11" t="inlineStr">
-        <is>
-          <t>Reuse basis / copyright duration</t>
-        </is>
-      </c>
-      <c r="AB45" s="11" t="inlineStr">
-        <is>
-          <t>Date / edition evidence</t>
-        </is>
-      </c>
-      <c r="AC45" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country evidence</t>
-        </is>
-      </c>
-      <c r="AD45" s="11" t="inlineStr">
-        <is>
-          <t>Additional evidence</t>
-        </is>
-      </c>
-      <c r="AE45" s="11" t="n"/>
+          <t>Watch the video</t>
+        </is>
+      </c>
+      <c r="AA45" s="11" t="n"/>
+      <c r="AB45" s="11" t="n"/>
+      <c r="AC45" s="11" t="n"/>
+      <c r="AD45" s="11" t="n"/>
+      <c r="AE45" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: https://sacred-texts.com/book/notes-on-the-folklore-of-the-fjort/v-the-vanishing-wife</t>
+        </is>
+      </c>
     </row>
     <row r="46" ht="91.5" customHeight="1" s="17">
       <c r="A46" s="7" t="inlineStr">
@@ -11078,19 +11064,19 @@
       </c>
       <c r="D76" s="13" t="inlineStr">
         <is>
-          <t>Titati</t>
+          <t>M'Bambou (Berce-moi)</t>
         </is>
       </c>
       <c r="E76" s="13" t="inlineStr">
         <is>
-          <t>Titati — English meaning not yet verified</t>
+          <t>Rock Me</t>
         </is>
       </c>
       <c r="F76" s="13" t="n"/>
       <c r="G76" s="13" t="n"/>
       <c r="H76" s="13" t="inlineStr">
         <is>
-          <t>Traditional Manding melody; instrumental version by Habib Koite</t>
+          <t>Sékouba Bambino</t>
         </is>
       </c>
       <c r="I76" s="13" t="inlineStr">
@@ -11110,57 +11096,65 @@
       </c>
       <c r="L76" s="13" t="inlineStr">
         <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="M76" s="14" t="n"/>
+          <t>Men</t>
+        </is>
+      </c>
+      <c r="M76" s="14" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
       <c r="N76" s="13" t="inlineStr">
         <is>
-          <t>Manding repertoire; instrumental version has no sung words</t>
+          <t>Malinke</t>
         </is>
       </c>
       <c r="O76" s="13" t="n"/>
       <c r="P76" s="13" t="inlineStr">
         <is>
-          <t>Song</t>
+          <t>Love song</t>
         </is>
       </c>
       <c r="Q76" s="13" t="inlineStr">
         <is>
-          <t>Unknown (traditional / collective authorship)</t>
-        </is>
-      </c>
-      <c r="R76" s="13" t="n"/>
+          <t>Sékouba Bambino</t>
+        </is>
+      </c>
+      <c r="R76" s="13" t="inlineStr">
+        <is>
+          <t>2017</t>
+        </is>
+      </c>
       <c r="S76" s="13" t="n"/>
       <c r="T76" s="13" t="inlineStr">
         <is>
-          <t>Performer explains its story as a lover seeking reciprocation. Album version is instrumental.</t>
+          <t>A tender love song in which the singer asks his beloved to cradle and rock him.</t>
         </is>
       </c>
       <c r="U76" s="13" t="inlineStr">
         <is>
-          <t>Koite interview about Afriki (2007) describes the melody as popular in both Mali and Guinea. Shared repertoire.</t>
+          <t>Official video on the Syllart Records YouTube channel.</t>
         </is>
       </c>
       <c r="V76" s="13" t="n"/>
       <c r="W76" s="13" t="inlineStr">
         <is>
-          <t>English interview. No sung text or English lyric verified.</t>
+          <t>Work changed (30 October 2026) after the sensitivity review: Habib Koité's instrumental, which had no words and was also used for Mali, is replaced by a love song by Guinea's best-known singer.</t>
         </is>
       </c>
       <c r="X76" s="13" t="inlineStr">
         <is>
-          <t>Lyric, musical setting, translation, performance and recording rights require separate review. Age or online access is not permission.</t>
+          <t>In copyright: described and linked only; no text or recording is reproduced here. Sensitivity review, 30 October 2026.</t>
         </is>
       </c>
       <c r="Y76" s="13" t="inlineStr">
         <is>
-          <t>Afropop Worldwide, Banning Eyre / Sean Barlow interview conducted June 2007; webpage dated 2025</t>
+          <t>Official video on the Syllart Records YouTube channel.</t>
         </is>
       </c>
       <c r="Z76" s="11" t="inlineStr">
         <is>
-          <t>Listen to the song</t>
+          <t>Watch the video</t>
         </is>
       </c>
       <c r="AA76" s="11" t="n"/>
@@ -11307,63 +11301,29 @@
       </c>
       <c r="D78" s="13" t="inlineStr">
         <is>
-          <t>The Negro Village</t>
+          <t>This Is the Dark Time, My Love</t>
         </is>
       </c>
       <c r="E78" s="13" t="inlineStr">
         <is>
-          <t>The Negro Village — passage on husband, wife and love</t>
-        </is>
-      </c>
-      <c r="F78" s="13" t="inlineStr">
-        <is>
-          <t>And yet there are, who will in strength maintain,
-The negro heart is foreign to all thought
-Which breathes of hopeful love, affection’s reign,
-Or nobler passions in the bosom wrought;
-Such reason in a blind conceit,
-Where prejudice and false pride meet,
-Yea! man is man with all emotions fraught.
-Their hearts can love with all the lavish strength,
-Impetuous fervour of ungoverned will,
-Running unbroken to its utmost length:
-Passion’s frenzy, but pure love’s offspring still;
-Unweaned by cold decorum’s laws,
-Cleaving persistent to its cause,
-Free and natural as the mountain rill.</t>
-        </is>
-      </c>
-      <c r="G78" s="13" t="inlineStr">
-        <is>
-          <t>And yet there are, who will in strength maintain,
-The negro heart is foreign to all thought
-Which breathes of hopeful love, affection’s reign,
-Or nobler passions in the bosom wrought;
-Such reason in a blind conceit,
-Where prejudice and false pride meet,
-Yea! man is man with all emotions fraught.
-Their hearts can love with all the lavish strength,
-Impetuous fervour of ungoverned will,
-Running unbroken to its utmost length:
-Passion’s frenzy, but pure love’s offspring still;
-Unweaned by cold decorum’s laws,
-Cleaving persistent to its cause,
-Free and natural as the mountain rill.</t>
-        </is>
-      </c>
+          <t>This Is the Dark Time, My Love</t>
+        </is>
+      </c>
+      <c r="F78" s="13" t="n"/>
+      <c r="G78" s="13" t="n"/>
       <c r="H78" s="13" t="inlineStr">
         <is>
-          <t>Egbert Martin, pen name Leo (c.1861–1890)</t>
+          <t>Martin Carter (1927–1997)</t>
         </is>
       </c>
       <c r="I78" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J78" s="13" t="inlineStr">
         <is>
-          <t>Named work (text)</t>
+          <t>Named work</t>
         </is>
       </c>
       <c r="K78" s="13" t="inlineStr">
@@ -11376,8 +11336,10 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M78" s="14" t="n">
-        <v>1883</v>
+      <c r="M78" s="14" t="inlineStr">
+        <is>
+          <t>1954</t>
+        </is>
       </c>
       <c r="N78" s="13" t="inlineStr">
         <is>
@@ -11387,81 +11349,60 @@
       <c r="O78" s="13" t="n"/>
       <c r="P78" s="13" t="inlineStr">
         <is>
-          <t>Lyric poem</t>
+          <t>Poem</t>
         </is>
       </c>
       <c r="Q78" s="13" t="inlineStr">
         <is>
-          <t>Man author</t>
+          <t>Martin Carter</t>
         </is>
       </c>
       <c r="R78" s="13" t="inlineStr">
         <is>
-          <t>1883, Leo’s Poetical Works</t>
-        </is>
-      </c>
-      <c r="S78" s="13" t="inlineStr">
-        <is>
-          <t>Historical work reproduced in linked digital source; modern editorial material is separate</t>
-        </is>
-      </c>
+          <t>1954</t>
+        </is>
+      </c>
+      <c r="S78" s="13" t="n"/>
       <c r="T78" s="13" t="inlineStr">
         <is>
-          <t>Within a wider village portrait, the poet describes a young wife and her affectionate husband, then affirms the intensity of their capacity for love.</t>
+          <t>A love poem written in a time of fear: the poet tells his beloved that the dark season has come, but speaks to her with tenderness and watchfulness while waiting for it to pass.</t>
         </is>
       </c>
       <c r="U78" s="13" t="inlineStr">
         <is>
-          <t>Lehigh University digital poetry anthology transcribes the 1883 poem. David Dabydeen’s biographical discussion documents Martin’s Georgetown connection and death in 1890.</t>
-        </is>
-      </c>
-      <c r="V78" s="13" t="inlineStr">
-        <is>
-          <t>Stanzas beginning with the youthful wife and continuing into the reflection on love</t>
-        </is>
-      </c>
+          <t>Martin Carter, Poems of Resistance from British Guiana (London: Lawrence &amp; Wishart, 1954).</t>
+        </is>
+      </c>
+      <c r="V78" s="13" t="n"/>
       <c r="W78" s="13" t="inlineStr">
         <is>
-          <t>Only the specified passage concerns romantic/marital love; the entire poem is not a love lyric. Its racial and Christian language reflects the nineteenth-century setting.
-Passage update (29 October 2026): Two consecutive stanzas, 14 lines: the poet answers the claim that Black people cannot feel deep love. Original English; no translation needed. Original English text; not a translation.</t>
+          <t>Work changed (30 October 2026) after the sensitivity review: Egbert Martin's 1883 poem, whose title and theme centred on race, is dropped; this is Guyana's best-known love poem, by its national poet.</t>
         </is>
       </c>
       <c r="X78" s="13" t="inlineStr">
         <is>
-          <t>Historical original text: standard life-plus-70 term has expired; author died 1890. Assessment excludes modern translations, commentary, editorial alterations, musical settings and recordings. Territorial and unusual publication-history exceptions are not comprehensively assessed.</t>
+          <t>In copyright: described and linked only; no text or recording is reproduced here. Sensitivity review, 30 October 2026.</t>
         </is>
       </c>
       <c r="Y78" s="13" t="inlineStr">
         <is>
-          <t>Lehigh University digital poetry anthology transcribes the 1883 poem. David Dabydeen’s biographical discussion documents Martin’s Georgetown connection and death in 1890.</t>
+          <t>Martin Carter, Poems of Resistance from British Guiana (London: Lawrence &amp; Wishart, 1954).</t>
         </is>
       </c>
       <c r="Z78" s="11" t="inlineStr">
         <is>
-          <t>Work / source text</t>
-        </is>
-      </c>
-      <c r="AA78" s="11" t="inlineStr">
-        <is>
-          <t>Reuse basis / copyright duration</t>
-        </is>
-      </c>
-      <c r="AB78" s="11" t="inlineStr">
-        <is>
-          <t>Date / edition evidence</t>
-        </is>
-      </c>
-      <c r="AC78" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country evidence</t>
-        </is>
-      </c>
-      <c r="AD78" s="11" t="inlineStr">
-        <is>
-          <t>Additional evidence</t>
-        </is>
-      </c>
-      <c r="AE78" s="11" t="n"/>
+          <t>Read the text</t>
+        </is>
+      </c>
+      <c r="AA78" s="11" t="n"/>
+      <c r="AB78" s="11" t="n"/>
+      <c r="AC78" s="11" t="n"/>
+      <c r="AD78" s="11" t="n"/>
+      <c r="AE78" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: https://scalar.lehigh.edu/african-american-poetry-a-digital-anthology/egbert-martin-leo-the-negro-village-1883.1</t>
+        </is>
+      </c>
     </row>
     <row r="79" ht="91.5" customHeight="1" s="17">
       <c r="A79" s="7" t="inlineStr">
@@ -12794,7 +12735,7 @@
 for the dark mole on that cheek I'd give up Samarkand and Bukhara.
 Bring the last of the wine, cupbearer: in paradise you won't find
 the banks of the Ruknabad or the flowered paths of Musalla.
-Ah, these playful gypsy girls, so charming, such trouble to the town,
+Ah, these playful wandering minstrel girls, so charming, such trouble to the town,
 have stripped the patience from my heart as Turks strip a table of its spoils.
 My love is incomplete, but my beloved's beauty does not need it:
 a lovely face has no use for powder, colour, beauty-spot or pencil.
@@ -12885,7 +12826,8 @@
         <is>
           <t>New English translation from the Persian; Gertrude Bell's 1897 translation is not used. Modern translations are separate. Mystical readings are possible.
 Passage update (29 October 2026): Complete ghazal, 9 couplets (18 half-lines). Persian text from Ganjoor (ghazal 3), with Ganjoor’s added short-vowel marks removed; the letters are unchanged. Fresh English translation by Claude (Anthropic AI); draft for editorial review.
-Revision (30 October 2026): retranslated from the Persian for the anthology review so that no line follows the wording of an earlier English version.</t>
+Revision (30 October 2026): retranslated from the Persian for the anthology review so that no line follows the wording of an earlier English version.
+Revision (30 October 2026, sensitivity review): lūliyān (line 5) translated as 'wandering minstrel girls' rather than with an ethnic slur.</t>
         </is>
       </c>
       <c r="X86" s="13" t="inlineStr">
@@ -16589,19 +16531,19 @@
       </c>
       <c r="D111" s="13" t="inlineStr">
         <is>
-          <t>I Get to Love You (Acoustic)</t>
+          <t>Nunidhey</t>
         </is>
       </c>
       <c r="E111" s="13" t="inlineStr">
         <is>
-          <t>I Get to Love You (Acoustic)</t>
+          <t>Nunidhey</t>
         </is>
       </c>
       <c r="F111" s="13" t="n"/>
       <c r="G111" s="13" t="n"/>
       <c r="H111" s="13" t="inlineStr">
         <is>
-          <t>Mysha Didi; original writers to confirm</t>
+          <t>Abdulla Livaaz</t>
         </is>
       </c>
       <c r="I111" s="13" t="inlineStr">
@@ -16621,68 +16563,76 @@
       </c>
       <c r="L111" s="13" t="inlineStr">
         <is>
-          <t>Women</t>
-        </is>
-      </c>
-      <c r="M111" s="14" t="n"/>
+          <t>Men</t>
+        </is>
+      </c>
+      <c r="M111" s="14" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
       <c r="N111" s="13" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Dhivehi</t>
         </is>
       </c>
       <c r="O111" s="13" t="n"/>
       <c r="P111" s="13" t="inlineStr">
         <is>
-          <t>Song / cover</t>
+          <t>Love song</t>
         </is>
       </c>
       <c r="Q111" s="13" t="inlineStr">
         <is>
-          <t>Woman (performer); authorship unknown or unconfirmed</t>
-        </is>
-      </c>
-      <c r="R111" s="13" t="n"/>
+          <t>Abdulla Livaaz</t>
+        </is>
+      </c>
+      <c r="R111" s="13" t="inlineStr">
+        <is>
+          <t>2026</t>
+        </is>
+      </c>
       <c r="S111" s="13" t="n"/>
       <c r="T111" s="13" t="inlineStr">
         <is>
-          <t>Named romantic wedding-ballad cover; exact lyric and credits not yet inspected.</t>
+          <t>A Dhivehi love song dedicated to those who love from a distance.</t>
         </is>
       </c>
       <c r="U111" s="13" t="inlineStr">
         <is>
-          <t>Tristar Records3March2023; Maldivian singer based Leeds performing international cover.</t>
+          <t>Official music video on Abdulla Livaaz's YouTube channel.</t>
         </is>
       </c>
       <c r="V111" s="13" t="n"/>
       <c r="W111" s="13" t="inlineStr">
         <is>
-          <t>Performance provenance only; not Maldivian composition or Dhivehi song.</t>
+          <t>Work changed (30 October 2026) after the sensitivity review: an English-language wedding cover is replaced by a love song in Dhivehi by a Maldivian singer-songwriter.</t>
         </is>
       </c>
       <c r="X111" s="13" t="inlineStr">
         <is>
-          <t>Review original text, edition and any translation separately. Website permission does not transfer to this book.</t>
+          <t>In copyright: described and linked only; no text or recording is reproduced here. Sensitivity review, 30 October 2026.</t>
         </is>
       </c>
       <c r="Y111" s="13" t="inlineStr">
         <is>
-          <t>Tristar distributor metadata; performer self-description</t>
+          <t>Official music video on Abdulla Livaaz's YouTube channel.</t>
         </is>
       </c>
       <c r="Z111" s="11" t="inlineStr">
         <is>
-          <t>Listen to the song</t>
+          <t>Watch the video</t>
         </is>
       </c>
       <c r="AA111" s="11" t="n"/>
       <c r="AB111" s="11" t="n"/>
       <c r="AC111" s="11" t="n"/>
-      <c r="AD111" s="11" t="inlineStr">
-        <is>
-          <t>addtoevent.co.uk</t>
-        </is>
-      </c>
-      <c r="AE111" s="11" t="n"/>
+      <c r="AD111" s="11" t="n"/>
+      <c r="AE111" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: https://open.spotify.com/track/1Pte35IwrE0KkvftaAofgw</t>
+        </is>
+      </c>
     </row>
     <row r="112" ht="60" customHeight="1" s="17">
       <c r="A112" s="7" t="inlineStr">
@@ -16702,19 +16652,19 @@
       </c>
       <c r="D112" s="13" t="inlineStr">
         <is>
-          <t>Titati</t>
+          <t>Je pense à toi</t>
         </is>
       </c>
       <c r="E112" s="13" t="inlineStr">
         <is>
-          <t>Titati — English meaning not yet verified</t>
+          <t>I Think of You</t>
         </is>
       </c>
       <c r="F112" s="13" t="n"/>
       <c r="G112" s="13" t="n"/>
       <c r="H112" s="13" t="inlineStr">
         <is>
-          <t>Traditional Manding melody; instrumental version by Habib Koite</t>
+          <t>Amadou &amp; Mariam</t>
         </is>
       </c>
       <c r="I112" s="13" t="inlineStr">
@@ -16734,57 +16684,65 @@
       </c>
       <c r="L112" s="13" t="inlineStr">
         <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="M112" s="14" t="n"/>
+          <t>Mixed</t>
+        </is>
+      </c>
+      <c r="M112" s="14" t="inlineStr">
+        <is>
+          <t>1998</t>
+        </is>
+      </c>
       <c r="N112" s="13" t="inlineStr">
         <is>
-          <t>Manding repertoire; instrumental version has no sung words</t>
+          <t>French and Bambara</t>
         </is>
       </c>
       <c r="O112" s="13" t="n"/>
       <c r="P112" s="13" t="inlineStr">
         <is>
-          <t>Song</t>
+          <t>Love song</t>
         </is>
       </c>
       <c r="Q112" s="13" t="inlineStr">
         <is>
-          <t>Unknown (traditional / collective authorship)</t>
-        </is>
-      </c>
-      <c r="R112" s="13" t="n"/>
+          <t>Amadou Bagayoko and Mariam Doumbia</t>
+        </is>
+      </c>
+      <c r="R112" s="13" t="inlineStr">
+        <is>
+          <t>1998</t>
+        </is>
+      </c>
       <c r="S112" s="13" t="n"/>
       <c r="T112" s="13" t="inlineStr">
         <is>
-          <t>Performer explains its story as a lover seeking reciprocation. Album version is instrumental.</t>
+          <t>A married couple sing to each other of how they think of one another all the time.</t>
         </is>
       </c>
       <c r="U112" s="13" t="inlineStr">
         <is>
-          <t>Koite interview about Afriki (2007) describes the melody as popular in both Mali and Guinea. Shared repertoire.</t>
+          <t>Official video on the Amadou &amp; Mariam VEVO channel; song first released on Sou ni tilé (1998).</t>
         </is>
       </c>
       <c r="V112" s="13" t="n"/>
       <c r="W112" s="13" t="inlineStr">
         <is>
-          <t>English interview. No sung text or English lyric verified.</t>
+          <t>Work changed (30 October 2026) after the sensitivity review: Habib Koité's instrumental, which had no words and was also used for Guinea, is replaced by Mali's best-loved love song.</t>
         </is>
       </c>
       <c r="X112" s="13" t="inlineStr">
         <is>
-          <t>Lyric, musical setting, translation, performance and recording rights require separate review. Age or online access is not permission.</t>
+          <t>In copyright: described and linked only; no text or recording is reproduced here. Sensitivity review, 30 October 2026.</t>
         </is>
       </c>
       <c r="Y112" s="13" t="inlineStr">
         <is>
-          <t>Afropop Worldwide, Banning Eyre / Sean Barlow interview conducted June 2007; webpage dated 2025</t>
+          <t>Official video on the Amadou &amp; Mariam VEVO channel; song first released on Sou ni tilé (1998).</t>
         </is>
       </c>
       <c r="Z112" s="11" t="inlineStr">
         <is>
-          <t>Listen to the song</t>
+          <t>Watch the video</t>
         </is>
       </c>
       <c r="AA112" s="11" t="n"/>
@@ -20491,7 +20449,7 @@
 the greeting of one who repays in full and never falls short.
 We do not greet the dwelling out of love for its ground,
 but for love of women like white gazelles that linger behind the herd,
-tall and slender, soft and full-breasted,
+tall and slender, soft and young,
 supple and graceful, from the noblest of Nahshal;
 and for one with long hair, gleaming where her skin is bare, tender,
 one of the modest, soft-voiced girls, her mouth sweet to kiss;
@@ -20576,7 +20534,8 @@
       </c>
       <c r="W137" s="13" t="inlineStr">
         <is>
-          <t>Work changed (30 October 2026): Saʿid al-Busaʿidi's poem, for which no printing before 1989 could be established, is replaced by the love prelude of a qasida by Oman's best-known classical poet. Couplets 8–14 of 21. Fresh English translation by Claude (Anthropic AI) made directly from the original; draft for editorial review.</t>
+          <t>Work changed (30 October 2026): Saʿid al-Busaʿidi's poem, for which no printing before 1989 could be established, is replaced by the love prelude of a qasida by Oman's best-known classical poet. Couplets 8–14 of 21. Fresh English translation by Claude (Anthropic AI) made directly from the original; draft for editorial review.
+Revision (30 October 2026, sensitivity review): line 5 rendered 'tall and slender, soft and young'.</t>
         </is>
       </c>
       <c r="X137" s="13" t="inlineStr">
@@ -23126,7 +23085,7 @@
       <c r="S154" s="13" t="n"/>
       <c r="T154" s="13" t="inlineStr">
         <is>
-          <t>Dance-floor attraction and sexual invitation; full song text and credits still to inspect.</t>
+          <t>The soca love song that made Vincentian music a worldwide hit.</t>
         </is>
       </c>
       <c r="U154" s="13" t="inlineStr">
@@ -23421,10 +23380,6 @@
 em que astro nenhum flutua
 mas se o teu olhar o fita
 na noite desponta a lua
-Se os escravos são comprados
-ó branca de além do mar
-homem livre eu, sou escravo
-comprado por teu olhar
 Meu olhar é retratista
 ò minha doce miragem
 senão diz-me porque tenho
@@ -23432,7 +23387,15 @@
 Roubei-te o primeiro beijo
 o segundo foi-me dado
 o terceiro, francamente,
-creio que me foi roubado</t>
+creio que me foi roubado
+Um dia a espuma dos mares
+ao ver em si meu amor
+Foi dizer baixinho à praia
+– a Vénus mudou de cor
+A nossa terra é tão bela
+duma beleza sem par
+E por ser assim formosa
+Fê-la sua amante o mar…</t>
         </is>
       </c>
       <c r="G157" s="13" t="inlineStr">
@@ -23441,10 +23404,6 @@
 in which no star is floating,
 but if your gaze rests on them,
 the moon rises in that night.
-If slaves are bought,
-O white woman from over the sea,
-I, a free man, am a slave
-bought by your gaze.
 My gaze is a portrait painter,
 O my sweet mirage;
 otherwise tell me why I carry
@@ -23452,7 +23411,15 @@
 I stole the first kiss from you,
 the second was given to me,
 the third, frankly,
-I believe was stolen from me.</t>
+I believe was stolen from me.
+One day the foam of the seas,
+seeing my love reflected in it,
+went and whispered to the shore:
+'Venus has changed her colour.'
+Our land is so lovely,
+of a beauty without equal,
+and because it is so fair
+the sea has made it his lover…</t>
         </is>
       </c>
       <c r="H157" s="13" t="inlineStr">
@@ -23511,7 +23478,7 @@
       </c>
       <c r="T157" s="13" t="inlineStr">
         <is>
-          <t>Love quatrains include exchanged kisses and praise of a dark-skinned beloved, alongside racial imagery shaped by colonial society.</t>
+          <t>Playful love quatrains: the beloved's gaze makes the moon rise, kisses are stolen and given, the sea foam mistakes her for Venus, and the island itself becomes the sea's lover.</t>
         </is>
       </c>
       <c r="U157" s="13" t="inlineStr">
@@ -23527,7 +23494,8 @@
       <c r="W157" s="13" t="inlineStr">
         <is>
           <t>The text contains racial comparisons requiring contextual reading. Modern commentary is separate. Composition date is not known; 1916 is the collection date.
-Passage update (29 October 2026): First four quatrains, 16 lines. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
+Passage update (29 October 2026): First four quatrains, 16 lines. Fresh English translation by Claude (Anthropic AI); draft for editorial review.
+Revision (30 October 2026, sensitivity review): re-excerpted to quatrains 1, 3, 4, 7 and 8 (20 lines), leaving out the quatrains built on slavery and skin-colour comparisons.</t>
         </is>
       </c>
       <c r="X157" s="13" t="inlineStr">
@@ -25101,151 +25069,108 @@
       </c>
       <c r="D168" s="13" t="inlineStr">
         <is>
-          <t>The Story of an African Farm</t>
+          <t>Ingoma Yakho Eyangivusayo</t>
         </is>
       </c>
       <c r="E168" s="13" t="inlineStr">
         <is>
-          <t>The Story of an African Farm</t>
-        </is>
-      </c>
-      <c r="F168" s="13" t="inlineStr">
-        <is>
-          <t>“But I’m sure you must be cold,” said Gregory, and put his hand under the cloak, and found there a small fist doubled up, soft, and very warm.
-He held it fast in his hand.
-“Oh, Em, I love you better than all the world besides! Tell me, do you love me a little?”
-“Yes, I do,” said Em, hesitating, and trying softly to free her hand.
-“Better than everything; better than all the world, darling?” he asked, bending down so low that the yellow hair was blown into his eyes.
-“I don’t know,” said Em, gravely. “I do love you very much; but I love my cousin who is at school, and Waldo, very much. You see I have known them so long!”
-“Oh, Em, do not talk to me so coldly!” Gregory cried, seizing the little arm that rested on the gate, and pressing it till she was half afraid.
-The herdsman had moved away to the other end of the kraal now, and the cows, busy with their calves, took no notice of the little human farce.
-“Em, if you talk so to me I will go mad! You must love me, love me better than all! You must give yourself to me. I have loved you since that first moment when I saw you walking by the stone wall with the jug in your hands. You were made for me, created for me! I will love you till I die! Oh, Em, do not be so cold, so cruel to me!”
-He held her arm so tightly that her fingers relaxed their hold, and the cloak fluttered down on to the ground, and the wind played more roughly than ever with the little yellow head.
-“I do love you very much,” she said; “but I do not know if I want to marry you. I love you better than Waldo, but I can’t tell if I love you better than Lyndall. If you would let me wait for a week I think perhaps I could tell you.”</t>
-        </is>
-      </c>
-      <c r="G168" s="13" t="inlineStr">
-        <is>
-          <t>“But I’m sure you must be cold,” said Gregory, and put his hand under the cloak, and found there a small fist doubled up, soft, and very warm.
-He held it fast in his hand.
-“Oh, Em, I love you better than all the world besides! Tell me, do you love me a little?”
-“Yes, I do,” said Em, hesitating, and trying softly to free her hand.
-“Better than everything; better than all the world, darling?” he asked, bending down so low that the yellow hair was blown into his eyes.
-“I don’t know,” said Em, gravely. “I do love you very much; but I love my cousin who is at school, and Waldo, very much. You see I have known them so long!”
-“Oh, Em, do not talk to me so coldly!” Gregory cried, seizing the little arm that rested on the gate, and pressing it till she was half afraid.
-The herdsman had moved away to the other end of the kraal now, and the cows, busy with their calves, took no notice of the little human farce.
-“Em, if you talk so to me I will go mad! You must love me, love me better than all! You must give yourself to me. I have loved you since that first moment when I saw you walking by the stone wall with the jug in your hands. You were made for me, created for me! I will love you till I die! Oh, Em, do not be so cold, so cruel to me!”
-He held her arm so tightly that her fingers relaxed their hold, and the cloak fluttered down on to the ground, and the wind played more roughly than ever with the little yellow head.
-“I do love you very much,” she said; “but I do not know if I want to marry you. I love you better than Waldo, but I can’t tell if I love you better than Lyndall. If you would let me wait for a week I think perhaps I could tell you.”</t>
-        </is>
-      </c>
+          <t>The Hundredth Song of Love</t>
+        </is>
+      </c>
+      <c r="F168" s="13" t="n"/>
+      <c r="G168" s="13" t="n"/>
       <c r="H168" s="13" t="inlineStr">
         <is>
-          <t>Olive Schreiner (published as Ralph Iron)</t>
+          <t>Mazisi Kunene (1930–2006)</t>
         </is>
       </c>
       <c r="I168" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J168" s="13" t="inlineStr">
         <is>
-          <t>Named literary work (original text)</t>
+          <t>Named work</t>
         </is>
       </c>
       <c r="K168" s="13" t="inlineStr">
         <is>
-          <t>Prose / novel</t>
+          <t>Poetry</t>
         </is>
       </c>
       <c r="L168" s="13" t="inlineStr">
         <is>
-          <t>Women</t>
-        </is>
-      </c>
-      <c r="M168" s="14" t="n">
-        <v>1883</v>
+          <t>Men</t>
+        </is>
+      </c>
+      <c r="M168" s="14" t="inlineStr">
+        <is>
+          <t>1997</t>
+        </is>
       </c>
       <c r="N168" s="13" t="inlineStr">
         <is>
-          <t>English</t>
+          <t>Zulu</t>
         </is>
       </c>
       <c r="O168" s="13" t="n"/>
       <c r="P168" s="13" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Poem</t>
         </is>
       </c>
       <c r="Q168" s="13" t="inlineStr">
         <is>
-          <t>Woman author</t>
+          <t>Mazisi Kunene</t>
         </is>
       </c>
       <c r="R168" s="13" t="inlineStr">
         <is>
-          <t>1883 first publication</t>
-        </is>
-      </c>
-      <c r="S168" s="13" t="inlineStr">
-        <is>
-          <t>Gutenberg digital edition: 1998; updated 2018</t>
-        </is>
-      </c>
+          <t>1997</t>
+        </is>
+      </c>
+      <c r="S168" s="13" t="n"/>
       <c r="T168" s="13" t="inlineStr">
         <is>
-          <t>Novel exploring romantic desire, marriage and women’s independence through Lyndall, Em and Gregory. Part II includes Em’s response to Gregory’s proposal and Lyndall’s reflections on love.</t>
+          <t>The poet wakes to find himself lifted by his beloved's hundred songs, dazzled by the flash of her eyes.</t>
         </is>
       </c>
       <c r="U168" s="13" t="inlineStr">
         <is>
-          <t>Project Gutenberg ebook 1441, released 1998, updated 2018; English original, author 1855–1920. South African Karoo setting and author’s literary association.</t>
-        </is>
-      </c>
-      <c r="V168" s="13" t="inlineStr">
-        <is>
-          <t>Part II, Em/Gregory courtship and Lyndall scenes; search “I do love you very much”</t>
-        </is>
-      </c>
+          <t>Mazisi Kunene, Igudu likaSomcabeko (1997); English version on Poetry International.</t>
+        </is>
+      </c>
+      <c r="V168" s="13" t="n"/>
       <c r="W168" s="13" t="inlineStr">
         <is>
-          <t>Prose novel rather than poem/song. Contains critical and painful relationships, not uniformly positive views. Historical racial language appears in the book. Gutenberg branding/licence separate from underlying novel.
-Passage update (29 October 2026): Eleven consecutive lines (one per paragraph or sentence) from Part II, Gregory’s declaration to Em at the cow-kraal gate. Original English; no translation needed. Original English text; not a translation.</t>
+          <t>Work changed (30 October 2026) after the sensitivity review: Olive Schreiner's settler novel is replaced by a recent love poem in Zulu by South Africa's first poet laureate.</t>
         </is>
       </c>
       <c r="X168" s="13" t="inlineStr">
         <is>
-          <t>Original text: standard life-plus-70 term expired; author died 1920. Reuse assessment applies to the original words, not modern translations, editorial additions, musical settings or recordings. Publication-history and territorial exceptions are not universally assessed.</t>
+          <t>In copyright: described and linked only; no text or recording is reproduced here. Sensitivity review, 30 October 2026.</t>
         </is>
       </c>
       <c r="Y168" s="13" t="inlineStr">
         <is>
-          <t>Project Gutenberg ebook 1441</t>
+          <t>Mazisi Kunene, Igudu likaSomcabeko (1997); English version on Poetry International.</t>
         </is>
       </c>
       <c r="Z168" s="11" t="inlineStr">
         <is>
-          <t>Original text</t>
-        </is>
-      </c>
-      <c r="AA168" s="11" t="inlineStr">
-        <is>
-          <t>Copyright duration rule</t>
-        </is>
-      </c>
-      <c r="AB168" s="11" t="inlineStr">
-        <is>
-          <t>Text / date evidence</t>
-        </is>
-      </c>
-      <c r="AC168" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country evidence</t>
-        </is>
-      </c>
+          <t>Read the text</t>
+        </is>
+      </c>
+      <c r="AA168" s="11" t="n"/>
+      <c r="AB168" s="11" t="n"/>
+      <c r="AC168" s="11" t="n"/>
       <c r="AD168" s="11" t="n"/>
-      <c r="AE168" s="11" t="n"/>
+      <c r="AE168" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: https://www.gutenberg.org/files/1441/1441-h/1441-h.htm</t>
+        </is>
+      </c>
     </row>
     <row r="169" ht="75.75" customHeight="1" s="17">
       <c r="A169" s="7" t="inlineStr">
@@ -26688,126 +26613,108 @@
       </c>
       <c r="D179" s="13" t="inlineStr">
         <is>
-          <t>L’intelligence des femmes</t>
+          <t>Utanipenda?</t>
         </is>
       </c>
       <c r="E179" s="13" t="inlineStr">
         <is>
-          <t>The Cleverness of Women</t>
+          <t>Will You Love Me?</t>
         </is>
       </c>
       <c r="F179" s="13" t="n"/>
       <c r="G179" s="13" t="n"/>
       <c r="H179" s="13" t="inlineStr">
         <is>
-          <t>Swahili oral narrators (unnamed); Carl Velten; René Basset, French version</t>
+          <t>Diamond Platnumz</t>
         </is>
       </c>
       <c r="I179" s="13" t="inlineStr">
         <is>
-          <t>Historical version only</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J179" s="13" t="inlineStr">
         <is>
-          <t>Named work (text)</t>
+          <t>Named work</t>
         </is>
       </c>
       <c r="K179" s="13" t="inlineStr">
         <is>
-          <t>Prose / folktale</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="L179" s="13" t="inlineStr">
         <is>
-          <t>Unknown</t>
-        </is>
-      </c>
-      <c r="M179" s="14" t="n">
-        <v>1903</v>
+          <t>Men</t>
+        </is>
+      </c>
+      <c r="M179" s="14" t="inlineStr">
+        <is>
+          <t>2015</t>
+        </is>
       </c>
       <c r="N179" s="13" t="inlineStr">
         <is>
-          <t>French historical version; Swahili source</t>
+          <t>Swahili</t>
         </is>
       </c>
       <c r="O179" s="13" t="n"/>
       <c r="P179" s="13" t="inlineStr">
         <is>
-          <t>Prose / folktale</t>
+          <t>Love song</t>
         </is>
       </c>
       <c r="Q179" s="13" t="inlineStr">
         <is>
-          <t>Original oral creator / attribution not established</t>
+          <t>Diamond Platnumz</t>
         </is>
       </c>
       <c r="R179" s="13" t="inlineStr">
         <is>
-          <t>French version 1903; Swahili/German source edition 1898</t>
-        </is>
-      </c>
-      <c r="S179" s="13" t="inlineStr">
-        <is>
-          <t>Historical work reproduced in linked digital source; modern editorial material is separate</t>
-        </is>
-      </c>
+          <t>2015</t>
+        </is>
+      </c>
+      <c r="S179" s="13" t="n"/>
       <c r="T179" s="13" t="inlineStr">
         <is>
-          <t>Interlocking stories of attraction, courtship, marriage and secret lovers demonstrate women’s ingenuity.</t>
+          <t>The singer asks his beloved whether she would still love him if he lost his fame and fortune.</t>
         </is>
       </c>
       <c r="U179" s="13" t="inlineStr">
         <is>
-          <t>Basset no.98, pp.233–252, places the Swahili tradition in the Zanzibar region and cites Velten’s 1898 Swahili text, pp.110–119, and German version, pp.178–191.</t>
-        </is>
-      </c>
-      <c r="V179" s="13" t="inlineStr">
-        <is>
-          <t>Opening love triangle and the vizier’s son’s courtship episodes</t>
-        </is>
-      </c>
+          <t>Official lyric video with English translation, on Diamond Platnumz's YouTube channel.</t>
+        </is>
+      </c>
+      <c r="V179" s="13" t="n"/>
       <c r="W179" s="13" t="inlineStr">
         <is>
-          <t>Includes adultery and polygamy; not an uncomplicated positive love story. The reusable text identified is the old French version, not a modern recording or a verified contemporary Swahili original.</t>
+          <t>Work changed (30 October 2026) after the sensitivity review: the tale collected under German colonial rule is replaced by a Swahili love song by Tanzania's biggest star.</t>
         </is>
       </c>
       <c r="X179" s="13" t="inlineStr">
         <is>
-          <t>Historical 1903 French version is public domain under standard life-plus-70 terms (Basset died 1924; Velten 1935); Commons marks the edition public domain. Native community rights and modern versions are separate.</t>
+          <t>In copyright: described and linked only; no text or recording is reproduced here. Sensitivity review, 30 October 2026.</t>
         </is>
       </c>
       <c r="Y179" s="13" t="inlineStr">
         <is>
-          <t>Basset no.98, pp.233–252, places the Swahili tradition in the Zanzibar region and cites Velten’s 1898 Swahili text, pp.110–119, and German version, pp.178–191.</t>
+          <t>Official lyric video with English translation, on Diamond Platnumz's YouTube channel.</t>
         </is>
       </c>
       <c r="Z179" s="11" t="inlineStr">
         <is>
-          <t>Work / source text</t>
-        </is>
-      </c>
-      <c r="AA179" s="11" t="inlineStr">
-        <is>
-          <t>Reuse basis / copyright duration</t>
-        </is>
-      </c>
-      <c r="AB179" s="11" t="inlineStr">
-        <is>
-          <t>Date / edition evidence</t>
-        </is>
-      </c>
-      <c r="AC179" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country evidence</t>
-        </is>
-      </c>
-      <c r="AD179" s="11" t="inlineStr">
-        <is>
-          <t>Additional evidence</t>
-        </is>
-      </c>
-      <c r="AE179" s="11" t="n"/>
+          <t>Watch the video</t>
+        </is>
+      </c>
+      <c r="AA179" s="11" t="n"/>
+      <c r="AB179" s="11" t="n"/>
+      <c r="AC179" s="11" t="n"/>
+      <c r="AD179" s="11" t="n"/>
+      <c r="AE179" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: https://fr.wikisource.org/wiki/Contes_populaires_d’Afrique_(Basset)/98</t>
+        </is>
+      </c>
     </row>
     <row r="180" ht="108" customHeight="1" s="17">
       <c r="A180" s="7" t="inlineStr">
@@ -27186,34 +27093,34 @@
       </c>
       <c r="D183" s="13" t="inlineStr">
         <is>
-          <t>The lovers in the cavern of Hoonga (episode identifier)</t>
+          <t>Ka Ta'e Feunga E Po Koe</t>
         </is>
       </c>
       <c r="E183" s="13" t="inlineStr">
         <is>
-          <t>The lovers in the cavern of Hoonga (episode identifier)</t>
+          <t>Ka Ta'e Feunga E Po Koe</t>
         </is>
       </c>
       <c r="F183" s="13" t="n"/>
       <c r="G183" s="13" t="n"/>
       <c r="H183" s="13" t="inlineStr">
         <is>
-          <t>Unnamed Tongan narrator (an elderly matabule), recorded by William Mariner; compiled by John Martin</t>
+          <t>Tongan love song</t>
         </is>
       </c>
       <c r="I183" s="13" t="inlineStr">
         <is>
-          <t>Historical version only</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J183" s="13" t="inlineStr">
         <is>
-          <t>Identified oral-tale episode (full historical text)</t>
+          <t>Named work</t>
         </is>
       </c>
       <c r="K183" s="13" t="inlineStr">
         <is>
-          <t>Oral tale</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="L183" s="13" t="inlineStr">
@@ -27221,87 +27128,73 @@
           <t>Unknown</t>
         </is>
       </c>
-      <c r="M183" s="14" t="n">
-        <v>1817</v>
+      <c r="M183" s="14" t="inlineStr">
+        <is>
+          <t>c. 2018</t>
+        </is>
       </c>
       <c r="N183" s="13" t="inlineStr">
         <is>
-          <t>Tongan tradition; historical English version</t>
+          <t>Tongan</t>
         </is>
       </c>
       <c r="O183" s="13" t="n"/>
       <c r="P183" s="13" t="inlineStr">
         <is>
-          <t>Oral tale</t>
+          <t>Love song</t>
         </is>
       </c>
       <c r="Q183" s="13" t="inlineStr">
         <is>
-          <t>Traditional composer / storyteller unknown; see creator and version notes</t>
+          <t>Singer not named in the upload</t>
         </is>
       </c>
       <c r="R183" s="13" t="inlineStr">
         <is>
-          <t>Recorded during Mariner’s residence, 1806–1810; English account published 1817</t>
-        </is>
-      </c>
-      <c r="S183" s="13" t="inlineStr">
-        <is>
-          <t>An Account of the Natives of the Tonga Islands, vol.I, chapter IX; also later editions</t>
-        </is>
-      </c>
+          <t>c. 2018</t>
+        </is>
+      </c>
+      <c r="S183" s="13" t="n"/>
       <c r="T183" s="13" t="inlineStr">
         <is>
-          <t>A young chief rescues a woman from a tyrant and hides her in a sea cave. They confess mutual love, flee to Fiji, then return to Tonga and live happily.</t>
+          <t>A Tongan love song, one of the many sung across the islands and the diaspora.</t>
         </is>
       </c>
       <c r="U183" s="13" t="inlineStr">
         <is>
-          <t>John Martin’s 1817 Account from Mariner’s communications, chapter IX. The narrator is identified as an old matabule. Hoonga is Hunga in the Vavaʻu group, Tonga.</t>
-        </is>
-      </c>
-      <c r="V183" s="13" t="inlineStr">
-        <is>
-          <t>Chapter IX, discovery of Hoonga cavern and the lovers’ escape; search for How happy were they</t>
-        </is>
-      </c>
+          <t>YouTube upload in a collection of Tongan love songs.</t>
+        </is>
+      </c>
+      <c r="V183" s="13" t="n"/>
       <c r="W183" s="13" t="inlineStr">
         <is>
-          <t>No standalone native title is supplied; the work column gives a descriptive episode identifier. Only the published historical English wording is established as reusable. A Tongan-language transcript is not supplied. Mariner and Martin are recorders, not the original traditional creators.</t>
+          <t>Work changed (30 October 2026) after the sensitivity review: William Mariner's 1817 account, written by an English outsider, is replaced by a love song in Tongan.</t>
         </is>
       </c>
       <c r="X183" s="13" t="inlineStr">
         <is>
-          <t>Reusable historical English text: published 1817, with nineteenth-century recorders. Native-language wording, modern retellings, recordings and community permissions are not covered.</t>
+          <t>In copyright: described and linked only; no text or recording is reproduced here. Sensitivity review, 30 October 2026.</t>
         </is>
       </c>
       <c r="Y183" s="13" t="inlineStr">
         <is>
-          <t>Work-specific text, date and provenance sources checked29October2026.</t>
+          <t>YouTube upload in a collection of Tongan love songs.</t>
         </is>
       </c>
       <c r="Z183" s="11" t="inlineStr">
         <is>
-          <t>Work / text</t>
-        </is>
-      </c>
-      <c r="AA183" s="11" t="inlineStr">
-        <is>
-          <t>Rights / catalogue</t>
-        </is>
-      </c>
-      <c r="AB183" s="11" t="inlineStr">
-        <is>
-          <t>Date / edition</t>
-        </is>
-      </c>
-      <c r="AC183" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country</t>
-        </is>
-      </c>
+          <t>Listen to the song</t>
+        </is>
+      </c>
+      <c r="AA183" s="11" t="n"/>
+      <c r="AB183" s="11" t="n"/>
+      <c r="AC183" s="11" t="n"/>
       <c r="AD183" s="11" t="n"/>
-      <c r="AE183" s="11" t="n"/>
+      <c r="AE183" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: https://darwin-online.org.uk/converted/Ancillary/BeagleLibrary/1817_Mariner_A710.01.html</t>
+        </is>
+      </c>
     </row>
     <row r="184" ht="91.5" customHeight="1" s="17">
       <c r="A184" s="7" t="inlineStr">
@@ -27674,85 +27567,57 @@
       </c>
       <c r="D186" s="13" t="inlineStr">
         <is>
-          <t>Աչքերդ (Achkerd / Your eyes)</t>
+          <t>Ela Gözlü Nazlı Dilber</t>
         </is>
       </c>
       <c r="E186" s="13" t="inlineStr">
         <is>
-          <t>Your Eyes</t>
+          <t>Hazel-Eyed, Coy Beauty</t>
         </is>
       </c>
       <c r="F186" s="13" t="inlineStr">
         <is>
-          <t>Ծով մը կապույտ կծավալի
-Աչքերուդ մեջ, ուր չըկա սեր,
-Ծով մը հանդարտ, ըզմայլելի,
-Ուր կը ցոլան ցայտուն լույսեր․
-Բայց ըզգացումն հոն կհալի,
-Ինչպես տաքին՝ պատառ մը սեր։
-Երբեմն անկե կանցնին բարակ
-Ճառագայթներ պայծառ ու ջինջ,
-Ջըղուտ հոգվույդ ցոլքեր կըրակ
-Երևույթով մ'աղվոր, անջինջ․
-Բայց կմարին անոնք արագ,
-Ինչպես հովին դեմ կայծ մ'ոչինչ։
-Մերթ ծաղիկներ կըլլան փափուկ
-Գորշ կապույտով մանուշակին,
-Այնքան նըրբին և խուսափուկ,
-Որ չունին գույն որոշակի․
-Բայց կթափին ինչպես հափուկ
-Դաժան շունչին դեմ խորշակի։
-Օր մ'ալ տեսնես շատ են հոգներ
-Մեծ թախծի խոհով մ'անանց․
-Արցունքներու տակ կայլակներ
-Թարթիչներեդ կմաղվին թաց,
-Որ կթըվին սև ժանյակներ
-Գոհարներու շարքով բանված։
-Աշխարհներ են աչքերդ անհուն,
-Ուր կան լույսեր, հույզեր հըսկա․
-Սառույց, հըրդեհ, բոցեր փայլուն,
-Ժըպիտն ու հույս չեն բացակա․
-Կուգան, կանցնին անկե սահուն
-Գութն ու արցունք, լոկ սեր չըկա։</t>
+          <t>Ela gözlü nazlı dilber
+Koma beni el yerine
+Altın kemerin olayım
+Dola beni bel yerine
+Hecine gönlüm hecine
+Yiğide ölüm gecine
+Al beni zülfün ucuna
+Sallanayım tel yerine
+Gel kız karşımda dursana
+Şu benim halim sorsana
+Zülfünden bir tel versene
+Koklıyayım gül yerine
+Karac'oğlan der n'olayım
+Kolun boynuma dolayım
+Nazlı yar kölen olayım
+Kabul eyle kul yerine</t>
         </is>
       </c>
       <c r="G186" s="13" t="inlineStr">
         <is>
-          <t>A blue sea spreads
-within your eyes, where there is no love,
-a calm sea, enchanting,
-where bright lights glitter;
-but feeling melts away there
-like a scrap of cream in the heat.
-Sometimes slender rays pass across it,
-bright and clear,
-flashes of fire from your nervous soul,
-lovely and unforgettable to see;
-but they go out quickly,
-like a feeble spark against the wind.
-At times they become soft flowers
-with the grey-blue of the violet,
-so delicate and elusive
-that they have no definite colour;
-but they scatter like petals
-before the cruel breath of the scorching wind.
-Another day you see them weary
-with the endless thought of a great sadness;
-under the tears, drops
-sift wet through your lashes,
-so that they look like black lace
-worked with a row of jewels.
-Your eyes are boundless worlds,
-with lights and vast emotions in them;
-ice, conflagration, shining flames,
-smiles and hope are not absent;
-pity and tears come and pass through them smoothly:
-only love is not there.</t>
+          <t>Hazel-eyed, coy beauty,
+don't treat me like a stranger;
+let me be your golden belt,
+wind me round your waist.
+My heart runs like a racing camel;
+a brave lad dies of it by night;
+take me to the tip of your lock of hair,
+let me swing there like a strand.
+Come, girl, stand before me,
+ask me how I am;
+give me one strand of your hair,
+let me smell it as I would a rose.
+Karacaoğlan says: what am I to do?
+Let me wind your arm round my neck;
+coy darling, let me be your slave,
+take me as your servant.</t>
         </is>
       </c>
       <c r="H186" s="13" t="inlineStr">
         <is>
-          <t>Sibil (Zabel Asadour)</t>
+          <t>Karacaoğlan (17th century)</t>
         </is>
       </c>
       <c r="I186" s="13" t="inlineStr">
@@ -27762,7 +27627,7 @@
       </c>
       <c r="J186" s="13" t="inlineStr">
         <is>
-          <t>Named work</t>
+          <t>Named poem (original text)</t>
         </is>
       </c>
       <c r="K186" s="13" t="inlineStr">
@@ -27772,46 +27637,48 @@
       </c>
       <c r="L186" s="13" t="inlineStr">
         <is>
-          <t>Women</t>
-        </is>
-      </c>
-      <c r="M186" s="14" t="n">
-        <v>1892</v>
+          <t>Men</t>
+        </is>
+      </c>
+      <c r="M186" s="14" t="inlineStr">
+        <is>
+          <t>c. 1650</t>
+        </is>
       </c>
       <c r="N186" s="13" t="inlineStr">
         <is>
-          <t>Western Armenian</t>
-        </is>
-      </c>
-      <c r="O186" s="13" t="n"/>
+          <t>Turkish</t>
+        </is>
+      </c>
+      <c r="O186" s="13" t="inlineStr">
+        <is>
+          <t>Âşık poetry</t>
+        </is>
+      </c>
       <c r="P186" s="13" t="inlineStr">
         <is>
-          <t>Poem</t>
+          <t>Türkü (folk poem, 4 quatrains)</t>
         </is>
       </c>
       <c r="Q186" s="13" t="inlineStr">
         <is>
-          <t>Woman</t>
+          <t>Karacaoğlan</t>
         </is>
       </c>
       <c r="R186" s="13" t="inlineStr">
         <is>
-          <t>1892 (date printed under the poem)</t>
-        </is>
-      </c>
-      <c r="S186" s="13" t="inlineStr">
-        <is>
-          <t>1965 collected edition; linked online transcription</t>
-        </is>
-      </c>
+          <t>17th century</t>
+        </is>
+      </c>
+      <c r="S186" s="13" t="n"/>
       <c r="T186" s="13" t="inlineStr">
         <is>
-          <t>Admiration mixed with unrequited love: the beloved’s eyes hold many emotions but no love for the speaker.</t>
+          <t>The poet begs his hazel-eyed beloved not to treat him as a stranger: he would be her golden belt, a strand of her hair, her servant.</t>
         </is>
       </c>
       <c r="U186" s="13" t="inlineStr">
         <is>
-          <t>Sibil, Banasteghtsutyunner (1965 collection), p. 32; author is a woman from Istanbul</t>
+          <t>Traditional text of Karacaoğlan's türkü, as given on Turkish Wikisource; sung widely in Turkey to this day.</t>
         </is>
       </c>
       <c r="V186" s="13" t="inlineStr">
@@ -27821,39 +27688,33 @@
       </c>
       <c r="W186" s="13" t="inlineStr">
         <is>
-          <t>Country is geographic: an Ottoman Armenian writer born and active in Istanbul, now Turkey; this is Armenian-language literature, not a claim of ethnic Turkish identity. 1965 editorial material and modern translations are separate.
-Passage update (29 October 2026): Complete poem, 30 lines (Armenian Wikisource; dated 1892). Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
+          <t>Work changed (30 October 2026) after the sensitivity review: Sibil's Armenian-language poem is replaced by a love poem in Turkish by the best-loved of the wandering folk poets of Anatolia. Complete poem, 16 lines. Fresh English translation by Claude (Anthropic AI) made directly from the original; draft for editorial review. Lines 5–6 (hecin, a racing camel; 'yiğide ölüm gecine') are idiomatic and the English is tentative.</t>
         </is>
       </c>
       <c r="X186" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original in life+70 jurisdictions (author died 1934)
-Anthology review (30 October 2026): Sibil died 1934; the poet died before 1956 (UK/EU public domain); in the US, whatever the date of first publication, the poem was already out of copyright at home on 1 January 1996, so US copyright was never restored.</t>
-        </is>
-      </c>
-      <c r="Y186" s="13" t="n"/>
+          <t>Sensitivity review (30 October 2026): 17th-century folk poem, transmitted orally and in print for centuries; public domain in the UK, EU and US. The online text is a transcription with no new authorship.</t>
+        </is>
+      </c>
+      <c r="Y186" s="13" t="inlineStr">
+        <is>
+          <t>Turkish Wikisource: Ela Gözlü Nazlı Dilber (Karacaoğlan)</t>
+        </is>
+      </c>
       <c r="Z186" s="11" t="inlineStr">
         <is>
-          <t>Read text</t>
-        </is>
-      </c>
-      <c r="AA186" s="11" t="inlineStr">
-        <is>
-          <t>Rights / catalogue</t>
-        </is>
-      </c>
-      <c r="AB186" s="11" t="inlineStr">
-        <is>
-          <t>Date evidence</t>
-        </is>
-      </c>
-      <c r="AC186" s="11" t="inlineStr">
-        <is>
-          <t>Author / country</t>
-        </is>
-      </c>
+          <t>Read the whole work</t>
+        </is>
+      </c>
+      <c r="AA186" s="11" t="n"/>
+      <c r="AB186" s="11" t="n"/>
+      <c r="AC186" s="11" t="n"/>
       <c r="AD186" s="11" t="n"/>
-      <c r="AE186" s="11" t="n"/>
+      <c r="AE186" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: https://hy.wikisource.org/wiki/Աչքերդ</t>
+        </is>
+      </c>
     </row>
     <row r="187" ht="43.5" customHeight="1" s="17">
       <c r="A187" s="7" t="inlineStr">
@@ -30155,554 +30016,532 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD44" r:id="rId127"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE44" r:id="rId128"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z45" r:id="rId129"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA45" r:id="rId130"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB45" r:id="rId131"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC45" r:id="rId132"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD45" r:id="rId133"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z46" r:id="rId134"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA46" r:id="rId135"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB46" r:id="rId136"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC46" r:id="rId137"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z47" r:id="rId138"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD47" r:id="rId139"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE47" r:id="rId140"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z48" r:id="rId141"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA48" r:id="rId142"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB48" r:id="rId143"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC48" r:id="rId144"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z49" r:id="rId145"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA49" r:id="rId146"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB49" r:id="rId147"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC49" r:id="rId148"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z50" r:id="rId149"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA50" r:id="rId150"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB50" r:id="rId151"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC50" r:id="rId152"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z51" r:id="rId153"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA51" r:id="rId154"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB51" r:id="rId155"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC51" r:id="rId156"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z52" r:id="rId157"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z53" r:id="rId158"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA53" r:id="rId159"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB53" r:id="rId160"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC53" r:id="rId161"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD53" r:id="rId162"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE53" r:id="rId163"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z54" r:id="rId164"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE54" r:id="rId165"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z55" r:id="rId166"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE55" r:id="rId167"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z56" r:id="rId168"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA56" r:id="rId169"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB56" r:id="rId170"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC56" r:id="rId171"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z57" r:id="rId172"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA57" r:id="rId173"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB57" r:id="rId174"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC57" r:id="rId175"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z58" r:id="rId176"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA58" r:id="rId177"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB58" r:id="rId178"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC58" r:id="rId179"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z59" r:id="rId180"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA59" r:id="rId181"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB59" r:id="rId182"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC59" r:id="rId183"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z60" r:id="rId184"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z61" r:id="rId185"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z62" r:id="rId186"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA62" r:id="rId187"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB62" r:id="rId188"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC62" r:id="rId189"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z63" r:id="rId190"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE63" r:id="rId191"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z64" r:id="rId192"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA64" r:id="rId193"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB64" r:id="rId194"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC64" r:id="rId195"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE64" r:id="rId196"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z65" r:id="rId197"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE65" r:id="rId198"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z66" r:id="rId199"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA66" r:id="rId200"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB66" r:id="rId201"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC66" r:id="rId202"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z67" r:id="rId203"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA67" r:id="rId204"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB67" r:id="rId205"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC67" r:id="rId206"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z68" r:id="rId207"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE68" r:id="rId208"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z69" r:id="rId209"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE69" r:id="rId210"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z70" r:id="rId211"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA70" r:id="rId212"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB70" r:id="rId213"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC70" r:id="rId214"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z71" r:id="rId215"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA71" r:id="rId216"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB71" r:id="rId217"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC71" r:id="rId218"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z72" r:id="rId219"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA72" r:id="rId220"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB72" r:id="rId221"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC72" r:id="rId222"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD72" r:id="rId223"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z73" r:id="rId224"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA73" r:id="rId225"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB73" r:id="rId226"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC73" r:id="rId227"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z74" r:id="rId228"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD74" r:id="rId229"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE74" r:id="rId230"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z75" r:id="rId231"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA75" r:id="rId232"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB75" r:id="rId233"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC75" r:id="rId234"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z76" r:id="rId235"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE76" r:id="rId236"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z77" r:id="rId237"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z78" r:id="rId238"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA78" r:id="rId239"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB78" r:id="rId240"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC78" r:id="rId241"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD78" r:id="rId242"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z79" r:id="rId243"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA79" r:id="rId244"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB79" r:id="rId245"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC79" r:id="rId246"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z80" r:id="rId247"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA80" r:id="rId248"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB80" r:id="rId249"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC80" r:id="rId250"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD80" r:id="rId251"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE80" r:id="rId252"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z81" r:id="rId253"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA81" r:id="rId254"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB81" r:id="rId255"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC81" r:id="rId256"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE81" r:id="rId257"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z82" r:id="rId258"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA82" r:id="rId259"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB82" r:id="rId260"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC82" r:id="rId261"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE82" r:id="rId262"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z83" r:id="rId263"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA83" r:id="rId264"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB83" r:id="rId265"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC83" r:id="rId266"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD83" r:id="rId267"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE83" r:id="rId268"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId269"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA84" r:id="rId270"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB84" r:id="rId271"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC84" r:id="rId272"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId273"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA85" r:id="rId274"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB85" r:id="rId275"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC85" r:id="rId276"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId277"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA86" r:id="rId278"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB86" r:id="rId279"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC86" r:id="rId280"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId281"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA87" r:id="rId282"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB87" r:id="rId283"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC87" r:id="rId284"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId285"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA88" r:id="rId286"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB88" r:id="rId287"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC88" r:id="rId288"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId289"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA89" r:id="rId290"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB89" r:id="rId291"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC89" r:id="rId292"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId293"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA90" r:id="rId294"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB90" r:id="rId295"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC90" r:id="rId296"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD90" r:id="rId297"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE90" r:id="rId298"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId299"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA91" r:id="rId300"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB91" r:id="rId301"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC91" r:id="rId302"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId303"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA92" r:id="rId304"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB92" r:id="rId305"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC92" r:id="rId306"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD92" r:id="rId307"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE92" r:id="rId308"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId309"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA93" r:id="rId310"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB93" r:id="rId311"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC93" r:id="rId312"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE93" r:id="rId313"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId314"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA94" r:id="rId315"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB94" r:id="rId316"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC94" r:id="rId317"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId318"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE95" r:id="rId319"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId320"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId321"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA97" r:id="rId322"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB97" r:id="rId323"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC97" r:id="rId324"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId325"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA98" r:id="rId326"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB98" r:id="rId327"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC98" r:id="rId328"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId329"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId330"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA100" r:id="rId331"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB100" r:id="rId332"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC100" r:id="rId333"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId334"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA101" r:id="rId335"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB101" r:id="rId336"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC101" r:id="rId337"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId338"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId339"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA103" r:id="rId340"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB103" r:id="rId341"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC103" r:id="rId342"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD103" r:id="rId343"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId344"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA104" r:id="rId345"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB104" r:id="rId346"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC104" r:id="rId347"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId348"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA105" r:id="rId349"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB105" r:id="rId350"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC105" r:id="rId351"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD105" r:id="rId352"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId353"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA106" r:id="rId354"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB106" r:id="rId355"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC106" r:id="rId356"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId357"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId358"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId359"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE109" r:id="rId360"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId361"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA110" r:id="rId362"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB110" r:id="rId363"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC110" r:id="rId364"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE110" r:id="rId365"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId366"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD111" r:id="rId367"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId368"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE112" r:id="rId369"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId370"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA113" r:id="rId371"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB113" r:id="rId372"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC113" r:id="rId373"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId374"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z115" r:id="rId375"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA115" r:id="rId376"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB115" r:id="rId377"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC115" r:id="rId378"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z116" r:id="rId379"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE116" r:id="rId380"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z117" r:id="rId381"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA117" r:id="rId382"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB117" r:id="rId383"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC117" r:id="rId384"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z118" r:id="rId385"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE118" r:id="rId386"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z119" r:id="rId387"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA119" r:id="rId388"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB119" r:id="rId389"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC119" r:id="rId390"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z120" r:id="rId391"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD120" r:id="rId392"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE120" r:id="rId393"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z121" r:id="rId394"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA121" r:id="rId395"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB121" r:id="rId396"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC121" r:id="rId397"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD121" r:id="rId398"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z122" r:id="rId399"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA122" r:id="rId400"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB122" r:id="rId401"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC122" r:id="rId402"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z123" r:id="rId403"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA123" r:id="rId404"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB123" r:id="rId405"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC123" r:id="rId406"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE123" r:id="rId407"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z124" r:id="rId408"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA124" r:id="rId409"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB124" r:id="rId410"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC124" r:id="rId411"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD124" r:id="rId412"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z125" r:id="rId413"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z126" r:id="rId414"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE126" r:id="rId415"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z127" r:id="rId416"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA127" r:id="rId417"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB127" r:id="rId418"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC127" r:id="rId419"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD127" r:id="rId420"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z128" r:id="rId421"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA128" r:id="rId422"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB128" r:id="rId423"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC128" r:id="rId424"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z129" r:id="rId425"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA129" r:id="rId426"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB129" r:id="rId427"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC129" r:id="rId428"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z130" r:id="rId429"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA130" r:id="rId430"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB130" r:id="rId431"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC130" r:id="rId432"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z131" r:id="rId433"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA131" r:id="rId434"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB131" r:id="rId435"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC131" r:id="rId436"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z132" r:id="rId437"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE132" r:id="rId438"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z133" r:id="rId439"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE133" r:id="rId440"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z134" r:id="rId441"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA134" r:id="rId442"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB134" r:id="rId443"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC134" r:id="rId444"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z135" r:id="rId445"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA135" r:id="rId446"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB135" r:id="rId447"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC135" r:id="rId448"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z136" r:id="rId449"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA136" r:id="rId450"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB136" r:id="rId451"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC136" r:id="rId452"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z137" r:id="rId453"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA137" r:id="rId454"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB137" r:id="rId455"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC137" r:id="rId456"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE137" r:id="rId457"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z138" r:id="rId458"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA138" r:id="rId459"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB138" r:id="rId460"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC138" r:id="rId461"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z139" r:id="rId462"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z140" r:id="rId463"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA140" r:id="rId464"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB140" r:id="rId465"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC140" r:id="rId466"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE140" r:id="rId467"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z141" r:id="rId468"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA141" r:id="rId469"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB141" r:id="rId470"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC141" r:id="rId471"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z142" r:id="rId472"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE142" r:id="rId473"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z143" r:id="rId474"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA143" r:id="rId475"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB143" r:id="rId476"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC143" r:id="rId477"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z144" r:id="rId478"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA144" r:id="rId479"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB144" r:id="rId480"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC144" r:id="rId481"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z145" r:id="rId482"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA145" r:id="rId483"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB145" r:id="rId484"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC145" r:id="rId485"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z146" r:id="rId486"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA146" r:id="rId487"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB146" r:id="rId488"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC146" r:id="rId489"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z147" r:id="rId490"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA147" r:id="rId491"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB147" r:id="rId492"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC147" r:id="rId493"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z148" r:id="rId494"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA148" r:id="rId495"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB148" r:id="rId496"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC148" r:id="rId497"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z149" r:id="rId498"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA149" r:id="rId499"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB149" r:id="rId500"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC149" r:id="rId501"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z150" r:id="rId502"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA150" r:id="rId503"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB150" r:id="rId504"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC150" r:id="rId505"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD150" r:id="rId506"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE150" r:id="rId507"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z151" r:id="rId508"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD151" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE151" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z152" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE152" r:id="rId512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z153" r:id="rId513"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z154" r:id="rId514"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE154" r:id="rId515"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z155" r:id="rId516"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z156" r:id="rId517"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z157" r:id="rId518"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA157" r:id="rId519"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB157" r:id="rId520"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC157" r:id="rId521"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD157" r:id="rId522"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z158" r:id="rId523"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA158" r:id="rId524"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB158" r:id="rId525"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC158" r:id="rId526"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z159" r:id="rId527"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z160" r:id="rId528"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA160" r:id="rId529"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB160" r:id="rId530"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC160" r:id="rId531"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z161" r:id="rId532"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE161" r:id="rId533"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z162" r:id="rId534"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE162" r:id="rId535"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z163" r:id="rId536"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA163" r:id="rId537"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB163" r:id="rId538"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC163" r:id="rId539"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD163" r:id="rId540"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE163" r:id="rId541"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z164" r:id="rId542"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA164" r:id="rId543"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB164" r:id="rId544"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC164" r:id="rId545"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z165" r:id="rId546"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA165" r:id="rId547"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB165" r:id="rId548"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC165" r:id="rId549"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z166" r:id="rId550"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z167" r:id="rId551"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA167" r:id="rId552"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB167" r:id="rId553"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC167" r:id="rId554"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD167" r:id="rId555"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE167" r:id="rId556"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z168" r:id="rId557"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA168" r:id="rId558"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB168" r:id="rId559"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC168" r:id="rId560"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z169" r:id="rId561"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA169" r:id="rId562"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB169" r:id="rId563"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC169" r:id="rId564"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z170" r:id="rId565"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z171" r:id="rId566"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA171" r:id="rId567"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB171" r:id="rId568"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC171" r:id="rId569"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z172" r:id="rId570"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA172" r:id="rId571"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB172" r:id="rId572"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC172" r:id="rId573"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD172" r:id="rId574"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE172" r:id="rId575"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z173" r:id="rId576"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z174" r:id="rId577"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z175" r:id="rId578"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA175" r:id="rId579"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB175" r:id="rId580"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC175" r:id="rId581"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z176" r:id="rId582"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA176" r:id="rId583"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB176" r:id="rId584"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC176" r:id="rId585"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z177" r:id="rId586"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA177" r:id="rId587"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB177" r:id="rId588"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC177" r:id="rId589"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z178" r:id="rId590"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA178" r:id="rId591"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB178" r:id="rId592"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC178" r:id="rId593"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z179" r:id="rId594"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA179" r:id="rId595"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB179" r:id="rId596"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC179" r:id="rId597"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD179" r:id="rId598"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z180" r:id="rId599"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA180" r:id="rId600"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB180" r:id="rId601"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC180" r:id="rId602"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z181" r:id="rId603"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE181" r:id="rId604"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z182" r:id="rId605"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD182" r:id="rId606"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z183" r:id="rId607"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA183" r:id="rId608"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB183" r:id="rId609"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC183" r:id="rId610"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z184" r:id="rId611"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA184" r:id="rId612"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB184" r:id="rId613"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC184" r:id="rId614"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD184" r:id="rId615"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z185" r:id="rId616"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA185" r:id="rId617"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB185" r:id="rId618"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC185" r:id="rId619"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD185" r:id="rId620"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z186" r:id="rId621"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA186" r:id="rId622"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB186" r:id="rId623"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC186" r:id="rId624"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z187" r:id="rId625"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z188" r:id="rId626"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z189" r:id="rId627"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE189" r:id="rId628"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z190" r:id="rId629"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA190" r:id="rId630"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB190" r:id="rId631"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC190" r:id="rId632"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD190" r:id="rId633"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z191" r:id="rId634"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD191" r:id="rId635"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE191" r:id="rId636"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z192" r:id="rId637"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA192" r:id="rId638"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB192" r:id="rId639"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC192" r:id="rId640"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z193" r:id="rId641"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA193" r:id="rId642"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB193" r:id="rId643"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC193" r:id="rId644"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z194" r:id="rId645"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA194" r:id="rId646"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB194" r:id="rId647"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC194" r:id="rId648"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z195" r:id="rId649"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA195" r:id="rId650"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB195" r:id="rId651"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC195" r:id="rId652"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z196" r:id="rId653"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA196" r:id="rId654"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB196" r:id="rId655"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC196" r:id="rId656"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z197" r:id="rId657"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA197" r:id="rId658"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB197" r:id="rId659"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC197" r:id="rId660"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z198" r:id="rId661"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA198" r:id="rId662"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB198" r:id="rId663"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC198" r:id="rId664"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE198" r:id="rId665"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z199" r:id="rId666"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA199" r:id="rId667"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB199" r:id="rId668"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC199" r:id="rId669"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE199" r:id="rId670"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z200" r:id="rId671"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z201" r:id="rId672"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE201" r:id="rId673"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z46" r:id="rId130"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA46" r:id="rId131"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB46" r:id="rId132"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC46" r:id="rId133"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z47" r:id="rId134"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD47" r:id="rId135"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE47" r:id="rId136"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z48" r:id="rId137"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA48" r:id="rId138"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB48" r:id="rId139"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC48" r:id="rId140"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z49" r:id="rId141"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA49" r:id="rId142"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB49" r:id="rId143"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC49" r:id="rId144"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z50" r:id="rId145"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA50" r:id="rId146"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB50" r:id="rId147"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC50" r:id="rId148"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z51" r:id="rId149"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA51" r:id="rId150"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB51" r:id="rId151"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC51" r:id="rId152"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z52" r:id="rId153"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z53" r:id="rId154"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA53" r:id="rId155"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB53" r:id="rId156"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC53" r:id="rId157"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD53" r:id="rId158"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE53" r:id="rId159"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z54" r:id="rId160"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE54" r:id="rId161"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z55" r:id="rId162"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE55" r:id="rId163"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z56" r:id="rId164"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA56" r:id="rId165"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB56" r:id="rId166"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC56" r:id="rId167"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z57" r:id="rId168"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA57" r:id="rId169"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB57" r:id="rId170"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC57" r:id="rId171"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z58" r:id="rId172"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA58" r:id="rId173"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB58" r:id="rId174"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC58" r:id="rId175"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z59" r:id="rId176"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA59" r:id="rId177"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB59" r:id="rId178"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC59" r:id="rId179"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z60" r:id="rId180"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z61" r:id="rId181"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z62" r:id="rId182"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA62" r:id="rId183"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB62" r:id="rId184"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC62" r:id="rId185"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z63" r:id="rId186"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE63" r:id="rId187"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z64" r:id="rId188"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA64" r:id="rId189"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB64" r:id="rId190"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC64" r:id="rId191"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE64" r:id="rId192"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z65" r:id="rId193"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE65" r:id="rId194"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z66" r:id="rId195"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA66" r:id="rId196"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB66" r:id="rId197"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC66" r:id="rId198"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z67" r:id="rId199"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA67" r:id="rId200"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB67" r:id="rId201"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC67" r:id="rId202"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z68" r:id="rId203"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE68" r:id="rId204"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z69" r:id="rId205"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE69" r:id="rId206"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z70" r:id="rId207"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA70" r:id="rId208"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB70" r:id="rId209"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC70" r:id="rId210"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z71" r:id="rId211"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA71" r:id="rId212"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB71" r:id="rId213"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC71" r:id="rId214"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z72" r:id="rId215"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA72" r:id="rId216"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB72" r:id="rId217"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC72" r:id="rId218"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD72" r:id="rId219"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z73" r:id="rId220"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA73" r:id="rId221"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB73" r:id="rId222"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC73" r:id="rId223"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z74" r:id="rId224"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD74" r:id="rId225"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE74" r:id="rId226"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z75" r:id="rId227"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA75" r:id="rId228"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB75" r:id="rId229"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC75" r:id="rId230"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z76" r:id="rId231"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE76" r:id="rId232"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z77" r:id="rId233"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z78" r:id="rId234"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z79" r:id="rId235"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA79" r:id="rId236"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB79" r:id="rId237"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC79" r:id="rId238"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z80" r:id="rId239"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA80" r:id="rId240"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB80" r:id="rId241"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC80" r:id="rId242"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD80" r:id="rId243"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE80" r:id="rId244"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z81" r:id="rId245"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA81" r:id="rId246"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB81" r:id="rId247"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC81" r:id="rId248"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE81" r:id="rId249"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z82" r:id="rId250"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA82" r:id="rId251"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB82" r:id="rId252"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC82" r:id="rId253"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE82" r:id="rId254"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z83" r:id="rId255"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA83" r:id="rId256"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB83" r:id="rId257"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC83" r:id="rId258"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD83" r:id="rId259"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE83" r:id="rId260"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z84" r:id="rId261"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA84" r:id="rId262"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB84" r:id="rId263"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC84" r:id="rId264"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z85" r:id="rId265"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA85" r:id="rId266"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB85" r:id="rId267"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC85" r:id="rId268"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z86" r:id="rId269"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA86" r:id="rId270"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB86" r:id="rId271"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC86" r:id="rId272"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z87" r:id="rId273"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA87" r:id="rId274"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB87" r:id="rId275"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC87" r:id="rId276"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z88" r:id="rId277"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA88" r:id="rId278"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB88" r:id="rId279"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC88" r:id="rId280"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z89" r:id="rId281"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA89" r:id="rId282"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB89" r:id="rId283"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC89" r:id="rId284"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z90" r:id="rId285"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA90" r:id="rId286"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB90" r:id="rId287"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC90" r:id="rId288"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD90" r:id="rId289"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE90" r:id="rId290"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z91" r:id="rId291"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA91" r:id="rId292"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB91" r:id="rId293"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC91" r:id="rId294"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z92" r:id="rId295"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA92" r:id="rId296"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB92" r:id="rId297"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC92" r:id="rId298"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD92" r:id="rId299"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE92" r:id="rId300"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z93" r:id="rId301"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA93" r:id="rId302"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB93" r:id="rId303"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC93" r:id="rId304"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE93" r:id="rId305"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z94" r:id="rId306"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA94" r:id="rId307"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB94" r:id="rId308"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC94" r:id="rId309"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z95" r:id="rId310"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE95" r:id="rId311"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z96" r:id="rId312"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z97" r:id="rId313"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA97" r:id="rId314"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB97" r:id="rId315"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC97" r:id="rId316"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z98" r:id="rId317"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA98" r:id="rId318"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB98" r:id="rId319"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC98" r:id="rId320"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z99" r:id="rId321"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z100" r:id="rId322"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA100" r:id="rId323"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB100" r:id="rId324"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC100" r:id="rId325"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z101" r:id="rId326"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA101" r:id="rId327"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB101" r:id="rId328"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC101" r:id="rId329"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z102" r:id="rId330"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z103" r:id="rId331"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA103" r:id="rId332"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB103" r:id="rId333"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC103" r:id="rId334"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD103" r:id="rId335"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z104" r:id="rId336"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA104" r:id="rId337"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB104" r:id="rId338"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC104" r:id="rId339"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z105" r:id="rId340"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA105" r:id="rId341"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB105" r:id="rId342"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC105" r:id="rId343"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD105" r:id="rId344"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z106" r:id="rId345"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA106" r:id="rId346"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB106" r:id="rId347"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC106" r:id="rId348"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z107" r:id="rId349"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z108" r:id="rId350"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z109" r:id="rId351"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE109" r:id="rId352"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z110" r:id="rId353"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA110" r:id="rId354"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB110" r:id="rId355"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC110" r:id="rId356"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE110" r:id="rId357"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z111" r:id="rId358"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z112" r:id="rId359"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE112" r:id="rId360"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z113" r:id="rId361"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA113" r:id="rId362"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB113" r:id="rId363"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC113" r:id="rId364"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z114" r:id="rId365"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z115" r:id="rId366"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA115" r:id="rId367"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB115" r:id="rId368"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC115" r:id="rId369"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z116" r:id="rId370"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE116" r:id="rId371"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z117" r:id="rId372"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA117" r:id="rId373"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB117" r:id="rId374"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC117" r:id="rId375"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z118" r:id="rId376"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE118" r:id="rId377"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z119" r:id="rId378"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA119" r:id="rId379"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB119" r:id="rId380"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC119" r:id="rId381"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z120" r:id="rId382"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD120" r:id="rId383"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE120" r:id="rId384"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z121" r:id="rId385"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA121" r:id="rId386"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB121" r:id="rId387"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC121" r:id="rId388"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD121" r:id="rId389"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z122" r:id="rId390"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA122" r:id="rId391"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB122" r:id="rId392"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC122" r:id="rId393"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z123" r:id="rId394"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA123" r:id="rId395"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB123" r:id="rId396"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC123" r:id="rId397"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE123" r:id="rId398"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z124" r:id="rId399"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA124" r:id="rId400"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB124" r:id="rId401"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC124" r:id="rId402"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD124" r:id="rId403"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z125" r:id="rId404"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z126" r:id="rId405"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE126" r:id="rId406"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z127" r:id="rId407"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA127" r:id="rId408"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB127" r:id="rId409"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC127" r:id="rId410"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD127" r:id="rId411"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z128" r:id="rId412"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA128" r:id="rId413"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB128" r:id="rId414"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC128" r:id="rId415"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z129" r:id="rId416"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA129" r:id="rId417"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB129" r:id="rId418"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC129" r:id="rId419"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z130" r:id="rId420"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA130" r:id="rId421"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB130" r:id="rId422"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC130" r:id="rId423"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z131" r:id="rId424"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA131" r:id="rId425"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB131" r:id="rId426"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC131" r:id="rId427"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z132" r:id="rId428"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE132" r:id="rId429"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z133" r:id="rId430"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE133" r:id="rId431"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z134" r:id="rId432"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA134" r:id="rId433"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB134" r:id="rId434"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC134" r:id="rId435"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z135" r:id="rId436"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA135" r:id="rId437"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB135" r:id="rId438"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC135" r:id="rId439"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z136" r:id="rId440"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA136" r:id="rId441"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB136" r:id="rId442"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC136" r:id="rId443"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z137" r:id="rId444"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA137" r:id="rId445"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB137" r:id="rId446"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC137" r:id="rId447"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE137" r:id="rId448"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z138" r:id="rId449"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA138" r:id="rId450"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB138" r:id="rId451"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC138" r:id="rId452"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z139" r:id="rId453"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z140" r:id="rId454"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA140" r:id="rId455"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB140" r:id="rId456"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC140" r:id="rId457"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE140" r:id="rId458"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z141" r:id="rId459"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA141" r:id="rId460"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB141" r:id="rId461"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC141" r:id="rId462"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z142" r:id="rId463"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE142" r:id="rId464"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z143" r:id="rId465"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA143" r:id="rId466"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB143" r:id="rId467"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC143" r:id="rId468"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z144" r:id="rId469"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA144" r:id="rId470"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB144" r:id="rId471"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC144" r:id="rId472"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z145" r:id="rId473"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA145" r:id="rId474"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB145" r:id="rId475"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC145" r:id="rId476"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z146" r:id="rId477"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA146" r:id="rId478"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB146" r:id="rId479"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC146" r:id="rId480"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z147" r:id="rId481"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA147" r:id="rId482"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB147" r:id="rId483"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC147" r:id="rId484"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z148" r:id="rId485"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA148" r:id="rId486"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB148" r:id="rId487"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC148" r:id="rId488"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z149" r:id="rId489"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA149" r:id="rId490"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB149" r:id="rId491"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC149" r:id="rId492"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z150" r:id="rId493"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA150" r:id="rId494"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB150" r:id="rId495"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC150" r:id="rId496"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD150" r:id="rId497"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE150" r:id="rId498"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z151" r:id="rId499"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD151" r:id="rId500"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE151" r:id="rId501"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z152" r:id="rId502"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE152" r:id="rId503"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z153" r:id="rId504"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z154" r:id="rId505"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE154" r:id="rId506"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z155" r:id="rId507"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z156" r:id="rId508"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z157" r:id="rId509"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA157" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB157" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC157" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD157" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z158" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA158" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB158" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC158" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z159" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z160" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA160" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB160" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC160" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z161" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE161" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z162" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE162" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z163" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA163" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB163" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC163" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD163" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE163" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z164" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA164" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB164" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC164" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z165" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA165" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB165" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC165" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z166" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z167" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA167" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB167" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC167" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD167" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE167" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z168" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z169" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA169" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB169" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC169" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z170" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z171" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA171" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB171" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC171" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z172" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA172" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB172" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC172" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD172" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE172" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z173" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z174" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z175" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA175" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB175" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC175" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z176" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA176" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB176" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC176" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z177" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA177" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB177" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC177" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z178" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA178" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB178" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC178" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z179" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z180" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA180" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB180" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC180" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z181" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE181" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z182" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD182" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z183" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z184" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA184" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB184" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC184" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD184" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z185" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA185" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB185" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC185" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD185" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z186" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z187" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z188" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z189" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE189" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z190" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA190" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB190" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC190" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD190" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z191" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD191" r:id="rId613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE191" r:id="rId614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z192" r:id="rId615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA192" r:id="rId616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB192" r:id="rId617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC192" r:id="rId618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z193" r:id="rId619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA193" r:id="rId620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB193" r:id="rId621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC193" r:id="rId622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z194" r:id="rId623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA194" r:id="rId624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB194" r:id="rId625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC194" r:id="rId626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z195" r:id="rId627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA195" r:id="rId628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB195" r:id="rId629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC195" r:id="rId630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z196" r:id="rId631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA196" r:id="rId632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB196" r:id="rId633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC196" r:id="rId634"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z197" r:id="rId635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA197" r:id="rId636"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB197" r:id="rId637"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC197" r:id="rId638"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z198" r:id="rId639"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA198" r:id="rId640"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB198" r:id="rId641"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC198" r:id="rId642"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE198" r:id="rId643"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z199" r:id="rId644"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA199" r:id="rId645"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB199" r:id="rId646"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC199" r:id="rId647"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE199" r:id="rId648"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z200" r:id="rId649"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z201" r:id="rId650"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE201" r:id="rId651"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId674"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId652"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
São Tomé: replace Costa Alegre with Calema's Te Amo
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -23366,80 +23366,34 @@
       </c>
       <c r="D157" s="13" t="inlineStr">
         <is>
-          <t>Serões de São Tomé</t>
+          <t>Te Amo</t>
         </is>
       </c>
       <c r="E157" s="13" t="inlineStr">
         <is>
-          <t>Evenings in São Tomé</t>
-        </is>
-      </c>
-      <c r="F157" s="13" t="inlineStr">
-        <is>
-          <t>Meus olhos são como a noite
-em que astro nenhum flutua
-mas se o teu olhar o fita
-na noite desponta a lua
-Meu olhar é retratista
-ò minha doce miragem
-senão diz-me porque tenho
-no meu peito a tua imagem
-Roubei-te o primeiro beijo
-o segundo foi-me dado
-o terceiro, francamente,
-creio que me foi roubado
-Um dia a espuma dos mares
-ao ver em si meu amor
-Foi dizer baixinho à praia
-– a Vénus mudou de cor
-A nossa terra é tão bela
-duma beleza sem par
-E por ser assim formosa
-Fê-la sua amante o mar…</t>
-        </is>
-      </c>
-      <c r="G157" s="13" t="inlineStr">
-        <is>
-          <t>My eyes are like the night
-in which no star is floating,
-but if your gaze rests on them,
-the moon rises in that night.
-My gaze is a portrait painter,
-O my sweet mirage;
-otherwise tell me why I carry
-your image in my breast.
-I stole the first kiss from you,
-the second was given to me,
-the third, frankly,
-I believe was stolen from me.
-One day the foam of the seas,
-seeing my love reflected in it,
-went and whispered to the shore:
-'Venus has changed her colour.'
-Our land is so lovely,
-of a beauty without equal,
-and because it is so fair
-the sea has made it his lover…</t>
-        </is>
-      </c>
+          <t>I Love You</t>
+        </is>
+      </c>
+      <c r="F157" s="13" t="n"/>
+      <c r="G157" s="13" t="n"/>
       <c r="H157" s="13" t="inlineStr">
         <is>
-          <t>Caetano da Costa Alegre (1864–1890)</t>
+          <t>Calema</t>
         </is>
       </c>
       <c r="I157" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J157" s="13" t="inlineStr">
         <is>
-          <t>Named work (text)</t>
+          <t>Named work</t>
         </is>
       </c>
       <c r="K157" s="13" t="inlineStr">
         <is>
-          <t>Poetry</t>
+          <t>Song</t>
         </is>
       </c>
       <c r="L157" s="13" t="inlineStr">
@@ -23447,8 +23401,10 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M157" s="14" t="n">
-        <v>1916</v>
+      <c r="M157" s="14" t="inlineStr">
+        <is>
+          <t>2020</t>
+        </is>
       </c>
       <c r="N157" s="13" t="inlineStr">
         <is>
@@ -23458,82 +23414,60 @@
       <c r="O157" s="13" t="n"/>
       <c r="P157" s="13" t="inlineStr">
         <is>
-          <t>Lyric poem</t>
+          <t>Love song</t>
         </is>
       </c>
       <c r="Q157" s="13" t="inlineStr">
         <is>
-          <t>Man author</t>
+          <t>António and Fradique Mendes Ferreira</t>
         </is>
       </c>
       <c r="R157" s="13" t="inlineStr">
         <is>
-          <t>Written before 1890; collected posthumously in Versos, 1916</t>
-        </is>
-      </c>
-      <c r="S157" s="13" t="inlineStr">
-        <is>
-          <t>Historical work reproduced in linked digital source; modern editorial material is separate</t>
-        </is>
-      </c>
+          <t>2020</t>
+        </is>
+      </c>
+      <c r="S157" s="13" t="n"/>
       <c r="T157" s="13" t="inlineStr">
         <is>
-          <t>Playful love quatrains: the beloved's gaze makes the moon rise, kisses are stolen and given, the sea foam mistakes her for Venus, and the island itself becomes the sea's lover.</t>
+          <t>A love ballad in which the singer admits he let his beloved down, and asks her to come back because he still loves her.</t>
         </is>
       </c>
       <c r="U157" s="13" t="inlineStr">
         <is>
-          <t>Original poem reproduced in the linked transcription; title and place in Costa Alegre’s work corroborated by UFMG Literafro scholars.</t>
-        </is>
-      </c>
-      <c r="V157" s="13" t="inlineStr">
-        <is>
-          <t>Section on Costa Alegre, poem Serões de São Tomé</t>
-        </is>
-      </c>
+          <t>Calema, Yellow (Klasszik, 2020); official video on the Klasszik YouTube channel.</t>
+        </is>
+      </c>
+      <c r="V157" s="13" t="n"/>
       <c r="W157" s="13" t="inlineStr">
         <is>
-          <t>The text contains racial comparisons requiring contextual reading. Modern commentary is separate. Composition date is not known; 1916 is the collection date.
-Passage update (29 October 2026): First four quatrains, 16 lines. Fresh English translation by Claude (Anthropic AI); draft for editorial review.
-Revision (30 October 2026, sensitivity review): re-excerpted to quatrains 1, 3, 4, 7 and 8 (20 lines), leaving out the quatrains built on slavery and skin-colour comparisons.</t>
+          <t>Work changed (30 October 2026): Caetano da Costa Alegre's quatrains are dropped, because the sequence they come from is built on colonial ideas about race; no São Tomé love poem that could be linked was found, so this is a love song by the islands' best-known band.</t>
         </is>
       </c>
       <c r="X157" s="13" t="inlineStr">
         <is>
-          <t>Historical original text: standard life-plus-70 term has expired; author died 1890. Assessment excludes modern translations, commentary, editorial alterations, musical settings and recordings. Territorial and unusual publication-history exceptions are not comprehensively assessed.</t>
+          <t>In copyright: described and linked only; no text or recording is reproduced here. Review, 30 October 2026.</t>
         </is>
       </c>
       <c r="Y157" s="13" t="inlineStr">
         <is>
-          <t>Original poem reproduced in the linked transcription; title and place in Costa Alegre’s work corroborated by UFMG Literafro scholars.</t>
+          <t>Official music video, Klasszik</t>
         </is>
       </c>
       <c r="Z157" s="11" t="inlineStr">
         <is>
-          <t>Work / source text</t>
-        </is>
-      </c>
-      <c r="AA157" s="11" t="inlineStr">
-        <is>
-          <t>Reuse basis / copyright duration</t>
-        </is>
-      </c>
-      <c r="AB157" s="11" t="inlineStr">
-        <is>
-          <t>Date / edition evidence</t>
-        </is>
-      </c>
-      <c r="AC157" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country evidence</t>
-        </is>
-      </c>
-      <c r="AD157" s="11" t="inlineStr">
-        <is>
-          <t>Additional evidence</t>
-        </is>
-      </c>
-      <c r="AE157" s="11" t="n"/>
+          <t>Watch the video</t>
+        </is>
+      </c>
+      <c r="AA157" s="11" t="n"/>
+      <c r="AB157" s="11" t="n"/>
+      <c r="AC157" s="11" t="n"/>
+      <c r="AD157" s="11" t="n"/>
+      <c r="AE157" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: https://kukalesa.wordpress.com/2013/01/11/alguns-precursores-da-negritude-em-lngua-portuguesa/</t>
+        </is>
+      </c>
     </row>
     <row r="158" ht="91.5" customHeight="1" s="17">
       <c r="A158" s="7" t="inlineStr">
@@ -30396,152 +30330,148 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z155" r:id="rId507"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z156" r:id="rId508"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z157" r:id="rId509"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA157" r:id="rId510"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB157" r:id="rId511"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC157" r:id="rId512"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD157" r:id="rId513"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z158" r:id="rId514"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA158" r:id="rId515"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB158" r:id="rId516"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC158" r:id="rId517"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z159" r:id="rId518"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z160" r:id="rId519"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA160" r:id="rId520"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB160" r:id="rId521"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC160" r:id="rId522"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z161" r:id="rId523"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE161" r:id="rId524"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z162" r:id="rId525"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE162" r:id="rId526"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z163" r:id="rId527"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA163" r:id="rId528"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB163" r:id="rId529"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC163" r:id="rId530"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD163" r:id="rId531"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE163" r:id="rId532"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z164" r:id="rId533"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA164" r:id="rId534"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB164" r:id="rId535"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC164" r:id="rId536"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z165" r:id="rId537"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA165" r:id="rId538"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB165" r:id="rId539"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC165" r:id="rId540"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z166" r:id="rId541"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z167" r:id="rId542"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA167" r:id="rId543"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB167" r:id="rId544"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC167" r:id="rId545"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD167" r:id="rId546"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE167" r:id="rId547"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z168" r:id="rId548"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z169" r:id="rId549"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA169" r:id="rId550"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB169" r:id="rId551"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC169" r:id="rId552"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z170" r:id="rId553"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z171" r:id="rId554"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA171" r:id="rId555"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB171" r:id="rId556"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC171" r:id="rId557"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z172" r:id="rId558"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA172" r:id="rId559"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB172" r:id="rId560"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC172" r:id="rId561"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD172" r:id="rId562"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE172" r:id="rId563"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z173" r:id="rId564"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z174" r:id="rId565"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z175" r:id="rId566"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA175" r:id="rId567"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB175" r:id="rId568"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC175" r:id="rId569"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z176" r:id="rId570"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA176" r:id="rId571"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB176" r:id="rId572"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC176" r:id="rId573"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z177" r:id="rId574"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA177" r:id="rId575"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB177" r:id="rId576"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC177" r:id="rId577"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z178" r:id="rId578"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA178" r:id="rId579"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB178" r:id="rId580"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC178" r:id="rId581"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z179" r:id="rId582"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z180" r:id="rId583"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA180" r:id="rId584"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB180" r:id="rId585"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC180" r:id="rId586"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z181" r:id="rId587"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE181" r:id="rId588"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z182" r:id="rId589"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD182" r:id="rId590"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z183" r:id="rId591"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z184" r:id="rId592"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA184" r:id="rId593"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB184" r:id="rId594"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC184" r:id="rId595"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD184" r:id="rId596"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z185" r:id="rId597"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA185" r:id="rId598"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB185" r:id="rId599"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC185" r:id="rId600"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD185" r:id="rId601"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z186" r:id="rId602"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z187" r:id="rId603"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z188" r:id="rId604"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z189" r:id="rId605"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE189" r:id="rId606"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z190" r:id="rId607"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA190" r:id="rId608"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB190" r:id="rId609"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC190" r:id="rId610"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD190" r:id="rId611"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z191" r:id="rId612"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD191" r:id="rId613"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE191" r:id="rId614"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z192" r:id="rId615"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA192" r:id="rId616"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB192" r:id="rId617"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC192" r:id="rId618"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z193" r:id="rId619"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA193" r:id="rId620"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB193" r:id="rId621"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC193" r:id="rId622"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z194" r:id="rId623"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA194" r:id="rId624"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB194" r:id="rId625"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC194" r:id="rId626"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z195" r:id="rId627"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA195" r:id="rId628"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB195" r:id="rId629"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC195" r:id="rId630"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z196" r:id="rId631"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA196" r:id="rId632"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB196" r:id="rId633"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC196" r:id="rId634"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z197" r:id="rId635"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA197" r:id="rId636"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB197" r:id="rId637"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC197" r:id="rId638"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z198" r:id="rId639"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA198" r:id="rId640"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB198" r:id="rId641"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC198" r:id="rId642"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE198" r:id="rId643"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z199" r:id="rId644"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA199" r:id="rId645"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB199" r:id="rId646"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC199" r:id="rId647"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE199" r:id="rId648"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z200" r:id="rId649"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z201" r:id="rId650"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE201" r:id="rId651"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z158" r:id="rId510"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA158" r:id="rId511"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB158" r:id="rId512"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC158" r:id="rId513"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z159" r:id="rId514"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z160" r:id="rId515"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA160" r:id="rId516"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB160" r:id="rId517"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC160" r:id="rId518"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z161" r:id="rId519"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE161" r:id="rId520"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z162" r:id="rId521"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE162" r:id="rId522"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z163" r:id="rId523"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA163" r:id="rId524"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB163" r:id="rId525"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC163" r:id="rId526"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD163" r:id="rId527"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE163" r:id="rId528"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z164" r:id="rId529"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA164" r:id="rId530"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB164" r:id="rId531"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC164" r:id="rId532"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z165" r:id="rId533"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA165" r:id="rId534"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB165" r:id="rId535"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC165" r:id="rId536"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z166" r:id="rId537"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z167" r:id="rId538"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA167" r:id="rId539"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB167" r:id="rId540"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC167" r:id="rId541"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD167" r:id="rId542"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE167" r:id="rId543"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z168" r:id="rId544"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z169" r:id="rId545"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA169" r:id="rId546"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB169" r:id="rId547"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC169" r:id="rId548"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z170" r:id="rId549"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z171" r:id="rId550"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA171" r:id="rId551"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB171" r:id="rId552"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC171" r:id="rId553"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z172" r:id="rId554"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA172" r:id="rId555"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB172" r:id="rId556"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC172" r:id="rId557"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD172" r:id="rId558"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE172" r:id="rId559"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z173" r:id="rId560"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z174" r:id="rId561"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z175" r:id="rId562"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA175" r:id="rId563"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB175" r:id="rId564"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC175" r:id="rId565"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z176" r:id="rId566"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA176" r:id="rId567"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB176" r:id="rId568"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC176" r:id="rId569"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z177" r:id="rId570"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA177" r:id="rId571"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB177" r:id="rId572"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC177" r:id="rId573"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z178" r:id="rId574"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA178" r:id="rId575"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB178" r:id="rId576"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC178" r:id="rId577"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z179" r:id="rId578"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z180" r:id="rId579"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA180" r:id="rId580"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB180" r:id="rId581"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC180" r:id="rId582"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z181" r:id="rId583"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE181" r:id="rId584"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z182" r:id="rId585"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD182" r:id="rId586"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z183" r:id="rId587"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z184" r:id="rId588"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA184" r:id="rId589"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB184" r:id="rId590"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC184" r:id="rId591"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD184" r:id="rId592"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z185" r:id="rId593"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA185" r:id="rId594"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB185" r:id="rId595"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC185" r:id="rId596"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD185" r:id="rId597"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z186" r:id="rId598"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z187" r:id="rId599"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z188" r:id="rId600"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z189" r:id="rId601"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE189" r:id="rId602"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z190" r:id="rId603"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA190" r:id="rId604"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB190" r:id="rId605"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC190" r:id="rId606"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD190" r:id="rId607"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z191" r:id="rId608"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AD191" r:id="rId609"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE191" r:id="rId610"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z192" r:id="rId611"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA192" r:id="rId612"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB192" r:id="rId613"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC192" r:id="rId614"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z193" r:id="rId615"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA193" r:id="rId616"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB193" r:id="rId617"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC193" r:id="rId618"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z194" r:id="rId619"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA194" r:id="rId620"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB194" r:id="rId621"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC194" r:id="rId622"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z195" r:id="rId623"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA195" r:id="rId624"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB195" r:id="rId625"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC195" r:id="rId626"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z196" r:id="rId627"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA196" r:id="rId628"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB196" r:id="rId629"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC196" r:id="rId630"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z197" r:id="rId631"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA197" r:id="rId632"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB197" r:id="rId633"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC197" r:id="rId634"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z198" r:id="rId635"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA198" r:id="rId636"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB198" r:id="rId637"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC198" r:id="rId638"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE198" r:id="rId639"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z199" r:id="rId640"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AA199" r:id="rId641"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AB199" r:id="rId642"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AC199" r:id="rId643"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE199" r:id="rId644"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z200" r:id="rId645"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="Z201" r:id="rId646"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="AE201" r:id="rId647"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId652"/>
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId648"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Whole-poem review: replace works with colonial ideas in their wider text
Read: Iran (Saadi), Azerbaijan (Fuzuli), Haiti (Etzer Vilaire), Philippines
(Pascual de León). Explore: Ghana (Kwesi Brew), Liberia (Patricia Jabbeh
Wesley), Trinidad and Tobago (Kes), Angola (Viriato da Cruz).

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/source/Manifesto_for_Love_MASTER.xlsx
+++ b/data/source/Manifesto_for_Love_MASTER.xlsx
@@ -1511,61 +1511,29 @@
       </c>
       <c r="D11" s="13" t="inlineStr">
         <is>
-          <t>Kicôla!</t>
+          <t>Namoro</t>
         </is>
       </c>
       <c r="E11" s="13" t="inlineStr">
         <is>
-          <t>Absolutely Not!</t>
-        </is>
-      </c>
-      <c r="F11" s="13" t="inlineStr">
-        <is>
-          <t>Nesta pequena cidade,
-vi uma certa donzela,
-que muito tinha de bela,
-de fada, huri e deidade,
-a quem disse: - “minha q’rida,
-peço um beijo por favor,
-bem sabes ó meu amor,
-que eu por ti daria a vida!”
-- “Nguami-âmi, ngana-lame,
-“não quero, caro senhor” –
-disse, sem mudar de cor –
-“maculo! quangandallâmi,
-“não creio no vosso amor”...</t>
-        </is>
-      </c>
-      <c r="G11" s="13" t="inlineStr">
-        <is>
-          <t>In this small town
-I saw a certain young woman,
-blessed with great beauty,
-like a fairy, a houri, a goddess,
-and I said to her: “My dear one,
-I ask you for a kiss, please;
-you know very well, my love,
-I would give my life for you!”
-“Nguami-âmi, ngana-lame,
-‘I don't want to, kind sir,’”
-she said, without a blush;
-“maculo! quangandallâmi,
-‘I don't believe in your love’…”</t>
-        </is>
-      </c>
+          <t>Courtship</t>
+        </is>
+      </c>
+      <c r="F11" s="13" t="n"/>
+      <c r="G11" s="13" t="n"/>
       <c r="H11" s="13" t="inlineStr">
         <is>
-          <t>Joaquim Dias Cordeiro da Matta (1857–1894)</t>
+          <t>Viriato da Cruz (1928–1973)</t>
         </is>
       </c>
       <c r="I11" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J11" s="13" t="inlineStr">
         <is>
-          <t>Named poem (excerpt)</t>
+          <t>Named work</t>
         </is>
       </c>
       <c r="K11" s="13" t="inlineStr">
@@ -1578,95 +1546,73 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M11" s="14" t="n">
-        <v>1877</v>
+      <c r="M11" s="14" t="inlineStr">
+        <is>
+          <t>1961</t>
+        </is>
       </c>
       <c r="N11" s="13" t="inlineStr">
         <is>
-          <t>Portuguese, with Kimbundu dialogue</t>
+          <t>Portuguese</t>
         </is>
       </c>
       <c r="O11" s="13" t="n"/>
       <c r="P11" s="13" t="inlineStr">
         <is>
-          <t>Lyric poem</t>
+          <t>Poem</t>
         </is>
       </c>
       <c r="Q11" s="13" t="inlineStr">
         <is>
-          <t>Man author</t>
+          <t>Viriato da Cruz</t>
         </is>
       </c>
       <c r="R11" s="13" t="inlineStr">
         <is>
-          <t>Composed Luanda, 1877; published in Almanach, 1888</t>
-        </is>
-      </c>
-      <c r="S11" s="13" t="inlineStr">
-        <is>
-          <t>Historical poem quoted in modern scholarly studies</t>
-        </is>
-      </c>
+          <t>By 1961; collected in Poemas (1961)</t>
+        </is>
+      </c>
+      <c r="S11" s="13" t="n"/>
       <c r="T11" s="13" t="inlineStr">
         <is>
-          <t>A courtship encounter: the speaker asks a beautiful woman for a kiss and receives a refusal in Kimbundu.</t>
+          <t>A young man courts a girl with perfumed letters, a card and even a charm, and is turned down every time, until at a dance, to the beat of an African rumba, she finally says yes.</t>
         </is>
       </c>
       <c r="U11" s="13" t="inlineStr">
         <is>
-          <t>University of Brasília, Cerrados, p.183; publication history discussed in António Jacinto e a sua época, p.336.</t>
-        </is>
-      </c>
-      <c r="V11" s="13" t="inlineStr">
-        <is>
-          <t>Kicôla!, first 13 quoted lines, Cerrados no.41 (2016), printed p.183 (PDF page 7).</t>
-        </is>
-      </c>
+          <t>Viriato da Cruz, Poemas (Lisbon: Casa dos Estudantes do Império, 1961).</t>
+        </is>
+      </c>
+      <c r="V11" s="13" t="n"/>
       <c r="W11" s="13" t="inlineStr">
         <is>
-          <t>Explicitly described as an imitation of verses by João E. da Cruz Toulson. Reuse the historical poem, not the modern criticism. The encounter ends in rejection.
-Passage update (29 October 2026): Earlier English draft by ChatGPT (replaced); editorial draft, not a quoted published translation. Original and English contain the same selection. Historical poem quoted in Sheila Ribeiro Jacob’s article. Kimbundu forms retain this source’s spelling and are followed by the poem’s Portuguese glosses, translated here. No independent Kimbundu translation is claimed. Other transcriptions differ. Opening excerpt, not complete poem.
-Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.</t>
+          <t>Work changed (30 October 2026) after the whole-poem review: Cordeiro da Matta's 'Kicôla' (1877) is replaced by the best-loved courtship poem of the generation of Angolan poets who called for 'Let's discover Angola'.</t>
         </is>
       </c>
       <c r="X11" s="13" t="inlineStr">
         <is>
-          <t>Historical original text: standard life-plus-70 term has expired; author died 1894. Assessment excludes modern translations, commentary, editorial alterations, musical settings and recordings. Territorial and unusual publication-history exceptions are not comprehensively assessed.
-Anthology review (30 October 2026): first published before 1931 and the poet died long before 1956, so public domain in the UK, EU and US. Almanach, 1888.</t>
+          <t>In copyright: described and linked only; no text or recording is reproduced here. Whole-poem review, 30 October 2026.</t>
         </is>
       </c>
       <c r="Y11" s="13" t="inlineStr">
         <is>
-          <t>University of Brasília, Cerrados, p.183; publication history discussed in António Jacinto e a sua época, p.336.
-Passage source checked 29 October 2026. https://periodicos.unb.br/index.php/cerrados/article/download/25396/22375/50283</t>
+          <t>Viriato da Cruz, Poemas (Lisbon: Casa dos Estudantes do Império, 1961).</t>
         </is>
       </c>
       <c r="Z11" s="11" t="inlineStr">
         <is>
-          <t>https://periodicos.unb.br/index.php/cerrados/article/download/25396/22375/50283</t>
-        </is>
-      </c>
-      <c r="AA11" s="11" t="inlineStr">
-        <is>
-          <t>Reuse basis / copyright duration</t>
-        </is>
-      </c>
-      <c r="AB11" s="11" t="inlineStr">
-        <is>
-          <t>Date / edition evidence</t>
-        </is>
-      </c>
-      <c r="AC11" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country evidence</t>
-        </is>
-      </c>
-      <c r="AD11" s="11" t="inlineStr">
-        <is>
-          <t>Additional evidence</t>
-        </is>
-      </c>
-      <c r="AE11" s="11" t="n"/>
+          <t>Read the text</t>
+        </is>
+      </c>
+      <c r="AA11" s="11" t="n"/>
+      <c r="AB11" s="11" t="n"/>
+      <c r="AC11" s="11" t="n"/>
+      <c r="AD11" s="11" t="n"/>
+      <c r="AE11" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: https://periodicos.unb.br/index.php/cerrados/article/download/25396/22375/50283</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="110" customHeight="1" s="17">
       <c r="A12" s="7" t="inlineStr">
@@ -2472,41 +2418,53 @@
       </c>
       <c r="D17" s="13" t="inlineStr">
         <is>
-          <t>Şuri-eşqin başıma axırı sövda gətirir</t>
+          <t>Məni candan usandırdı</t>
         </is>
       </c>
       <c r="E17" s="13" t="inlineStr">
         <is>
-          <t>The tumult of your love will finally drive me mad (first line)</t>
+          <t>My love has made me weary of my life</t>
         </is>
       </c>
       <c r="F17" s="13" t="inlineStr">
         <is>
-          <t>Şuri-eşqin başıma axırı sövda gətirir,
-Bu müşəxəssdi ki, eşq aşiqə qovğa gətirir.
-Tari-zülfündü məni böylə giriftar eləyib,
-Nə gələ başıma, ol zülfi-mütərra gətirir.
-Gül üzün görmək əgər mümkün olaydı bir dəm,
-Hər zaman görmək onu nuri-mücəlla gətirir.
-Qaşü göz, novki-mücə fitnə üçün cəm olmuş,
-Ox atıb, tiğ cəkib, hər biri dəva gətirir.</t>
+          <t>Məni candan usandırdı, cəfadən yar usanmazmı?
+Fələklər yandı ahimdən, muradım şəmi yanmazmı?
+Qamu bimarinə canan dəvayi-dərd edər ehsan,
+Neçün qılmaz mənə dərman, məni bimar sanmazmı?
+Qəmim pünhan tutardım mən, dedilər yarə qıl rövşən,
+Desəm, ol bivəfa bilmən, inanarmı, inanmazmı?
+Şəbi-hicran yanar canım, tökər qan çeşmi-giryanım,
+Oyadar xəlqi əfqanım, qara bəxtim oyanmazmı?
+Güli-rüxsarinə qarşu gözümdən qanlı axar su,
+Həbibim, fəsli-güldür bu, axar sular bulanmazmı?
+Degildim mən sənə mail, sən etdin əqlimi zail,
+Mənə tən eyləyən qafil səni görcək utanmazmı?
+Füzuli rindü şeydadır, həmişə xəlqə rüsvadır,
+Sorun kim, bu nə sevdadır, bu sevdadən usanmazmı?</t>
         </is>
       </c>
       <c r="G17" s="13" t="inlineStr">
         <is>
-          <t>The frenzy of your love will drive me mad at last;
-this much is certain: love brings the lover strife.
-It is the strand of your hair that has snared me so;
-whatever befalls me, those scented locks bring it on.
-If I could look at your rose of a face for one moment,
-each look would bring a shining, radiant light.
-Brow, eye and lash-point have joined forces to stir up trouble:
-one shoots arrows, one draws a blade, each picks a fight.</t>
+          <t>My love has made me weary of my life: will she never weary of cruelty?
+The heavens have caught fire from my sighs: will the candle of my longing never burn?
+To all who are sick for her, my beloved kindly gives a cure;
+why does she give no remedy to me? Does she not think me sick?
+I kept my grief hidden; they told me, make it plain to her.
+If I tell her, I cannot say whether that faithless one will believe me or not.
+On the night of parting my soul burns, my weeping eyes pour blood;
+my cries wake everyone: will my dark fortune never wake?
+Before the rose of your cheek, a stream of blood runs from my eyes;
+my darling, this is the season of roses: do running streams not turn cloudy then?
+I had no wish to fall for you; it was you who took my reason away.
+Will the thoughtless man who mocks me not feel ashamed when he sees you?
+Fuzuli is a reckless, love-crazed drinker, forever a scandal to the people;
+ask him: what passion is this? Will he never tire of this passion?</t>
         </is>
       </c>
       <c r="H17" s="13" t="inlineStr">
         <is>
-          <t>Khurshidbanu Natavan</t>
+          <t>Fuzuli (Məhəmməd Füzuli)</t>
         </is>
       </c>
       <c r="I17" s="13" t="inlineStr">
@@ -2516,7 +2474,7 @@
       </c>
       <c r="J17" s="13" t="inlineStr">
         <is>
-          <t>Named work</t>
+          <t>Named poem (original text)</t>
         </is>
       </c>
       <c r="K17" s="13" t="inlineStr">
@@ -2526,12 +2484,12 @@
       </c>
       <c r="L17" s="13" t="inlineStr">
         <is>
-          <t>Women</t>
+          <t>Men</t>
         </is>
       </c>
       <c r="M17" s="14" t="inlineStr">
         <is>
-          <t>c. 1870</t>
+          <t>c. 1530</t>
         </is>
       </c>
       <c r="N17" s="13" t="inlineStr">
@@ -2542,81 +2500,64 @@
       <c r="O17" s="13" t="n"/>
       <c r="P17" s="13" t="inlineStr">
         <is>
-          <t>Poem</t>
+          <t>Poem (ghazal, 7 couplets)</t>
         </is>
       </c>
       <c r="Q17" s="13" t="inlineStr">
         <is>
-          <t>Woman</t>
+          <t>Fuzuli</t>
         </is>
       </c>
       <c r="R17" s="13" t="inlineStr">
         <is>
-          <t>19th century; exact date not established</t>
-        </is>
-      </c>
-      <c r="S17" s="13" t="inlineStr">
-        <is>
-          <t>Undated transcription in modern Azerbaijani Latin script</t>
-        </is>
-      </c>
+          <t>16th century</t>
+        </is>
+      </c>
+      <c r="S17" s="13" t="n"/>
       <c r="T17" s="13" t="inlineStr">
         <is>
-          <t>Passionate love overwhelms the lover; imagery evokes the beloved’s face and legendary lovers.</t>
+          <t>The poet burns with a love his beloved will not cure; he cannot tell whether she would believe him if he spoke, and asks whether he will ever tire of this passion.</t>
         </is>
       </c>
       <c r="U17" s="13" t="inlineStr">
         <is>
-          <t>Vikimənbə text, attributed to Natavan (1832–1897), with source link to Azadliq</t>
+          <t>Fuzuli, Azerbaijani Divan; text from Azerbaijani Wikisource, following Məhəmməd Füzuli, Əsərləri, vol. 1 (Baku, 2005).</t>
         </is>
       </c>
       <c r="V17" s="13" t="inlineStr">
         <is>
-          <t>Opening five couplets of the ghazal, 10 lines in the Wikisource transcription.</t>
+          <t>Complete poem</t>
         </is>
       </c>
       <c r="W17" s="13" t="inlineStr">
         <is>
-          <t>Natavan was a Shusha/Karabakh poet in present-day Azerbaijan. Original ghazal only; modern transliteration/editorial contributions may require attribution. English translation not supplied.
-Passage update (29 October 2026): Earlier English draft by ChatGPT (replaced); editorial draft, not a quoted published translation. Original and English contain the same selection. Latin transcription follows Wikisource, including cəkib as printed. Final couplet retains a historical dark-hair/light-face military conceit involving Abyssinia and Rum. Classical vocabulary merits specialist review.
-Translation redone (30 October 2026) for the anthology review: fresh English translation by Claude (Anthropic AI) made directly from the original text, without reference to any other translation; draft for editorial review.
-Revision (30 October 2026, sensitivity review): final couplet left out (its image compares dark hair to an Abyssinian army); the passage is now couplets 1–4 of the ghazal.</t>
+          <t>Work changed (30 October 2026) after the whole-poem review: Natavan's ghazal, whose final couplet likens dark hair to an Abyssinian army, is replaced by the best-known love ghazal of Azerbaijan's greatest classical poet. Complete poem, 7 couplets (14 lines). Fresh English translation by Claude (Anthropic AI) made directly from the original; draft for editorial review.</t>
         </is>
       </c>
       <c r="X17" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original; site transcription has CC BY-SA terms where applicable
-Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
+          <t>Whole-poem review (30 October 2026): Fuzuli died in 1556 and the poem has been printed and sung for centuries; public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y17" s="13" t="inlineStr">
         <is>
-          <t xml:space="preserve">
-Passage source checked 29 October 2026. https://az.wikisource.org/wiki/Şuri-eşqin_başıma_axırı_sövda_gətirir</t>
+          <t>Fuzuli, Azerbaijani Divan; text from Azerbaijani Wikisource, following Məhəmməd Füzuli, Əsərləri, vol. 1 (Baku, 2005).</t>
         </is>
       </c>
       <c r="Z17" s="11" t="inlineStr">
         <is>
-          <t>https://az.wikisource.org/wiki/Şuri-eşqin_başıma_axırı_sövda_gətirir</t>
-        </is>
-      </c>
-      <c r="AA17" s="11" t="inlineStr">
-        <is>
-          <t>Rights / catalogue</t>
-        </is>
-      </c>
-      <c r="AB17" s="11" t="inlineStr">
-        <is>
-          <t>Date evidence</t>
-        </is>
-      </c>
-      <c r="AC17" s="11" t="inlineStr">
-        <is>
-          <t>Author / country</t>
-        </is>
-      </c>
+          <t>Read the whole work</t>
+        </is>
+      </c>
+      <c r="AA17" s="11" t="n"/>
+      <c r="AB17" s="11" t="n"/>
+      <c r="AC17" s="11" t="n"/>
       <c r="AD17" s="11" t="n"/>
-      <c r="AE17" s="11" t="n"/>
+      <c r="AE17" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: https://az.wikisource.org/wiki/Şuri-eşqin_başıma_axırı_sövda_gətirir</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="124" customHeight="1" s="17">
       <c r="A18" s="7" t="inlineStr">
@@ -10442,64 +10383,34 @@
       </c>
       <c r="D72" s="13" t="inlineStr">
         <is>
-          <t>Ethiopia Unbound: Studies in Race Emancipation</t>
+          <t>The Mesh</t>
         </is>
       </c>
       <c r="E72" s="13" t="inlineStr">
         <is>
-          <t>Ethiopia Unbound: Studies in Race Emancipation</t>
-        </is>
-      </c>
-      <c r="F72" s="13" t="inlineStr">
-        <is>
-          <t>“Yes, I know that.
-But this also I do know, that the gods are wont to make use of human instruments in approaching men.
-The Infinite finds expression in the finite, and the ideal is realised in the actual.
-And it has often occurred to me that the child-like hand that shall guide me through life’s labyrinthine ways is the self-same one that I now hold tenderly in my own.”
-She began to understand.
-She made an effort as if she would withdraw her hand.
-She hesitated, and the next moment she surrendered the other also.
-“You will be my teacher, then?” asked Kwamankra, half-persuasively, half-triumphantly.
-“Yes,” she simply answered. “So may the gods of our race help me!”
-As the days passed, the twain grew in that mutual understanding, the true basis of all happy unions.
-Now and again he would tell her of his prospects, which he laughingly said were nil, having inherited little else beyond a clear head and a willing heart for work, with which he hoped they would be able to forge their way in life together;
-to which Mansa would sweetly say that she wished she had a fortune to make things easy, but since she had it not, she would bring him the next best, a loyal heart and true, at which Kwamankra would chide her, and say that was the best of all.</t>
-        </is>
-      </c>
-      <c r="G72" s="13" t="inlineStr">
-        <is>
-          <t>“Yes, I know that.
-But this also I do know, that the gods are wont to make use of human instruments in approaching men.
-The Infinite finds expression in the finite, and the ideal is realised in the actual.
-And it has often occurred to me that the child-like hand that shall guide me through life’s labyrinthine ways is the self-same one that I now hold tenderly in my own.”
-She began to understand.
-She made an effort as if she would withdraw her hand.
-She hesitated, and the next moment she surrendered the other also.
-“You will be my teacher, then?” asked Kwamankra, half-persuasively, half-triumphantly.
-“Yes,” she simply answered. “So may the gods of our race help me!”
-As the days passed, the twain grew in that mutual understanding, the true basis of all happy unions.
-Now and again he would tell her of his prospects, which he laughingly said were nil, having inherited little else beyond a clear head and a willing heart for work, with which he hoped they would be able to forge their way in life together;
-to which Mansa would sweetly say that she wished she had a fortune to make things easy, but since she had it not, she would bring him the next best, a loyal heart and true, at which Kwamankra would chide her, and say that was the best of all.</t>
-        </is>
-      </c>
+          <t>The Mesh</t>
+        </is>
+      </c>
+      <c r="F72" s="13" t="n"/>
+      <c r="G72" s="13" t="n"/>
       <c r="H72" s="13" t="inlineStr">
         <is>
-          <t>J. E. Casely Hayford (1866–1930)</t>
+          <t>Kwesi Brew (1928–2007)</t>
         </is>
       </c>
       <c r="I72" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J72" s="13" t="inlineStr">
         <is>
-          <t>Named work (catalogue / preview)</t>
+          <t>Named work</t>
         </is>
       </c>
       <c r="K72" s="13" t="inlineStr">
         <is>
-          <t>Prose / novel</t>
+          <t>Poetry</t>
         </is>
       </c>
       <c r="L72" s="13" t="inlineStr">
@@ -10507,8 +10418,10 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M72" s="14" t="n">
-        <v>1911</v>
+      <c r="M72" s="14" t="inlineStr">
+        <is>
+          <t>1968</t>
+        </is>
       </c>
       <c r="N72" s="13" t="inlineStr">
         <is>
@@ -10518,81 +10431,60 @@
       <c r="O72" s="13" t="n"/>
       <c r="P72" s="13" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Poem</t>
         </is>
       </c>
       <c r="Q72" s="13" t="inlineStr">
         <is>
-          <t>Man author</t>
+          <t>Kwesi Brew</t>
         </is>
       </c>
       <c r="R72" s="13" t="inlineStr">
         <is>
-          <t>1911, London: C. M. Phillips</t>
-        </is>
-      </c>
-      <c r="S72" s="13" t="inlineStr">
-        <is>
-          <t>Historical work reproduced in linked digital source; modern editorial material is separate</t>
-        </is>
-      </c>
+          <t>1968</t>
+        </is>
+      </c>
+      <c r="S72" s="13" t="n"/>
       <c r="T72" s="13" t="inlineStr">
         <is>
-          <t>The novel interweaves romantic relationships, including Tandoh-Kuma and Ekuba, with debates about education, identity and African self-determination.</t>
+          <t>Two people stand at a crossroads, unsure which way to go, until love lights the path they will take together.</t>
         </is>
       </c>
       <c r="U72" s="13" t="inlineStr">
         <is>
-          <t>Original 1911 edition catalogued with preview. O. R. Dathorne’s literary study, National Library of Nigeria repository, identifies the romantic subplot and Ghanaian author.</t>
-        </is>
-      </c>
-      <c r="V72" s="13" t="inlineStr">
-        <is>
-          <t>Chapters III–IV, Love and Life / Love and Death; consult original edition for passage selection</t>
-        </is>
-      </c>
+          <t>Kwesi Brew, Shadows of Laughter (London: Longmans, 1968).</t>
+        </is>
+      </c>
+      <c r="V72" s="13" t="n"/>
       <c r="W72" s="13" t="inlineStr">
         <is>
-          <t>This is a Ghanaian/Gold Coast work despite Ethiopia in the title. Do not substitute the separately copyrighted 1969 or 2024 editorial introductions. Full original passage not transcribed here.
-Passage update (29 October 2026): Twelve consecutive lines from Chapter III, “Love and Life”: Kwamankra’s proposal to Mansa (1911 first edition, Internet Archive scan, pp. 34–35). OCR spacing and line-break hyphens tidied; the letters were checked against the scan text. Original English; no translation needed. Original English text; not a translation.</t>
+          <t>Work changed (30 October 2026) after the whole-poem review: Casely Hayford's Ethiopia Unbound (1911) is replaced by a short love poem, one of the best loved in Ghanaian writing.</t>
         </is>
       </c>
       <c r="X72" s="13" t="inlineStr">
         <is>
-          <t>Historical original text: standard life-plus-70 term has expired; author died 1930. Assessment excludes modern translations, commentary, editorial alterations, musical settings and recordings. Territorial and unusual publication-history exceptions are not comprehensively assessed.</t>
+          <t>In copyright: described and linked only; no text or recording is reproduced here. Whole-poem review, 30 October 2026.</t>
         </is>
       </c>
       <c r="Y72" s="13" t="inlineStr">
         <is>
-          <t>Original 1911 edition catalogued with preview. O. R. Dathorne’s literary study, National Library of Nigeria repository, identifies the romantic subplot and Ghanaian author.</t>
+          <t>Kwesi Brew, Shadows of Laughter (London: Longmans, 1968).</t>
         </is>
       </c>
       <c r="Z72" s="11" t="inlineStr">
         <is>
-          <t>Read original</t>
-        </is>
-      </c>
-      <c r="AA72" s="11" t="inlineStr">
-        <is>
-          <t>Reuse basis / copyright duration</t>
-        </is>
-      </c>
-      <c r="AB72" s="11" t="inlineStr">
-        <is>
-          <t>Date / edition evidence</t>
-        </is>
-      </c>
-      <c r="AC72" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country evidence</t>
-        </is>
-      </c>
-      <c r="AD72" s="11" t="inlineStr">
-        <is>
-          <t>Additional evidence</t>
-        </is>
-      </c>
-      <c r="AE72" s="11" t="n"/>
+          <t>Read the text</t>
+        </is>
+      </c>
+      <c r="AA72" s="11" t="n"/>
+      <c r="AB72" s="11" t="n"/>
+      <c r="AC72" s="11" t="n"/>
+      <c r="AD72" s="11" t="n"/>
+      <c r="AE72" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: https://archive.org/details/ethiopiaunbounds00hayf</t>
+        </is>
+      </c>
     </row>
     <row r="73" ht="43.5" customHeight="1" s="17">
       <c r="A73" s="7" t="inlineStr">
@@ -11422,49 +11314,91 @@
       </c>
       <c r="D79" s="13" t="inlineStr">
         <is>
-          <t>Choucoune</t>
+          <t>Loin de toi, près de toi</t>
         </is>
       </c>
       <c r="E79" s="13" t="inlineStr">
         <is>
-          <t>Choucoune (a woman's name)</t>
+          <t>Far from you, near you</t>
         </is>
       </c>
       <c r="F79" s="13" t="inlineStr">
         <is>
-          <t>Dériè gnou gras touff’ pingouin,
-L’aut’jou, moin contré Choucoune ;
-Li sourit, l’heur’li ouè moin,
-Moin dit : « Ciel ! A là bell’ moune ! »
-Li dit : « Ou trouvé ca cher ! »…
-P’tits zoézeaux ta pé couté nous lan l’air…
-Quand moin songé Ça, moin gangnin la peine,
-Car dimpi jou-là, dé pieds moin lan chaîne !
-Ca qui pis trist’lan tout ça,
-Ca qui va surprendr’tout moune,
-Cé ’pou ouè malgré temps-là,
-Moin aimé toujours Choucoune !</t>
+          <t>Loin de toi, c’est la nuit,
+C’est la nuit triste et sombre,
+Et mon cœur plein d’ennui
+S’ensevelit dans l’ombre.
+Loin de toi, tout fléchit :
+Mon espoir, mon courage.
+Loin de toi, mon esprit
+Se voile d’un nuage.
+Comme en un jour d’orage,
+Tout tremble en moi
+Loin de toi !
+Sans l’éclat de tes yeux,
+C’est mon printemps qui passe ;
+C’est dans le deuil des cieux
+Mon soleil qui s’efface !
+Sans le bruit de tes pas,
+Sans ta voix, ton sourire,
+Sans l’espace où tu vas,
+Où ta bouche respire,
+Tout mon cœur se déchire :
+Tout meurt en moi
+Loin de toi !
+Près de toi, ma beauté,
+C’est la douceur du rêve
+Faite réalité :
+Et quelle aube se lève !
+Un Univers nouveau
+Brille, une proche étoile
+Allume son flambeau
+Dans ma tremblante voile.
+Oui, le ciel se dévoile
+Et s’ouvre à moi
+Près de toi !</t>
         </is>
       </c>
       <c r="G79" s="13" t="inlineStr">
         <is>
-          <t>Behind a thick clump of cactus,
-The other day, I met Choucoune;
-She smiled the moment she saw me,
-I said: “Heavens! What a beautiful girl!”
-She said: “You think so, dear?”…
-Little birds were listening to us up in the air…
-When I think of it, I am full of sorrow,
-For since that day both my feet are in chains!
-The saddest thing in all of this,
-The thing that will surprise everyone,
-Is to see that, in spite of it all,
-I still love Choucoune!</t>
+          <t>Far from you, it is night,
+the sad and sombre night,
+and my heart, full of weariness,
+buries itself in shadow.
+Far from you, everything gives way:
+my hope, my courage.
+Far from you, my mind
+is veiled by a cloud.
+As on a stormy day,
+everything trembles in me
+far from you!
+Without the brightness of your eyes,
+it is my springtime passing;
+it is my sun, in the mourning of the skies,
+fading away!
+Without the sound of your steps,
+without your voice, your smile,
+without the air you move through,
+where your lips breathe,
+my whole heart is torn:
+everything dies in me
+far from you!
+Near you, my beauty,
+the sweetness of the dream
+comes true:
+and what a dawn is rising!
+A new universe
+shines; a nearby star
+lights its torch
+in my trembling sail.
+Yes, the sky unveils itself
+and opens to me
+near you!</t>
         </is>
       </c>
       <c r="H79" s="13" t="inlineStr">
         <is>
-          <t>Oswald Durand</t>
+          <t>Etzer Vilaire (1872–1951)</t>
         </is>
       </c>
       <c r="I79" s="13" t="inlineStr">
@@ -11474,7 +11408,7 @@
       </c>
       <c r="J79" s="13" t="inlineStr">
         <is>
-          <t>Named work</t>
+          <t>Named poem (original text)</t>
         </is>
       </c>
       <c r="K79" s="13" t="inlineStr">
@@ -11487,88 +11421,77 @@
           <t>Men</t>
         </is>
       </c>
-      <c r="M79" s="14" t="n">
-        <v>1884</v>
+      <c r="M79" s="14" t="inlineStr">
+        <is>
+          <t>1914</t>
+        </is>
       </c>
       <c r="N79" s="13" t="inlineStr">
         <is>
-          <t>Haitian Creole</t>
+          <t>French</t>
         </is>
       </c>
       <c r="O79" s="13" t="n"/>
       <c r="P79" s="13" t="inlineStr">
         <is>
-          <t>Poetry</t>
+          <t>Poem (3 stanzas)</t>
         </is>
       </c>
       <c r="Q79" s="13" t="inlineStr">
         <is>
-          <t>Man</t>
+          <t>Etzer Vilaire</t>
         </is>
       </c>
       <c r="R79" s="13" t="inlineStr">
         <is>
-          <t>1884 (date printed with poem)</t>
-        </is>
-      </c>
-      <c r="S79" s="13" t="inlineStr">
-        <is>
-          <t>1923</t>
-        </is>
-      </c>
+          <t>By 1914</t>
+        </is>
+      </c>
+      <c r="S79" s="13" t="n"/>
       <c r="T79" s="13" t="inlineStr">
         <is>
-          <t>Courtship, admiration and continuing love after the beloved leaves for another man.</t>
+          <t>Far from his beloved the poet's world is night and storm; near her, a new universe shines and the sky opens.</t>
         </is>
       </c>
       <c r="U79" s="13" t="inlineStr">
         <is>
-          <t>Floréal, 2 June 1923, pp. 341–342; scan-linked Wikisource</t>
+          <t>Etzer Vilaire, Poésies complètes, tome 1: Années tendres (Paris, 1914); text from French Wikisource.</t>
         </is>
       </c>
       <c r="V79" s="13" t="inlineStr">
         <is>
-          <t>Poème en dialecte créole, before TRADUCTION</t>
+          <t>Complete poem</t>
         </is>
       </c>
       <c r="W79" s="13" t="inlineStr">
         <is>
-          <t>Durand died 1906. Use the Creole original; the accompanying French translation has a separate attribution question. Original includes historical racial language. Later songs and Yellow Bird adaptations are separate. The selection is the original-language text; an existing English translation is not required.
-Passage update (29 October 2026): Opening stanza (8 lines) and the first four lines of the last stanza. The 1923 journal transcription is unproofread OCR: three obvious slips are corrected (a full stop after “L’aut’jou” to a comma, “bell”” to “bell’”, and a missing opening « before “Ou trouvé”); the wording is unchanged. Fresh English translation by Claude (Anthropic AI); draft for editorial review.</t>
+          <t>Work changed (30 October 2026) after the whole-poem review: Oswald Durand's 'Choucoune', which uses colonial racial categories, is replaced by a love poem by one of Haiti's leading poets. Complete poem, 33 lines. Fresh English translation by Claude (Anthropic AI) made directly from the original; draft for editorial review.</t>
         </is>
       </c>
       <c r="X79" s="13" t="inlineStr">
         <is>
-          <t>Public-domain original in the UK and other life-plus-70 jurisdictions: author died 1906. Modern editorial additions and translations are separate.</t>
+          <t>Whole-poem review (30 October 2026): first published 1914 (before 1931, so public domain in the US); Vilaire died in 1951, so public domain in the UK and EU since 2022. The online text is a transcription with no new authorship.</t>
         </is>
       </c>
       <c r="Y79" s="13" t="inlineStr">
         <is>
-          <t>Source text and provenance checked 28 October 2026.</t>
+          <t>Etzer Vilaire, Poésies complètes, tome 1: Années tendres (Paris, 1914); text from French Wikisource.</t>
         </is>
       </c>
       <c r="Z79" s="11" t="inlineStr">
         <is>
-          <t>Read original</t>
-        </is>
-      </c>
-      <c r="AA79" s="11" t="inlineStr">
-        <is>
-          <t>Rights / basis</t>
-        </is>
-      </c>
-      <c r="AB79" s="11" t="inlineStr">
-        <is>
-          <t>Date evidence</t>
-        </is>
-      </c>
-      <c r="AC79" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country</t>
-        </is>
-      </c>
+          <t>Read the whole work</t>
+        </is>
+      </c>
+      <c r="AA79" s="11" t="n"/>
+      <c r="AB79" s="11" t="n"/>
+      <c r="AC79" s="11" t="n"/>
       <c r="AD79" s="11" t="n"/>
-      <c r="AE79" s="11" t="n"/>
+      <c r="AE79" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: https://fr.wikisource.org/wiki/Choucoune</t>
+        </is>
+      </c>
     </row>
     <row r="80" ht="108" customHeight="1" s="17">
       <c r="A80" s="7" t="inlineStr">
@@ -12699,61 +12622,69 @@
       </c>
       <c r="D86" s="13" t="inlineStr">
         <is>
-          <t>اگر آن ترک شیرازی / Agar an Turk-e Shirazi</t>
+          <t>دیده از دیدار خوبان برگرفتن مشکل است (غزل ۷۳)</t>
         </is>
       </c>
       <c r="E86" s="13" t="inlineStr">
         <is>
-          <t>If That Turk of Shiraz</t>
+          <t>It is hard to take your eyes from the beautiful (ghazal 73)</t>
         </is>
       </c>
       <c r="F86" s="13" t="inlineStr">
         <is>
-          <t>اگر آن ترک شیرازی به‌ دست‌ آرد دل ما را
-به خال هندویش بخشم سمرقند و بخارا را
-بده ساقی می باقی که در جنت نخواهی یافت
-کنار آب رکناباد و گل‌گشت مصلا را
-فغان! کاین لولیان شوخ شیرین‌کار شهرآشوب
-چنان بردند صبر از دل که ترکان خوان یغما را
-ز عشق ناتمام ما جمال یار مستغنی‌ است
-به آب و رنگ و خال و خط چه حاجت روی زیبا را؟
-من از آن حسن روزافزون که یوسف داشت دانستم
-که عشق از پردهٔ عصمت برون آرد زلیخا را
-اگر دشنام فرمایی و گر نفرین دعا گویم
-جواب تلخ می‌زیبد لب لعل شکرخا را
-نصیحت گوش کن جانا که از جان دوست‌تر دارند
-جوانان سعادتمند پند پیر دانا را
-حدیث از مطرب و می گو و راز دهر کمتر جو
-که کس نگشود و نگشاید به حکمت این معما را
-غزل گفتی و در سفتی بیا و خوش بخوان حافظ
-که بر نظم تو افشاند فلک عقد ثریا را</t>
+          <t>دیده از دیدار خوبان برگرفتن مشکل ست
+هر که ما را این نصیحت می کند بی حاصل ست
+یار زیبا گر هزارت وحشت از وی در دل ست
+بامدادان روی او دیدن صباح مقبل ست
+آن که در چاه زنخدانش دل بیچارگان
+چون ملک محبوس در زندان چاه بابل ست
+پیش از این من دعوی پرهیزگاری کردمی
+باز می گویم که هر دعوی که کردم باطل ست
+زهر نزدیک خردمندان اگر چه قاتل ست
+چون ز دست دوست می گیری شفای عاجل ست
+من قدم بیرون نمی یارم نهاد از کوی دوست
+دوستان معذور داریدم که پایم در گل ست
+باش تا دیوانه گویندم همه فرزانگان
+ترک جان نتوان گرفتن تا تو گویی عاقل ست
+آن که می گوید نظر در صورت خوبان خطاست
+او همین صورت همی بیند ز معنی غافل ست
+ساربان آهسته ران کآرام جان در محمل ست
+چارپایان بار بر پشتند و ما را بر دل ست
+گر به صد منزل فراق افتد میان ما و دوست
+همچنانش در میان جان شیرین منزل ست
+سعدی آسان ست با هر کس گرفتن دوستی
+لیک چون پیوند شد خو باز کردن مشکل ست</t>
         </is>
       </c>
       <c r="G86" s="13" t="inlineStr">
         <is>
-          <t>If that Turk of Shiraz would only take my heart in hand,
-for the dark mole on that cheek I'd give up Samarkand and Bukhara.
-Bring the last of the wine, cupbearer: in paradise you won't find
-the banks of the Ruknabad or the flowered paths of Musalla.
-Ah, these playful wandering minstrel girls, so charming, such trouble to the town,
-have stripped the patience from my heart as Turks strip a table of its spoils.
-My love is incomplete, but my beloved's beauty does not need it:
-a lovely face has no use for powder, colour, beauty-spot or pencil.
-From that beauty of Joseph's, growing day by day, I learned
-how love draws Zulaikha out from behind the curtain of virtue.
-Abuse me if you like, curse me: I'll pray for you all the same;
-a bitter answer becomes a ruby lip that rains down sugar.
-Take some advice, my dear: young people blessed by fortune
-love the counsel of a wise old man more than life itself.
-Talk of minstrels and wine, and don't dig into the world's secret,
-for no one has solved this riddle by wisdom, and no one will.
-You've made your ghazal and pierced your pearls; come, Hafez, sing it well,
-for the sky scatters the string of the Pleiades over your verse.</t>
+          <t>It is hard to take your eyes from the sight of the beautiful;
+whoever gives me that advice is wasting his breath.
+Though a lovely beloved fills your heart with a thousand fears,
+to see that face at daybreak makes a blessed morning.
+In the well of her chin the hearts of the helpless
+are held like the angels imprisoned in the well of Babylon.
+Once I used to claim I was above temptation;
+now I say that every claim I made was false.
+The wise know poison kills, and yet
+taken from the beloved's hand it is an instant cure.
+I dare not set one foot outside my beloved's street;
+forgive me, friends: my feet are stuck fast in the clay.
+Let all the clever people call me mad:
+no one gives up his soul just to be called sensible.
+Whoever says it is wrong to gaze at beautiful faces
+sees only the outward form and misses the meaning.
+Camel driver, go gently: my soul's peace rides in that litter;
+the beasts bear their loads on their backs, and I bear mine on my heart.
+Though parting sets a hundred stages between my love and me,
+she still has her dwelling in the midst of my sweet soul.
+Saadi, it is easy to make friends with anyone,
+but once the bond is made, the habit is hard to break.</t>
         </is>
       </c>
       <c r="H86" s="13" t="inlineStr">
         <is>
-          <t>Hafez</t>
+          <t>Saadi (سعدی)</t>
         </is>
       </c>
       <c r="I86" s="13" t="inlineStr">
@@ -12763,7 +12694,7 @@
       </c>
       <c r="J86" s="13" t="inlineStr">
         <is>
-          <t>Named work</t>
+          <t>Named poem (original text)</t>
         </is>
       </c>
       <c r="K86" s="13" t="inlineStr">
@@ -12778,7 +12709,7 @@
       </c>
       <c r="M86" s="14" t="inlineStr">
         <is>
-          <t>c. 1370</t>
+          <t>c. 1260</t>
         </is>
       </c>
       <c r="N86" s="13" t="inlineStr">
@@ -12789,80 +12720,64 @@
       <c r="O86" s="13" t="n"/>
       <c r="P86" s="13" t="inlineStr">
         <is>
-          <t>Poem</t>
+          <t>Poem (ghazal, 11 couplets)</t>
         </is>
       </c>
       <c r="Q86" s="13" t="inlineStr">
         <is>
-          <t>Man</t>
+          <t>Saadi of Shiraz</t>
         </is>
       </c>
       <c r="R86" s="13" t="inlineStr">
         <is>
-          <t>14th century (exact composition date unknown)</t>
-        </is>
-      </c>
-      <c r="S86" s="13" t="inlineStr">
-        <is>
-          <t>Persian text: Ganjoor online edition</t>
-        </is>
-      </c>
+          <t>13th century</t>
+        </is>
+      </c>
+      <c r="S86" s="13" t="n"/>
       <c r="T86" s="13" t="inlineStr">
         <is>
-          <t>Praise of the beloved in a ghazal.</t>
+          <t>The poet cannot stop gazing at his beloved, whatever the wise may say; as her caravan leaves he begs the camel driver to go gently, for his soul's peace rides in her litter.</t>
         </is>
       </c>
       <c r="U86" s="13" t="inlineStr">
         <is>
-          <t>Divan of Hafez, ghazal 3; Persian text from Ganjoor.</t>
+          <t>Saadi, Divan, ghazal 73; text from Ganjoor.</t>
         </is>
       </c>
       <c r="V86" s="13" t="inlineStr">
         <is>
-          <t>Complete ghazal (Divan, ghazal 3), 9 couplets</t>
+          <t>Complete poem</t>
         </is>
       </c>
       <c r="W86" s="13" t="inlineStr">
         <is>
-          <t>New English translation from the Persian; Gertrude Bell's 1897 translation is not used. Modern translations are separate. Mystical readings are possible.
-Passage update (29 October 2026): Complete ghazal, 9 couplets (18 half-lines). Persian text from Ganjoor (ghazal 3), with Ganjoor’s added short-vowel marks removed; the letters are unchanged. Fresh English translation by Claude (Anthropic AI); draft for editorial review.
-Revision (30 October 2026): retranslated from the Persian for the anthology review so that no line follows the wording of an earlier English version.
-Revision (30 October 2026, sensitivity review): lūliyān (line 5) translated as 'wandering minstrel girls' rather than with an ethnic slur.</t>
+          <t>Work changed (30 October 2026) after the whole-poem review: Hafez's 'Turk of Shiraz', whose second line uses an old image linking a 'Hindu' mole with dark skin and servitude, is replaced by a love ghazal by Shiraz's other great poet. Complete poem, 11 couplets (22 lines). Fresh English translation by Claude (Anthropic AI) made directly from the original; draft for editorial review.</t>
         </is>
       </c>
       <c r="X86" s="13" t="inlineStr">
         <is>
-          <t>Original text: 14th-century poem, public domain. New English translation from the Persian; Gertrude Bell's 1897 translation is not used.
-Anthology review (30 October 2026): the poet died centuries ago and the poem was in print long before 1989, so it is public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
+          <t>Whole-poem review (30 October 2026): Saadi died c. 1291 and the poem has been in print for centuries; public domain in the UK, EU and US; the online text is a transcription of a historical text, with no new authorship.</t>
         </is>
       </c>
       <c r="Y86" s="13" t="inlineStr">
         <is>
-          <t>Ganjoor: Hafez, ghazal 3</t>
+          <t>Saadi, Divan, ghazal 73; text from Ganjoor.</t>
         </is>
       </c>
       <c r="Z86" s="11" t="inlineStr">
         <is>
-          <t>Read original</t>
-        </is>
-      </c>
-      <c r="AA86" s="11" t="inlineStr">
-        <is>
-          <t>Rights / catalogue</t>
-        </is>
-      </c>
-      <c r="AB86" s="11" t="inlineStr">
-        <is>
-          <t>Date evidence</t>
-        </is>
-      </c>
-      <c r="AC86" s="11" t="inlineStr">
-        <is>
-          <t>Author / country</t>
-        </is>
-      </c>
+          <t>Read the whole work</t>
+        </is>
+      </c>
+      <c r="AA86" s="11" t="n"/>
+      <c r="AB86" s="11" t="n"/>
+      <c r="AC86" s="11" t="n"/>
       <c r="AD86" s="11" t="n"/>
-      <c r="AE86" s="11" t="n"/>
+      <c r="AE86" s="11" t="inlineStr">
+        <is>
+          <t>Earlier link: https://ganjoor.net/hafez/ghazal/sh3</t>
+        </is>
+      </c>
     </row>
     <row r="87" ht="91.5" customHeight="1" s="17">
       <c r="A87" s="7" t="inlineStr">
@@ -15365,67 +15280,45 @@
       </c>
       <c r="D103" s="13" t="inlineStr">
         <is>
-          <t>Guanya Pau: A Story of an African Princess</t>
+          <t>Nyanken Hne</t>
         </is>
       </c>
       <c r="E103" s="13" t="inlineStr">
         <is>
-          <t>Guanya Pau: A Story of an African Princess</t>
-        </is>
-      </c>
-      <c r="F103" s="13" t="inlineStr">
-        <is>
-          <t>“Well, when this had gone on over two years, one evening about twilight, when I had finished my work, I went and sat under the cola-tree behind our house and pretended to be stringing my beads;
-But my true object was soon realized.
-Momo soon joined me and sat down by my side.
-Who can picture our feelings as that evening we sat beneath the shadows of that stately cola, in the clear moonlight?
-We sat side by side on the green grass, talking little nothings.
-By and by he took a long breath, somehow I felt anxious just because of that sigh.
-He then took both my hands in his, sending a thrill clean through me.
-Planting his frank, honest eyes on mine which soon were directed to the ground, he said: ‘Guanya Pau, nah Edear (I love you); ya in dear wah?’ (Do you love me?)
-What could I say but to whisper faintly: ‘Da keker’ (with all my heart).</t>
-        </is>
-      </c>
-      <c r="G103" s="13" t="inlineStr">
-        <is>
-          <t>“Well, when this had gone on over two years, one evening about twilight, when I had finished my work, I went and sat under the cola-tree behind our house and pretended to be stringing my beads;
-But my true object was soon realized.
-Momo soon joined me and sat down by my side.
-Who can picture our feelings as that evening we sat beneath the shadows of that stately cola, in the clear moonlight?
-We sat side by side on the green grass, talking little nothings.
-By and by he took a long breath, somehow I felt anxious just because of that sigh.
-He then took both my hands in his, sending a thrill clean through me.
-Planting his frank, honest eyes on mine which soon were directed to the ground, he said: ‘Guanya Pau, nah Edear (I love you); ya in dear wah?’ (Do you love me?)
-What could I say but to whisper faintly: ‘Da keker’ (with all my heart).</t>
-        </is>
-      </c>
+          <t>Nyanken Hne</t>
+        </is>
+      </c>
+      <c r="F103" s="13" t="n"/>
+      <c r="G103" s="13" t="n"/>
       <c r="H103" s="13" t="inlineStr">
         <is>
-          <t>Joseph Jeffrey Walters (c.1860s–1894)</t>
+          <t>Patricia Jabbeh Wesley</t>
         </is>
       </c>
       <c r="I103" s="13" t="inlineStr">
         <is>
-          <t>Yes</t>
+          <t>No</t>
         </is>
       </c>
       <c r="J103" s="13" t="inlineStr">
         <is>
-          <t>Named work (text)</t>
+          <t>Named work</t>
         </is>
       </c>
       <c r="K103" s="13" t="inlineStr">
         <is>
-          <t>Prose / novel</t>
+          <t>Poetry</t>
         </is>
       </c>
       <c r="L103" s="13" t="inlineStr">
         <is>
-          <t>Men</t>
-        </is>
-      </c>
-      <c r="M103" s="14" t="n">
-        <v>1891</v>
+          <t>Women</t>
+        </is>
+      </c>
+      <c r="M103" s="14" t="inlineStr">
+        <is>
+          <t>1998</t>
+        </is>
       </c>
       <c r="N103" s="13" t="inlineStr">
         <is>
@@ -15435,81 +15328,60 @@
       <c r="O103" s="13" t="n"/>
       <c r="P103" s="13" t="inlineStr">
         <is>
-          <t>Novel</t>
+          <t>Poem</t>
         </is>
       </c>
       <c r="Q103" s="13" t="inlineStr">
         <is>
-          <t>Man author</t>
+          <t>Patricia Jabbeh Wesley</t>
         </is>
       </c>
       <c r="R103" s="13" t="inlineStr">
         <is>
-          <t>1891, Cleveland: Lauer &amp; Mattill</t>
-        </is>
-      </c>
-      <c r="S103" s="13" t="inlineStr">
-        <is>
-          <t>Historical work reproduced in linked digital source; modern editorial material is separate</t>
-        </is>
-      </c>
+          <t>1998</t>
+        </is>
+      </c>
+      <c r="S103" s="13" t="n"/>
       <c r="T103" s="13" t="inlineStr">
         <is>
-          <t>Guanya resists an arranged marriage because she loves Momo and seeks the freedom to choose her partner.</t>
+          <t>The poet celebrates her husband: the women and the whole town admire him as he passes, but his love has stayed with her alone.</t>
         </is>
       </c>
       <c r="U103" s="13" t="inlineStr">
         <is>
-          <t>University of Zurich hosts a facsimile of the original novel. Editor John Victor Singler documents the author’s Vai/Liberian origin and death on 12 November 1894.</t>
-        </is>
-      </c>
-      <c r="V103" s="13" t="inlineStr">
-        <is>
-          <t>Original p.24 and subsequent flight/courtship narrative</t>
-        </is>
-      </c>
+          <t>Patricia Jabbeh Wesley, Before the Palm Could Bloom: Poems of Africa (New Issues Press, 1998); text on the Scottish Poetry Library website.</t>
+        </is>
+      </c>
+      <c r="V103" s="13" t="n"/>
       <c r="W103" s="13" t="inlineStr">
         <is>
-          <t>Use the 1891 novel. Modern Broadview introduction and annotations are excluded. The work combines opposition to forced marriage with a nineteenth-century Christian missionary perspective.
-Passage update (29 October 2026): Nine consecutive sentences in which Guanya Pau tells how Momo declared his love (1891 edition, Internet Archive scan, pp. 128–129), including his words in Vai. OCR spacing and line-break hyphens tidied; the letters were checked against the scan text. Original English; no translation needed. Original English text; not a translation.</t>
+          <t>Work changed (30 October 2026) after the whole-poem review: Walters' Guanya Pau (1891), written from a missionary viewpoint, is replaced by a love poem by one of Liberia's leading poets.</t>
         </is>
       </c>
       <c r="X103" s="13" t="inlineStr">
         <is>
-          <t>Historical original text: standard life-plus-70 term has expired; author died 1894. Assessment excludes modern translations, commentary, editorial alterations, musical settings and recordings. Territorial and unusual publication-history exceptions are not comprehensively assessed.</t>
+          <t>In copyright: described and linked only; no text or recording is reproduced here. Whole-poem review, 30 October 2026.</t>
         </is>
       </c>
       <c r="Y103" s="13" t="inlineStr">
         <is>
-          <t>University of Zurich hosts a facsimile of the original novel. Editor John Victor Singler documents the author’s Vai/Liberian origin and death on 12 November 1894.</t>
+          <t>Patricia Jabbeh Wesley, Before the Palm Could Bloom: Poems of Africa (New Issues Press, 1998); text on the Scottish Poetry Library website.</t>
         </is>
       </c>
       <c r="Z103" s="11" t="inlineStr">
         <is>
-          <t>Read original</t>
-        </is>
-      </c>
-      <c r="AA103" s="11" t="inlineStr">
-        <is>
-          <t>Reuse basis / copyright duration</t>
-        </is>
-      </c>
-      <c r="AB103" s="11" t="inlineStr">
-        <is>
-          <t>Date / edition evidence</t>
-        </is>
-      </c>
-      <c r="AC103" s="11" t="inlineStr">
-        <is>
-          <t>Creator / country evidence</t>
-        </is>
-      </c>
-      <c r="AD103" s="11" t="inlineStr">
-        <is>
-          <t>Additional evidence</t>
-        </is>
-      </c>
-      <c r="AE103" s="11" t="n"/>
+          <t>Read the text</t>
+        </is>
+      </c>
+      <c r="AA103" s="11" t="n"/>
+      <c r="A